<commit_message>
📊 Horarios actualizados Línea 141 - 1785
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-03-21.xlsx
+++ b/data/horarios-141-2026-03-21.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E7"/>
+  <dimension ref="A1:E8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 01:19:36</t>
+          <t>Última actualización: 02:14:10</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 2</t>
+          <t>Total filas: 3</t>
         </is>
       </c>
     </row>
@@ -473,21 +473,21 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>01:19:36</t>
+          <t>02:14:10</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>01:58</t>
+          <t>02:57</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>215_ALUAR</t>
         </is>
       </c>
       <c r="D6" t="n">
-        <v>39</v>
+        <v>43</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
@@ -498,23 +498,48 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>01:19:36</t>
+          <t>02:14:10</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>02:56</t>
+          <t>03:48</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>215_ALUAR</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D7" t="n">
+        <v>94</v>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>02:14:10</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>03:51</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>83_ESC 6_ALUAR</t>
+        </is>
+      </c>
+      <c r="D8" t="n">
         <v>97</v>
       </c>
-      <c r="E7" t="inlineStr">
+      <c r="E8" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -544,7 +569,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 01:19:36</t>
+          <t>Última actualización: 02:14:10</t>
         </is>
       </c>
     </row>
@@ -585,12 +610,12 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>01:19:36</t>
+          <t>02:14:10</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>02:56</t>
+          <t>02:57</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -599,7 +624,7 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>97</v>
+        <v>43</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
@@ -631,7 +656,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 01:19:36</t>
+          <t>Última actualización: 02:14:10</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 1786
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-03-21.xlsx
+++ b/data/horarios-141-2026-03-21.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E8"/>
+  <dimension ref="A1:E11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 02:14:10</t>
+          <t>Última actualización: 02:55:00</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 3</t>
+          <t>Total filas: 6</t>
         </is>
       </c>
     </row>
@@ -473,7 +473,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>02:14:10</t>
+          <t>02:55:00</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -487,7 +487,7 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>43</v>
+        <v>2</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
@@ -498,7 +498,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>02:14:10</t>
+          <t>02:55:00</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -512,7 +512,7 @@
         </is>
       </c>
       <c r="D7" t="n">
-        <v>94</v>
+        <v>53</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
@@ -523,7 +523,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>02:14:10</t>
+          <t>02:55:00</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -537,9 +537,84 @@
         </is>
       </c>
       <c r="D8" t="n">
+        <v>56</v>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>02:55:00</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>04:32</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D9" t="n">
         <v>97</v>
       </c>
-      <c r="E8" t="inlineStr">
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>02:55:00</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>04:48</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D10" t="n">
+        <v>113</v>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>02:55:00</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>04:48</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D11" t="n">
+        <v>113</v>
+      </c>
+      <c r="E11" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -556,7 +631,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E6"/>
+  <dimension ref="A1:E7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -569,14 +644,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 02:14:10</t>
+          <t>Última actualización: 02:55:00</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 1</t>
+          <t>Total filas: 2</t>
         </is>
       </c>
     </row>
@@ -610,7 +685,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>02:14:10</t>
+          <t>02:55:00</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -624,9 +699,34 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>43</v>
+        <v>2</v>
       </c>
       <c r="E6" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>02:55:00</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>04:48</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D7" t="n">
+        <v>113</v>
+      </c>
+      <c r="E7" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -656,7 +756,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 02:14:10</t>
+          <t>Última actualización: 02:55:00</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 1787
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-03-21.xlsx
+++ b/data/horarios-141-2026-03-21.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E11"/>
+  <dimension ref="A1:E12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 02:55:00</t>
+          <t>Última actualización: 03:29:30</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 6</t>
+          <t>Total filas: 7</t>
         </is>
       </c>
     </row>
@@ -473,21 +473,21 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>02:55:00</t>
+          <t>03:29:30</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>02:57</t>
+          <t>03:48</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>215_ALUAR</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D6" t="n">
-        <v>2</v>
+        <v>19</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
@@ -498,21 +498,21 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>02:55:00</t>
+          <t>03:29:30</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>03:48</t>
+          <t>03:50</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>83_ESC 6_ALUAR</t>
         </is>
       </c>
       <c r="D7" t="n">
-        <v>53</v>
+        <v>21</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
@@ -523,21 +523,21 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>02:55:00</t>
+          <t>03:29:30</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>03:51</t>
+          <t>04:32</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>83_ESC 6_ALUAR</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D8" t="n">
-        <v>56</v>
+        <v>63</v>
       </c>
       <c r="E8" t="inlineStr">
         <is>
@@ -548,21 +548,21 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>02:55:00</t>
+          <t>03:29:30</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>04:32</t>
+          <t>04:48</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D9" t="n">
-        <v>97</v>
+        <v>79</v>
       </c>
       <c r="E9" t="inlineStr">
         <is>
@@ -573,7 +573,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>02:55:00</t>
+          <t>03:29:30</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -583,11 +583,11 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D10" t="n">
-        <v>113</v>
+        <v>79</v>
       </c>
       <c r="E10" t="inlineStr">
         <is>
@@ -598,23 +598,48 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>02:55:00</t>
+          <t>03:29:30</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>04:48</t>
+          <t>05:06</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D11" t="n">
-        <v>113</v>
+        <v>97</v>
       </c>
       <c r="E11" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>03:29:30</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>05:20</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D12" t="n">
+        <v>111</v>
+      </c>
+      <c r="E12" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -631,7 +656,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E7"/>
+  <dimension ref="A1:E6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -644,14 +669,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 02:55:00</t>
+          <t>Última actualización: 03:29:30</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 2</t>
+          <t>Total filas: 1</t>
         </is>
       </c>
     </row>
@@ -685,48 +710,23 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>02:55:00</t>
+          <t>03:29:30</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>02:57</t>
+          <t>04:48</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>215_ALUAR</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D6" t="n">
-        <v>2</v>
+        <v>79</v>
       </c>
       <c r="E6" t="inlineStr">
-        <is>
-          <t>LP1912</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>02:55:00</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>04:48</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>215A_EL PATO</t>
-        </is>
-      </c>
-      <c r="D7" t="n">
-        <v>113</v>
-      </c>
-      <c r="E7" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -756,7 +756,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 02:55:00</t>
+          <t>Última actualización: 03:29:30</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 1788
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-03-21.xlsx
+++ b/data/horarios-141-2026-03-21.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E12"/>
+  <dimension ref="A1:E18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 03:29:30</t>
+          <t>Última actualización: 04:08:30</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 7</t>
+          <t>Total filas: 13</t>
         </is>
       </c>
     </row>
@@ -473,12 +473,12 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>03:29:30</t>
+          <t>04:08:30</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>03:48</t>
+          <t>04:32</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -487,7 +487,7 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>19</v>
+        <v>24</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
@@ -498,21 +498,21 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>03:29:30</t>
+          <t>04:08:30</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>03:50</t>
+          <t>04:48</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>83_ESC 6_ALUAR</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D7" t="n">
-        <v>21</v>
+        <v>40</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
@@ -523,21 +523,21 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>03:29:30</t>
+          <t>04:08:30</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>04:32</t>
+          <t>04:48</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D8" t="n">
-        <v>63</v>
+        <v>40</v>
       </c>
       <c r="E8" t="inlineStr">
         <is>
@@ -548,21 +548,21 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>03:29:30</t>
+          <t>04:08:30</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>04:48</t>
+          <t>05:06</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D9" t="n">
-        <v>79</v>
+        <v>58</v>
       </c>
       <c r="E9" t="inlineStr">
         <is>
@@ -573,21 +573,21 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>03:29:30</t>
+          <t>04:08:30</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>04:48</t>
+          <t>05:09</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D10" t="n">
-        <v>79</v>
+        <v>61</v>
       </c>
       <c r="E10" t="inlineStr">
         <is>
@@ -598,21 +598,21 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>03:29:30</t>
+          <t>04:08:30</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>05:06</t>
+          <t>05:20</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D11" t="n">
-        <v>97</v>
+        <v>72</v>
       </c>
       <c r="E11" t="inlineStr">
         <is>
@@ -623,23 +623,173 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>03:29:30</t>
+          <t>04:08:30</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>05:20</t>
+          <t>05:29</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D12" t="n">
-        <v>111</v>
+        <v>81</v>
       </c>
       <c r="E12" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>04:08:30</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>05:29</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D13" t="n">
+        <v>81</v>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>04:08:30</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>05:30</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D14" t="n">
+        <v>82</v>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>04:08:30</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>05:40</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>14X44_ABASTO</t>
+        </is>
+      </c>
+      <c r="D15" t="n">
+        <v>92</v>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>04:08:30</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>05:42</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>84_COLONIA URQUIZA-ESC 49</t>
+        </is>
+      </c>
+      <c r="D16" t="n">
+        <v>94</v>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>04:08:30</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>05:45</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D17" t="n">
+        <v>97</v>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>04:08:30</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>05:48</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D18" t="n">
+        <v>100</v>
+      </c>
+      <c r="E18" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -656,7 +806,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E6"/>
+  <dimension ref="A1:E8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -669,14 +819,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 03:29:30</t>
+          <t>Última actualización: 04:08:30</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 1</t>
+          <t>Total filas: 3</t>
         </is>
       </c>
     </row>
@@ -710,7 +860,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>03:29:30</t>
+          <t>04:08:30</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -724,9 +874,59 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>79</v>
+        <v>40</v>
       </c>
       <c r="E6" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>04:08:30</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>05:29</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D7" t="n">
+        <v>81</v>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>04:08:30</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>05:48</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D8" t="n">
+        <v>100</v>
+      </c>
+      <c r="E8" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -743,7 +943,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A3"/>
+  <dimension ref="A1:E7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -756,14 +956,91 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 03:29:30</t>
+          <t>Última actualización: 04:08:30</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 0</t>
+          <t>Total filas: 2</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Hora_Scrap</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Hora_Llegada</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Linea</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Minutos</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Parada</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>04:08:30</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>05:29</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D6" t="n">
+        <v>81</v>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>04:08:30</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>06:04</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>215A_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D7" t="n">
+        <v>116</v>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>L6173</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 1789
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-03-21.xlsx
+++ b/data/horarios-141-2026-03-21.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E18"/>
+  <dimension ref="A1:E33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 04:08:30</t>
+          <t>Última actualización: 04:43:08</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 13</t>
+          <t>Total filas: 28</t>
         </is>
       </c>
     </row>
@@ -498,21 +498,21 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>04:08:30</t>
+          <t>04:43:08</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>04:48</t>
+          <t>04:47</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>215_EL PELIGRO</t>
         </is>
       </c>
       <c r="D7" t="n">
-        <v>40</v>
+        <v>4</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
@@ -533,7 +533,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D8" t="n">
@@ -553,16 +553,16 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>05:06</t>
+          <t>04:48</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D9" t="n">
-        <v>58</v>
+        <v>40</v>
       </c>
       <c r="E9" t="inlineStr">
         <is>
@@ -573,21 +573,21 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>04:08:30</t>
+          <t>04:43:08</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>05:09</t>
+          <t>04:53</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D10" t="n">
-        <v>61</v>
+        <v>10</v>
       </c>
       <c r="E10" t="inlineStr">
         <is>
@@ -603,16 +603,16 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>05:20</t>
+          <t>05:06</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D11" t="n">
-        <v>72</v>
+        <v>58</v>
       </c>
       <c r="E11" t="inlineStr">
         <is>
@@ -628,16 +628,16 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>05:29</t>
+          <t>05:09</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D12" t="n">
-        <v>81</v>
+        <v>61</v>
       </c>
       <c r="E12" t="inlineStr">
         <is>
@@ -648,21 +648,21 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>04:08:30</t>
+          <t>04:43:08</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>05:29</t>
+          <t>05:12</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D13" t="n">
-        <v>81</v>
+        <v>29</v>
       </c>
       <c r="E13" t="inlineStr">
         <is>
@@ -678,16 +678,16 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>05:30</t>
+          <t>05:20</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D14" t="n">
-        <v>82</v>
+        <v>72</v>
       </c>
       <c r="E14" t="inlineStr">
         <is>
@@ -698,21 +698,21 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>04:08:30</t>
+          <t>04:43:08</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>05:40</t>
+          <t>05:22</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>14X44_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D15" t="n">
-        <v>92</v>
+        <v>39</v>
       </c>
       <c r="E15" t="inlineStr">
         <is>
@@ -728,16 +728,16 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>05:42</t>
+          <t>05:29</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>84_COLONIA URQUIZA-ESC 49</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D16" t="n">
-        <v>94</v>
+        <v>81</v>
       </c>
       <c r="E16" t="inlineStr">
         <is>
@@ -753,16 +753,16 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>05:45</t>
+          <t>05:29</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D17" t="n">
-        <v>97</v>
+        <v>81</v>
       </c>
       <c r="E17" t="inlineStr">
         <is>
@@ -778,18 +778,393 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
+          <t>05:30</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D18" t="n">
+        <v>82</v>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>04:43:08</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>05:32</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>81_EL PELIGRO</t>
+        </is>
+      </c>
+      <c r="D19" t="n">
+        <v>49</v>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>04:08:30</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>05:40</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>14X44_ABASTO</t>
+        </is>
+      </c>
+      <c r="D20" t="n">
+        <v>92</v>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>04:08:30</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>05:42</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>84_COLONIA URQUIZA-ESC 49</t>
+        </is>
+      </c>
+      <c r="D21" t="n">
+        <v>94</v>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>04:43:08</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>05:44</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D22" t="n">
+        <v>61</v>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>04:08:30</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>05:45</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D23" t="n">
+        <v>97</v>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>04:08:30</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
           <t>05:48</t>
         </is>
       </c>
-      <c r="C18" t="inlineStr">
+      <c r="C24" t="inlineStr">
         <is>
           <t>215A_EL PATO</t>
         </is>
       </c>
-      <c r="D18" t="n">
+      <c r="D24" t="n">
         <v>100</v>
       </c>
-      <c r="E18" t="inlineStr">
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>04:43:08</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>05:52</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>17_ROMERO</t>
+        </is>
+      </c>
+      <c r="D25" t="n">
+        <v>69</v>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>04:43:08</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>06:01</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D26" t="n">
+        <v>78</v>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>04:43:08</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>06:04</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D27" t="n">
+        <v>81</v>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>04:43:08</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>06:11</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D28" t="n">
+        <v>88</v>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>04:43:08</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>06:24</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D29" t="n">
+        <v>101</v>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>04:43:08</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>06:27</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D30" t="n">
+        <v>104</v>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>04:43:08</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>06:31</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D31" t="n">
+        <v>108</v>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>04:43:08</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>06:31</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>17X38_ROMERO</t>
+        </is>
+      </c>
+      <c r="D32" t="n">
+        <v>108</v>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>04:43:08</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>06:39</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>225_C ROCA-H SUR</t>
+        </is>
+      </c>
+      <c r="D33" t="n">
+        <v>116</v>
+      </c>
+      <c r="E33" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -806,7 +1181,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E8"/>
+  <dimension ref="A1:E10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -819,14 +1194,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 04:08:30</t>
+          <t>Última actualización: 04:43:08</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 3</t>
+          <t>Total filas: 5</t>
         </is>
       </c>
     </row>
@@ -860,21 +1235,21 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>04:08:30</t>
+          <t>04:43:08</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>04:48</t>
+          <t>04:47</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>215_EL PELIGRO</t>
         </is>
       </c>
       <c r="D6" t="n">
-        <v>40</v>
+        <v>4</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
@@ -890,16 +1265,16 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>05:29</t>
+          <t>04:48</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D7" t="n">
-        <v>81</v>
+        <v>40</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
@@ -915,18 +1290,68 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
+          <t>05:29</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D8" t="n">
+        <v>81</v>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>04:08:30</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
           <t>05:48</t>
         </is>
       </c>
-      <c r="C8" t="inlineStr">
+      <c r="C9" t="inlineStr">
         <is>
           <t>215A_EL PATO</t>
         </is>
       </c>
-      <c r="D8" t="n">
+      <c r="D9" t="n">
         <v>100</v>
       </c>
-      <c r="E8" t="inlineStr">
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>04:43:08</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>06:11</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D10" t="n">
+        <v>88</v>
+      </c>
+      <c r="E10" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -943,7 +1368,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E7"/>
+  <dimension ref="A1:E8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -956,14 +1381,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 04:08:30</t>
+          <t>Última actualización: 04:43:08</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 2</t>
+          <t>Total filas: 3</t>
         </is>
       </c>
     </row>
@@ -1039,6 +1464,31 @@
         <v>116</v>
       </c>
       <c r="E7" t="inlineStr">
+        <is>
+          <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>04:43:08</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>06:05</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>215A_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D8" t="n">
+        <v>82</v>
+      </c>
+      <c r="E8" t="inlineStr">
         <is>
           <t>L6173</t>
         </is>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 1790
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-03-21.xlsx
+++ b/data/horarios-141-2026-03-21.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E33"/>
+  <dimension ref="A1:E36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 04:43:08</t>
+          <t>Última actualización: 04:59:30</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 28</t>
+          <t>Total filas: 31</t>
         </is>
       </c>
     </row>
@@ -533,7 +533,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D8" t="n">
@@ -558,7 +558,7 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D9" t="n">
@@ -648,12 +648,12 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>04:43:08</t>
+          <t>04:59:30</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>05:12</t>
+          <t>05:11</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -662,7 +662,7 @@
         </is>
       </c>
       <c r="D13" t="n">
-        <v>29</v>
+        <v>12</v>
       </c>
       <c r="E13" t="inlineStr">
         <is>
@@ -673,21 +673,21 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>04:08:30</t>
+          <t>04:43:08</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>05:20</t>
+          <t>05:12</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D14" t="n">
-        <v>72</v>
+        <v>29</v>
       </c>
       <c r="E14" t="inlineStr">
         <is>
@@ -698,21 +698,21 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>04:43:08</t>
+          <t>04:08:30</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>05:22</t>
+          <t>05:20</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D15" t="n">
-        <v>39</v>
+        <v>72</v>
       </c>
       <c r="E15" t="inlineStr">
         <is>
@@ -723,12 +723,12 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>04:08:30</t>
+          <t>04:59:30</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>05:29</t>
+          <t>05:22</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -737,7 +737,7 @@
         </is>
       </c>
       <c r="D16" t="n">
-        <v>81</v>
+        <v>23</v>
       </c>
       <c r="E16" t="inlineStr">
         <is>
@@ -758,7 +758,7 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D17" t="n">
@@ -778,16 +778,16 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>05:30</t>
+          <t>05:29</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D18" t="n">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="E18" t="inlineStr">
         <is>
@@ -798,21 +798,21 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>04:43:08</t>
+          <t>04:08:30</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>05:32</t>
+          <t>05:30</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>81_EL PELIGRO</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D19" t="n">
-        <v>49</v>
+        <v>82</v>
       </c>
       <c r="E19" t="inlineStr">
         <is>
@@ -823,21 +823,21 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>04:08:30</t>
+          <t>04:59:30</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>05:40</t>
+          <t>05:32</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>14X44_ABASTO</t>
+          <t>81_EL PELIGRO</t>
         </is>
       </c>
       <c r="D20" t="n">
-        <v>92</v>
+        <v>33</v>
       </c>
       <c r="E20" t="inlineStr">
         <is>
@@ -853,16 +853,16 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>05:42</t>
+          <t>05:40</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>84_COLONIA URQUIZA-ESC 49</t>
+          <t>14X44_ABASTO</t>
         </is>
       </c>
       <c r="D21" t="n">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="E21" t="inlineStr">
         <is>
@@ -873,21 +873,21 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>04:43:08</t>
+          <t>04:08:30</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>05:44</t>
+          <t>05:42</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>84_COLONIA URQUIZA-ESC 49</t>
         </is>
       </c>
       <c r="D22" t="n">
-        <v>61</v>
+        <v>94</v>
       </c>
       <c r="E22" t="inlineStr">
         <is>
@@ -898,21 +898,21 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>04:08:30</t>
+          <t>04:59:30</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>05:45</t>
+          <t>05:44</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D23" t="n">
-        <v>97</v>
+        <v>45</v>
       </c>
       <c r="E23" t="inlineStr">
         <is>
@@ -928,16 +928,16 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>05:48</t>
+          <t>05:45</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D24" t="n">
-        <v>100</v>
+        <v>97</v>
       </c>
       <c r="E24" t="inlineStr">
         <is>
@@ -948,21 +948,21 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>04:43:08</t>
+          <t>04:08:30</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>05:52</t>
+          <t>05:48</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D25" t="n">
-        <v>69</v>
+        <v>100</v>
       </c>
       <c r="E25" t="inlineStr">
         <is>
@@ -973,21 +973,21 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>04:43:08</t>
+          <t>04:59:30</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>06:01</t>
+          <t>05:52</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D26" t="n">
-        <v>78</v>
+        <v>53</v>
       </c>
       <c r="E26" t="inlineStr">
         <is>
@@ -998,21 +998,21 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>04:43:08</t>
+          <t>04:59:30</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>06:04</t>
+          <t>06:01</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D27" t="n">
-        <v>81</v>
+        <v>62</v>
       </c>
       <c r="E27" t="inlineStr">
         <is>
@@ -1023,21 +1023,21 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>04:43:08</t>
+          <t>04:59:30</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>06:11</t>
+          <t>06:04</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D28" t="n">
-        <v>88</v>
+        <v>65</v>
       </c>
       <c r="E28" t="inlineStr">
         <is>
@@ -1048,21 +1048,21 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>04:43:08</t>
+          <t>04:59:30</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>06:24</t>
+          <t>06:11</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D29" t="n">
-        <v>101</v>
+        <v>72</v>
       </c>
       <c r="E29" t="inlineStr">
         <is>
@@ -1073,21 +1073,21 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>04:43:08</t>
+          <t>04:59:30</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>06:27</t>
+          <t>06:24</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D30" t="n">
-        <v>104</v>
+        <v>85</v>
       </c>
       <c r="E30" t="inlineStr">
         <is>
@@ -1098,21 +1098,21 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>04:43:08</t>
+          <t>04:59:30</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>06:31</t>
+          <t>06:27</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D31" t="n">
-        <v>108</v>
+        <v>88</v>
       </c>
       <c r="E31" t="inlineStr">
         <is>
@@ -1123,7 +1123,7 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>04:43:08</t>
+          <t>04:59:30</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -1133,11 +1133,11 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D32" t="n">
-        <v>108</v>
+        <v>92</v>
       </c>
       <c r="E32" t="inlineStr">
         <is>
@@ -1148,23 +1148,98 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>04:43:08</t>
+          <t>04:59:30</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
+          <t>06:31</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>17X38_ROMERO</t>
+        </is>
+      </c>
+      <c r="D33" t="n">
+        <v>92</v>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>04:59:30</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
           <t>06:39</t>
         </is>
       </c>
-      <c r="C33" t="inlineStr">
+      <c r="C34" t="inlineStr">
         <is>
           <t>225_C ROCA-H SUR</t>
         </is>
       </c>
-      <c r="D33" t="n">
-        <v>116</v>
-      </c>
-      <c r="E33" t="inlineStr">
+      <c r="D34" t="n">
+        <v>100</v>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>04:59:30</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>06:51</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D35" t="n">
+        <v>112</v>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>04:59:30</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>06:54</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D36" t="n">
+        <v>115</v>
+      </c>
+      <c r="E36" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -1181,7 +1256,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E10"/>
+  <dimension ref="A1:E11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1194,14 +1269,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 04:43:08</t>
+          <t>Última actualización: 04:59:30</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 5</t>
+          <t>Total filas: 6</t>
         </is>
       </c>
     </row>
@@ -1335,7 +1410,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>04:43:08</t>
+          <t>04:59:30</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -1349,9 +1424,34 @@
         </is>
       </c>
       <c r="D10" t="n">
-        <v>88</v>
+        <v>72</v>
       </c>
       <c r="E10" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>04:59:30</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>06:51</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D11" t="n">
+        <v>112</v>
+      </c>
+      <c r="E11" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -1381,7 +1481,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 04:43:08</t>
+          <t>Última actualización: 04:59:30</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 1791
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-03-21.xlsx
+++ b/data/horarios-141-2026-03-21.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E36"/>
+  <dimension ref="A1:E42"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 04:59:30</t>
+          <t>Última actualización: 05:33:31</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 31</t>
+          <t>Total filas: 37</t>
         </is>
       </c>
     </row>
@@ -898,7 +898,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>04:59:30</t>
+          <t>05:33:31</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -912,7 +912,7 @@
         </is>
       </c>
       <c r="D23" t="n">
-        <v>45</v>
+        <v>11</v>
       </c>
       <c r="E23" t="inlineStr">
         <is>
@@ -973,7 +973,7 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>04:59:30</t>
+          <t>05:33:31</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -987,7 +987,7 @@
         </is>
       </c>
       <c r="D26" t="n">
-        <v>53</v>
+        <v>19</v>
       </c>
       <c r="E26" t="inlineStr">
         <is>
@@ -1023,12 +1023,12 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>04:59:30</t>
+          <t>05:33:31</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>06:04</t>
+          <t>06:03</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
@@ -1037,7 +1037,7 @@
         </is>
       </c>
       <c r="D28" t="n">
-        <v>65</v>
+        <v>30</v>
       </c>
       <c r="E28" t="inlineStr">
         <is>
@@ -1053,16 +1053,16 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>06:11</t>
+          <t>06:04</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D29" t="n">
-        <v>72</v>
+        <v>65</v>
       </c>
       <c r="E29" t="inlineStr">
         <is>
@@ -1073,21 +1073,21 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>04:59:30</t>
+          <t>05:33:31</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>06:24</t>
+          <t>06:11</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D30" t="n">
-        <v>85</v>
+        <v>38</v>
       </c>
       <c r="E30" t="inlineStr">
         <is>
@@ -1098,21 +1098,21 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>04:59:30</t>
+          <t>05:33:31</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>06:27</t>
+          <t>06:24</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D31" t="n">
-        <v>88</v>
+        <v>51</v>
       </c>
       <c r="E31" t="inlineStr">
         <is>
@@ -1123,21 +1123,21 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>04:59:30</t>
+          <t>05:33:31</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>06:31</t>
+          <t>06:27</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D32" t="n">
-        <v>92</v>
+        <v>54</v>
       </c>
       <c r="E32" t="inlineStr">
         <is>
@@ -1148,7 +1148,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>04:59:30</t>
+          <t>05:33:31</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -1162,7 +1162,7 @@
         </is>
       </c>
       <c r="D33" t="n">
-        <v>92</v>
+        <v>58</v>
       </c>
       <c r="E33" t="inlineStr">
         <is>
@@ -1173,21 +1173,21 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>04:59:30</t>
+          <t>05:33:31</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>06:39</t>
+          <t>06:31</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>225_C ROCA-H SUR</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D34" t="n">
-        <v>100</v>
+        <v>58</v>
       </c>
       <c r="E34" t="inlineStr">
         <is>
@@ -1198,21 +1198,21 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>04:59:30</t>
+          <t>05:33:31</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>06:51</t>
+          <t>06:39</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>225_C ROCA-H SUR</t>
         </is>
       </c>
       <c r="D35" t="n">
-        <v>112</v>
+        <v>66</v>
       </c>
       <c r="E35" t="inlineStr">
         <is>
@@ -1228,18 +1228,168 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
+          <t>06:51</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D36" t="n">
+        <v>112</v>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>05:33:31</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
           <t>06:54</t>
         </is>
       </c>
-      <c r="C36" t="inlineStr">
+      <c r="C37" t="inlineStr">
         <is>
           <t>14_ABASTO</t>
         </is>
       </c>
-      <c r="D36" t="n">
-        <v>115</v>
-      </c>
-      <c r="E36" t="inlineStr">
+      <c r="D37" t="n">
+        <v>81</v>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>05:33:31</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>07:01</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D38" t="n">
+        <v>88</v>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>05:33:31</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>07:04</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>225_GOMEZ</t>
+        </is>
+      </c>
+      <c r="D39" t="n">
+        <v>91</v>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>05:33:31</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>07:06</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D40" t="n">
+        <v>93</v>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>05:33:31</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>07:13</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>14X44_ABASTO</t>
+        </is>
+      </c>
+      <c r="D41" t="n">
+        <v>100</v>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>05:33:31</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>07:21</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D42" t="n">
+        <v>108</v>
+      </c>
+      <c r="E42" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -1256,7 +1406,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E11"/>
+  <dimension ref="A1:E13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1269,14 +1419,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 04:59:30</t>
+          <t>Última actualización: 05:33:31</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 6</t>
+          <t>Total filas: 8</t>
         </is>
       </c>
     </row>
@@ -1410,7 +1560,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>04:59:30</t>
+          <t>05:33:31</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -1424,7 +1574,7 @@
         </is>
       </c>
       <c r="D10" t="n">
-        <v>72</v>
+        <v>38</v>
       </c>
       <c r="E10" t="inlineStr">
         <is>
@@ -1452,6 +1602,56 @@
         <v>112</v>
       </c>
       <c r="E11" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>05:33:31</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>07:06</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D12" t="n">
+        <v>93</v>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>05:33:31</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>07:21</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D13" t="n">
+        <v>108</v>
+      </c>
+      <c r="E13" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -1468,7 +1668,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E8"/>
+  <dimension ref="A1:E9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1481,14 +1681,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 04:59:30</t>
+          <t>Última actualización: 05:33:31</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 3</t>
+          <t>Total filas: 4</t>
         </is>
       </c>
     </row>
@@ -1589,6 +1789,31 @@
         <v>82</v>
       </c>
       <c r="E8" t="inlineStr">
+        <is>
+          <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>05:33:31</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>07:27</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>215A_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D9" t="n">
+        <v>114</v>
+      </c>
+      <c r="E9" t="inlineStr">
         <is>
           <t>L6173</t>
         </is>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 1792
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-03-21.xlsx
+++ b/data/horarios-141-2026-03-21.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E42"/>
+  <dimension ref="A1:E48"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 05:33:31</t>
+          <t>Última actualización: 06:00:32</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 37</t>
+          <t>Total filas: 43</t>
         </is>
       </c>
     </row>
@@ -533,7 +533,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D8" t="n">
@@ -558,7 +558,7 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D9" t="n">
@@ -1023,7 +1023,7 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>05:33:31</t>
+          <t>06:00:32</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -1037,7 +1037,7 @@
         </is>
       </c>
       <c r="D28" t="n">
-        <v>30</v>
+        <v>3</v>
       </c>
       <c r="E28" t="inlineStr">
         <is>
@@ -1073,7 +1073,7 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>05:33:31</t>
+          <t>06:00:32</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -1087,7 +1087,7 @@
         </is>
       </c>
       <c r="D30" t="n">
-        <v>38</v>
+        <v>11</v>
       </c>
       <c r="E30" t="inlineStr">
         <is>
@@ -1098,7 +1098,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>05:33:31</t>
+          <t>06:00:32</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -1112,7 +1112,7 @@
         </is>
       </c>
       <c r="D31" t="n">
-        <v>51</v>
+        <v>24</v>
       </c>
       <c r="E31" t="inlineStr">
         <is>
@@ -1123,7 +1123,7 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>05:33:31</t>
+          <t>06:00:32</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -1137,7 +1137,7 @@
         </is>
       </c>
       <c r="D32" t="n">
-        <v>54</v>
+        <v>27</v>
       </c>
       <c r="E32" t="inlineStr">
         <is>
@@ -1148,7 +1148,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>05:33:31</t>
+          <t>06:00:32</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -1158,11 +1158,11 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D33" t="n">
-        <v>58</v>
+        <v>31</v>
       </c>
       <c r="E33" t="inlineStr">
         <is>
@@ -1173,7 +1173,7 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>05:33:31</t>
+          <t>06:00:32</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -1183,11 +1183,11 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D34" t="n">
-        <v>58</v>
+        <v>31</v>
       </c>
       <c r="E34" t="inlineStr">
         <is>
@@ -1198,7 +1198,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>05:33:31</t>
+          <t>06:00:32</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -1212,7 +1212,7 @@
         </is>
       </c>
       <c r="D35" t="n">
-        <v>66</v>
+        <v>39</v>
       </c>
       <c r="E35" t="inlineStr">
         <is>
@@ -1248,7 +1248,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>05:33:31</t>
+          <t>06:00:32</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -1262,7 +1262,7 @@
         </is>
       </c>
       <c r="D37" t="n">
-        <v>81</v>
+        <v>54</v>
       </c>
       <c r="E37" t="inlineStr">
         <is>
@@ -1273,7 +1273,7 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>05:33:31</t>
+          <t>06:00:32</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
@@ -1287,7 +1287,7 @@
         </is>
       </c>
       <c r="D38" t="n">
-        <v>88</v>
+        <v>61</v>
       </c>
       <c r="E38" t="inlineStr">
         <is>
@@ -1298,7 +1298,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>05:33:31</t>
+          <t>06:00:32</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -1312,7 +1312,7 @@
         </is>
       </c>
       <c r="D39" t="n">
-        <v>91</v>
+        <v>64</v>
       </c>
       <c r="E39" t="inlineStr">
         <is>
@@ -1323,7 +1323,7 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>05:33:31</t>
+          <t>06:00:32</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
@@ -1337,7 +1337,7 @@
         </is>
       </c>
       <c r="D40" t="n">
-        <v>93</v>
+        <v>66</v>
       </c>
       <c r="E40" t="inlineStr">
         <is>
@@ -1348,7 +1348,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>05:33:31</t>
+          <t>06:00:32</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
@@ -1362,7 +1362,7 @@
         </is>
       </c>
       <c r="D41" t="n">
-        <v>100</v>
+        <v>73</v>
       </c>
       <c r="E41" t="inlineStr">
         <is>
@@ -1373,7 +1373,7 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>05:33:31</t>
+          <t>06:00:32</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -1387,9 +1387,159 @@
         </is>
       </c>
       <c r="D42" t="n">
-        <v>108</v>
+        <v>81</v>
       </c>
       <c r="E42" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>06:00:32</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>07:29</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D43" t="n">
+        <v>89</v>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>06:00:32</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>07:33</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D44" t="n">
+        <v>93</v>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>06:00:32</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>07:36</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D45" t="n">
+        <v>96</v>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>06:00:32</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>07:36</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>17X38_ROMERO</t>
+        </is>
+      </c>
+      <c r="D46" t="n">
+        <v>96</v>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>06:00:32</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>07:43</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D47" t="n">
+        <v>103</v>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>06:00:32</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>07:49</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D48" t="n">
+        <v>109</v>
+      </c>
+      <c r="E48" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -1419,7 +1569,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 05:33:31</t>
+          <t>Última actualización: 06:00:32</t>
         </is>
       </c>
     </row>
@@ -1560,7 +1710,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>05:33:31</t>
+          <t>06:00:32</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -1574,7 +1724,7 @@
         </is>
       </c>
       <c r="D10" t="n">
-        <v>38</v>
+        <v>11</v>
       </c>
       <c r="E10" t="inlineStr">
         <is>
@@ -1610,7 +1760,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>05:33:31</t>
+          <t>06:00:32</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -1624,7 +1774,7 @@
         </is>
       </c>
       <c r="D12" t="n">
-        <v>93</v>
+        <v>66</v>
       </c>
       <c r="E12" t="inlineStr">
         <is>
@@ -1635,7 +1785,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>05:33:31</t>
+          <t>06:00:32</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -1649,7 +1799,7 @@
         </is>
       </c>
       <c r="D13" t="n">
-        <v>108</v>
+        <v>81</v>
       </c>
       <c r="E13" t="inlineStr">
         <is>
@@ -1681,7 +1831,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 05:33:31</t>
+          <t>Última actualización: 06:00:32</t>
         </is>
       </c>
     </row>
@@ -1797,7 +1947,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>05:33:31</t>
+          <t>06:00:32</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -1811,7 +1961,7 @@
         </is>
       </c>
       <c r="D9" t="n">
-        <v>114</v>
+        <v>87</v>
       </c>
       <c r="E9" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 1793
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-03-21.xlsx
+++ b/data/horarios-141-2026-03-21.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E48"/>
+  <dimension ref="A1:E59"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 06:00:32</t>
+          <t>Última actualización: 06:42:23</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 43</t>
+          <t>Total filas: 54</t>
         </is>
       </c>
     </row>
@@ -533,7 +533,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D8" t="n">
@@ -558,7 +558,7 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D9" t="n">
@@ -1223,7 +1223,7 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>04:59:30</t>
+          <t>06:42:23</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
@@ -1237,7 +1237,7 @@
         </is>
       </c>
       <c r="D36" t="n">
-        <v>112</v>
+        <v>9</v>
       </c>
       <c r="E36" t="inlineStr">
         <is>
@@ -1248,7 +1248,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>06:00:32</t>
+          <t>06:42:23</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -1262,7 +1262,7 @@
         </is>
       </c>
       <c r="D37" t="n">
-        <v>54</v>
+        <v>12</v>
       </c>
       <c r="E37" t="inlineStr">
         <is>
@@ -1273,7 +1273,7 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>06:00:32</t>
+          <t>06:42:23</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
@@ -1287,7 +1287,7 @@
         </is>
       </c>
       <c r="D38" t="n">
-        <v>61</v>
+        <v>19</v>
       </c>
       <c r="E38" t="inlineStr">
         <is>
@@ -1298,7 +1298,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>06:00:32</t>
+          <t>06:42:23</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -1312,7 +1312,7 @@
         </is>
       </c>
       <c r="D39" t="n">
-        <v>64</v>
+        <v>22</v>
       </c>
       <c r="E39" t="inlineStr">
         <is>
@@ -1348,21 +1348,21 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>06:00:32</t>
+          <t>06:42:23</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>07:13</t>
+          <t>07:07</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>14X44_ABASTO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D41" t="n">
-        <v>73</v>
+        <v>25</v>
       </c>
       <c r="E41" t="inlineStr">
         <is>
@@ -1378,16 +1378,16 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>07:21</t>
+          <t>07:13</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>14X44_ABASTO</t>
         </is>
       </c>
       <c r="D42" t="n">
-        <v>81</v>
+        <v>73</v>
       </c>
       <c r="E42" t="inlineStr">
         <is>
@@ -1398,21 +1398,21 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>06:00:32</t>
+          <t>06:42:23</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>07:29</t>
+          <t>07:14</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>14X44_ABASTO</t>
         </is>
       </c>
       <c r="D43" t="n">
-        <v>89</v>
+        <v>32</v>
       </c>
       <c r="E43" t="inlineStr">
         <is>
@@ -1423,21 +1423,21 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>06:00:32</t>
+          <t>06:42:23</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>07:33</t>
+          <t>07:21</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D44" t="n">
-        <v>93</v>
+        <v>39</v>
       </c>
       <c r="E44" t="inlineStr">
         <is>
@@ -1448,21 +1448,21 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>06:00:32</t>
+          <t>06:42:23</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>07:36</t>
+          <t>07:24</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D45" t="n">
-        <v>96</v>
+        <v>42</v>
       </c>
       <c r="E45" t="inlineStr">
         <is>
@@ -1473,21 +1473,21 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>06:00:32</t>
+          <t>06:42:23</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>07:36</t>
+          <t>07:29</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D46" t="n">
-        <v>96</v>
+        <v>47</v>
       </c>
       <c r="E46" t="inlineStr">
         <is>
@@ -1498,21 +1498,21 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>06:00:32</t>
+          <t>06:42:23</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>07:43</t>
+          <t>07:33</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D47" t="n">
-        <v>103</v>
+        <v>51</v>
       </c>
       <c r="E47" t="inlineStr">
         <is>
@@ -1528,18 +1528,293 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
+          <t>07:36</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D48" t="n">
+        <v>96</v>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>06:42:23</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>07:36</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>17X38_ROMERO</t>
+        </is>
+      </c>
+      <c r="D49" t="n">
+        <v>54</v>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>06:42:23</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>07:37</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D50" t="n">
+        <v>55</v>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>06:00:32</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>07:43</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D51" t="n">
+        <v>103</v>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>06:42:23</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>07:44</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D52" t="n">
+        <v>62</v>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>06:42:23</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
           <t>07:49</t>
         </is>
       </c>
-      <c r="C48" t="inlineStr">
+      <c r="C53" t="inlineStr">
         <is>
           <t>15_ABASTO</t>
         </is>
       </c>
-      <c r="D48" t="n">
-        <v>109</v>
-      </c>
-      <c r="E48" t="inlineStr">
+      <c r="D53" t="n">
+        <v>67</v>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>06:42:23</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>07:58</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D54" t="n">
+        <v>76</v>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>06:42:23</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>07:59</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D55" t="n">
+        <v>77</v>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>06:42:23</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>08:03</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>17X38_ROMERO</t>
+        </is>
+      </c>
+      <c r="D56" t="n">
+        <v>81</v>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>06:42:23</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>08:14</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D57" t="n">
+        <v>92</v>
+      </c>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>06:42:23</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>08:19</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D58" t="n">
+        <v>97</v>
+      </c>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>06:42:23</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>08:34</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D59" t="n">
+        <v>112</v>
+      </c>
+      <c r="E59" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -1556,7 +1831,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E13"/>
+  <dimension ref="A1:E15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1569,14 +1844,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 06:00:32</t>
+          <t>Última actualización: 06:42:23</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 8</t>
+          <t>Total filas: 10</t>
         </is>
       </c>
     </row>
@@ -1735,7 +2010,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>04:59:30</t>
+          <t>06:42:23</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -1749,7 +2024,7 @@
         </is>
       </c>
       <c r="D11" t="n">
-        <v>112</v>
+        <v>9</v>
       </c>
       <c r="E11" t="inlineStr">
         <is>
@@ -1785,23 +2060,73 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>06:00:32</t>
+          <t>06:42:23</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
+          <t>07:07</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D13" t="n">
+        <v>25</v>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>06:42:23</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
           <t>07:21</t>
         </is>
       </c>
-      <c r="C13" t="inlineStr">
+      <c r="C14" t="inlineStr">
         <is>
           <t>215A_EL PATO</t>
         </is>
       </c>
-      <c r="D13" t="n">
-        <v>81</v>
-      </c>
-      <c r="E13" t="inlineStr">
+      <c r="D14" t="n">
+        <v>39</v>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>06:42:23</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>08:34</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D15" t="n">
+        <v>112</v>
+      </c>
+      <c r="E15" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -1818,7 +2143,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E9"/>
+  <dimension ref="A1:E12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1831,14 +2156,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 06:00:32</t>
+          <t>Última actualización: 06:42:23</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 4</t>
+          <t>Total filas: 7</t>
         </is>
       </c>
     </row>
@@ -1966,6 +2291,81 @@
       <c r="E9" t="inlineStr">
         <is>
           <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>06:42:23</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>07:42</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>215A_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D10" t="n">
+        <v>60</v>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>06:42:23</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>08:10</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>215A_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D11" t="n">
+        <v>88</v>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>06:42:23</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>08:23</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D12" t="n">
+        <v>101</v>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>L6203</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 1794
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-03-21.xlsx
+++ b/data/horarios-141-2026-03-21.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E59"/>
+  <dimension ref="A1:E64"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 06:42:23</t>
+          <t>Última actualización: 06:59:30</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 54</t>
+          <t>Total filas: 59</t>
         </is>
       </c>
     </row>
@@ -758,7 +758,7 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D17" t="n">
@@ -783,7 +783,7 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D18" t="n">
@@ -1273,7 +1273,7 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>06:42:23</t>
+          <t>06:59:30</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
@@ -1287,7 +1287,7 @@
         </is>
       </c>
       <c r="D38" t="n">
-        <v>19</v>
+        <v>2</v>
       </c>
       <c r="E38" t="inlineStr">
         <is>
@@ -1298,7 +1298,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>06:42:23</t>
+          <t>06:59:30</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -1312,7 +1312,7 @@
         </is>
       </c>
       <c r="D39" t="n">
-        <v>22</v>
+        <v>5</v>
       </c>
       <c r="E39" t="inlineStr">
         <is>
@@ -1323,7 +1323,7 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>06:00:32</t>
+          <t>06:59:30</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
@@ -1337,7 +1337,7 @@
         </is>
       </c>
       <c r="D40" t="n">
-        <v>66</v>
+        <v>7</v>
       </c>
       <c r="E40" t="inlineStr">
         <is>
@@ -1373,7 +1373,7 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>06:00:32</t>
+          <t>06:59:30</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -1387,7 +1387,7 @@
         </is>
       </c>
       <c r="D42" t="n">
-        <v>73</v>
+        <v>14</v>
       </c>
       <c r="E42" t="inlineStr">
         <is>
@@ -1423,7 +1423,7 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>06:42:23</t>
+          <t>06:59:30</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
@@ -1437,7 +1437,7 @@
         </is>
       </c>
       <c r="D44" t="n">
-        <v>39</v>
+        <v>22</v>
       </c>
       <c r="E44" t="inlineStr">
         <is>
@@ -1473,7 +1473,7 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>06:42:23</t>
+          <t>06:59:30</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
@@ -1487,7 +1487,7 @@
         </is>
       </c>
       <c r="D46" t="n">
-        <v>47</v>
+        <v>30</v>
       </c>
       <c r="E46" t="inlineStr">
         <is>
@@ -1498,7 +1498,7 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>06:42:23</t>
+          <t>06:59:30</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
@@ -1512,7 +1512,7 @@
         </is>
       </c>
       <c r="D47" t="n">
-        <v>51</v>
+        <v>34</v>
       </c>
       <c r="E47" t="inlineStr">
         <is>
@@ -1523,7 +1523,7 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>06:00:32</t>
+          <t>06:59:30</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
@@ -1537,7 +1537,7 @@
         </is>
       </c>
       <c r="D48" t="n">
-        <v>96</v>
+        <v>37</v>
       </c>
       <c r="E48" t="inlineStr">
         <is>
@@ -1548,7 +1548,7 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>06:42:23</t>
+          <t>06:59:30</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
@@ -1562,7 +1562,7 @@
         </is>
       </c>
       <c r="D49" t="n">
-        <v>54</v>
+        <v>37</v>
       </c>
       <c r="E49" t="inlineStr">
         <is>
@@ -1598,7 +1598,7 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>06:00:32</t>
+          <t>06:59:30</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
@@ -1612,7 +1612,7 @@
         </is>
       </c>
       <c r="D51" t="n">
-        <v>103</v>
+        <v>44</v>
       </c>
       <c r="E51" t="inlineStr">
         <is>
@@ -1648,7 +1648,7 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>06:42:23</t>
+          <t>06:59:30</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
@@ -1662,7 +1662,7 @@
         </is>
       </c>
       <c r="D53" t="n">
-        <v>67</v>
+        <v>50</v>
       </c>
       <c r="E53" t="inlineStr">
         <is>
@@ -1673,12 +1673,12 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>06:42:23</t>
+          <t>06:59:30</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>07:58</t>
+          <t>07:55</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
@@ -1687,7 +1687,7 @@
         </is>
       </c>
       <c r="D54" t="n">
-        <v>76</v>
+        <v>56</v>
       </c>
       <c r="E54" t="inlineStr">
         <is>
@@ -1703,16 +1703,16 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>07:59</t>
+          <t>07:58</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D55" t="n">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="E55" t="inlineStr">
         <is>
@@ -1723,21 +1723,21 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>06:42:23</t>
+          <t>06:59:30</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>08:03</t>
+          <t>07:59</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D56" t="n">
-        <v>81</v>
+        <v>60</v>
       </c>
       <c r="E56" t="inlineStr">
         <is>
@@ -1748,21 +1748,21 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>06:42:23</t>
+          <t>06:59:30</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>08:14</t>
+          <t>08:01</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D57" t="n">
-        <v>92</v>
+        <v>62</v>
       </c>
       <c r="E57" t="inlineStr">
         <is>
@@ -1773,21 +1773,21 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>06:42:23</t>
+          <t>06:59:30</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>08:19</t>
+          <t>08:03</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D58" t="n">
-        <v>97</v>
+        <v>64</v>
       </c>
       <c r="E58" t="inlineStr">
         <is>
@@ -1798,23 +1798,148 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>06:42:23</t>
+          <t>06:59:30</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
+          <t>08:14</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D59" t="n">
+        <v>75</v>
+      </c>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>06:59:30</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>08:19</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D60" t="n">
+        <v>80</v>
+      </c>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>06:59:30</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>08:29</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D61" t="n">
+        <v>90</v>
+      </c>
+      <c r="E61" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>06:59:30</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
           <t>08:34</t>
         </is>
       </c>
-      <c r="C59" t="inlineStr">
+      <c r="C62" t="inlineStr">
         <is>
           <t>215C_EL PATO</t>
         </is>
       </c>
-      <c r="D59" t="n">
+      <c r="D62" t="n">
+        <v>95</v>
+      </c>
+      <c r="E62" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>06:59:30</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>08:48</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D63" t="n">
+        <v>109</v>
+      </c>
+      <c r="E63" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>06:59:30</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>08:51</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>16_P MOR-SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D64" t="n">
         <v>112</v>
       </c>
-      <c r="E59" t="inlineStr">
+      <c r="E64" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -1831,7 +1956,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E15"/>
+  <dimension ref="A1:E16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1844,14 +1969,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 06:42:23</t>
+          <t>Última actualización: 06:59:30</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 10</t>
+          <t>Total filas: 11</t>
         </is>
       </c>
     </row>
@@ -2035,7 +2160,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>06:00:32</t>
+          <t>06:59:30</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -2049,7 +2174,7 @@
         </is>
       </c>
       <c r="D12" t="n">
-        <v>66</v>
+        <v>7</v>
       </c>
       <c r="E12" t="inlineStr">
         <is>
@@ -2085,7 +2210,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>06:42:23</t>
+          <t>06:59:30</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -2099,7 +2224,7 @@
         </is>
       </c>
       <c r="D14" t="n">
-        <v>39</v>
+        <v>22</v>
       </c>
       <c r="E14" t="inlineStr">
         <is>
@@ -2110,7 +2235,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>06:42:23</t>
+          <t>06:59:30</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -2124,9 +2249,34 @@
         </is>
       </c>
       <c r="D15" t="n">
-        <v>112</v>
+        <v>95</v>
       </c>
       <c r="E15" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>06:59:30</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>08:48</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D16" t="n">
+        <v>109</v>
+      </c>
+      <c r="E16" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -2156,7 +2306,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 06:42:23</t>
+          <t>Última actualización: 06:59:30</t>
         </is>
       </c>
     </row>
@@ -2297,7 +2447,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>06:42:23</t>
+          <t>06:59:30</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -2311,7 +2461,7 @@
         </is>
       </c>
       <c r="D10" t="n">
-        <v>60</v>
+        <v>43</v>
       </c>
       <c r="E10" t="inlineStr">
         <is>
@@ -2322,7 +2472,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>06:42:23</t>
+          <t>06:59:30</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -2336,7 +2486,7 @@
         </is>
       </c>
       <c r="D11" t="n">
-        <v>88</v>
+        <v>71</v>
       </c>
       <c r="E11" t="inlineStr">
         <is>
@@ -2347,7 +2497,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>06:42:23</t>
+          <t>06:59:30</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -2361,7 +2511,7 @@
         </is>
       </c>
       <c r="D12" t="n">
-        <v>101</v>
+        <v>84</v>
       </c>
       <c r="E12" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 1795
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-03-21.xlsx
+++ b/data/horarios-141-2026-03-21.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E64"/>
+  <dimension ref="A1:E71"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 06:59:30</t>
+          <t>Última actualización: 07:27:35</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 59</t>
+          <t>Total filas: 66</t>
         </is>
       </c>
     </row>
@@ -1473,21 +1473,21 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>06:59:30</t>
+          <t>07:27:35</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>07:29</t>
+          <t>07:27</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D46" t="n">
-        <v>30</v>
+        <v>0</v>
       </c>
       <c r="E46" t="inlineStr">
         <is>
@@ -1498,21 +1498,21 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>06:59:30</t>
+          <t>07:27:35</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>07:33</t>
+          <t>07:29</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D47" t="n">
-        <v>34</v>
+        <v>2</v>
       </c>
       <c r="E47" t="inlineStr">
         <is>
@@ -1528,16 +1528,16 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>07:36</t>
+          <t>07:33</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D48" t="n">
-        <v>37</v>
+        <v>34</v>
       </c>
       <c r="E48" t="inlineStr">
         <is>
@@ -1548,7 +1548,7 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>06:59:30</t>
+          <t>07:27:35</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
@@ -1558,11 +1558,11 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D49" t="n">
-        <v>37</v>
+        <v>9</v>
       </c>
       <c r="E49" t="inlineStr">
         <is>
@@ -1573,21 +1573,21 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>06:42:23</t>
+          <t>07:27:35</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>07:37</t>
+          <t>07:36</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D50" t="n">
-        <v>55</v>
+        <v>9</v>
       </c>
       <c r="E50" t="inlineStr">
         <is>
@@ -1598,21 +1598,21 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>06:59:30</t>
+          <t>06:42:23</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>07:43</t>
+          <t>07:37</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D51" t="n">
-        <v>44</v>
+        <v>55</v>
       </c>
       <c r="E51" t="inlineStr">
         <is>
@@ -1623,12 +1623,12 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>06:42:23</t>
+          <t>07:27:35</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>07:44</t>
+          <t>07:43</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
@@ -1637,7 +1637,7 @@
         </is>
       </c>
       <c r="D52" t="n">
-        <v>62</v>
+        <v>16</v>
       </c>
       <c r="E52" t="inlineStr">
         <is>
@@ -1648,21 +1648,21 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>06:59:30</t>
+          <t>06:42:23</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>07:49</t>
+          <t>07:44</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D53" t="n">
-        <v>50</v>
+        <v>62</v>
       </c>
       <c r="E53" t="inlineStr">
         <is>
@@ -1673,21 +1673,21 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>06:59:30</t>
+          <t>07:27:35</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>07:55</t>
+          <t>07:49</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D54" t="n">
-        <v>56</v>
+        <v>22</v>
       </c>
       <c r="E54" t="inlineStr">
         <is>
@@ -1698,12 +1698,12 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>06:42:23</t>
+          <t>07:27:35</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>07:58</t>
+          <t>07:54</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
@@ -1712,7 +1712,7 @@
         </is>
       </c>
       <c r="D55" t="n">
-        <v>76</v>
+        <v>27</v>
       </c>
       <c r="E55" t="inlineStr">
         <is>
@@ -1728,16 +1728,16 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>07:59</t>
+          <t>07:55</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D56" t="n">
-        <v>60</v>
+        <v>56</v>
       </c>
       <c r="E56" t="inlineStr">
         <is>
@@ -1748,21 +1748,21 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>06:59:30</t>
+          <t>07:27:35</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>08:01</t>
+          <t>07:58</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D57" t="n">
-        <v>62</v>
+        <v>31</v>
       </c>
       <c r="E57" t="inlineStr">
         <is>
@@ -1773,21 +1773,21 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>06:59:30</t>
+          <t>07:27:35</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>08:03</t>
+          <t>07:59</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D58" t="n">
-        <v>64</v>
+        <v>32</v>
       </c>
       <c r="E58" t="inlineStr">
         <is>
@@ -1798,21 +1798,21 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>06:59:30</t>
+          <t>07:27:35</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>08:14</t>
+          <t>08:01</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D59" t="n">
-        <v>75</v>
+        <v>34</v>
       </c>
       <c r="E59" t="inlineStr">
         <is>
@@ -1823,21 +1823,21 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>06:59:30</t>
+          <t>07:27:35</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>08:19</t>
+          <t>08:03</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D60" t="n">
-        <v>80</v>
+        <v>36</v>
       </c>
       <c r="E60" t="inlineStr">
         <is>
@@ -1853,16 +1853,16 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>08:29</t>
+          <t>08:14</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D61" t="n">
-        <v>90</v>
+        <v>75</v>
       </c>
       <c r="E61" t="inlineStr">
         <is>
@@ -1873,21 +1873,21 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>06:59:30</t>
+          <t>07:27:35</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>08:34</t>
+          <t>08:19</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D62" t="n">
-        <v>95</v>
+        <v>52</v>
       </c>
       <c r="E62" t="inlineStr">
         <is>
@@ -1898,21 +1898,21 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>06:59:30</t>
+          <t>07:27:35</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>08:48</t>
+          <t>08:19</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D63" t="n">
-        <v>109</v>
+        <v>52</v>
       </c>
       <c r="E63" t="inlineStr">
         <is>
@@ -1923,23 +1923,198 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>06:59:30</t>
+          <t>07:27:35</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
         <is>
+          <t>08:29</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D64" t="n">
+        <v>62</v>
+      </c>
+      <c r="E64" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>07:27:35</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>08:34</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D65" t="n">
+        <v>67</v>
+      </c>
+      <c r="E65" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>07:27:35</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>08:48</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D66" t="n">
+        <v>81</v>
+      </c>
+      <c r="E66" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>07:27:35</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
           <t>08:51</t>
         </is>
       </c>
-      <c r="C64" t="inlineStr">
+      <c r="C67" t="inlineStr">
         <is>
           <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
-      <c r="D64" t="n">
+      <c r="D67" t="n">
+        <v>84</v>
+      </c>
+      <c r="E67" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>07:27:35</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>08:59</t>
+        </is>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D68" t="n">
+        <v>92</v>
+      </c>
+      <c r="E68" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>07:27:35</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>09:14</t>
+        </is>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D69" t="n">
+        <v>107</v>
+      </c>
+      <c r="E69" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>07:27:35</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>09:16</t>
+        </is>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D70" t="n">
+        <v>109</v>
+      </c>
+      <c r="E70" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>07:27:35</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>09:19</t>
+        </is>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>215_EL PELIGRO</t>
+        </is>
+      </c>
+      <c r="D71" t="n">
         <v>112</v>
       </c>
-      <c r="E64" t="inlineStr">
+      <c r="E71" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -1956,7 +2131,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E16"/>
+  <dimension ref="A1:E18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1969,14 +2144,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 06:59:30</t>
+          <t>Última actualización: 07:27:35</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 11</t>
+          <t>Total filas: 13</t>
         </is>
       </c>
     </row>
@@ -2235,7 +2410,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>06:59:30</t>
+          <t>07:27:35</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -2249,7 +2424,7 @@
         </is>
       </c>
       <c r="D15" t="n">
-        <v>95</v>
+        <v>67</v>
       </c>
       <c r="E15" t="inlineStr">
         <is>
@@ -2260,7 +2435,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>06:59:30</t>
+          <t>07:27:35</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -2274,9 +2449,59 @@
         </is>
       </c>
       <c r="D16" t="n">
-        <v>109</v>
+        <v>81</v>
       </c>
       <c r="E16" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>07:27:35</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>08:59</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D17" t="n">
+        <v>92</v>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>07:27:35</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>09:19</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>215_EL PELIGRO</t>
+        </is>
+      </c>
+      <c r="D18" t="n">
+        <v>112</v>
+      </c>
+      <c r="E18" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -2293,7 +2518,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E12"/>
+  <dimension ref="A1:E15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2306,14 +2531,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 06:59:30</t>
+          <t>Última actualización: 07:27:35</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 7</t>
+          <t>Total filas: 10</t>
         </is>
       </c>
     </row>
@@ -2472,12 +2697,12 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>06:59:30</t>
+          <t>07:27:35</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>08:10</t>
+          <t>07:45</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -2486,7 +2711,7 @@
         </is>
       </c>
       <c r="D11" t="n">
-        <v>71</v>
+        <v>18</v>
       </c>
       <c r="E11" t="inlineStr">
         <is>
@@ -2502,20 +2727,95 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
+          <t>08:10</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>215A_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D12" t="n">
+        <v>71</v>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>07:27:35</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>08:22</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D13" t="n">
+        <v>55</v>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>06:59:30</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
           <t>08:23</t>
         </is>
       </c>
-      <c r="C12" t="inlineStr">
+      <c r="C14" t="inlineStr">
         <is>
           <t>215C_LA PLATA</t>
         </is>
       </c>
-      <c r="D12" t="n">
+      <c r="D14" t="n">
         <v>84</v>
       </c>
-      <c r="E12" t="inlineStr">
+      <c r="E14" t="inlineStr">
         <is>
           <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>07:27:35</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>08:33</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>215A_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D15" t="n">
+        <v>66</v>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>L6173</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 1796
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-03-21.xlsx
+++ b/data/horarios-141-2026-03-21.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E71"/>
+  <dimension ref="A1:E83"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 07:27:35</t>
+          <t>Última actualización: 07:51:37</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 66</t>
+          <t>Total filas: 78</t>
         </is>
       </c>
     </row>
@@ -1698,21 +1698,21 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>07:27:35</t>
+          <t>07:51:37</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>07:54</t>
+          <t>07:52</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D55" t="n">
-        <v>27</v>
+        <v>1</v>
       </c>
       <c r="E55" t="inlineStr">
         <is>
@@ -1723,12 +1723,12 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>06:59:30</t>
+          <t>07:27:35</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>07:55</t>
+          <t>07:54</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
@@ -1737,7 +1737,7 @@
         </is>
       </c>
       <c r="D56" t="n">
-        <v>56</v>
+        <v>27</v>
       </c>
       <c r="E56" t="inlineStr">
         <is>
@@ -1748,12 +1748,12 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>07:27:35</t>
+          <t>06:59:30</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>07:58</t>
+          <t>07:55</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
@@ -1762,7 +1762,7 @@
         </is>
       </c>
       <c r="D57" t="n">
-        <v>31</v>
+        <v>56</v>
       </c>
       <c r="E57" t="inlineStr">
         <is>
@@ -1773,21 +1773,21 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>07:27:35</t>
+          <t>07:51:37</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>07:59</t>
+          <t>07:58</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D58" t="n">
-        <v>32</v>
+        <v>7</v>
       </c>
       <c r="E58" t="inlineStr">
         <is>
@@ -1798,21 +1798,21 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>07:27:35</t>
+          <t>07:51:37</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>08:01</t>
+          <t>07:59</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D59" t="n">
-        <v>34</v>
+        <v>8</v>
       </c>
       <c r="E59" t="inlineStr">
         <is>
@@ -1823,21 +1823,21 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>07:27:35</t>
+          <t>07:51:37</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>08:03</t>
+          <t>08:01</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D60" t="n">
-        <v>36</v>
+        <v>10</v>
       </c>
       <c r="E60" t="inlineStr">
         <is>
@@ -1848,21 +1848,21 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>06:59:30</t>
+          <t>07:51:37</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>08:14</t>
+          <t>08:03</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D61" t="n">
-        <v>75</v>
+        <v>12</v>
       </c>
       <c r="E61" t="inlineStr">
         <is>
@@ -1873,12 +1873,12 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>07:27:35</t>
+          <t>06:59:30</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>08:19</t>
+          <t>08:14</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
@@ -1887,7 +1887,7 @@
         </is>
       </c>
       <c r="D62" t="n">
-        <v>52</v>
+        <v>75</v>
       </c>
       <c r="E62" t="inlineStr">
         <is>
@@ -1898,21 +1898,21 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>07:27:35</t>
+          <t>07:51:37</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>08:19</t>
+          <t>08:17</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D63" t="n">
-        <v>52</v>
+        <v>26</v>
       </c>
       <c r="E63" t="inlineStr">
         <is>
@@ -1923,21 +1923,21 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>07:27:35</t>
+          <t>07:51:37</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>08:29</t>
+          <t>08:19</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D64" t="n">
-        <v>62</v>
+        <v>28</v>
       </c>
       <c r="E64" t="inlineStr">
         <is>
@@ -1948,21 +1948,21 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>07:27:35</t>
+          <t>07:51:37</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>08:34</t>
+          <t>08:19</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D65" t="n">
-        <v>67</v>
+        <v>28</v>
       </c>
       <c r="E65" t="inlineStr">
         <is>
@@ -1978,16 +1978,16 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>08:48</t>
+          <t>08:19</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D66" t="n">
-        <v>81</v>
+        <v>52</v>
       </c>
       <c r="E66" t="inlineStr">
         <is>
@@ -1998,21 +1998,21 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>07:27:35</t>
+          <t>07:51:37</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>08:51</t>
+          <t>08:22</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D67" t="n">
-        <v>84</v>
+        <v>31</v>
       </c>
       <c r="E67" t="inlineStr">
         <is>
@@ -2023,21 +2023,21 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>07:27:35</t>
+          <t>07:51:37</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>08:59</t>
+          <t>08:29</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D68" t="n">
-        <v>92</v>
+        <v>38</v>
       </c>
       <c r="E68" t="inlineStr">
         <is>
@@ -2048,21 +2048,21 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>07:27:35</t>
+          <t>07:51:37</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>09:14</t>
+          <t>08:33</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D69" t="n">
-        <v>107</v>
+        <v>42</v>
       </c>
       <c r="E69" t="inlineStr">
         <is>
@@ -2078,16 +2078,16 @@
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>09:16</t>
+          <t>08:34</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D70" t="n">
-        <v>109</v>
+        <v>67</v>
       </c>
       <c r="E70" t="inlineStr">
         <is>
@@ -2098,23 +2098,323 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
+          <t>07:51:37</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>08:48</t>
+        </is>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D71" t="n">
+        <v>57</v>
+      </c>
+      <c r="E71" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
           <t>07:27:35</t>
         </is>
       </c>
-      <c r="B71" t="inlineStr">
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>08:51</t>
+        </is>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>16_P MOR-SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D72" t="n">
+        <v>84</v>
+      </c>
+      <c r="E72" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>07:51:37</t>
+        </is>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>08:59</t>
+        </is>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D73" t="n">
+        <v>68</v>
+      </c>
+      <c r="E73" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>07:51:37</t>
+        </is>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>09:03</t>
+        </is>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>17X38_ROMERO</t>
+        </is>
+      </c>
+      <c r="D74" t="n">
+        <v>72</v>
+      </c>
+      <c r="E74" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>07:51:37</t>
+        </is>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>09:10</t>
+        </is>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>16_P MOR-SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D75" t="n">
+        <v>79</v>
+      </c>
+      <c r="E75" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>07:51:37</t>
+        </is>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>09:14</t>
+        </is>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D76" t="n">
+        <v>83</v>
+      </c>
+      <c r="E76" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>07:27:35</t>
+        </is>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>09:16</t>
+        </is>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D77" t="n">
+        <v>109</v>
+      </c>
+      <c r="E77" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>07:51:37</t>
+        </is>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>09:18</t>
+        </is>
+      </c>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>215_EL PELIGRO</t>
+        </is>
+      </c>
+      <c r="D78" t="n">
+        <v>87</v>
+      </c>
+      <c r="E78" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>07:27:35</t>
+        </is>
+      </c>
+      <c r="B79" t="inlineStr">
         <is>
           <t>09:19</t>
         </is>
       </c>
-      <c r="C71" t="inlineStr">
+      <c r="C79" t="inlineStr">
         <is>
           <t>215_EL PELIGRO</t>
         </is>
       </c>
-      <c r="D71" t="n">
+      <c r="D79" t="n">
         <v>112</v>
       </c>
-      <c r="E71" t="inlineStr">
+      <c r="E79" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>07:51:37</t>
+        </is>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>09:20</t>
+        </is>
+      </c>
+      <c r="C80" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D80" t="n">
+        <v>89</v>
+      </c>
+      <c r="E80" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>07:51:37</t>
+        </is>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>09:29</t>
+        </is>
+      </c>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D81" t="n">
+        <v>98</v>
+      </c>
+      <c r="E81" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t>07:51:37</t>
+        </is>
+      </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>09:34</t>
+        </is>
+      </c>
+      <c r="C82" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D82" t="n">
+        <v>103</v>
+      </c>
+      <c r="E82" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>07:51:37</t>
+        </is>
+      </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>09:44</t>
+        </is>
+      </c>
+      <c r="C83" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D83" t="n">
+        <v>113</v>
+      </c>
+      <c r="E83" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -2131,7 +2431,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E18"/>
+  <dimension ref="A1:E21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2144,14 +2444,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 07:27:35</t>
+          <t>Última actualización: 07:51:37</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 13</t>
+          <t>Total filas: 16</t>
         </is>
       </c>
     </row>
@@ -2410,21 +2710,21 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>07:27:35</t>
+          <t>07:51:37</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>08:34</t>
+          <t>08:17</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D15" t="n">
-        <v>67</v>
+        <v>26</v>
       </c>
       <c r="E15" t="inlineStr">
         <is>
@@ -2435,21 +2735,21 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>07:27:35</t>
+          <t>07:51:37</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>08:48</t>
+          <t>08:33</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D16" t="n">
-        <v>81</v>
+        <v>42</v>
       </c>
       <c r="E16" t="inlineStr">
         <is>
@@ -2465,16 +2765,16 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>08:59</t>
+          <t>08:34</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D17" t="n">
-        <v>92</v>
+        <v>67</v>
       </c>
       <c r="E17" t="inlineStr">
         <is>
@@ -2485,23 +2785,98 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
+          <t>07:51:37</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>08:48</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D18" t="n">
+        <v>57</v>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>07:51:37</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>08:59</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D19" t="n">
+        <v>68</v>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>07:51:37</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>09:18</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>215_EL PELIGRO</t>
+        </is>
+      </c>
+      <c r="D20" t="n">
+        <v>87</v>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
           <t>07:27:35</t>
         </is>
       </c>
-      <c r="B18" t="inlineStr">
+      <c r="B21" t="inlineStr">
         <is>
           <t>09:19</t>
         </is>
       </c>
-      <c r="C18" t="inlineStr">
+      <c r="C21" t="inlineStr">
         <is>
           <t>215_EL PELIGRO</t>
         </is>
       </c>
-      <c r="D18" t="n">
+      <c r="D21" t="n">
         <v>112</v>
       </c>
-      <c r="E18" t="inlineStr">
+      <c r="E21" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -2518,7 +2893,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E15"/>
+  <dimension ref="A1:E17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2531,14 +2906,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 07:27:35</t>
+          <t>Última actualización: 07:51:37</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 10</t>
+          <t>Total filas: 12</t>
         </is>
       </c>
     </row>
@@ -2797,23 +3172,73 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
+          <t>07:51:37</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>08:25</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D15" t="n">
+        <v>34</v>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>07:51:37</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>08:30</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>215A_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D16" t="n">
+        <v>39</v>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
           <t>07:27:35</t>
         </is>
       </c>
-      <c r="B15" t="inlineStr">
+      <c r="B17" t="inlineStr">
         <is>
           <t>08:33</t>
         </is>
       </c>
-      <c r="C15" t="inlineStr">
+      <c r="C17" t="inlineStr">
         <is>
           <t>215A_LA PLATA</t>
         </is>
       </c>
-      <c r="D15" t="n">
+      <c r="D17" t="n">
         <v>66</v>
       </c>
-      <c r="E15" t="inlineStr">
+      <c r="E17" t="inlineStr">
         <is>
           <t>L6173</t>
         </is>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 1797
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-03-21.xlsx
+++ b/data/horarios-141-2026-03-21.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E83"/>
+  <dimension ref="A1:E99"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 07:51:37</t>
+          <t>Última actualización: 08:14:14</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 78</t>
+          <t>Total filas: 94</t>
         </is>
       </c>
     </row>
@@ -533,7 +533,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D8" t="n">
@@ -558,7 +558,7 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D9" t="n">
@@ -758,7 +758,7 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D17" t="n">
@@ -783,7 +783,7 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D18" t="n">
@@ -1558,7 +1558,7 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D49" t="n">
@@ -1583,7 +1583,7 @@
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D50" t="n">
@@ -1898,21 +1898,21 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>07:51:37</t>
+          <t>08:14:14</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>08:17</t>
+          <t>08:14</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D63" t="n">
-        <v>26</v>
+        <v>0</v>
       </c>
       <c r="E63" t="inlineStr">
         <is>
@@ -1923,21 +1923,21 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>07:51:37</t>
+          <t>08:14:14</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>08:19</t>
+          <t>08:14</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D64" t="n">
-        <v>28</v>
+        <v>0</v>
       </c>
       <c r="E64" t="inlineStr">
         <is>
@@ -1953,16 +1953,16 @@
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>08:19</t>
+          <t>08:17</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D65" t="n">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="E65" t="inlineStr">
         <is>
@@ -1973,7 +1973,7 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>07:27:35</t>
+          <t>07:51:37</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
@@ -1983,11 +1983,11 @@
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D66" t="n">
-        <v>52</v>
+        <v>28</v>
       </c>
       <c r="E66" t="inlineStr">
         <is>
@@ -2003,16 +2003,16 @@
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>08:22</t>
+          <t>08:19</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D67" t="n">
-        <v>31</v>
+        <v>28</v>
       </c>
       <c r="E67" t="inlineStr">
         <is>
@@ -2023,21 +2023,21 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>07:51:37</t>
+          <t>07:27:35</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>08:29</t>
+          <t>08:19</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D68" t="n">
-        <v>38</v>
+        <v>52</v>
       </c>
       <c r="E68" t="inlineStr">
         <is>
@@ -2048,21 +2048,21 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>07:51:37</t>
+          <t>08:14:14</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>08:33</t>
+          <t>08:20</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D69" t="n">
-        <v>42</v>
+        <v>6</v>
       </c>
       <c r="E69" t="inlineStr">
         <is>
@@ -2073,21 +2073,21 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>07:27:35</t>
+          <t>08:14:14</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>08:34</t>
+          <t>08:21</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D70" t="n">
-        <v>67</v>
+        <v>7</v>
       </c>
       <c r="E70" t="inlineStr">
         <is>
@@ -2098,21 +2098,21 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>07:51:37</t>
+          <t>08:14:14</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>08:48</t>
+          <t>08:22</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D71" t="n">
-        <v>57</v>
+        <v>8</v>
       </c>
       <c r="E71" t="inlineStr">
         <is>
@@ -2123,21 +2123,21 @@
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>07:27:35</t>
+          <t>07:51:37</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>08:51</t>
+          <t>08:29</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D72" t="n">
-        <v>84</v>
+        <v>38</v>
       </c>
       <c r="E72" t="inlineStr">
         <is>
@@ -2148,21 +2148,21 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>07:51:37</t>
+          <t>08:14:14</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>08:59</t>
+          <t>08:30</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D73" t="n">
-        <v>68</v>
+        <v>16</v>
       </c>
       <c r="E73" t="inlineStr">
         <is>
@@ -2178,16 +2178,16 @@
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>09:03</t>
+          <t>08:33</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D74" t="n">
-        <v>72</v>
+        <v>42</v>
       </c>
       <c r="E74" t="inlineStr">
         <is>
@@ -2198,21 +2198,21 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>07:51:37</t>
+          <t>08:14:14</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>09:10</t>
+          <t>08:34</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D75" t="n">
-        <v>79</v>
+        <v>20</v>
       </c>
       <c r="E75" t="inlineStr">
         <is>
@@ -2223,21 +2223,21 @@
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>07:51:37</t>
+          <t>08:14:14</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>09:14</t>
+          <t>08:42</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D76" t="n">
-        <v>83</v>
+        <v>28</v>
       </c>
       <c r="E76" t="inlineStr">
         <is>
@@ -2248,21 +2248,21 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>07:27:35</t>
+          <t>08:14:14</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>09:16</t>
+          <t>08:44</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D77" t="n">
-        <v>109</v>
+        <v>30</v>
       </c>
       <c r="E77" t="inlineStr">
         <is>
@@ -2273,21 +2273,21 @@
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>07:51:37</t>
+          <t>08:14:14</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>09:18</t>
+          <t>08:48</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>215_EL PELIGRO</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D78" t="n">
-        <v>87</v>
+        <v>34</v>
       </c>
       <c r="E78" t="inlineStr">
         <is>
@@ -2303,16 +2303,16 @@
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>09:19</t>
+          <t>08:51</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>215_EL PELIGRO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D79" t="n">
-        <v>112</v>
+        <v>84</v>
       </c>
       <c r="E79" t="inlineStr">
         <is>
@@ -2328,16 +2328,16 @@
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>09:20</t>
+          <t>08:59</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D80" t="n">
-        <v>89</v>
+        <v>68</v>
       </c>
       <c r="E80" t="inlineStr">
         <is>
@@ -2348,21 +2348,21 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>07:51:37</t>
+          <t>08:14:14</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>09:29</t>
+          <t>09:00</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D81" t="n">
-        <v>98</v>
+        <v>46</v>
       </c>
       <c r="E81" t="inlineStr">
         <is>
@@ -2373,21 +2373,21 @@
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>07:51:37</t>
+          <t>08:14:14</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>09:34</t>
+          <t>09:03</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D82" t="n">
-        <v>103</v>
+        <v>49</v>
       </c>
       <c r="E82" t="inlineStr">
         <is>
@@ -2403,18 +2403,418 @@
       </c>
       <c r="B83" t="inlineStr">
         <is>
+          <t>09:10</t>
+        </is>
+      </c>
+      <c r="C83" t="inlineStr">
+        <is>
+          <t>16_P MOR-SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D83" t="n">
+        <v>79</v>
+      </c>
+      <c r="E83" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="inlineStr">
+        <is>
+          <t>07:51:37</t>
+        </is>
+      </c>
+      <c r="B84" t="inlineStr">
+        <is>
+          <t>09:14</t>
+        </is>
+      </c>
+      <c r="C84" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D84" t="n">
+        <v>83</v>
+      </c>
+      <c r="E84" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="inlineStr">
+        <is>
+          <t>08:14:14</t>
+        </is>
+      </c>
+      <c r="B85" t="inlineStr">
+        <is>
+          <t>09:15</t>
+        </is>
+      </c>
+      <c r="C85" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D85" t="n">
+        <v>61</v>
+      </c>
+      <c r="E85" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="inlineStr">
+        <is>
+          <t>07:27:35</t>
+        </is>
+      </c>
+      <c r="B86" t="inlineStr">
+        <is>
+          <t>09:16</t>
+        </is>
+      </c>
+      <c r="C86" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D86" t="n">
+        <v>109</v>
+      </c>
+      <c r="E86" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t>08:14:14</t>
+        </is>
+      </c>
+      <c r="B87" t="inlineStr">
+        <is>
+          <t>09:18</t>
+        </is>
+      </c>
+      <c r="C87" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D87" t="n">
+        <v>64</v>
+      </c>
+      <c r="E87" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="inlineStr">
+        <is>
+          <t>07:51:37</t>
+        </is>
+      </c>
+      <c r="B88" t="inlineStr">
+        <is>
+          <t>09:18</t>
+        </is>
+      </c>
+      <c r="C88" t="inlineStr">
+        <is>
+          <t>215_EL PELIGRO</t>
+        </is>
+      </c>
+      <c r="D88" t="n">
+        <v>87</v>
+      </c>
+      <c r="E88" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="inlineStr">
+        <is>
+          <t>08:14:14</t>
+        </is>
+      </c>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>09:19</t>
+        </is>
+      </c>
+      <c r="C89" t="inlineStr">
+        <is>
+          <t>215_EL PELIGRO</t>
+        </is>
+      </c>
+      <c r="D89" t="n">
+        <v>65</v>
+      </c>
+      <c r="E89" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="inlineStr">
+        <is>
+          <t>07:51:37</t>
+        </is>
+      </c>
+      <c r="B90" t="inlineStr">
+        <is>
+          <t>09:20</t>
+        </is>
+      </c>
+      <c r="C90" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D90" t="n">
+        <v>89</v>
+      </c>
+      <c r="E90" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="inlineStr">
+        <is>
+          <t>07:51:37</t>
+        </is>
+      </c>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t>09:29</t>
+        </is>
+      </c>
+      <c r="C91" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D91" t="n">
+        <v>98</v>
+      </c>
+      <c r="E91" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="inlineStr">
+        <is>
+          <t>08:14:14</t>
+        </is>
+      </c>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t>09:33</t>
+        </is>
+      </c>
+      <c r="C92" t="inlineStr">
+        <is>
+          <t>16_P MOR-SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D92" t="n">
+        <v>79</v>
+      </c>
+      <c r="E92" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="inlineStr">
+        <is>
+          <t>08:14:14</t>
+        </is>
+      </c>
+      <c r="B93" t="inlineStr">
+        <is>
+          <t>09:33</t>
+        </is>
+      </c>
+      <c r="C93" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D93" t="n">
+        <v>79</v>
+      </c>
+      <c r="E93" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="inlineStr">
+        <is>
+          <t>08:14:14</t>
+        </is>
+      </c>
+      <c r="B94" t="inlineStr">
+        <is>
+          <t>09:34</t>
+        </is>
+      </c>
+      <c r="C94" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D94" t="n">
+        <v>80</v>
+      </c>
+      <c r="E94" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="inlineStr">
+        <is>
+          <t>07:51:37</t>
+        </is>
+      </c>
+      <c r="B95" t="inlineStr">
+        <is>
           <t>09:44</t>
         </is>
       </c>
-      <c r="C83" t="inlineStr">
+      <c r="C95" t="inlineStr">
         <is>
           <t>14_ABASTO</t>
         </is>
       </c>
-      <c r="D83" t="n">
+      <c r="D95" t="n">
         <v>113</v>
       </c>
-      <c r="E83" t="inlineStr">
+      <c r="E95" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="inlineStr">
+        <is>
+          <t>08:14:14</t>
+        </is>
+      </c>
+      <c r="B96" t="inlineStr">
+        <is>
+          <t>09:45</t>
+        </is>
+      </c>
+      <c r="C96" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D96" t="n">
+        <v>91</v>
+      </c>
+      <c r="E96" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="inlineStr">
+        <is>
+          <t>08:14:14</t>
+        </is>
+      </c>
+      <c r="B97" t="inlineStr">
+        <is>
+          <t>09:51</t>
+        </is>
+      </c>
+      <c r="C97" t="inlineStr">
+        <is>
+          <t>16_P MOR-SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D97" t="n">
+        <v>97</v>
+      </c>
+      <c r="E97" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="inlineStr">
+        <is>
+          <t>08:14:14</t>
+        </is>
+      </c>
+      <c r="B98" t="inlineStr">
+        <is>
+          <t>09:56</t>
+        </is>
+      </c>
+      <c r="C98" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D98" t="n">
+        <v>102</v>
+      </c>
+      <c r="E98" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="inlineStr">
+        <is>
+          <t>08:14:14</t>
+        </is>
+      </c>
+      <c r="B99" t="inlineStr">
+        <is>
+          <t>10:04</t>
+        </is>
+      </c>
+      <c r="C99" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D99" t="n">
+        <v>110</v>
+      </c>
+      <c r="E99" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -2431,7 +2831,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E21"/>
+  <dimension ref="A1:E23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2444,14 +2844,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 07:51:37</t>
+          <t>Última actualización: 08:14:14</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 16</t>
+          <t>Total filas: 18</t>
         </is>
       </c>
     </row>
@@ -2760,7 +3160,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>07:27:35</t>
+          <t>08:14:14</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -2774,7 +3174,7 @@
         </is>
       </c>
       <c r="D17" t="n">
-        <v>67</v>
+        <v>20</v>
       </c>
       <c r="E17" t="inlineStr">
         <is>
@@ -2785,7 +3185,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>07:51:37</t>
+          <t>08:14:14</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -2799,7 +3199,7 @@
         </is>
       </c>
       <c r="D18" t="n">
-        <v>57</v>
+        <v>34</v>
       </c>
       <c r="E18" t="inlineStr">
         <is>
@@ -2835,21 +3235,21 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>07:51:37</t>
+          <t>08:14:14</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>09:18</t>
+          <t>09:00</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>215_EL PELIGRO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D20" t="n">
-        <v>87</v>
+        <v>46</v>
       </c>
       <c r="E20" t="inlineStr">
         <is>
@@ -2860,23 +3260,73 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>07:27:35</t>
+          <t>07:51:37</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
+          <t>09:18</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>215_EL PELIGRO</t>
+        </is>
+      </c>
+      <c r="D21" t="n">
+        <v>87</v>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>08:14:14</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
           <t>09:19</t>
         </is>
       </c>
-      <c r="C21" t="inlineStr">
+      <c r="C22" t="inlineStr">
         <is>
           <t>215_EL PELIGRO</t>
         </is>
       </c>
-      <c r="D21" t="n">
-        <v>112</v>
-      </c>
-      <c r="E21" t="inlineStr">
+      <c r="D22" t="n">
+        <v>65</v>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>08:14:14</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>10:04</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D23" t="n">
+        <v>110</v>
+      </c>
+      <c r="E23" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -2893,7 +3343,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E17"/>
+  <dimension ref="A1:E21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2906,14 +3356,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 07:51:37</t>
+          <t>Última actualización: 08:14:14</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 12</t>
+          <t>Total filas: 16</t>
         </is>
       </c>
     </row>
@@ -3197,50 +3647,150 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>07:51:37</t>
+          <t>08:14:14</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>08:30</t>
+          <t>08:28</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>215A_LA PLATA</t>
+          <t>215C_LA PLATA</t>
         </is>
       </c>
       <c r="D16" t="n">
-        <v>39</v>
+        <v>14</v>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>L6173</t>
+          <t>L6203</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
+          <t>07:51:37</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>08:30</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>215A_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D17" t="n">
+        <v>39</v>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>08:14:14</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>08:32</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>215A_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D18" t="n">
+        <v>18</v>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
           <t>07:27:35</t>
         </is>
       </c>
-      <c r="B17" t="inlineStr">
+      <c r="B19" t="inlineStr">
         <is>
           <t>08:33</t>
         </is>
       </c>
-      <c r="C17" t="inlineStr">
+      <c r="C19" t="inlineStr">
         <is>
           <t>215A_LA PLATA</t>
         </is>
       </c>
-      <c r="D17" t="n">
+      <c r="D19" t="n">
         <v>66</v>
       </c>
-      <c r="E17" t="inlineStr">
+      <c r="E19" t="inlineStr">
         <is>
           <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>08:14:14</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>08:52</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>215A_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D20" t="n">
+        <v>38</v>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>08:14:14</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>09:56</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D21" t="n">
+        <v>102</v>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>L6203</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 1798
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-03-21.xlsx
+++ b/data/horarios-141-2026-03-21.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E99"/>
+  <dimension ref="A1:E112"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 08:14:14</t>
+          <t>Última actualización: 08:36:09</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 94</t>
+          <t>Total filas: 107</t>
         </is>
       </c>
     </row>
@@ -1558,7 +1558,7 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D49" t="n">
@@ -1583,7 +1583,7 @@
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D50" t="n">
@@ -1873,7 +1873,7 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>06:59:30</t>
+          <t>08:14:14</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
@@ -1883,11 +1883,11 @@
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D62" t="n">
-        <v>75</v>
+        <v>0</v>
       </c>
       <c r="E62" t="inlineStr">
         <is>
@@ -1908,7 +1908,7 @@
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D63" t="n">
@@ -1923,7 +1923,7 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>08:14:14</t>
+          <t>06:59:30</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
@@ -1933,11 +1933,11 @@
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D64" t="n">
-        <v>0</v>
+        <v>75</v>
       </c>
       <c r="E64" t="inlineStr">
         <is>
@@ -1973,7 +1973,7 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>07:51:37</t>
+          <t>07:27:35</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
@@ -1983,11 +1983,11 @@
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D66" t="n">
-        <v>28</v>
+        <v>52</v>
       </c>
       <c r="E66" t="inlineStr">
         <is>
@@ -2008,7 +2008,7 @@
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D67" t="n">
@@ -2023,7 +2023,7 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>07:27:35</t>
+          <t>07:51:37</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
@@ -2033,11 +2033,11 @@
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D68" t="n">
-        <v>52</v>
+        <v>28</v>
       </c>
       <c r="E68" t="inlineStr">
         <is>
@@ -2223,21 +2223,21 @@
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>08:14:14</t>
+          <t>08:36:09</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>08:42</t>
+          <t>08:36</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D76" t="n">
-        <v>28</v>
+        <v>0</v>
       </c>
       <c r="E76" t="inlineStr">
         <is>
@@ -2248,21 +2248,21 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>08:14:14</t>
+          <t>08:36:09</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>08:44</t>
+          <t>08:36</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D77" t="n">
-        <v>30</v>
+        <v>0</v>
       </c>
       <c r="E77" t="inlineStr">
         <is>
@@ -2273,21 +2273,21 @@
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>08:14:14</t>
+          <t>08:36:09</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>08:48</t>
+          <t>08:37</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D78" t="n">
-        <v>34</v>
+        <v>1</v>
       </c>
       <c r="E78" t="inlineStr">
         <is>
@@ -2298,21 +2298,21 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>07:27:35</t>
+          <t>08:14:14</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>08:51</t>
+          <t>08:42</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D79" t="n">
-        <v>84</v>
+        <v>28</v>
       </c>
       <c r="E79" t="inlineStr">
         <is>
@@ -2323,21 +2323,21 @@
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>07:51:37</t>
+          <t>08:36:09</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>08:59</t>
+          <t>08:44</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D80" t="n">
-        <v>68</v>
+        <v>8</v>
       </c>
       <c r="E80" t="inlineStr">
         <is>
@@ -2348,21 +2348,21 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>08:14:14</t>
+          <t>08:36:09</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>09:00</t>
+          <t>08:48</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D81" t="n">
-        <v>46</v>
+        <v>12</v>
       </c>
       <c r="E81" t="inlineStr">
         <is>
@@ -2373,21 +2373,21 @@
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>08:14:14</t>
+          <t>07:27:35</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>09:03</t>
+          <t>08:51</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D82" t="n">
-        <v>49</v>
+        <v>84</v>
       </c>
       <c r="E82" t="inlineStr">
         <is>
@@ -2403,16 +2403,16 @@
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>09:10</t>
+          <t>08:59</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D83" t="n">
-        <v>79</v>
+        <v>68</v>
       </c>
       <c r="E83" t="inlineStr">
         <is>
@@ -2423,21 +2423,21 @@
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>07:51:37</t>
+          <t>08:36:09</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>09:14</t>
+          <t>09:00</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D84" t="n">
-        <v>83</v>
+        <v>24</v>
       </c>
       <c r="E84" t="inlineStr">
         <is>
@@ -2448,21 +2448,21 @@
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>08:14:14</t>
+          <t>08:36:09</t>
         </is>
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>09:15</t>
+          <t>09:01</t>
         </is>
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D85" t="n">
-        <v>61</v>
+        <v>25</v>
       </c>
       <c r="E85" t="inlineStr">
         <is>
@@ -2473,21 +2473,21 @@
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>07:27:35</t>
+          <t>08:36:09</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>09:16</t>
+          <t>09:03</t>
         </is>
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D86" t="n">
-        <v>109</v>
+        <v>27</v>
       </c>
       <c r="E86" t="inlineStr">
         <is>
@@ -2498,21 +2498,21 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>08:14:14</t>
+          <t>08:36:09</t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>09:18</t>
+          <t>09:04</t>
         </is>
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D87" t="n">
-        <v>64</v>
+        <v>28</v>
       </c>
       <c r="E87" t="inlineStr">
         <is>
@@ -2528,16 +2528,16 @@
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>09:18</t>
+          <t>09:10</t>
         </is>
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>215_EL PELIGRO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D88" t="n">
-        <v>87</v>
+        <v>79</v>
       </c>
       <c r="E88" t="inlineStr">
         <is>
@@ -2548,21 +2548,21 @@
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>08:14:14</t>
+          <t>07:51:37</t>
         </is>
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>09:19</t>
+          <t>09:14</t>
         </is>
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>215_EL PELIGRO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D89" t="n">
-        <v>65</v>
+        <v>83</v>
       </c>
       <c r="E89" t="inlineStr">
         <is>
@@ -2573,21 +2573,21 @@
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>07:51:37</t>
+          <t>08:36:09</t>
         </is>
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>09:20</t>
+          <t>09:15</t>
         </is>
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D90" t="n">
-        <v>89</v>
+        <v>39</v>
       </c>
       <c r="E90" t="inlineStr">
         <is>
@@ -2598,21 +2598,21 @@
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>07:51:37</t>
+          <t>07:27:35</t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>09:29</t>
+          <t>09:16</t>
         </is>
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D91" t="n">
-        <v>98</v>
+        <v>109</v>
       </c>
       <c r="E91" t="inlineStr">
         <is>
@@ -2623,21 +2623,21 @@
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>08:14:14</t>
+          <t>08:36:09</t>
         </is>
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>09:33</t>
+          <t>09:17</t>
         </is>
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D92" t="n">
-        <v>79</v>
+        <v>41</v>
       </c>
       <c r="E92" t="inlineStr">
         <is>
@@ -2653,16 +2653,16 @@
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>09:33</t>
+          <t>09:18</t>
         </is>
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D93" t="n">
-        <v>79</v>
+        <v>64</v>
       </c>
       <c r="E93" t="inlineStr">
         <is>
@@ -2673,21 +2673,21 @@
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>08:14:14</t>
+          <t>07:51:37</t>
         </is>
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>09:34</t>
+          <t>09:18</t>
         </is>
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>215_EL PELIGRO</t>
         </is>
       </c>
       <c r="D94" t="n">
-        <v>80</v>
+        <v>87</v>
       </c>
       <c r="E94" t="inlineStr">
         <is>
@@ -2698,21 +2698,21 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>07:51:37</t>
+          <t>08:36:09</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>09:44</t>
+          <t>09:19</t>
         </is>
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>215_EL PELIGRO</t>
         </is>
       </c>
       <c r="D95" t="n">
-        <v>113</v>
+        <v>43</v>
       </c>
       <c r="E95" t="inlineStr">
         <is>
@@ -2723,21 +2723,21 @@
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>08:14:14</t>
+          <t>07:51:37</t>
         </is>
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>09:45</t>
+          <t>09:20</t>
         </is>
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D96" t="n">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="E96" t="inlineStr">
         <is>
@@ -2748,21 +2748,21 @@
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>08:14:14</t>
+          <t>07:51:37</t>
         </is>
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>09:51</t>
+          <t>09:29</t>
         </is>
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D97" t="n">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="E97" t="inlineStr">
         <is>
@@ -2773,21 +2773,21 @@
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>08:14:14</t>
+          <t>08:36:09</t>
         </is>
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>09:56</t>
+          <t>09:29</t>
         </is>
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D98" t="n">
-        <v>102</v>
+        <v>53</v>
       </c>
       <c r="E98" t="inlineStr">
         <is>
@@ -2803,18 +2803,343 @@
       </c>
       <c r="B99" t="inlineStr">
         <is>
+          <t>09:33</t>
+        </is>
+      </c>
+      <c r="C99" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D99" t="n">
+        <v>79</v>
+      </c>
+      <c r="E99" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="inlineStr">
+        <is>
+          <t>08:14:14</t>
+        </is>
+      </c>
+      <c r="B100" t="inlineStr">
+        <is>
+          <t>09:33</t>
+        </is>
+      </c>
+      <c r="C100" t="inlineStr">
+        <is>
+          <t>16_P MOR-SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D100" t="n">
+        <v>79</v>
+      </c>
+      <c r="E100" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="inlineStr">
+        <is>
+          <t>08:36:09</t>
+        </is>
+      </c>
+      <c r="B101" t="inlineStr">
+        <is>
+          <t>09:34</t>
+        </is>
+      </c>
+      <c r="C101" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D101" t="n">
+        <v>58</v>
+      </c>
+      <c r="E101" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" t="inlineStr">
+        <is>
+          <t>07:51:37</t>
+        </is>
+      </c>
+      <c r="B102" t="inlineStr">
+        <is>
+          <t>09:44</t>
+        </is>
+      </c>
+      <c r="C102" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D102" t="n">
+        <v>113</v>
+      </c>
+      <c r="E102" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="inlineStr">
+        <is>
+          <t>08:36:09</t>
+        </is>
+      </c>
+      <c r="B103" t="inlineStr">
+        <is>
+          <t>09:45</t>
+        </is>
+      </c>
+      <c r="C103" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D103" t="n">
+        <v>69</v>
+      </c>
+      <c r="E103" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" t="inlineStr">
+        <is>
+          <t>08:36:09</t>
+        </is>
+      </c>
+      <c r="B104" t="inlineStr">
+        <is>
+          <t>09:51</t>
+        </is>
+      </c>
+      <c r="C104" t="inlineStr">
+        <is>
+          <t>16_P MOR-SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D104" t="n">
+        <v>75</v>
+      </c>
+      <c r="E104" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" t="inlineStr">
+        <is>
+          <t>08:36:09</t>
+        </is>
+      </c>
+      <c r="B105" t="inlineStr">
+        <is>
+          <t>09:54</t>
+        </is>
+      </c>
+      <c r="C105" t="inlineStr">
+        <is>
+          <t>16_P MOR-SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D105" t="n">
+        <v>78</v>
+      </c>
+      <c r="E105" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" t="inlineStr">
+        <is>
+          <t>08:36:09</t>
+        </is>
+      </c>
+      <c r="B106" t="inlineStr">
+        <is>
+          <t>09:56</t>
+        </is>
+      </c>
+      <c r="C106" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D106" t="n">
+        <v>80</v>
+      </c>
+      <c r="E106" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" t="inlineStr">
+        <is>
+          <t>08:36:09</t>
+        </is>
+      </c>
+      <c r="B107" t="inlineStr">
+        <is>
           <t>10:04</t>
         </is>
       </c>
-      <c r="C99" t="inlineStr">
+      <c r="C107" t="inlineStr">
         <is>
           <t>215C_EL PATO</t>
         </is>
       </c>
-      <c r="D99" t="n">
-        <v>110</v>
-      </c>
-      <c r="E99" t="inlineStr">
+      <c r="D107" t="n">
+        <v>88</v>
+      </c>
+      <c r="E107" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" t="inlineStr">
+        <is>
+          <t>08:36:09</t>
+        </is>
+      </c>
+      <c r="B108" t="inlineStr">
+        <is>
+          <t>10:09</t>
+        </is>
+      </c>
+      <c r="C108" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D108" t="n">
+        <v>93</v>
+      </c>
+      <c r="E108" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" t="inlineStr">
+        <is>
+          <t>08:36:09</t>
+        </is>
+      </c>
+      <c r="B109" t="inlineStr">
+        <is>
+          <t>10:19</t>
+        </is>
+      </c>
+      <c r="C109" t="inlineStr">
+        <is>
+          <t>17_ROMERO</t>
+        </is>
+      </c>
+      <c r="D109" t="n">
+        <v>103</v>
+      </c>
+      <c r="E109" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" t="inlineStr">
+        <is>
+          <t>08:36:09</t>
+        </is>
+      </c>
+      <c r="B110" t="inlineStr">
+        <is>
+          <t>10:20</t>
+        </is>
+      </c>
+      <c r="C110" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D110" t="n">
+        <v>104</v>
+      </c>
+      <c r="E110" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" t="inlineStr">
+        <is>
+          <t>08:36:09</t>
+        </is>
+      </c>
+      <c r="B111" t="inlineStr">
+        <is>
+          <t>10:33</t>
+        </is>
+      </c>
+      <c r="C111" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D111" t="n">
+        <v>117</v>
+      </c>
+      <c r="E111" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" t="inlineStr">
+        <is>
+          <t>08:36:09</t>
+        </is>
+      </c>
+      <c r="B112" t="inlineStr">
+        <is>
+          <t>10:34</t>
+        </is>
+      </c>
+      <c r="C112" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D112" t="n">
+        <v>118</v>
+      </c>
+      <c r="E112" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -2831,7 +3156,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E23"/>
+  <dimension ref="A1:E24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2844,14 +3169,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 08:14:14</t>
+          <t>Última actualización: 08:36:09</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 18</t>
+          <t>Total filas: 19</t>
         </is>
       </c>
     </row>
@@ -3185,21 +3510,21 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>08:14:14</t>
+          <t>08:36:09</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>08:48</t>
+          <t>08:36</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D18" t="n">
-        <v>34</v>
+        <v>0</v>
       </c>
       <c r="E18" t="inlineStr">
         <is>
@@ -3210,21 +3535,21 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>07:51:37</t>
+          <t>08:36:09</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>08:59</t>
+          <t>08:48</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D19" t="n">
-        <v>68</v>
+        <v>12</v>
       </c>
       <c r="E19" t="inlineStr">
         <is>
@@ -3235,12 +3560,12 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>08:14:14</t>
+          <t>07:51:37</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>09:00</t>
+          <t>08:59</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -3249,7 +3574,7 @@
         </is>
       </c>
       <c r="D20" t="n">
-        <v>46</v>
+        <v>68</v>
       </c>
       <c r="E20" t="inlineStr">
         <is>
@@ -3260,21 +3585,21 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>07:51:37</t>
+          <t>08:36:09</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>09:18</t>
+          <t>09:00</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>215_EL PELIGRO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D21" t="n">
-        <v>87</v>
+        <v>24</v>
       </c>
       <c r="E21" t="inlineStr">
         <is>
@@ -3285,12 +3610,12 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>08:14:14</t>
+          <t>07:51:37</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>09:19</t>
+          <t>09:18</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
@@ -3299,7 +3624,7 @@
         </is>
       </c>
       <c r="D22" t="n">
-        <v>65</v>
+        <v>87</v>
       </c>
       <c r="E22" t="inlineStr">
         <is>
@@ -3310,23 +3635,48 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>08:14:14</t>
+          <t>08:36:09</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
+          <t>09:19</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>215_EL PELIGRO</t>
+        </is>
+      </c>
+      <c r="D23" t="n">
+        <v>43</v>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>08:36:09</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
           <t>10:04</t>
         </is>
       </c>
-      <c r="C23" t="inlineStr">
+      <c r="C24" t="inlineStr">
         <is>
           <t>215C_EL PATO</t>
         </is>
       </c>
-      <c r="D23" t="n">
-        <v>110</v>
-      </c>
-      <c r="E23" t="inlineStr">
+      <c r="D24" t="n">
+        <v>88</v>
+      </c>
+      <c r="E24" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -3343,7 +3693,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E21"/>
+  <dimension ref="A1:E24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3356,14 +3706,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 08:14:14</t>
+          <t>Última actualización: 08:36:09</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 16</t>
+          <t>Total filas: 19</t>
         </is>
       </c>
     </row>
@@ -3747,7 +4097,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>08:14:14</t>
+          <t>08:36:09</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -3761,7 +4111,7 @@
         </is>
       </c>
       <c r="D20" t="n">
-        <v>38</v>
+        <v>16</v>
       </c>
       <c r="E20" t="inlineStr">
         <is>
@@ -3791,6 +4141,81 @@
       <c r="E21" t="inlineStr">
         <is>
           <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>08:36:09</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>09:59</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D22" t="n">
+        <v>83</v>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>08:36:09</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>10:11</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>215A_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D23" t="n">
+        <v>95</v>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>08:36:09</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>10:22</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>215B_LP-P MOR-1 Y 57</t>
+        </is>
+      </c>
+      <c r="D24" t="n">
+        <v>106</v>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>L6173</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 1799
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-03-21.xlsx
+++ b/data/horarios-141-2026-03-21.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E112"/>
+  <dimension ref="A1:E122"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 08:36:09</t>
+          <t>Última actualización: 08:50:55</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 107</t>
+          <t>Total filas: 117</t>
         </is>
       </c>
     </row>
@@ -533,7 +533,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D8" t="n">
@@ -558,7 +558,7 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D9" t="n">
@@ -758,7 +758,7 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D17" t="n">
@@ -783,7 +783,7 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D18" t="n">
@@ -1158,7 +1158,7 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D33" t="n">
@@ -1183,7 +1183,7 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D34" t="n">
@@ -1898,7 +1898,7 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>08:14:14</t>
+          <t>06:59:30</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
@@ -1908,11 +1908,11 @@
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D63" t="n">
-        <v>0</v>
+        <v>75</v>
       </c>
       <c r="E63" t="inlineStr">
         <is>
@@ -1923,7 +1923,7 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>06:59:30</t>
+          <t>08:14:14</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
@@ -1933,11 +1933,11 @@
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D64" t="n">
-        <v>75</v>
+        <v>0</v>
       </c>
       <c r="E64" t="inlineStr">
         <is>
@@ -1973,7 +1973,7 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>07:27:35</t>
+          <t>07:51:37</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
@@ -1983,11 +1983,11 @@
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D66" t="n">
-        <v>52</v>
+        <v>28</v>
       </c>
       <c r="E66" t="inlineStr">
         <is>
@@ -2023,7 +2023,7 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>07:51:37</t>
+          <t>07:27:35</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
@@ -2033,11 +2033,11 @@
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D68" t="n">
-        <v>28</v>
+        <v>52</v>
       </c>
       <c r="E68" t="inlineStr">
         <is>
@@ -2373,7 +2373,7 @@
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>07:27:35</t>
+          <t>08:50:55</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
@@ -2383,11 +2383,11 @@
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D82" t="n">
-        <v>84</v>
+        <v>1</v>
       </c>
       <c r="E82" t="inlineStr">
         <is>
@@ -2398,21 +2398,21 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>07:51:37</t>
+          <t>08:50:55</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>08:59</t>
+          <t>08:51</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D83" t="n">
-        <v>68</v>
+        <v>1</v>
       </c>
       <c r="E83" t="inlineStr">
         <is>
@@ -2423,21 +2423,21 @@
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>08:36:09</t>
+          <t>07:27:35</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>09:00</t>
+          <t>08:51</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D84" t="n">
-        <v>24</v>
+        <v>84</v>
       </c>
       <c r="E84" t="inlineStr">
         <is>
@@ -2448,21 +2448,21 @@
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>08:36:09</t>
+          <t>08:50:55</t>
         </is>
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>09:01</t>
+          <t>08:59</t>
         </is>
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D85" t="n">
-        <v>25</v>
+        <v>9</v>
       </c>
       <c r="E85" t="inlineStr">
         <is>
@@ -2478,16 +2478,16 @@
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>09:03</t>
+          <t>09:00</t>
         </is>
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D86" t="n">
-        <v>27</v>
+        <v>24</v>
       </c>
       <c r="E86" t="inlineStr">
         <is>
@@ -2498,21 +2498,21 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>08:36:09</t>
+          <t>08:50:55</t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>09:04</t>
+          <t>09:01</t>
         </is>
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D87" t="n">
-        <v>28</v>
+        <v>11</v>
       </c>
       <c r="E87" t="inlineStr">
         <is>
@@ -2523,21 +2523,21 @@
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>07:51:37</t>
+          <t>08:50:55</t>
         </is>
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>09:10</t>
+          <t>09:03</t>
         </is>
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D88" t="n">
-        <v>79</v>
+        <v>13</v>
       </c>
       <c r="E88" t="inlineStr">
         <is>
@@ -2548,21 +2548,21 @@
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>07:51:37</t>
+          <t>08:36:09</t>
         </is>
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>09:14</t>
+          <t>09:04</t>
         </is>
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D89" t="n">
-        <v>83</v>
+        <v>28</v>
       </c>
       <c r="E89" t="inlineStr">
         <is>
@@ -2573,21 +2573,21 @@
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>08:36:09</t>
+          <t>07:51:37</t>
         </is>
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>09:15</t>
+          <t>09:10</t>
         </is>
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D90" t="n">
-        <v>39</v>
+        <v>79</v>
       </c>
       <c r="E90" t="inlineStr">
         <is>
@@ -2598,21 +2598,21 @@
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>07:27:35</t>
+          <t>08:50:55</t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>09:16</t>
+          <t>09:14</t>
         </is>
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D91" t="n">
-        <v>109</v>
+        <v>24</v>
       </c>
       <c r="E91" t="inlineStr">
         <is>
@@ -2628,16 +2628,16 @@
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>09:17</t>
+          <t>09:15</t>
         </is>
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D92" t="n">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="E92" t="inlineStr">
         <is>
@@ -2648,12 +2648,12 @@
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>08:14:14</t>
+          <t>08:50:55</t>
         </is>
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>09:18</t>
+          <t>09:16</t>
         </is>
       </c>
       <c r="C93" t="inlineStr">
@@ -2662,7 +2662,7 @@
         </is>
       </c>
       <c r="D93" t="n">
-        <v>64</v>
+        <v>26</v>
       </c>
       <c r="E93" t="inlineStr">
         <is>
@@ -2673,21 +2673,21 @@
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>07:51:37</t>
+          <t>08:36:09</t>
         </is>
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>09:18</t>
+          <t>09:17</t>
         </is>
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>215_EL PELIGRO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D94" t="n">
-        <v>87</v>
+        <v>41</v>
       </c>
       <c r="E94" t="inlineStr">
         <is>
@@ -2698,21 +2698,21 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>08:36:09</t>
+          <t>08:14:14</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>09:19</t>
+          <t>09:18</t>
         </is>
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>215_EL PELIGRO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D95" t="n">
-        <v>43</v>
+        <v>64</v>
       </c>
       <c r="E95" t="inlineStr">
         <is>
@@ -2723,21 +2723,21 @@
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>07:51:37</t>
+          <t>08:50:55</t>
         </is>
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>09:20</t>
+          <t>09:18</t>
         </is>
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D96" t="n">
-        <v>89</v>
+        <v>28</v>
       </c>
       <c r="E96" t="inlineStr">
         <is>
@@ -2748,21 +2748,21 @@
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>07:51:37</t>
+          <t>08:50:55</t>
         </is>
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>09:29</t>
+          <t>09:18</t>
         </is>
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>215_EL PELIGRO</t>
         </is>
       </c>
       <c r="D97" t="n">
-        <v>98</v>
+        <v>28</v>
       </c>
       <c r="E97" t="inlineStr">
         <is>
@@ -2778,16 +2778,16 @@
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>09:29</t>
+          <t>09:19</t>
         </is>
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215_EL PELIGRO</t>
         </is>
       </c>
       <c r="D98" t="n">
-        <v>53</v>
+        <v>43</v>
       </c>
       <c r="E98" t="inlineStr">
         <is>
@@ -2798,21 +2798,21 @@
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>08:14:14</t>
+          <t>07:51:37</t>
         </is>
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>09:33</t>
+          <t>09:20</t>
         </is>
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D99" t="n">
-        <v>79</v>
+        <v>89</v>
       </c>
       <c r="E99" t="inlineStr">
         <is>
@@ -2823,21 +2823,21 @@
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>08:14:14</t>
+          <t>08:50:55</t>
         </is>
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>09:33</t>
+          <t>09:21</t>
         </is>
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D100" t="n">
-        <v>79</v>
+        <v>31</v>
       </c>
       <c r="E100" t="inlineStr">
         <is>
@@ -2848,21 +2848,21 @@
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>08:36:09</t>
+          <t>07:51:37</t>
         </is>
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>09:34</t>
+          <t>09:29</t>
         </is>
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D101" t="n">
-        <v>58</v>
+        <v>98</v>
       </c>
       <c r="E101" t="inlineStr">
         <is>
@@ -2873,21 +2873,21 @@
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>07:51:37</t>
+          <t>08:36:09</t>
         </is>
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>09:44</t>
+          <t>09:29</t>
         </is>
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D102" t="n">
-        <v>113</v>
+        <v>53</v>
       </c>
       <c r="E102" t="inlineStr">
         <is>
@@ -2898,21 +2898,21 @@
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>08:36:09</t>
+          <t>08:14:14</t>
         </is>
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>09:45</t>
+          <t>09:33</t>
         </is>
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D103" t="n">
-        <v>69</v>
+        <v>79</v>
       </c>
       <c r="E103" t="inlineStr">
         <is>
@@ -2923,21 +2923,21 @@
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>08:36:09</t>
+          <t>08:50:55</t>
         </is>
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>09:51</t>
+          <t>09:33</t>
         </is>
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D104" t="n">
-        <v>75</v>
+        <v>43</v>
       </c>
       <c r="E104" t="inlineStr">
         <is>
@@ -2948,21 +2948,21 @@
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>08:36:09</t>
+          <t>08:50:55</t>
         </is>
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>09:54</t>
+          <t>09:34</t>
         </is>
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D105" t="n">
-        <v>78</v>
+        <v>44</v>
       </c>
       <c r="E105" t="inlineStr">
         <is>
@@ -2973,21 +2973,21 @@
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>08:36:09</t>
+          <t>08:50:55</t>
         </is>
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>09:56</t>
+          <t>09:44</t>
         </is>
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D106" t="n">
-        <v>80</v>
+        <v>54</v>
       </c>
       <c r="E106" t="inlineStr">
         <is>
@@ -3003,16 +3003,16 @@
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>10:04</t>
+          <t>09:45</t>
         </is>
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D107" t="n">
-        <v>88</v>
+        <v>69</v>
       </c>
       <c r="E107" t="inlineStr">
         <is>
@@ -3023,21 +3023,21 @@
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>08:36:09</t>
+          <t>08:50:55</t>
         </is>
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>10:09</t>
+          <t>09:51</t>
         </is>
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D108" t="n">
-        <v>93</v>
+        <v>61</v>
       </c>
       <c r="E108" t="inlineStr">
         <is>
@@ -3053,16 +3053,16 @@
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>10:19</t>
+          <t>09:54</t>
         </is>
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D109" t="n">
-        <v>103</v>
+        <v>78</v>
       </c>
       <c r="E109" t="inlineStr">
         <is>
@@ -3073,12 +3073,12 @@
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>08:36:09</t>
+          <t>08:50:55</t>
         </is>
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>10:20</t>
+          <t>09:56</t>
         </is>
       </c>
       <c r="C110" t="inlineStr">
@@ -3087,7 +3087,7 @@
         </is>
       </c>
       <c r="D110" t="n">
-        <v>104</v>
+        <v>66</v>
       </c>
       <c r="E110" t="inlineStr">
         <is>
@@ -3098,21 +3098,21 @@
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>08:36:09</t>
+          <t>08:50:55</t>
         </is>
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>10:33</t>
+          <t>10:03</t>
         </is>
       </c>
       <c r="C111" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D111" t="n">
-        <v>117</v>
+        <v>73</v>
       </c>
       <c r="E111" t="inlineStr">
         <is>
@@ -3128,18 +3128,268 @@
       </c>
       <c r="B112" t="inlineStr">
         <is>
+          <t>10:04</t>
+        </is>
+      </c>
+      <c r="C112" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D112" t="n">
+        <v>88</v>
+      </c>
+      <c r="E112" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" t="inlineStr">
+        <is>
+          <t>08:50:55</t>
+        </is>
+      </c>
+      <c r="B113" t="inlineStr">
+        <is>
+          <t>10:07</t>
+        </is>
+      </c>
+      <c r="C113" t="inlineStr">
+        <is>
+          <t>16_P MOR-SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D113" t="n">
+        <v>77</v>
+      </c>
+      <c r="E113" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" t="inlineStr">
+        <is>
+          <t>08:50:55</t>
+        </is>
+      </c>
+      <c r="B114" t="inlineStr">
+        <is>
+          <t>10:08</t>
+        </is>
+      </c>
+      <c r="C114" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D114" t="n">
+        <v>78</v>
+      </c>
+      <c r="E114" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" t="inlineStr">
+        <is>
+          <t>08:36:09</t>
+        </is>
+      </c>
+      <c r="B115" t="inlineStr">
+        <is>
+          <t>10:09</t>
+        </is>
+      </c>
+      <c r="C115" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D115" t="n">
+        <v>93</v>
+      </c>
+      <c r="E115" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" t="inlineStr">
+        <is>
+          <t>08:50:55</t>
+        </is>
+      </c>
+      <c r="B116" t="inlineStr">
+        <is>
+          <t>10:18</t>
+        </is>
+      </c>
+      <c r="C116" t="inlineStr">
+        <is>
+          <t>17_ROMERO</t>
+        </is>
+      </c>
+      <c r="D116" t="n">
+        <v>88</v>
+      </c>
+      <c r="E116" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" t="inlineStr">
+        <is>
+          <t>08:36:09</t>
+        </is>
+      </c>
+      <c r="B117" t="inlineStr">
+        <is>
+          <t>10:19</t>
+        </is>
+      </c>
+      <c r="C117" t="inlineStr">
+        <is>
+          <t>17_ROMERO</t>
+        </is>
+      </c>
+      <c r="D117" t="n">
+        <v>103</v>
+      </c>
+      <c r="E117" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" t="inlineStr">
+        <is>
+          <t>08:50:55</t>
+        </is>
+      </c>
+      <c r="B118" t="inlineStr">
+        <is>
+          <t>10:20</t>
+        </is>
+      </c>
+      <c r="C118" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D118" t="n">
+        <v>90</v>
+      </c>
+      <c r="E118" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" t="inlineStr">
+        <is>
+          <t>08:50:55</t>
+        </is>
+      </c>
+      <c r="B119" t="inlineStr">
+        <is>
+          <t>10:32</t>
+        </is>
+      </c>
+      <c r="C119" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D119" t="n">
+        <v>102</v>
+      </c>
+      <c r="E119" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" t="inlineStr">
+        <is>
+          <t>08:36:09</t>
+        </is>
+      </c>
+      <c r="B120" t="inlineStr">
+        <is>
+          <t>10:33</t>
+        </is>
+      </c>
+      <c r="C120" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D120" t="n">
+        <v>117</v>
+      </c>
+      <c r="E120" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" t="inlineStr">
+        <is>
+          <t>08:50:55</t>
+        </is>
+      </c>
+      <c r="B121" t="inlineStr">
+        <is>
           <t>10:34</t>
         </is>
       </c>
-      <c r="C112" t="inlineStr">
+      <c r="C121" t="inlineStr">
         <is>
           <t>15_ABASTO</t>
         </is>
       </c>
-      <c r="D112" t="n">
-        <v>118</v>
-      </c>
-      <c r="E112" t="inlineStr">
+      <c r="D121" t="n">
+        <v>104</v>
+      </c>
+      <c r="E121" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" t="inlineStr">
+        <is>
+          <t>08:50:55</t>
+        </is>
+      </c>
+      <c r="B122" t="inlineStr">
+        <is>
+          <t>10:43</t>
+        </is>
+      </c>
+      <c r="C122" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D122" t="n">
+        <v>113</v>
+      </c>
+      <c r="E122" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -3156,7 +3406,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E24"/>
+  <dimension ref="A1:E26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3169,14 +3419,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 08:36:09</t>
+          <t>Última actualización: 08:50:55</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 19</t>
+          <t>Total filas: 21</t>
         </is>
       </c>
     </row>
@@ -3560,21 +3810,21 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>07:51:37</t>
+          <t>08:50:55</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>08:59</t>
+          <t>08:51</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D20" t="n">
-        <v>68</v>
+        <v>1</v>
       </c>
       <c r="E20" t="inlineStr">
         <is>
@@ -3585,12 +3835,12 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>08:36:09</t>
+          <t>08:50:55</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>09:00</t>
+          <t>08:59</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
@@ -3599,7 +3849,7 @@
         </is>
       </c>
       <c r="D21" t="n">
-        <v>24</v>
+        <v>9</v>
       </c>
       <c r="E21" t="inlineStr">
         <is>
@@ -3610,21 +3860,21 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>07:51:37</t>
+          <t>08:36:09</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>09:18</t>
+          <t>09:00</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>215_EL PELIGRO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D22" t="n">
-        <v>87</v>
+        <v>24</v>
       </c>
       <c r="E22" t="inlineStr">
         <is>
@@ -3635,12 +3885,12 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>08:36:09</t>
+          <t>08:50:55</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>09:19</t>
+          <t>09:18</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
@@ -3649,7 +3899,7 @@
         </is>
       </c>
       <c r="D23" t="n">
-        <v>43</v>
+        <v>28</v>
       </c>
       <c r="E23" t="inlineStr">
         <is>
@@ -3665,18 +3915,68 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
+          <t>09:19</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>215_EL PELIGRO</t>
+        </is>
+      </c>
+      <c r="D24" t="n">
+        <v>43</v>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>08:50:55</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>10:03</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D25" t="n">
+        <v>73</v>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>08:36:09</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
           <t>10:04</t>
         </is>
       </c>
-      <c r="C24" t="inlineStr">
+      <c r="C26" t="inlineStr">
         <is>
           <t>215C_EL PATO</t>
         </is>
       </c>
-      <c r="D24" t="n">
+      <c r="D26" t="n">
         <v>88</v>
       </c>
-      <c r="E24" t="inlineStr">
+      <c r="E26" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -3693,7 +3993,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E24"/>
+  <dimension ref="A1:E28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3706,14 +4006,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 08:36:09</t>
+          <t>Última actualización: 08:50:55</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 19</t>
+          <t>Total filas: 23</t>
         </is>
       </c>
     </row>
@@ -4097,12 +4397,12 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>08:36:09</t>
+          <t>08:50:55</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>08:52</t>
+          <t>08:51</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -4111,7 +4411,7 @@
         </is>
       </c>
       <c r="D20" t="n">
-        <v>16</v>
+        <v>1</v>
       </c>
       <c r="E20" t="inlineStr">
         <is>
@@ -4122,37 +4422,37 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>08:14:14</t>
+          <t>08:36:09</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>09:56</t>
+          <t>08:52</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>215C_LA PLATA</t>
+          <t>215A_LA PLATA</t>
         </is>
       </c>
       <c r="D21" t="n">
-        <v>102</v>
+        <v>16</v>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>L6203</t>
+          <t>L6173</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>08:36:09</t>
+          <t>08:50:55</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>09:59</t>
+          <t>09:55</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
@@ -4161,7 +4461,7 @@
         </is>
       </c>
       <c r="D22" t="n">
-        <v>83</v>
+        <v>65</v>
       </c>
       <c r="E22" t="inlineStr">
         <is>
@@ -4172,25 +4472,25 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>08:36:09</t>
+          <t>08:14:14</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>10:11</t>
+          <t>09:56</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>215A_LA PLATA</t>
+          <t>215C_LA PLATA</t>
         </is>
       </c>
       <c r="D23" t="n">
-        <v>95</v>
+        <v>102</v>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>L6173</t>
+          <t>L6203</t>
         </is>
       </c>
     </row>
@@ -4202,18 +4502,118 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
+          <t>09:59</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D24" t="n">
+        <v>83</v>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>08:36:09</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>10:11</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>215A_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D25" t="n">
+        <v>95</v>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>08:50:55</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>10:13</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>215A_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D26" t="n">
+        <v>83</v>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>08:50:55</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>10:21</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>215B_LP-P MOR-1 Y 57</t>
+        </is>
+      </c>
+      <c r="D27" t="n">
+        <v>91</v>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>08:36:09</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
           <t>10:22</t>
         </is>
       </c>
-      <c r="C24" t="inlineStr">
+      <c r="C28" t="inlineStr">
         <is>
           <t>215B_LP-P MOR-1 Y 57</t>
         </is>
       </c>
-      <c r="D24" t="n">
+      <c r="D28" t="n">
         <v>106</v>
       </c>
-      <c r="E24" t="inlineStr">
+      <c r="E28" t="inlineStr">
         <is>
           <t>L6173</t>
         </is>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 1800
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-03-21.xlsx
+++ b/data/horarios-141-2026-03-21.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E122"/>
+  <dimension ref="A1:E135"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 08:50:55</t>
+          <t>Última actualización: 09:23:24</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 117</t>
+          <t>Total filas: 130</t>
         </is>
       </c>
     </row>
@@ -1158,7 +1158,7 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D33" t="n">
@@ -1183,7 +1183,7 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D34" t="n">
@@ -1873,7 +1873,7 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>08:14:14</t>
+          <t>06:59:30</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
@@ -1883,11 +1883,11 @@
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D62" t="n">
-        <v>0</v>
+        <v>75</v>
       </c>
       <c r="E62" t="inlineStr">
         <is>
@@ -1898,7 +1898,7 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>06:59:30</t>
+          <t>08:14:14</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
@@ -1908,11 +1908,11 @@
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D63" t="n">
-        <v>75</v>
+        <v>0</v>
       </c>
       <c r="E63" t="inlineStr">
         <is>
@@ -1973,7 +1973,7 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>07:51:37</t>
+          <t>07:27:35</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
@@ -1983,11 +1983,11 @@
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D66" t="n">
-        <v>28</v>
+        <v>52</v>
       </c>
       <c r="E66" t="inlineStr">
         <is>
@@ -2023,7 +2023,7 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>07:27:35</t>
+          <t>07:51:37</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
@@ -2033,11 +2033,11 @@
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D68" t="n">
-        <v>52</v>
+        <v>28</v>
       </c>
       <c r="E68" t="inlineStr">
         <is>
@@ -2233,7 +2233,7 @@
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D76" t="n">
@@ -2258,7 +2258,7 @@
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D77" t="n">
@@ -2373,7 +2373,7 @@
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>08:50:55</t>
+          <t>07:27:35</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
@@ -2383,11 +2383,11 @@
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D82" t="n">
-        <v>1</v>
+        <v>84</v>
       </c>
       <c r="E82" t="inlineStr">
         <is>
@@ -2423,7 +2423,7 @@
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>07:27:35</t>
+          <t>08:50:55</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
@@ -2433,11 +2433,11 @@
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D84" t="n">
-        <v>84</v>
+        <v>1</v>
       </c>
       <c r="E84" t="inlineStr">
         <is>
@@ -2698,7 +2698,7 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>08:14:14</t>
+          <t>08:50:55</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
@@ -2708,11 +2708,11 @@
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D95" t="n">
-        <v>64</v>
+        <v>28</v>
       </c>
       <c r="E95" t="inlineStr">
         <is>
@@ -2723,7 +2723,7 @@
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>08:50:55</t>
+          <t>08:14:14</t>
         </is>
       </c>
       <c r="B96" t="inlineStr">
@@ -2733,11 +2733,11 @@
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D96" t="n">
-        <v>28</v>
+        <v>64</v>
       </c>
       <c r="E96" t="inlineStr">
         <is>
@@ -2848,21 +2848,21 @@
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>07:51:37</t>
+          <t>09:23:24</t>
         </is>
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>09:29</t>
+          <t>09:24</t>
         </is>
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D101" t="n">
-        <v>98</v>
+        <v>1</v>
       </c>
       <c r="E101" t="inlineStr">
         <is>
@@ -2873,7 +2873,7 @@
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>08:36:09</t>
+          <t>07:51:37</t>
         </is>
       </c>
       <c r="B102" t="inlineStr">
@@ -2883,11 +2883,11 @@
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D102" t="n">
-        <v>53</v>
+        <v>98</v>
       </c>
       <c r="E102" t="inlineStr">
         <is>
@@ -2898,21 +2898,21 @@
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>08:14:14</t>
+          <t>08:36:09</t>
         </is>
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>09:33</t>
+          <t>09:29</t>
         </is>
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D103" t="n">
-        <v>79</v>
+        <v>53</v>
       </c>
       <c r="E103" t="inlineStr">
         <is>
@@ -2923,7 +2923,7 @@
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>08:50:55</t>
+          <t>08:14:14</t>
         </is>
       </c>
       <c r="B104" t="inlineStr">
@@ -2933,11 +2933,11 @@
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D104" t="n">
-        <v>43</v>
+        <v>79</v>
       </c>
       <c r="E104" t="inlineStr">
         <is>
@@ -2948,21 +2948,21 @@
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>08:50:55</t>
+          <t>09:23:24</t>
         </is>
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>09:34</t>
+          <t>09:33</t>
         </is>
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D105" t="n">
-        <v>44</v>
+        <v>10</v>
       </c>
       <c r="E105" t="inlineStr">
         <is>
@@ -2973,21 +2973,21 @@
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>08:50:55</t>
+          <t>09:23:24</t>
         </is>
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>09:44</t>
+          <t>09:34</t>
         </is>
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D106" t="n">
-        <v>54</v>
+        <v>11</v>
       </c>
       <c r="E106" t="inlineStr">
         <is>
@@ -2998,21 +2998,21 @@
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>08:36:09</t>
+          <t>09:23:24</t>
         </is>
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>09:45</t>
+          <t>09:41</t>
         </is>
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D107" t="n">
-        <v>69</v>
+        <v>18</v>
       </c>
       <c r="E107" t="inlineStr">
         <is>
@@ -3023,21 +3023,21 @@
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>08:50:55</t>
+          <t>09:23:24</t>
         </is>
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>09:51</t>
+          <t>09:44</t>
         </is>
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D108" t="n">
-        <v>61</v>
+        <v>21</v>
       </c>
       <c r="E108" t="inlineStr">
         <is>
@@ -3053,16 +3053,16 @@
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>09:54</t>
+          <t>09:45</t>
         </is>
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D109" t="n">
-        <v>78</v>
+        <v>69</v>
       </c>
       <c r="E109" t="inlineStr">
         <is>
@@ -3073,21 +3073,21 @@
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>08:50:55</t>
+          <t>09:23:24</t>
         </is>
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>09:56</t>
+          <t>09:51</t>
         </is>
       </c>
       <c r="C110" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D110" t="n">
-        <v>66</v>
+        <v>28</v>
       </c>
       <c r="E110" t="inlineStr">
         <is>
@@ -3098,21 +3098,21 @@
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>08:50:55</t>
+          <t>09:23:24</t>
         </is>
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>10:03</t>
+          <t>09:51</t>
         </is>
       </c>
       <c r="C111" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D111" t="n">
-        <v>73</v>
+        <v>28</v>
       </c>
       <c r="E111" t="inlineStr">
         <is>
@@ -3128,16 +3128,16 @@
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>10:04</t>
+          <t>09:54</t>
         </is>
       </c>
       <c r="C112" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D112" t="n">
-        <v>88</v>
+        <v>78</v>
       </c>
       <c r="E112" t="inlineStr">
         <is>
@@ -3148,21 +3148,21 @@
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>08:50:55</t>
+          <t>09:23:24</t>
         </is>
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>10:07</t>
+          <t>09:56</t>
         </is>
       </c>
       <c r="C113" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D113" t="n">
-        <v>77</v>
+        <v>33</v>
       </c>
       <c r="E113" t="inlineStr">
         <is>
@@ -3173,21 +3173,21 @@
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>08:50:55</t>
+          <t>09:23:24</t>
         </is>
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>10:08</t>
+          <t>10:03</t>
         </is>
       </c>
       <c r="C114" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D114" t="n">
-        <v>78</v>
+        <v>40</v>
       </c>
       <c r="E114" t="inlineStr">
         <is>
@@ -3198,21 +3198,21 @@
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>08:36:09</t>
+          <t>08:50:55</t>
         </is>
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>10:09</t>
+          <t>10:03</t>
         </is>
       </c>
       <c r="C115" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D115" t="n">
-        <v>93</v>
+        <v>73</v>
       </c>
       <c r="E115" t="inlineStr">
         <is>
@@ -3223,21 +3223,21 @@
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t>08:50:55</t>
+          <t>09:23:24</t>
         </is>
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t>10:18</t>
+          <t>10:04</t>
         </is>
       </c>
       <c r="C116" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D116" t="n">
-        <v>88</v>
+        <v>41</v>
       </c>
       <c r="E116" t="inlineStr">
         <is>
@@ -3248,21 +3248,21 @@
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
-          <t>08:36:09</t>
+          <t>08:50:55</t>
         </is>
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>10:19</t>
+          <t>10:07</t>
         </is>
       </c>
       <c r="C117" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D117" t="n">
-        <v>103</v>
+        <v>77</v>
       </c>
       <c r="E117" t="inlineStr">
         <is>
@@ -3278,16 +3278,16 @@
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t>10:20</t>
+          <t>10:08</t>
         </is>
       </c>
       <c r="C118" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D118" t="n">
-        <v>90</v>
+        <v>78</v>
       </c>
       <c r="E118" t="inlineStr">
         <is>
@@ -3298,21 +3298,21 @@
     <row r="119">
       <c r="A119" t="inlineStr">
         <is>
-          <t>08:50:55</t>
+          <t>08:36:09</t>
         </is>
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t>10:32</t>
+          <t>10:09</t>
         </is>
       </c>
       <c r="C119" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D119" t="n">
-        <v>102</v>
+        <v>93</v>
       </c>
       <c r="E119" t="inlineStr">
         <is>
@@ -3323,21 +3323,21 @@
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t>08:36:09</t>
+          <t>09:23:24</t>
         </is>
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>10:33</t>
+          <t>10:14</t>
         </is>
       </c>
       <c r="C120" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D120" t="n">
-        <v>117</v>
+        <v>51</v>
       </c>
       <c r="E120" t="inlineStr">
         <is>
@@ -3353,16 +3353,16 @@
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>10:34</t>
+          <t>10:18</t>
         </is>
       </c>
       <c r="C121" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D121" t="n">
-        <v>104</v>
+        <v>88</v>
       </c>
       <c r="E121" t="inlineStr">
         <is>
@@ -3373,23 +3373,348 @@
     <row r="122">
       <c r="A122" t="inlineStr">
         <is>
+          <t>09:23:24</t>
+        </is>
+      </c>
+      <c r="B122" t="inlineStr">
+        <is>
+          <t>10:19</t>
+        </is>
+      </c>
+      <c r="C122" t="inlineStr">
+        <is>
+          <t>17_ROMERO</t>
+        </is>
+      </c>
+      <c r="D122" t="n">
+        <v>56</v>
+      </c>
+      <c r="E122" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" t="inlineStr">
+        <is>
+          <t>09:23:24</t>
+        </is>
+      </c>
+      <c r="B123" t="inlineStr">
+        <is>
+          <t>10:20</t>
+        </is>
+      </c>
+      <c r="C123" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D123" t="n">
+        <v>57</v>
+      </c>
+      <c r="E123" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" t="inlineStr">
+        <is>
           <t>08:50:55</t>
         </is>
       </c>
-      <c r="B122" t="inlineStr">
+      <c r="B124" t="inlineStr">
+        <is>
+          <t>10:32</t>
+        </is>
+      </c>
+      <c r="C124" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D124" t="n">
+        <v>102</v>
+      </c>
+      <c r="E124" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" t="inlineStr">
+        <is>
+          <t>08:36:09</t>
+        </is>
+      </c>
+      <c r="B125" t="inlineStr">
+        <is>
+          <t>10:33</t>
+        </is>
+      </c>
+      <c r="C125" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D125" t="n">
+        <v>117</v>
+      </c>
+      <c r="E125" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" t="inlineStr">
+        <is>
+          <t>08:50:55</t>
+        </is>
+      </c>
+      <c r="B126" t="inlineStr">
+        <is>
+          <t>10:34</t>
+        </is>
+      </c>
+      <c r="C126" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D126" t="n">
+        <v>104</v>
+      </c>
+      <c r="E126" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" t="inlineStr">
+        <is>
+          <t>09:23:24</t>
+        </is>
+      </c>
+      <c r="B127" t="inlineStr">
         <is>
           <t>10:43</t>
         </is>
       </c>
-      <c r="C122" t="inlineStr">
+      <c r="C127" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D127" t="n">
+        <v>80</v>
+      </c>
+      <c r="E127" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" t="inlineStr">
+        <is>
+          <t>08:50:55</t>
+        </is>
+      </c>
+      <c r="B128" t="inlineStr">
+        <is>
+          <t>10:43</t>
+        </is>
+      </c>
+      <c r="C128" t="inlineStr">
         <is>
           <t>10_OLMOS</t>
         </is>
       </c>
-      <c r="D122" t="n">
+      <c r="D128" t="n">
         <v>113</v>
       </c>
-      <c r="E122" t="inlineStr">
+      <c r="E128" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" t="inlineStr">
+        <is>
+          <t>09:23:24</t>
+        </is>
+      </c>
+      <c r="B129" t="inlineStr">
+        <is>
+          <t>10:44</t>
+        </is>
+      </c>
+      <c r="C129" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D129" t="n">
+        <v>81</v>
+      </c>
+      <c r="E129" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" t="inlineStr">
+        <is>
+          <t>09:23:24</t>
+        </is>
+      </c>
+      <c r="B130" t="inlineStr">
+        <is>
+          <t>10:56</t>
+        </is>
+      </c>
+      <c r="C130" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D130" t="n">
+        <v>93</v>
+      </c>
+      <c r="E130" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" t="inlineStr">
+        <is>
+          <t>09:23:24</t>
+        </is>
+      </c>
+      <c r="B131" t="inlineStr">
+        <is>
+          <t>10:57</t>
+        </is>
+      </c>
+      <c r="C131" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D131" t="n">
+        <v>94</v>
+      </c>
+      <c r="E131" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" t="inlineStr">
+        <is>
+          <t>09:23:24</t>
+        </is>
+      </c>
+      <c r="B132" t="inlineStr">
+        <is>
+          <t>11:04</t>
+        </is>
+      </c>
+      <c r="C132" t="inlineStr">
+        <is>
+          <t>17_ROMERO</t>
+        </is>
+      </c>
+      <c r="D132" t="n">
+        <v>101</v>
+      </c>
+      <c r="E132" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" t="inlineStr">
+        <is>
+          <t>09:23:24</t>
+        </is>
+      </c>
+      <c r="B133" t="inlineStr">
+        <is>
+          <t>11:08</t>
+        </is>
+      </c>
+      <c r="C133" t="inlineStr">
+        <is>
+          <t>225_C ROCA-H SUR</t>
+        </is>
+      </c>
+      <c r="D133" t="n">
+        <v>105</v>
+      </c>
+      <c r="E133" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" t="inlineStr">
+        <is>
+          <t>09:23:24</t>
+        </is>
+      </c>
+      <c r="B134" t="inlineStr">
+        <is>
+          <t>11:19</t>
+        </is>
+      </c>
+      <c r="C134" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D134" t="n">
+        <v>116</v>
+      </c>
+      <c r="E134" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" t="inlineStr">
+        <is>
+          <t>09:23:24</t>
+        </is>
+      </c>
+      <c r="B135" t="inlineStr">
+        <is>
+          <t>11:20</t>
+        </is>
+      </c>
+      <c r="C135" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D135" t="n">
+        <v>117</v>
+      </c>
+      <c r="E135" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -3406,7 +3731,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E26"/>
+  <dimension ref="A1:E27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3419,14 +3744,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 08:50:55</t>
+          <t>Última actualización: 09:23:24</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 21</t>
+          <t>Total filas: 22</t>
         </is>
       </c>
     </row>
@@ -3960,7 +4285,7 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>08:36:09</t>
+          <t>09:23:24</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -3974,9 +4299,34 @@
         </is>
       </c>
       <c r="D26" t="n">
-        <v>88</v>
+        <v>41</v>
       </c>
       <c r="E26" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>09:23:24</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>11:19</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D27" t="n">
+        <v>116</v>
+      </c>
+      <c r="E27" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -3993,7 +4343,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E28"/>
+  <dimension ref="A1:E29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4006,14 +4356,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 08:50:55</t>
+          <t>Última actualización: 09:23:24</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 23</t>
+          <t>Total filas: 24</t>
         </is>
       </c>
     </row>
@@ -4497,7 +4847,7 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>08:36:09</t>
+          <t>09:23:24</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -4511,7 +4861,7 @@
         </is>
       </c>
       <c r="D24" t="n">
-        <v>83</v>
+        <v>36</v>
       </c>
       <c r="E24" t="inlineStr">
         <is>
@@ -4597,7 +4947,7 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>08:36:09</t>
+          <t>09:23:24</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -4611,9 +4961,34 @@
         </is>
       </c>
       <c r="D28" t="n">
-        <v>106</v>
+        <v>59</v>
       </c>
       <c r="E28" t="inlineStr">
+        <is>
+          <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>09:23:24</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>10:24</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>215A_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D29" t="n">
+        <v>61</v>
+      </c>
+      <c r="E29" t="inlineStr">
         <is>
           <t>L6173</t>
         </is>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 1801
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-03-21.xlsx
+++ b/data/horarios-141-2026-03-21.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E135"/>
+  <dimension ref="A1:E150"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 09:23:24</t>
+          <t>Última actualización: 10:14:52</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 130</t>
+          <t>Total filas: 145</t>
         </is>
       </c>
     </row>
@@ -1158,7 +1158,7 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D33" t="n">
@@ -1183,7 +1183,7 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D34" t="n">
@@ -1558,7 +1558,7 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D49" t="n">
@@ -1583,7 +1583,7 @@
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D50" t="n">
@@ -1973,7 +1973,7 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>07:27:35</t>
+          <t>07:51:37</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
@@ -1983,11 +1983,11 @@
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D66" t="n">
-        <v>52</v>
+        <v>28</v>
       </c>
       <c r="E66" t="inlineStr">
         <is>
@@ -2023,7 +2023,7 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>07:51:37</t>
+          <t>07:27:35</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
@@ -2033,11 +2033,11 @@
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D68" t="n">
-        <v>28</v>
+        <v>52</v>
       </c>
       <c r="E68" t="inlineStr">
         <is>
@@ -2233,7 +2233,7 @@
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D76" t="n">
@@ -2258,7 +2258,7 @@
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D77" t="n">
@@ -2873,7 +2873,7 @@
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>07:51:37</t>
+          <t>08:36:09</t>
         </is>
       </c>
       <c r="B102" t="inlineStr">
@@ -2883,11 +2883,11 @@
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D102" t="n">
-        <v>98</v>
+        <v>53</v>
       </c>
       <c r="E102" t="inlineStr">
         <is>
@@ -2898,7 +2898,7 @@
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>08:36:09</t>
+          <t>07:51:37</t>
         </is>
       </c>
       <c r="B103" t="inlineStr">
@@ -2908,11 +2908,11 @@
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D103" t="n">
-        <v>53</v>
+        <v>98</v>
       </c>
       <c r="E103" t="inlineStr">
         <is>
@@ -2923,7 +2923,7 @@
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>08:14:14</t>
+          <t>09:23:24</t>
         </is>
       </c>
       <c r="B104" t="inlineStr">
@@ -2933,11 +2933,11 @@
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D104" t="n">
-        <v>79</v>
+        <v>10</v>
       </c>
       <c r="E104" t="inlineStr">
         <is>
@@ -2948,7 +2948,7 @@
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>09:23:24</t>
+          <t>08:14:14</t>
         </is>
       </c>
       <c r="B105" t="inlineStr">
@@ -2958,11 +2958,11 @@
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D105" t="n">
-        <v>10</v>
+        <v>79</v>
       </c>
       <c r="E105" t="inlineStr">
         <is>
@@ -3348,21 +3348,21 @@
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>08:50:55</t>
+          <t>10:14:52</t>
         </is>
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>10:18</t>
+          <t>10:15</t>
         </is>
       </c>
       <c r="C121" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D121" t="n">
-        <v>88</v>
+        <v>1</v>
       </c>
       <c r="E121" t="inlineStr">
         <is>
@@ -3373,21 +3373,21 @@
     <row r="122">
       <c r="A122" t="inlineStr">
         <is>
-          <t>09:23:24</t>
+          <t>10:14:52</t>
         </is>
       </c>
       <c r="B122" t="inlineStr">
         <is>
-          <t>10:19</t>
+          <t>10:16</t>
         </is>
       </c>
       <c r="C122" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D122" t="n">
-        <v>56</v>
+        <v>2</v>
       </c>
       <c r="E122" t="inlineStr">
         <is>
@@ -3398,21 +3398,21 @@
     <row r="123">
       <c r="A123" t="inlineStr">
         <is>
-          <t>09:23:24</t>
+          <t>08:50:55</t>
         </is>
       </c>
       <c r="B123" t="inlineStr">
         <is>
-          <t>10:20</t>
+          <t>10:18</t>
         </is>
       </c>
       <c r="C123" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D123" t="n">
-        <v>57</v>
+        <v>88</v>
       </c>
       <c r="E123" t="inlineStr">
         <is>
@@ -3423,21 +3423,21 @@
     <row r="124">
       <c r="A124" t="inlineStr">
         <is>
-          <t>08:50:55</t>
+          <t>09:23:24</t>
         </is>
       </c>
       <c r="B124" t="inlineStr">
         <is>
-          <t>10:32</t>
+          <t>10:19</t>
         </is>
       </c>
       <c r="C124" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D124" t="n">
-        <v>102</v>
+        <v>56</v>
       </c>
       <c r="E124" t="inlineStr">
         <is>
@@ -3448,21 +3448,21 @@
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>08:36:09</t>
+          <t>10:14:52</t>
         </is>
       </c>
       <c r="B125" t="inlineStr">
         <is>
-          <t>10:33</t>
+          <t>10:20</t>
         </is>
       </c>
       <c r="C125" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D125" t="n">
-        <v>117</v>
+        <v>6</v>
       </c>
       <c r="E125" t="inlineStr">
         <is>
@@ -3473,21 +3473,21 @@
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t>08:50:55</t>
+          <t>10:14:52</t>
         </is>
       </c>
       <c r="B126" t="inlineStr">
         <is>
-          <t>10:34</t>
+          <t>10:32</t>
         </is>
       </c>
       <c r="C126" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D126" t="n">
-        <v>104</v>
+        <v>18</v>
       </c>
       <c r="E126" t="inlineStr">
         <is>
@@ -3498,21 +3498,21 @@
     <row r="127">
       <c r="A127" t="inlineStr">
         <is>
-          <t>09:23:24</t>
+          <t>08:36:09</t>
         </is>
       </c>
       <c r="B127" t="inlineStr">
         <is>
-          <t>10:43</t>
+          <t>10:33</t>
         </is>
       </c>
       <c r="C127" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D127" t="n">
-        <v>80</v>
+        <v>117</v>
       </c>
       <c r="E127" t="inlineStr">
         <is>
@@ -3523,21 +3523,21 @@
     <row r="128">
       <c r="A128" t="inlineStr">
         <is>
-          <t>08:50:55</t>
+          <t>10:14:52</t>
         </is>
       </c>
       <c r="B128" t="inlineStr">
         <is>
-          <t>10:43</t>
+          <t>10:33</t>
         </is>
       </c>
       <c r="C128" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D128" t="n">
-        <v>113</v>
+        <v>19</v>
       </c>
       <c r="E128" t="inlineStr">
         <is>
@@ -3548,21 +3548,21 @@
     <row r="129">
       <c r="A129" t="inlineStr">
         <is>
-          <t>09:23:24</t>
+          <t>10:14:52</t>
         </is>
       </c>
       <c r="B129" t="inlineStr">
         <is>
-          <t>10:44</t>
+          <t>10:34</t>
         </is>
       </c>
       <c r="C129" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D129" t="n">
-        <v>81</v>
+        <v>20</v>
       </c>
       <c r="E129" t="inlineStr">
         <is>
@@ -3573,21 +3573,21 @@
     <row r="130">
       <c r="A130" t="inlineStr">
         <is>
-          <t>09:23:24</t>
+          <t>10:14:52</t>
         </is>
       </c>
       <c r="B130" t="inlineStr">
         <is>
-          <t>10:56</t>
+          <t>10:41</t>
         </is>
       </c>
       <c r="C130" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D130" t="n">
-        <v>93</v>
+        <v>27</v>
       </c>
       <c r="E130" t="inlineStr">
         <is>
@@ -3598,21 +3598,21 @@
     <row r="131">
       <c r="A131" t="inlineStr">
         <is>
-          <t>09:23:24</t>
+          <t>10:14:52</t>
         </is>
       </c>
       <c r="B131" t="inlineStr">
         <is>
-          <t>10:57</t>
+          <t>10:43</t>
         </is>
       </c>
       <c r="C131" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D131" t="n">
-        <v>94</v>
+        <v>29</v>
       </c>
       <c r="E131" t="inlineStr">
         <is>
@@ -3628,16 +3628,16 @@
       </c>
       <c r="B132" t="inlineStr">
         <is>
-          <t>11:04</t>
+          <t>10:43</t>
         </is>
       </c>
       <c r="C132" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D132" t="n">
-        <v>101</v>
+        <v>80</v>
       </c>
       <c r="E132" t="inlineStr">
         <is>
@@ -3653,16 +3653,16 @@
       </c>
       <c r="B133" t="inlineStr">
         <is>
-          <t>11:08</t>
+          <t>10:44</t>
         </is>
       </c>
       <c r="C133" t="inlineStr">
         <is>
-          <t>225_C ROCA-H SUR</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D133" t="n">
-        <v>105</v>
+        <v>81</v>
       </c>
       <c r="E133" t="inlineStr">
         <is>
@@ -3673,21 +3673,21 @@
     <row r="134">
       <c r="A134" t="inlineStr">
         <is>
-          <t>09:23:24</t>
+          <t>10:14:52</t>
         </is>
       </c>
       <c r="B134" t="inlineStr">
         <is>
-          <t>11:19</t>
+          <t>10:51</t>
         </is>
       </c>
       <c r="C134" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D134" t="n">
-        <v>116</v>
+        <v>37</v>
       </c>
       <c r="E134" t="inlineStr">
         <is>
@@ -3698,23 +3698,398 @@
     <row r="135">
       <c r="A135" t="inlineStr">
         <is>
+          <t>10:14:52</t>
+        </is>
+      </c>
+      <c r="B135" t="inlineStr">
+        <is>
+          <t>10:56</t>
+        </is>
+      </c>
+      <c r="C135" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D135" t="n">
+        <v>42</v>
+      </c>
+      <c r="E135" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" t="inlineStr">
+        <is>
           <t>09:23:24</t>
         </is>
       </c>
-      <c r="B135" t="inlineStr">
+      <c r="B136" t="inlineStr">
+        <is>
+          <t>10:57</t>
+        </is>
+      </c>
+      <c r="C136" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D136" t="n">
+        <v>94</v>
+      </c>
+      <c r="E136" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137" t="inlineStr">
+        <is>
+          <t>10:14:52</t>
+        </is>
+      </c>
+      <c r="B137" t="inlineStr">
+        <is>
+          <t>10:59</t>
+        </is>
+      </c>
+      <c r="C137" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D137" t="n">
+        <v>45</v>
+      </c>
+      <c r="E137" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" t="inlineStr">
+        <is>
+          <t>10:14:52</t>
+        </is>
+      </c>
+      <c r="B138" t="inlineStr">
+        <is>
+          <t>11:03</t>
+        </is>
+      </c>
+      <c r="C138" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D138" t="n">
+        <v>49</v>
+      </c>
+      <c r="E138" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" t="inlineStr">
+        <is>
+          <t>10:14:52</t>
+        </is>
+      </c>
+      <c r="B139" t="inlineStr">
+        <is>
+          <t>11:04</t>
+        </is>
+      </c>
+      <c r="C139" t="inlineStr">
+        <is>
+          <t>17_ROMERO</t>
+        </is>
+      </c>
+      <c r="D139" t="n">
+        <v>50</v>
+      </c>
+      <c r="E139" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" t="inlineStr">
+        <is>
+          <t>10:14:52</t>
+        </is>
+      </c>
+      <c r="B140" t="inlineStr">
+        <is>
+          <t>11:07</t>
+        </is>
+      </c>
+      <c r="C140" t="inlineStr">
+        <is>
+          <t>225_C ROCA-H SUR</t>
+        </is>
+      </c>
+      <c r="D140" t="n">
+        <v>53</v>
+      </c>
+      <c r="E140" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" t="inlineStr">
+        <is>
+          <t>09:23:24</t>
+        </is>
+      </c>
+      <c r="B141" t="inlineStr">
+        <is>
+          <t>11:08</t>
+        </is>
+      </c>
+      <c r="C141" t="inlineStr">
+        <is>
+          <t>225_C ROCA-H SUR</t>
+        </is>
+      </c>
+      <c r="D141" t="n">
+        <v>105</v>
+      </c>
+      <c r="E141" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" t="inlineStr">
+        <is>
+          <t>10:14:52</t>
+        </is>
+      </c>
+      <c r="B142" t="inlineStr">
+        <is>
+          <t>11:18</t>
+        </is>
+      </c>
+      <c r="C142" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D142" t="n">
+        <v>64</v>
+      </c>
+      <c r="E142" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" t="inlineStr">
+        <is>
+          <t>09:23:24</t>
+        </is>
+      </c>
+      <c r="B143" t="inlineStr">
+        <is>
+          <t>11:19</t>
+        </is>
+      </c>
+      <c r="C143" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D143" t="n">
+        <v>116</v>
+      </c>
+      <c r="E143" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144" t="inlineStr">
+        <is>
+          <t>10:14:52</t>
+        </is>
+      </c>
+      <c r="B144" t="inlineStr">
         <is>
           <t>11:20</t>
         </is>
       </c>
-      <c r="C135" t="inlineStr">
+      <c r="C144" t="inlineStr">
         <is>
           <t>11_ETCHEVERRY</t>
         </is>
       </c>
-      <c r="D135" t="n">
-        <v>117</v>
-      </c>
-      <c r="E135" t="inlineStr">
+      <c r="D144" t="n">
+        <v>66</v>
+      </c>
+      <c r="E144" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="145">
+      <c r="A145" t="inlineStr">
+        <is>
+          <t>10:14:52</t>
+        </is>
+      </c>
+      <c r="B145" t="inlineStr">
+        <is>
+          <t>11:32</t>
+        </is>
+      </c>
+      <c r="C145" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D145" t="n">
+        <v>78</v>
+      </c>
+      <c r="E145" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="146">
+      <c r="A146" t="inlineStr">
+        <is>
+          <t>10:14:52</t>
+        </is>
+      </c>
+      <c r="B146" t="inlineStr">
+        <is>
+          <t>11:34</t>
+        </is>
+      </c>
+      <c r="C146" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D146" t="n">
+        <v>80</v>
+      </c>
+      <c r="E146" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="147">
+      <c r="A147" t="inlineStr">
+        <is>
+          <t>10:14:52</t>
+        </is>
+      </c>
+      <c r="B147" t="inlineStr">
+        <is>
+          <t>11:40</t>
+        </is>
+      </c>
+      <c r="C147" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D147" t="n">
+        <v>86</v>
+      </c>
+      <c r="E147" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="148">
+      <c r="A148" t="inlineStr">
+        <is>
+          <t>10:14:52</t>
+        </is>
+      </c>
+      <c r="B148" t="inlineStr">
+        <is>
+          <t>11:44</t>
+        </is>
+      </c>
+      <c r="C148" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D148" t="n">
+        <v>90</v>
+      </c>
+      <c r="E148" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149" t="inlineStr">
+        <is>
+          <t>10:14:52</t>
+        </is>
+      </c>
+      <c r="B149" t="inlineStr">
+        <is>
+          <t>11:55</t>
+        </is>
+      </c>
+      <c r="C149" t="inlineStr">
+        <is>
+          <t>225_GOMEZ</t>
+        </is>
+      </c>
+      <c r="D149" t="n">
+        <v>101</v>
+      </c>
+      <c r="E149" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="150">
+      <c r="A150" t="inlineStr">
+        <is>
+          <t>10:14:52</t>
+        </is>
+      </c>
+      <c r="B150" t="inlineStr">
+        <is>
+          <t>12:04</t>
+        </is>
+      </c>
+      <c r="C150" t="inlineStr">
+        <is>
+          <t>17_ROMERO</t>
+        </is>
+      </c>
+      <c r="D150" t="n">
+        <v>110</v>
+      </c>
+      <c r="E150" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -3731,7 +4106,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E27"/>
+  <dimension ref="A1:E30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3744,14 +4119,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 09:23:24</t>
+          <t>Última actualización: 10:14:52</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 22</t>
+          <t>Total filas: 25</t>
         </is>
       </c>
     </row>
@@ -4310,23 +4685,98 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
+          <t>10:14:52</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>11:18</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D27" t="n">
+        <v>64</v>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
           <t>09:23:24</t>
         </is>
       </c>
-      <c r="B27" t="inlineStr">
+      <c r="B28" t="inlineStr">
         <is>
           <t>11:19</t>
         </is>
       </c>
-      <c r="C27" t="inlineStr">
+      <c r="C28" t="inlineStr">
         <is>
           <t>215C_EL PATO</t>
         </is>
       </c>
-      <c r="D27" t="n">
+      <c r="D28" t="n">
         <v>116</v>
       </c>
-      <c r="E27" t="inlineStr">
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>10:14:52</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>11:32</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D29" t="n">
+        <v>78</v>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>10:14:52</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>11:44</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D30" t="n">
+        <v>90</v>
+      </c>
+      <c r="E30" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -4343,7 +4793,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E29"/>
+  <dimension ref="A1:E32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4356,14 +4806,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 09:23:24</t>
+          <t>Última actualización: 10:14:52</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 24</t>
+          <t>Total filas: 27</t>
         </is>
       </c>
     </row>
@@ -4922,21 +5372,21 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>08:50:55</t>
+          <t>10:14:52</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>10:21</t>
+          <t>10:17</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>215B_LP-P MOR-1 Y 57</t>
+          <t>215A_LA PLATA</t>
         </is>
       </c>
       <c r="D27" t="n">
-        <v>91</v>
+        <v>3</v>
       </c>
       <c r="E27" t="inlineStr">
         <is>
@@ -4947,12 +5397,12 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>09:23:24</t>
+          <t>10:14:52</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>10:22</t>
+          <t>10:21</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
@@ -4961,7 +5411,7 @@
         </is>
       </c>
       <c r="D28" t="n">
-        <v>59</v>
+        <v>7</v>
       </c>
       <c r="E28" t="inlineStr">
         <is>
@@ -4977,20 +5427,95 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
+          <t>10:22</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>215B_LP-P MOR-1 Y 57</t>
+        </is>
+      </c>
+      <c r="D29" t="n">
+        <v>59</v>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>09:23:24</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
           <t>10:24</t>
         </is>
       </c>
-      <c r="C29" t="inlineStr">
+      <c r="C30" t="inlineStr">
         <is>
           <t>215A_LA PLATA</t>
         </is>
       </c>
-      <c r="D29" t="n">
+      <c r="D30" t="n">
         <v>61</v>
       </c>
-      <c r="E29" t="inlineStr">
+      <c r="E30" t="inlineStr">
         <is>
           <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>10:14:52</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>11:34</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>215A_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D31" t="n">
+        <v>80</v>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>10:14:52</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>11:55</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D32" t="n">
+        <v>101</v>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>L6203</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 1802
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-03-21.xlsx
+++ b/data/horarios-141-2026-03-21.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E150"/>
+  <dimension ref="A1:E167"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 10:14:52</t>
+          <t>Última actualización: 10:52:37</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 145</t>
+          <t>Total filas: 162</t>
         </is>
       </c>
     </row>
@@ -1873,7 +1873,7 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>06:59:30</t>
+          <t>08:14:14</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
@@ -1883,11 +1883,11 @@
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D62" t="n">
-        <v>75</v>
+        <v>0</v>
       </c>
       <c r="E62" t="inlineStr">
         <is>
@@ -1898,7 +1898,7 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>08:14:14</t>
+          <t>06:59:30</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
@@ -1908,11 +1908,11 @@
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D63" t="n">
-        <v>0</v>
+        <v>75</v>
       </c>
       <c r="E63" t="inlineStr">
         <is>
@@ -2233,7 +2233,7 @@
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D76" t="n">
@@ -2258,7 +2258,7 @@
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D77" t="n">
@@ -2373,7 +2373,7 @@
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>07:27:35</t>
+          <t>08:50:55</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
@@ -2383,11 +2383,11 @@
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D82" t="n">
-        <v>84</v>
+        <v>1</v>
       </c>
       <c r="E82" t="inlineStr">
         <is>
@@ -2408,7 +2408,7 @@
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D83" t="n">
@@ -2423,7 +2423,7 @@
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>08:50:55</t>
+          <t>07:27:35</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
@@ -2433,11 +2433,11 @@
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D84" t="n">
-        <v>1</v>
+        <v>84</v>
       </c>
       <c r="E84" t="inlineStr">
         <is>
@@ -2723,7 +2723,7 @@
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>08:14:14</t>
+          <t>08:50:55</t>
         </is>
       </c>
       <c r="B96" t="inlineStr">
@@ -2733,11 +2733,11 @@
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>215_EL PELIGRO</t>
         </is>
       </c>
       <c r="D96" t="n">
-        <v>64</v>
+        <v>28</v>
       </c>
       <c r="E96" t="inlineStr">
         <is>
@@ -2748,7 +2748,7 @@
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>08:50:55</t>
+          <t>08:14:14</t>
         </is>
       </c>
       <c r="B97" t="inlineStr">
@@ -2758,11 +2758,11 @@
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>215_EL PELIGRO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D97" t="n">
-        <v>28</v>
+        <v>64</v>
       </c>
       <c r="E97" t="inlineStr">
         <is>
@@ -2923,7 +2923,7 @@
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>09:23:24</t>
+          <t>08:14:14</t>
         </is>
       </c>
       <c r="B104" t="inlineStr">
@@ -2933,11 +2933,11 @@
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D104" t="n">
-        <v>10</v>
+        <v>79</v>
       </c>
       <c r="E104" t="inlineStr">
         <is>
@@ -2948,7 +2948,7 @@
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>08:14:14</t>
+          <t>09:23:24</t>
         </is>
       </c>
       <c r="B105" t="inlineStr">
@@ -2958,11 +2958,11 @@
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D105" t="n">
-        <v>79</v>
+        <v>10</v>
       </c>
       <c r="E105" t="inlineStr">
         <is>
@@ -3598,7 +3598,7 @@
     <row r="131">
       <c r="A131" t="inlineStr">
         <is>
-          <t>10:14:52</t>
+          <t>09:23:24</t>
         </is>
       </c>
       <c r="B131" t="inlineStr">
@@ -3608,11 +3608,11 @@
       </c>
       <c r="C131" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D131" t="n">
-        <v>29</v>
+        <v>80</v>
       </c>
       <c r="E131" t="inlineStr">
         <is>
@@ -3623,7 +3623,7 @@
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t>09:23:24</t>
+          <t>10:14:52</t>
         </is>
       </c>
       <c r="B132" t="inlineStr">
@@ -3633,11 +3633,11 @@
       </c>
       <c r="C132" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D132" t="n">
-        <v>80</v>
+        <v>29</v>
       </c>
       <c r="E132" t="inlineStr">
         <is>
@@ -3698,21 +3698,21 @@
     <row r="135">
       <c r="A135" t="inlineStr">
         <is>
-          <t>10:14:52</t>
+          <t>10:52:37</t>
         </is>
       </c>
       <c r="B135" t="inlineStr">
         <is>
-          <t>10:56</t>
+          <t>10:52</t>
         </is>
       </c>
       <c r="C135" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D135" t="n">
-        <v>42</v>
+        <v>0</v>
       </c>
       <c r="E135" t="inlineStr">
         <is>
@@ -3723,21 +3723,21 @@
     <row r="136">
       <c r="A136" t="inlineStr">
         <is>
-          <t>09:23:24</t>
+          <t>10:52:37</t>
         </is>
       </c>
       <c r="B136" t="inlineStr">
         <is>
-          <t>10:57</t>
+          <t>10:53</t>
         </is>
       </c>
       <c r="C136" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D136" t="n">
-        <v>94</v>
+        <v>1</v>
       </c>
       <c r="E136" t="inlineStr">
         <is>
@@ -3748,21 +3748,21 @@
     <row r="137">
       <c r="A137" t="inlineStr">
         <is>
-          <t>10:14:52</t>
+          <t>10:52:37</t>
         </is>
       </c>
       <c r="B137" t="inlineStr">
         <is>
-          <t>10:59</t>
+          <t>10:54</t>
         </is>
       </c>
       <c r="C137" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D137" t="n">
-        <v>45</v>
+        <v>2</v>
       </c>
       <c r="E137" t="inlineStr">
         <is>
@@ -3778,16 +3778,16 @@
       </c>
       <c r="B138" t="inlineStr">
         <is>
-          <t>11:03</t>
+          <t>10:56</t>
         </is>
       </c>
       <c r="C138" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D138" t="n">
-        <v>49</v>
+        <v>42</v>
       </c>
       <c r="E138" t="inlineStr">
         <is>
@@ -3798,21 +3798,21 @@
     <row r="139">
       <c r="A139" t="inlineStr">
         <is>
-          <t>10:14:52</t>
+          <t>09:23:24</t>
         </is>
       </c>
       <c r="B139" t="inlineStr">
         <is>
-          <t>11:04</t>
+          <t>10:57</t>
         </is>
       </c>
       <c r="C139" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D139" t="n">
-        <v>50</v>
+        <v>94</v>
       </c>
       <c r="E139" t="inlineStr">
         <is>
@@ -3828,16 +3828,16 @@
       </c>
       <c r="B140" t="inlineStr">
         <is>
-          <t>11:07</t>
+          <t>10:59</t>
         </is>
       </c>
       <c r="C140" t="inlineStr">
         <is>
-          <t>225_C ROCA-H SUR</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D140" t="n">
-        <v>53</v>
+        <v>45</v>
       </c>
       <c r="E140" t="inlineStr">
         <is>
@@ -3848,21 +3848,21 @@
     <row r="141">
       <c r="A141" t="inlineStr">
         <is>
-          <t>09:23:24</t>
+          <t>10:52:37</t>
         </is>
       </c>
       <c r="B141" t="inlineStr">
         <is>
-          <t>11:08</t>
+          <t>11:01</t>
         </is>
       </c>
       <c r="C141" t="inlineStr">
         <is>
-          <t>225_C ROCA-H SUR</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D141" t="n">
-        <v>105</v>
+        <v>9</v>
       </c>
       <c r="E141" t="inlineStr">
         <is>
@@ -3878,16 +3878,16 @@
       </c>
       <c r="B142" t="inlineStr">
         <is>
-          <t>11:18</t>
+          <t>11:03</t>
         </is>
       </c>
       <c r="C142" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D142" t="n">
-        <v>64</v>
+        <v>49</v>
       </c>
       <c r="E142" t="inlineStr">
         <is>
@@ -3898,21 +3898,21 @@
     <row r="143">
       <c r="A143" t="inlineStr">
         <is>
-          <t>09:23:24</t>
+          <t>10:52:37</t>
         </is>
       </c>
       <c r="B143" t="inlineStr">
         <is>
-          <t>11:19</t>
+          <t>11:03</t>
         </is>
       </c>
       <c r="C143" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D143" t="n">
-        <v>116</v>
+        <v>11</v>
       </c>
       <c r="E143" t="inlineStr">
         <is>
@@ -3923,21 +3923,21 @@
     <row r="144">
       <c r="A144" t="inlineStr">
         <is>
-          <t>10:14:52</t>
+          <t>10:52:37</t>
         </is>
       </c>
       <c r="B144" t="inlineStr">
         <is>
-          <t>11:20</t>
+          <t>11:04</t>
         </is>
       </c>
       <c r="C144" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D144" t="n">
-        <v>66</v>
+        <v>12</v>
       </c>
       <c r="E144" t="inlineStr">
         <is>
@@ -3953,16 +3953,16 @@
       </c>
       <c r="B145" t="inlineStr">
         <is>
-          <t>11:32</t>
+          <t>11:07</t>
         </is>
       </c>
       <c r="C145" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>225_C ROCA-H SUR</t>
         </is>
       </c>
       <c r="D145" t="n">
-        <v>78</v>
+        <v>53</v>
       </c>
       <c r="E145" t="inlineStr">
         <is>
@@ -3973,21 +3973,21 @@
     <row r="146">
       <c r="A146" t="inlineStr">
         <is>
-          <t>10:14:52</t>
+          <t>10:52:37</t>
         </is>
       </c>
       <c r="B146" t="inlineStr">
         <is>
-          <t>11:34</t>
+          <t>11:08</t>
         </is>
       </c>
       <c r="C146" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>225_C ROCA-H SUR</t>
         </is>
       </c>
       <c r="D146" t="n">
-        <v>80</v>
+        <v>16</v>
       </c>
       <c r="E146" t="inlineStr">
         <is>
@@ -3998,21 +3998,21 @@
     <row r="147">
       <c r="A147" t="inlineStr">
         <is>
-          <t>10:14:52</t>
+          <t>10:52:37</t>
         </is>
       </c>
       <c r="B147" t="inlineStr">
         <is>
-          <t>11:40</t>
+          <t>11:14</t>
         </is>
       </c>
       <c r="C147" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D147" t="n">
-        <v>86</v>
+        <v>22</v>
       </c>
       <c r="E147" t="inlineStr">
         <is>
@@ -4023,21 +4023,21 @@
     <row r="148">
       <c r="A148" t="inlineStr">
         <is>
-          <t>10:14:52</t>
+          <t>10:52:37</t>
         </is>
       </c>
       <c r="B148" t="inlineStr">
         <is>
-          <t>11:44</t>
+          <t>11:18</t>
         </is>
       </c>
       <c r="C148" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D148" t="n">
-        <v>90</v>
+        <v>26</v>
       </c>
       <c r="E148" t="inlineStr">
         <is>
@@ -4048,21 +4048,21 @@
     <row r="149">
       <c r="A149" t="inlineStr">
         <is>
-          <t>10:14:52</t>
+          <t>09:23:24</t>
         </is>
       </c>
       <c r="B149" t="inlineStr">
         <is>
-          <t>11:55</t>
+          <t>11:19</t>
         </is>
       </c>
       <c r="C149" t="inlineStr">
         <is>
-          <t>225_GOMEZ</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D149" t="n">
-        <v>101</v>
+        <v>116</v>
       </c>
       <c r="E149" t="inlineStr">
         <is>
@@ -4073,23 +4073,448 @@
     <row r="150">
       <c r="A150" t="inlineStr">
         <is>
+          <t>10:52:37</t>
+        </is>
+      </c>
+      <c r="B150" t="inlineStr">
+        <is>
+          <t>11:20</t>
+        </is>
+      </c>
+      <c r="C150" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D150" t="n">
+        <v>28</v>
+      </c>
+      <c r="E150" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="151">
+      <c r="A151" t="inlineStr">
+        <is>
           <t>10:14:52</t>
         </is>
       </c>
-      <c r="B150" t="inlineStr">
+      <c r="B151" t="inlineStr">
+        <is>
+          <t>11:32</t>
+        </is>
+      </c>
+      <c r="C151" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D151" t="n">
+        <v>78</v>
+      </c>
+      <c r="E151" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="152">
+      <c r="A152" t="inlineStr">
+        <is>
+          <t>10:52:37</t>
+        </is>
+      </c>
+      <c r="B152" t="inlineStr">
+        <is>
+          <t>11:32</t>
+        </is>
+      </c>
+      <c r="C152" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D152" t="n">
+        <v>40</v>
+      </c>
+      <c r="E152" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="153">
+      <c r="A153" t="inlineStr">
+        <is>
+          <t>10:52:37</t>
+        </is>
+      </c>
+      <c r="B153" t="inlineStr">
+        <is>
+          <t>11:33</t>
+        </is>
+      </c>
+      <c r="C153" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D153" t="n">
+        <v>41</v>
+      </c>
+      <c r="E153" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="154">
+      <c r="A154" t="inlineStr">
+        <is>
+          <t>10:52:37</t>
+        </is>
+      </c>
+      <c r="B154" t="inlineStr">
+        <is>
+          <t>11:33</t>
+        </is>
+      </c>
+      <c r="C154" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D154" t="n">
+        <v>41</v>
+      </c>
+      <c r="E154" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="155">
+      <c r="A155" t="inlineStr">
+        <is>
+          <t>10:14:52</t>
+        </is>
+      </c>
+      <c r="B155" t="inlineStr">
+        <is>
+          <t>11:34</t>
+        </is>
+      </c>
+      <c r="C155" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D155" t="n">
+        <v>80</v>
+      </c>
+      <c r="E155" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="156">
+      <c r="A156" t="inlineStr">
+        <is>
+          <t>10:14:52</t>
+        </is>
+      </c>
+      <c r="B156" t="inlineStr">
+        <is>
+          <t>11:40</t>
+        </is>
+      </c>
+      <c r="C156" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D156" t="n">
+        <v>86</v>
+      </c>
+      <c r="E156" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="157">
+      <c r="A157" t="inlineStr">
+        <is>
+          <t>10:52:37</t>
+        </is>
+      </c>
+      <c r="B157" t="inlineStr">
+        <is>
+          <t>11:41</t>
+        </is>
+      </c>
+      <c r="C157" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D157" t="n">
+        <v>49</v>
+      </c>
+      <c r="E157" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="158">
+      <c r="A158" t="inlineStr">
+        <is>
+          <t>10:52:37</t>
+        </is>
+      </c>
+      <c r="B158" t="inlineStr">
+        <is>
+          <t>11:44</t>
+        </is>
+      </c>
+      <c r="C158" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D158" t="n">
+        <v>52</v>
+      </c>
+      <c r="E158" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="159">
+      <c r="A159" t="inlineStr">
+        <is>
+          <t>10:52:37</t>
+        </is>
+      </c>
+      <c r="B159" t="inlineStr">
+        <is>
+          <t>11:49</t>
+        </is>
+      </c>
+      <c r="C159" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D159" t="n">
+        <v>57</v>
+      </c>
+      <c r="E159" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="160">
+      <c r="A160" t="inlineStr">
+        <is>
+          <t>10:14:52</t>
+        </is>
+      </c>
+      <c r="B160" t="inlineStr">
+        <is>
+          <t>11:55</t>
+        </is>
+      </c>
+      <c r="C160" t="inlineStr">
+        <is>
+          <t>225_GOMEZ</t>
+        </is>
+      </c>
+      <c r="D160" t="n">
+        <v>101</v>
+      </c>
+      <c r="E160" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="161">
+      <c r="A161" t="inlineStr">
+        <is>
+          <t>10:52:37</t>
+        </is>
+      </c>
+      <c r="B161" t="inlineStr">
+        <is>
+          <t>11:56</t>
+        </is>
+      </c>
+      <c r="C161" t="inlineStr">
+        <is>
+          <t>225_GOMEZ</t>
+        </is>
+      </c>
+      <c r="D161" t="n">
+        <v>64</v>
+      </c>
+      <c r="E161" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="162">
+      <c r="A162" t="inlineStr">
+        <is>
+          <t>10:52:37</t>
+        </is>
+      </c>
+      <c r="B162" t="inlineStr">
         <is>
           <t>12:04</t>
         </is>
       </c>
-      <c r="C150" t="inlineStr">
+      <c r="C162" t="inlineStr">
         <is>
           <t>17_ROMERO</t>
         </is>
       </c>
-      <c r="D150" t="n">
-        <v>110</v>
-      </c>
-      <c r="E150" t="inlineStr">
+      <c r="D162" t="n">
+        <v>72</v>
+      </c>
+      <c r="E162" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="163">
+      <c r="A163" t="inlineStr">
+        <is>
+          <t>10:52:37</t>
+        </is>
+      </c>
+      <c r="B163" t="inlineStr">
+        <is>
+          <t>12:08</t>
+        </is>
+      </c>
+      <c r="C163" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D163" t="n">
+        <v>76</v>
+      </c>
+      <c r="E163" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="164">
+      <c r="A164" t="inlineStr">
+        <is>
+          <t>10:52:37</t>
+        </is>
+      </c>
+      <c r="B164" t="inlineStr">
+        <is>
+          <t>12:20</t>
+        </is>
+      </c>
+      <c r="C164" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D164" t="n">
+        <v>88</v>
+      </c>
+      <c r="E164" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="165">
+      <c r="A165" t="inlineStr">
+        <is>
+          <t>10:52:37</t>
+        </is>
+      </c>
+      <c r="B165" t="inlineStr">
+        <is>
+          <t>12:32</t>
+        </is>
+      </c>
+      <c r="C165" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D165" t="n">
+        <v>100</v>
+      </c>
+      <c r="E165" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="166">
+      <c r="A166" t="inlineStr">
+        <is>
+          <t>10:52:37</t>
+        </is>
+      </c>
+      <c r="B166" t="inlineStr">
+        <is>
+          <t>12:33</t>
+        </is>
+      </c>
+      <c r="C166" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D166" t="n">
+        <v>101</v>
+      </c>
+      <c r="E166" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="167">
+      <c r="A167" t="inlineStr">
+        <is>
+          <t>10:52:37</t>
+        </is>
+      </c>
+      <c r="B167" t="inlineStr">
+        <is>
+          <t>12:51</t>
+        </is>
+      </c>
+      <c r="C167" t="inlineStr">
+        <is>
+          <t>16_P MOR-SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D167" t="n">
+        <v>119</v>
+      </c>
+      <c r="E167" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -4106,7 +4531,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E30"/>
+  <dimension ref="A1:E32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4119,14 +4544,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 10:14:52</t>
+          <t>Última actualización: 10:52:37</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 25</t>
+          <t>Total filas: 27</t>
         </is>
       </c>
     </row>
@@ -4685,7 +5110,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>10:14:52</t>
+          <t>10:52:37</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -4699,7 +5124,7 @@
         </is>
       </c>
       <c r="D27" t="n">
-        <v>64</v>
+        <v>26</v>
       </c>
       <c r="E27" t="inlineStr">
         <is>
@@ -4760,23 +5185,73 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>10:14:52</t>
+          <t>10:52:37</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
+          <t>11:33</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D30" t="n">
+        <v>41</v>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>10:52:37</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
           <t>11:44</t>
         </is>
       </c>
-      <c r="C30" t="inlineStr">
+      <c r="C31" t="inlineStr">
         <is>
           <t>215B_EL PATO</t>
         </is>
       </c>
-      <c r="D30" t="n">
-        <v>90</v>
-      </c>
-      <c r="E30" t="inlineStr">
+      <c r="D31" t="n">
+        <v>52</v>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>10:52:37</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>12:33</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D32" t="n">
+        <v>101</v>
+      </c>
+      <c r="E32" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -4806,7 +5281,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 10:14:52</t>
+          <t>Última actualización: 10:52:37</t>
         </is>
       </c>
     </row>
@@ -5497,7 +5972,7 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>10:14:52</t>
+          <t>10:52:37</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -5511,7 +5986,7 @@
         </is>
       </c>
       <c r="D32" t="n">
-        <v>101</v>
+        <v>63</v>
       </c>
       <c r="E32" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 1803
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-03-21.xlsx
+++ b/data/horarios-141-2026-03-21.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E167"/>
+  <dimension ref="A1:E176"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 10:52:37</t>
+          <t>Última actualización: 11:16:36</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 162</t>
+          <t>Total filas: 171</t>
         </is>
       </c>
     </row>
@@ -1158,7 +1158,7 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D33" t="n">
@@ -1183,7 +1183,7 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D34" t="n">
@@ -1558,7 +1558,7 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D49" t="n">
@@ -1583,7 +1583,7 @@
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D50" t="n">
@@ -1883,7 +1883,7 @@
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D62" t="n">
@@ -1933,7 +1933,7 @@
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D64" t="n">
@@ -1998,7 +1998,7 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>07:51:37</t>
+          <t>07:27:35</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
@@ -2008,11 +2008,11 @@
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D67" t="n">
-        <v>28</v>
+        <v>52</v>
       </c>
       <c r="E67" t="inlineStr">
         <is>
@@ -2023,7 +2023,7 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>07:27:35</t>
+          <t>07:51:37</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
@@ -2033,11 +2033,11 @@
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D68" t="n">
-        <v>52</v>
+        <v>28</v>
       </c>
       <c r="E68" t="inlineStr">
         <is>
@@ -2233,7 +2233,7 @@
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D76" t="n">
@@ -2258,7 +2258,7 @@
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D77" t="n">
@@ -2383,7 +2383,7 @@
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D82" t="n">
@@ -2408,7 +2408,7 @@
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D83" t="n">
@@ -2708,7 +2708,7 @@
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215_EL PELIGRO</t>
         </is>
       </c>
       <c r="D95" t="n">
@@ -2733,7 +2733,7 @@
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>215_EL PELIGRO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D96" t="n">
@@ -2873,7 +2873,7 @@
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>08:36:09</t>
+          <t>07:51:37</t>
         </is>
       </c>
       <c r="B102" t="inlineStr">
@@ -2883,11 +2883,11 @@
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D102" t="n">
-        <v>53</v>
+        <v>98</v>
       </c>
       <c r="E102" t="inlineStr">
         <is>
@@ -2898,7 +2898,7 @@
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>07:51:37</t>
+          <t>08:36:09</t>
         </is>
       </c>
       <c r="B103" t="inlineStr">
@@ -2908,11 +2908,11 @@
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D103" t="n">
-        <v>98</v>
+        <v>53</v>
       </c>
       <c r="E103" t="inlineStr">
         <is>
@@ -3498,7 +3498,7 @@
     <row r="127">
       <c r="A127" t="inlineStr">
         <is>
-          <t>08:36:09</t>
+          <t>10:14:52</t>
         </is>
       </c>
       <c r="B127" t="inlineStr">
@@ -3508,11 +3508,11 @@
       </c>
       <c r="C127" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D127" t="n">
-        <v>117</v>
+        <v>19</v>
       </c>
       <c r="E127" t="inlineStr">
         <is>
@@ -3523,7 +3523,7 @@
     <row r="128">
       <c r="A128" t="inlineStr">
         <is>
-          <t>10:14:52</t>
+          <t>08:36:09</t>
         </is>
       </c>
       <c r="B128" t="inlineStr">
@@ -3533,11 +3533,11 @@
       </c>
       <c r="C128" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D128" t="n">
-        <v>19</v>
+        <v>117</v>
       </c>
       <c r="E128" t="inlineStr">
         <is>
@@ -3873,7 +3873,7 @@
     <row r="142">
       <c r="A142" t="inlineStr">
         <is>
-          <t>10:14:52</t>
+          <t>10:52:37</t>
         </is>
       </c>
       <c r="B142" t="inlineStr">
@@ -3883,11 +3883,11 @@
       </c>
       <c r="C142" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D142" t="n">
-        <v>49</v>
+        <v>11</v>
       </c>
       <c r="E142" t="inlineStr">
         <is>
@@ -3898,7 +3898,7 @@
     <row r="143">
       <c r="A143" t="inlineStr">
         <is>
-          <t>10:52:37</t>
+          <t>10:14:52</t>
         </is>
       </c>
       <c r="B143" t="inlineStr">
@@ -3908,11 +3908,11 @@
       </c>
       <c r="C143" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D143" t="n">
-        <v>11</v>
+        <v>49</v>
       </c>
       <c r="E143" t="inlineStr">
         <is>
@@ -4023,21 +4023,21 @@
     <row r="148">
       <c r="A148" t="inlineStr">
         <is>
-          <t>10:52:37</t>
+          <t>11:16:36</t>
         </is>
       </c>
       <c r="B148" t="inlineStr">
         <is>
-          <t>11:18</t>
+          <t>11:17</t>
         </is>
       </c>
       <c r="C148" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D148" t="n">
-        <v>26</v>
+        <v>1</v>
       </c>
       <c r="E148" t="inlineStr">
         <is>
@@ -4048,12 +4048,12 @@
     <row r="149">
       <c r="A149" t="inlineStr">
         <is>
-          <t>09:23:24</t>
+          <t>10:52:37</t>
         </is>
       </c>
       <c r="B149" t="inlineStr">
         <is>
-          <t>11:19</t>
+          <t>11:18</t>
         </is>
       </c>
       <c r="C149" t="inlineStr">
@@ -4062,7 +4062,7 @@
         </is>
       </c>
       <c r="D149" t="n">
-        <v>116</v>
+        <v>26</v>
       </c>
       <c r="E149" t="inlineStr">
         <is>
@@ -4073,21 +4073,21 @@
     <row r="150">
       <c r="A150" t="inlineStr">
         <is>
-          <t>10:52:37</t>
+          <t>09:23:24</t>
         </is>
       </c>
       <c r="B150" t="inlineStr">
         <is>
-          <t>11:20</t>
+          <t>11:19</t>
         </is>
       </c>
       <c r="C150" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D150" t="n">
-        <v>28</v>
+        <v>116</v>
       </c>
       <c r="E150" t="inlineStr">
         <is>
@@ -4098,21 +4098,21 @@
     <row r="151">
       <c r="A151" t="inlineStr">
         <is>
-          <t>10:14:52</t>
+          <t>11:16:36</t>
         </is>
       </c>
       <c r="B151" t="inlineStr">
         <is>
-          <t>11:32</t>
+          <t>11:20</t>
         </is>
       </c>
       <c r="C151" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D151" t="n">
-        <v>78</v>
+        <v>4</v>
       </c>
       <c r="E151" t="inlineStr">
         <is>
@@ -4123,7 +4123,7 @@
     <row r="152">
       <c r="A152" t="inlineStr">
         <is>
-          <t>10:52:37</t>
+          <t>11:16:36</t>
         </is>
       </c>
       <c r="B152" t="inlineStr">
@@ -4137,7 +4137,7 @@
         </is>
       </c>
       <c r="D152" t="n">
-        <v>40</v>
+        <v>16</v>
       </c>
       <c r="E152" t="inlineStr">
         <is>
@@ -4148,21 +4148,21 @@
     <row r="153">
       <c r="A153" t="inlineStr">
         <is>
-          <t>10:52:37</t>
+          <t>10:14:52</t>
         </is>
       </c>
       <c r="B153" t="inlineStr">
         <is>
-          <t>11:33</t>
+          <t>11:32</t>
         </is>
       </c>
       <c r="C153" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D153" t="n">
-        <v>41</v>
+        <v>78</v>
       </c>
       <c r="E153" t="inlineStr">
         <is>
@@ -4173,7 +4173,7 @@
     <row r="154">
       <c r="A154" t="inlineStr">
         <is>
-          <t>10:52:37</t>
+          <t>11:16:36</t>
         </is>
       </c>
       <c r="B154" t="inlineStr">
@@ -4187,7 +4187,7 @@
         </is>
       </c>
       <c r="D154" t="n">
-        <v>41</v>
+        <v>17</v>
       </c>
       <c r="E154" t="inlineStr">
         <is>
@@ -4198,21 +4198,21 @@
     <row r="155">
       <c r="A155" t="inlineStr">
         <is>
-          <t>10:14:52</t>
+          <t>11:16:36</t>
         </is>
       </c>
       <c r="B155" t="inlineStr">
         <is>
-          <t>11:34</t>
+          <t>11:33</t>
         </is>
       </c>
       <c r="C155" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D155" t="n">
-        <v>80</v>
+        <v>17</v>
       </c>
       <c r="E155" t="inlineStr">
         <is>
@@ -4228,16 +4228,16 @@
       </c>
       <c r="B156" t="inlineStr">
         <is>
-          <t>11:40</t>
+          <t>11:34</t>
         </is>
       </c>
       <c r="C156" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D156" t="n">
-        <v>86</v>
+        <v>80</v>
       </c>
       <c r="E156" t="inlineStr">
         <is>
@@ -4248,21 +4248,21 @@
     <row r="157">
       <c r="A157" t="inlineStr">
         <is>
-          <t>10:52:37</t>
+          <t>10:14:52</t>
         </is>
       </c>
       <c r="B157" t="inlineStr">
         <is>
-          <t>11:41</t>
+          <t>11:40</t>
         </is>
       </c>
       <c r="C157" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D157" t="n">
-        <v>49</v>
+        <v>86</v>
       </c>
       <c r="E157" t="inlineStr">
         <is>
@@ -4273,21 +4273,21 @@
     <row r="158">
       <c r="A158" t="inlineStr">
         <is>
-          <t>10:52:37</t>
+          <t>11:16:36</t>
         </is>
       </c>
       <c r="B158" t="inlineStr">
         <is>
-          <t>11:44</t>
+          <t>11:41</t>
         </is>
       </c>
       <c r="C158" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D158" t="n">
-        <v>52</v>
+        <v>25</v>
       </c>
       <c r="E158" t="inlineStr">
         <is>
@@ -4298,21 +4298,21 @@
     <row r="159">
       <c r="A159" t="inlineStr">
         <is>
-          <t>10:52:37</t>
+          <t>11:16:36</t>
         </is>
       </c>
       <c r="B159" t="inlineStr">
         <is>
-          <t>11:49</t>
+          <t>11:44</t>
         </is>
       </c>
       <c r="C159" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D159" t="n">
-        <v>57</v>
+        <v>28</v>
       </c>
       <c r="E159" t="inlineStr">
         <is>
@@ -4323,21 +4323,21 @@
     <row r="160">
       <c r="A160" t="inlineStr">
         <is>
-          <t>10:14:52</t>
+          <t>11:16:36</t>
         </is>
       </c>
       <c r="B160" t="inlineStr">
         <is>
-          <t>11:55</t>
+          <t>11:49</t>
         </is>
       </c>
       <c r="C160" t="inlineStr">
         <is>
-          <t>225_GOMEZ</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D160" t="n">
-        <v>101</v>
+        <v>33</v>
       </c>
       <c r="E160" t="inlineStr">
         <is>
@@ -4348,21 +4348,21 @@
     <row r="161">
       <c r="A161" t="inlineStr">
         <is>
-          <t>10:52:37</t>
+          <t>11:16:36</t>
         </is>
       </c>
       <c r="B161" t="inlineStr">
         <is>
-          <t>11:56</t>
+          <t>11:51</t>
         </is>
       </c>
       <c r="C161" t="inlineStr">
         <is>
-          <t>225_GOMEZ</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D161" t="n">
-        <v>64</v>
+        <v>35</v>
       </c>
       <c r="E161" t="inlineStr">
         <is>
@@ -4373,21 +4373,21 @@
     <row r="162">
       <c r="A162" t="inlineStr">
         <is>
-          <t>10:52:37</t>
+          <t>10:14:52</t>
         </is>
       </c>
       <c r="B162" t="inlineStr">
         <is>
-          <t>12:04</t>
+          <t>11:55</t>
         </is>
       </c>
       <c r="C162" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>225_GOMEZ</t>
         </is>
       </c>
       <c r="D162" t="n">
-        <v>72</v>
+        <v>101</v>
       </c>
       <c r="E162" t="inlineStr">
         <is>
@@ -4398,21 +4398,21 @@
     <row r="163">
       <c r="A163" t="inlineStr">
         <is>
-          <t>10:52:37</t>
+          <t>11:16:36</t>
         </is>
       </c>
       <c r="B163" t="inlineStr">
         <is>
-          <t>12:08</t>
+          <t>11:56</t>
         </is>
       </c>
       <c r="C163" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>225_GOMEZ</t>
         </is>
       </c>
       <c r="D163" t="n">
-        <v>76</v>
+        <v>40</v>
       </c>
       <c r="E163" t="inlineStr">
         <is>
@@ -4423,21 +4423,21 @@
     <row r="164">
       <c r="A164" t="inlineStr">
         <is>
-          <t>10:52:37</t>
+          <t>11:16:36</t>
         </is>
       </c>
       <c r="B164" t="inlineStr">
         <is>
-          <t>12:20</t>
+          <t>12:04</t>
         </is>
       </c>
       <c r="C164" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D164" t="n">
-        <v>88</v>
+        <v>48</v>
       </c>
       <c r="E164" t="inlineStr">
         <is>
@@ -4448,21 +4448,21 @@
     <row r="165">
       <c r="A165" t="inlineStr">
         <is>
-          <t>10:52:37</t>
+          <t>11:16:36</t>
         </is>
       </c>
       <c r="B165" t="inlineStr">
         <is>
-          <t>12:32</t>
+          <t>12:04</t>
         </is>
       </c>
       <c r="C165" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D165" t="n">
-        <v>100</v>
+        <v>48</v>
       </c>
       <c r="E165" t="inlineStr">
         <is>
@@ -4473,21 +4473,21 @@
     <row r="166">
       <c r="A166" t="inlineStr">
         <is>
-          <t>10:52:37</t>
+          <t>11:16:36</t>
         </is>
       </c>
       <c r="B166" t="inlineStr">
         <is>
-          <t>12:33</t>
+          <t>12:08</t>
         </is>
       </c>
       <c r="C166" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D166" t="n">
-        <v>101</v>
+        <v>52</v>
       </c>
       <c r="E166" t="inlineStr">
         <is>
@@ -4498,23 +4498,248 @@
     <row r="167">
       <c r="A167" t="inlineStr">
         <is>
+          <t>11:16:36</t>
+        </is>
+      </c>
+      <c r="B167" t="inlineStr">
+        <is>
+          <t>12:19</t>
+        </is>
+      </c>
+      <c r="C167" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D167" t="n">
+        <v>63</v>
+      </c>
+      <c r="E167" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="168">
+      <c r="A168" t="inlineStr">
+        <is>
+          <t>11:16:36</t>
+        </is>
+      </c>
+      <c r="B168" t="inlineStr">
+        <is>
+          <t>12:20</t>
+        </is>
+      </c>
+      <c r="C168" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D168" t="n">
+        <v>64</v>
+      </c>
+      <c r="E168" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="169">
+      <c r="A169" t="inlineStr">
+        <is>
+          <t>11:16:36</t>
+        </is>
+      </c>
+      <c r="B169" t="inlineStr">
+        <is>
+          <t>12:21</t>
+        </is>
+      </c>
+      <c r="C169" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D169" t="n">
+        <v>65</v>
+      </c>
+      <c r="E169" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="170">
+      <c r="A170" t="inlineStr">
+        <is>
+          <t>11:16:36</t>
+        </is>
+      </c>
+      <c r="B170" t="inlineStr">
+        <is>
+          <t>12:32</t>
+        </is>
+      </c>
+      <c r="C170" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D170" t="n">
+        <v>76</v>
+      </c>
+      <c r="E170" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="171">
+      <c r="A171" t="inlineStr">
+        <is>
           <t>10:52:37</t>
         </is>
       </c>
-      <c r="B167" t="inlineStr">
+      <c r="B171" t="inlineStr">
+        <is>
+          <t>12:33</t>
+        </is>
+      </c>
+      <c r="C171" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D171" t="n">
+        <v>101</v>
+      </c>
+      <c r="E171" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="172">
+      <c r="A172" t="inlineStr">
+        <is>
+          <t>11:16:36</t>
+        </is>
+      </c>
+      <c r="B172" t="inlineStr">
+        <is>
+          <t>12:34</t>
+        </is>
+      </c>
+      <c r="C172" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D172" t="n">
+        <v>78</v>
+      </c>
+      <c r="E172" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="173">
+      <c r="A173" t="inlineStr">
+        <is>
+          <t>11:16:36</t>
+        </is>
+      </c>
+      <c r="B173" t="inlineStr">
         <is>
           <t>12:51</t>
         </is>
       </c>
-      <c r="C167" t="inlineStr">
+      <c r="C173" t="inlineStr">
         <is>
           <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
-      <c r="D167" t="n">
-        <v>119</v>
-      </c>
-      <c r="E167" t="inlineStr">
+      <c r="D173" t="n">
+        <v>95</v>
+      </c>
+      <c r="E173" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="174">
+      <c r="A174" t="inlineStr">
+        <is>
+          <t>11:16:36</t>
+        </is>
+      </c>
+      <c r="B174" t="inlineStr">
+        <is>
+          <t>12:57</t>
+        </is>
+      </c>
+      <c r="C174" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D174" t="n">
+        <v>101</v>
+      </c>
+      <c r="E174" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="175">
+      <c r="A175" t="inlineStr">
+        <is>
+          <t>11:16:36</t>
+        </is>
+      </c>
+      <c r="B175" t="inlineStr">
+        <is>
+          <t>13:02</t>
+        </is>
+      </c>
+      <c r="C175" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D175" t="n">
+        <v>106</v>
+      </c>
+      <c r="E175" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="176">
+      <c r="A176" t="inlineStr">
+        <is>
+          <t>11:16:36</t>
+        </is>
+      </c>
+      <c r="B176" t="inlineStr">
+        <is>
+          <t>13:04</t>
+        </is>
+      </c>
+      <c r="C176" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D176" t="n">
+        <v>108</v>
+      </c>
+      <c r="E176" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -4531,7 +4756,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E32"/>
+  <dimension ref="A1:E34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4544,14 +4769,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 10:52:37</t>
+          <t>Última actualización: 11:16:36</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 27</t>
+          <t>Total filas: 29</t>
         </is>
       </c>
     </row>
@@ -5185,7 +5410,7 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>10:52:37</t>
+          <t>11:16:36</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -5199,7 +5424,7 @@
         </is>
       </c>
       <c r="D30" t="n">
-        <v>41</v>
+        <v>17</v>
       </c>
       <c r="E30" t="inlineStr">
         <is>
@@ -5210,7 +5435,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>10:52:37</t>
+          <t>11:16:36</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -5224,7 +5449,7 @@
         </is>
       </c>
       <c r="D31" t="n">
-        <v>52</v>
+        <v>28</v>
       </c>
       <c r="E31" t="inlineStr">
         <is>
@@ -5252,6 +5477,56 @@
         <v>101</v>
       </c>
       <c r="E32" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>11:16:36</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>12:34</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D33" t="n">
+        <v>78</v>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>11:16:36</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>13:04</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D34" t="n">
+        <v>108</v>
+      </c>
+      <c r="E34" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -5268,7 +5543,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E32"/>
+  <dimension ref="A1:E34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5281,14 +5556,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 10:52:37</t>
+          <t>Última actualización: 11:16:36</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 27</t>
+          <t>Total filas: 29</t>
         </is>
       </c>
     </row>
@@ -5972,7 +6247,7 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>10:52:37</t>
+          <t>11:16:36</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -5986,11 +6261,61 @@
         </is>
       </c>
       <c r="D32" t="n">
-        <v>63</v>
+        <v>39</v>
       </c>
       <c r="E32" t="inlineStr">
         <is>
           <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>11:16:36</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>12:55</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D33" t="n">
+        <v>99</v>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>11:16:36</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>13:11</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>215A_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D34" t="n">
+        <v>115</v>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>L6173</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 1804
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-03-21.xlsx
+++ b/data/horarios-141-2026-03-21.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E176"/>
+  <dimension ref="A1:E185"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 11:16:36</t>
+          <t>Última actualización: 11:46:24</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 171</t>
+          <t>Total filas: 180</t>
         </is>
       </c>
     </row>
@@ -1158,7 +1158,7 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D33" t="n">
@@ -1183,7 +1183,7 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D34" t="n">
@@ -1558,7 +1558,7 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D49" t="n">
@@ -1583,7 +1583,7 @@
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D50" t="n">
@@ -1883,7 +1883,7 @@
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D62" t="n">
@@ -1898,7 +1898,7 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>06:59:30</t>
+          <t>08:14:14</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
@@ -1908,11 +1908,11 @@
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D63" t="n">
-        <v>75</v>
+        <v>0</v>
       </c>
       <c r="E63" t="inlineStr">
         <is>
@@ -1923,7 +1923,7 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>08:14:14</t>
+          <t>06:59:30</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
@@ -1933,11 +1933,11 @@
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D64" t="n">
-        <v>0</v>
+        <v>75</v>
       </c>
       <c r="E64" t="inlineStr">
         <is>
@@ -1983,7 +1983,7 @@
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D66" t="n">
@@ -1998,7 +1998,7 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>07:27:35</t>
+          <t>07:51:37</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
@@ -2008,11 +2008,11 @@
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D67" t="n">
-        <v>52</v>
+        <v>28</v>
       </c>
       <c r="E67" t="inlineStr">
         <is>
@@ -2023,7 +2023,7 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>07:51:37</t>
+          <t>07:27:35</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
@@ -2033,11 +2033,11 @@
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D68" t="n">
-        <v>28</v>
+        <v>52</v>
       </c>
       <c r="E68" t="inlineStr">
         <is>
@@ -2233,7 +2233,7 @@
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D76" t="n">
@@ -2258,7 +2258,7 @@
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D77" t="n">
@@ -2708,7 +2708,7 @@
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>215_EL PELIGRO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D95" t="n">
@@ -2733,7 +2733,7 @@
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215_EL PELIGRO</t>
         </is>
       </c>
       <c r="D96" t="n">
@@ -2873,7 +2873,7 @@
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>07:51:37</t>
+          <t>08:36:09</t>
         </is>
       </c>
       <c r="B102" t="inlineStr">
@@ -2883,11 +2883,11 @@
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D102" t="n">
-        <v>98</v>
+        <v>53</v>
       </c>
       <c r="E102" t="inlineStr">
         <is>
@@ -2898,7 +2898,7 @@
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>08:36:09</t>
+          <t>07:51:37</t>
         </is>
       </c>
       <c r="B103" t="inlineStr">
@@ -2908,11 +2908,11 @@
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D103" t="n">
-        <v>53</v>
+        <v>98</v>
       </c>
       <c r="E103" t="inlineStr">
         <is>
@@ -2923,7 +2923,7 @@
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>08:14:14</t>
+          <t>09:23:24</t>
         </is>
       </c>
       <c r="B104" t="inlineStr">
@@ -2933,11 +2933,11 @@
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D104" t="n">
-        <v>79</v>
+        <v>10</v>
       </c>
       <c r="E104" t="inlineStr">
         <is>
@@ -2948,7 +2948,7 @@
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>09:23:24</t>
+          <t>08:14:14</t>
         </is>
       </c>
       <c r="B105" t="inlineStr">
@@ -2958,11 +2958,11 @@
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D105" t="n">
-        <v>10</v>
+        <v>79</v>
       </c>
       <c r="E105" t="inlineStr">
         <is>
@@ -3598,7 +3598,7 @@
     <row r="131">
       <c r="A131" t="inlineStr">
         <is>
-          <t>09:23:24</t>
+          <t>10:14:52</t>
         </is>
       </c>
       <c r="B131" t="inlineStr">
@@ -3608,11 +3608,11 @@
       </c>
       <c r="C131" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D131" t="n">
-        <v>80</v>
+        <v>29</v>
       </c>
       <c r="E131" t="inlineStr">
         <is>
@@ -3623,7 +3623,7 @@
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t>10:14:52</t>
+          <t>09:23:24</t>
         </is>
       </c>
       <c r="B132" t="inlineStr">
@@ -3633,11 +3633,11 @@
       </c>
       <c r="C132" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D132" t="n">
-        <v>29</v>
+        <v>80</v>
       </c>
       <c r="E132" t="inlineStr">
         <is>
@@ -4123,7 +4123,7 @@
     <row r="152">
       <c r="A152" t="inlineStr">
         <is>
-          <t>11:16:36</t>
+          <t>10:14:52</t>
         </is>
       </c>
       <c r="B152" t="inlineStr">
@@ -4133,11 +4133,11 @@
       </c>
       <c r="C152" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D152" t="n">
-        <v>16</v>
+        <v>78</v>
       </c>
       <c r="E152" t="inlineStr">
         <is>
@@ -4148,7 +4148,7 @@
     <row r="153">
       <c r="A153" t="inlineStr">
         <is>
-          <t>10:14:52</t>
+          <t>11:16:36</t>
         </is>
       </c>
       <c r="B153" t="inlineStr">
@@ -4158,11 +4158,11 @@
       </c>
       <c r="C153" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D153" t="n">
-        <v>78</v>
+        <v>16</v>
       </c>
       <c r="E153" t="inlineStr">
         <is>
@@ -4183,7 +4183,7 @@
       </c>
       <c r="C154" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D154" t="n">
@@ -4208,7 +4208,7 @@
       </c>
       <c r="C155" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D155" t="n">
@@ -4323,7 +4323,7 @@
     <row r="160">
       <c r="A160" t="inlineStr">
         <is>
-          <t>11:16:36</t>
+          <t>11:46:24</t>
         </is>
       </c>
       <c r="B160" t="inlineStr">
@@ -4337,7 +4337,7 @@
         </is>
       </c>
       <c r="D160" t="n">
-        <v>33</v>
+        <v>3</v>
       </c>
       <c r="E160" t="inlineStr">
         <is>
@@ -4348,7 +4348,7 @@
     <row r="161">
       <c r="A161" t="inlineStr">
         <is>
-          <t>11:16:36</t>
+          <t>11:46:24</t>
         </is>
       </c>
       <c r="B161" t="inlineStr">
@@ -4362,7 +4362,7 @@
         </is>
       </c>
       <c r="D161" t="n">
-        <v>35</v>
+        <v>5</v>
       </c>
       <c r="E161" t="inlineStr">
         <is>
@@ -4398,7 +4398,7 @@
     <row r="163">
       <c r="A163" t="inlineStr">
         <is>
-          <t>11:16:36</t>
+          <t>11:46:24</t>
         </is>
       </c>
       <c r="B163" t="inlineStr">
@@ -4412,7 +4412,7 @@
         </is>
       </c>
       <c r="D163" t="n">
-        <v>40</v>
+        <v>10</v>
       </c>
       <c r="E163" t="inlineStr">
         <is>
@@ -4423,12 +4423,12 @@
     <row r="164">
       <c r="A164" t="inlineStr">
         <is>
-          <t>11:16:36</t>
+          <t>11:46:24</t>
         </is>
       </c>
       <c r="B164" t="inlineStr">
         <is>
-          <t>12:04</t>
+          <t>12:03</t>
         </is>
       </c>
       <c r="C164" t="inlineStr">
@@ -4437,7 +4437,7 @@
         </is>
       </c>
       <c r="D164" t="n">
-        <v>48</v>
+        <v>17</v>
       </c>
       <c r="E164" t="inlineStr">
         <is>
@@ -4458,7 +4458,7 @@
       </c>
       <c r="C165" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D165" t="n">
@@ -4473,21 +4473,21 @@
     <row r="166">
       <c r="A166" t="inlineStr">
         <is>
-          <t>11:16:36</t>
+          <t>11:46:24</t>
         </is>
       </c>
       <c r="B166" t="inlineStr">
         <is>
-          <t>12:08</t>
+          <t>12:04</t>
         </is>
       </c>
       <c r="C166" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D166" t="n">
-        <v>52</v>
+        <v>18</v>
       </c>
       <c r="E166" t="inlineStr">
         <is>
@@ -4503,16 +4503,16 @@
       </c>
       <c r="B167" t="inlineStr">
         <is>
-          <t>12:19</t>
+          <t>12:08</t>
         </is>
       </c>
       <c r="C167" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D167" t="n">
-        <v>63</v>
+        <v>52</v>
       </c>
       <c r="E167" t="inlineStr">
         <is>
@@ -4523,21 +4523,21 @@
     <row r="168">
       <c r="A168" t="inlineStr">
         <is>
-          <t>11:16:36</t>
+          <t>11:46:24</t>
         </is>
       </c>
       <c r="B168" t="inlineStr">
         <is>
-          <t>12:20</t>
+          <t>12:19</t>
         </is>
       </c>
       <c r="C168" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D168" t="n">
-        <v>64</v>
+        <v>33</v>
       </c>
       <c r="E168" t="inlineStr">
         <is>
@@ -4548,21 +4548,21 @@
     <row r="169">
       <c r="A169" t="inlineStr">
         <is>
-          <t>11:16:36</t>
+          <t>11:46:24</t>
         </is>
       </c>
       <c r="B169" t="inlineStr">
         <is>
-          <t>12:21</t>
+          <t>12:20</t>
         </is>
       </c>
       <c r="C169" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D169" t="n">
-        <v>65</v>
+        <v>34</v>
       </c>
       <c r="E169" t="inlineStr">
         <is>
@@ -4573,21 +4573,21 @@
     <row r="170">
       <c r="A170" t="inlineStr">
         <is>
-          <t>11:16:36</t>
+          <t>11:46:24</t>
         </is>
       </c>
       <c r="B170" t="inlineStr">
         <is>
-          <t>12:32</t>
+          <t>12:21</t>
         </is>
       </c>
       <c r="C170" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D170" t="n">
-        <v>76</v>
+        <v>35</v>
       </c>
       <c r="E170" t="inlineStr">
         <is>
@@ -4598,21 +4598,21 @@
     <row r="171">
       <c r="A171" t="inlineStr">
         <is>
-          <t>10:52:37</t>
+          <t>11:46:24</t>
         </is>
       </c>
       <c r="B171" t="inlineStr">
         <is>
-          <t>12:33</t>
+          <t>12:32</t>
         </is>
       </c>
       <c r="C171" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D171" t="n">
-        <v>101</v>
+        <v>46</v>
       </c>
       <c r="E171" t="inlineStr">
         <is>
@@ -4623,12 +4623,12 @@
     <row r="172">
       <c r="A172" t="inlineStr">
         <is>
-          <t>11:16:36</t>
+          <t>10:52:37</t>
         </is>
       </c>
       <c r="B172" t="inlineStr">
         <is>
-          <t>12:34</t>
+          <t>12:33</t>
         </is>
       </c>
       <c r="C172" t="inlineStr">
@@ -4637,7 +4637,7 @@
         </is>
       </c>
       <c r="D172" t="n">
-        <v>78</v>
+        <v>101</v>
       </c>
       <c r="E172" t="inlineStr">
         <is>
@@ -4648,21 +4648,21 @@
     <row r="173">
       <c r="A173" t="inlineStr">
         <is>
-          <t>11:16:36</t>
+          <t>11:46:24</t>
         </is>
       </c>
       <c r="B173" t="inlineStr">
         <is>
-          <t>12:51</t>
+          <t>12:34</t>
         </is>
       </c>
       <c r="C173" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D173" t="n">
-        <v>95</v>
+        <v>48</v>
       </c>
       <c r="E173" t="inlineStr">
         <is>
@@ -4673,12 +4673,12 @@
     <row r="174">
       <c r="A174" t="inlineStr">
         <is>
-          <t>11:16:36</t>
+          <t>11:46:24</t>
         </is>
       </c>
       <c r="B174" t="inlineStr">
         <is>
-          <t>12:57</t>
+          <t>12:37</t>
         </is>
       </c>
       <c r="C174" t="inlineStr">
@@ -4687,7 +4687,7 @@
         </is>
       </c>
       <c r="D174" t="n">
-        <v>101</v>
+        <v>51</v>
       </c>
       <c r="E174" t="inlineStr">
         <is>
@@ -4698,21 +4698,21 @@
     <row r="175">
       <c r="A175" t="inlineStr">
         <is>
-          <t>11:16:36</t>
+          <t>11:46:24</t>
         </is>
       </c>
       <c r="B175" t="inlineStr">
         <is>
-          <t>13:02</t>
+          <t>12:47</t>
         </is>
       </c>
       <c r="C175" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D175" t="n">
-        <v>106</v>
+        <v>61</v>
       </c>
       <c r="E175" t="inlineStr">
         <is>
@@ -4723,23 +4723,248 @@
     <row r="176">
       <c r="A176" t="inlineStr">
         <is>
+          <t>11:46:24</t>
+        </is>
+      </c>
+      <c r="B176" t="inlineStr">
+        <is>
+          <t>12:51</t>
+        </is>
+      </c>
+      <c r="C176" t="inlineStr">
+        <is>
+          <t>16_P MOR-SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D176" t="n">
+        <v>65</v>
+      </c>
+      <c r="E176" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="177">
+      <c r="A177" t="inlineStr">
+        <is>
           <t>11:16:36</t>
         </is>
       </c>
-      <c r="B176" t="inlineStr">
+      <c r="B177" t="inlineStr">
+        <is>
+          <t>12:57</t>
+        </is>
+      </c>
+      <c r="C177" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D177" t="n">
+        <v>101</v>
+      </c>
+      <c r="E177" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="178">
+      <c r="A178" t="inlineStr">
+        <is>
+          <t>11:46:24</t>
+        </is>
+      </c>
+      <c r="B178" t="inlineStr">
+        <is>
+          <t>13:02</t>
+        </is>
+      </c>
+      <c r="C178" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D178" t="n">
+        <v>76</v>
+      </c>
+      <c r="E178" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="179">
+      <c r="A179" t="inlineStr">
+        <is>
+          <t>11:46:24</t>
+        </is>
+      </c>
+      <c r="B179" t="inlineStr">
+        <is>
+          <t>13:03</t>
+        </is>
+      </c>
+      <c r="C179" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D179" t="n">
+        <v>77</v>
+      </c>
+      <c r="E179" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="180">
+      <c r="A180" t="inlineStr">
+        <is>
+          <t>11:46:24</t>
+        </is>
+      </c>
+      <c r="B180" t="inlineStr">
         <is>
           <t>13:04</t>
         </is>
       </c>
-      <c r="C176" t="inlineStr">
+      <c r="C180" t="inlineStr">
         <is>
           <t>215C_EL PATO</t>
         </is>
       </c>
-      <c r="D176" t="n">
-        <v>108</v>
-      </c>
-      <c r="E176" t="inlineStr">
+      <c r="D180" t="n">
+        <v>78</v>
+      </c>
+      <c r="E180" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="181">
+      <c r="A181" t="inlineStr">
+        <is>
+          <t>11:46:24</t>
+        </is>
+      </c>
+      <c r="B181" t="inlineStr">
+        <is>
+          <t>13:17</t>
+        </is>
+      </c>
+      <c r="C181" t="inlineStr">
+        <is>
+          <t>11X44_P_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D181" t="n">
+        <v>91</v>
+      </c>
+      <c r="E181" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="182">
+      <c r="A182" t="inlineStr">
+        <is>
+          <t>11:46:24</t>
+        </is>
+      </c>
+      <c r="B182" t="inlineStr">
+        <is>
+          <t>13:19</t>
+        </is>
+      </c>
+      <c r="C182" t="inlineStr">
+        <is>
+          <t>215_ALUAR</t>
+        </is>
+      </c>
+      <c r="D182" t="n">
+        <v>93</v>
+      </c>
+      <c r="E182" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="183">
+      <c r="A183" t="inlineStr">
+        <is>
+          <t>11:46:24</t>
+        </is>
+      </c>
+      <c r="B183" t="inlineStr">
+        <is>
+          <t>13:32</t>
+        </is>
+      </c>
+      <c r="C183" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D183" t="n">
+        <v>106</v>
+      </c>
+      <c r="E183" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="184">
+      <c r="A184" t="inlineStr">
+        <is>
+          <t>11:46:24</t>
+        </is>
+      </c>
+      <c r="B184" t="inlineStr">
+        <is>
+          <t>13:38</t>
+        </is>
+      </c>
+      <c r="C184" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D184" t="n">
+        <v>112</v>
+      </c>
+      <c r="E184" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="185">
+      <c r="A185" t="inlineStr">
+        <is>
+          <t>11:46:24</t>
+        </is>
+      </c>
+      <c r="B185" t="inlineStr">
+        <is>
+          <t>13:41</t>
+        </is>
+      </c>
+      <c r="C185" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D185" t="n">
+        <v>115</v>
+      </c>
+      <c r="E185" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -4756,7 +4981,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E34"/>
+  <dimension ref="A1:E36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4769,14 +4994,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 11:16:36</t>
+          <t>Última actualización: 11:46:24</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 29</t>
+          <t>Total filas: 31</t>
         </is>
       </c>
     </row>
@@ -5485,7 +5710,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>11:16:36</t>
+          <t>11:46:24</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -5499,7 +5724,7 @@
         </is>
       </c>
       <c r="D33" t="n">
-        <v>78</v>
+        <v>48</v>
       </c>
       <c r="E33" t="inlineStr">
         <is>
@@ -5510,7 +5735,7 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>11:16:36</t>
+          <t>11:46:24</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -5524,9 +5749,59 @@
         </is>
       </c>
       <c r="D34" t="n">
-        <v>108</v>
+        <v>78</v>
       </c>
       <c r="E34" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>11:46:24</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>13:19</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>215_ALUAR</t>
+        </is>
+      </c>
+      <c r="D35" t="n">
+        <v>93</v>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>11:46:24</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>13:38</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D36" t="n">
+        <v>112</v>
+      </c>
+      <c r="E36" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -5543,7 +5818,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E34"/>
+  <dimension ref="A1:E37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5556,14 +5831,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 11:16:36</t>
+          <t>Última actualización: 11:46:24</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 29</t>
+          <t>Total filas: 32</t>
         </is>
       </c>
     </row>
@@ -6272,12 +6547,12 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>11:16:36</t>
+          <t>11:46:24</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>12:55</t>
+          <t>11:56</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
@@ -6286,7 +6561,7 @@
         </is>
       </c>
       <c r="D33" t="n">
-        <v>99</v>
+        <v>10</v>
       </c>
       <c r="E33" t="inlineStr">
         <is>
@@ -6302,18 +6577,93 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
+          <t>12:55</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D34" t="n">
+        <v>99</v>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>11:46:24</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>12:56</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D35" t="n">
+        <v>70</v>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>11:46:24</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
           <t>13:11</t>
         </is>
       </c>
-      <c r="C34" t="inlineStr">
+      <c r="C36" t="inlineStr">
         <is>
           <t>215A_LA PLATA</t>
         </is>
       </c>
-      <c r="D34" t="n">
-        <v>115</v>
-      </c>
-      <c r="E34" t="inlineStr">
+      <c r="D36" t="n">
+        <v>85</v>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>11:46:24</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>13:22</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>215B_LP-P MOR-1 Y 57</t>
+        </is>
+      </c>
+      <c r="D37" t="n">
+        <v>96</v>
+      </c>
+      <c r="E37" t="inlineStr">
         <is>
           <t>L6173</t>
         </is>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 1805
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-03-21.xlsx
+++ b/data/horarios-141-2026-03-21.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E185"/>
+  <dimension ref="A1:E194"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 11:46:24</t>
+          <t>Última actualización: 12:00:15</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 180</t>
+          <t>Total filas: 189</t>
         </is>
       </c>
     </row>
@@ -758,7 +758,7 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D17" t="n">
@@ -783,7 +783,7 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D18" t="n">
@@ -1558,7 +1558,7 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D49" t="n">
@@ -1583,7 +1583,7 @@
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D50" t="n">
@@ -1898,7 +1898,7 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>08:14:14</t>
+          <t>06:59:30</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
@@ -1908,11 +1908,11 @@
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D63" t="n">
-        <v>0</v>
+        <v>75</v>
       </c>
       <c r="E63" t="inlineStr">
         <is>
@@ -1923,7 +1923,7 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>06:59:30</t>
+          <t>08:14:14</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
@@ -1933,11 +1933,11 @@
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D64" t="n">
-        <v>75</v>
+        <v>0</v>
       </c>
       <c r="E64" t="inlineStr">
         <is>
@@ -2373,7 +2373,7 @@
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>08:50:55</t>
+          <t>07:27:35</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
@@ -2383,11 +2383,11 @@
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D82" t="n">
-        <v>1</v>
+        <v>84</v>
       </c>
       <c r="E82" t="inlineStr">
         <is>
@@ -2423,7 +2423,7 @@
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>07:27:35</t>
+          <t>08:50:55</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
@@ -2433,11 +2433,11 @@
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D84" t="n">
-        <v>84</v>
+        <v>1</v>
       </c>
       <c r="E84" t="inlineStr">
         <is>
@@ -2698,7 +2698,7 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>08:50:55</t>
+          <t>08:14:14</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
@@ -2708,11 +2708,11 @@
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D95" t="n">
-        <v>28</v>
+        <v>64</v>
       </c>
       <c r="E95" t="inlineStr">
         <is>
@@ -2733,7 +2733,7 @@
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>215_EL PELIGRO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D96" t="n">
@@ -2748,7 +2748,7 @@
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>08:14:14</t>
+          <t>08:50:55</t>
         </is>
       </c>
       <c r="B97" t="inlineStr">
@@ -2758,11 +2758,11 @@
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>215_EL PELIGRO</t>
         </is>
       </c>
       <c r="D97" t="n">
-        <v>64</v>
+        <v>28</v>
       </c>
       <c r="E97" t="inlineStr">
         <is>
@@ -2873,7 +2873,7 @@
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>08:36:09</t>
+          <t>07:51:37</t>
         </is>
       </c>
       <c r="B102" t="inlineStr">
@@ -2883,11 +2883,11 @@
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D102" t="n">
-        <v>53</v>
+        <v>98</v>
       </c>
       <c r="E102" t="inlineStr">
         <is>
@@ -2898,7 +2898,7 @@
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>07:51:37</t>
+          <t>08:36:09</t>
         </is>
       </c>
       <c r="B103" t="inlineStr">
@@ -2908,11 +2908,11 @@
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D103" t="n">
-        <v>98</v>
+        <v>53</v>
       </c>
       <c r="E103" t="inlineStr">
         <is>
@@ -2923,7 +2923,7 @@
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>09:23:24</t>
+          <t>08:14:14</t>
         </is>
       </c>
       <c r="B104" t="inlineStr">
@@ -2933,11 +2933,11 @@
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D104" t="n">
-        <v>10</v>
+        <v>79</v>
       </c>
       <c r="E104" t="inlineStr">
         <is>
@@ -2948,7 +2948,7 @@
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>08:14:14</t>
+          <t>09:23:24</t>
         </is>
       </c>
       <c r="B105" t="inlineStr">
@@ -2958,11 +2958,11 @@
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D105" t="n">
-        <v>79</v>
+        <v>10</v>
       </c>
       <c r="E105" t="inlineStr">
         <is>
@@ -3173,7 +3173,7 @@
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>09:23:24</t>
+          <t>08:50:55</t>
         </is>
       </c>
       <c r="B114" t="inlineStr">
@@ -3183,11 +3183,11 @@
       </c>
       <c r="C114" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D114" t="n">
-        <v>40</v>
+        <v>73</v>
       </c>
       <c r="E114" t="inlineStr">
         <is>
@@ -3198,7 +3198,7 @@
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>08:50:55</t>
+          <t>09:23:24</t>
         </is>
       </c>
       <c r="B115" t="inlineStr">
@@ -3208,11 +3208,11 @@
       </c>
       <c r="C115" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D115" t="n">
-        <v>73</v>
+        <v>40</v>
       </c>
       <c r="E115" t="inlineStr">
         <is>
@@ -3498,7 +3498,7 @@
     <row r="127">
       <c r="A127" t="inlineStr">
         <is>
-          <t>10:14:52</t>
+          <t>08:36:09</t>
         </is>
       </c>
       <c r="B127" t="inlineStr">
@@ -3508,11 +3508,11 @@
       </c>
       <c r="C127" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D127" t="n">
-        <v>19</v>
+        <v>117</v>
       </c>
       <c r="E127" t="inlineStr">
         <is>
@@ -3523,7 +3523,7 @@
     <row r="128">
       <c r="A128" t="inlineStr">
         <is>
-          <t>08:36:09</t>
+          <t>10:14:52</t>
         </is>
       </c>
       <c r="B128" t="inlineStr">
@@ -3533,11 +3533,11 @@
       </c>
       <c r="C128" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D128" t="n">
-        <v>117</v>
+        <v>19</v>
       </c>
       <c r="E128" t="inlineStr">
         <is>
@@ -3873,7 +3873,7 @@
     <row r="142">
       <c r="A142" t="inlineStr">
         <is>
-          <t>10:52:37</t>
+          <t>10:14:52</t>
         </is>
       </c>
       <c r="B142" t="inlineStr">
@@ -3883,11 +3883,11 @@
       </c>
       <c r="C142" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D142" t="n">
-        <v>11</v>
+        <v>49</v>
       </c>
       <c r="E142" t="inlineStr">
         <is>
@@ -3898,7 +3898,7 @@
     <row r="143">
       <c r="A143" t="inlineStr">
         <is>
-          <t>10:14:52</t>
+          <t>10:52:37</t>
         </is>
       </c>
       <c r="B143" t="inlineStr">
@@ -3908,11 +3908,11 @@
       </c>
       <c r="C143" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D143" t="n">
-        <v>49</v>
+        <v>11</v>
       </c>
       <c r="E143" t="inlineStr">
         <is>
@@ -4423,21 +4423,21 @@
     <row r="164">
       <c r="A164" t="inlineStr">
         <is>
-          <t>11:46:24</t>
+          <t>12:00:15</t>
         </is>
       </c>
       <c r="B164" t="inlineStr">
         <is>
-          <t>12:03</t>
+          <t>12:01</t>
         </is>
       </c>
       <c r="C164" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D164" t="n">
-        <v>17</v>
+        <v>1</v>
       </c>
       <c r="E164" t="inlineStr">
         <is>
@@ -4448,12 +4448,12 @@
     <row r="165">
       <c r="A165" t="inlineStr">
         <is>
-          <t>11:16:36</t>
+          <t>12:00:15</t>
         </is>
       </c>
       <c r="B165" t="inlineStr">
         <is>
-          <t>12:04</t>
+          <t>12:03</t>
         </is>
       </c>
       <c r="C165" t="inlineStr">
@@ -4462,7 +4462,7 @@
         </is>
       </c>
       <c r="D165" t="n">
-        <v>48</v>
+        <v>3</v>
       </c>
       <c r="E165" t="inlineStr">
         <is>
@@ -4473,7 +4473,7 @@
     <row r="166">
       <c r="A166" t="inlineStr">
         <is>
-          <t>11:46:24</t>
+          <t>11:16:36</t>
         </is>
       </c>
       <c r="B166" t="inlineStr">
@@ -4483,11 +4483,11 @@
       </c>
       <c r="C166" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D166" t="n">
-        <v>18</v>
+        <v>48</v>
       </c>
       <c r="E166" t="inlineStr">
         <is>
@@ -4498,21 +4498,21 @@
     <row r="167">
       <c r="A167" t="inlineStr">
         <is>
-          <t>11:16:36</t>
+          <t>12:00:15</t>
         </is>
       </c>
       <c r="B167" t="inlineStr">
         <is>
-          <t>12:08</t>
+          <t>12:04</t>
         </is>
       </c>
       <c r="C167" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D167" t="n">
-        <v>52</v>
+        <v>4</v>
       </c>
       <c r="E167" t="inlineStr">
         <is>
@@ -4523,21 +4523,21 @@
     <row r="168">
       <c r="A168" t="inlineStr">
         <is>
-          <t>11:46:24</t>
+          <t>11:16:36</t>
         </is>
       </c>
       <c r="B168" t="inlineStr">
         <is>
-          <t>12:19</t>
+          <t>12:08</t>
         </is>
       </c>
       <c r="C168" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D168" t="n">
-        <v>33</v>
+        <v>52</v>
       </c>
       <c r="E168" t="inlineStr">
         <is>
@@ -4548,21 +4548,21 @@
     <row r="169">
       <c r="A169" t="inlineStr">
         <is>
-          <t>11:46:24</t>
+          <t>12:00:15</t>
         </is>
       </c>
       <c r="B169" t="inlineStr">
         <is>
-          <t>12:20</t>
+          <t>12:19</t>
         </is>
       </c>
       <c r="C169" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D169" t="n">
-        <v>34</v>
+        <v>19</v>
       </c>
       <c r="E169" t="inlineStr">
         <is>
@@ -4573,21 +4573,21 @@
     <row r="170">
       <c r="A170" t="inlineStr">
         <is>
-          <t>11:46:24</t>
+          <t>12:00:15</t>
         </is>
       </c>
       <c r="B170" t="inlineStr">
         <is>
-          <t>12:21</t>
+          <t>12:20</t>
         </is>
       </c>
       <c r="C170" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D170" t="n">
-        <v>35</v>
+        <v>20</v>
       </c>
       <c r="E170" t="inlineStr">
         <is>
@@ -4598,21 +4598,21 @@
     <row r="171">
       <c r="A171" t="inlineStr">
         <is>
-          <t>11:46:24</t>
+          <t>12:00:15</t>
         </is>
       </c>
       <c r="B171" t="inlineStr">
         <is>
-          <t>12:32</t>
+          <t>12:21</t>
         </is>
       </c>
       <c r="C171" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D171" t="n">
-        <v>46</v>
+        <v>21</v>
       </c>
       <c r="E171" t="inlineStr">
         <is>
@@ -4623,21 +4623,21 @@
     <row r="172">
       <c r="A172" t="inlineStr">
         <is>
-          <t>10:52:37</t>
+          <t>11:46:24</t>
         </is>
       </c>
       <c r="B172" t="inlineStr">
         <is>
-          <t>12:33</t>
+          <t>12:32</t>
         </is>
       </c>
       <c r="C172" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D172" t="n">
-        <v>101</v>
+        <v>46</v>
       </c>
       <c r="E172" t="inlineStr">
         <is>
@@ -4648,12 +4648,12 @@
     <row r="173">
       <c r="A173" t="inlineStr">
         <is>
-          <t>11:46:24</t>
+          <t>10:52:37</t>
         </is>
       </c>
       <c r="B173" t="inlineStr">
         <is>
-          <t>12:34</t>
+          <t>12:33</t>
         </is>
       </c>
       <c r="C173" t="inlineStr">
@@ -4662,7 +4662,7 @@
         </is>
       </c>
       <c r="D173" t="n">
-        <v>48</v>
+        <v>101</v>
       </c>
       <c r="E173" t="inlineStr">
         <is>
@@ -4673,21 +4673,21 @@
     <row r="174">
       <c r="A174" t="inlineStr">
         <is>
-          <t>11:46:24</t>
+          <t>12:00:15</t>
         </is>
       </c>
       <c r="B174" t="inlineStr">
         <is>
-          <t>12:37</t>
+          <t>12:33</t>
         </is>
       </c>
       <c r="C174" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D174" t="n">
-        <v>51</v>
+        <v>33</v>
       </c>
       <c r="E174" t="inlineStr">
         <is>
@@ -4698,21 +4698,21 @@
     <row r="175">
       <c r="A175" t="inlineStr">
         <is>
-          <t>11:46:24</t>
+          <t>12:00:15</t>
         </is>
       </c>
       <c r="B175" t="inlineStr">
         <is>
-          <t>12:47</t>
+          <t>12:34</t>
         </is>
       </c>
       <c r="C175" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D175" t="n">
-        <v>61</v>
+        <v>34</v>
       </c>
       <c r="E175" t="inlineStr">
         <is>
@@ -4723,21 +4723,21 @@
     <row r="176">
       <c r="A176" t="inlineStr">
         <is>
-          <t>11:46:24</t>
+          <t>12:00:15</t>
         </is>
       </c>
       <c r="B176" t="inlineStr">
         <is>
-          <t>12:51</t>
+          <t>12:37</t>
         </is>
       </c>
       <c r="C176" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D176" t="n">
-        <v>65</v>
+        <v>37</v>
       </c>
       <c r="E176" t="inlineStr">
         <is>
@@ -4748,21 +4748,21 @@
     <row r="177">
       <c r="A177" t="inlineStr">
         <is>
-          <t>11:16:36</t>
+          <t>12:00:15</t>
         </is>
       </c>
       <c r="B177" t="inlineStr">
         <is>
-          <t>12:57</t>
+          <t>12:47</t>
         </is>
       </c>
       <c r="C177" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D177" t="n">
-        <v>101</v>
+        <v>47</v>
       </c>
       <c r="E177" t="inlineStr">
         <is>
@@ -4773,21 +4773,21 @@
     <row r="178">
       <c r="A178" t="inlineStr">
         <is>
-          <t>11:46:24</t>
+          <t>12:00:15</t>
         </is>
       </c>
       <c r="B178" t="inlineStr">
         <is>
-          <t>13:02</t>
+          <t>12:49</t>
         </is>
       </c>
       <c r="C178" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D178" t="n">
-        <v>76</v>
+        <v>49</v>
       </c>
       <c r="E178" t="inlineStr">
         <is>
@@ -4798,21 +4798,21 @@
     <row r="179">
       <c r="A179" t="inlineStr">
         <is>
-          <t>11:46:24</t>
+          <t>12:00:15</t>
         </is>
       </c>
       <c r="B179" t="inlineStr">
         <is>
-          <t>13:03</t>
+          <t>12:51</t>
         </is>
       </c>
       <c r="C179" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D179" t="n">
-        <v>77</v>
+        <v>51</v>
       </c>
       <c r="E179" t="inlineStr">
         <is>
@@ -4823,21 +4823,21 @@
     <row r="180">
       <c r="A180" t="inlineStr">
         <is>
-          <t>11:46:24</t>
+          <t>11:16:36</t>
         </is>
       </c>
       <c r="B180" t="inlineStr">
         <is>
-          <t>13:04</t>
+          <t>12:57</t>
         </is>
       </c>
       <c r="C180" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D180" t="n">
-        <v>78</v>
+        <v>101</v>
       </c>
       <c r="E180" t="inlineStr">
         <is>
@@ -4853,16 +4853,16 @@
       </c>
       <c r="B181" t="inlineStr">
         <is>
-          <t>13:17</t>
+          <t>13:02</t>
         </is>
       </c>
       <c r="C181" t="inlineStr">
         <is>
-          <t>11X44_P_ETCHEVERRY</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D181" t="n">
-        <v>91</v>
+        <v>76</v>
       </c>
       <c r="E181" t="inlineStr">
         <is>
@@ -4878,16 +4878,16 @@
       </c>
       <c r="B182" t="inlineStr">
         <is>
-          <t>13:19</t>
+          <t>13:03</t>
         </is>
       </c>
       <c r="C182" t="inlineStr">
         <is>
-          <t>215_ALUAR</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D182" t="n">
-        <v>93</v>
+        <v>77</v>
       </c>
       <c r="E182" t="inlineStr">
         <is>
@@ -4898,12 +4898,12 @@
     <row r="183">
       <c r="A183" t="inlineStr">
         <is>
-          <t>11:46:24</t>
+          <t>12:00:15</t>
         </is>
       </c>
       <c r="B183" t="inlineStr">
         <is>
-          <t>13:32</t>
+          <t>13:03</t>
         </is>
       </c>
       <c r="C183" t="inlineStr">
@@ -4912,7 +4912,7 @@
         </is>
       </c>
       <c r="D183" t="n">
-        <v>106</v>
+        <v>63</v>
       </c>
       <c r="E183" t="inlineStr">
         <is>
@@ -4923,21 +4923,21 @@
     <row r="184">
       <c r="A184" t="inlineStr">
         <is>
-          <t>11:46:24</t>
+          <t>12:00:15</t>
         </is>
       </c>
       <c r="B184" t="inlineStr">
         <is>
-          <t>13:38</t>
+          <t>13:04</t>
         </is>
       </c>
       <c r="C184" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D184" t="n">
-        <v>112</v>
+        <v>64</v>
       </c>
       <c r="E184" t="inlineStr">
         <is>
@@ -4948,23 +4948,248 @@
     <row r="185">
       <c r="A185" t="inlineStr">
         <is>
+          <t>12:00:15</t>
+        </is>
+      </c>
+      <c r="B185" t="inlineStr">
+        <is>
+          <t>13:04</t>
+        </is>
+      </c>
+      <c r="C185" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D185" t="n">
+        <v>64</v>
+      </c>
+      <c r="E185" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="186">
+      <c r="A186" t="inlineStr">
+        <is>
+          <t>12:00:15</t>
+        </is>
+      </c>
+      <c r="B186" t="inlineStr">
+        <is>
+          <t>13:17</t>
+        </is>
+      </c>
+      <c r="C186" t="inlineStr">
+        <is>
+          <t>11X44_P_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D186" t="n">
+        <v>77</v>
+      </c>
+      <c r="E186" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="187">
+      <c r="A187" t="inlineStr">
+        <is>
+          <t>12:00:15</t>
+        </is>
+      </c>
+      <c r="B187" t="inlineStr">
+        <is>
+          <t>13:19</t>
+        </is>
+      </c>
+      <c r="C187" t="inlineStr">
+        <is>
+          <t>215_ALUAR</t>
+        </is>
+      </c>
+      <c r="D187" t="n">
+        <v>79</v>
+      </c>
+      <c r="E187" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="188">
+      <c r="A188" t="inlineStr">
+        <is>
           <t>11:46:24</t>
         </is>
       </c>
-      <c r="B185" t="inlineStr">
+      <c r="B188" t="inlineStr">
+        <is>
+          <t>13:32</t>
+        </is>
+      </c>
+      <c r="C188" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D188" t="n">
+        <v>106</v>
+      </c>
+      <c r="E188" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="189">
+      <c r="A189" t="inlineStr">
+        <is>
+          <t>12:00:15</t>
+        </is>
+      </c>
+      <c r="B189" t="inlineStr">
+        <is>
+          <t>13:33</t>
+        </is>
+      </c>
+      <c r="C189" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D189" t="n">
+        <v>93</v>
+      </c>
+      <c r="E189" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="190">
+      <c r="A190" t="inlineStr">
+        <is>
+          <t>12:00:15</t>
+        </is>
+      </c>
+      <c r="B190" t="inlineStr">
+        <is>
+          <t>13:38</t>
+        </is>
+      </c>
+      <c r="C190" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D190" t="n">
+        <v>98</v>
+      </c>
+      <c r="E190" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="191">
+      <c r="A191" t="inlineStr">
+        <is>
+          <t>11:46:24</t>
+        </is>
+      </c>
+      <c r="B191" t="inlineStr">
         <is>
           <t>13:41</t>
         </is>
       </c>
-      <c r="C185" t="inlineStr">
+      <c r="C191" t="inlineStr">
         <is>
           <t>16_SANTA ANA</t>
         </is>
       </c>
-      <c r="D185" t="n">
+      <c r="D191" t="n">
         <v>115</v>
       </c>
-      <c r="E185" t="inlineStr">
+      <c r="E191" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="192">
+      <c r="A192" t="inlineStr">
+        <is>
+          <t>12:00:15</t>
+        </is>
+      </c>
+      <c r="B192" t="inlineStr">
+        <is>
+          <t>13:47</t>
+        </is>
+      </c>
+      <c r="C192" t="inlineStr">
+        <is>
+          <t>225_GOMEZ</t>
+        </is>
+      </c>
+      <c r="D192" t="n">
+        <v>107</v>
+      </c>
+      <c r="E192" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="193">
+      <c r="A193" t="inlineStr">
+        <is>
+          <t>12:00:15</t>
+        </is>
+      </c>
+      <c r="B193" t="inlineStr">
+        <is>
+          <t>13:51</t>
+        </is>
+      </c>
+      <c r="C193" t="inlineStr">
+        <is>
+          <t>16_P MOR-SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D193" t="n">
+        <v>111</v>
+      </c>
+      <c r="E193" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="194">
+      <c r="A194" t="inlineStr">
+        <is>
+          <t>12:00:15</t>
+        </is>
+      </c>
+      <c r="B194" t="inlineStr">
+        <is>
+          <t>13:59</t>
+        </is>
+      </c>
+      <c r="C194" t="inlineStr">
+        <is>
+          <t>17_ROMERO</t>
+        </is>
+      </c>
+      <c r="D194" t="n">
+        <v>119</v>
+      </c>
+      <c r="E194" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -4994,7 +5219,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 11:46:24</t>
+          <t>Última actualización: 12:00:15</t>
         </is>
       </c>
     </row>
@@ -5710,7 +5935,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>11:46:24</t>
+          <t>12:00:15</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -5724,7 +5949,7 @@
         </is>
       </c>
       <c r="D33" t="n">
-        <v>48</v>
+        <v>34</v>
       </c>
       <c r="E33" t="inlineStr">
         <is>
@@ -5735,7 +5960,7 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>11:46:24</t>
+          <t>12:00:15</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -5749,7 +5974,7 @@
         </is>
       </c>
       <c r="D34" t="n">
-        <v>78</v>
+        <v>64</v>
       </c>
       <c r="E34" t="inlineStr">
         <is>
@@ -5760,7 +5985,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>11:46:24</t>
+          <t>12:00:15</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -5774,7 +5999,7 @@
         </is>
       </c>
       <c r="D35" t="n">
-        <v>93</v>
+        <v>79</v>
       </c>
       <c r="E35" t="inlineStr">
         <is>
@@ -5785,7 +6010,7 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>11:46:24</t>
+          <t>12:00:15</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
@@ -5799,7 +6024,7 @@
         </is>
       </c>
       <c r="D36" t="n">
-        <v>112</v>
+        <v>98</v>
       </c>
       <c r="E36" t="inlineStr">
         <is>
@@ -5818,7 +6043,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E37"/>
+  <dimension ref="A1:E38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5831,14 +6056,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 11:46:24</t>
+          <t>Última actualización: 12:00:15</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 32</t>
+          <t>Total filas: 33</t>
         </is>
       </c>
     </row>
@@ -6597,7 +6822,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>11:46:24</t>
+          <t>12:00:15</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -6611,7 +6836,7 @@
         </is>
       </c>
       <c r="D35" t="n">
-        <v>70</v>
+        <v>56</v>
       </c>
       <c r="E35" t="inlineStr">
         <is>
@@ -6622,7 +6847,7 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>11:46:24</t>
+          <t>12:00:15</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
@@ -6636,7 +6861,7 @@
         </is>
       </c>
       <c r="D36" t="n">
-        <v>85</v>
+        <v>71</v>
       </c>
       <c r="E36" t="inlineStr">
         <is>
@@ -6647,7 +6872,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>11:46:24</t>
+          <t>12:00:15</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -6661,11 +6886,36 @@
         </is>
       </c>
       <c r="D37" t="n">
-        <v>96</v>
+        <v>82</v>
       </c>
       <c r="E37" t="inlineStr">
         <is>
           <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>12:00:15</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>13:56</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D38" t="n">
+        <v>116</v>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>L6203</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 1806
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-03-21.xlsx
+++ b/data/horarios-141-2026-03-21.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E194"/>
+  <dimension ref="A1:E202"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 12:00:15</t>
+          <t>Última actualización: 12:28:38</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 189</t>
+          <t>Total filas: 197</t>
         </is>
       </c>
     </row>
@@ -758,7 +758,7 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D17" t="n">
@@ -783,7 +783,7 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D18" t="n">
@@ -1558,7 +1558,7 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D49" t="n">
@@ -1583,7 +1583,7 @@
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D50" t="n">
@@ -1983,7 +1983,7 @@
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D66" t="n">
@@ -1998,7 +1998,7 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>07:51:37</t>
+          <t>07:27:35</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
@@ -2008,11 +2008,11 @@
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D67" t="n">
-        <v>28</v>
+        <v>52</v>
       </c>
       <c r="E67" t="inlineStr">
         <is>
@@ -2023,7 +2023,7 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>07:27:35</t>
+          <t>07:51:37</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
@@ -2033,11 +2033,11 @@
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D68" t="n">
-        <v>52</v>
+        <v>28</v>
       </c>
       <c r="E68" t="inlineStr">
         <is>
@@ -2233,7 +2233,7 @@
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D76" t="n">
@@ -2258,7 +2258,7 @@
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D77" t="n">
@@ -2373,7 +2373,7 @@
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>07:27:35</t>
+          <t>08:50:55</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
@@ -2383,11 +2383,11 @@
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D82" t="n">
-        <v>84</v>
+        <v>1</v>
       </c>
       <c r="E82" t="inlineStr">
         <is>
@@ -2398,7 +2398,7 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>08:50:55</t>
+          <t>07:27:35</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
@@ -2408,11 +2408,11 @@
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D83" t="n">
-        <v>1</v>
+        <v>84</v>
       </c>
       <c r="E83" t="inlineStr">
         <is>
@@ -2433,7 +2433,7 @@
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D84" t="n">
@@ -2733,7 +2733,7 @@
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215_EL PELIGRO</t>
         </is>
       </c>
       <c r="D96" t="n">
@@ -2758,7 +2758,7 @@
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>215_EL PELIGRO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D97" t="n">
@@ -2923,7 +2923,7 @@
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>08:14:14</t>
+          <t>09:23:24</t>
         </is>
       </c>
       <c r="B104" t="inlineStr">
@@ -2933,11 +2933,11 @@
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D104" t="n">
-        <v>79</v>
+        <v>10</v>
       </c>
       <c r="E104" t="inlineStr">
         <is>
@@ -2948,7 +2948,7 @@
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>09:23:24</t>
+          <t>08:14:14</t>
         </is>
       </c>
       <c r="B105" t="inlineStr">
@@ -2958,11 +2958,11 @@
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D105" t="n">
-        <v>10</v>
+        <v>79</v>
       </c>
       <c r="E105" t="inlineStr">
         <is>
@@ -3083,7 +3083,7 @@
       </c>
       <c r="C110" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D110" t="n">
@@ -3108,7 +3108,7 @@
       </c>
       <c r="C111" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D111" t="n">
@@ -3598,7 +3598,7 @@
     <row r="131">
       <c r="A131" t="inlineStr">
         <is>
-          <t>10:14:52</t>
+          <t>09:23:24</t>
         </is>
       </c>
       <c r="B131" t="inlineStr">
@@ -3608,11 +3608,11 @@
       </c>
       <c r="C131" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D131" t="n">
-        <v>29</v>
+        <v>80</v>
       </c>
       <c r="E131" t="inlineStr">
         <is>
@@ -3623,7 +3623,7 @@
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t>09:23:24</t>
+          <t>10:14:52</t>
         </is>
       </c>
       <c r="B132" t="inlineStr">
@@ -3633,11 +3633,11 @@
       </c>
       <c r="C132" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D132" t="n">
-        <v>80</v>
+        <v>29</v>
       </c>
       <c r="E132" t="inlineStr">
         <is>
@@ -3873,7 +3873,7 @@
     <row r="142">
       <c r="A142" t="inlineStr">
         <is>
-          <t>10:14:52</t>
+          <t>10:52:37</t>
         </is>
       </c>
       <c r="B142" t="inlineStr">
@@ -3883,11 +3883,11 @@
       </c>
       <c r="C142" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D142" t="n">
-        <v>49</v>
+        <v>11</v>
       </c>
       <c r="E142" t="inlineStr">
         <is>
@@ -3898,7 +3898,7 @@
     <row r="143">
       <c r="A143" t="inlineStr">
         <is>
-          <t>10:52:37</t>
+          <t>10:14:52</t>
         </is>
       </c>
       <c r="B143" t="inlineStr">
@@ -3908,11 +3908,11 @@
       </c>
       <c r="C143" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D143" t="n">
-        <v>11</v>
+        <v>49</v>
       </c>
       <c r="E143" t="inlineStr">
         <is>
@@ -4183,7 +4183,7 @@
       </c>
       <c r="C154" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D154" t="n">
@@ -4208,7 +4208,7 @@
       </c>
       <c r="C155" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D155" t="n">
@@ -4473,7 +4473,7 @@
     <row r="166">
       <c r="A166" t="inlineStr">
         <is>
-          <t>11:16:36</t>
+          <t>12:00:15</t>
         </is>
       </c>
       <c r="B166" t="inlineStr">
@@ -4483,11 +4483,11 @@
       </c>
       <c r="C166" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D166" t="n">
-        <v>48</v>
+        <v>4</v>
       </c>
       <c r="E166" t="inlineStr">
         <is>
@@ -4498,7 +4498,7 @@
     <row r="167">
       <c r="A167" t="inlineStr">
         <is>
-          <t>12:00:15</t>
+          <t>11:16:36</t>
         </is>
       </c>
       <c r="B167" t="inlineStr">
@@ -4508,11 +4508,11 @@
       </c>
       <c r="C167" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D167" t="n">
-        <v>4</v>
+        <v>48</v>
       </c>
       <c r="E167" t="inlineStr">
         <is>
@@ -4623,7 +4623,7 @@
     <row r="172">
       <c r="A172" t="inlineStr">
         <is>
-          <t>11:46:24</t>
+          <t>12:28:38</t>
         </is>
       </c>
       <c r="B172" t="inlineStr">
@@ -4637,7 +4637,7 @@
         </is>
       </c>
       <c r="D172" t="n">
-        <v>46</v>
+        <v>4</v>
       </c>
       <c r="E172" t="inlineStr">
         <is>
@@ -4648,7 +4648,7 @@
     <row r="173">
       <c r="A173" t="inlineStr">
         <is>
-          <t>10:52:37</t>
+          <t>12:28:38</t>
         </is>
       </c>
       <c r="B173" t="inlineStr">
@@ -4662,7 +4662,7 @@
         </is>
       </c>
       <c r="D173" t="n">
-        <v>101</v>
+        <v>5</v>
       </c>
       <c r="E173" t="inlineStr">
         <is>
@@ -4673,7 +4673,7 @@
     <row r="174">
       <c r="A174" t="inlineStr">
         <is>
-          <t>12:00:15</t>
+          <t>12:28:38</t>
         </is>
       </c>
       <c r="B174" t="inlineStr">
@@ -4683,11 +4683,11 @@
       </c>
       <c r="C174" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D174" t="n">
-        <v>33</v>
+        <v>5</v>
       </c>
       <c r="E174" t="inlineStr">
         <is>
@@ -4703,16 +4703,16 @@
       </c>
       <c r="B175" t="inlineStr">
         <is>
-          <t>12:34</t>
+          <t>12:33</t>
         </is>
       </c>
       <c r="C175" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D175" t="n">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="E175" t="inlineStr">
         <is>
@@ -4728,16 +4728,16 @@
       </c>
       <c r="B176" t="inlineStr">
         <is>
-          <t>12:37</t>
+          <t>12:34</t>
         </is>
       </c>
       <c r="C176" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D176" t="n">
-        <v>37</v>
+        <v>34</v>
       </c>
       <c r="E176" t="inlineStr">
         <is>
@@ -4748,21 +4748,21 @@
     <row r="177">
       <c r="A177" t="inlineStr">
         <is>
-          <t>12:00:15</t>
+          <t>12:28:38</t>
         </is>
       </c>
       <c r="B177" t="inlineStr">
         <is>
-          <t>12:47</t>
+          <t>12:36</t>
         </is>
       </c>
       <c r="C177" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D177" t="n">
-        <v>47</v>
+        <v>8</v>
       </c>
       <c r="E177" t="inlineStr">
         <is>
@@ -4778,16 +4778,16 @@
       </c>
       <c r="B178" t="inlineStr">
         <is>
-          <t>12:49</t>
+          <t>12:37</t>
         </is>
       </c>
       <c r="C178" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D178" t="n">
-        <v>49</v>
+        <v>37</v>
       </c>
       <c r="E178" t="inlineStr">
         <is>
@@ -4798,21 +4798,21 @@
     <row r="179">
       <c r="A179" t="inlineStr">
         <is>
-          <t>12:00:15</t>
+          <t>12:28:38</t>
         </is>
       </c>
       <c r="B179" t="inlineStr">
         <is>
-          <t>12:51</t>
+          <t>12:47</t>
         </is>
       </c>
       <c r="C179" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D179" t="n">
-        <v>51</v>
+        <v>19</v>
       </c>
       <c r="E179" t="inlineStr">
         <is>
@@ -4823,21 +4823,21 @@
     <row r="180">
       <c r="A180" t="inlineStr">
         <is>
-          <t>11:16:36</t>
+          <t>12:28:38</t>
         </is>
       </c>
       <c r="B180" t="inlineStr">
         <is>
-          <t>12:57</t>
+          <t>12:49</t>
         </is>
       </c>
       <c r="C180" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D180" t="n">
-        <v>101</v>
+        <v>21</v>
       </c>
       <c r="E180" t="inlineStr">
         <is>
@@ -4848,21 +4848,21 @@
     <row r="181">
       <c r="A181" t="inlineStr">
         <is>
-          <t>11:46:24</t>
+          <t>12:28:38</t>
         </is>
       </c>
       <c r="B181" t="inlineStr">
         <is>
-          <t>13:02</t>
+          <t>12:51</t>
         </is>
       </c>
       <c r="C181" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D181" t="n">
-        <v>76</v>
+        <v>23</v>
       </c>
       <c r="E181" t="inlineStr">
         <is>
@@ -4873,21 +4873,21 @@
     <row r="182">
       <c r="A182" t="inlineStr">
         <is>
-          <t>11:46:24</t>
+          <t>11:16:36</t>
         </is>
       </c>
       <c r="B182" t="inlineStr">
         <is>
-          <t>13:03</t>
+          <t>12:57</t>
         </is>
       </c>
       <c r="C182" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D182" t="n">
-        <v>77</v>
+        <v>101</v>
       </c>
       <c r="E182" t="inlineStr">
         <is>
@@ -4898,21 +4898,21 @@
     <row r="183">
       <c r="A183" t="inlineStr">
         <is>
-          <t>12:00:15</t>
+          <t>12:28:38</t>
         </is>
       </c>
       <c r="B183" t="inlineStr">
         <is>
-          <t>13:03</t>
+          <t>13:01</t>
         </is>
       </c>
       <c r="C183" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D183" t="n">
-        <v>63</v>
+        <v>33</v>
       </c>
       <c r="E183" t="inlineStr">
         <is>
@@ -4923,21 +4923,21 @@
     <row r="184">
       <c r="A184" t="inlineStr">
         <is>
-          <t>12:00:15</t>
+          <t>12:28:38</t>
         </is>
       </c>
       <c r="B184" t="inlineStr">
         <is>
-          <t>13:04</t>
+          <t>13:02</t>
         </is>
       </c>
       <c r="C184" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D184" t="n">
-        <v>64</v>
+        <v>34</v>
       </c>
       <c r="E184" t="inlineStr">
         <is>
@@ -4948,12 +4948,12 @@
     <row r="185">
       <c r="A185" t="inlineStr">
         <is>
-          <t>12:00:15</t>
+          <t>12:28:38</t>
         </is>
       </c>
       <c r="B185" t="inlineStr">
         <is>
-          <t>13:04</t>
+          <t>13:03</t>
         </is>
       </c>
       <c r="C185" t="inlineStr">
@@ -4962,7 +4962,7 @@
         </is>
       </c>
       <c r="D185" t="n">
-        <v>64</v>
+        <v>35</v>
       </c>
       <c r="E185" t="inlineStr">
         <is>
@@ -4978,16 +4978,16 @@
       </c>
       <c r="B186" t="inlineStr">
         <is>
-          <t>13:17</t>
+          <t>13:03</t>
         </is>
       </c>
       <c r="C186" t="inlineStr">
         <is>
-          <t>11X44_P_ETCHEVERRY</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D186" t="n">
-        <v>77</v>
+        <v>63</v>
       </c>
       <c r="E186" t="inlineStr">
         <is>
@@ -4998,21 +4998,21 @@
     <row r="187">
       <c r="A187" t="inlineStr">
         <is>
-          <t>12:00:15</t>
+          <t>12:28:38</t>
         </is>
       </c>
       <c r="B187" t="inlineStr">
         <is>
-          <t>13:19</t>
+          <t>13:03</t>
         </is>
       </c>
       <c r="C187" t="inlineStr">
         <is>
-          <t>215_ALUAR</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D187" t="n">
-        <v>79</v>
+        <v>35</v>
       </c>
       <c r="E187" t="inlineStr">
         <is>
@@ -5023,21 +5023,21 @@
     <row r="188">
       <c r="A188" t="inlineStr">
         <is>
-          <t>11:46:24</t>
+          <t>12:00:15</t>
         </is>
       </c>
       <c r="B188" t="inlineStr">
         <is>
-          <t>13:32</t>
+          <t>13:04</t>
         </is>
       </c>
       <c r="C188" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D188" t="n">
-        <v>106</v>
+        <v>64</v>
       </c>
       <c r="E188" t="inlineStr">
         <is>
@@ -5053,16 +5053,16 @@
       </c>
       <c r="B189" t="inlineStr">
         <is>
-          <t>13:33</t>
+          <t>13:04</t>
         </is>
       </c>
       <c r="C189" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D189" t="n">
-        <v>93</v>
+        <v>64</v>
       </c>
       <c r="E189" t="inlineStr">
         <is>
@@ -5073,21 +5073,21 @@
     <row r="190">
       <c r="A190" t="inlineStr">
         <is>
-          <t>12:00:15</t>
+          <t>12:28:38</t>
         </is>
       </c>
       <c r="B190" t="inlineStr">
         <is>
-          <t>13:38</t>
+          <t>13:17</t>
         </is>
       </c>
       <c r="C190" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>11X44_P_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D190" t="n">
-        <v>98</v>
+        <v>49</v>
       </c>
       <c r="E190" t="inlineStr">
         <is>
@@ -5098,21 +5098,21 @@
     <row r="191">
       <c r="A191" t="inlineStr">
         <is>
-          <t>11:46:24</t>
+          <t>12:28:38</t>
         </is>
       </c>
       <c r="B191" t="inlineStr">
         <is>
-          <t>13:41</t>
+          <t>13:18</t>
         </is>
       </c>
       <c r="C191" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>215_ALUAR</t>
         </is>
       </c>
       <c r="D191" t="n">
-        <v>115</v>
+        <v>50</v>
       </c>
       <c r="E191" t="inlineStr">
         <is>
@@ -5128,16 +5128,16 @@
       </c>
       <c r="B192" t="inlineStr">
         <is>
-          <t>13:47</t>
+          <t>13:19</t>
         </is>
       </c>
       <c r="C192" t="inlineStr">
         <is>
-          <t>225_GOMEZ</t>
+          <t>215_ALUAR</t>
         </is>
       </c>
       <c r="D192" t="n">
-        <v>107</v>
+        <v>79</v>
       </c>
       <c r="E192" t="inlineStr">
         <is>
@@ -5148,21 +5148,21 @@
     <row r="193">
       <c r="A193" t="inlineStr">
         <is>
-          <t>12:00:15</t>
+          <t>12:28:38</t>
         </is>
       </c>
       <c r="B193" t="inlineStr">
         <is>
-          <t>13:51</t>
+          <t>13:21</t>
         </is>
       </c>
       <c r="C193" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D193" t="n">
-        <v>111</v>
+        <v>53</v>
       </c>
       <c r="E193" t="inlineStr">
         <is>
@@ -5173,23 +5173,223 @@
     <row r="194">
       <c r="A194" t="inlineStr">
         <is>
+          <t>12:28:38</t>
+        </is>
+      </c>
+      <c r="B194" t="inlineStr">
+        <is>
+          <t>13:32</t>
+        </is>
+      </c>
+      <c r="C194" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D194" t="n">
+        <v>64</v>
+      </c>
+      <c r="E194" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="195">
+      <c r="A195" t="inlineStr">
+        <is>
           <t>12:00:15</t>
         </is>
       </c>
-      <c r="B194" t="inlineStr">
+      <c r="B195" t="inlineStr">
+        <is>
+          <t>13:33</t>
+        </is>
+      </c>
+      <c r="C195" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D195" t="n">
+        <v>93</v>
+      </c>
+      <c r="E195" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="196">
+      <c r="A196" t="inlineStr">
+        <is>
+          <t>12:28:38</t>
+        </is>
+      </c>
+      <c r="B196" t="inlineStr">
+        <is>
+          <t>13:38</t>
+        </is>
+      </c>
+      <c r="C196" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D196" t="n">
+        <v>70</v>
+      </c>
+      <c r="E196" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="197">
+      <c r="A197" t="inlineStr">
+        <is>
+          <t>11:46:24</t>
+        </is>
+      </c>
+      <c r="B197" t="inlineStr">
+        <is>
+          <t>13:41</t>
+        </is>
+      </c>
+      <c r="C197" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D197" t="n">
+        <v>115</v>
+      </c>
+      <c r="E197" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="198">
+      <c r="A198" t="inlineStr">
+        <is>
+          <t>12:28:38</t>
+        </is>
+      </c>
+      <c r="B198" t="inlineStr">
+        <is>
+          <t>13:47</t>
+        </is>
+      </c>
+      <c r="C198" t="inlineStr">
+        <is>
+          <t>225_GOMEZ</t>
+        </is>
+      </c>
+      <c r="D198" t="n">
+        <v>79</v>
+      </c>
+      <c r="E198" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="199">
+      <c r="A199" t="inlineStr">
+        <is>
+          <t>12:28:38</t>
+        </is>
+      </c>
+      <c r="B199" t="inlineStr">
+        <is>
+          <t>13:51</t>
+        </is>
+      </c>
+      <c r="C199" t="inlineStr">
+        <is>
+          <t>16_P MOR-SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D199" t="n">
+        <v>83</v>
+      </c>
+      <c r="E199" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="200">
+      <c r="A200" t="inlineStr">
+        <is>
+          <t>12:28:38</t>
+        </is>
+      </c>
+      <c r="B200" t="inlineStr">
         <is>
           <t>13:59</t>
         </is>
       </c>
-      <c r="C194" t="inlineStr">
+      <c r="C200" t="inlineStr">
         <is>
           <t>17_ROMERO</t>
         </is>
       </c>
-      <c r="D194" t="n">
-        <v>119</v>
-      </c>
-      <c r="E194" t="inlineStr">
+      <c r="D200" t="n">
+        <v>91</v>
+      </c>
+      <c r="E200" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="201">
+      <c r="A201" t="inlineStr">
+        <is>
+          <t>12:28:38</t>
+        </is>
+      </c>
+      <c r="B201" t="inlineStr">
+        <is>
+          <t>14:16</t>
+        </is>
+      </c>
+      <c r="C201" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D201" t="n">
+        <v>108</v>
+      </c>
+      <c r="E201" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="202">
+      <c r="A202" t="inlineStr">
+        <is>
+          <t>12:28:38</t>
+        </is>
+      </c>
+      <c r="B202" t="inlineStr">
+        <is>
+          <t>14:17</t>
+        </is>
+      </c>
+      <c r="C202" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D202" t="n">
+        <v>109</v>
+      </c>
+      <c r="E202" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -5206,7 +5406,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E36"/>
+  <dimension ref="A1:E38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5219,14 +5419,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 12:00:15</t>
+          <t>Última actualización: 12:28:38</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 31</t>
+          <t>Total filas: 33</t>
         </is>
       </c>
     </row>
@@ -5910,7 +6110,7 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>10:52:37</t>
+          <t>12:28:38</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -5924,7 +6124,7 @@
         </is>
       </c>
       <c r="D32" t="n">
-        <v>101</v>
+        <v>5</v>
       </c>
       <c r="E32" t="inlineStr">
         <is>
@@ -5960,12 +6160,12 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>12:00:15</t>
+          <t>12:28:38</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>13:04</t>
+          <t>13:03</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
@@ -5974,7 +6174,7 @@
         </is>
       </c>
       <c r="D34" t="n">
-        <v>64</v>
+        <v>35</v>
       </c>
       <c r="E34" t="inlineStr">
         <is>
@@ -5990,16 +6190,16 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>13:19</t>
+          <t>13:04</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>215_ALUAR</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D35" t="n">
-        <v>79</v>
+        <v>64</v>
       </c>
       <c r="E35" t="inlineStr">
         <is>
@@ -6010,23 +6210,73 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
+          <t>12:28:38</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>13:18</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>215_ALUAR</t>
+        </is>
+      </c>
+      <c r="D36" t="n">
+        <v>50</v>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
           <t>12:00:15</t>
         </is>
       </c>
-      <c r="B36" t="inlineStr">
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>13:19</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>215_ALUAR</t>
+        </is>
+      </c>
+      <c r="D37" t="n">
+        <v>79</v>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>12:28:38</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
         <is>
           <t>13:38</t>
         </is>
       </c>
-      <c r="C36" t="inlineStr">
+      <c r="C38" t="inlineStr">
         <is>
           <t>215A_EL PATO</t>
         </is>
       </c>
-      <c r="D36" t="n">
-        <v>98</v>
-      </c>
-      <c r="E36" t="inlineStr">
+      <c r="D38" t="n">
+        <v>70</v>
+      </c>
+      <c r="E38" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -6043,7 +6293,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E38"/>
+  <dimension ref="A1:E41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6056,14 +6306,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 12:00:15</t>
+          <t>Última actualización: 12:28:38</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 33</t>
+          <t>Total filas: 36</t>
         </is>
       </c>
     </row>
@@ -6797,7 +7047,7 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>11:16:36</t>
+          <t>12:28:38</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -6811,7 +7061,7 @@
         </is>
       </c>
       <c r="D34" t="n">
-        <v>99</v>
+        <v>27</v>
       </c>
       <c r="E34" t="inlineStr">
         <is>
@@ -6847,12 +7097,12 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>12:00:15</t>
+          <t>12:28:38</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>13:11</t>
+          <t>13:10</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
@@ -6861,7 +7111,7 @@
         </is>
       </c>
       <c r="D36" t="n">
-        <v>71</v>
+        <v>42</v>
       </c>
       <c r="E36" t="inlineStr">
         <is>
@@ -6877,16 +7127,16 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>13:22</t>
+          <t>13:11</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>215B_LP-P MOR-1 Y 57</t>
+          <t>215A_LA PLATA</t>
         </is>
       </c>
       <c r="D37" t="n">
-        <v>82</v>
+        <v>71</v>
       </c>
       <c r="E37" t="inlineStr">
         <is>
@@ -6897,23 +7147,98 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
+          <t>12:28:38</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>13:21</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>215B_LP-P MOR-1 Y 57</t>
+        </is>
+      </c>
+      <c r="D38" t="n">
+        <v>53</v>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
           <t>12:00:15</t>
         </is>
       </c>
-      <c r="B38" t="inlineStr">
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>13:22</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>215B_LP-P MOR-1 Y 57</t>
+        </is>
+      </c>
+      <c r="D39" t="n">
+        <v>82</v>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>12:28:38</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>13:55</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D40" t="n">
+        <v>87</v>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>12:00:15</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
         <is>
           <t>13:56</t>
         </is>
       </c>
-      <c r="C38" t="inlineStr">
+      <c r="C41" t="inlineStr">
         <is>
           <t>215C_LA PLATA</t>
         </is>
       </c>
-      <c r="D38" t="n">
+      <c r="D41" t="n">
         <v>116</v>
       </c>
-      <c r="E38" t="inlineStr">
+      <c r="E41" t="inlineStr">
         <is>
           <t>L6203</t>
         </is>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 1807
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-03-21.xlsx
+++ b/data/horarios-141-2026-03-21.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E202"/>
+  <dimension ref="A1:E208"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 12:28:38</t>
+          <t>Última actualización: 12:48:06</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 197</t>
+          <t>Total filas: 203</t>
         </is>
       </c>
     </row>
@@ -758,7 +758,7 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D17" t="n">
@@ -783,7 +783,7 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D18" t="n">
@@ -1158,7 +1158,7 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D33" t="n">
@@ -1183,7 +1183,7 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D34" t="n">
@@ -1558,7 +1558,7 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D49" t="n">
@@ -1583,7 +1583,7 @@
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D50" t="n">
@@ -1883,7 +1883,7 @@
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D62" t="n">
@@ -1898,7 +1898,7 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>06:59:30</t>
+          <t>08:14:14</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
@@ -1908,11 +1908,11 @@
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D63" t="n">
-        <v>75</v>
+        <v>0</v>
       </c>
       <c r="E63" t="inlineStr">
         <is>
@@ -1923,7 +1923,7 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>08:14:14</t>
+          <t>06:59:30</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
@@ -1933,11 +1933,11 @@
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D64" t="n">
-        <v>0</v>
+        <v>75</v>
       </c>
       <c r="E64" t="inlineStr">
         <is>
@@ -1983,7 +1983,7 @@
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D66" t="n">
@@ -1998,7 +1998,7 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>07:27:35</t>
+          <t>07:51:37</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
@@ -2008,11 +2008,11 @@
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D67" t="n">
-        <v>52</v>
+        <v>28</v>
       </c>
       <c r="E67" t="inlineStr">
         <is>
@@ -2023,7 +2023,7 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>07:51:37</t>
+          <t>07:27:35</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
@@ -2033,11 +2033,11 @@
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D68" t="n">
-        <v>28</v>
+        <v>52</v>
       </c>
       <c r="E68" t="inlineStr">
         <is>
@@ -2233,7 +2233,7 @@
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D76" t="n">
@@ -2258,7 +2258,7 @@
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D77" t="n">
@@ -2383,7 +2383,7 @@
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D82" t="n">
@@ -2433,7 +2433,7 @@
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D84" t="n">
@@ -2733,7 +2733,7 @@
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>215_EL PELIGRO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D96" t="n">
@@ -2758,7 +2758,7 @@
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215_EL PELIGRO</t>
         </is>
       </c>
       <c r="D97" t="n">
@@ -2873,7 +2873,7 @@
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>07:51:37</t>
+          <t>08:36:09</t>
         </is>
       </c>
       <c r="B102" t="inlineStr">
@@ -2883,11 +2883,11 @@
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D102" t="n">
-        <v>98</v>
+        <v>53</v>
       </c>
       <c r="E102" t="inlineStr">
         <is>
@@ -2898,7 +2898,7 @@
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>08:36:09</t>
+          <t>07:51:37</t>
         </is>
       </c>
       <c r="B103" t="inlineStr">
@@ -2908,11 +2908,11 @@
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D103" t="n">
-        <v>53</v>
+        <v>98</v>
       </c>
       <c r="E103" t="inlineStr">
         <is>
@@ -3498,7 +3498,7 @@
     <row r="127">
       <c r="A127" t="inlineStr">
         <is>
-          <t>08:36:09</t>
+          <t>10:14:52</t>
         </is>
       </c>
       <c r="B127" t="inlineStr">
@@ -3508,11 +3508,11 @@
       </c>
       <c r="C127" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D127" t="n">
-        <v>117</v>
+        <v>19</v>
       </c>
       <c r="E127" t="inlineStr">
         <is>
@@ -3523,7 +3523,7 @@
     <row r="128">
       <c r="A128" t="inlineStr">
         <is>
-          <t>10:14:52</t>
+          <t>08:36:09</t>
         </is>
       </c>
       <c r="B128" t="inlineStr">
@@ -3533,11 +3533,11 @@
       </c>
       <c r="C128" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D128" t="n">
-        <v>19</v>
+        <v>117</v>
       </c>
       <c r="E128" t="inlineStr">
         <is>
@@ -3873,7 +3873,7 @@
     <row r="142">
       <c r="A142" t="inlineStr">
         <is>
-          <t>10:52:37</t>
+          <t>10:14:52</t>
         </is>
       </c>
       <c r="B142" t="inlineStr">
@@ -3883,11 +3883,11 @@
       </c>
       <c r="C142" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D142" t="n">
-        <v>11</v>
+        <v>49</v>
       </c>
       <c r="E142" t="inlineStr">
         <is>
@@ -3898,7 +3898,7 @@
     <row r="143">
       <c r="A143" t="inlineStr">
         <is>
-          <t>10:14:52</t>
+          <t>10:52:37</t>
         </is>
       </c>
       <c r="B143" t="inlineStr">
@@ -3908,11 +3908,11 @@
       </c>
       <c r="C143" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D143" t="n">
-        <v>49</v>
+        <v>11</v>
       </c>
       <c r="E143" t="inlineStr">
         <is>
@@ -4123,7 +4123,7 @@
     <row r="152">
       <c r="A152" t="inlineStr">
         <is>
-          <t>10:14:52</t>
+          <t>11:16:36</t>
         </is>
       </c>
       <c r="B152" t="inlineStr">
@@ -4133,11 +4133,11 @@
       </c>
       <c r="C152" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D152" t="n">
-        <v>78</v>
+        <v>16</v>
       </c>
       <c r="E152" t="inlineStr">
         <is>
@@ -4148,7 +4148,7 @@
     <row r="153">
       <c r="A153" t="inlineStr">
         <is>
-          <t>11:16:36</t>
+          <t>10:14:52</t>
         </is>
       </c>
       <c r="B153" t="inlineStr">
@@ -4158,11 +4158,11 @@
       </c>
       <c r="C153" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D153" t="n">
-        <v>16</v>
+        <v>78</v>
       </c>
       <c r="E153" t="inlineStr">
         <is>
@@ -4183,7 +4183,7 @@
       </c>
       <c r="C154" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D154" t="n">
@@ -4208,7 +4208,7 @@
       </c>
       <c r="C155" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D155" t="n">
@@ -4648,7 +4648,7 @@
     <row r="173">
       <c r="A173" t="inlineStr">
         <is>
-          <t>12:28:38</t>
+          <t>12:00:15</t>
         </is>
       </c>
       <c r="B173" t="inlineStr">
@@ -4658,11 +4658,11 @@
       </c>
       <c r="C173" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D173" t="n">
-        <v>5</v>
+        <v>33</v>
       </c>
       <c r="E173" t="inlineStr">
         <is>
@@ -4683,7 +4683,7 @@
       </c>
       <c r="C174" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D174" t="n">
@@ -4698,7 +4698,7 @@
     <row r="175">
       <c r="A175" t="inlineStr">
         <is>
-          <t>12:00:15</t>
+          <t>12:28:38</t>
         </is>
       </c>
       <c r="B175" t="inlineStr">
@@ -4708,11 +4708,11 @@
       </c>
       <c r="C175" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D175" t="n">
-        <v>33</v>
+        <v>5</v>
       </c>
       <c r="E175" t="inlineStr">
         <is>
@@ -4823,21 +4823,21 @@
     <row r="180">
       <c r="A180" t="inlineStr">
         <is>
-          <t>12:28:38</t>
+          <t>12:48:06</t>
         </is>
       </c>
       <c r="B180" t="inlineStr">
         <is>
-          <t>12:49</t>
+          <t>12:48</t>
         </is>
       </c>
       <c r="C180" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D180" t="n">
-        <v>21</v>
+        <v>0</v>
       </c>
       <c r="E180" t="inlineStr">
         <is>
@@ -4848,21 +4848,21 @@
     <row r="181">
       <c r="A181" t="inlineStr">
         <is>
-          <t>12:28:38</t>
+          <t>12:48:06</t>
         </is>
       </c>
       <c r="B181" t="inlineStr">
         <is>
-          <t>12:51</t>
+          <t>12:49</t>
         </is>
       </c>
       <c r="C181" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D181" t="n">
-        <v>23</v>
+        <v>1</v>
       </c>
       <c r="E181" t="inlineStr">
         <is>
@@ -4873,21 +4873,21 @@
     <row r="182">
       <c r="A182" t="inlineStr">
         <is>
-          <t>11:16:36</t>
+          <t>12:48:06</t>
         </is>
       </c>
       <c r="B182" t="inlineStr">
         <is>
-          <t>12:57</t>
+          <t>12:51</t>
         </is>
       </c>
       <c r="C182" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D182" t="n">
-        <v>101</v>
+        <v>3</v>
       </c>
       <c r="E182" t="inlineStr">
         <is>
@@ -4898,21 +4898,21 @@
     <row r="183">
       <c r="A183" t="inlineStr">
         <is>
-          <t>12:28:38</t>
+          <t>11:16:36</t>
         </is>
       </c>
       <c r="B183" t="inlineStr">
         <is>
-          <t>13:01</t>
+          <t>12:57</t>
         </is>
       </c>
       <c r="C183" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D183" t="n">
-        <v>33</v>
+        <v>101</v>
       </c>
       <c r="E183" t="inlineStr">
         <is>
@@ -4923,21 +4923,21 @@
     <row r="184">
       <c r="A184" t="inlineStr">
         <is>
-          <t>12:28:38</t>
+          <t>12:48:06</t>
         </is>
       </c>
       <c r="B184" t="inlineStr">
         <is>
-          <t>13:02</t>
+          <t>13:01</t>
         </is>
       </c>
       <c r="C184" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D184" t="n">
-        <v>34</v>
+        <v>13</v>
       </c>
       <c r="E184" t="inlineStr">
         <is>
@@ -4953,16 +4953,16 @@
       </c>
       <c r="B185" t="inlineStr">
         <is>
-          <t>13:03</t>
+          <t>13:02</t>
         </is>
       </c>
       <c r="C185" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D185" t="n">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="E185" t="inlineStr">
         <is>
@@ -4973,7 +4973,7 @@
     <row r="186">
       <c r="A186" t="inlineStr">
         <is>
-          <t>12:00:15</t>
+          <t>12:28:38</t>
         </is>
       </c>
       <c r="B186" t="inlineStr">
@@ -4983,11 +4983,11 @@
       </c>
       <c r="C186" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D186" t="n">
-        <v>63</v>
+        <v>35</v>
       </c>
       <c r="E186" t="inlineStr">
         <is>
@@ -5023,21 +5023,21 @@
     <row r="188">
       <c r="A188" t="inlineStr">
         <is>
-          <t>12:00:15</t>
+          <t>12:48:06</t>
         </is>
       </c>
       <c r="B188" t="inlineStr">
         <is>
-          <t>13:04</t>
+          <t>13:03</t>
         </is>
       </c>
       <c r="C188" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D188" t="n">
-        <v>64</v>
+        <v>15</v>
       </c>
       <c r="E188" t="inlineStr">
         <is>
@@ -5048,7 +5048,7 @@
     <row r="189">
       <c r="A189" t="inlineStr">
         <is>
-          <t>12:00:15</t>
+          <t>12:48:06</t>
         </is>
       </c>
       <c r="B189" t="inlineStr">
@@ -5062,7 +5062,7 @@
         </is>
       </c>
       <c r="D189" t="n">
-        <v>64</v>
+        <v>16</v>
       </c>
       <c r="E189" t="inlineStr">
         <is>
@@ -5073,21 +5073,21 @@
     <row r="190">
       <c r="A190" t="inlineStr">
         <is>
-          <t>12:28:38</t>
+          <t>12:48:06</t>
         </is>
       </c>
       <c r="B190" t="inlineStr">
         <is>
-          <t>13:17</t>
+          <t>13:04</t>
         </is>
       </c>
       <c r="C190" t="inlineStr">
         <is>
-          <t>11X44_P_ETCHEVERRY</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D190" t="n">
-        <v>49</v>
+        <v>16</v>
       </c>
       <c r="E190" t="inlineStr">
         <is>
@@ -5098,21 +5098,21 @@
     <row r="191">
       <c r="A191" t="inlineStr">
         <is>
-          <t>12:28:38</t>
+          <t>12:48:06</t>
         </is>
       </c>
       <c r="B191" t="inlineStr">
         <is>
-          <t>13:18</t>
+          <t>13:17</t>
         </is>
       </c>
       <c r="C191" t="inlineStr">
         <is>
-          <t>215_ALUAR</t>
+          <t>11X44_P_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D191" t="n">
-        <v>50</v>
+        <v>29</v>
       </c>
       <c r="E191" t="inlineStr">
         <is>
@@ -5123,12 +5123,12 @@
     <row r="192">
       <c r="A192" t="inlineStr">
         <is>
-          <t>12:00:15</t>
+          <t>12:28:38</t>
         </is>
       </c>
       <c r="B192" t="inlineStr">
         <is>
-          <t>13:19</t>
+          <t>13:18</t>
         </is>
       </c>
       <c r="C192" t="inlineStr">
@@ -5137,7 +5137,7 @@
         </is>
       </c>
       <c r="D192" t="n">
-        <v>79</v>
+        <v>50</v>
       </c>
       <c r="E192" t="inlineStr">
         <is>
@@ -5148,21 +5148,21 @@
     <row r="193">
       <c r="A193" t="inlineStr">
         <is>
-          <t>12:28:38</t>
+          <t>12:48:06</t>
         </is>
       </c>
       <c r="B193" t="inlineStr">
         <is>
-          <t>13:21</t>
+          <t>13:19</t>
         </is>
       </c>
       <c r="C193" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>215_ALUAR</t>
         </is>
       </c>
       <c r="D193" t="n">
-        <v>53</v>
+        <v>31</v>
       </c>
       <c r="E193" t="inlineStr">
         <is>
@@ -5173,21 +5173,21 @@
     <row r="194">
       <c r="A194" t="inlineStr">
         <is>
-          <t>12:28:38</t>
+          <t>12:48:06</t>
         </is>
       </c>
       <c r="B194" t="inlineStr">
         <is>
-          <t>13:32</t>
+          <t>13:21</t>
         </is>
       </c>
       <c r="C194" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D194" t="n">
-        <v>64</v>
+        <v>33</v>
       </c>
       <c r="E194" t="inlineStr">
         <is>
@@ -5198,12 +5198,12 @@
     <row r="195">
       <c r="A195" t="inlineStr">
         <is>
-          <t>12:00:15</t>
+          <t>12:28:38</t>
         </is>
       </c>
       <c r="B195" t="inlineStr">
         <is>
-          <t>13:33</t>
+          <t>13:32</t>
         </is>
       </c>
       <c r="C195" t="inlineStr">
@@ -5212,7 +5212,7 @@
         </is>
       </c>
       <c r="D195" t="n">
-        <v>93</v>
+        <v>64</v>
       </c>
       <c r="E195" t="inlineStr">
         <is>
@@ -5223,21 +5223,21 @@
     <row r="196">
       <c r="A196" t="inlineStr">
         <is>
-          <t>12:28:38</t>
+          <t>12:48:06</t>
         </is>
       </c>
       <c r="B196" t="inlineStr">
         <is>
-          <t>13:38</t>
+          <t>13:33</t>
         </is>
       </c>
       <c r="C196" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D196" t="n">
-        <v>70</v>
+        <v>45</v>
       </c>
       <c r="E196" t="inlineStr">
         <is>
@@ -5248,21 +5248,21 @@
     <row r="197">
       <c r="A197" t="inlineStr">
         <is>
-          <t>11:46:24</t>
+          <t>12:48:06</t>
         </is>
       </c>
       <c r="B197" t="inlineStr">
         <is>
-          <t>13:41</t>
+          <t>13:38</t>
         </is>
       </c>
       <c r="C197" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D197" t="n">
-        <v>115</v>
+        <v>50</v>
       </c>
       <c r="E197" t="inlineStr">
         <is>
@@ -5273,21 +5273,21 @@
     <row r="198">
       <c r="A198" t="inlineStr">
         <is>
-          <t>12:28:38</t>
+          <t>12:48:06</t>
         </is>
       </c>
       <c r="B198" t="inlineStr">
         <is>
-          <t>13:47</t>
+          <t>13:38</t>
         </is>
       </c>
       <c r="C198" t="inlineStr">
         <is>
-          <t>225_GOMEZ</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D198" t="n">
-        <v>79</v>
+        <v>50</v>
       </c>
       <c r="E198" t="inlineStr">
         <is>
@@ -5298,21 +5298,21 @@
     <row r="199">
       <c r="A199" t="inlineStr">
         <is>
-          <t>12:28:38</t>
+          <t>11:46:24</t>
         </is>
       </c>
       <c r="B199" t="inlineStr">
         <is>
-          <t>13:51</t>
+          <t>13:41</t>
         </is>
       </c>
       <c r="C199" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D199" t="n">
-        <v>83</v>
+        <v>115</v>
       </c>
       <c r="E199" t="inlineStr">
         <is>
@@ -5323,21 +5323,21 @@
     <row r="200">
       <c r="A200" t="inlineStr">
         <is>
-          <t>12:28:38</t>
+          <t>12:48:06</t>
         </is>
       </c>
       <c r="B200" t="inlineStr">
         <is>
-          <t>13:59</t>
+          <t>13:47</t>
         </is>
       </c>
       <c r="C200" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>225_GOMEZ</t>
         </is>
       </c>
       <c r="D200" t="n">
-        <v>91</v>
+        <v>59</v>
       </c>
       <c r="E200" t="inlineStr">
         <is>
@@ -5348,21 +5348,21 @@
     <row r="201">
       <c r="A201" t="inlineStr">
         <is>
-          <t>12:28:38</t>
+          <t>12:48:06</t>
         </is>
       </c>
       <c r="B201" t="inlineStr">
         <is>
-          <t>14:16</t>
+          <t>13:51</t>
         </is>
       </c>
       <c r="C201" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D201" t="n">
-        <v>108</v>
+        <v>63</v>
       </c>
       <c r="E201" t="inlineStr">
         <is>
@@ -5373,23 +5373,173 @@
     <row r="202">
       <c r="A202" t="inlineStr">
         <is>
+          <t>12:48:06</t>
+        </is>
+      </c>
+      <c r="B202" t="inlineStr">
+        <is>
+          <t>13:59</t>
+        </is>
+      </c>
+      <c r="C202" t="inlineStr">
+        <is>
+          <t>17_ROMERO</t>
+        </is>
+      </c>
+      <c r="D202" t="n">
+        <v>71</v>
+      </c>
+      <c r="E202" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="203">
+      <c r="A203" t="inlineStr">
+        <is>
           <t>12:28:38</t>
         </is>
       </c>
-      <c r="B202" t="inlineStr">
+      <c r="B203" t="inlineStr">
+        <is>
+          <t>14:16</t>
+        </is>
+      </c>
+      <c r="C203" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D203" t="n">
+        <v>108</v>
+      </c>
+      <c r="E203" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="204">
+      <c r="A204" t="inlineStr">
+        <is>
+          <t>12:48:06</t>
+        </is>
+      </c>
+      <c r="B204" t="inlineStr">
         <is>
           <t>14:17</t>
         </is>
       </c>
-      <c r="C202" t="inlineStr">
+      <c r="C204" t="inlineStr">
         <is>
           <t>10_OLMOS</t>
         </is>
       </c>
-      <c r="D202" t="n">
-        <v>109</v>
-      </c>
-      <c r="E202" t="inlineStr">
+      <c r="D204" t="n">
+        <v>89</v>
+      </c>
+      <c r="E204" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="205">
+      <c r="A205" t="inlineStr">
+        <is>
+          <t>12:48:06</t>
+        </is>
+      </c>
+      <c r="B205" t="inlineStr">
+        <is>
+          <t>14:17</t>
+        </is>
+      </c>
+      <c r="C205" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D205" t="n">
+        <v>89</v>
+      </c>
+      <c r="E205" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="206">
+      <c r="A206" t="inlineStr">
+        <is>
+          <t>12:48:06</t>
+        </is>
+      </c>
+      <c r="B206" t="inlineStr">
+        <is>
+          <t>14:19</t>
+        </is>
+      </c>
+      <c r="C206" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D206" t="n">
+        <v>91</v>
+      </c>
+      <c r="E206" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="207">
+      <c r="A207" t="inlineStr">
+        <is>
+          <t>12:48:06</t>
+        </is>
+      </c>
+      <c r="B207" t="inlineStr">
+        <is>
+          <t>14:33</t>
+        </is>
+      </c>
+      <c r="C207" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D207" t="n">
+        <v>105</v>
+      </c>
+      <c r="E207" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="208">
+      <c r="A208" t="inlineStr">
+        <is>
+          <t>12:48:06</t>
+        </is>
+      </c>
+      <c r="B208" t="inlineStr">
+        <is>
+          <t>14:38</t>
+        </is>
+      </c>
+      <c r="C208" t="inlineStr">
+        <is>
+          <t>15X38_ABASTO</t>
+        </is>
+      </c>
+      <c r="D208" t="n">
+        <v>110</v>
+      </c>
+      <c r="E208" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -5406,7 +5556,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E38"/>
+  <dimension ref="A1:E39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5419,14 +5569,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 12:28:38</t>
+          <t>Última actualización: 12:48:06</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 33</t>
+          <t>Total filas: 34</t>
         </is>
       </c>
     </row>
@@ -6185,7 +6335,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>12:00:15</t>
+          <t>12:48:06</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -6199,7 +6349,7 @@
         </is>
       </c>
       <c r="D35" t="n">
-        <v>64</v>
+        <v>16</v>
       </c>
       <c r="E35" t="inlineStr">
         <is>
@@ -6235,7 +6385,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>12:00:15</t>
+          <t>12:48:06</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -6249,7 +6399,7 @@
         </is>
       </c>
       <c r="D37" t="n">
-        <v>79</v>
+        <v>31</v>
       </c>
       <c r="E37" t="inlineStr">
         <is>
@@ -6260,7 +6410,7 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>12:28:38</t>
+          <t>12:48:06</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
@@ -6274,9 +6424,34 @@
         </is>
       </c>
       <c r="D38" t="n">
-        <v>70</v>
+        <v>50</v>
       </c>
       <c r="E38" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>12:48:06</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>14:19</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D39" t="n">
+        <v>91</v>
+      </c>
+      <c r="E39" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -6293,7 +6468,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E41"/>
+  <dimension ref="A1:E42"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6306,14 +6481,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 12:28:38</t>
+          <t>Última actualización: 12:48:06</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 36</t>
+          <t>Total filas: 37</t>
         </is>
       </c>
     </row>
@@ -7072,7 +7247,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>12:00:15</t>
+          <t>12:48:06</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -7086,7 +7261,7 @@
         </is>
       </c>
       <c r="D35" t="n">
-        <v>56</v>
+        <v>8</v>
       </c>
       <c r="E35" t="inlineStr">
         <is>
@@ -7122,7 +7297,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>12:00:15</t>
+          <t>12:48:06</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -7136,7 +7311,7 @@
         </is>
       </c>
       <c r="D37" t="n">
-        <v>71</v>
+        <v>23</v>
       </c>
       <c r="E37" t="inlineStr">
         <is>
@@ -7172,7 +7347,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>12:00:15</t>
+          <t>12:48:06</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -7186,7 +7361,7 @@
         </is>
       </c>
       <c r="D39" t="n">
-        <v>82</v>
+        <v>34</v>
       </c>
       <c r="E39" t="inlineStr">
         <is>
@@ -7239,6 +7414,31 @@
         <v>116</v>
       </c>
       <c r="E41" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>12:48:06</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>13:57</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D42" t="n">
+        <v>69</v>
+      </c>
+      <c r="E42" t="inlineStr">
         <is>
           <t>L6203</t>
         </is>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 1808
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-03-21.xlsx
+++ b/data/horarios-141-2026-03-21.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E208"/>
+  <dimension ref="A1:E213"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 12:48:06</t>
+          <t>Última actualización: 13:00:14</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 203</t>
+          <t>Total filas: 208</t>
         </is>
       </c>
     </row>
@@ -758,7 +758,7 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D17" t="n">
@@ -783,7 +783,7 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D18" t="n">
@@ -1158,7 +1158,7 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D33" t="n">
@@ -1183,7 +1183,7 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D34" t="n">
@@ -1883,7 +1883,7 @@
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D62" t="n">
@@ -1898,7 +1898,7 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>08:14:14</t>
+          <t>06:59:30</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
@@ -1908,11 +1908,11 @@
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D63" t="n">
-        <v>0</v>
+        <v>75</v>
       </c>
       <c r="E63" t="inlineStr">
         <is>
@@ -1923,7 +1923,7 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>06:59:30</t>
+          <t>08:14:14</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
@@ -1933,11 +1933,11 @@
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D64" t="n">
-        <v>75</v>
+        <v>0</v>
       </c>
       <c r="E64" t="inlineStr">
         <is>
@@ -2233,7 +2233,7 @@
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D76" t="n">
@@ -2258,7 +2258,7 @@
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D77" t="n">
@@ -2398,7 +2398,7 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>07:27:35</t>
+          <t>08:50:55</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
@@ -2408,11 +2408,11 @@
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D83" t="n">
-        <v>84</v>
+        <v>1</v>
       </c>
       <c r="E83" t="inlineStr">
         <is>
@@ -2423,7 +2423,7 @@
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>08:50:55</t>
+          <t>07:27:35</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
@@ -2433,11 +2433,11 @@
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D84" t="n">
-        <v>1</v>
+        <v>84</v>
       </c>
       <c r="E84" t="inlineStr">
         <is>
@@ -2698,7 +2698,7 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>08:14:14</t>
+          <t>08:50:55</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
@@ -2708,11 +2708,11 @@
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>215_EL PELIGRO</t>
         </is>
       </c>
       <c r="D95" t="n">
-        <v>64</v>
+        <v>28</v>
       </c>
       <c r="E95" t="inlineStr">
         <is>
@@ -2748,7 +2748,7 @@
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>08:50:55</t>
+          <t>08:14:14</t>
         </is>
       </c>
       <c r="B97" t="inlineStr">
@@ -2758,11 +2758,11 @@
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>215_EL PELIGRO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D97" t="n">
-        <v>28</v>
+        <v>64</v>
       </c>
       <c r="E97" t="inlineStr">
         <is>
@@ -2923,7 +2923,7 @@
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>09:23:24</t>
+          <t>08:14:14</t>
         </is>
       </c>
       <c r="B104" t="inlineStr">
@@ -2933,11 +2933,11 @@
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D104" t="n">
-        <v>10</v>
+        <v>79</v>
       </c>
       <c r="E104" t="inlineStr">
         <is>
@@ -2948,7 +2948,7 @@
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>08:14:14</t>
+          <t>09:23:24</t>
         </is>
       </c>
       <c r="B105" t="inlineStr">
@@ -2958,11 +2958,11 @@
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D105" t="n">
-        <v>79</v>
+        <v>10</v>
       </c>
       <c r="E105" t="inlineStr">
         <is>
@@ -3173,7 +3173,7 @@
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>08:50:55</t>
+          <t>09:23:24</t>
         </is>
       </c>
       <c r="B114" t="inlineStr">
@@ -3183,11 +3183,11 @@
       </c>
       <c r="C114" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D114" t="n">
-        <v>73</v>
+        <v>40</v>
       </c>
       <c r="E114" t="inlineStr">
         <is>
@@ -3198,7 +3198,7 @@
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>09:23:24</t>
+          <t>08:50:55</t>
         </is>
       </c>
       <c r="B115" t="inlineStr">
@@ -3208,11 +3208,11 @@
       </c>
       <c r="C115" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D115" t="n">
-        <v>40</v>
+        <v>73</v>
       </c>
       <c r="E115" t="inlineStr">
         <is>
@@ -3873,7 +3873,7 @@
     <row r="142">
       <c r="A142" t="inlineStr">
         <is>
-          <t>10:14:52</t>
+          <t>10:52:37</t>
         </is>
       </c>
       <c r="B142" t="inlineStr">
@@ -3883,11 +3883,11 @@
       </c>
       <c r="C142" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D142" t="n">
-        <v>49</v>
+        <v>11</v>
       </c>
       <c r="E142" t="inlineStr">
         <is>
@@ -3898,7 +3898,7 @@
     <row r="143">
       <c r="A143" t="inlineStr">
         <is>
-          <t>10:52:37</t>
+          <t>10:14:52</t>
         </is>
       </c>
       <c r="B143" t="inlineStr">
@@ -3908,11 +3908,11 @@
       </c>
       <c r="C143" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D143" t="n">
-        <v>11</v>
+        <v>49</v>
       </c>
       <c r="E143" t="inlineStr">
         <is>
@@ -4473,7 +4473,7 @@
     <row r="166">
       <c r="A166" t="inlineStr">
         <is>
-          <t>12:00:15</t>
+          <t>11:16:36</t>
         </is>
       </c>
       <c r="B166" t="inlineStr">
@@ -4483,11 +4483,11 @@
       </c>
       <c r="C166" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D166" t="n">
-        <v>4</v>
+        <v>48</v>
       </c>
       <c r="E166" t="inlineStr">
         <is>
@@ -4498,7 +4498,7 @@
     <row r="167">
       <c r="A167" t="inlineStr">
         <is>
-          <t>11:16:36</t>
+          <t>12:00:15</t>
         </is>
       </c>
       <c r="B167" t="inlineStr">
@@ -4508,11 +4508,11 @@
       </c>
       <c r="C167" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D167" t="n">
-        <v>48</v>
+        <v>4</v>
       </c>
       <c r="E167" t="inlineStr">
         <is>
@@ -4923,21 +4923,21 @@
     <row r="184">
       <c r="A184" t="inlineStr">
         <is>
-          <t>12:48:06</t>
+          <t>13:00:14</t>
         </is>
       </c>
       <c r="B184" t="inlineStr">
         <is>
-          <t>13:01</t>
+          <t>13:00</t>
         </is>
       </c>
       <c r="C184" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D184" t="n">
-        <v>13</v>
+        <v>0</v>
       </c>
       <c r="E184" t="inlineStr">
         <is>
@@ -4948,21 +4948,21 @@
     <row r="185">
       <c r="A185" t="inlineStr">
         <is>
-          <t>12:28:38</t>
+          <t>12:48:06</t>
         </is>
       </c>
       <c r="B185" t="inlineStr">
         <is>
-          <t>13:02</t>
+          <t>13:01</t>
         </is>
       </c>
       <c r="C185" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D185" t="n">
-        <v>34</v>
+        <v>13</v>
       </c>
       <c r="E185" t="inlineStr">
         <is>
@@ -4978,16 +4978,16 @@
       </c>
       <c r="B186" t="inlineStr">
         <is>
-          <t>13:03</t>
+          <t>13:02</t>
         </is>
       </c>
       <c r="C186" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D186" t="n">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="E186" t="inlineStr">
         <is>
@@ -5008,7 +5008,7 @@
       </c>
       <c r="C187" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D187" t="n">
@@ -5023,7 +5023,7 @@
     <row r="188">
       <c r="A188" t="inlineStr">
         <is>
-          <t>12:48:06</t>
+          <t>12:28:38</t>
         </is>
       </c>
       <c r="B188" t="inlineStr">
@@ -5033,11 +5033,11 @@
       </c>
       <c r="C188" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D188" t="n">
-        <v>15</v>
+        <v>35</v>
       </c>
       <c r="E188" t="inlineStr">
         <is>
@@ -5048,21 +5048,21 @@
     <row r="189">
       <c r="A189" t="inlineStr">
         <is>
-          <t>12:48:06</t>
+          <t>13:00:14</t>
         </is>
       </c>
       <c r="B189" t="inlineStr">
         <is>
-          <t>13:04</t>
+          <t>13:03</t>
         </is>
       </c>
       <c r="C189" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D189" t="n">
-        <v>16</v>
+        <v>3</v>
       </c>
       <c r="E189" t="inlineStr">
         <is>
@@ -5073,7 +5073,7 @@
     <row r="190">
       <c r="A190" t="inlineStr">
         <is>
-          <t>12:48:06</t>
+          <t>13:00:14</t>
         </is>
       </c>
       <c r="B190" t="inlineStr">
@@ -5083,11 +5083,11 @@
       </c>
       <c r="C190" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D190" t="n">
-        <v>16</v>
+        <v>4</v>
       </c>
       <c r="E190" t="inlineStr">
         <is>
@@ -5103,16 +5103,16 @@
       </c>
       <c r="B191" t="inlineStr">
         <is>
-          <t>13:17</t>
+          <t>13:04</t>
         </is>
       </c>
       <c r="C191" t="inlineStr">
         <is>
-          <t>11X44_P_ETCHEVERRY</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D191" t="n">
-        <v>29</v>
+        <v>16</v>
       </c>
       <c r="E191" t="inlineStr">
         <is>
@@ -5123,21 +5123,21 @@
     <row r="192">
       <c r="A192" t="inlineStr">
         <is>
-          <t>12:28:38</t>
+          <t>13:00:14</t>
         </is>
       </c>
       <c r="B192" t="inlineStr">
         <is>
-          <t>13:18</t>
+          <t>13:17</t>
         </is>
       </c>
       <c r="C192" t="inlineStr">
         <is>
-          <t>215_ALUAR</t>
+          <t>11X44_P_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D192" t="n">
-        <v>50</v>
+        <v>17</v>
       </c>
       <c r="E192" t="inlineStr">
         <is>
@@ -5148,12 +5148,12 @@
     <row r="193">
       <c r="A193" t="inlineStr">
         <is>
-          <t>12:48:06</t>
+          <t>12:28:38</t>
         </is>
       </c>
       <c r="B193" t="inlineStr">
         <is>
-          <t>13:19</t>
+          <t>13:18</t>
         </is>
       </c>
       <c r="C193" t="inlineStr">
@@ -5162,7 +5162,7 @@
         </is>
       </c>
       <c r="D193" t="n">
-        <v>31</v>
+        <v>50</v>
       </c>
       <c r="E193" t="inlineStr">
         <is>
@@ -5173,21 +5173,21 @@
     <row r="194">
       <c r="A194" t="inlineStr">
         <is>
-          <t>12:48:06</t>
+          <t>13:00:14</t>
         </is>
       </c>
       <c r="B194" t="inlineStr">
         <is>
-          <t>13:21</t>
+          <t>13:19</t>
         </is>
       </c>
       <c r="C194" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>215_ALUAR</t>
         </is>
       </c>
       <c r="D194" t="n">
-        <v>33</v>
+        <v>19</v>
       </c>
       <c r="E194" t="inlineStr">
         <is>
@@ -5198,21 +5198,21 @@
     <row r="195">
       <c r="A195" t="inlineStr">
         <is>
-          <t>12:28:38</t>
+          <t>13:00:14</t>
         </is>
       </c>
       <c r="B195" t="inlineStr">
         <is>
-          <t>13:32</t>
+          <t>13:21</t>
         </is>
       </c>
       <c r="C195" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D195" t="n">
-        <v>64</v>
+        <v>21</v>
       </c>
       <c r="E195" t="inlineStr">
         <is>
@@ -5223,12 +5223,12 @@
     <row r="196">
       <c r="A196" t="inlineStr">
         <is>
-          <t>12:48:06</t>
+          <t>12:28:38</t>
         </is>
       </c>
       <c r="B196" t="inlineStr">
         <is>
-          <t>13:33</t>
+          <t>13:32</t>
         </is>
       </c>
       <c r="C196" t="inlineStr">
@@ -5237,7 +5237,7 @@
         </is>
       </c>
       <c r="D196" t="n">
-        <v>45</v>
+        <v>64</v>
       </c>
       <c r="E196" t="inlineStr">
         <is>
@@ -5248,21 +5248,21 @@
     <row r="197">
       <c r="A197" t="inlineStr">
         <is>
-          <t>12:48:06</t>
+          <t>13:00:14</t>
         </is>
       </c>
       <c r="B197" t="inlineStr">
         <is>
-          <t>13:38</t>
+          <t>13:33</t>
         </is>
       </c>
       <c r="C197" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D197" t="n">
-        <v>50</v>
+        <v>33</v>
       </c>
       <c r="E197" t="inlineStr">
         <is>
@@ -5278,16 +5278,16 @@
       </c>
       <c r="B198" t="inlineStr">
         <is>
-          <t>13:38</t>
+          <t>13:33</t>
         </is>
       </c>
       <c r="C198" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D198" t="n">
-        <v>50</v>
+        <v>45</v>
       </c>
       <c r="E198" t="inlineStr">
         <is>
@@ -5298,21 +5298,21 @@
     <row r="199">
       <c r="A199" t="inlineStr">
         <is>
-          <t>11:46:24</t>
+          <t>13:00:14</t>
         </is>
       </c>
       <c r="B199" t="inlineStr">
         <is>
-          <t>13:41</t>
+          <t>13:38</t>
         </is>
       </c>
       <c r="C199" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D199" t="n">
-        <v>115</v>
+        <v>38</v>
       </c>
       <c r="E199" t="inlineStr">
         <is>
@@ -5328,16 +5328,16 @@
       </c>
       <c r="B200" t="inlineStr">
         <is>
-          <t>13:47</t>
+          <t>13:38</t>
         </is>
       </c>
       <c r="C200" t="inlineStr">
         <is>
-          <t>225_GOMEZ</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D200" t="n">
-        <v>59</v>
+        <v>50</v>
       </c>
       <c r="E200" t="inlineStr">
         <is>
@@ -5348,21 +5348,21 @@
     <row r="201">
       <c r="A201" t="inlineStr">
         <is>
-          <t>12:48:06</t>
+          <t>13:00:14</t>
         </is>
       </c>
       <c r="B201" t="inlineStr">
         <is>
-          <t>13:51</t>
+          <t>13:41</t>
         </is>
       </c>
       <c r="C201" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D201" t="n">
-        <v>63</v>
+        <v>41</v>
       </c>
       <c r="E201" t="inlineStr">
         <is>
@@ -5373,21 +5373,21 @@
     <row r="202">
       <c r="A202" t="inlineStr">
         <is>
-          <t>12:48:06</t>
+          <t>13:00:14</t>
         </is>
       </c>
       <c r="B202" t="inlineStr">
         <is>
-          <t>13:59</t>
+          <t>13:47</t>
         </is>
       </c>
       <c r="C202" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>225_GOMEZ</t>
         </is>
       </c>
       <c r="D202" t="n">
-        <v>71</v>
+        <v>47</v>
       </c>
       <c r="E202" t="inlineStr">
         <is>
@@ -5398,21 +5398,21 @@
     <row r="203">
       <c r="A203" t="inlineStr">
         <is>
-          <t>12:28:38</t>
+          <t>13:00:14</t>
         </is>
       </c>
       <c r="B203" t="inlineStr">
         <is>
-          <t>14:16</t>
+          <t>13:51</t>
         </is>
       </c>
       <c r="C203" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D203" t="n">
-        <v>108</v>
+        <v>51</v>
       </c>
       <c r="E203" t="inlineStr">
         <is>
@@ -5423,21 +5423,21 @@
     <row r="204">
       <c r="A204" t="inlineStr">
         <is>
-          <t>12:48:06</t>
+          <t>13:00:14</t>
         </is>
       </c>
       <c r="B204" t="inlineStr">
         <is>
-          <t>14:17</t>
+          <t>13:59</t>
         </is>
       </c>
       <c r="C204" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D204" t="n">
-        <v>89</v>
+        <v>59</v>
       </c>
       <c r="E204" t="inlineStr">
         <is>
@@ -5448,21 +5448,21 @@
     <row r="205">
       <c r="A205" t="inlineStr">
         <is>
-          <t>12:48:06</t>
+          <t>13:00:14</t>
         </is>
       </c>
       <c r="B205" t="inlineStr">
         <is>
-          <t>14:17</t>
+          <t>14:03</t>
         </is>
       </c>
       <c r="C205" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D205" t="n">
-        <v>89</v>
+        <v>63</v>
       </c>
       <c r="E205" t="inlineStr">
         <is>
@@ -5473,21 +5473,21 @@
     <row r="206">
       <c r="A206" t="inlineStr">
         <is>
-          <t>12:48:06</t>
+          <t>12:28:38</t>
         </is>
       </c>
       <c r="B206" t="inlineStr">
         <is>
-          <t>14:19</t>
+          <t>14:16</t>
         </is>
       </c>
       <c r="C206" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D206" t="n">
-        <v>91</v>
+        <v>108</v>
       </c>
       <c r="E206" t="inlineStr">
         <is>
@@ -5498,21 +5498,21 @@
     <row r="207">
       <c r="A207" t="inlineStr">
         <is>
-          <t>12:48:06</t>
+          <t>13:00:14</t>
         </is>
       </c>
       <c r="B207" t="inlineStr">
         <is>
-          <t>14:33</t>
+          <t>14:17</t>
         </is>
       </c>
       <c r="C207" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D207" t="n">
-        <v>105</v>
+        <v>77</v>
       </c>
       <c r="E207" t="inlineStr">
         <is>
@@ -5523,23 +5523,148 @@
     <row r="208">
       <c r="A208" t="inlineStr">
         <is>
-          <t>12:48:06</t>
+          <t>13:00:14</t>
         </is>
       </c>
       <c r="B208" t="inlineStr">
         <is>
+          <t>14:17</t>
+        </is>
+      </c>
+      <c r="C208" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D208" t="n">
+        <v>77</v>
+      </c>
+      <c r="E208" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="209">
+      <c r="A209" t="inlineStr">
+        <is>
+          <t>13:00:14</t>
+        </is>
+      </c>
+      <c r="B209" t="inlineStr">
+        <is>
+          <t>14:19</t>
+        </is>
+      </c>
+      <c r="C209" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D209" t="n">
+        <v>79</v>
+      </c>
+      <c r="E209" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="210">
+      <c r="A210" t="inlineStr">
+        <is>
+          <t>13:00:14</t>
+        </is>
+      </c>
+      <c r="B210" t="inlineStr">
+        <is>
+          <t>14:33</t>
+        </is>
+      </c>
+      <c r="C210" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D210" t="n">
+        <v>93</v>
+      </c>
+      <c r="E210" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="211">
+      <c r="A211" t="inlineStr">
+        <is>
+          <t>13:00:14</t>
+        </is>
+      </c>
+      <c r="B211" t="inlineStr">
+        <is>
           <t>14:38</t>
         </is>
       </c>
-      <c r="C208" t="inlineStr">
+      <c r="C211" t="inlineStr">
         <is>
           <t>15X38_ABASTO</t>
         </is>
       </c>
-      <c r="D208" t="n">
-        <v>110</v>
-      </c>
-      <c r="E208" t="inlineStr">
+      <c r="D211" t="n">
+        <v>98</v>
+      </c>
+      <c r="E211" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="212">
+      <c r="A212" t="inlineStr">
+        <is>
+          <t>13:00:14</t>
+        </is>
+      </c>
+      <c r="B212" t="inlineStr">
+        <is>
+          <t>14:47</t>
+        </is>
+      </c>
+      <c r="C212" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D212" t="n">
+        <v>107</v>
+      </c>
+      <c r="E212" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="213">
+      <c r="A213" t="inlineStr">
+        <is>
+          <t>13:00:14</t>
+        </is>
+      </c>
+      <c r="B213" t="inlineStr">
+        <is>
+          <t>14:51</t>
+        </is>
+      </c>
+      <c r="C213" t="inlineStr">
+        <is>
+          <t>16_P MOR-SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D213" t="n">
+        <v>111</v>
+      </c>
+      <c r="E213" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -5569,7 +5694,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 12:48:06</t>
+          <t>Última actualización: 13:00:14</t>
         </is>
       </c>
     </row>
@@ -6335,7 +6460,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>12:48:06</t>
+          <t>13:00:14</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -6349,7 +6474,7 @@
         </is>
       </c>
       <c r="D35" t="n">
-        <v>16</v>
+        <v>4</v>
       </c>
       <c r="E35" t="inlineStr">
         <is>
@@ -6385,7 +6510,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>12:48:06</t>
+          <t>13:00:14</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -6399,7 +6524,7 @@
         </is>
       </c>
       <c r="D37" t="n">
-        <v>31</v>
+        <v>19</v>
       </c>
       <c r="E37" t="inlineStr">
         <is>
@@ -6410,7 +6535,7 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>12:48:06</t>
+          <t>13:00:14</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
@@ -6424,7 +6549,7 @@
         </is>
       </c>
       <c r="D38" t="n">
-        <v>50</v>
+        <v>38</v>
       </c>
       <c r="E38" t="inlineStr">
         <is>
@@ -6435,7 +6560,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>12:48:06</t>
+          <t>13:00:14</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -6449,7 +6574,7 @@
         </is>
       </c>
       <c r="D39" t="n">
-        <v>91</v>
+        <v>79</v>
       </c>
       <c r="E39" t="inlineStr">
         <is>
@@ -6468,7 +6593,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E42"/>
+  <dimension ref="A1:E43"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6481,14 +6606,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 12:48:06</t>
+          <t>Última actualización: 13:00:14</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 37</t>
+          <t>Total filas: 38</t>
         </is>
       </c>
     </row>
@@ -7297,7 +7422,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>12:48:06</t>
+          <t>13:00:14</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -7311,7 +7436,7 @@
         </is>
       </c>
       <c r="D37" t="n">
-        <v>23</v>
+        <v>11</v>
       </c>
       <c r="E37" t="inlineStr">
         <is>
@@ -7347,7 +7472,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>12:48:06</t>
+          <t>13:00:14</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -7361,7 +7486,7 @@
         </is>
       </c>
       <c r="D39" t="n">
-        <v>34</v>
+        <v>22</v>
       </c>
       <c r="E39" t="inlineStr">
         <is>
@@ -7397,7 +7522,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>12:00:15</t>
+          <t>13:00:14</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
@@ -7411,7 +7536,7 @@
         </is>
       </c>
       <c r="D41" t="n">
-        <v>116</v>
+        <v>56</v>
       </c>
       <c r="E41" t="inlineStr">
         <is>
@@ -7439,6 +7564,31 @@
         <v>69</v>
       </c>
       <c r="E42" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>13:00:14</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>14:46</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D43" t="n">
+        <v>106</v>
+      </c>
+      <c r="E43" t="inlineStr">
         <is>
           <t>L6203</t>
         </is>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 1809
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-03-21.xlsx
+++ b/data/horarios-141-2026-03-21.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E213"/>
+  <dimension ref="A1:E228"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 13:00:14</t>
+          <t>Última actualización: 13:32:57</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 208</t>
+          <t>Total filas: 223</t>
         </is>
       </c>
     </row>
@@ -758,7 +758,7 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D17" t="n">
@@ -783,7 +783,7 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D18" t="n">
@@ -1158,7 +1158,7 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D33" t="n">
@@ -1183,7 +1183,7 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D34" t="n">
@@ -1873,7 +1873,7 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>08:14:14</t>
+          <t>06:59:30</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
@@ -1883,11 +1883,11 @@
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D62" t="n">
-        <v>0</v>
+        <v>75</v>
       </c>
       <c r="E62" t="inlineStr">
         <is>
@@ -1898,7 +1898,7 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>06:59:30</t>
+          <t>08:14:14</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
@@ -1908,11 +1908,11 @@
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D63" t="n">
-        <v>75</v>
+        <v>0</v>
       </c>
       <c r="E63" t="inlineStr">
         <is>
@@ -1998,7 +1998,7 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>07:51:37</t>
+          <t>07:27:35</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
@@ -2008,11 +2008,11 @@
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D67" t="n">
-        <v>28</v>
+        <v>52</v>
       </c>
       <c r="E67" t="inlineStr">
         <is>
@@ -2023,7 +2023,7 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>07:27:35</t>
+          <t>07:51:37</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
@@ -2033,11 +2033,11 @@
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D68" t="n">
-        <v>52</v>
+        <v>28</v>
       </c>
       <c r="E68" t="inlineStr">
         <is>
@@ -2233,7 +2233,7 @@
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D76" t="n">
@@ -2258,7 +2258,7 @@
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D77" t="n">
@@ -2383,7 +2383,7 @@
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D82" t="n">
@@ -2398,7 +2398,7 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>08:50:55</t>
+          <t>07:27:35</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
@@ -2408,11 +2408,11 @@
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D83" t="n">
-        <v>1</v>
+        <v>84</v>
       </c>
       <c r="E83" t="inlineStr">
         <is>
@@ -2423,7 +2423,7 @@
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>07:27:35</t>
+          <t>08:50:55</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
@@ -2433,11 +2433,11 @@
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D84" t="n">
-        <v>84</v>
+        <v>1</v>
       </c>
       <c r="E84" t="inlineStr">
         <is>
@@ -2698,7 +2698,7 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>08:50:55</t>
+          <t>08:14:14</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
@@ -2708,11 +2708,11 @@
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>215_EL PELIGRO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D95" t="n">
-        <v>28</v>
+        <v>64</v>
       </c>
       <c r="E95" t="inlineStr">
         <is>
@@ -2733,7 +2733,7 @@
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215_EL PELIGRO</t>
         </is>
       </c>
       <c r="D96" t="n">
@@ -2748,7 +2748,7 @@
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>08:14:14</t>
+          <t>08:50:55</t>
         </is>
       </c>
       <c r="B97" t="inlineStr">
@@ -2758,11 +2758,11 @@
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D97" t="n">
-        <v>64</v>
+        <v>28</v>
       </c>
       <c r="E97" t="inlineStr">
         <is>
@@ -2873,7 +2873,7 @@
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>08:36:09</t>
+          <t>07:51:37</t>
         </is>
       </c>
       <c r="B102" t="inlineStr">
@@ -2883,11 +2883,11 @@
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D102" t="n">
-        <v>53</v>
+        <v>98</v>
       </c>
       <c r="E102" t="inlineStr">
         <is>
@@ -2898,7 +2898,7 @@
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>07:51:37</t>
+          <t>08:36:09</t>
         </is>
       </c>
       <c r="B103" t="inlineStr">
@@ -2908,11 +2908,11 @@
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D103" t="n">
-        <v>98</v>
+        <v>53</v>
       </c>
       <c r="E103" t="inlineStr">
         <is>
@@ -2923,7 +2923,7 @@
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>08:14:14</t>
+          <t>09:23:24</t>
         </is>
       </c>
       <c r="B104" t="inlineStr">
@@ -2933,11 +2933,11 @@
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D104" t="n">
-        <v>79</v>
+        <v>10</v>
       </c>
       <c r="E104" t="inlineStr">
         <is>
@@ -2948,7 +2948,7 @@
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>09:23:24</t>
+          <t>08:14:14</t>
         </is>
       </c>
       <c r="B105" t="inlineStr">
@@ -2958,11 +2958,11 @@
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D105" t="n">
-        <v>10</v>
+        <v>79</v>
       </c>
       <c r="E105" t="inlineStr">
         <is>
@@ -3083,7 +3083,7 @@
       </c>
       <c r="C110" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D110" t="n">
@@ -3108,7 +3108,7 @@
       </c>
       <c r="C111" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D111" t="n">
@@ -3173,7 +3173,7 @@
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>09:23:24</t>
+          <t>08:50:55</t>
         </is>
       </c>
       <c r="B114" t="inlineStr">
@@ -3183,11 +3183,11 @@
       </c>
       <c r="C114" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D114" t="n">
-        <v>40</v>
+        <v>73</v>
       </c>
       <c r="E114" t="inlineStr">
         <is>
@@ -3198,7 +3198,7 @@
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>08:50:55</t>
+          <t>09:23:24</t>
         </is>
       </c>
       <c r="B115" t="inlineStr">
@@ -3208,11 +3208,11 @@
       </c>
       <c r="C115" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D115" t="n">
-        <v>73</v>
+        <v>40</v>
       </c>
       <c r="E115" t="inlineStr">
         <is>
@@ -3498,7 +3498,7 @@
     <row r="127">
       <c r="A127" t="inlineStr">
         <is>
-          <t>10:14:52</t>
+          <t>08:36:09</t>
         </is>
       </c>
       <c r="B127" t="inlineStr">
@@ -3508,11 +3508,11 @@
       </c>
       <c r="C127" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D127" t="n">
-        <v>19</v>
+        <v>117</v>
       </c>
       <c r="E127" t="inlineStr">
         <is>
@@ -3523,7 +3523,7 @@
     <row r="128">
       <c r="A128" t="inlineStr">
         <is>
-          <t>08:36:09</t>
+          <t>10:14:52</t>
         </is>
       </c>
       <c r="B128" t="inlineStr">
@@ -3533,11 +3533,11 @@
       </c>
       <c r="C128" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D128" t="n">
-        <v>117</v>
+        <v>19</v>
       </c>
       <c r="E128" t="inlineStr">
         <is>
@@ -3598,7 +3598,7 @@
     <row r="131">
       <c r="A131" t="inlineStr">
         <is>
-          <t>09:23:24</t>
+          <t>10:14:52</t>
         </is>
       </c>
       <c r="B131" t="inlineStr">
@@ -3608,11 +3608,11 @@
       </c>
       <c r="C131" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D131" t="n">
-        <v>80</v>
+        <v>29</v>
       </c>
       <c r="E131" t="inlineStr">
         <is>
@@ -3623,7 +3623,7 @@
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t>10:14:52</t>
+          <t>09:23:24</t>
         </is>
       </c>
       <c r="B132" t="inlineStr">
@@ -3633,11 +3633,11 @@
       </c>
       <c r="C132" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D132" t="n">
-        <v>29</v>
+        <v>80</v>
       </c>
       <c r="E132" t="inlineStr">
         <is>
@@ -4123,7 +4123,7 @@
     <row r="152">
       <c r="A152" t="inlineStr">
         <is>
-          <t>11:16:36</t>
+          <t>10:14:52</t>
         </is>
       </c>
       <c r="B152" t="inlineStr">
@@ -4133,11 +4133,11 @@
       </c>
       <c r="C152" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D152" t="n">
-        <v>16</v>
+        <v>78</v>
       </c>
       <c r="E152" t="inlineStr">
         <is>
@@ -4148,7 +4148,7 @@
     <row r="153">
       <c r="A153" t="inlineStr">
         <is>
-          <t>10:14:52</t>
+          <t>11:16:36</t>
         </is>
       </c>
       <c r="B153" t="inlineStr">
@@ -4158,11 +4158,11 @@
       </c>
       <c r="C153" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D153" t="n">
-        <v>78</v>
+        <v>16</v>
       </c>
       <c r="E153" t="inlineStr">
         <is>
@@ -4183,7 +4183,7 @@
       </c>
       <c r="C154" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D154" t="n">
@@ -4208,7 +4208,7 @@
       </c>
       <c r="C155" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D155" t="n">
@@ -4648,7 +4648,7 @@
     <row r="173">
       <c r="A173" t="inlineStr">
         <is>
-          <t>12:00:15</t>
+          <t>12:28:38</t>
         </is>
       </c>
       <c r="B173" t="inlineStr">
@@ -4658,11 +4658,11 @@
       </c>
       <c r="C173" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D173" t="n">
-        <v>33</v>
+        <v>5</v>
       </c>
       <c r="E173" t="inlineStr">
         <is>
@@ -4698,7 +4698,7 @@
     <row r="175">
       <c r="A175" t="inlineStr">
         <is>
-          <t>12:28:38</t>
+          <t>12:00:15</t>
         </is>
       </c>
       <c r="B175" t="inlineStr">
@@ -4708,11 +4708,11 @@
       </c>
       <c r="C175" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D175" t="n">
-        <v>5</v>
+        <v>33</v>
       </c>
       <c r="E175" t="inlineStr">
         <is>
@@ -4998,7 +4998,7 @@
     <row r="187">
       <c r="A187" t="inlineStr">
         <is>
-          <t>12:28:38</t>
+          <t>13:00:14</t>
         </is>
       </c>
       <c r="B187" t="inlineStr">
@@ -5008,11 +5008,11 @@
       </c>
       <c r="C187" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D187" t="n">
-        <v>35</v>
+        <v>3</v>
       </c>
       <c r="E187" t="inlineStr">
         <is>
@@ -5048,7 +5048,7 @@
     <row r="189">
       <c r="A189" t="inlineStr">
         <is>
-          <t>13:00:14</t>
+          <t>12:28:38</t>
         </is>
       </c>
       <c r="B189" t="inlineStr">
@@ -5058,11 +5058,11 @@
       </c>
       <c r="C189" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D189" t="n">
-        <v>3</v>
+        <v>35</v>
       </c>
       <c r="E189" t="inlineStr">
         <is>
@@ -5073,7 +5073,7 @@
     <row r="190">
       <c r="A190" t="inlineStr">
         <is>
-          <t>13:00:14</t>
+          <t>12:48:06</t>
         </is>
       </c>
       <c r="B190" t="inlineStr">
@@ -5083,11 +5083,11 @@
       </c>
       <c r="C190" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D190" t="n">
-        <v>4</v>
+        <v>16</v>
       </c>
       <c r="E190" t="inlineStr">
         <is>
@@ -5098,7 +5098,7 @@
     <row r="191">
       <c r="A191" t="inlineStr">
         <is>
-          <t>12:48:06</t>
+          <t>13:00:14</t>
         </is>
       </c>
       <c r="B191" t="inlineStr">
@@ -5108,11 +5108,11 @@
       </c>
       <c r="C191" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D191" t="n">
-        <v>16</v>
+        <v>4</v>
       </c>
       <c r="E191" t="inlineStr">
         <is>
@@ -5223,7 +5223,7 @@
     <row r="196">
       <c r="A196" t="inlineStr">
         <is>
-          <t>12:28:38</t>
+          <t>13:32:57</t>
         </is>
       </c>
       <c r="B196" t="inlineStr">
@@ -5237,7 +5237,7 @@
         </is>
       </c>
       <c r="D196" t="n">
-        <v>64</v>
+        <v>0</v>
       </c>
       <c r="E196" t="inlineStr">
         <is>
@@ -5298,12 +5298,12 @@
     <row r="199">
       <c r="A199" t="inlineStr">
         <is>
-          <t>13:00:14</t>
+          <t>13:32:57</t>
         </is>
       </c>
       <c r="B199" t="inlineStr">
         <is>
-          <t>13:38</t>
+          <t>13:37</t>
         </is>
       </c>
       <c r="C199" t="inlineStr">
@@ -5312,7 +5312,7 @@
         </is>
       </c>
       <c r="D199" t="n">
-        <v>38</v>
+        <v>5</v>
       </c>
       <c r="E199" t="inlineStr">
         <is>
@@ -5323,7 +5323,7 @@
     <row r="200">
       <c r="A200" t="inlineStr">
         <is>
-          <t>12:48:06</t>
+          <t>13:00:14</t>
         </is>
       </c>
       <c r="B200" t="inlineStr">
@@ -5333,11 +5333,11 @@
       </c>
       <c r="C200" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D200" t="n">
-        <v>50</v>
+        <v>38</v>
       </c>
       <c r="E200" t="inlineStr">
         <is>
@@ -5348,21 +5348,21 @@
     <row r="201">
       <c r="A201" t="inlineStr">
         <is>
-          <t>13:00:14</t>
+          <t>12:48:06</t>
         </is>
       </c>
       <c r="B201" t="inlineStr">
         <is>
-          <t>13:41</t>
+          <t>13:38</t>
         </is>
       </c>
       <c r="C201" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D201" t="n">
-        <v>41</v>
+        <v>50</v>
       </c>
       <c r="E201" t="inlineStr">
         <is>
@@ -5373,21 +5373,21 @@
     <row r="202">
       <c r="A202" t="inlineStr">
         <is>
-          <t>13:00:14</t>
+          <t>13:32:57</t>
         </is>
       </c>
       <c r="B202" t="inlineStr">
         <is>
-          <t>13:47</t>
+          <t>13:41</t>
         </is>
       </c>
       <c r="C202" t="inlineStr">
         <is>
-          <t>225_GOMEZ</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D202" t="n">
-        <v>47</v>
+        <v>9</v>
       </c>
       <c r="E202" t="inlineStr">
         <is>
@@ -5398,21 +5398,21 @@
     <row r="203">
       <c r="A203" t="inlineStr">
         <is>
-          <t>13:00:14</t>
+          <t>13:32:57</t>
         </is>
       </c>
       <c r="B203" t="inlineStr">
         <is>
-          <t>13:51</t>
+          <t>13:46</t>
         </is>
       </c>
       <c r="C203" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>225_GOMEZ</t>
         </is>
       </c>
       <c r="D203" t="n">
-        <v>51</v>
+        <v>14</v>
       </c>
       <c r="E203" t="inlineStr">
         <is>
@@ -5428,16 +5428,16 @@
       </c>
       <c r="B204" t="inlineStr">
         <is>
-          <t>13:59</t>
+          <t>13:47</t>
         </is>
       </c>
       <c r="C204" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>225_GOMEZ</t>
         </is>
       </c>
       <c r="D204" t="n">
-        <v>59</v>
+        <v>47</v>
       </c>
       <c r="E204" t="inlineStr">
         <is>
@@ -5448,21 +5448,21 @@
     <row r="205">
       <c r="A205" t="inlineStr">
         <is>
-          <t>13:00:14</t>
+          <t>13:32:57</t>
         </is>
       </c>
       <c r="B205" t="inlineStr">
         <is>
-          <t>14:03</t>
+          <t>13:51</t>
         </is>
       </c>
       <c r="C205" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D205" t="n">
-        <v>63</v>
+        <v>19</v>
       </c>
       <c r="E205" t="inlineStr">
         <is>
@@ -5473,21 +5473,21 @@
     <row r="206">
       <c r="A206" t="inlineStr">
         <is>
-          <t>12:28:38</t>
+          <t>13:32:57</t>
         </is>
       </c>
       <c r="B206" t="inlineStr">
         <is>
-          <t>14:16</t>
+          <t>13:58</t>
         </is>
       </c>
       <c r="C206" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D206" t="n">
-        <v>108</v>
+        <v>26</v>
       </c>
       <c r="E206" t="inlineStr">
         <is>
@@ -5503,16 +5503,16 @@
       </c>
       <c r="B207" t="inlineStr">
         <is>
-          <t>14:17</t>
+          <t>13:59</t>
         </is>
       </c>
       <c r="C207" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D207" t="n">
-        <v>77</v>
+        <v>59</v>
       </c>
       <c r="E207" t="inlineStr">
         <is>
@@ -5523,21 +5523,21 @@
     <row r="208">
       <c r="A208" t="inlineStr">
         <is>
-          <t>13:00:14</t>
+          <t>13:32:57</t>
         </is>
       </c>
       <c r="B208" t="inlineStr">
         <is>
-          <t>14:17</t>
+          <t>13:59</t>
         </is>
       </c>
       <c r="C208" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D208" t="n">
-        <v>77</v>
+        <v>27</v>
       </c>
       <c r="E208" t="inlineStr">
         <is>
@@ -5548,21 +5548,21 @@
     <row r="209">
       <c r="A209" t="inlineStr">
         <is>
-          <t>13:00:14</t>
+          <t>13:32:57</t>
         </is>
       </c>
       <c r="B209" t="inlineStr">
         <is>
-          <t>14:19</t>
+          <t>14:02</t>
         </is>
       </c>
       <c r="C209" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D209" t="n">
-        <v>79</v>
+        <v>30</v>
       </c>
       <c r="E209" t="inlineStr">
         <is>
@@ -5578,16 +5578,16 @@
       </c>
       <c r="B210" t="inlineStr">
         <is>
-          <t>14:33</t>
+          <t>14:03</t>
         </is>
       </c>
       <c r="C210" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D210" t="n">
-        <v>93</v>
+        <v>63</v>
       </c>
       <c r="E210" t="inlineStr">
         <is>
@@ -5598,21 +5598,21 @@
     <row r="211">
       <c r="A211" t="inlineStr">
         <is>
-          <t>13:00:14</t>
+          <t>13:32:57</t>
         </is>
       </c>
       <c r="B211" t="inlineStr">
         <is>
-          <t>14:38</t>
+          <t>14:03</t>
         </is>
       </c>
       <c r="C211" t="inlineStr">
         <is>
-          <t>15X38_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D211" t="n">
-        <v>98</v>
+        <v>31</v>
       </c>
       <c r="E211" t="inlineStr">
         <is>
@@ -5623,12 +5623,12 @@
     <row r="212">
       <c r="A212" t="inlineStr">
         <is>
-          <t>13:00:14</t>
+          <t>13:32:57</t>
         </is>
       </c>
       <c r="B212" t="inlineStr">
         <is>
-          <t>14:47</t>
+          <t>14:16</t>
         </is>
       </c>
       <c r="C212" t="inlineStr">
@@ -5637,7 +5637,7 @@
         </is>
       </c>
       <c r="D212" t="n">
-        <v>107</v>
+        <v>44</v>
       </c>
       <c r="E212" t="inlineStr">
         <is>
@@ -5648,23 +5648,398 @@
     <row r="213">
       <c r="A213" t="inlineStr">
         <is>
+          <t>13:32:57</t>
+        </is>
+      </c>
+      <c r="B213" t="inlineStr">
+        <is>
+          <t>14:16</t>
+        </is>
+      </c>
+      <c r="C213" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D213" t="n">
+        <v>44</v>
+      </c>
+      <c r="E213" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="214">
+      <c r="A214" t="inlineStr">
+        <is>
           <t>13:00:14</t>
         </is>
       </c>
-      <c r="B213" t="inlineStr">
+      <c r="B214" t="inlineStr">
+        <is>
+          <t>14:17</t>
+        </is>
+      </c>
+      <c r="C214" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D214" t="n">
+        <v>77</v>
+      </c>
+      <c r="E214" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="215">
+      <c r="A215" t="inlineStr">
+        <is>
+          <t>13:00:14</t>
+        </is>
+      </c>
+      <c r="B215" t="inlineStr">
+        <is>
+          <t>14:17</t>
+        </is>
+      </c>
+      <c r="C215" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D215" t="n">
+        <v>77</v>
+      </c>
+      <c r="E215" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="216">
+      <c r="A216" t="inlineStr">
+        <is>
+          <t>13:32:57</t>
+        </is>
+      </c>
+      <c r="B216" t="inlineStr">
+        <is>
+          <t>14:18</t>
+        </is>
+      </c>
+      <c r="C216" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D216" t="n">
+        <v>46</v>
+      </c>
+      <c r="E216" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="217">
+      <c r="A217" t="inlineStr">
+        <is>
+          <t>13:00:14</t>
+        </is>
+      </c>
+      <c r="B217" t="inlineStr">
+        <is>
+          <t>14:19</t>
+        </is>
+      </c>
+      <c r="C217" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D217" t="n">
+        <v>79</v>
+      </c>
+      <c r="E217" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="218">
+      <c r="A218" t="inlineStr">
+        <is>
+          <t>13:32:57</t>
+        </is>
+      </c>
+      <c r="B218" t="inlineStr">
+        <is>
+          <t>14:21</t>
+        </is>
+      </c>
+      <c r="C218" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D218" t="n">
+        <v>49</v>
+      </c>
+      <c r="E218" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="219">
+      <c r="A219" t="inlineStr">
+        <is>
+          <t>13:32:57</t>
+        </is>
+      </c>
+      <c r="B219" t="inlineStr">
+        <is>
+          <t>14:32</t>
+        </is>
+      </c>
+      <c r="C219" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D219" t="n">
+        <v>60</v>
+      </c>
+      <c r="E219" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="220">
+      <c r="A220" t="inlineStr">
+        <is>
+          <t>13:00:14</t>
+        </is>
+      </c>
+      <c r="B220" t="inlineStr">
+        <is>
+          <t>14:33</t>
+        </is>
+      </c>
+      <c r="C220" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D220" t="n">
+        <v>93</v>
+      </c>
+      <c r="E220" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="221">
+      <c r="A221" t="inlineStr">
+        <is>
+          <t>13:32:57</t>
+        </is>
+      </c>
+      <c r="B221" t="inlineStr">
+        <is>
+          <t>14:38</t>
+        </is>
+      </c>
+      <c r="C221" t="inlineStr">
+        <is>
+          <t>15X38_ABASTO</t>
+        </is>
+      </c>
+      <c r="D221" t="n">
+        <v>66</v>
+      </c>
+      <c r="E221" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="222">
+      <c r="A222" t="inlineStr">
+        <is>
+          <t>13:32:57</t>
+        </is>
+      </c>
+      <c r="B222" t="inlineStr">
+        <is>
+          <t>14:46</t>
+        </is>
+      </c>
+      <c r="C222" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D222" t="n">
+        <v>74</v>
+      </c>
+      <c r="E222" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="223">
+      <c r="A223" t="inlineStr">
+        <is>
+          <t>13:00:14</t>
+        </is>
+      </c>
+      <c r="B223" t="inlineStr">
+        <is>
+          <t>14:47</t>
+        </is>
+      </c>
+      <c r="C223" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D223" t="n">
+        <v>107</v>
+      </c>
+      <c r="E223" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="224">
+      <c r="A224" t="inlineStr">
+        <is>
+          <t>13:32:57</t>
+        </is>
+      </c>
+      <c r="B224" t="inlineStr">
         <is>
           <t>14:51</t>
         </is>
       </c>
-      <c r="C213" t="inlineStr">
+      <c r="C224" t="inlineStr">
         <is>
           <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
-      <c r="D213" t="n">
+      <c r="D224" t="n">
+        <v>79</v>
+      </c>
+      <c r="E224" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="225">
+      <c r="A225" t="inlineStr">
+        <is>
+          <t>13:32:57</t>
+        </is>
+      </c>
+      <c r="B225" t="inlineStr">
+        <is>
+          <t>14:58</t>
+        </is>
+      </c>
+      <c r="C225" t="inlineStr">
+        <is>
+          <t>81_EL PELIGRO</t>
+        </is>
+      </c>
+      <c r="D225" t="n">
+        <v>86</v>
+      </c>
+      <c r="E225" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="226">
+      <c r="A226" t="inlineStr">
+        <is>
+          <t>13:32:57</t>
+        </is>
+      </c>
+      <c r="B226" t="inlineStr">
+        <is>
+          <t>14:59</t>
+        </is>
+      </c>
+      <c r="C226" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D226" t="n">
+        <v>87</v>
+      </c>
+      <c r="E226" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="227">
+      <c r="A227" t="inlineStr">
+        <is>
+          <t>13:32:57</t>
+        </is>
+      </c>
+      <c r="B227" t="inlineStr">
+        <is>
+          <t>15:18</t>
+        </is>
+      </c>
+      <c r="C227" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D227" t="n">
+        <v>106</v>
+      </c>
+      <c r="E227" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="228">
+      <c r="A228" t="inlineStr">
+        <is>
+          <t>13:32:57</t>
+        </is>
+      </c>
+      <c r="B228" t="inlineStr">
+        <is>
+          <t>15:23</t>
+        </is>
+      </c>
+      <c r="C228" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D228" t="n">
         <v>111</v>
       </c>
-      <c r="E213" t="inlineStr">
+      <c r="E228" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -5681,7 +6056,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E39"/>
+  <dimension ref="A1:E43"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5694,14 +6069,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 13:00:14</t>
+          <t>Última actualización: 13:32:57</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 34</t>
+          <t>Total filas: 38</t>
         </is>
       </c>
     </row>
@@ -6535,12 +6910,12 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>13:00:14</t>
+          <t>13:32:57</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>13:38</t>
+          <t>13:37</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
@@ -6549,7 +6924,7 @@
         </is>
       </c>
       <c r="D38" t="n">
-        <v>38</v>
+        <v>5</v>
       </c>
       <c r="E38" t="inlineStr">
         <is>
@@ -6565,18 +6940,118 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
+          <t>13:38</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D39" t="n">
+        <v>38</v>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>13:32:57</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>14:18</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D40" t="n">
+        <v>46</v>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>13:00:14</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
           <t>14:19</t>
         </is>
       </c>
-      <c r="C39" t="inlineStr">
+      <c r="C41" t="inlineStr">
         <is>
           <t>215C_EL PATO</t>
         </is>
       </c>
-      <c r="D39" t="n">
+      <c r="D41" t="n">
         <v>79</v>
       </c>
-      <c r="E39" t="inlineStr">
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>13:32:57</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>14:59</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D42" t="n">
+        <v>87</v>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>13:32:57</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>15:18</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D43" t="n">
+        <v>106</v>
+      </c>
+      <c r="E43" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -6593,7 +7068,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E43"/>
+  <dimension ref="A1:E45"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6606,14 +7081,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 13:00:14</t>
+          <t>Última actualización: 13:32:57</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 38</t>
+          <t>Total filas: 40</t>
         </is>
       </c>
     </row>
@@ -7547,7 +8022,7 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>12:48:06</t>
+          <t>13:32:57</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -7561,7 +8036,7 @@
         </is>
       </c>
       <c r="D42" t="n">
-        <v>69</v>
+        <v>25</v>
       </c>
       <c r="E42" t="inlineStr">
         <is>
@@ -7572,25 +8047,75 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
+          <t>13:32:57</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>14:45</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D43" t="n">
+        <v>73</v>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
           <t>13:00:14</t>
         </is>
       </c>
-      <c r="B43" t="inlineStr">
+      <c r="B44" t="inlineStr">
         <is>
           <t>14:46</t>
         </is>
       </c>
-      <c r="C43" t="inlineStr">
+      <c r="C44" t="inlineStr">
         <is>
           <t>215C_LA PLATA</t>
         </is>
       </c>
-      <c r="D43" t="n">
+      <c r="D44" t="n">
         <v>106</v>
       </c>
-      <c r="E43" t="inlineStr">
+      <c r="E44" t="inlineStr">
         <is>
           <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>13:32:57</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>15:05</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>215A_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D45" t="n">
+        <v>93</v>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>L6173</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 1810
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-03-21.xlsx
+++ b/data/horarios-141-2026-03-21.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E228"/>
+  <dimension ref="A1:E236"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 13:32:57</t>
+          <t>Última actualización: 13:57:43</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 223</t>
+          <t>Total filas: 231</t>
         </is>
       </c>
     </row>
@@ -758,7 +758,7 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D17" t="n">
@@ -783,7 +783,7 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D18" t="n">
@@ -1873,7 +1873,7 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>06:59:30</t>
+          <t>08:14:14</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
@@ -1883,11 +1883,11 @@
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D62" t="n">
-        <v>75</v>
+        <v>0</v>
       </c>
       <c r="E62" t="inlineStr">
         <is>
@@ -1923,7 +1923,7 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>08:14:14</t>
+          <t>06:59:30</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
@@ -1933,11 +1933,11 @@
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D64" t="n">
-        <v>0</v>
+        <v>75</v>
       </c>
       <c r="E64" t="inlineStr">
         <is>
@@ -1973,7 +1973,7 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>07:51:37</t>
+          <t>07:27:35</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
@@ -1983,11 +1983,11 @@
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D66" t="n">
-        <v>28</v>
+        <v>52</v>
       </c>
       <c r="E66" t="inlineStr">
         <is>
@@ -1998,7 +1998,7 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>07:27:35</t>
+          <t>07:51:37</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
@@ -2008,11 +2008,11 @@
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D67" t="n">
-        <v>52</v>
+        <v>28</v>
       </c>
       <c r="E67" t="inlineStr">
         <is>
@@ -2033,7 +2033,7 @@
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D68" t="n">
@@ -2383,7 +2383,7 @@
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D82" t="n">
@@ -2398,7 +2398,7 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>07:27:35</t>
+          <t>08:50:55</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
@@ -2408,11 +2408,11 @@
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D83" t="n">
-        <v>84</v>
+        <v>1</v>
       </c>
       <c r="E83" t="inlineStr">
         <is>
@@ -2423,7 +2423,7 @@
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>08:50:55</t>
+          <t>07:27:35</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
@@ -2433,11 +2433,11 @@
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D84" t="n">
-        <v>1</v>
+        <v>84</v>
       </c>
       <c r="E84" t="inlineStr">
         <is>
@@ -3083,7 +3083,7 @@
       </c>
       <c r="C110" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D110" t="n">
@@ -3108,7 +3108,7 @@
       </c>
       <c r="C111" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D111" t="n">
@@ -3173,7 +3173,7 @@
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>08:50:55</t>
+          <t>09:23:24</t>
         </is>
       </c>
       <c r="B114" t="inlineStr">
@@ -3183,11 +3183,11 @@
       </c>
       <c r="C114" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D114" t="n">
-        <v>73</v>
+        <v>40</v>
       </c>
       <c r="E114" t="inlineStr">
         <is>
@@ -3198,7 +3198,7 @@
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>09:23:24</t>
+          <t>08:50:55</t>
         </is>
       </c>
       <c r="B115" t="inlineStr">
@@ -3208,11 +3208,11 @@
       </c>
       <c r="C115" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D115" t="n">
-        <v>40</v>
+        <v>73</v>
       </c>
       <c r="E115" t="inlineStr">
         <is>
@@ -3498,7 +3498,7 @@
     <row r="127">
       <c r="A127" t="inlineStr">
         <is>
-          <t>08:36:09</t>
+          <t>10:14:52</t>
         </is>
       </c>
       <c r="B127" t="inlineStr">
@@ -3508,11 +3508,11 @@
       </c>
       <c r="C127" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D127" t="n">
-        <v>117</v>
+        <v>19</v>
       </c>
       <c r="E127" t="inlineStr">
         <is>
@@ -3523,7 +3523,7 @@
     <row r="128">
       <c r="A128" t="inlineStr">
         <is>
-          <t>10:14:52</t>
+          <t>08:36:09</t>
         </is>
       </c>
       <c r="B128" t="inlineStr">
@@ -3533,11 +3533,11 @@
       </c>
       <c r="C128" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D128" t="n">
-        <v>19</v>
+        <v>117</v>
       </c>
       <c r="E128" t="inlineStr">
         <is>
@@ -3598,7 +3598,7 @@
     <row r="131">
       <c r="A131" t="inlineStr">
         <is>
-          <t>10:14:52</t>
+          <t>09:23:24</t>
         </is>
       </c>
       <c r="B131" t="inlineStr">
@@ -3608,11 +3608,11 @@
       </c>
       <c r="C131" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D131" t="n">
-        <v>29</v>
+        <v>80</v>
       </c>
       <c r="E131" t="inlineStr">
         <is>
@@ -3623,7 +3623,7 @@
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t>09:23:24</t>
+          <t>10:14:52</t>
         </is>
       </c>
       <c r="B132" t="inlineStr">
@@ -3633,11 +3633,11 @@
       </c>
       <c r="C132" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D132" t="n">
-        <v>80</v>
+        <v>29</v>
       </c>
       <c r="E132" t="inlineStr">
         <is>
@@ -4123,7 +4123,7 @@
     <row r="152">
       <c r="A152" t="inlineStr">
         <is>
-          <t>10:14:52</t>
+          <t>11:16:36</t>
         </is>
       </c>
       <c r="B152" t="inlineStr">
@@ -4133,11 +4133,11 @@
       </c>
       <c r="C152" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D152" t="n">
-        <v>78</v>
+        <v>16</v>
       </c>
       <c r="E152" t="inlineStr">
         <is>
@@ -4148,7 +4148,7 @@
     <row r="153">
       <c r="A153" t="inlineStr">
         <is>
-          <t>11:16:36</t>
+          <t>10:14:52</t>
         </is>
       </c>
       <c r="B153" t="inlineStr">
@@ -4158,11 +4158,11 @@
       </c>
       <c r="C153" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D153" t="n">
-        <v>16</v>
+        <v>78</v>
       </c>
       <c r="E153" t="inlineStr">
         <is>
@@ -4183,7 +4183,7 @@
       </c>
       <c r="C154" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D154" t="n">
@@ -4208,7 +4208,7 @@
       </c>
       <c r="C155" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D155" t="n">
@@ -4473,7 +4473,7 @@
     <row r="166">
       <c r="A166" t="inlineStr">
         <is>
-          <t>11:16:36</t>
+          <t>12:00:15</t>
         </is>
       </c>
       <c r="B166" t="inlineStr">
@@ -4483,11 +4483,11 @@
       </c>
       <c r="C166" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D166" t="n">
-        <v>48</v>
+        <v>4</v>
       </c>
       <c r="E166" t="inlineStr">
         <is>
@@ -4498,7 +4498,7 @@
     <row r="167">
       <c r="A167" t="inlineStr">
         <is>
-          <t>12:00:15</t>
+          <t>11:16:36</t>
         </is>
       </c>
       <c r="B167" t="inlineStr">
@@ -4508,11 +4508,11 @@
       </c>
       <c r="C167" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D167" t="n">
-        <v>4</v>
+        <v>48</v>
       </c>
       <c r="E167" t="inlineStr">
         <is>
@@ -4648,7 +4648,7 @@
     <row r="173">
       <c r="A173" t="inlineStr">
         <is>
-          <t>12:28:38</t>
+          <t>12:00:15</t>
         </is>
       </c>
       <c r="B173" t="inlineStr">
@@ -4658,11 +4658,11 @@
       </c>
       <c r="C173" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D173" t="n">
-        <v>5</v>
+        <v>33</v>
       </c>
       <c r="E173" t="inlineStr">
         <is>
@@ -4698,7 +4698,7 @@
     <row r="175">
       <c r="A175" t="inlineStr">
         <is>
-          <t>12:00:15</t>
+          <t>12:28:38</t>
         </is>
       </c>
       <c r="B175" t="inlineStr">
@@ -4708,11 +4708,11 @@
       </c>
       <c r="C175" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D175" t="n">
-        <v>33</v>
+        <v>5</v>
       </c>
       <c r="E175" t="inlineStr">
         <is>
@@ -4998,7 +4998,7 @@
     <row r="187">
       <c r="A187" t="inlineStr">
         <is>
-          <t>13:00:14</t>
+          <t>12:28:38</t>
         </is>
       </c>
       <c r="B187" t="inlineStr">
@@ -5008,11 +5008,11 @@
       </c>
       <c r="C187" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D187" t="n">
-        <v>3</v>
+        <v>35</v>
       </c>
       <c r="E187" t="inlineStr">
         <is>
@@ -5033,7 +5033,7 @@
       </c>
       <c r="C188" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D188" t="n">
@@ -5048,7 +5048,7 @@
     <row r="189">
       <c r="A189" t="inlineStr">
         <is>
-          <t>12:28:38</t>
+          <t>13:00:14</t>
         </is>
       </c>
       <c r="B189" t="inlineStr">
@@ -5058,11 +5058,11 @@
       </c>
       <c r="C189" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D189" t="n">
-        <v>35</v>
+        <v>3</v>
       </c>
       <c r="E189" t="inlineStr">
         <is>
@@ -5498,7 +5498,7 @@
     <row r="207">
       <c r="A207" t="inlineStr">
         <is>
-          <t>13:00:14</t>
+          <t>13:57:43</t>
         </is>
       </c>
       <c r="B207" t="inlineStr">
@@ -5512,7 +5512,7 @@
         </is>
       </c>
       <c r="D207" t="n">
-        <v>59</v>
+        <v>2</v>
       </c>
       <c r="E207" t="inlineStr">
         <is>
@@ -5548,7 +5548,7 @@
     <row r="209">
       <c r="A209" t="inlineStr">
         <is>
-          <t>13:32:57</t>
+          <t>13:57:43</t>
         </is>
       </c>
       <c r="B209" t="inlineStr">
@@ -5562,7 +5562,7 @@
         </is>
       </c>
       <c r="D209" t="n">
-        <v>30</v>
+        <v>5</v>
       </c>
       <c r="E209" t="inlineStr">
         <is>
@@ -5598,7 +5598,7 @@
     <row r="211">
       <c r="A211" t="inlineStr">
         <is>
-          <t>13:32:57</t>
+          <t>13:57:43</t>
         </is>
       </c>
       <c r="B211" t="inlineStr">
@@ -5612,7 +5612,7 @@
         </is>
       </c>
       <c r="D211" t="n">
-        <v>31</v>
+        <v>6</v>
       </c>
       <c r="E211" t="inlineStr">
         <is>
@@ -5648,7 +5648,7 @@
     <row r="213">
       <c r="A213" t="inlineStr">
         <is>
-          <t>13:32:57</t>
+          <t>13:57:43</t>
         </is>
       </c>
       <c r="B213" t="inlineStr">
@@ -5662,7 +5662,7 @@
         </is>
       </c>
       <c r="D213" t="n">
-        <v>44</v>
+        <v>19</v>
       </c>
       <c r="E213" t="inlineStr">
         <is>
@@ -5683,7 +5683,7 @@
       </c>
       <c r="C214" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D214" t="n">
@@ -5698,7 +5698,7 @@
     <row r="215">
       <c r="A215" t="inlineStr">
         <is>
-          <t>13:00:14</t>
+          <t>13:57:43</t>
         </is>
       </c>
       <c r="B215" t="inlineStr">
@@ -5708,11 +5708,11 @@
       </c>
       <c r="C215" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D215" t="n">
-        <v>77</v>
+        <v>20</v>
       </c>
       <c r="E215" t="inlineStr">
         <is>
@@ -5723,7 +5723,7 @@
     <row r="216">
       <c r="A216" t="inlineStr">
         <is>
-          <t>13:32:57</t>
+          <t>13:57:43</t>
         </is>
       </c>
       <c r="B216" t="inlineStr">
@@ -5737,7 +5737,7 @@
         </is>
       </c>
       <c r="D216" t="n">
-        <v>46</v>
+        <v>21</v>
       </c>
       <c r="E216" t="inlineStr">
         <is>
@@ -5773,7 +5773,7 @@
     <row r="218">
       <c r="A218" t="inlineStr">
         <is>
-          <t>13:32:57</t>
+          <t>13:57:43</t>
         </is>
       </c>
       <c r="B218" t="inlineStr">
@@ -5787,7 +5787,7 @@
         </is>
       </c>
       <c r="D218" t="n">
-        <v>49</v>
+        <v>24</v>
       </c>
       <c r="E218" t="inlineStr">
         <is>
@@ -5798,21 +5798,21 @@
     <row r="219">
       <c r="A219" t="inlineStr">
         <is>
-          <t>13:32:57</t>
+          <t>13:57:43</t>
         </is>
       </c>
       <c r="B219" t="inlineStr">
         <is>
-          <t>14:32</t>
+          <t>14:24</t>
         </is>
       </c>
       <c r="C219" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D219" t="n">
-        <v>60</v>
+        <v>27</v>
       </c>
       <c r="E219" t="inlineStr">
         <is>
@@ -5823,12 +5823,12 @@
     <row r="220">
       <c r="A220" t="inlineStr">
         <is>
-          <t>13:00:14</t>
+          <t>13:57:43</t>
         </is>
       </c>
       <c r="B220" t="inlineStr">
         <is>
-          <t>14:33</t>
+          <t>14:32</t>
         </is>
       </c>
       <c r="C220" t="inlineStr">
@@ -5837,7 +5837,7 @@
         </is>
       </c>
       <c r="D220" t="n">
-        <v>93</v>
+        <v>35</v>
       </c>
       <c r="E220" t="inlineStr">
         <is>
@@ -5848,21 +5848,21 @@
     <row r="221">
       <c r="A221" t="inlineStr">
         <is>
-          <t>13:32:57</t>
+          <t>13:00:14</t>
         </is>
       </c>
       <c r="B221" t="inlineStr">
         <is>
-          <t>14:38</t>
+          <t>14:33</t>
         </is>
       </c>
       <c r="C221" t="inlineStr">
         <is>
-          <t>15X38_ABASTO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D221" t="n">
-        <v>66</v>
+        <v>93</v>
       </c>
       <c r="E221" t="inlineStr">
         <is>
@@ -5873,21 +5873,21 @@
     <row r="222">
       <c r="A222" t="inlineStr">
         <is>
-          <t>13:32:57</t>
+          <t>13:57:43</t>
         </is>
       </c>
       <c r="B222" t="inlineStr">
         <is>
-          <t>14:46</t>
+          <t>14:38</t>
         </is>
       </c>
       <c r="C222" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>15X38_ABASTO</t>
         </is>
       </c>
       <c r="D222" t="n">
-        <v>74</v>
+        <v>41</v>
       </c>
       <c r="E222" t="inlineStr">
         <is>
@@ -5898,12 +5898,12 @@
     <row r="223">
       <c r="A223" t="inlineStr">
         <is>
-          <t>13:00:14</t>
+          <t>13:32:57</t>
         </is>
       </c>
       <c r="B223" t="inlineStr">
         <is>
-          <t>14:47</t>
+          <t>14:46</t>
         </is>
       </c>
       <c r="C223" t="inlineStr">
@@ -5912,7 +5912,7 @@
         </is>
       </c>
       <c r="D223" t="n">
-        <v>107</v>
+        <v>74</v>
       </c>
       <c r="E223" t="inlineStr">
         <is>
@@ -5923,21 +5923,21 @@
     <row r="224">
       <c r="A224" t="inlineStr">
         <is>
-          <t>13:32:57</t>
+          <t>13:57:43</t>
         </is>
       </c>
       <c r="B224" t="inlineStr">
         <is>
-          <t>14:51</t>
+          <t>14:47</t>
         </is>
       </c>
       <c r="C224" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D224" t="n">
-        <v>79</v>
+        <v>50</v>
       </c>
       <c r="E224" t="inlineStr">
         <is>
@@ -5948,21 +5948,21 @@
     <row r="225">
       <c r="A225" t="inlineStr">
         <is>
-          <t>13:32:57</t>
+          <t>13:57:43</t>
         </is>
       </c>
       <c r="B225" t="inlineStr">
         <is>
-          <t>14:58</t>
+          <t>14:51</t>
         </is>
       </c>
       <c r="C225" t="inlineStr">
         <is>
-          <t>81_EL PELIGRO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D225" t="n">
-        <v>86</v>
+        <v>54</v>
       </c>
       <c r="E225" t="inlineStr">
         <is>
@@ -5978,16 +5978,16 @@
       </c>
       <c r="B226" t="inlineStr">
         <is>
-          <t>14:59</t>
+          <t>14:58</t>
         </is>
       </c>
       <c r="C226" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>81_EL PELIGRO</t>
         </is>
       </c>
       <c r="D226" t="n">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="E226" t="inlineStr">
         <is>
@@ -5998,21 +5998,21 @@
     <row r="227">
       <c r="A227" t="inlineStr">
         <is>
-          <t>13:32:57</t>
+          <t>13:57:43</t>
         </is>
       </c>
       <c r="B227" t="inlineStr">
         <is>
-          <t>15:18</t>
+          <t>14:59</t>
         </is>
       </c>
       <c r="C227" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>81_EL PELIGRO</t>
         </is>
       </c>
       <c r="D227" t="n">
-        <v>106</v>
+        <v>62</v>
       </c>
       <c r="E227" t="inlineStr">
         <is>
@@ -6023,23 +6023,223 @@
     <row r="228">
       <c r="A228" t="inlineStr">
         <is>
+          <t>13:57:43</t>
+        </is>
+      </c>
+      <c r="B228" t="inlineStr">
+        <is>
+          <t>14:59</t>
+        </is>
+      </c>
+      <c r="C228" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D228" t="n">
+        <v>62</v>
+      </c>
+      <c r="E228" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="229">
+      <c r="A229" t="inlineStr">
+        <is>
+          <t>13:57:43</t>
+        </is>
+      </c>
+      <c r="B229" t="inlineStr">
+        <is>
+          <t>15:18</t>
+        </is>
+      </c>
+      <c r="C229" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D229" t="n">
+        <v>81</v>
+      </c>
+      <c r="E229" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="230">
+      <c r="A230" t="inlineStr">
+        <is>
           <t>13:32:57</t>
         </is>
       </c>
-      <c r="B228" t="inlineStr">
+      <c r="B230" t="inlineStr">
         <is>
           <t>15:23</t>
         </is>
       </c>
-      <c r="C228" t="inlineStr">
+      <c r="C230" t="inlineStr">
         <is>
           <t>11_ETCHEVERRY</t>
         </is>
       </c>
-      <c r="D228" t="n">
+      <c r="D230" t="n">
         <v>111</v>
       </c>
-      <c r="E228" t="inlineStr">
+      <c r="E230" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="231">
+      <c r="A231" t="inlineStr">
+        <is>
+          <t>13:57:43</t>
+        </is>
+      </c>
+      <c r="B231" t="inlineStr">
+        <is>
+          <t>15:38</t>
+        </is>
+      </c>
+      <c r="C231" t="inlineStr">
+        <is>
+          <t>17X38_ROMERO</t>
+        </is>
+      </c>
+      <c r="D231" t="n">
+        <v>101</v>
+      </c>
+      <c r="E231" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="232">
+      <c r="A232" t="inlineStr">
+        <is>
+          <t>13:57:43</t>
+        </is>
+      </c>
+      <c r="B232" t="inlineStr">
+        <is>
+          <t>15:41</t>
+        </is>
+      </c>
+      <c r="C232" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D232" t="n">
+        <v>104</v>
+      </c>
+      <c r="E232" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="233">
+      <c r="A233" t="inlineStr">
+        <is>
+          <t>13:57:43</t>
+        </is>
+      </c>
+      <c r="B233" t="inlineStr">
+        <is>
+          <t>15:47</t>
+        </is>
+      </c>
+      <c r="C233" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D233" t="n">
+        <v>110</v>
+      </c>
+      <c r="E233" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="234">
+      <c r="A234" t="inlineStr">
+        <is>
+          <t>13:57:43</t>
+        </is>
+      </c>
+      <c r="B234" t="inlineStr">
+        <is>
+          <t>15:51</t>
+        </is>
+      </c>
+      <c r="C234" t="inlineStr">
+        <is>
+          <t>16_P MOR-SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D234" t="n">
+        <v>114</v>
+      </c>
+      <c r="E234" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="235">
+      <c r="A235" t="inlineStr">
+        <is>
+          <t>13:57:43</t>
+        </is>
+      </c>
+      <c r="B235" t="inlineStr">
+        <is>
+          <t>15:54</t>
+        </is>
+      </c>
+      <c r="C235" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D235" t="n">
+        <v>117</v>
+      </c>
+      <c r="E235" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="236">
+      <c r="A236" t="inlineStr">
+        <is>
+          <t>13:57:43</t>
+        </is>
+      </c>
+      <c r="B236" t="inlineStr">
+        <is>
+          <t>15:56</t>
+        </is>
+      </c>
+      <c r="C236" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D236" t="n">
+        <v>119</v>
+      </c>
+      <c r="E236" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -6069,7 +6269,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 13:32:57</t>
+          <t>Última actualización: 13:57:43</t>
         </is>
       </c>
     </row>
@@ -6960,7 +7160,7 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>13:32:57</t>
+          <t>13:57:43</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
@@ -6974,7 +7174,7 @@
         </is>
       </c>
       <c r="D40" t="n">
-        <v>46</v>
+        <v>21</v>
       </c>
       <c r="E40" t="inlineStr">
         <is>
@@ -7010,7 +7210,7 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>13:32:57</t>
+          <t>13:57:43</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -7024,7 +7224,7 @@
         </is>
       </c>
       <c r="D42" t="n">
-        <v>87</v>
+        <v>62</v>
       </c>
       <c r="E42" t="inlineStr">
         <is>
@@ -7035,7 +7235,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>13:32:57</t>
+          <t>13:57:43</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
@@ -7049,7 +7249,7 @@
         </is>
       </c>
       <c r="D43" t="n">
-        <v>106</v>
+        <v>81</v>
       </c>
       <c r="E43" t="inlineStr">
         <is>
@@ -7068,7 +7268,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E45"/>
+  <dimension ref="A1:E46"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -7081,14 +7281,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 13:32:57</t>
+          <t>Última actualización: 13:57:43</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 40</t>
+          <t>Total filas: 41</t>
         </is>
       </c>
     </row>
@@ -8047,12 +8247,12 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>13:32:57</t>
+          <t>13:57:43</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>14:45</t>
+          <t>13:59</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
@@ -8061,7 +8261,7 @@
         </is>
       </c>
       <c r="D43" t="n">
-        <v>73</v>
+        <v>2</v>
       </c>
       <c r="E43" t="inlineStr">
         <is>
@@ -8072,12 +8272,12 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>13:00:14</t>
+          <t>13:57:43</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>14:46</t>
+          <t>14:45</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
@@ -8086,7 +8286,7 @@
         </is>
       </c>
       <c r="D44" t="n">
-        <v>106</v>
+        <v>48</v>
       </c>
       <c r="E44" t="inlineStr">
         <is>
@@ -8097,23 +8297,48 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>13:32:57</t>
+          <t>13:00:14</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
+          <t>14:46</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D45" t="n">
+        <v>106</v>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>13:57:43</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
           <t>15:05</t>
         </is>
       </c>
-      <c r="C45" t="inlineStr">
+      <c r="C46" t="inlineStr">
         <is>
           <t>215A_LA PLATA</t>
         </is>
       </c>
-      <c r="D45" t="n">
-        <v>93</v>
-      </c>
-      <c r="E45" t="inlineStr">
+      <c r="D46" t="n">
+        <v>68</v>
+      </c>
+      <c r="E46" t="inlineStr">
         <is>
           <t>L6173</t>
         </is>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 1811
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-03-21.xlsx
+++ b/data/horarios-141-2026-03-21.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E236"/>
+  <dimension ref="A1:E243"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 13:57:43</t>
+          <t>Última actualización: 14:21:42</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 231</t>
+          <t>Total filas: 238</t>
         </is>
       </c>
     </row>
@@ -1158,7 +1158,7 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D33" t="n">
@@ -1183,7 +1183,7 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D34" t="n">
@@ -1883,7 +1883,7 @@
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D62" t="n">
@@ -1898,7 +1898,7 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>08:14:14</t>
+          <t>06:59:30</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
@@ -1908,11 +1908,11 @@
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D63" t="n">
-        <v>0</v>
+        <v>75</v>
       </c>
       <c r="E63" t="inlineStr">
         <is>
@@ -1923,7 +1923,7 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>06:59:30</t>
+          <t>08:14:14</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
@@ -1933,11 +1933,11 @@
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D64" t="n">
-        <v>75</v>
+        <v>0</v>
       </c>
       <c r="E64" t="inlineStr">
         <is>
@@ -1973,7 +1973,7 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>07:27:35</t>
+          <t>07:51:37</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
@@ -1983,11 +1983,11 @@
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D66" t="n">
-        <v>52</v>
+        <v>28</v>
       </c>
       <c r="E66" t="inlineStr">
         <is>
@@ -2008,7 +2008,7 @@
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D67" t="n">
@@ -2023,7 +2023,7 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>07:51:37</t>
+          <t>07:27:35</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
@@ -2033,11 +2033,11 @@
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D68" t="n">
-        <v>28</v>
+        <v>52</v>
       </c>
       <c r="E68" t="inlineStr">
         <is>
@@ -2233,7 +2233,7 @@
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D76" t="n">
@@ -2258,7 +2258,7 @@
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D77" t="n">
@@ -2373,7 +2373,7 @@
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>08:50:55</t>
+          <t>07:27:35</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
@@ -2383,11 +2383,11 @@
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D82" t="n">
-        <v>1</v>
+        <v>84</v>
       </c>
       <c r="E82" t="inlineStr">
         <is>
@@ -2408,7 +2408,7 @@
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D83" t="n">
@@ -2423,7 +2423,7 @@
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>07:27:35</t>
+          <t>08:50:55</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
@@ -2433,11 +2433,11 @@
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D84" t="n">
-        <v>84</v>
+        <v>1</v>
       </c>
       <c r="E84" t="inlineStr">
         <is>
@@ -2733,7 +2733,7 @@
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>215_EL PELIGRO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D96" t="n">
@@ -2758,7 +2758,7 @@
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215_EL PELIGRO</t>
         </is>
       </c>
       <c r="D97" t="n">
@@ -2873,7 +2873,7 @@
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>07:51:37</t>
+          <t>08:36:09</t>
         </is>
       </c>
       <c r="B102" t="inlineStr">
@@ -2883,11 +2883,11 @@
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D102" t="n">
-        <v>98</v>
+        <v>53</v>
       </c>
       <c r="E102" t="inlineStr">
         <is>
@@ -2898,7 +2898,7 @@
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>08:36:09</t>
+          <t>07:51:37</t>
         </is>
       </c>
       <c r="B103" t="inlineStr">
@@ -2908,11 +2908,11 @@
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D103" t="n">
-        <v>53</v>
+        <v>98</v>
       </c>
       <c r="E103" t="inlineStr">
         <is>
@@ -3083,7 +3083,7 @@
       </c>
       <c r="C110" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D110" t="n">
@@ -3108,7 +3108,7 @@
       </c>
       <c r="C111" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D111" t="n">
@@ -3498,7 +3498,7 @@
     <row r="127">
       <c r="A127" t="inlineStr">
         <is>
-          <t>10:14:52</t>
+          <t>08:36:09</t>
         </is>
       </c>
       <c r="B127" t="inlineStr">
@@ -3508,11 +3508,11 @@
       </c>
       <c r="C127" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D127" t="n">
-        <v>19</v>
+        <v>117</v>
       </c>
       <c r="E127" t="inlineStr">
         <is>
@@ -3523,7 +3523,7 @@
     <row r="128">
       <c r="A128" t="inlineStr">
         <is>
-          <t>08:36:09</t>
+          <t>10:14:52</t>
         </is>
       </c>
       <c r="B128" t="inlineStr">
@@ -3533,11 +3533,11 @@
       </c>
       <c r="C128" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D128" t="n">
-        <v>117</v>
+        <v>19</v>
       </c>
       <c r="E128" t="inlineStr">
         <is>
@@ -3873,7 +3873,7 @@
     <row r="142">
       <c r="A142" t="inlineStr">
         <is>
-          <t>10:52:37</t>
+          <t>10:14:52</t>
         </is>
       </c>
       <c r="B142" t="inlineStr">
@@ -3883,11 +3883,11 @@
       </c>
       <c r="C142" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D142" t="n">
-        <v>11</v>
+        <v>49</v>
       </c>
       <c r="E142" t="inlineStr">
         <is>
@@ -3898,7 +3898,7 @@
     <row r="143">
       <c r="A143" t="inlineStr">
         <is>
-          <t>10:14:52</t>
+          <t>10:52:37</t>
         </is>
       </c>
       <c r="B143" t="inlineStr">
@@ -3908,11 +3908,11 @@
       </c>
       <c r="C143" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D143" t="n">
-        <v>49</v>
+        <v>11</v>
       </c>
       <c r="E143" t="inlineStr">
         <is>
@@ -4183,7 +4183,7 @@
       </c>
       <c r="C154" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D154" t="n">
@@ -4208,7 +4208,7 @@
       </c>
       <c r="C155" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D155" t="n">
@@ -4473,7 +4473,7 @@
     <row r="166">
       <c r="A166" t="inlineStr">
         <is>
-          <t>12:00:15</t>
+          <t>11:16:36</t>
         </is>
       </c>
       <c r="B166" t="inlineStr">
@@ -4483,11 +4483,11 @@
       </c>
       <c r="C166" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D166" t="n">
-        <v>4</v>
+        <v>48</v>
       </c>
       <c r="E166" t="inlineStr">
         <is>
@@ -4498,7 +4498,7 @@
     <row r="167">
       <c r="A167" t="inlineStr">
         <is>
-          <t>11:16:36</t>
+          <t>12:00:15</t>
         </is>
       </c>
       <c r="B167" t="inlineStr">
@@ -4508,11 +4508,11 @@
       </c>
       <c r="C167" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D167" t="n">
-        <v>48</v>
+        <v>4</v>
       </c>
       <c r="E167" t="inlineStr">
         <is>
@@ -5323,7 +5323,7 @@
     <row r="200">
       <c r="A200" t="inlineStr">
         <is>
-          <t>13:00:14</t>
+          <t>12:48:06</t>
         </is>
       </c>
       <c r="B200" t="inlineStr">
@@ -5333,11 +5333,11 @@
       </c>
       <c r="C200" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D200" t="n">
-        <v>38</v>
+        <v>50</v>
       </c>
       <c r="E200" t="inlineStr">
         <is>
@@ -5348,7 +5348,7 @@
     <row r="201">
       <c r="A201" t="inlineStr">
         <is>
-          <t>12:48:06</t>
+          <t>13:00:14</t>
         </is>
       </c>
       <c r="B201" t="inlineStr">
@@ -5358,11 +5358,11 @@
       </c>
       <c r="C201" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D201" t="n">
-        <v>50</v>
+        <v>38</v>
       </c>
       <c r="E201" t="inlineStr">
         <is>
@@ -5498,7 +5498,7 @@
     <row r="207">
       <c r="A207" t="inlineStr">
         <is>
-          <t>13:57:43</t>
+          <t>13:32:57</t>
         </is>
       </c>
       <c r="B207" t="inlineStr">
@@ -5508,11 +5508,11 @@
       </c>
       <c r="C207" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D207" t="n">
-        <v>2</v>
+        <v>27</v>
       </c>
       <c r="E207" t="inlineStr">
         <is>
@@ -5523,7 +5523,7 @@
     <row r="208">
       <c r="A208" t="inlineStr">
         <is>
-          <t>13:32:57</t>
+          <t>13:57:43</t>
         </is>
       </c>
       <c r="B208" t="inlineStr">
@@ -5533,11 +5533,11 @@
       </c>
       <c r="C208" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D208" t="n">
-        <v>27</v>
+        <v>2</v>
       </c>
       <c r="E208" t="inlineStr">
         <is>
@@ -5623,7 +5623,7 @@
     <row r="212">
       <c r="A212" t="inlineStr">
         <is>
-          <t>13:32:57</t>
+          <t>13:57:43</t>
         </is>
       </c>
       <c r="B212" t="inlineStr">
@@ -5633,11 +5633,11 @@
       </c>
       <c r="C212" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D212" t="n">
-        <v>44</v>
+        <v>19</v>
       </c>
       <c r="E212" t="inlineStr">
         <is>
@@ -5648,7 +5648,7 @@
     <row r="213">
       <c r="A213" t="inlineStr">
         <is>
-          <t>13:57:43</t>
+          <t>13:32:57</t>
         </is>
       </c>
       <c r="B213" t="inlineStr">
@@ -5658,11 +5658,11 @@
       </c>
       <c r="C213" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D213" t="n">
-        <v>19</v>
+        <v>44</v>
       </c>
       <c r="E213" t="inlineStr">
         <is>
@@ -5773,7 +5773,7 @@
     <row r="218">
       <c r="A218" t="inlineStr">
         <is>
-          <t>13:57:43</t>
+          <t>14:21:42</t>
         </is>
       </c>
       <c r="B218" t="inlineStr">
@@ -5787,7 +5787,7 @@
         </is>
       </c>
       <c r="D218" t="n">
-        <v>24</v>
+        <v>0</v>
       </c>
       <c r="E218" t="inlineStr">
         <is>
@@ -5798,21 +5798,21 @@
     <row r="219">
       <c r="A219" t="inlineStr">
         <is>
-          <t>13:57:43</t>
+          <t>14:21:42</t>
         </is>
       </c>
       <c r="B219" t="inlineStr">
         <is>
-          <t>14:24</t>
+          <t>14:23</t>
         </is>
       </c>
       <c r="C219" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D219" t="n">
-        <v>27</v>
+        <v>2</v>
       </c>
       <c r="E219" t="inlineStr">
         <is>
@@ -5828,16 +5828,16 @@
       </c>
       <c r="B220" t="inlineStr">
         <is>
-          <t>14:32</t>
+          <t>14:24</t>
         </is>
       </c>
       <c r="C220" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D220" t="n">
-        <v>35</v>
+        <v>27</v>
       </c>
       <c r="E220" t="inlineStr">
         <is>
@@ -5848,12 +5848,12 @@
     <row r="221">
       <c r="A221" t="inlineStr">
         <is>
-          <t>13:00:14</t>
+          <t>13:57:43</t>
         </is>
       </c>
       <c r="B221" t="inlineStr">
         <is>
-          <t>14:33</t>
+          <t>14:32</t>
         </is>
       </c>
       <c r="C221" t="inlineStr">
@@ -5862,7 +5862,7 @@
         </is>
       </c>
       <c r="D221" t="n">
-        <v>93</v>
+        <v>35</v>
       </c>
       <c r="E221" t="inlineStr">
         <is>
@@ -5873,21 +5873,21 @@
     <row r="222">
       <c r="A222" t="inlineStr">
         <is>
-          <t>13:57:43</t>
+          <t>13:00:14</t>
         </is>
       </c>
       <c r="B222" t="inlineStr">
         <is>
-          <t>14:38</t>
+          <t>14:33</t>
         </is>
       </c>
       <c r="C222" t="inlineStr">
         <is>
-          <t>15X38_ABASTO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D222" t="n">
-        <v>41</v>
+        <v>93</v>
       </c>
       <c r="E222" t="inlineStr">
         <is>
@@ -5898,21 +5898,21 @@
     <row r="223">
       <c r="A223" t="inlineStr">
         <is>
-          <t>13:32:57</t>
+          <t>14:21:42</t>
         </is>
       </c>
       <c r="B223" t="inlineStr">
         <is>
-          <t>14:46</t>
+          <t>14:33</t>
         </is>
       </c>
       <c r="C223" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D223" t="n">
-        <v>74</v>
+        <v>12</v>
       </c>
       <c r="E223" t="inlineStr">
         <is>
@@ -5923,21 +5923,21 @@
     <row r="224">
       <c r="A224" t="inlineStr">
         <is>
-          <t>13:57:43</t>
+          <t>14:21:42</t>
         </is>
       </c>
       <c r="B224" t="inlineStr">
         <is>
-          <t>14:47</t>
+          <t>14:38</t>
         </is>
       </c>
       <c r="C224" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>15X38_ABASTO</t>
         </is>
       </c>
       <c r="D224" t="n">
-        <v>50</v>
+        <v>17</v>
       </c>
       <c r="E224" t="inlineStr">
         <is>
@@ -5948,21 +5948,21 @@
     <row r="225">
       <c r="A225" t="inlineStr">
         <is>
-          <t>13:57:43</t>
+          <t>13:32:57</t>
         </is>
       </c>
       <c r="B225" t="inlineStr">
         <is>
-          <t>14:51</t>
+          <t>14:46</t>
         </is>
       </c>
       <c r="C225" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D225" t="n">
-        <v>54</v>
+        <v>74</v>
       </c>
       <c r="E225" t="inlineStr">
         <is>
@@ -5973,21 +5973,21 @@
     <row r="226">
       <c r="A226" t="inlineStr">
         <is>
-          <t>13:32:57</t>
+          <t>14:21:42</t>
         </is>
       </c>
       <c r="B226" t="inlineStr">
         <is>
-          <t>14:58</t>
+          <t>14:47</t>
         </is>
       </c>
       <c r="C226" t="inlineStr">
         <is>
-          <t>81_EL PELIGRO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D226" t="n">
-        <v>86</v>
+        <v>26</v>
       </c>
       <c r="E226" t="inlineStr">
         <is>
@@ -5998,21 +5998,21 @@
     <row r="227">
       <c r="A227" t="inlineStr">
         <is>
-          <t>13:57:43</t>
+          <t>14:21:42</t>
         </is>
       </c>
       <c r="B227" t="inlineStr">
         <is>
-          <t>14:59</t>
+          <t>14:49</t>
         </is>
       </c>
       <c r="C227" t="inlineStr">
         <is>
-          <t>81_EL PELIGRO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D227" t="n">
-        <v>62</v>
+        <v>28</v>
       </c>
       <c r="E227" t="inlineStr">
         <is>
@@ -6023,21 +6023,21 @@
     <row r="228">
       <c r="A228" t="inlineStr">
         <is>
-          <t>13:57:43</t>
+          <t>14:21:42</t>
         </is>
       </c>
       <c r="B228" t="inlineStr">
         <is>
-          <t>14:59</t>
+          <t>14:51</t>
         </is>
       </c>
       <c r="C228" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D228" t="n">
-        <v>62</v>
+        <v>30</v>
       </c>
       <c r="E228" t="inlineStr">
         <is>
@@ -6048,21 +6048,21 @@
     <row r="229">
       <c r="A229" t="inlineStr">
         <is>
-          <t>13:57:43</t>
+          <t>13:32:57</t>
         </is>
       </c>
       <c r="B229" t="inlineStr">
         <is>
-          <t>15:18</t>
+          <t>14:58</t>
         </is>
       </c>
       <c r="C229" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>81_EL PELIGRO</t>
         </is>
       </c>
       <c r="D229" t="n">
-        <v>81</v>
+        <v>86</v>
       </c>
       <c r="E229" t="inlineStr">
         <is>
@@ -6073,21 +6073,21 @@
     <row r="230">
       <c r="A230" t="inlineStr">
         <is>
-          <t>13:32:57</t>
+          <t>14:21:42</t>
         </is>
       </c>
       <c r="B230" t="inlineStr">
         <is>
-          <t>15:23</t>
+          <t>14:59</t>
         </is>
       </c>
       <c r="C230" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>81_EL PELIGRO</t>
         </is>
       </c>
       <c r="D230" t="n">
-        <v>111</v>
+        <v>38</v>
       </c>
       <c r="E230" t="inlineStr">
         <is>
@@ -6098,21 +6098,21 @@
     <row r="231">
       <c r="A231" t="inlineStr">
         <is>
-          <t>13:57:43</t>
+          <t>14:21:42</t>
         </is>
       </c>
       <c r="B231" t="inlineStr">
         <is>
-          <t>15:38</t>
+          <t>14:59</t>
         </is>
       </c>
       <c r="C231" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D231" t="n">
-        <v>101</v>
+        <v>38</v>
       </c>
       <c r="E231" t="inlineStr">
         <is>
@@ -6123,21 +6123,21 @@
     <row r="232">
       <c r="A232" t="inlineStr">
         <is>
-          <t>13:57:43</t>
+          <t>14:21:42</t>
         </is>
       </c>
       <c r="B232" t="inlineStr">
         <is>
-          <t>15:41</t>
+          <t>15:11</t>
         </is>
       </c>
       <c r="C232" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D232" t="n">
-        <v>104</v>
+        <v>50</v>
       </c>
       <c r="E232" t="inlineStr">
         <is>
@@ -6148,21 +6148,21 @@
     <row r="233">
       <c r="A233" t="inlineStr">
         <is>
-          <t>13:57:43</t>
+          <t>14:21:42</t>
         </is>
       </c>
       <c r="B233" t="inlineStr">
         <is>
-          <t>15:47</t>
+          <t>15:18</t>
         </is>
       </c>
       <c r="C233" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D233" t="n">
-        <v>110</v>
+        <v>57</v>
       </c>
       <c r="E233" t="inlineStr">
         <is>
@@ -6173,21 +6173,21 @@
     <row r="234">
       <c r="A234" t="inlineStr">
         <is>
-          <t>13:57:43</t>
+          <t>14:21:42</t>
         </is>
       </c>
       <c r="B234" t="inlineStr">
         <is>
-          <t>15:51</t>
+          <t>15:23</t>
         </is>
       </c>
       <c r="C234" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D234" t="n">
-        <v>114</v>
+        <v>62</v>
       </c>
       <c r="E234" t="inlineStr">
         <is>
@@ -6198,21 +6198,21 @@
     <row r="235">
       <c r="A235" t="inlineStr">
         <is>
-          <t>13:57:43</t>
+          <t>14:21:42</t>
         </is>
       </c>
       <c r="B235" t="inlineStr">
         <is>
-          <t>15:54</t>
+          <t>15:38</t>
         </is>
       </c>
       <c r="C235" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D235" t="n">
-        <v>117</v>
+        <v>77</v>
       </c>
       <c r="E235" t="inlineStr">
         <is>
@@ -6223,23 +6223,198 @@
     <row r="236">
       <c r="A236" t="inlineStr">
         <is>
+          <t>14:21:42</t>
+        </is>
+      </c>
+      <c r="B236" t="inlineStr">
+        <is>
+          <t>15:41</t>
+        </is>
+      </c>
+      <c r="C236" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D236" t="n">
+        <v>80</v>
+      </c>
+      <c r="E236" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="237">
+      <c r="A237" t="inlineStr">
+        <is>
+          <t>14:21:42</t>
+        </is>
+      </c>
+      <c r="B237" t="inlineStr">
+        <is>
+          <t>15:47</t>
+        </is>
+      </c>
+      <c r="C237" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D237" t="n">
+        <v>86</v>
+      </c>
+      <c r="E237" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="238">
+      <c r="A238" t="inlineStr">
+        <is>
+          <t>14:21:42</t>
+        </is>
+      </c>
+      <c r="B238" t="inlineStr">
+        <is>
+          <t>15:51</t>
+        </is>
+      </c>
+      <c r="C238" t="inlineStr">
+        <is>
+          <t>16_P MOR-SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D238" t="n">
+        <v>90</v>
+      </c>
+      <c r="E238" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="239">
+      <c r="A239" t="inlineStr">
+        <is>
+          <t>14:21:42</t>
+        </is>
+      </c>
+      <c r="B239" t="inlineStr">
+        <is>
+          <t>15:54</t>
+        </is>
+      </c>
+      <c r="C239" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D239" t="n">
+        <v>93</v>
+      </c>
+      <c r="E239" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="240">
+      <c r="A240" t="inlineStr">
+        <is>
           <t>13:57:43</t>
         </is>
       </c>
-      <c r="B236" t="inlineStr">
+      <c r="B240" t="inlineStr">
         <is>
           <t>15:56</t>
         </is>
       </c>
-      <c r="C236" t="inlineStr">
+      <c r="C240" t="inlineStr">
         <is>
           <t>27_EL RETIRO</t>
         </is>
       </c>
-      <c r="D236" t="n">
+      <c r="D240" t="n">
         <v>119</v>
       </c>
-      <c r="E236" t="inlineStr">
+      <c r="E240" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="241">
+      <c r="A241" t="inlineStr">
+        <is>
+          <t>14:21:42</t>
+        </is>
+      </c>
+      <c r="B241" t="inlineStr">
+        <is>
+          <t>15:57</t>
+        </is>
+      </c>
+      <c r="C241" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D241" t="n">
+        <v>96</v>
+      </c>
+      <c r="E241" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="242">
+      <c r="A242" t="inlineStr">
+        <is>
+          <t>14:21:42</t>
+        </is>
+      </c>
+      <c r="B242" t="inlineStr">
+        <is>
+          <t>16:09</t>
+        </is>
+      </c>
+      <c r="C242" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D242" t="n">
+        <v>108</v>
+      </c>
+      <c r="E242" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="243">
+      <c r="A243" t="inlineStr">
+        <is>
+          <t>14:21:42</t>
+        </is>
+      </c>
+      <c r="B243" t="inlineStr">
+        <is>
+          <t>16:11</t>
+        </is>
+      </c>
+      <c r="C243" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D243" t="n">
+        <v>110</v>
+      </c>
+      <c r="E243" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -6269,7 +6444,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 13:57:43</t>
+          <t>Última actualización: 14:21:42</t>
         </is>
       </c>
     </row>
@@ -7210,7 +7385,7 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>13:57:43</t>
+          <t>14:21:42</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -7224,7 +7399,7 @@
         </is>
       </c>
       <c r="D42" t="n">
-        <v>62</v>
+        <v>38</v>
       </c>
       <c r="E42" t="inlineStr">
         <is>
@@ -7235,7 +7410,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>13:57:43</t>
+          <t>14:21:42</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
@@ -7249,7 +7424,7 @@
         </is>
       </c>
       <c r="D43" t="n">
-        <v>81</v>
+        <v>57</v>
       </c>
       <c r="E43" t="inlineStr">
         <is>
@@ -7268,7 +7443,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E46"/>
+  <dimension ref="A1:E48"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -7281,14 +7456,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 13:57:43</t>
+          <t>Última actualización: 14:21:42</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 41</t>
+          <t>Total filas: 43</t>
         </is>
       </c>
     </row>
@@ -8272,7 +8447,7 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>13:57:43</t>
+          <t>14:21:42</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
@@ -8286,7 +8461,7 @@
         </is>
       </c>
       <c r="D44" t="n">
-        <v>48</v>
+        <v>24</v>
       </c>
       <c r="E44" t="inlineStr">
         <is>
@@ -8341,6 +8516,56 @@
       <c r="E46" t="inlineStr">
         <is>
           <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>14:21:42</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>15:06</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>215A_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D47" t="n">
+        <v>45</v>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>14:21:42</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>15:45</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D48" t="n">
+        <v>84</v>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>L6203</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 1812
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-03-21.xlsx
+++ b/data/horarios-141-2026-03-21.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E243"/>
+  <dimension ref="A1:E251"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 14:21:42</t>
+          <t>Última actualización: 14:46:40</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 238</t>
+          <t>Total filas: 246</t>
         </is>
       </c>
     </row>
@@ -1873,7 +1873,7 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>08:14:14</t>
+          <t>06:59:30</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
@@ -1883,11 +1883,11 @@
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D62" t="n">
-        <v>0</v>
+        <v>75</v>
       </c>
       <c r="E62" t="inlineStr">
         <is>
@@ -1898,7 +1898,7 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>06:59:30</t>
+          <t>08:14:14</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
@@ -1908,11 +1908,11 @@
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D63" t="n">
-        <v>75</v>
+        <v>0</v>
       </c>
       <c r="E63" t="inlineStr">
         <is>
@@ -1933,7 +1933,7 @@
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D64" t="n">
@@ -1998,7 +1998,7 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>07:51:37</t>
+          <t>07:27:35</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
@@ -2008,11 +2008,11 @@
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D67" t="n">
-        <v>28</v>
+        <v>52</v>
       </c>
       <c r="E67" t="inlineStr">
         <is>
@@ -2023,7 +2023,7 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>07:27:35</t>
+          <t>07:51:37</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
@@ -2033,11 +2033,11 @@
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D68" t="n">
-        <v>52</v>
+        <v>28</v>
       </c>
       <c r="E68" t="inlineStr">
         <is>
@@ -2373,7 +2373,7 @@
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>07:27:35</t>
+          <t>08:50:55</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
@@ -2383,11 +2383,11 @@
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D82" t="n">
-        <v>84</v>
+        <v>1</v>
       </c>
       <c r="E82" t="inlineStr">
         <is>
@@ -2408,7 +2408,7 @@
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D83" t="n">
@@ -2423,7 +2423,7 @@
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>08:50:55</t>
+          <t>07:27:35</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
@@ -2433,11 +2433,11 @@
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D84" t="n">
-        <v>1</v>
+        <v>84</v>
       </c>
       <c r="E84" t="inlineStr">
         <is>
@@ -2698,7 +2698,7 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>08:14:14</t>
+          <t>08:50:55</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
@@ -2708,11 +2708,11 @@
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D95" t="n">
-        <v>64</v>
+        <v>28</v>
       </c>
       <c r="E95" t="inlineStr">
         <is>
@@ -2733,7 +2733,7 @@
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215_EL PELIGRO</t>
         </is>
       </c>
       <c r="D96" t="n">
@@ -2748,7 +2748,7 @@
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>08:50:55</t>
+          <t>08:14:14</t>
         </is>
       </c>
       <c r="B97" t="inlineStr">
@@ -2758,11 +2758,11 @@
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>215_EL PELIGRO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D97" t="n">
-        <v>28</v>
+        <v>64</v>
       </c>
       <c r="E97" t="inlineStr">
         <is>
@@ -2873,7 +2873,7 @@
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>08:36:09</t>
+          <t>07:51:37</t>
         </is>
       </c>
       <c r="B102" t="inlineStr">
@@ -2883,11 +2883,11 @@
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D102" t="n">
-        <v>53</v>
+        <v>98</v>
       </c>
       <c r="E102" t="inlineStr">
         <is>
@@ -2898,7 +2898,7 @@
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>07:51:37</t>
+          <t>08:36:09</t>
         </is>
       </c>
       <c r="B103" t="inlineStr">
@@ -2908,11 +2908,11 @@
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D103" t="n">
-        <v>98</v>
+        <v>53</v>
       </c>
       <c r="E103" t="inlineStr">
         <is>
@@ -3173,7 +3173,7 @@
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>09:23:24</t>
+          <t>08:50:55</t>
         </is>
       </c>
       <c r="B114" t="inlineStr">
@@ -3183,11 +3183,11 @@
       </c>
       <c r="C114" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D114" t="n">
-        <v>40</v>
+        <v>73</v>
       </c>
       <c r="E114" t="inlineStr">
         <is>
@@ -3198,7 +3198,7 @@
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>08:50:55</t>
+          <t>09:23:24</t>
         </is>
       </c>
       <c r="B115" t="inlineStr">
@@ -3208,11 +3208,11 @@
       </c>
       <c r="C115" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D115" t="n">
-        <v>73</v>
+        <v>40</v>
       </c>
       <c r="E115" t="inlineStr">
         <is>
@@ -3598,7 +3598,7 @@
     <row r="131">
       <c r="A131" t="inlineStr">
         <is>
-          <t>09:23:24</t>
+          <t>10:14:52</t>
         </is>
       </c>
       <c r="B131" t="inlineStr">
@@ -3608,11 +3608,11 @@
       </c>
       <c r="C131" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D131" t="n">
-        <v>80</v>
+        <v>29</v>
       </c>
       <c r="E131" t="inlineStr">
         <is>
@@ -3623,7 +3623,7 @@
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t>10:14:52</t>
+          <t>09:23:24</t>
         </is>
       </c>
       <c r="B132" t="inlineStr">
@@ -3633,11 +3633,11 @@
       </c>
       <c r="C132" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D132" t="n">
-        <v>29</v>
+        <v>80</v>
       </c>
       <c r="E132" t="inlineStr">
         <is>
@@ -5673,7 +5673,7 @@
     <row r="214">
       <c r="A214" t="inlineStr">
         <is>
-          <t>13:00:14</t>
+          <t>13:57:43</t>
         </is>
       </c>
       <c r="B214" t="inlineStr">
@@ -5683,11 +5683,11 @@
       </c>
       <c r="C214" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D214" t="n">
-        <v>77</v>
+        <v>20</v>
       </c>
       <c r="E214" t="inlineStr">
         <is>
@@ -5698,7 +5698,7 @@
     <row r="215">
       <c r="A215" t="inlineStr">
         <is>
-          <t>13:57:43</t>
+          <t>13:00:14</t>
         </is>
       </c>
       <c r="B215" t="inlineStr">
@@ -5708,11 +5708,11 @@
       </c>
       <c r="C215" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D215" t="n">
-        <v>20</v>
+        <v>77</v>
       </c>
       <c r="E215" t="inlineStr">
         <is>
@@ -5873,7 +5873,7 @@
     <row r="222">
       <c r="A222" t="inlineStr">
         <is>
-          <t>13:00:14</t>
+          <t>14:21:42</t>
         </is>
       </c>
       <c r="B222" t="inlineStr">
@@ -5883,11 +5883,11 @@
       </c>
       <c r="C222" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D222" t="n">
-        <v>93</v>
+        <v>12</v>
       </c>
       <c r="E222" t="inlineStr">
         <is>
@@ -5898,7 +5898,7 @@
     <row r="223">
       <c r="A223" t="inlineStr">
         <is>
-          <t>14:21:42</t>
+          <t>13:00:14</t>
         </is>
       </c>
       <c r="B223" t="inlineStr">
@@ -5908,11 +5908,11 @@
       </c>
       <c r="C223" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D223" t="n">
-        <v>12</v>
+        <v>93</v>
       </c>
       <c r="E223" t="inlineStr">
         <is>
@@ -5973,7 +5973,7 @@
     <row r="226">
       <c r="A226" t="inlineStr">
         <is>
-          <t>14:21:42</t>
+          <t>14:46:39</t>
         </is>
       </c>
       <c r="B226" t="inlineStr">
@@ -5983,11 +5983,11 @@
       </c>
       <c r="C226" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D226" t="n">
-        <v>26</v>
+        <v>1</v>
       </c>
       <c r="E226" t="inlineStr">
         <is>
@@ -5998,21 +5998,21 @@
     <row r="227">
       <c r="A227" t="inlineStr">
         <is>
-          <t>14:21:42</t>
+          <t>14:46:39</t>
         </is>
       </c>
       <c r="B227" t="inlineStr">
         <is>
-          <t>14:49</t>
+          <t>14:47</t>
         </is>
       </c>
       <c r="C227" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D227" t="n">
-        <v>28</v>
+        <v>1</v>
       </c>
       <c r="E227" t="inlineStr">
         <is>
@@ -6028,16 +6028,16 @@
       </c>
       <c r="B228" t="inlineStr">
         <is>
-          <t>14:51</t>
+          <t>14:49</t>
         </is>
       </c>
       <c r="C228" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D228" t="n">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="E228" t="inlineStr">
         <is>
@@ -6048,21 +6048,21 @@
     <row r="229">
       <c r="A229" t="inlineStr">
         <is>
-          <t>13:32:57</t>
+          <t>14:46:39</t>
         </is>
       </c>
       <c r="B229" t="inlineStr">
         <is>
-          <t>14:58</t>
+          <t>14:51</t>
         </is>
       </c>
       <c r="C229" t="inlineStr">
         <is>
-          <t>81_EL PELIGRO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D229" t="n">
-        <v>86</v>
+        <v>5</v>
       </c>
       <c r="E229" t="inlineStr">
         <is>
@@ -6073,12 +6073,12 @@
     <row r="230">
       <c r="A230" t="inlineStr">
         <is>
-          <t>14:21:42</t>
+          <t>13:32:57</t>
         </is>
       </c>
       <c r="B230" t="inlineStr">
         <is>
-          <t>14:59</t>
+          <t>14:58</t>
         </is>
       </c>
       <c r="C230" t="inlineStr">
@@ -6087,7 +6087,7 @@
         </is>
       </c>
       <c r="D230" t="n">
-        <v>38</v>
+        <v>86</v>
       </c>
       <c r="E230" t="inlineStr">
         <is>
@@ -6098,7 +6098,7 @@
     <row r="231">
       <c r="A231" t="inlineStr">
         <is>
-          <t>14:21:42</t>
+          <t>14:46:39</t>
         </is>
       </c>
       <c r="B231" t="inlineStr">
@@ -6108,11 +6108,11 @@
       </c>
       <c r="C231" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>81_EL PELIGRO</t>
         </is>
       </c>
       <c r="D231" t="n">
-        <v>38</v>
+        <v>13</v>
       </c>
       <c r="E231" t="inlineStr">
         <is>
@@ -6123,21 +6123,21 @@
     <row r="232">
       <c r="A232" t="inlineStr">
         <is>
-          <t>14:21:42</t>
+          <t>14:46:39</t>
         </is>
       </c>
       <c r="B232" t="inlineStr">
         <is>
-          <t>15:11</t>
+          <t>14:59</t>
         </is>
       </c>
       <c r="C232" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D232" t="n">
-        <v>50</v>
+        <v>13</v>
       </c>
       <c r="E232" t="inlineStr">
         <is>
@@ -6148,21 +6148,21 @@
     <row r="233">
       <c r="A233" t="inlineStr">
         <is>
-          <t>14:21:42</t>
+          <t>14:46:39</t>
         </is>
       </c>
       <c r="B233" t="inlineStr">
         <is>
-          <t>15:18</t>
+          <t>15:01</t>
         </is>
       </c>
       <c r="C233" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D233" t="n">
-        <v>57</v>
+        <v>15</v>
       </c>
       <c r="E233" t="inlineStr">
         <is>
@@ -6173,21 +6173,21 @@
     <row r="234">
       <c r="A234" t="inlineStr">
         <is>
-          <t>14:21:42</t>
+          <t>14:46:39</t>
         </is>
       </c>
       <c r="B234" t="inlineStr">
         <is>
-          <t>15:23</t>
+          <t>15:03</t>
         </is>
       </c>
       <c r="C234" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D234" t="n">
-        <v>62</v>
+        <v>17</v>
       </c>
       <c r="E234" t="inlineStr">
         <is>
@@ -6198,21 +6198,21 @@
     <row r="235">
       <c r="A235" t="inlineStr">
         <is>
-          <t>14:21:42</t>
+          <t>14:46:39</t>
         </is>
       </c>
       <c r="B235" t="inlineStr">
         <is>
-          <t>15:38</t>
+          <t>15:11</t>
         </is>
       </c>
       <c r="C235" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D235" t="n">
-        <v>77</v>
+        <v>25</v>
       </c>
       <c r="E235" t="inlineStr">
         <is>
@@ -6223,21 +6223,21 @@
     <row r="236">
       <c r="A236" t="inlineStr">
         <is>
-          <t>14:21:42</t>
+          <t>14:46:39</t>
         </is>
       </c>
       <c r="B236" t="inlineStr">
         <is>
-          <t>15:41</t>
+          <t>15:11</t>
         </is>
       </c>
       <c r="C236" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D236" t="n">
-        <v>80</v>
+        <v>25</v>
       </c>
       <c r="E236" t="inlineStr">
         <is>
@@ -6248,21 +6248,21 @@
     <row r="237">
       <c r="A237" t="inlineStr">
         <is>
-          <t>14:21:42</t>
+          <t>14:46:39</t>
         </is>
       </c>
       <c r="B237" t="inlineStr">
         <is>
-          <t>15:47</t>
+          <t>15:18</t>
         </is>
       </c>
       <c r="C237" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D237" t="n">
-        <v>86</v>
+        <v>32</v>
       </c>
       <c r="E237" t="inlineStr">
         <is>
@@ -6273,21 +6273,21 @@
     <row r="238">
       <c r="A238" t="inlineStr">
         <is>
-          <t>14:21:42</t>
+          <t>14:46:39</t>
         </is>
       </c>
       <c r="B238" t="inlineStr">
         <is>
-          <t>15:51</t>
+          <t>15:23</t>
         </is>
       </c>
       <c r="C238" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D238" t="n">
-        <v>90</v>
+        <v>37</v>
       </c>
       <c r="E238" t="inlineStr">
         <is>
@@ -6298,21 +6298,21 @@
     <row r="239">
       <c r="A239" t="inlineStr">
         <is>
-          <t>14:21:42</t>
+          <t>14:46:39</t>
         </is>
       </c>
       <c r="B239" t="inlineStr">
         <is>
-          <t>15:54</t>
+          <t>15:38</t>
         </is>
       </c>
       <c r="C239" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D239" t="n">
-        <v>93</v>
+        <v>52</v>
       </c>
       <c r="E239" t="inlineStr">
         <is>
@@ -6323,21 +6323,21 @@
     <row r="240">
       <c r="A240" t="inlineStr">
         <is>
-          <t>13:57:43</t>
+          <t>14:46:39</t>
         </is>
       </c>
       <c r="B240" t="inlineStr">
         <is>
-          <t>15:56</t>
+          <t>15:41</t>
         </is>
       </c>
       <c r="C240" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D240" t="n">
-        <v>119</v>
+        <v>55</v>
       </c>
       <c r="E240" t="inlineStr">
         <is>
@@ -6348,21 +6348,21 @@
     <row r="241">
       <c r="A241" t="inlineStr">
         <is>
-          <t>14:21:42</t>
+          <t>14:46:39</t>
         </is>
       </c>
       <c r="B241" t="inlineStr">
         <is>
-          <t>15:57</t>
+          <t>15:47</t>
         </is>
       </c>
       <c r="C241" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D241" t="n">
-        <v>96</v>
+        <v>61</v>
       </c>
       <c r="E241" t="inlineStr">
         <is>
@@ -6373,21 +6373,21 @@
     <row r="242">
       <c r="A242" t="inlineStr">
         <is>
-          <t>14:21:42</t>
+          <t>14:46:39</t>
         </is>
       </c>
       <c r="B242" t="inlineStr">
         <is>
-          <t>16:09</t>
+          <t>15:51</t>
         </is>
       </c>
       <c r="C242" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D242" t="n">
-        <v>108</v>
+        <v>65</v>
       </c>
       <c r="E242" t="inlineStr">
         <is>
@@ -6398,23 +6398,223 @@
     <row r="243">
       <c r="A243" t="inlineStr">
         <is>
+          <t>14:46:39</t>
+        </is>
+      </c>
+      <c r="B243" t="inlineStr">
+        <is>
+          <t>15:54</t>
+        </is>
+      </c>
+      <c r="C243" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D243" t="n">
+        <v>68</v>
+      </c>
+      <c r="E243" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="244">
+      <c r="A244" t="inlineStr">
+        <is>
+          <t>14:46:39</t>
+        </is>
+      </c>
+      <c r="B244" t="inlineStr">
+        <is>
+          <t>15:54</t>
+        </is>
+      </c>
+      <c r="C244" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D244" t="n">
+        <v>68</v>
+      </c>
+      <c r="E244" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="245">
+      <c r="A245" t="inlineStr">
+        <is>
+          <t>13:57:43</t>
+        </is>
+      </c>
+      <c r="B245" t="inlineStr">
+        <is>
+          <t>15:56</t>
+        </is>
+      </c>
+      <c r="C245" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D245" t="n">
+        <v>119</v>
+      </c>
+      <c r="E245" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="246">
+      <c r="A246" t="inlineStr">
+        <is>
           <t>14:21:42</t>
         </is>
       </c>
-      <c r="B243" t="inlineStr">
+      <c r="B246" t="inlineStr">
+        <is>
+          <t>15:57</t>
+        </is>
+      </c>
+      <c r="C246" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D246" t="n">
+        <v>96</v>
+      </c>
+      <c r="E246" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="247">
+      <c r="A247" t="inlineStr">
+        <is>
+          <t>14:46:39</t>
+        </is>
+      </c>
+      <c r="B247" t="inlineStr">
+        <is>
+          <t>16:09</t>
+        </is>
+      </c>
+      <c r="C247" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D247" t="n">
+        <v>83</v>
+      </c>
+      <c r="E247" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="248">
+      <c r="A248" t="inlineStr">
+        <is>
+          <t>14:46:39</t>
+        </is>
+      </c>
+      <c r="B248" t="inlineStr">
         <is>
           <t>16:11</t>
         </is>
       </c>
-      <c r="C243" t="inlineStr">
+      <c r="C248" t="inlineStr">
         <is>
           <t>14_ABASTO</t>
         </is>
       </c>
-      <c r="D243" t="n">
-        <v>110</v>
-      </c>
-      <c r="E243" t="inlineStr">
+      <c r="D248" t="n">
+        <v>85</v>
+      </c>
+      <c r="E248" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="249">
+      <c r="A249" t="inlineStr">
+        <is>
+          <t>14:46:39</t>
+        </is>
+      </c>
+      <c r="B249" t="inlineStr">
+        <is>
+          <t>16:23</t>
+        </is>
+      </c>
+      <c r="C249" t="inlineStr">
+        <is>
+          <t>215_ALUAR</t>
+        </is>
+      </c>
+      <c r="D249" t="n">
+        <v>97</v>
+      </c>
+      <c r="E249" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="250">
+      <c r="A250" t="inlineStr">
+        <is>
+          <t>14:46:39</t>
+        </is>
+      </c>
+      <c r="B250" t="inlineStr">
+        <is>
+          <t>16:35</t>
+        </is>
+      </c>
+      <c r="C250" t="inlineStr">
+        <is>
+          <t>17X38_ROMERO</t>
+        </is>
+      </c>
+      <c r="D250" t="n">
+        <v>109</v>
+      </c>
+      <c r="E250" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="251">
+      <c r="A251" t="inlineStr">
+        <is>
+          <t>14:46:39</t>
+        </is>
+      </c>
+      <c r="B251" t="inlineStr">
+        <is>
+          <t>16:35</t>
+        </is>
+      </c>
+      <c r="C251" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D251" t="n">
+        <v>109</v>
+      </c>
+      <c r="E251" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -6431,7 +6631,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E43"/>
+  <dimension ref="A1:E44"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6444,14 +6644,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 14:21:42</t>
+          <t>Última actualización: 14:46:40</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 38</t>
+          <t>Total filas: 39</t>
         </is>
       </c>
     </row>
@@ -7385,7 +7585,7 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>14:21:42</t>
+          <t>14:46:39</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -7399,7 +7599,7 @@
         </is>
       </c>
       <c r="D42" t="n">
-        <v>38</v>
+        <v>13</v>
       </c>
       <c r="E42" t="inlineStr">
         <is>
@@ -7410,7 +7610,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>14:21:42</t>
+          <t>14:46:39</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
@@ -7424,9 +7624,34 @@
         </is>
       </c>
       <c r="D43" t="n">
-        <v>57</v>
+        <v>32</v>
       </c>
       <c r="E43" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>14:46:39</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>16:23</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>215_ALUAR</t>
+        </is>
+      </c>
+      <c r="D44" t="n">
+        <v>97</v>
+      </c>
+      <c r="E44" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -7443,7 +7668,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E48"/>
+  <dimension ref="A1:E50"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -7456,14 +7681,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 14:21:42</t>
+          <t>Última actualización: 14:46:40</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 43</t>
+          <t>Total filas: 45</t>
         </is>
       </c>
     </row>
@@ -8472,7 +8697,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>13:00:14</t>
+          <t>14:46:39</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
@@ -8486,7 +8711,7 @@
         </is>
       </c>
       <c r="D45" t="n">
-        <v>106</v>
+        <v>0</v>
       </c>
       <c r="E45" t="inlineStr">
         <is>
@@ -8547,25 +8772,75 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>14:21:42</t>
+          <t>14:46:39</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
+          <t>15:10</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>215A_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D48" t="n">
+        <v>24</v>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>14:46:39</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
           <t>15:45</t>
         </is>
       </c>
-      <c r="C48" t="inlineStr">
+      <c r="C49" t="inlineStr">
         <is>
           <t>215C_LA PLATA</t>
         </is>
       </c>
-      <c r="D48" t="n">
-        <v>84</v>
-      </c>
-      <c r="E48" t="inlineStr">
+      <c r="D49" t="n">
+        <v>59</v>
+      </c>
+      <c r="E49" t="inlineStr">
         <is>
           <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>14:46:39</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>16:42</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>215B_LP-P MOR-1 Y 57</t>
+        </is>
+      </c>
+      <c r="D50" t="n">
+        <v>116</v>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>L6173</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 1813
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-03-21.xlsx
+++ b/data/horarios-141-2026-03-21.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E251"/>
+  <dimension ref="A1:E267"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 14:46:40</t>
+          <t>Última actualización: 14:59:00</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 246</t>
+          <t>Total filas: 262</t>
         </is>
       </c>
     </row>
@@ -1158,7 +1158,7 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D33" t="n">
@@ -1183,7 +1183,7 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D34" t="n">
@@ -1873,7 +1873,7 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>06:59:30</t>
+          <t>08:14:14</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
@@ -1883,11 +1883,11 @@
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D62" t="n">
-        <v>75</v>
+        <v>0</v>
       </c>
       <c r="E62" t="inlineStr">
         <is>
@@ -1923,7 +1923,7 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>08:14:14</t>
+          <t>06:59:30</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
@@ -1933,11 +1933,11 @@
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D64" t="n">
-        <v>0</v>
+        <v>75</v>
       </c>
       <c r="E64" t="inlineStr">
         <is>
@@ -1998,7 +1998,7 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>07:27:35</t>
+          <t>07:51:37</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
@@ -2008,11 +2008,11 @@
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D67" t="n">
-        <v>52</v>
+        <v>28</v>
       </c>
       <c r="E67" t="inlineStr">
         <is>
@@ -2023,7 +2023,7 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>07:51:37</t>
+          <t>07:27:35</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
@@ -2033,11 +2033,11 @@
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D68" t="n">
-        <v>28</v>
+        <v>52</v>
       </c>
       <c r="E68" t="inlineStr">
         <is>
@@ -2233,7 +2233,7 @@
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D76" t="n">
@@ -2258,7 +2258,7 @@
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D77" t="n">
@@ -2383,7 +2383,7 @@
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D82" t="n">
@@ -2408,7 +2408,7 @@
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D83" t="n">
@@ -2698,7 +2698,7 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>08:50:55</t>
+          <t>08:14:14</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
@@ -2708,11 +2708,11 @@
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D95" t="n">
-        <v>28</v>
+        <v>64</v>
       </c>
       <c r="E95" t="inlineStr">
         <is>
@@ -2733,7 +2733,7 @@
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>215_EL PELIGRO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D96" t="n">
@@ -2748,7 +2748,7 @@
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>08:14:14</t>
+          <t>08:50:55</t>
         </is>
       </c>
       <c r="B97" t="inlineStr">
@@ -2758,11 +2758,11 @@
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>215_EL PELIGRO</t>
         </is>
       </c>
       <c r="D97" t="n">
-        <v>64</v>
+        <v>28</v>
       </c>
       <c r="E97" t="inlineStr">
         <is>
@@ -2923,7 +2923,7 @@
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>09:23:24</t>
+          <t>08:14:14</t>
         </is>
       </c>
       <c r="B104" t="inlineStr">
@@ -2933,11 +2933,11 @@
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D104" t="n">
-        <v>10</v>
+        <v>79</v>
       </c>
       <c r="E104" t="inlineStr">
         <is>
@@ -2948,7 +2948,7 @@
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>08:14:14</t>
+          <t>09:23:24</t>
         </is>
       </c>
       <c r="B105" t="inlineStr">
@@ -2958,11 +2958,11 @@
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D105" t="n">
-        <v>79</v>
+        <v>10</v>
       </c>
       <c r="E105" t="inlineStr">
         <is>
@@ -3173,7 +3173,7 @@
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>08:50:55</t>
+          <t>09:23:24</t>
         </is>
       </c>
       <c r="B114" t="inlineStr">
@@ -3183,11 +3183,11 @@
       </c>
       <c r="C114" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D114" t="n">
-        <v>73</v>
+        <v>40</v>
       </c>
       <c r="E114" t="inlineStr">
         <is>
@@ -3198,7 +3198,7 @@
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>09:23:24</t>
+          <t>08:50:55</t>
         </is>
       </c>
       <c r="B115" t="inlineStr">
@@ -3208,11 +3208,11 @@
       </c>
       <c r="C115" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D115" t="n">
-        <v>40</v>
+        <v>73</v>
       </c>
       <c r="E115" t="inlineStr">
         <is>
@@ -3598,7 +3598,7 @@
     <row r="131">
       <c r="A131" t="inlineStr">
         <is>
-          <t>10:14:52</t>
+          <t>09:23:24</t>
         </is>
       </c>
       <c r="B131" t="inlineStr">
@@ -3608,11 +3608,11 @@
       </c>
       <c r="C131" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D131" t="n">
-        <v>29</v>
+        <v>80</v>
       </c>
       <c r="E131" t="inlineStr">
         <is>
@@ -3623,7 +3623,7 @@
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t>09:23:24</t>
+          <t>10:14:52</t>
         </is>
       </c>
       <c r="B132" t="inlineStr">
@@ -3633,11 +3633,11 @@
       </c>
       <c r="C132" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D132" t="n">
-        <v>80</v>
+        <v>29</v>
       </c>
       <c r="E132" t="inlineStr">
         <is>
@@ -4473,7 +4473,7 @@
     <row r="166">
       <c r="A166" t="inlineStr">
         <is>
-          <t>11:16:36</t>
+          <t>12:00:15</t>
         </is>
       </c>
       <c r="B166" t="inlineStr">
@@ -4483,11 +4483,11 @@
       </c>
       <c r="C166" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D166" t="n">
-        <v>48</v>
+        <v>4</v>
       </c>
       <c r="E166" t="inlineStr">
         <is>
@@ -4498,7 +4498,7 @@
     <row r="167">
       <c r="A167" t="inlineStr">
         <is>
-          <t>12:00:15</t>
+          <t>11:16:36</t>
         </is>
       </c>
       <c r="B167" t="inlineStr">
@@ -4508,11 +4508,11 @@
       </c>
       <c r="C167" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D167" t="n">
-        <v>4</v>
+        <v>48</v>
       </c>
       <c r="E167" t="inlineStr">
         <is>
@@ -4648,7 +4648,7 @@
     <row r="173">
       <c r="A173" t="inlineStr">
         <is>
-          <t>12:00:15</t>
+          <t>12:28:38</t>
         </is>
       </c>
       <c r="B173" t="inlineStr">
@@ -4658,11 +4658,11 @@
       </c>
       <c r="C173" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D173" t="n">
-        <v>33</v>
+        <v>5</v>
       </c>
       <c r="E173" t="inlineStr">
         <is>
@@ -4698,7 +4698,7 @@
     <row r="175">
       <c r="A175" t="inlineStr">
         <is>
-          <t>12:28:38</t>
+          <t>12:00:15</t>
         </is>
       </c>
       <c r="B175" t="inlineStr">
@@ -4708,11 +4708,11 @@
       </c>
       <c r="C175" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D175" t="n">
-        <v>5</v>
+        <v>33</v>
       </c>
       <c r="E175" t="inlineStr">
         <is>
@@ -5008,7 +5008,7 @@
       </c>
       <c r="C187" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D187" t="n">
@@ -5033,7 +5033,7 @@
       </c>
       <c r="C188" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D188" t="n">
@@ -5073,7 +5073,7 @@
     <row r="190">
       <c r="A190" t="inlineStr">
         <is>
-          <t>12:48:06</t>
+          <t>13:00:14</t>
         </is>
       </c>
       <c r="B190" t="inlineStr">
@@ -5083,11 +5083,11 @@
       </c>
       <c r="C190" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D190" t="n">
-        <v>16</v>
+        <v>4</v>
       </c>
       <c r="E190" t="inlineStr">
         <is>
@@ -5098,7 +5098,7 @@
     <row r="191">
       <c r="A191" t="inlineStr">
         <is>
-          <t>13:00:14</t>
+          <t>12:48:06</t>
         </is>
       </c>
       <c r="B191" t="inlineStr">
@@ -5108,11 +5108,11 @@
       </c>
       <c r="C191" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D191" t="n">
-        <v>4</v>
+        <v>16</v>
       </c>
       <c r="E191" t="inlineStr">
         <is>
@@ -5323,7 +5323,7 @@
     <row r="200">
       <c r="A200" t="inlineStr">
         <is>
-          <t>12:48:06</t>
+          <t>13:00:14</t>
         </is>
       </c>
       <c r="B200" t="inlineStr">
@@ -5333,11 +5333,11 @@
       </c>
       <c r="C200" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D200" t="n">
-        <v>50</v>
+        <v>38</v>
       </c>
       <c r="E200" t="inlineStr">
         <is>
@@ -5348,7 +5348,7 @@
     <row r="201">
       <c r="A201" t="inlineStr">
         <is>
-          <t>13:00:14</t>
+          <t>12:48:06</t>
         </is>
       </c>
       <c r="B201" t="inlineStr">
@@ -5358,11 +5358,11 @@
       </c>
       <c r="C201" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D201" t="n">
-        <v>38</v>
+        <v>50</v>
       </c>
       <c r="E201" t="inlineStr">
         <is>
@@ -5573,7 +5573,7 @@
     <row r="210">
       <c r="A210" t="inlineStr">
         <is>
-          <t>13:00:14</t>
+          <t>13:57:43</t>
         </is>
       </c>
       <c r="B210" t="inlineStr">
@@ -5583,11 +5583,11 @@
       </c>
       <c r="C210" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D210" t="n">
-        <v>63</v>
+        <v>6</v>
       </c>
       <c r="E210" t="inlineStr">
         <is>
@@ -5598,7 +5598,7 @@
     <row r="211">
       <c r="A211" t="inlineStr">
         <is>
-          <t>13:57:43</t>
+          <t>13:00:14</t>
         </is>
       </c>
       <c r="B211" t="inlineStr">
@@ -5608,11 +5608,11 @@
       </c>
       <c r="C211" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D211" t="n">
-        <v>6</v>
+        <v>63</v>
       </c>
       <c r="E211" t="inlineStr">
         <is>
@@ -5623,7 +5623,7 @@
     <row r="212">
       <c r="A212" t="inlineStr">
         <is>
-          <t>13:57:43</t>
+          <t>13:32:57</t>
         </is>
       </c>
       <c r="B212" t="inlineStr">
@@ -5633,11 +5633,11 @@
       </c>
       <c r="C212" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D212" t="n">
-        <v>19</v>
+        <v>44</v>
       </c>
       <c r="E212" t="inlineStr">
         <is>
@@ -5648,7 +5648,7 @@
     <row r="213">
       <c r="A213" t="inlineStr">
         <is>
-          <t>13:32:57</t>
+          <t>13:57:43</t>
         </is>
       </c>
       <c r="B213" t="inlineStr">
@@ -5658,11 +5658,11 @@
       </c>
       <c r="C213" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D213" t="n">
-        <v>44</v>
+        <v>19</v>
       </c>
       <c r="E213" t="inlineStr">
         <is>
@@ -6098,7 +6098,7 @@
     <row r="231">
       <c r="A231" t="inlineStr">
         <is>
-          <t>14:46:39</t>
+          <t>14:59:00</t>
         </is>
       </c>
       <c r="B231" t="inlineStr">
@@ -6112,7 +6112,7 @@
         </is>
       </c>
       <c r="D231" t="n">
-        <v>13</v>
+        <v>0</v>
       </c>
       <c r="E231" t="inlineStr">
         <is>
@@ -6148,21 +6148,21 @@
     <row r="233">
       <c r="A233" t="inlineStr">
         <is>
-          <t>14:46:39</t>
+          <t>14:59:00</t>
         </is>
       </c>
       <c r="B233" t="inlineStr">
         <is>
-          <t>15:01</t>
+          <t>15:00</t>
         </is>
       </c>
       <c r="C233" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D233" t="n">
-        <v>15</v>
+        <v>1</v>
       </c>
       <c r="E233" t="inlineStr">
         <is>
@@ -6173,21 +6173,21 @@
     <row r="234">
       <c r="A234" t="inlineStr">
         <is>
-          <t>14:46:39</t>
+          <t>14:59:00</t>
         </is>
       </c>
       <c r="B234" t="inlineStr">
         <is>
-          <t>15:03</t>
+          <t>15:01</t>
         </is>
       </c>
       <c r="C234" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D234" t="n">
-        <v>17</v>
+        <v>2</v>
       </c>
       <c r="E234" t="inlineStr">
         <is>
@@ -6203,16 +6203,16 @@
       </c>
       <c r="B235" t="inlineStr">
         <is>
-          <t>15:11</t>
+          <t>15:01</t>
         </is>
       </c>
       <c r="C235" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D235" t="n">
-        <v>25</v>
+        <v>15</v>
       </c>
       <c r="E235" t="inlineStr">
         <is>
@@ -6223,21 +6223,21 @@
     <row r="236">
       <c r="A236" t="inlineStr">
         <is>
-          <t>14:46:39</t>
+          <t>14:59:00</t>
         </is>
       </c>
       <c r="B236" t="inlineStr">
         <is>
-          <t>15:11</t>
+          <t>15:02</t>
         </is>
       </c>
       <c r="C236" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D236" t="n">
-        <v>25</v>
+        <v>3</v>
       </c>
       <c r="E236" t="inlineStr">
         <is>
@@ -6253,16 +6253,16 @@
       </c>
       <c r="B237" t="inlineStr">
         <is>
-          <t>15:18</t>
+          <t>15:03</t>
         </is>
       </c>
       <c r="C237" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D237" t="n">
-        <v>32</v>
+        <v>17</v>
       </c>
       <c r="E237" t="inlineStr">
         <is>
@@ -6273,21 +6273,21 @@
     <row r="238">
       <c r="A238" t="inlineStr">
         <is>
-          <t>14:46:39</t>
+          <t>14:59:00</t>
         </is>
       </c>
       <c r="B238" t="inlineStr">
         <is>
-          <t>15:23</t>
+          <t>15:04</t>
         </is>
       </c>
       <c r="C238" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D238" t="n">
-        <v>37</v>
+        <v>5</v>
       </c>
       <c r="E238" t="inlineStr">
         <is>
@@ -6298,21 +6298,21 @@
     <row r="239">
       <c r="A239" t="inlineStr">
         <is>
-          <t>14:46:39</t>
+          <t>14:59:00</t>
         </is>
       </c>
       <c r="B239" t="inlineStr">
         <is>
-          <t>15:38</t>
+          <t>15:11</t>
         </is>
       </c>
       <c r="C239" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D239" t="n">
-        <v>52</v>
+        <v>12</v>
       </c>
       <c r="E239" t="inlineStr">
         <is>
@@ -6328,16 +6328,16 @@
       </c>
       <c r="B240" t="inlineStr">
         <is>
-          <t>15:41</t>
+          <t>15:11</t>
         </is>
       </c>
       <c r="C240" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D240" t="n">
-        <v>55</v>
+        <v>25</v>
       </c>
       <c r="E240" t="inlineStr">
         <is>
@@ -6353,16 +6353,16 @@
       </c>
       <c r="B241" t="inlineStr">
         <is>
-          <t>15:47</t>
+          <t>15:18</t>
         </is>
       </c>
       <c r="C241" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D241" t="n">
-        <v>61</v>
+        <v>32</v>
       </c>
       <c r="E241" t="inlineStr">
         <is>
@@ -6373,21 +6373,21 @@
     <row r="242">
       <c r="A242" t="inlineStr">
         <is>
-          <t>14:46:39</t>
+          <t>14:59:00</t>
         </is>
       </c>
       <c r="B242" t="inlineStr">
         <is>
-          <t>15:51</t>
+          <t>15:19</t>
         </is>
       </c>
       <c r="C242" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D242" t="n">
-        <v>65</v>
+        <v>20</v>
       </c>
       <c r="E242" t="inlineStr">
         <is>
@@ -6403,16 +6403,16 @@
       </c>
       <c r="B243" t="inlineStr">
         <is>
-          <t>15:54</t>
+          <t>15:23</t>
         </is>
       </c>
       <c r="C243" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D243" t="n">
-        <v>68</v>
+        <v>37</v>
       </c>
       <c r="E243" t="inlineStr">
         <is>
@@ -6423,21 +6423,21 @@
     <row r="244">
       <c r="A244" t="inlineStr">
         <is>
-          <t>14:46:39</t>
+          <t>14:59:00</t>
         </is>
       </c>
       <c r="B244" t="inlineStr">
         <is>
-          <t>15:54</t>
+          <t>15:24</t>
         </is>
       </c>
       <c r="C244" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D244" t="n">
-        <v>68</v>
+        <v>25</v>
       </c>
       <c r="E244" t="inlineStr">
         <is>
@@ -6448,21 +6448,21 @@
     <row r="245">
       <c r="A245" t="inlineStr">
         <is>
-          <t>13:57:43</t>
+          <t>14:59:00</t>
         </is>
       </c>
       <c r="B245" t="inlineStr">
         <is>
-          <t>15:56</t>
+          <t>15:27</t>
         </is>
       </c>
       <c r="C245" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D245" t="n">
-        <v>119</v>
+        <v>28</v>
       </c>
       <c r="E245" t="inlineStr">
         <is>
@@ -6473,21 +6473,21 @@
     <row r="246">
       <c r="A246" t="inlineStr">
         <is>
-          <t>14:21:42</t>
+          <t>14:46:39</t>
         </is>
       </c>
       <c r="B246" t="inlineStr">
         <is>
-          <t>15:57</t>
+          <t>15:38</t>
         </is>
       </c>
       <c r="C246" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D246" t="n">
-        <v>96</v>
+        <v>52</v>
       </c>
       <c r="E246" t="inlineStr">
         <is>
@@ -6498,21 +6498,21 @@
     <row r="247">
       <c r="A247" t="inlineStr">
         <is>
-          <t>14:46:39</t>
+          <t>14:59:00</t>
         </is>
       </c>
       <c r="B247" t="inlineStr">
         <is>
-          <t>16:09</t>
+          <t>15:39</t>
         </is>
       </c>
       <c r="C247" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D247" t="n">
-        <v>83</v>
+        <v>40</v>
       </c>
       <c r="E247" t="inlineStr">
         <is>
@@ -6528,16 +6528,16 @@
       </c>
       <c r="B248" t="inlineStr">
         <is>
-          <t>16:11</t>
+          <t>15:41</t>
         </is>
       </c>
       <c r="C248" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D248" t="n">
-        <v>85</v>
+        <v>55</v>
       </c>
       <c r="E248" t="inlineStr">
         <is>
@@ -6548,21 +6548,21 @@
     <row r="249">
       <c r="A249" t="inlineStr">
         <is>
-          <t>14:46:39</t>
+          <t>14:59:00</t>
         </is>
       </c>
       <c r="B249" t="inlineStr">
         <is>
-          <t>16:23</t>
+          <t>15:42</t>
         </is>
       </c>
       <c r="C249" t="inlineStr">
         <is>
-          <t>215_ALUAR</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D249" t="n">
-        <v>97</v>
+        <v>43</v>
       </c>
       <c r="E249" t="inlineStr">
         <is>
@@ -6578,16 +6578,16 @@
       </c>
       <c r="B250" t="inlineStr">
         <is>
-          <t>16:35</t>
+          <t>15:47</t>
         </is>
       </c>
       <c r="C250" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D250" t="n">
-        <v>109</v>
+        <v>61</v>
       </c>
       <c r="E250" t="inlineStr">
         <is>
@@ -6598,23 +6598,423 @@
     <row r="251">
       <c r="A251" t="inlineStr">
         <is>
+          <t>14:59:00</t>
+        </is>
+      </c>
+      <c r="B251" t="inlineStr">
+        <is>
+          <t>15:48</t>
+        </is>
+      </c>
+      <c r="C251" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D251" t="n">
+        <v>49</v>
+      </c>
+      <c r="E251" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="252">
+      <c r="A252" t="inlineStr">
+        <is>
+          <t>14:59:00</t>
+        </is>
+      </c>
+      <c r="B252" t="inlineStr">
+        <is>
+          <t>15:51</t>
+        </is>
+      </c>
+      <c r="C252" t="inlineStr">
+        <is>
+          <t>16_P MOR-SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D252" t="n">
+        <v>52</v>
+      </c>
+      <c r="E252" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="253">
+      <c r="A253" t="inlineStr">
+        <is>
+          <t>14:59:00</t>
+        </is>
+      </c>
+      <c r="B253" t="inlineStr">
+        <is>
+          <t>15:54</t>
+        </is>
+      </c>
+      <c r="C253" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D253" t="n">
+        <v>55</v>
+      </c>
+      <c r="E253" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="254">
+      <c r="A254" t="inlineStr">
+        <is>
           <t>14:46:39</t>
         </is>
       </c>
-      <c r="B251" t="inlineStr">
+      <c r="B254" t="inlineStr">
+        <is>
+          <t>15:54</t>
+        </is>
+      </c>
+      <c r="C254" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D254" t="n">
+        <v>68</v>
+      </c>
+      <c r="E254" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="255">
+      <c r="A255" t="inlineStr">
+        <is>
+          <t>13:57:43</t>
+        </is>
+      </c>
+      <c r="B255" t="inlineStr">
+        <is>
+          <t>15:56</t>
+        </is>
+      </c>
+      <c r="C255" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D255" t="n">
+        <v>119</v>
+      </c>
+      <c r="E255" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="256">
+      <c r="A256" t="inlineStr">
+        <is>
+          <t>14:59:00</t>
+        </is>
+      </c>
+      <c r="B256" t="inlineStr">
+        <is>
+          <t>15:57</t>
+        </is>
+      </c>
+      <c r="C256" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D256" t="n">
+        <v>58</v>
+      </c>
+      <c r="E256" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="257">
+      <c r="A257" t="inlineStr">
+        <is>
+          <t>14:59:00</t>
+        </is>
+      </c>
+      <c r="B257" t="inlineStr">
+        <is>
+          <t>16:09</t>
+        </is>
+      </c>
+      <c r="C257" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D257" t="n">
+        <v>70</v>
+      </c>
+      <c r="E257" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="258">
+      <c r="A258" t="inlineStr">
+        <is>
+          <t>14:46:39</t>
+        </is>
+      </c>
+      <c r="B258" t="inlineStr">
+        <is>
+          <t>16:11</t>
+        </is>
+      </c>
+      <c r="C258" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D258" t="n">
+        <v>85</v>
+      </c>
+      <c r="E258" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="259">
+      <c r="A259" t="inlineStr">
+        <is>
+          <t>14:59:00</t>
+        </is>
+      </c>
+      <c r="B259" t="inlineStr">
+        <is>
+          <t>16:12</t>
+        </is>
+      </c>
+      <c r="C259" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D259" t="n">
+        <v>73</v>
+      </c>
+      <c r="E259" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="260">
+      <c r="A260" t="inlineStr">
+        <is>
+          <t>14:46:39</t>
+        </is>
+      </c>
+      <c r="B260" t="inlineStr">
+        <is>
+          <t>16:23</t>
+        </is>
+      </c>
+      <c r="C260" t="inlineStr">
+        <is>
+          <t>215_ALUAR</t>
+        </is>
+      </c>
+      <c r="D260" t="n">
+        <v>97</v>
+      </c>
+      <c r="E260" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="261">
+      <c r="A261" t="inlineStr">
+        <is>
+          <t>14:59:00</t>
+        </is>
+      </c>
+      <c r="B261" t="inlineStr">
+        <is>
+          <t>16:24</t>
+        </is>
+      </c>
+      <c r="C261" t="inlineStr">
+        <is>
+          <t>215_ALUAR</t>
+        </is>
+      </c>
+      <c r="D261" t="n">
+        <v>85</v>
+      </c>
+      <c r="E261" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="262">
+      <c r="A262" t="inlineStr">
+        <is>
+          <t>14:59:00</t>
+        </is>
+      </c>
+      <c r="B262" t="inlineStr">
+        <is>
+          <t>16:25</t>
+        </is>
+      </c>
+      <c r="C262" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D262" t="n">
+        <v>86</v>
+      </c>
+      <c r="E262" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="263">
+      <c r="A263" t="inlineStr">
+        <is>
+          <t>14:59:00</t>
+        </is>
+      </c>
+      <c r="B263" t="inlineStr">
         <is>
           <t>16:35</t>
         </is>
       </c>
-      <c r="C251" t="inlineStr">
+      <c r="C263" t="inlineStr">
+        <is>
+          <t>17X38_ROMERO</t>
+        </is>
+      </c>
+      <c r="D263" t="n">
+        <v>96</v>
+      </c>
+      <c r="E263" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="264">
+      <c r="A264" t="inlineStr">
+        <is>
+          <t>14:46:39</t>
+        </is>
+      </c>
+      <c r="B264" t="inlineStr">
+        <is>
+          <t>16:35</t>
+        </is>
+      </c>
+      <c r="C264" t="inlineStr">
         <is>
           <t>11_ETCHEVERRY</t>
         </is>
       </c>
-      <c r="D251" t="n">
+      <c r="D264" t="n">
         <v>109</v>
       </c>
-      <c r="E251" t="inlineStr">
+      <c r="E264" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="265">
+      <c r="A265" t="inlineStr">
+        <is>
+          <t>14:59:00</t>
+        </is>
+      </c>
+      <c r="B265" t="inlineStr">
+        <is>
+          <t>16:36</t>
+        </is>
+      </c>
+      <c r="C265" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D265" t="n">
+        <v>97</v>
+      </c>
+      <c r="E265" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="266">
+      <c r="A266" t="inlineStr">
+        <is>
+          <t>14:59:00</t>
+        </is>
+      </c>
+      <c r="B266" t="inlineStr">
+        <is>
+          <t>16:47</t>
+        </is>
+      </c>
+      <c r="C266" t="inlineStr">
+        <is>
+          <t>225_GOMEZ</t>
+        </is>
+      </c>
+      <c r="D266" t="n">
+        <v>108</v>
+      </c>
+      <c r="E266" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="267">
+      <c r="A267" t="inlineStr">
+        <is>
+          <t>14:59:00</t>
+        </is>
+      </c>
+      <c r="B267" t="inlineStr">
+        <is>
+          <t>16:51</t>
+        </is>
+      </c>
+      <c r="C267" t="inlineStr">
+        <is>
+          <t>16_P MOR-SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D267" t="n">
+        <v>112</v>
+      </c>
+      <c r="E267" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -6631,7 +7031,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E44"/>
+  <dimension ref="A1:E47"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6644,14 +7044,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 14:46:40</t>
+          <t>Última actualización: 14:59:00</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 39</t>
+          <t>Total filas: 42</t>
         </is>
       </c>
     </row>
@@ -7610,21 +8010,21 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>14:46:39</t>
+          <t>14:59:00</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>15:18</t>
+          <t>15:00</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D43" t="n">
-        <v>32</v>
+        <v>1</v>
       </c>
       <c r="E43" t="inlineStr">
         <is>
@@ -7640,18 +8040,93 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
+          <t>15:18</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D44" t="n">
+        <v>32</v>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>14:59:00</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>15:19</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D45" t="n">
+        <v>20</v>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>14:46:39</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
           <t>16:23</t>
         </is>
       </c>
-      <c r="C44" t="inlineStr">
+      <c r="C46" t="inlineStr">
         <is>
           <t>215_ALUAR</t>
         </is>
       </c>
-      <c r="D44" t="n">
+      <c r="D46" t="n">
         <v>97</v>
       </c>
-      <c r="E44" t="inlineStr">
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>14:59:00</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>16:24</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>215_ALUAR</t>
+        </is>
+      </c>
+      <c r="D47" t="n">
+        <v>85</v>
+      </c>
+      <c r="E47" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -7668,7 +8143,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E50"/>
+  <dimension ref="A1:E53"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -7681,14 +8156,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 14:46:40</t>
+          <t>Última actualización: 14:59:00</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 45</t>
+          <t>Total filas: 48</t>
         </is>
       </c>
     </row>
@@ -8772,7 +9247,7 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>14:46:39</t>
+          <t>14:59:00</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
@@ -8786,7 +9261,7 @@
         </is>
       </c>
       <c r="D48" t="n">
-        <v>24</v>
+        <v>11</v>
       </c>
       <c r="E48" t="inlineStr">
         <is>
@@ -8822,25 +9297,100 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
+          <t>14:59:00</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>15:46</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D50" t="n">
+        <v>47</v>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
           <t>14:46:39</t>
         </is>
       </c>
-      <c r="B50" t="inlineStr">
+      <c r="B51" t="inlineStr">
         <is>
           <t>16:42</t>
         </is>
       </c>
-      <c r="C50" t="inlineStr">
+      <c r="C51" t="inlineStr">
         <is>
           <t>215B_LP-P MOR-1 Y 57</t>
         </is>
       </c>
-      <c r="D50" t="n">
+      <c r="D51" t="n">
         <v>116</v>
       </c>
-      <c r="E50" t="inlineStr">
+      <c r="E51" t="inlineStr">
         <is>
           <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>14:59:00</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>16:43</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>215B_LP-P MOR-1 Y 57</t>
+        </is>
+      </c>
+      <c r="D52" t="n">
+        <v>104</v>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>14:59:00</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>16:56</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D53" t="n">
+        <v>117</v>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>L6203</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 1814
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-03-21.xlsx
+++ b/data/horarios-141-2026-03-21.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E267"/>
+  <dimension ref="A1:E275"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 14:59:00</t>
+          <t>Última actualización: 15:34:45</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 262</t>
+          <t>Total filas: 270</t>
         </is>
       </c>
     </row>
@@ -758,7 +758,7 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D17" t="n">
@@ -783,7 +783,7 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D18" t="n">
@@ -1158,7 +1158,7 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D33" t="n">
@@ -1183,7 +1183,7 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D34" t="n">
@@ -1558,7 +1558,7 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D49" t="n">
@@ -1583,7 +1583,7 @@
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D50" t="n">
@@ -1983,7 +1983,7 @@
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D66" t="n">
@@ -2008,7 +2008,7 @@
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D67" t="n">
@@ -2373,7 +2373,7 @@
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>08:50:55</t>
+          <t>07:27:35</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
@@ -2383,11 +2383,11 @@
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D82" t="n">
-        <v>1</v>
+        <v>84</v>
       </c>
       <c r="E82" t="inlineStr">
         <is>
@@ -2423,7 +2423,7 @@
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>07:27:35</t>
+          <t>08:50:55</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
@@ -2433,11 +2433,11 @@
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D84" t="n">
-        <v>84</v>
+        <v>1</v>
       </c>
       <c r="E84" t="inlineStr">
         <is>
@@ -2698,7 +2698,7 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>08:14:14</t>
+          <t>08:50:55</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
@@ -2708,11 +2708,11 @@
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>215_EL PELIGRO</t>
         </is>
       </c>
       <c r="D95" t="n">
-        <v>64</v>
+        <v>28</v>
       </c>
       <c r="E95" t="inlineStr">
         <is>
@@ -2723,7 +2723,7 @@
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>08:50:55</t>
+          <t>08:14:14</t>
         </is>
       </c>
       <c r="B96" t="inlineStr">
@@ -2733,11 +2733,11 @@
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D96" t="n">
-        <v>28</v>
+        <v>64</v>
       </c>
       <c r="E96" t="inlineStr">
         <is>
@@ -2758,7 +2758,7 @@
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>215_EL PELIGRO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D97" t="n">
@@ -3083,7 +3083,7 @@
       </c>
       <c r="C110" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D110" t="n">
@@ -3108,7 +3108,7 @@
       </c>
       <c r="C111" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D111" t="n">
@@ -3173,7 +3173,7 @@
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>09:23:24</t>
+          <t>08:50:55</t>
         </is>
       </c>
       <c r="B114" t="inlineStr">
@@ -3183,11 +3183,11 @@
       </c>
       <c r="C114" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D114" t="n">
-        <v>40</v>
+        <v>73</v>
       </c>
       <c r="E114" t="inlineStr">
         <is>
@@ -3198,7 +3198,7 @@
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>08:50:55</t>
+          <t>09:23:24</t>
         </is>
       </c>
       <c r="B115" t="inlineStr">
@@ -3208,11 +3208,11 @@
       </c>
       <c r="C115" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D115" t="n">
-        <v>73</v>
+        <v>40</v>
       </c>
       <c r="E115" t="inlineStr">
         <is>
@@ -4123,7 +4123,7 @@
     <row r="152">
       <c r="A152" t="inlineStr">
         <is>
-          <t>11:16:36</t>
+          <t>10:14:52</t>
         </is>
       </c>
       <c r="B152" t="inlineStr">
@@ -4133,11 +4133,11 @@
       </c>
       <c r="C152" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D152" t="n">
-        <v>16</v>
+        <v>78</v>
       </c>
       <c r="E152" t="inlineStr">
         <is>
@@ -4148,7 +4148,7 @@
     <row r="153">
       <c r="A153" t="inlineStr">
         <is>
-          <t>10:14:52</t>
+          <t>11:16:36</t>
         </is>
       </c>
       <c r="B153" t="inlineStr">
@@ -4158,11 +4158,11 @@
       </c>
       <c r="C153" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D153" t="n">
-        <v>78</v>
+        <v>16</v>
       </c>
       <c r="E153" t="inlineStr">
         <is>
@@ -4183,7 +4183,7 @@
       </c>
       <c r="C154" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D154" t="n">
@@ -4208,7 +4208,7 @@
       </c>
       <c r="C155" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D155" t="n">
@@ -4658,7 +4658,7 @@
       </c>
       <c r="C173" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D173" t="n">
@@ -4683,7 +4683,7 @@
       </c>
       <c r="C174" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D174" t="n">
@@ -5248,7 +5248,7 @@
     <row r="197">
       <c r="A197" t="inlineStr">
         <is>
-          <t>13:00:14</t>
+          <t>12:48:06</t>
         </is>
       </c>
       <c r="B197" t="inlineStr">
@@ -5258,11 +5258,11 @@
       </c>
       <c r="C197" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D197" t="n">
-        <v>33</v>
+        <v>45</v>
       </c>
       <c r="E197" t="inlineStr">
         <is>
@@ -5273,7 +5273,7 @@
     <row r="198">
       <c r="A198" t="inlineStr">
         <is>
-          <t>12:48:06</t>
+          <t>13:00:14</t>
         </is>
       </c>
       <c r="B198" t="inlineStr">
@@ -5283,11 +5283,11 @@
       </c>
       <c r="C198" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D198" t="n">
-        <v>45</v>
+        <v>33</v>
       </c>
       <c r="E198" t="inlineStr">
         <is>
@@ -5498,7 +5498,7 @@
     <row r="207">
       <c r="A207" t="inlineStr">
         <is>
-          <t>13:32:57</t>
+          <t>13:57:43</t>
         </is>
       </c>
       <c r="B207" t="inlineStr">
@@ -5508,11 +5508,11 @@
       </c>
       <c r="C207" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D207" t="n">
-        <v>27</v>
+        <v>2</v>
       </c>
       <c r="E207" t="inlineStr">
         <is>
@@ -5523,7 +5523,7 @@
     <row r="208">
       <c r="A208" t="inlineStr">
         <is>
-          <t>13:57:43</t>
+          <t>13:32:57</t>
         </is>
       </c>
       <c r="B208" t="inlineStr">
@@ -5533,11 +5533,11 @@
       </c>
       <c r="C208" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D208" t="n">
-        <v>2</v>
+        <v>27</v>
       </c>
       <c r="E208" t="inlineStr">
         <is>
@@ -6298,7 +6298,7 @@
     <row r="239">
       <c r="A239" t="inlineStr">
         <is>
-          <t>14:59:00</t>
+          <t>14:46:39</t>
         </is>
       </c>
       <c r="B239" t="inlineStr">
@@ -6308,11 +6308,11 @@
       </c>
       <c r="C239" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D239" t="n">
-        <v>12</v>
+        <v>25</v>
       </c>
       <c r="E239" t="inlineStr">
         <is>
@@ -6323,7 +6323,7 @@
     <row r="240">
       <c r="A240" t="inlineStr">
         <is>
-          <t>14:46:39</t>
+          <t>14:59:00</t>
         </is>
       </c>
       <c r="B240" t="inlineStr">
@@ -6333,11 +6333,11 @@
       </c>
       <c r="C240" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D240" t="n">
-        <v>25</v>
+        <v>12</v>
       </c>
       <c r="E240" t="inlineStr">
         <is>
@@ -6473,21 +6473,21 @@
     <row r="246">
       <c r="A246" t="inlineStr">
         <is>
-          <t>14:46:39</t>
+          <t>15:34:45</t>
         </is>
       </c>
       <c r="B246" t="inlineStr">
         <is>
-          <t>15:38</t>
+          <t>15:34</t>
         </is>
       </c>
       <c r="C246" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D246" t="n">
-        <v>52</v>
+        <v>0</v>
       </c>
       <c r="E246" t="inlineStr">
         <is>
@@ -6498,21 +6498,21 @@
     <row r="247">
       <c r="A247" t="inlineStr">
         <is>
-          <t>14:59:00</t>
+          <t>15:34:45</t>
         </is>
       </c>
       <c r="B247" t="inlineStr">
         <is>
-          <t>15:39</t>
+          <t>15:35</t>
         </is>
       </c>
       <c r="C247" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D247" t="n">
-        <v>40</v>
+        <v>1</v>
       </c>
       <c r="E247" t="inlineStr">
         <is>
@@ -6523,21 +6523,21 @@
     <row r="248">
       <c r="A248" t="inlineStr">
         <is>
-          <t>14:46:39</t>
+          <t>15:34:45</t>
         </is>
       </c>
       <c r="B248" t="inlineStr">
         <is>
-          <t>15:41</t>
+          <t>15:38</t>
         </is>
       </c>
       <c r="C248" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D248" t="n">
-        <v>55</v>
+        <v>4</v>
       </c>
       <c r="E248" t="inlineStr">
         <is>
@@ -6553,16 +6553,16 @@
       </c>
       <c r="B249" t="inlineStr">
         <is>
-          <t>15:42</t>
+          <t>15:39</t>
         </is>
       </c>
       <c r="C249" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D249" t="n">
-        <v>43</v>
+        <v>40</v>
       </c>
       <c r="E249" t="inlineStr">
         <is>
@@ -6573,21 +6573,21 @@
     <row r="250">
       <c r="A250" t="inlineStr">
         <is>
-          <t>14:46:39</t>
+          <t>15:34:45</t>
         </is>
       </c>
       <c r="B250" t="inlineStr">
         <is>
-          <t>15:47</t>
+          <t>15:41</t>
         </is>
       </c>
       <c r="C250" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D250" t="n">
-        <v>61</v>
+        <v>7</v>
       </c>
       <c r="E250" t="inlineStr">
         <is>
@@ -6603,16 +6603,16 @@
       </c>
       <c r="B251" t="inlineStr">
         <is>
-          <t>15:48</t>
+          <t>15:42</t>
         </is>
       </c>
       <c r="C251" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D251" t="n">
-        <v>49</v>
+        <v>43</v>
       </c>
       <c r="E251" t="inlineStr">
         <is>
@@ -6623,21 +6623,21 @@
     <row r="252">
       <c r="A252" t="inlineStr">
         <is>
-          <t>14:59:00</t>
+          <t>15:34:45</t>
         </is>
       </c>
       <c r="B252" t="inlineStr">
         <is>
-          <t>15:51</t>
+          <t>15:47</t>
         </is>
       </c>
       <c r="C252" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D252" t="n">
-        <v>52</v>
+        <v>13</v>
       </c>
       <c r="E252" t="inlineStr">
         <is>
@@ -6653,16 +6653,16 @@
       </c>
       <c r="B253" t="inlineStr">
         <is>
-          <t>15:54</t>
+          <t>15:48</t>
         </is>
       </c>
       <c r="C253" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D253" t="n">
-        <v>55</v>
+        <v>49</v>
       </c>
       <c r="E253" t="inlineStr">
         <is>
@@ -6673,21 +6673,21 @@
     <row r="254">
       <c r="A254" t="inlineStr">
         <is>
-          <t>14:46:39</t>
+          <t>15:34:45</t>
         </is>
       </c>
       <c r="B254" t="inlineStr">
         <is>
-          <t>15:54</t>
+          <t>15:51</t>
         </is>
       </c>
       <c r="C254" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D254" t="n">
-        <v>68</v>
+        <v>17</v>
       </c>
       <c r="E254" t="inlineStr">
         <is>
@@ -6698,21 +6698,21 @@
     <row r="255">
       <c r="A255" t="inlineStr">
         <is>
-          <t>13:57:43</t>
+          <t>15:34:45</t>
         </is>
       </c>
       <c r="B255" t="inlineStr">
         <is>
-          <t>15:56</t>
+          <t>15:54</t>
         </is>
       </c>
       <c r="C255" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D255" t="n">
-        <v>119</v>
+        <v>20</v>
       </c>
       <c r="E255" t="inlineStr">
         <is>
@@ -6723,12 +6723,12 @@
     <row r="256">
       <c r="A256" t="inlineStr">
         <is>
-          <t>14:59:00</t>
+          <t>14:46:39</t>
         </is>
       </c>
       <c r="B256" t="inlineStr">
         <is>
-          <t>15:57</t>
+          <t>15:54</t>
         </is>
       </c>
       <c r="C256" t="inlineStr">
@@ -6737,7 +6737,7 @@
         </is>
       </c>
       <c r="D256" t="n">
-        <v>58</v>
+        <v>68</v>
       </c>
       <c r="E256" t="inlineStr">
         <is>
@@ -6748,21 +6748,21 @@
     <row r="257">
       <c r="A257" t="inlineStr">
         <is>
-          <t>14:59:00</t>
+          <t>15:34:45</t>
         </is>
       </c>
       <c r="B257" t="inlineStr">
         <is>
-          <t>16:09</t>
+          <t>15:56</t>
         </is>
       </c>
       <c r="C257" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D257" t="n">
-        <v>70</v>
+        <v>22</v>
       </c>
       <c r="E257" t="inlineStr">
         <is>
@@ -6773,21 +6773,21 @@
     <row r="258">
       <c r="A258" t="inlineStr">
         <is>
-          <t>14:46:39</t>
+          <t>14:59:00</t>
         </is>
       </c>
       <c r="B258" t="inlineStr">
         <is>
-          <t>16:11</t>
+          <t>15:57</t>
         </is>
       </c>
       <c r="C258" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D258" t="n">
-        <v>85</v>
+        <v>58</v>
       </c>
       <c r="E258" t="inlineStr">
         <is>
@@ -6798,21 +6798,21 @@
     <row r="259">
       <c r="A259" t="inlineStr">
         <is>
-          <t>14:59:00</t>
+          <t>15:34:45</t>
         </is>
       </c>
       <c r="B259" t="inlineStr">
         <is>
-          <t>16:12</t>
+          <t>16:09</t>
         </is>
       </c>
       <c r="C259" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D259" t="n">
-        <v>73</v>
+        <v>35</v>
       </c>
       <c r="E259" t="inlineStr">
         <is>
@@ -6823,21 +6823,21 @@
     <row r="260">
       <c r="A260" t="inlineStr">
         <is>
-          <t>14:46:39</t>
+          <t>15:34:45</t>
         </is>
       </c>
       <c r="B260" t="inlineStr">
         <is>
-          <t>16:23</t>
+          <t>16:11</t>
         </is>
       </c>
       <c r="C260" t="inlineStr">
         <is>
-          <t>215_ALUAR</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D260" t="n">
-        <v>97</v>
+        <v>37</v>
       </c>
       <c r="E260" t="inlineStr">
         <is>
@@ -6853,16 +6853,16 @@
       </c>
       <c r="B261" t="inlineStr">
         <is>
-          <t>16:24</t>
+          <t>16:12</t>
         </is>
       </c>
       <c r="C261" t="inlineStr">
         <is>
-          <t>215_ALUAR</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D261" t="n">
-        <v>85</v>
+        <v>73</v>
       </c>
       <c r="E261" t="inlineStr">
         <is>
@@ -6873,12 +6873,12 @@
     <row r="262">
       <c r="A262" t="inlineStr">
         <is>
-          <t>14:59:00</t>
+          <t>15:34:45</t>
         </is>
       </c>
       <c r="B262" t="inlineStr">
         <is>
-          <t>16:25</t>
+          <t>16:23</t>
         </is>
       </c>
       <c r="C262" t="inlineStr">
@@ -6887,7 +6887,7 @@
         </is>
       </c>
       <c r="D262" t="n">
-        <v>86</v>
+        <v>49</v>
       </c>
       <c r="E262" t="inlineStr">
         <is>
@@ -6898,21 +6898,21 @@
     <row r="263">
       <c r="A263" t="inlineStr">
         <is>
-          <t>14:59:00</t>
+          <t>15:34:45</t>
         </is>
       </c>
       <c r="B263" t="inlineStr">
         <is>
-          <t>16:35</t>
+          <t>16:23</t>
         </is>
       </c>
       <c r="C263" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>215_ALUAR</t>
         </is>
       </c>
       <c r="D263" t="n">
-        <v>96</v>
+        <v>49</v>
       </c>
       <c r="E263" t="inlineStr">
         <is>
@@ -6923,21 +6923,21 @@
     <row r="264">
       <c r="A264" t="inlineStr">
         <is>
-          <t>14:46:39</t>
+          <t>14:59:00</t>
         </is>
       </c>
       <c r="B264" t="inlineStr">
         <is>
-          <t>16:35</t>
+          <t>16:24</t>
         </is>
       </c>
       <c r="C264" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>215_ALUAR</t>
         </is>
       </c>
       <c r="D264" t="n">
-        <v>109</v>
+        <v>85</v>
       </c>
       <c r="E264" t="inlineStr">
         <is>
@@ -6953,16 +6953,16 @@
       </c>
       <c r="B265" t="inlineStr">
         <is>
-          <t>16:36</t>
+          <t>16:25</t>
         </is>
       </c>
       <c r="C265" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D265" t="n">
-        <v>97</v>
+        <v>86</v>
       </c>
       <c r="E265" t="inlineStr">
         <is>
@@ -6973,21 +6973,21 @@
     <row r="266">
       <c r="A266" t="inlineStr">
         <is>
-          <t>14:59:00</t>
+          <t>15:34:45</t>
         </is>
       </c>
       <c r="B266" t="inlineStr">
         <is>
-          <t>16:47</t>
+          <t>16:35</t>
         </is>
       </c>
       <c r="C266" t="inlineStr">
         <is>
-          <t>225_GOMEZ</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D266" t="n">
-        <v>108</v>
+        <v>61</v>
       </c>
       <c r="E266" t="inlineStr">
         <is>
@@ -6998,23 +6998,223 @@
     <row r="267">
       <c r="A267" t="inlineStr">
         <is>
+          <t>15:34:45</t>
+        </is>
+      </c>
+      <c r="B267" t="inlineStr">
+        <is>
+          <t>16:35</t>
+        </is>
+      </c>
+      <c r="C267" t="inlineStr">
+        <is>
+          <t>17X38_ROMERO</t>
+        </is>
+      </c>
+      <c r="D267" t="n">
+        <v>61</v>
+      </c>
+      <c r="E267" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="268">
+      <c r="A268" t="inlineStr">
+        <is>
+          <t>15:34:45</t>
+        </is>
+      </c>
+      <c r="B268" t="inlineStr">
+        <is>
+          <t>16:36</t>
+        </is>
+      </c>
+      <c r="C268" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D268" t="n">
+        <v>62</v>
+      </c>
+      <c r="E268" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="269">
+      <c r="A269" t="inlineStr">
+        <is>
           <t>14:59:00</t>
         </is>
       </c>
-      <c r="B267" t="inlineStr">
+      <c r="B269" t="inlineStr">
+        <is>
+          <t>16:36</t>
+        </is>
+      </c>
+      <c r="C269" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D269" t="n">
+        <v>97</v>
+      </c>
+      <c r="E269" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="270">
+      <c r="A270" t="inlineStr">
+        <is>
+          <t>15:34:45</t>
+        </is>
+      </c>
+      <c r="B270" t="inlineStr">
+        <is>
+          <t>16:47</t>
+        </is>
+      </c>
+      <c r="C270" t="inlineStr">
+        <is>
+          <t>225_GOMEZ</t>
+        </is>
+      </c>
+      <c r="D270" t="n">
+        <v>73</v>
+      </c>
+      <c r="E270" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="271">
+      <c r="A271" t="inlineStr">
+        <is>
+          <t>15:34:45</t>
+        </is>
+      </c>
+      <c r="B271" t="inlineStr">
         <is>
           <t>16:51</t>
         </is>
       </c>
-      <c r="C267" t="inlineStr">
+      <c r="C271" t="inlineStr">
         <is>
           <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
-      <c r="D267" t="n">
-        <v>112</v>
-      </c>
-      <c r="E267" t="inlineStr">
+      <c r="D271" t="n">
+        <v>77</v>
+      </c>
+      <c r="E271" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="272">
+      <c r="A272" t="inlineStr">
+        <is>
+          <t>15:34:45</t>
+        </is>
+      </c>
+      <c r="B272" t="inlineStr">
+        <is>
+          <t>16:59</t>
+        </is>
+      </c>
+      <c r="C272" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D272" t="n">
+        <v>85</v>
+      </c>
+      <c r="E272" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="273">
+      <c r="A273" t="inlineStr">
+        <is>
+          <t>15:34:45</t>
+        </is>
+      </c>
+      <c r="B273" t="inlineStr">
+        <is>
+          <t>16:59</t>
+        </is>
+      </c>
+      <c r="C273" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D273" t="n">
+        <v>85</v>
+      </c>
+      <c r="E273" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="274">
+      <c r="A274" t="inlineStr">
+        <is>
+          <t>15:34:45</t>
+        </is>
+      </c>
+      <c r="B274" t="inlineStr">
+        <is>
+          <t>17:11</t>
+        </is>
+      </c>
+      <c r="C274" t="inlineStr">
+        <is>
+          <t>17_ROMERO</t>
+        </is>
+      </c>
+      <c r="D274" t="n">
+        <v>97</v>
+      </c>
+      <c r="E274" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="275">
+      <c r="A275" t="inlineStr">
+        <is>
+          <t>15:34:45</t>
+        </is>
+      </c>
+      <c r="B275" t="inlineStr">
+        <is>
+          <t>17:19</t>
+        </is>
+      </c>
+      <c r="C275" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D275" t="n">
+        <v>105</v>
+      </c>
+      <c r="E275" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -7031,7 +7231,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E47"/>
+  <dimension ref="A1:E48"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -7044,14 +7244,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 14:59:00</t>
+          <t>Última actualización: 15:34:45</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 42</t>
+          <t>Total filas: 43</t>
         </is>
       </c>
     </row>
@@ -8085,7 +8285,7 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>14:46:39</t>
+          <t>15:34:45</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
@@ -8099,7 +8299,7 @@
         </is>
       </c>
       <c r="D46" t="n">
-        <v>97</v>
+        <v>49</v>
       </c>
       <c r="E46" t="inlineStr">
         <is>
@@ -8127,6 +8327,31 @@
         <v>85</v>
       </c>
       <c r="E47" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>15:34:45</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>16:59</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D48" t="n">
+        <v>85</v>
+      </c>
+      <c r="E48" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -8143,7 +8368,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E53"/>
+  <dimension ref="A1:E54"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -8156,14 +8381,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 14:59:00</t>
+          <t>Última actualización: 15:34:45</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 48</t>
+          <t>Total filas: 49</t>
         </is>
       </c>
     </row>
@@ -9272,7 +9497,7 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>14:46:39</t>
+          <t>15:34:45</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
@@ -9286,7 +9511,7 @@
         </is>
       </c>
       <c r="D49" t="n">
-        <v>59</v>
+        <v>11</v>
       </c>
       <c r="E49" t="inlineStr">
         <is>
@@ -9322,7 +9547,7 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>14:46:39</t>
+          <t>15:34:45</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
@@ -9336,7 +9561,7 @@
         </is>
       </c>
       <c r="D51" t="n">
-        <v>116</v>
+        <v>68</v>
       </c>
       <c r="E51" t="inlineStr">
         <is>
@@ -9372,23 +9597,48 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
+          <t>15:34:45</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>16:55</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D53" t="n">
+        <v>81</v>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
           <t>14:59:00</t>
         </is>
       </c>
-      <c r="B53" t="inlineStr">
+      <c r="B54" t="inlineStr">
         <is>
           <t>16:56</t>
         </is>
       </c>
-      <c r="C53" t="inlineStr">
+      <c r="C54" t="inlineStr">
         <is>
           <t>215C_LA PLATA</t>
         </is>
       </c>
-      <c r="D53" t="n">
+      <c r="D54" t="n">
         <v>117</v>
       </c>
-      <c r="E53" t="inlineStr">
+      <c r="E54" t="inlineStr">
         <is>
           <t>L6203</t>
         </is>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 1815
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-03-21.xlsx
+++ b/data/horarios-141-2026-03-21.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E275"/>
+  <dimension ref="A1:E289"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 15:34:45</t>
+          <t>Última actualización: 16:01:44</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 270</t>
+          <t>Total filas: 284</t>
         </is>
       </c>
     </row>
@@ -1158,7 +1158,7 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D33" t="n">
@@ -1183,7 +1183,7 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D34" t="n">
@@ -1883,7 +1883,7 @@
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D62" t="n">
@@ -1908,7 +1908,7 @@
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D63" t="n">
@@ -1973,7 +1973,7 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>07:51:37</t>
+          <t>07:27:35</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
@@ -1983,11 +1983,11 @@
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D66" t="n">
-        <v>28</v>
+        <v>52</v>
       </c>
       <c r="E66" t="inlineStr">
         <is>
@@ -2023,7 +2023,7 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>07:27:35</t>
+          <t>07:51:37</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
@@ -2033,11 +2033,11 @@
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D68" t="n">
-        <v>52</v>
+        <v>28</v>
       </c>
       <c r="E68" t="inlineStr">
         <is>
@@ -2233,7 +2233,7 @@
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D76" t="n">
@@ -2258,7 +2258,7 @@
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D77" t="n">
@@ -2708,7 +2708,7 @@
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>215_EL PELIGRO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D95" t="n">
@@ -2723,7 +2723,7 @@
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>08:14:14</t>
+          <t>08:50:55</t>
         </is>
       </c>
       <c r="B96" t="inlineStr">
@@ -2733,11 +2733,11 @@
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>215_EL PELIGRO</t>
         </is>
       </c>
       <c r="D96" t="n">
-        <v>64</v>
+        <v>28</v>
       </c>
       <c r="E96" t="inlineStr">
         <is>
@@ -2748,7 +2748,7 @@
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>08:50:55</t>
+          <t>08:14:14</t>
         </is>
       </c>
       <c r="B97" t="inlineStr">
@@ -2758,11 +2758,11 @@
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D97" t="n">
-        <v>28</v>
+        <v>64</v>
       </c>
       <c r="E97" t="inlineStr">
         <is>
@@ -2873,7 +2873,7 @@
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>07:51:37</t>
+          <t>08:36:09</t>
         </is>
       </c>
       <c r="B102" t="inlineStr">
@@ -2883,11 +2883,11 @@
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D102" t="n">
-        <v>98</v>
+        <v>53</v>
       </c>
       <c r="E102" t="inlineStr">
         <is>
@@ -2898,7 +2898,7 @@
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>08:36:09</t>
+          <t>07:51:37</t>
         </is>
       </c>
       <c r="B103" t="inlineStr">
@@ -2908,11 +2908,11 @@
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D103" t="n">
-        <v>53</v>
+        <v>98</v>
       </c>
       <c r="E103" t="inlineStr">
         <is>
@@ -3083,7 +3083,7 @@
       </c>
       <c r="C110" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D110" t="n">
@@ -3108,7 +3108,7 @@
       </c>
       <c r="C111" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D111" t="n">
@@ -3173,7 +3173,7 @@
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>08:50:55</t>
+          <t>09:23:24</t>
         </is>
       </c>
       <c r="B114" t="inlineStr">
@@ -3183,11 +3183,11 @@
       </c>
       <c r="C114" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D114" t="n">
-        <v>73</v>
+        <v>40</v>
       </c>
       <c r="E114" t="inlineStr">
         <is>
@@ -3198,7 +3198,7 @@
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>09:23:24</t>
+          <t>08:50:55</t>
         </is>
       </c>
       <c r="B115" t="inlineStr">
@@ -3208,11 +3208,11 @@
       </c>
       <c r="C115" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D115" t="n">
-        <v>40</v>
+        <v>73</v>
       </c>
       <c r="E115" t="inlineStr">
         <is>
@@ -4123,7 +4123,7 @@
     <row r="152">
       <c r="A152" t="inlineStr">
         <is>
-          <t>10:14:52</t>
+          <t>11:16:36</t>
         </is>
       </c>
       <c r="B152" t="inlineStr">
@@ -4133,11 +4133,11 @@
       </c>
       <c r="C152" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D152" t="n">
-        <v>78</v>
+        <v>16</v>
       </c>
       <c r="E152" t="inlineStr">
         <is>
@@ -4148,7 +4148,7 @@
     <row r="153">
       <c r="A153" t="inlineStr">
         <is>
-          <t>11:16:36</t>
+          <t>10:14:52</t>
         </is>
       </c>
       <c r="B153" t="inlineStr">
@@ -4158,11 +4158,11 @@
       </c>
       <c r="C153" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D153" t="n">
-        <v>16</v>
+        <v>78</v>
       </c>
       <c r="E153" t="inlineStr">
         <is>
@@ -4183,7 +4183,7 @@
       </c>
       <c r="C154" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D154" t="n">
@@ -4208,7 +4208,7 @@
       </c>
       <c r="C155" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D155" t="n">
@@ -4473,7 +4473,7 @@
     <row r="166">
       <c r="A166" t="inlineStr">
         <is>
-          <t>12:00:15</t>
+          <t>11:16:36</t>
         </is>
       </c>
       <c r="B166" t="inlineStr">
@@ -4483,11 +4483,11 @@
       </c>
       <c r="C166" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D166" t="n">
-        <v>4</v>
+        <v>48</v>
       </c>
       <c r="E166" t="inlineStr">
         <is>
@@ -4498,7 +4498,7 @@
     <row r="167">
       <c r="A167" t="inlineStr">
         <is>
-          <t>11:16:36</t>
+          <t>12:00:15</t>
         </is>
       </c>
       <c r="B167" t="inlineStr">
@@ -4508,11 +4508,11 @@
       </c>
       <c r="C167" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D167" t="n">
-        <v>48</v>
+        <v>4</v>
       </c>
       <c r="E167" t="inlineStr">
         <is>
@@ -4998,7 +4998,7 @@
     <row r="187">
       <c r="A187" t="inlineStr">
         <is>
-          <t>12:28:38</t>
+          <t>13:00:14</t>
         </is>
       </c>
       <c r="B187" t="inlineStr">
@@ -5008,11 +5008,11 @@
       </c>
       <c r="C187" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D187" t="n">
-        <v>35</v>
+        <v>3</v>
       </c>
       <c r="E187" t="inlineStr">
         <is>
@@ -5033,7 +5033,7 @@
       </c>
       <c r="C188" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D188" t="n">
@@ -5048,7 +5048,7 @@
     <row r="189">
       <c r="A189" t="inlineStr">
         <is>
-          <t>13:00:14</t>
+          <t>12:28:38</t>
         </is>
       </c>
       <c r="B189" t="inlineStr">
@@ -5058,11 +5058,11 @@
       </c>
       <c r="C189" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D189" t="n">
-        <v>3</v>
+        <v>35</v>
       </c>
       <c r="E189" t="inlineStr">
         <is>
@@ -5073,7 +5073,7 @@
     <row r="190">
       <c r="A190" t="inlineStr">
         <is>
-          <t>13:00:14</t>
+          <t>12:48:06</t>
         </is>
       </c>
       <c r="B190" t="inlineStr">
@@ -5083,11 +5083,11 @@
       </c>
       <c r="C190" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D190" t="n">
-        <v>4</v>
+        <v>16</v>
       </c>
       <c r="E190" t="inlineStr">
         <is>
@@ -5098,7 +5098,7 @@
     <row r="191">
       <c r="A191" t="inlineStr">
         <is>
-          <t>12:48:06</t>
+          <t>13:00:14</t>
         </is>
       </c>
       <c r="B191" t="inlineStr">
@@ -5108,11 +5108,11 @@
       </c>
       <c r="C191" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D191" t="n">
-        <v>16</v>
+        <v>4</v>
       </c>
       <c r="E191" t="inlineStr">
         <is>
@@ -5323,7 +5323,7 @@
     <row r="200">
       <c r="A200" t="inlineStr">
         <is>
-          <t>13:00:14</t>
+          <t>12:48:06</t>
         </is>
       </c>
       <c r="B200" t="inlineStr">
@@ -5333,11 +5333,11 @@
       </c>
       <c r="C200" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D200" t="n">
-        <v>38</v>
+        <v>50</v>
       </c>
       <c r="E200" t="inlineStr">
         <is>
@@ -5348,7 +5348,7 @@
     <row r="201">
       <c r="A201" t="inlineStr">
         <is>
-          <t>12:48:06</t>
+          <t>13:00:14</t>
         </is>
       </c>
       <c r="B201" t="inlineStr">
@@ -5358,11 +5358,11 @@
       </c>
       <c r="C201" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D201" t="n">
-        <v>50</v>
+        <v>38</v>
       </c>
       <c r="E201" t="inlineStr">
         <is>
@@ -5623,7 +5623,7 @@
     <row r="212">
       <c r="A212" t="inlineStr">
         <is>
-          <t>13:32:57</t>
+          <t>13:57:43</t>
         </is>
       </c>
       <c r="B212" t="inlineStr">
@@ -5633,11 +5633,11 @@
       </c>
       <c r="C212" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D212" t="n">
-        <v>44</v>
+        <v>19</v>
       </c>
       <c r="E212" t="inlineStr">
         <is>
@@ -5648,7 +5648,7 @@
     <row r="213">
       <c r="A213" t="inlineStr">
         <is>
-          <t>13:57:43</t>
+          <t>13:32:57</t>
         </is>
       </c>
       <c r="B213" t="inlineStr">
@@ -5658,11 +5658,11 @@
       </c>
       <c r="C213" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D213" t="n">
-        <v>19</v>
+        <v>44</v>
       </c>
       <c r="E213" t="inlineStr">
         <is>
@@ -5673,7 +5673,7 @@
     <row r="214">
       <c r="A214" t="inlineStr">
         <is>
-          <t>13:57:43</t>
+          <t>13:00:14</t>
         </is>
       </c>
       <c r="B214" t="inlineStr">
@@ -5683,11 +5683,11 @@
       </c>
       <c r="C214" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D214" t="n">
-        <v>20</v>
+        <v>77</v>
       </c>
       <c r="E214" t="inlineStr">
         <is>
@@ -5698,7 +5698,7 @@
     <row r="215">
       <c r="A215" t="inlineStr">
         <is>
-          <t>13:00:14</t>
+          <t>13:57:43</t>
         </is>
       </c>
       <c r="B215" t="inlineStr">
@@ -5708,11 +5708,11 @@
       </c>
       <c r="C215" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D215" t="n">
-        <v>77</v>
+        <v>20</v>
       </c>
       <c r="E215" t="inlineStr">
         <is>
@@ -5873,7 +5873,7 @@
     <row r="222">
       <c r="A222" t="inlineStr">
         <is>
-          <t>14:21:42</t>
+          <t>13:00:14</t>
         </is>
       </c>
       <c r="B222" t="inlineStr">
@@ -5883,11 +5883,11 @@
       </c>
       <c r="C222" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D222" t="n">
-        <v>12</v>
+        <v>93</v>
       </c>
       <c r="E222" t="inlineStr">
         <is>
@@ -5898,7 +5898,7 @@
     <row r="223">
       <c r="A223" t="inlineStr">
         <is>
-          <t>13:00:14</t>
+          <t>14:21:42</t>
         </is>
       </c>
       <c r="B223" t="inlineStr">
@@ -5908,11 +5908,11 @@
       </c>
       <c r="C223" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D223" t="n">
-        <v>93</v>
+        <v>12</v>
       </c>
       <c r="E223" t="inlineStr">
         <is>
@@ -5983,7 +5983,7 @@
       </c>
       <c r="C226" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D226" t="n">
@@ -6008,7 +6008,7 @@
       </c>
       <c r="C227" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D227" t="n">
@@ -6098,7 +6098,7 @@
     <row r="231">
       <c r="A231" t="inlineStr">
         <is>
-          <t>14:59:00</t>
+          <t>14:46:39</t>
         </is>
       </c>
       <c r="B231" t="inlineStr">
@@ -6108,11 +6108,11 @@
       </c>
       <c r="C231" t="inlineStr">
         <is>
-          <t>81_EL PELIGRO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D231" t="n">
-        <v>0</v>
+        <v>13</v>
       </c>
       <c r="E231" t="inlineStr">
         <is>
@@ -6123,7 +6123,7 @@
     <row r="232">
       <c r="A232" t="inlineStr">
         <is>
-          <t>14:46:39</t>
+          <t>14:59:00</t>
         </is>
       </c>
       <c r="B232" t="inlineStr">
@@ -6133,11 +6133,11 @@
       </c>
       <c r="C232" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>81_EL PELIGRO</t>
         </is>
       </c>
       <c r="D232" t="n">
-        <v>13</v>
+        <v>0</v>
       </c>
       <c r="E232" t="inlineStr">
         <is>
@@ -6173,7 +6173,7 @@
     <row r="234">
       <c r="A234" t="inlineStr">
         <is>
-          <t>14:59:00</t>
+          <t>14:46:39</t>
         </is>
       </c>
       <c r="B234" t="inlineStr">
@@ -6183,11 +6183,11 @@
       </c>
       <c r="C234" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D234" t="n">
-        <v>2</v>
+        <v>15</v>
       </c>
       <c r="E234" t="inlineStr">
         <is>
@@ -6198,7 +6198,7 @@
     <row r="235">
       <c r="A235" t="inlineStr">
         <is>
-          <t>14:46:39</t>
+          <t>14:59:00</t>
         </is>
       </c>
       <c r="B235" t="inlineStr">
@@ -6208,11 +6208,11 @@
       </c>
       <c r="C235" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D235" t="n">
-        <v>15</v>
+        <v>2</v>
       </c>
       <c r="E235" t="inlineStr">
         <is>
@@ -6698,7 +6698,7 @@
     <row r="255">
       <c r="A255" t="inlineStr">
         <is>
-          <t>15:34:45</t>
+          <t>14:46:39</t>
         </is>
       </c>
       <c r="B255" t="inlineStr">
@@ -6708,11 +6708,11 @@
       </c>
       <c r="C255" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D255" t="n">
-        <v>20</v>
+        <v>68</v>
       </c>
       <c r="E255" t="inlineStr">
         <is>
@@ -6723,7 +6723,7 @@
     <row r="256">
       <c r="A256" t="inlineStr">
         <is>
-          <t>14:46:39</t>
+          <t>15:34:45</t>
         </is>
       </c>
       <c r="B256" t="inlineStr">
@@ -6733,11 +6733,11 @@
       </c>
       <c r="C256" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D256" t="n">
-        <v>68</v>
+        <v>20</v>
       </c>
       <c r="E256" t="inlineStr">
         <is>
@@ -6798,21 +6798,21 @@
     <row r="259">
       <c r="A259" t="inlineStr">
         <is>
-          <t>15:34:45</t>
+          <t>16:01:44</t>
         </is>
       </c>
       <c r="B259" t="inlineStr">
         <is>
-          <t>16:09</t>
+          <t>16:01</t>
         </is>
       </c>
       <c r="C259" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D259" t="n">
-        <v>35</v>
+        <v>0</v>
       </c>
       <c r="E259" t="inlineStr">
         <is>
@@ -6823,21 +6823,21 @@
     <row r="260">
       <c r="A260" t="inlineStr">
         <is>
-          <t>15:34:45</t>
+          <t>16:01:44</t>
         </is>
       </c>
       <c r="B260" t="inlineStr">
         <is>
-          <t>16:11</t>
+          <t>16:03</t>
         </is>
       </c>
       <c r="C260" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D260" t="n">
-        <v>37</v>
+        <v>2</v>
       </c>
       <c r="E260" t="inlineStr">
         <is>
@@ -6848,21 +6848,21 @@
     <row r="261">
       <c r="A261" t="inlineStr">
         <is>
-          <t>14:59:00</t>
+          <t>16:01:44</t>
         </is>
       </c>
       <c r="B261" t="inlineStr">
         <is>
-          <t>16:12</t>
+          <t>16:09</t>
         </is>
       </c>
       <c r="C261" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D261" t="n">
-        <v>73</v>
+        <v>8</v>
       </c>
       <c r="E261" t="inlineStr">
         <is>
@@ -6873,21 +6873,21 @@
     <row r="262">
       <c r="A262" t="inlineStr">
         <is>
-          <t>15:34:45</t>
+          <t>16:01:44</t>
         </is>
       </c>
       <c r="B262" t="inlineStr">
         <is>
-          <t>16:23</t>
+          <t>16:11</t>
         </is>
       </c>
       <c r="C262" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D262" t="n">
-        <v>49</v>
+        <v>10</v>
       </c>
       <c r="E262" t="inlineStr">
         <is>
@@ -6898,21 +6898,21 @@
     <row r="263">
       <c r="A263" t="inlineStr">
         <is>
-          <t>15:34:45</t>
+          <t>14:59:00</t>
         </is>
       </c>
       <c r="B263" t="inlineStr">
         <is>
-          <t>16:23</t>
+          <t>16:12</t>
         </is>
       </c>
       <c r="C263" t="inlineStr">
         <is>
-          <t>215_ALUAR</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D263" t="n">
-        <v>49</v>
+        <v>73</v>
       </c>
       <c r="E263" t="inlineStr">
         <is>
@@ -6923,21 +6923,21 @@
     <row r="264">
       <c r="A264" t="inlineStr">
         <is>
-          <t>14:59:00</t>
+          <t>16:01:44</t>
         </is>
       </c>
       <c r="B264" t="inlineStr">
         <is>
-          <t>16:24</t>
+          <t>16:23</t>
         </is>
       </c>
       <c r="C264" t="inlineStr">
         <is>
-          <t>215_ALUAR</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D264" t="n">
-        <v>85</v>
+        <v>22</v>
       </c>
       <c r="E264" t="inlineStr">
         <is>
@@ -6948,21 +6948,21 @@
     <row r="265">
       <c r="A265" t="inlineStr">
         <is>
-          <t>14:59:00</t>
+          <t>16:01:44</t>
         </is>
       </c>
       <c r="B265" t="inlineStr">
         <is>
-          <t>16:25</t>
+          <t>16:23</t>
         </is>
       </c>
       <c r="C265" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>215_ALUAR</t>
         </is>
       </c>
       <c r="D265" t="n">
-        <v>86</v>
+        <v>22</v>
       </c>
       <c r="E265" t="inlineStr">
         <is>
@@ -6973,21 +6973,21 @@
     <row r="266">
       <c r="A266" t="inlineStr">
         <is>
-          <t>15:34:45</t>
+          <t>14:59:00</t>
         </is>
       </c>
       <c r="B266" t="inlineStr">
         <is>
-          <t>16:35</t>
+          <t>16:24</t>
         </is>
       </c>
       <c r="C266" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>215_ALUAR</t>
         </is>
       </c>
       <c r="D266" t="n">
-        <v>61</v>
+        <v>85</v>
       </c>
       <c r="E266" t="inlineStr">
         <is>
@@ -6998,21 +6998,21 @@
     <row r="267">
       <c r="A267" t="inlineStr">
         <is>
-          <t>15:34:45</t>
+          <t>14:59:00</t>
         </is>
       </c>
       <c r="B267" t="inlineStr">
         <is>
-          <t>16:35</t>
+          <t>16:25</t>
         </is>
       </c>
       <c r="C267" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D267" t="n">
-        <v>61</v>
+        <v>86</v>
       </c>
       <c r="E267" t="inlineStr">
         <is>
@@ -7023,12 +7023,12 @@
     <row r="268">
       <c r="A268" t="inlineStr">
         <is>
-          <t>15:34:45</t>
+          <t>16:01:44</t>
         </is>
       </c>
       <c r="B268" t="inlineStr">
         <is>
-          <t>16:36</t>
+          <t>16:33</t>
         </is>
       </c>
       <c r="C268" t="inlineStr">
@@ -7037,7 +7037,7 @@
         </is>
       </c>
       <c r="D268" t="n">
-        <v>62</v>
+        <v>32</v>
       </c>
       <c r="E268" t="inlineStr">
         <is>
@@ -7048,12 +7048,12 @@
     <row r="269">
       <c r="A269" t="inlineStr">
         <is>
-          <t>14:59:00</t>
+          <t>16:01:44</t>
         </is>
       </c>
       <c r="B269" t="inlineStr">
         <is>
-          <t>16:36</t>
+          <t>16:35</t>
         </is>
       </c>
       <c r="C269" t="inlineStr">
@@ -7062,7 +7062,7 @@
         </is>
       </c>
       <c r="D269" t="n">
-        <v>97</v>
+        <v>34</v>
       </c>
       <c r="E269" t="inlineStr">
         <is>
@@ -7073,21 +7073,21 @@
     <row r="270">
       <c r="A270" t="inlineStr">
         <is>
-          <t>15:34:45</t>
+          <t>16:01:44</t>
         </is>
       </c>
       <c r="B270" t="inlineStr">
         <is>
-          <t>16:47</t>
+          <t>16:35</t>
         </is>
       </c>
       <c r="C270" t="inlineStr">
         <is>
-          <t>225_GOMEZ</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D270" t="n">
-        <v>73</v>
+        <v>34</v>
       </c>
       <c r="E270" t="inlineStr">
         <is>
@@ -7103,16 +7103,16 @@
       </c>
       <c r="B271" t="inlineStr">
         <is>
-          <t>16:51</t>
+          <t>16:36</t>
         </is>
       </c>
       <c r="C271" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D271" t="n">
-        <v>77</v>
+        <v>62</v>
       </c>
       <c r="E271" t="inlineStr">
         <is>
@@ -7123,21 +7123,21 @@
     <row r="272">
       <c r="A272" t="inlineStr">
         <is>
-          <t>15:34:45</t>
+          <t>14:59:00</t>
         </is>
       </c>
       <c r="B272" t="inlineStr">
         <is>
-          <t>16:59</t>
+          <t>16:36</t>
         </is>
       </c>
       <c r="C272" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D272" t="n">
-        <v>85</v>
+        <v>97</v>
       </c>
       <c r="E272" t="inlineStr">
         <is>
@@ -7148,21 +7148,21 @@
     <row r="273">
       <c r="A273" t="inlineStr">
         <is>
-          <t>15:34:45</t>
+          <t>16:01:44</t>
         </is>
       </c>
       <c r="B273" t="inlineStr">
         <is>
-          <t>16:59</t>
+          <t>16:47</t>
         </is>
       </c>
       <c r="C273" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>225_GOMEZ</t>
         </is>
       </c>
       <c r="D273" t="n">
-        <v>85</v>
+        <v>46</v>
       </c>
       <c r="E273" t="inlineStr">
         <is>
@@ -7173,21 +7173,21 @@
     <row r="274">
       <c r="A274" t="inlineStr">
         <is>
-          <t>15:34:45</t>
+          <t>16:01:44</t>
         </is>
       </c>
       <c r="B274" t="inlineStr">
         <is>
-          <t>17:11</t>
+          <t>16:48</t>
         </is>
       </c>
       <c r="C274" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D274" t="n">
-        <v>97</v>
+        <v>47</v>
       </c>
       <c r="E274" t="inlineStr">
         <is>
@@ -7198,23 +7198,373 @@
     <row r="275">
       <c r="A275" t="inlineStr">
         <is>
+          <t>16:01:44</t>
+        </is>
+      </c>
+      <c r="B275" t="inlineStr">
+        <is>
+          <t>16:51</t>
+        </is>
+      </c>
+      <c r="C275" t="inlineStr">
+        <is>
+          <t>16_P MOR-SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D275" t="n">
+        <v>50</v>
+      </c>
+      <c r="E275" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="276">
+      <c r="A276" t="inlineStr">
+        <is>
+          <t>16:01:44</t>
+        </is>
+      </c>
+      <c r="B276" t="inlineStr">
+        <is>
+          <t>16:59</t>
+        </is>
+      </c>
+      <c r="C276" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D276" t="n">
+        <v>58</v>
+      </c>
+      <c r="E276" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="277">
+      <c r="A277" t="inlineStr">
+        <is>
+          <t>16:01:44</t>
+        </is>
+      </c>
+      <c r="B277" t="inlineStr">
+        <is>
+          <t>16:59</t>
+        </is>
+      </c>
+      <c r="C277" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D277" t="n">
+        <v>58</v>
+      </c>
+      <c r="E277" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="278">
+      <c r="A278" t="inlineStr">
+        <is>
+          <t>16:01:44</t>
+        </is>
+      </c>
+      <c r="B278" t="inlineStr">
+        <is>
+          <t>17:11</t>
+        </is>
+      </c>
+      <c r="C278" t="inlineStr">
+        <is>
+          <t>17_ROMERO</t>
+        </is>
+      </c>
+      <c r="D278" t="n">
+        <v>70</v>
+      </c>
+      <c r="E278" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="279">
+      <c r="A279" t="inlineStr">
+        <is>
           <t>15:34:45</t>
         </is>
       </c>
-      <c r="B275" t="inlineStr">
+      <c r="B279" t="inlineStr">
         <is>
           <t>17:19</t>
         </is>
       </c>
-      <c r="C275" t="inlineStr">
+      <c r="C279" t="inlineStr">
         <is>
           <t>16_SANTA ANA</t>
         </is>
       </c>
-      <c r="D275" t="n">
+      <c r="D279" t="n">
         <v>105</v>
       </c>
-      <c r="E275" t="inlineStr">
+      <c r="E279" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="280">
+      <c r="A280" t="inlineStr">
+        <is>
+          <t>16:01:44</t>
+        </is>
+      </c>
+      <c r="B280" t="inlineStr">
+        <is>
+          <t>17:21</t>
+        </is>
+      </c>
+      <c r="C280" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D280" t="n">
+        <v>80</v>
+      </c>
+      <c r="E280" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="281">
+      <c r="A281" t="inlineStr">
+        <is>
+          <t>16:01:44</t>
+        </is>
+      </c>
+      <c r="B281" t="inlineStr">
+        <is>
+          <t>17:23</t>
+        </is>
+      </c>
+      <c r="C281" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D281" t="n">
+        <v>82</v>
+      </c>
+      <c r="E281" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="282">
+      <c r="A282" t="inlineStr">
+        <is>
+          <t>16:01:44</t>
+        </is>
+      </c>
+      <c r="B282" t="inlineStr">
+        <is>
+          <t>17:35</t>
+        </is>
+      </c>
+      <c r="C282" t="inlineStr">
+        <is>
+          <t>17X38_ROMERO</t>
+        </is>
+      </c>
+      <c r="D282" t="n">
+        <v>94</v>
+      </c>
+      <c r="E282" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="283">
+      <c r="A283" t="inlineStr">
+        <is>
+          <t>16:01:44</t>
+        </is>
+      </c>
+      <c r="B283" t="inlineStr">
+        <is>
+          <t>17:35</t>
+        </is>
+      </c>
+      <c r="C283" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D283" t="n">
+        <v>94</v>
+      </c>
+      <c r="E283" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="284">
+      <c r="A284" t="inlineStr">
+        <is>
+          <t>16:01:44</t>
+        </is>
+      </c>
+      <c r="B284" t="inlineStr">
+        <is>
+          <t>17:38</t>
+        </is>
+      </c>
+      <c r="C284" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D284" t="n">
+        <v>97</v>
+      </c>
+      <c r="E284" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="285">
+      <c r="A285" t="inlineStr">
+        <is>
+          <t>16:01:44</t>
+        </is>
+      </c>
+      <c r="B285" t="inlineStr">
+        <is>
+          <t>17:47</t>
+        </is>
+      </c>
+      <c r="C285" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D285" t="n">
+        <v>106</v>
+      </c>
+      <c r="E285" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="286">
+      <c r="A286" t="inlineStr">
+        <is>
+          <t>16:01:44</t>
+        </is>
+      </c>
+      <c r="B286" t="inlineStr">
+        <is>
+          <t>17:47</t>
+        </is>
+      </c>
+      <c r="C286" t="inlineStr">
+        <is>
+          <t>215_EL PELIGRO</t>
+        </is>
+      </c>
+      <c r="D286" t="n">
+        <v>106</v>
+      </c>
+      <c r="E286" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="287">
+      <c r="A287" t="inlineStr">
+        <is>
+          <t>16:01:44</t>
+        </is>
+      </c>
+      <c r="B287" t="inlineStr">
+        <is>
+          <t>17:51</t>
+        </is>
+      </c>
+      <c r="C287" t="inlineStr">
+        <is>
+          <t>16_P MOR-SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D287" t="n">
+        <v>110</v>
+      </c>
+      <c r="E287" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="288">
+      <c r="A288" t="inlineStr">
+        <is>
+          <t>16:01:44</t>
+        </is>
+      </c>
+      <c r="B288" t="inlineStr">
+        <is>
+          <t>17:59</t>
+        </is>
+      </c>
+      <c r="C288" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D288" t="n">
+        <v>118</v>
+      </c>
+      <c r="E288" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="289">
+      <c r="A289" t="inlineStr">
+        <is>
+          <t>16:01:44</t>
+        </is>
+      </c>
+      <c r="B289" t="inlineStr">
+        <is>
+          <t>17:59</t>
+        </is>
+      </c>
+      <c r="C289" t="inlineStr">
+        <is>
+          <t>17_ROMERO</t>
+        </is>
+      </c>
+      <c r="D289" t="n">
+        <v>118</v>
+      </c>
+      <c r="E289" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -7231,7 +7581,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E48"/>
+  <dimension ref="A1:E50"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -7244,14 +7594,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 15:34:45</t>
+          <t>Última actualización: 16:01:44</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 43</t>
+          <t>Total filas: 45</t>
         </is>
       </c>
     </row>
@@ -8285,7 +8635,7 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>15:34:45</t>
+          <t>16:01:44</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
@@ -8299,7 +8649,7 @@
         </is>
       </c>
       <c r="D46" t="n">
-        <v>49</v>
+        <v>22</v>
       </c>
       <c r="E46" t="inlineStr">
         <is>
@@ -8335,7 +8685,7 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>15:34:45</t>
+          <t>16:01:44</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
@@ -8349,9 +8699,59 @@
         </is>
       </c>
       <c r="D48" t="n">
-        <v>85</v>
+        <v>58</v>
       </c>
       <c r="E48" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>16:01:44</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>17:47</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>215_EL PELIGRO</t>
+        </is>
+      </c>
+      <c r="D49" t="n">
+        <v>106</v>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>16:01:44</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>17:47</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D50" t="n">
+        <v>106</v>
+      </c>
+      <c r="E50" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -8381,7 +8781,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 15:34:45</t>
+          <t>Última actualización: 16:01:44</t>
         </is>
       </c>
     </row>
@@ -9547,7 +9947,7 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>15:34:45</t>
+          <t>16:01:44</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
@@ -9561,7 +9961,7 @@
         </is>
       </c>
       <c r="D51" t="n">
-        <v>68</v>
+        <v>41</v>
       </c>
       <c r="E51" t="inlineStr">
         <is>
@@ -9597,7 +9997,7 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>15:34:45</t>
+          <t>16:01:44</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
@@ -9611,7 +10011,7 @@
         </is>
       </c>
       <c r="D53" t="n">
-        <v>81</v>
+        <v>54</v>
       </c>
       <c r="E53" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 1816
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-03-21.xlsx
+++ b/data/horarios-141-2026-03-21.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E289"/>
+  <dimension ref="A1:E301"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 16:01:44</t>
+          <t>Última actualización: 16:33:34</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 284</t>
+          <t>Total filas: 296</t>
         </is>
       </c>
     </row>
@@ -1973,7 +1973,7 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>07:27:35</t>
+          <t>07:51:37</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
@@ -1983,11 +1983,11 @@
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D66" t="n">
-        <v>52</v>
+        <v>28</v>
       </c>
       <c r="E66" t="inlineStr">
         <is>
@@ -2008,7 +2008,7 @@
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D67" t="n">
@@ -2023,7 +2023,7 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>07:51:37</t>
+          <t>07:27:35</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
@@ -2033,11 +2033,11 @@
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D68" t="n">
-        <v>28</v>
+        <v>52</v>
       </c>
       <c r="E68" t="inlineStr">
         <is>
@@ -2698,7 +2698,7 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>08:50:55</t>
+          <t>08:14:14</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
@@ -2708,11 +2708,11 @@
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D95" t="n">
-        <v>28</v>
+        <v>64</v>
       </c>
       <c r="E95" t="inlineStr">
         <is>
@@ -2733,7 +2733,7 @@
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>215_EL PELIGRO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D96" t="n">
@@ -2748,7 +2748,7 @@
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>08:14:14</t>
+          <t>08:50:55</t>
         </is>
       </c>
       <c r="B97" t="inlineStr">
@@ -2758,11 +2758,11 @@
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>215_EL PELIGRO</t>
         </is>
       </c>
       <c r="D97" t="n">
-        <v>64</v>
+        <v>28</v>
       </c>
       <c r="E97" t="inlineStr">
         <is>
@@ -2923,7 +2923,7 @@
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>08:14:14</t>
+          <t>09:23:24</t>
         </is>
       </c>
       <c r="B104" t="inlineStr">
@@ -2933,11 +2933,11 @@
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D104" t="n">
-        <v>79</v>
+        <v>10</v>
       </c>
       <c r="E104" t="inlineStr">
         <is>
@@ -2948,7 +2948,7 @@
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>09:23:24</t>
+          <t>08:14:14</t>
         </is>
       </c>
       <c r="B105" t="inlineStr">
@@ -2958,11 +2958,11 @@
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D105" t="n">
-        <v>10</v>
+        <v>79</v>
       </c>
       <c r="E105" t="inlineStr">
         <is>
@@ -3083,7 +3083,7 @@
       </c>
       <c r="C110" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D110" t="n">
@@ -3108,7 +3108,7 @@
       </c>
       <c r="C111" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D111" t="n">
@@ -3173,7 +3173,7 @@
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>09:23:24</t>
+          <t>08:50:55</t>
         </is>
       </c>
       <c r="B114" t="inlineStr">
@@ -3183,11 +3183,11 @@
       </c>
       <c r="C114" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D114" t="n">
-        <v>40</v>
+        <v>73</v>
       </c>
       <c r="E114" t="inlineStr">
         <is>
@@ -3198,7 +3198,7 @@
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>08:50:55</t>
+          <t>09:23:24</t>
         </is>
       </c>
       <c r="B115" t="inlineStr">
@@ -3208,11 +3208,11 @@
       </c>
       <c r="C115" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D115" t="n">
-        <v>73</v>
+        <v>40</v>
       </c>
       <c r="E115" t="inlineStr">
         <is>
@@ -3598,7 +3598,7 @@
     <row r="131">
       <c r="A131" t="inlineStr">
         <is>
-          <t>09:23:24</t>
+          <t>10:14:52</t>
         </is>
       </c>
       <c r="B131" t="inlineStr">
@@ -3608,11 +3608,11 @@
       </c>
       <c r="C131" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D131" t="n">
-        <v>80</v>
+        <v>29</v>
       </c>
       <c r="E131" t="inlineStr">
         <is>
@@ -3623,7 +3623,7 @@
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t>10:14:52</t>
+          <t>09:23:24</t>
         </is>
       </c>
       <c r="B132" t="inlineStr">
@@ -3633,11 +3633,11 @@
       </c>
       <c r="C132" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D132" t="n">
-        <v>29</v>
+        <v>80</v>
       </c>
       <c r="E132" t="inlineStr">
         <is>
@@ -4648,7 +4648,7 @@
     <row r="173">
       <c r="A173" t="inlineStr">
         <is>
-          <t>12:28:38</t>
+          <t>12:00:15</t>
         </is>
       </c>
       <c r="B173" t="inlineStr">
@@ -4658,11 +4658,11 @@
       </c>
       <c r="C173" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D173" t="n">
-        <v>5</v>
+        <v>33</v>
       </c>
       <c r="E173" t="inlineStr">
         <is>
@@ -4683,7 +4683,7 @@
       </c>
       <c r="C174" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D174" t="n">
@@ -4698,7 +4698,7 @@
     <row r="175">
       <c r="A175" t="inlineStr">
         <is>
-          <t>12:00:15</t>
+          <t>12:28:38</t>
         </is>
       </c>
       <c r="B175" t="inlineStr">
@@ -4708,11 +4708,11 @@
       </c>
       <c r="C175" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D175" t="n">
-        <v>33</v>
+        <v>5</v>
       </c>
       <c r="E175" t="inlineStr">
         <is>
@@ -4998,7 +4998,7 @@
     <row r="187">
       <c r="A187" t="inlineStr">
         <is>
-          <t>13:00:14</t>
+          <t>12:28:38</t>
         </is>
       </c>
       <c r="B187" t="inlineStr">
@@ -5008,11 +5008,11 @@
       </c>
       <c r="C187" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D187" t="n">
-        <v>3</v>
+        <v>35</v>
       </c>
       <c r="E187" t="inlineStr">
         <is>
@@ -5033,7 +5033,7 @@
       </c>
       <c r="C188" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D188" t="n">
@@ -5048,7 +5048,7 @@
     <row r="189">
       <c r="A189" t="inlineStr">
         <is>
-          <t>12:28:38</t>
+          <t>13:00:14</t>
         </is>
       </c>
       <c r="B189" t="inlineStr">
@@ -5058,11 +5058,11 @@
       </c>
       <c r="C189" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D189" t="n">
-        <v>35</v>
+        <v>3</v>
       </c>
       <c r="E189" t="inlineStr">
         <is>
@@ -5073,7 +5073,7 @@
     <row r="190">
       <c r="A190" t="inlineStr">
         <is>
-          <t>12:48:06</t>
+          <t>13:00:14</t>
         </is>
       </c>
       <c r="B190" t="inlineStr">
@@ -5083,11 +5083,11 @@
       </c>
       <c r="C190" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D190" t="n">
-        <v>16</v>
+        <v>4</v>
       </c>
       <c r="E190" t="inlineStr">
         <is>
@@ -5098,7 +5098,7 @@
     <row r="191">
       <c r="A191" t="inlineStr">
         <is>
-          <t>13:00:14</t>
+          <t>12:48:06</t>
         </is>
       </c>
       <c r="B191" t="inlineStr">
@@ -5108,11 +5108,11 @@
       </c>
       <c r="C191" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D191" t="n">
-        <v>4</v>
+        <v>16</v>
       </c>
       <c r="E191" t="inlineStr">
         <is>
@@ -5498,7 +5498,7 @@
     <row r="207">
       <c r="A207" t="inlineStr">
         <is>
-          <t>13:57:43</t>
+          <t>13:32:57</t>
         </is>
       </c>
       <c r="B207" t="inlineStr">
@@ -5508,11 +5508,11 @@
       </c>
       <c r="C207" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D207" t="n">
-        <v>2</v>
+        <v>27</v>
       </c>
       <c r="E207" t="inlineStr">
         <is>
@@ -5523,7 +5523,7 @@
     <row r="208">
       <c r="A208" t="inlineStr">
         <is>
-          <t>13:32:57</t>
+          <t>13:57:43</t>
         </is>
       </c>
       <c r="B208" t="inlineStr">
@@ -5533,11 +5533,11 @@
       </c>
       <c r="C208" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D208" t="n">
-        <v>27</v>
+        <v>2</v>
       </c>
       <c r="E208" t="inlineStr">
         <is>
@@ -5573,7 +5573,7 @@
     <row r="210">
       <c r="A210" t="inlineStr">
         <is>
-          <t>13:57:43</t>
+          <t>13:00:14</t>
         </is>
       </c>
       <c r="B210" t="inlineStr">
@@ -5583,11 +5583,11 @@
       </c>
       <c r="C210" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D210" t="n">
-        <v>6</v>
+        <v>63</v>
       </c>
       <c r="E210" t="inlineStr">
         <is>
@@ -5598,7 +5598,7 @@
     <row r="211">
       <c r="A211" t="inlineStr">
         <is>
-          <t>13:00:14</t>
+          <t>13:57:43</t>
         </is>
       </c>
       <c r="B211" t="inlineStr">
@@ -5608,11 +5608,11 @@
       </c>
       <c r="C211" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D211" t="n">
-        <v>63</v>
+        <v>6</v>
       </c>
       <c r="E211" t="inlineStr">
         <is>
@@ -5873,7 +5873,7 @@
     <row r="222">
       <c r="A222" t="inlineStr">
         <is>
-          <t>13:00:14</t>
+          <t>14:21:42</t>
         </is>
       </c>
       <c r="B222" t="inlineStr">
@@ -5883,11 +5883,11 @@
       </c>
       <c r="C222" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D222" t="n">
-        <v>93</v>
+        <v>12</v>
       </c>
       <c r="E222" t="inlineStr">
         <is>
@@ -5898,7 +5898,7 @@
     <row r="223">
       <c r="A223" t="inlineStr">
         <is>
-          <t>14:21:42</t>
+          <t>13:00:14</t>
         </is>
       </c>
       <c r="B223" t="inlineStr">
@@ -5908,11 +5908,11 @@
       </c>
       <c r="C223" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D223" t="n">
-        <v>12</v>
+        <v>93</v>
       </c>
       <c r="E223" t="inlineStr">
         <is>
@@ -5983,7 +5983,7 @@
       </c>
       <c r="C226" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D226" t="n">
@@ -6008,7 +6008,7 @@
       </c>
       <c r="C227" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D227" t="n">
@@ -6298,7 +6298,7 @@
     <row r="239">
       <c r="A239" t="inlineStr">
         <is>
-          <t>14:46:39</t>
+          <t>14:59:00</t>
         </is>
       </c>
       <c r="B239" t="inlineStr">
@@ -6308,11 +6308,11 @@
       </c>
       <c r="C239" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D239" t="n">
-        <v>25</v>
+        <v>12</v>
       </c>
       <c r="E239" t="inlineStr">
         <is>
@@ -6323,7 +6323,7 @@
     <row r="240">
       <c r="A240" t="inlineStr">
         <is>
-          <t>14:59:00</t>
+          <t>14:46:39</t>
         </is>
       </c>
       <c r="B240" t="inlineStr">
@@ -6333,11 +6333,11 @@
       </c>
       <c r="C240" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D240" t="n">
-        <v>12</v>
+        <v>25</v>
       </c>
       <c r="E240" t="inlineStr">
         <is>
@@ -7023,7 +7023,7 @@
     <row r="268">
       <c r="A268" t="inlineStr">
         <is>
-          <t>16:01:44</t>
+          <t>16:33:34</t>
         </is>
       </c>
       <c r="B268" t="inlineStr">
@@ -7037,7 +7037,7 @@
         </is>
       </c>
       <c r="D268" t="n">
-        <v>32</v>
+        <v>0</v>
       </c>
       <c r="E268" t="inlineStr">
         <is>
@@ -7048,12 +7048,12 @@
     <row r="269">
       <c r="A269" t="inlineStr">
         <is>
-          <t>16:01:44</t>
+          <t>16:33:34</t>
         </is>
       </c>
       <c r="B269" t="inlineStr">
         <is>
-          <t>16:35</t>
+          <t>16:33</t>
         </is>
       </c>
       <c r="C269" t="inlineStr">
@@ -7062,7 +7062,7 @@
         </is>
       </c>
       <c r="D269" t="n">
-        <v>34</v>
+        <v>0</v>
       </c>
       <c r="E269" t="inlineStr">
         <is>
@@ -7073,7 +7073,7 @@
     <row r="270">
       <c r="A270" t="inlineStr">
         <is>
-          <t>16:01:44</t>
+          <t>16:33:34</t>
         </is>
       </c>
       <c r="B270" t="inlineStr">
@@ -7087,7 +7087,7 @@
         </is>
       </c>
       <c r="D270" t="n">
-        <v>34</v>
+        <v>2</v>
       </c>
       <c r="E270" t="inlineStr">
         <is>
@@ -7098,21 +7098,21 @@
     <row r="271">
       <c r="A271" t="inlineStr">
         <is>
-          <t>15:34:45</t>
+          <t>16:01:44</t>
         </is>
       </c>
       <c r="B271" t="inlineStr">
         <is>
-          <t>16:36</t>
+          <t>16:35</t>
         </is>
       </c>
       <c r="C271" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D271" t="n">
-        <v>62</v>
+        <v>34</v>
       </c>
       <c r="E271" t="inlineStr">
         <is>
@@ -7148,21 +7148,21 @@
     <row r="273">
       <c r="A273" t="inlineStr">
         <is>
-          <t>16:01:44</t>
+          <t>15:34:45</t>
         </is>
       </c>
       <c r="B273" t="inlineStr">
         <is>
-          <t>16:47</t>
+          <t>16:36</t>
         </is>
       </c>
       <c r="C273" t="inlineStr">
         <is>
-          <t>225_GOMEZ</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D273" t="n">
-        <v>46</v>
+        <v>62</v>
       </c>
       <c r="E273" t="inlineStr">
         <is>
@@ -7173,21 +7173,21 @@
     <row r="274">
       <c r="A274" t="inlineStr">
         <is>
-          <t>16:01:44</t>
+          <t>16:33:34</t>
         </is>
       </c>
       <c r="B274" t="inlineStr">
         <is>
-          <t>16:48</t>
+          <t>16:37</t>
         </is>
       </c>
       <c r="C274" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>225_GOMEZ</t>
         </is>
       </c>
       <c r="D274" t="n">
-        <v>47</v>
+        <v>4</v>
       </c>
       <c r="E274" t="inlineStr">
         <is>
@@ -7203,16 +7203,16 @@
       </c>
       <c r="B275" t="inlineStr">
         <is>
-          <t>16:51</t>
+          <t>16:47</t>
         </is>
       </c>
       <c r="C275" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>225_GOMEZ</t>
         </is>
       </c>
       <c r="D275" t="n">
-        <v>50</v>
+        <v>46</v>
       </c>
       <c r="E275" t="inlineStr">
         <is>
@@ -7223,21 +7223,21 @@
     <row r="276">
       <c r="A276" t="inlineStr">
         <is>
-          <t>16:01:44</t>
+          <t>16:33:34</t>
         </is>
       </c>
       <c r="B276" t="inlineStr">
         <is>
-          <t>16:59</t>
+          <t>16:48</t>
         </is>
       </c>
       <c r="C276" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D276" t="n">
-        <v>58</v>
+        <v>15</v>
       </c>
       <c r="E276" t="inlineStr">
         <is>
@@ -7248,21 +7248,21 @@
     <row r="277">
       <c r="A277" t="inlineStr">
         <is>
-          <t>16:01:44</t>
+          <t>16:33:34</t>
         </is>
       </c>
       <c r="B277" t="inlineStr">
         <is>
-          <t>16:59</t>
+          <t>16:51</t>
         </is>
       </c>
       <c r="C277" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D277" t="n">
-        <v>58</v>
+        <v>18</v>
       </c>
       <c r="E277" t="inlineStr">
         <is>
@@ -7273,21 +7273,21 @@
     <row r="278">
       <c r="A278" t="inlineStr">
         <is>
-          <t>16:01:44</t>
+          <t>16:33:34</t>
         </is>
       </c>
       <c r="B278" t="inlineStr">
         <is>
-          <t>17:11</t>
+          <t>16:59</t>
         </is>
       </c>
       <c r="C278" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D278" t="n">
-        <v>70</v>
+        <v>26</v>
       </c>
       <c r="E278" t="inlineStr">
         <is>
@@ -7298,21 +7298,21 @@
     <row r="279">
       <c r="A279" t="inlineStr">
         <is>
-          <t>15:34:45</t>
+          <t>16:01:44</t>
         </is>
       </c>
       <c r="B279" t="inlineStr">
         <is>
-          <t>17:19</t>
+          <t>16:59</t>
         </is>
       </c>
       <c r="C279" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D279" t="n">
-        <v>105</v>
+        <v>58</v>
       </c>
       <c r="E279" t="inlineStr">
         <is>
@@ -7323,21 +7323,21 @@
     <row r="280">
       <c r="A280" t="inlineStr">
         <is>
-          <t>16:01:44</t>
+          <t>16:33:34</t>
         </is>
       </c>
       <c r="B280" t="inlineStr">
         <is>
-          <t>17:21</t>
+          <t>17:00</t>
         </is>
       </c>
       <c r="C280" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D280" t="n">
-        <v>80</v>
+        <v>27</v>
       </c>
       <c r="E280" t="inlineStr">
         <is>
@@ -7348,21 +7348,21 @@
     <row r="281">
       <c r="A281" t="inlineStr">
         <is>
-          <t>16:01:44</t>
+          <t>16:33:34</t>
         </is>
       </c>
       <c r="B281" t="inlineStr">
         <is>
-          <t>17:23</t>
+          <t>17:03</t>
         </is>
       </c>
       <c r="C281" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D281" t="n">
-        <v>82</v>
+        <v>30</v>
       </c>
       <c r="E281" t="inlineStr">
         <is>
@@ -7378,16 +7378,16 @@
       </c>
       <c r="B282" t="inlineStr">
         <is>
-          <t>17:35</t>
+          <t>17:11</t>
         </is>
       </c>
       <c r="C282" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D282" t="n">
-        <v>94</v>
+        <v>70</v>
       </c>
       <c r="E282" t="inlineStr">
         <is>
@@ -7398,21 +7398,21 @@
     <row r="283">
       <c r="A283" t="inlineStr">
         <is>
-          <t>16:01:44</t>
+          <t>16:33:34</t>
         </is>
       </c>
       <c r="B283" t="inlineStr">
         <is>
-          <t>17:35</t>
+          <t>17:12</t>
         </is>
       </c>
       <c r="C283" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D283" t="n">
-        <v>94</v>
+        <v>39</v>
       </c>
       <c r="E283" t="inlineStr">
         <is>
@@ -7423,21 +7423,21 @@
     <row r="284">
       <c r="A284" t="inlineStr">
         <is>
-          <t>16:01:44</t>
+          <t>15:34:45</t>
         </is>
       </c>
       <c r="B284" t="inlineStr">
         <is>
-          <t>17:38</t>
+          <t>17:19</t>
         </is>
       </c>
       <c r="C284" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D284" t="n">
-        <v>97</v>
+        <v>105</v>
       </c>
       <c r="E284" t="inlineStr">
         <is>
@@ -7448,21 +7448,21 @@
     <row r="285">
       <c r="A285" t="inlineStr">
         <is>
-          <t>16:01:44</t>
+          <t>16:33:34</t>
         </is>
       </c>
       <c r="B285" t="inlineStr">
         <is>
-          <t>17:47</t>
+          <t>17:21</t>
         </is>
       </c>
       <c r="C285" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D285" t="n">
-        <v>106</v>
+        <v>48</v>
       </c>
       <c r="E285" t="inlineStr">
         <is>
@@ -7473,21 +7473,21 @@
     <row r="286">
       <c r="A286" t="inlineStr">
         <is>
-          <t>16:01:44</t>
+          <t>16:33:34</t>
         </is>
       </c>
       <c r="B286" t="inlineStr">
         <is>
-          <t>17:47</t>
+          <t>17:23</t>
         </is>
       </c>
       <c r="C286" t="inlineStr">
         <is>
-          <t>215_EL PELIGRO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D286" t="n">
-        <v>106</v>
+        <v>50</v>
       </c>
       <c r="E286" t="inlineStr">
         <is>
@@ -7498,21 +7498,21 @@
     <row r="287">
       <c r="A287" t="inlineStr">
         <is>
-          <t>16:01:44</t>
+          <t>16:33:34</t>
         </is>
       </c>
       <c r="B287" t="inlineStr">
         <is>
-          <t>17:51</t>
+          <t>17:24</t>
         </is>
       </c>
       <c r="C287" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D287" t="n">
-        <v>110</v>
+        <v>51</v>
       </c>
       <c r="E287" t="inlineStr">
         <is>
@@ -7523,12 +7523,12 @@
     <row r="288">
       <c r="A288" t="inlineStr">
         <is>
-          <t>16:01:44</t>
+          <t>16:33:34</t>
         </is>
       </c>
       <c r="B288" t="inlineStr">
         <is>
-          <t>17:59</t>
+          <t>17:35</t>
         </is>
       </c>
       <c r="C288" t="inlineStr">
@@ -7537,7 +7537,7 @@
         </is>
       </c>
       <c r="D288" t="n">
-        <v>118</v>
+        <v>62</v>
       </c>
       <c r="E288" t="inlineStr">
         <is>
@@ -7548,23 +7548,323 @@
     <row r="289">
       <c r="A289" t="inlineStr">
         <is>
+          <t>16:33:34</t>
+        </is>
+      </c>
+      <c r="B289" t="inlineStr">
+        <is>
+          <t>17:35</t>
+        </is>
+      </c>
+      <c r="C289" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D289" t="n">
+        <v>62</v>
+      </c>
+      <c r="E289" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="290">
+      <c r="A290" t="inlineStr">
+        <is>
+          <t>16:33:34</t>
+        </is>
+      </c>
+      <c r="B290" t="inlineStr">
+        <is>
+          <t>17:35</t>
+        </is>
+      </c>
+      <c r="C290" t="inlineStr">
+        <is>
+          <t>17X38_ROMERO</t>
+        </is>
+      </c>
+      <c r="D290" t="n">
+        <v>62</v>
+      </c>
+      <c r="E290" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="291">
+      <c r="A291" t="inlineStr">
+        <is>
           <t>16:01:44</t>
         </is>
       </c>
-      <c r="B289" t="inlineStr">
+      <c r="B291" t="inlineStr">
+        <is>
+          <t>17:38</t>
+        </is>
+      </c>
+      <c r="C291" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D291" t="n">
+        <v>97</v>
+      </c>
+      <c r="E291" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="292">
+      <c r="A292" t="inlineStr">
+        <is>
+          <t>16:33:34</t>
+        </is>
+      </c>
+      <c r="B292" t="inlineStr">
+        <is>
+          <t>17:41</t>
+        </is>
+      </c>
+      <c r="C292" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D292" t="n">
+        <v>68</v>
+      </c>
+      <c r="E292" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="293">
+      <c r="A293" t="inlineStr">
+        <is>
+          <t>16:33:34</t>
+        </is>
+      </c>
+      <c r="B293" t="inlineStr">
+        <is>
+          <t>17:47</t>
+        </is>
+      </c>
+      <c r="C293" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D293" t="n">
+        <v>74</v>
+      </c>
+      <c r="E293" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="294">
+      <c r="A294" t="inlineStr">
+        <is>
+          <t>16:01:44</t>
+        </is>
+      </c>
+      <c r="B294" t="inlineStr">
+        <is>
+          <t>17:47</t>
+        </is>
+      </c>
+      <c r="C294" t="inlineStr">
+        <is>
+          <t>215_EL PELIGRO</t>
+        </is>
+      </c>
+      <c r="D294" t="n">
+        <v>106</v>
+      </c>
+      <c r="E294" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="295">
+      <c r="A295" t="inlineStr">
+        <is>
+          <t>16:33:34</t>
+        </is>
+      </c>
+      <c r="B295" t="inlineStr">
+        <is>
+          <t>17:48</t>
+        </is>
+      </c>
+      <c r="C295" t="inlineStr">
+        <is>
+          <t>215_EL PELIGRO</t>
+        </is>
+      </c>
+      <c r="D295" t="n">
+        <v>75</v>
+      </c>
+      <c r="E295" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="296">
+      <c r="A296" t="inlineStr">
+        <is>
+          <t>16:33:34</t>
+        </is>
+      </c>
+      <c r="B296" t="inlineStr">
+        <is>
+          <t>17:51</t>
+        </is>
+      </c>
+      <c r="C296" t="inlineStr">
+        <is>
+          <t>16_P MOR-SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D296" t="n">
+        <v>78</v>
+      </c>
+      <c r="E296" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="297">
+      <c r="A297" t="inlineStr">
+        <is>
+          <t>16:01:44</t>
+        </is>
+      </c>
+      <c r="B297" t="inlineStr">
         <is>
           <t>17:59</t>
         </is>
       </c>
-      <c r="C289" t="inlineStr">
+      <c r="C297" t="inlineStr">
         <is>
           <t>17_ROMERO</t>
         </is>
       </c>
-      <c r="D289" t="n">
+      <c r="D297" t="n">
         <v>118</v>
       </c>
-      <c r="E289" t="inlineStr">
+      <c r="E297" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="298">
+      <c r="A298" t="inlineStr">
+        <is>
+          <t>16:33:34</t>
+        </is>
+      </c>
+      <c r="B298" t="inlineStr">
+        <is>
+          <t>17:59</t>
+        </is>
+      </c>
+      <c r="C298" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D298" t="n">
+        <v>86</v>
+      </c>
+      <c r="E298" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="299">
+      <c r="A299" t="inlineStr">
+        <is>
+          <t>16:33:34</t>
+        </is>
+      </c>
+      <c r="B299" t="inlineStr">
+        <is>
+          <t>18:00</t>
+        </is>
+      </c>
+      <c r="C299" t="inlineStr">
+        <is>
+          <t>17_ROMERO</t>
+        </is>
+      </c>
+      <c r="D299" t="n">
+        <v>87</v>
+      </c>
+      <c r="E299" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="300">
+      <c r="A300" t="inlineStr">
+        <is>
+          <t>16:33:34</t>
+        </is>
+      </c>
+      <c r="B300" t="inlineStr">
+        <is>
+          <t>18:11</t>
+        </is>
+      </c>
+      <c r="C300" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D300" t="n">
+        <v>98</v>
+      </c>
+      <c r="E300" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="301">
+      <c r="A301" t="inlineStr">
+        <is>
+          <t>16:33:34</t>
+        </is>
+      </c>
+      <c r="B301" t="inlineStr">
+        <is>
+          <t>18:23</t>
+        </is>
+      </c>
+      <c r="C301" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D301" t="n">
+        <v>110</v>
+      </c>
+      <c r="E301" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -7581,7 +7881,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E50"/>
+  <dimension ref="A1:E52"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -7594,14 +7894,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 16:01:44</t>
+          <t>Última actualización: 16:33:34</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 45</t>
+          <t>Total filas: 47</t>
         </is>
       </c>
     </row>
@@ -8710,21 +9010,21 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>16:01:44</t>
+          <t>16:33:34</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>17:47</t>
+          <t>17:00</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>215_EL PELIGRO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D49" t="n">
-        <v>106</v>
+        <v>27</v>
       </c>
       <c r="E49" t="inlineStr">
         <is>
@@ -8745,13 +9045,63 @@
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>215_EL PELIGRO</t>
         </is>
       </c>
       <c r="D50" t="n">
         <v>106</v>
       </c>
       <c r="E50" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>16:33:34</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>17:47</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D51" t="n">
+        <v>74</v>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>16:33:34</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>17:48</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>215_EL PELIGRO</t>
+        </is>
+      </c>
+      <c r="D52" t="n">
+        <v>75</v>
+      </c>
+      <c r="E52" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -8768,7 +9118,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E54"/>
+  <dimension ref="A1:E55"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -8781,14 +9131,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 16:01:44</t>
+          <t>Última actualización: 16:33:34</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 49</t>
+          <t>Total filas: 50</t>
         </is>
       </c>
     </row>
@@ -9972,7 +10322,7 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>14:59:00</t>
+          <t>16:33:34</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
@@ -9986,7 +10336,7 @@
         </is>
       </c>
       <c r="D52" t="n">
-        <v>104</v>
+        <v>10</v>
       </c>
       <c r="E52" t="inlineStr">
         <is>
@@ -9997,7 +10347,7 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>16:01:44</t>
+          <t>16:33:34</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
@@ -10011,7 +10361,7 @@
         </is>
       </c>
       <c r="D53" t="n">
-        <v>54</v>
+        <v>22</v>
       </c>
       <c r="E53" t="inlineStr">
         <is>
@@ -10039,6 +10389,31 @@
         <v>117</v>
       </c>
       <c r="E54" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>16:33:34</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>18:25</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D55" t="n">
+        <v>112</v>
+      </c>
+      <c r="E55" t="inlineStr">
         <is>
           <t>L6203</t>
         </is>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 1817
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-03-21.xlsx
+++ b/data/horarios-141-2026-03-21.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E301"/>
+  <dimension ref="A1:E313"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 16:33:34</t>
+          <t>Última actualización: 16:49:09</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 296</t>
+          <t>Total filas: 308</t>
         </is>
       </c>
     </row>
@@ -533,7 +533,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D8" t="n">
@@ -558,7 +558,7 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D9" t="n">
@@ -758,7 +758,7 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D17" t="n">
@@ -783,7 +783,7 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D18" t="n">
@@ -1558,7 +1558,7 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D49" t="n">
@@ -1583,7 +1583,7 @@
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D50" t="n">
@@ -1873,7 +1873,7 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>08:14:14</t>
+          <t>06:59:30</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
@@ -1883,11 +1883,11 @@
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D62" t="n">
-        <v>0</v>
+        <v>75</v>
       </c>
       <c r="E62" t="inlineStr">
         <is>
@@ -1923,7 +1923,7 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>06:59:30</t>
+          <t>08:14:14</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
@@ -1933,11 +1933,11 @@
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D64" t="n">
-        <v>75</v>
+        <v>0</v>
       </c>
       <c r="E64" t="inlineStr">
         <is>
@@ -1973,7 +1973,7 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>07:51:37</t>
+          <t>07:27:35</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
@@ -1983,11 +1983,11 @@
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D66" t="n">
-        <v>28</v>
+        <v>52</v>
       </c>
       <c r="E66" t="inlineStr">
         <is>
@@ -2023,7 +2023,7 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>07:27:35</t>
+          <t>07:51:37</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
@@ -2033,11 +2033,11 @@
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D68" t="n">
-        <v>52</v>
+        <v>28</v>
       </c>
       <c r="E68" t="inlineStr">
         <is>
@@ -2698,7 +2698,7 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>08:14:14</t>
+          <t>08:50:55</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
@@ -2708,11 +2708,11 @@
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>215_EL PELIGRO</t>
         </is>
       </c>
       <c r="D95" t="n">
-        <v>64</v>
+        <v>28</v>
       </c>
       <c r="E95" t="inlineStr">
         <is>
@@ -2748,7 +2748,7 @@
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>08:50:55</t>
+          <t>08:14:14</t>
         </is>
       </c>
       <c r="B97" t="inlineStr">
@@ -2758,11 +2758,11 @@
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>215_EL PELIGRO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D97" t="n">
-        <v>28</v>
+        <v>64</v>
       </c>
       <c r="E97" t="inlineStr">
         <is>
@@ -3173,7 +3173,7 @@
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>08:50:55</t>
+          <t>09:23:24</t>
         </is>
       </c>
       <c r="B114" t="inlineStr">
@@ -3183,11 +3183,11 @@
       </c>
       <c r="C114" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D114" t="n">
-        <v>73</v>
+        <v>40</v>
       </c>
       <c r="E114" t="inlineStr">
         <is>
@@ -3198,7 +3198,7 @@
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>09:23:24</t>
+          <t>08:50:55</t>
         </is>
       </c>
       <c r="B115" t="inlineStr">
@@ -3208,11 +3208,11 @@
       </c>
       <c r="C115" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D115" t="n">
-        <v>40</v>
+        <v>73</v>
       </c>
       <c r="E115" t="inlineStr">
         <is>
@@ -3598,7 +3598,7 @@
     <row r="131">
       <c r="A131" t="inlineStr">
         <is>
-          <t>10:14:52</t>
+          <t>09:23:24</t>
         </is>
       </c>
       <c r="B131" t="inlineStr">
@@ -3608,11 +3608,11 @@
       </c>
       <c r="C131" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D131" t="n">
-        <v>29</v>
+        <v>80</v>
       </c>
       <c r="E131" t="inlineStr">
         <is>
@@ -3623,7 +3623,7 @@
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t>09:23:24</t>
+          <t>10:14:52</t>
         </is>
       </c>
       <c r="B132" t="inlineStr">
@@ -3633,11 +3633,11 @@
       </c>
       <c r="C132" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D132" t="n">
-        <v>80</v>
+        <v>29</v>
       </c>
       <c r="E132" t="inlineStr">
         <is>
@@ -3873,7 +3873,7 @@
     <row r="142">
       <c r="A142" t="inlineStr">
         <is>
-          <t>10:14:52</t>
+          <t>10:52:37</t>
         </is>
       </c>
       <c r="B142" t="inlineStr">
@@ -3883,11 +3883,11 @@
       </c>
       <c r="C142" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D142" t="n">
-        <v>49</v>
+        <v>11</v>
       </c>
       <c r="E142" t="inlineStr">
         <is>
@@ -3898,7 +3898,7 @@
     <row r="143">
       <c r="A143" t="inlineStr">
         <is>
-          <t>10:52:37</t>
+          <t>10:14:52</t>
         </is>
       </c>
       <c r="B143" t="inlineStr">
@@ -3908,11 +3908,11 @@
       </c>
       <c r="C143" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D143" t="n">
-        <v>11</v>
+        <v>49</v>
       </c>
       <c r="E143" t="inlineStr">
         <is>
@@ -4123,7 +4123,7 @@
     <row r="152">
       <c r="A152" t="inlineStr">
         <is>
-          <t>11:16:36</t>
+          <t>10:14:52</t>
         </is>
       </c>
       <c r="B152" t="inlineStr">
@@ -4133,11 +4133,11 @@
       </c>
       <c r="C152" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D152" t="n">
-        <v>16</v>
+        <v>78</v>
       </c>
       <c r="E152" t="inlineStr">
         <is>
@@ -4148,7 +4148,7 @@
     <row r="153">
       <c r="A153" t="inlineStr">
         <is>
-          <t>10:14:52</t>
+          <t>11:16:36</t>
         </is>
       </c>
       <c r="B153" t="inlineStr">
@@ -4158,11 +4158,11 @@
       </c>
       <c r="C153" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D153" t="n">
-        <v>78</v>
+        <v>16</v>
       </c>
       <c r="E153" t="inlineStr">
         <is>
@@ -4183,7 +4183,7 @@
       </c>
       <c r="C154" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D154" t="n">
@@ -4208,7 +4208,7 @@
       </c>
       <c r="C155" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D155" t="n">
@@ -4683,7 +4683,7 @@
       </c>
       <c r="C174" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D174" t="n">
@@ -4708,7 +4708,7 @@
       </c>
       <c r="C175" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D175" t="n">
@@ -5008,7 +5008,7 @@
       </c>
       <c r="C187" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D187" t="n">
@@ -5023,7 +5023,7 @@
     <row r="188">
       <c r="A188" t="inlineStr">
         <is>
-          <t>12:28:38</t>
+          <t>13:00:14</t>
         </is>
       </c>
       <c r="B188" t="inlineStr">
@@ -5033,11 +5033,11 @@
       </c>
       <c r="C188" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D188" t="n">
-        <v>35</v>
+        <v>3</v>
       </c>
       <c r="E188" t="inlineStr">
         <is>
@@ -5048,7 +5048,7 @@
     <row r="189">
       <c r="A189" t="inlineStr">
         <is>
-          <t>13:00:14</t>
+          <t>12:28:38</t>
         </is>
       </c>
       <c r="B189" t="inlineStr">
@@ -5058,11 +5058,11 @@
       </c>
       <c r="C189" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D189" t="n">
-        <v>3</v>
+        <v>35</v>
       </c>
       <c r="E189" t="inlineStr">
         <is>
@@ -5498,7 +5498,7 @@
     <row r="207">
       <c r="A207" t="inlineStr">
         <is>
-          <t>13:32:57</t>
+          <t>13:57:43</t>
         </is>
       </c>
       <c r="B207" t="inlineStr">
@@ -5508,11 +5508,11 @@
       </c>
       <c r="C207" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D207" t="n">
-        <v>27</v>
+        <v>2</v>
       </c>
       <c r="E207" t="inlineStr">
         <is>
@@ -5523,7 +5523,7 @@
     <row r="208">
       <c r="A208" t="inlineStr">
         <is>
-          <t>13:57:43</t>
+          <t>13:32:57</t>
         </is>
       </c>
       <c r="B208" t="inlineStr">
@@ -5533,11 +5533,11 @@
       </c>
       <c r="C208" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D208" t="n">
-        <v>2</v>
+        <v>27</v>
       </c>
       <c r="E208" t="inlineStr">
         <is>
@@ -5573,7 +5573,7 @@
     <row r="210">
       <c r="A210" t="inlineStr">
         <is>
-          <t>13:00:14</t>
+          <t>13:57:43</t>
         </is>
       </c>
       <c r="B210" t="inlineStr">
@@ -5583,11 +5583,11 @@
       </c>
       <c r="C210" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D210" t="n">
-        <v>63</v>
+        <v>6</v>
       </c>
       <c r="E210" t="inlineStr">
         <is>
@@ -5598,7 +5598,7 @@
     <row r="211">
       <c r="A211" t="inlineStr">
         <is>
-          <t>13:57:43</t>
+          <t>13:00:14</t>
         </is>
       </c>
       <c r="B211" t="inlineStr">
@@ -5608,11 +5608,11 @@
       </c>
       <c r="C211" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D211" t="n">
-        <v>6</v>
+        <v>63</v>
       </c>
       <c r="E211" t="inlineStr">
         <is>
@@ -6098,7 +6098,7 @@
     <row r="231">
       <c r="A231" t="inlineStr">
         <is>
-          <t>14:46:39</t>
+          <t>14:59:00</t>
         </is>
       </c>
       <c r="B231" t="inlineStr">
@@ -6108,11 +6108,11 @@
       </c>
       <c r="C231" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>81_EL PELIGRO</t>
         </is>
       </c>
       <c r="D231" t="n">
-        <v>13</v>
+        <v>0</v>
       </c>
       <c r="E231" t="inlineStr">
         <is>
@@ -6123,7 +6123,7 @@
     <row r="232">
       <c r="A232" t="inlineStr">
         <is>
-          <t>14:59:00</t>
+          <t>14:46:39</t>
         </is>
       </c>
       <c r="B232" t="inlineStr">
@@ -6133,11 +6133,11 @@
       </c>
       <c r="C232" t="inlineStr">
         <is>
-          <t>81_EL PELIGRO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D232" t="n">
-        <v>0</v>
+        <v>13</v>
       </c>
       <c r="E232" t="inlineStr">
         <is>
@@ -6698,7 +6698,7 @@
     <row r="255">
       <c r="A255" t="inlineStr">
         <is>
-          <t>14:46:39</t>
+          <t>15:34:45</t>
         </is>
       </c>
       <c r="B255" t="inlineStr">
@@ -6708,11 +6708,11 @@
       </c>
       <c r="C255" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D255" t="n">
-        <v>68</v>
+        <v>20</v>
       </c>
       <c r="E255" t="inlineStr">
         <is>
@@ -6723,7 +6723,7 @@
     <row r="256">
       <c r="A256" t="inlineStr">
         <is>
-          <t>15:34:45</t>
+          <t>14:46:39</t>
         </is>
       </c>
       <c r="B256" t="inlineStr">
@@ -6733,11 +6733,11 @@
       </c>
       <c r="C256" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D256" t="n">
-        <v>20</v>
+        <v>68</v>
       </c>
       <c r="E256" t="inlineStr">
         <is>
@@ -7123,7 +7123,7 @@
     <row r="272">
       <c r="A272" t="inlineStr">
         <is>
-          <t>14:59:00</t>
+          <t>15:34:45</t>
         </is>
       </c>
       <c r="B272" t="inlineStr">
@@ -7133,11 +7133,11 @@
       </c>
       <c r="C272" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D272" t="n">
-        <v>97</v>
+        <v>62</v>
       </c>
       <c r="E272" t="inlineStr">
         <is>
@@ -7148,7 +7148,7 @@
     <row r="273">
       <c r="A273" t="inlineStr">
         <is>
-          <t>15:34:45</t>
+          <t>14:59:00</t>
         </is>
       </c>
       <c r="B273" t="inlineStr">
@@ -7158,11 +7158,11 @@
       </c>
       <c r="C273" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D273" t="n">
-        <v>62</v>
+        <v>97</v>
       </c>
       <c r="E273" t="inlineStr">
         <is>
@@ -7248,12 +7248,12 @@
     <row r="277">
       <c r="A277" t="inlineStr">
         <is>
-          <t>16:33:34</t>
+          <t>16:49:09</t>
         </is>
       </c>
       <c r="B277" t="inlineStr">
         <is>
-          <t>16:51</t>
+          <t>16:49</t>
         </is>
       </c>
       <c r="C277" t="inlineStr">
@@ -7262,7 +7262,7 @@
         </is>
       </c>
       <c r="D277" t="n">
-        <v>18</v>
+        <v>0</v>
       </c>
       <c r="E277" t="inlineStr">
         <is>
@@ -7273,21 +7273,21 @@
     <row r="278">
       <c r="A278" t="inlineStr">
         <is>
-          <t>16:33:34</t>
+          <t>16:49:09</t>
         </is>
       </c>
       <c r="B278" t="inlineStr">
         <is>
-          <t>16:59</t>
+          <t>16:50</t>
         </is>
       </c>
       <c r="C278" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D278" t="n">
-        <v>26</v>
+        <v>1</v>
       </c>
       <c r="E278" t="inlineStr">
         <is>
@@ -7298,21 +7298,21 @@
     <row r="279">
       <c r="A279" t="inlineStr">
         <is>
-          <t>16:01:44</t>
+          <t>16:49:09</t>
         </is>
       </c>
       <c r="B279" t="inlineStr">
         <is>
-          <t>16:59</t>
+          <t>16:51</t>
         </is>
       </c>
       <c r="C279" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D279" t="n">
-        <v>58</v>
+        <v>2</v>
       </c>
       <c r="E279" t="inlineStr">
         <is>
@@ -7323,12 +7323,12 @@
     <row r="280">
       <c r="A280" t="inlineStr">
         <is>
-          <t>16:33:34</t>
+          <t>16:01:44</t>
         </is>
       </c>
       <c r="B280" t="inlineStr">
         <is>
-          <t>17:00</t>
+          <t>16:59</t>
         </is>
       </c>
       <c r="C280" t="inlineStr">
@@ -7337,7 +7337,7 @@
         </is>
       </c>
       <c r="D280" t="n">
-        <v>27</v>
+        <v>58</v>
       </c>
       <c r="E280" t="inlineStr">
         <is>
@@ -7353,16 +7353,16 @@
       </c>
       <c r="B281" t="inlineStr">
         <is>
-          <t>17:03</t>
+          <t>16:59</t>
         </is>
       </c>
       <c r="C281" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D281" t="n">
-        <v>30</v>
+        <v>26</v>
       </c>
       <c r="E281" t="inlineStr">
         <is>
@@ -7373,21 +7373,21 @@
     <row r="282">
       <c r="A282" t="inlineStr">
         <is>
-          <t>16:01:44</t>
+          <t>16:49:09</t>
         </is>
       </c>
       <c r="B282" t="inlineStr">
         <is>
-          <t>17:11</t>
+          <t>17:00</t>
         </is>
       </c>
       <c r="C282" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D282" t="n">
-        <v>70</v>
+        <v>11</v>
       </c>
       <c r="E282" t="inlineStr">
         <is>
@@ -7398,21 +7398,21 @@
     <row r="283">
       <c r="A283" t="inlineStr">
         <is>
-          <t>16:33:34</t>
+          <t>16:49:09</t>
         </is>
       </c>
       <c r="B283" t="inlineStr">
         <is>
-          <t>17:12</t>
+          <t>17:00</t>
         </is>
       </c>
       <c r="C283" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D283" t="n">
-        <v>39</v>
+        <v>11</v>
       </c>
       <c r="E283" t="inlineStr">
         <is>
@@ -7423,21 +7423,21 @@
     <row r="284">
       <c r="A284" t="inlineStr">
         <is>
-          <t>15:34:45</t>
+          <t>16:49:09</t>
         </is>
       </c>
       <c r="B284" t="inlineStr">
         <is>
-          <t>17:19</t>
+          <t>17:03</t>
         </is>
       </c>
       <c r="C284" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D284" t="n">
-        <v>105</v>
+        <v>14</v>
       </c>
       <c r="E284" t="inlineStr">
         <is>
@@ -7448,21 +7448,21 @@
     <row r="285">
       <c r="A285" t="inlineStr">
         <is>
-          <t>16:33:34</t>
+          <t>16:01:44</t>
         </is>
       </c>
       <c r="B285" t="inlineStr">
         <is>
-          <t>17:21</t>
+          <t>17:11</t>
         </is>
       </c>
       <c r="C285" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D285" t="n">
-        <v>48</v>
+        <v>70</v>
       </c>
       <c r="E285" t="inlineStr">
         <is>
@@ -7473,21 +7473,21 @@
     <row r="286">
       <c r="A286" t="inlineStr">
         <is>
-          <t>16:33:34</t>
+          <t>16:49:09</t>
         </is>
       </c>
       <c r="B286" t="inlineStr">
         <is>
-          <t>17:23</t>
+          <t>17:12</t>
         </is>
       </c>
       <c r="C286" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D286" t="n">
-        <v>50</v>
+        <v>23</v>
       </c>
       <c r="E286" t="inlineStr">
         <is>
@@ -7498,21 +7498,21 @@
     <row r="287">
       <c r="A287" t="inlineStr">
         <is>
-          <t>16:33:34</t>
+          <t>15:34:45</t>
         </is>
       </c>
       <c r="B287" t="inlineStr">
         <is>
-          <t>17:24</t>
+          <t>17:19</t>
         </is>
       </c>
       <c r="C287" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D287" t="n">
-        <v>51</v>
+        <v>105</v>
       </c>
       <c r="E287" t="inlineStr">
         <is>
@@ -7523,21 +7523,21 @@
     <row r="288">
       <c r="A288" t="inlineStr">
         <is>
-          <t>16:33:34</t>
+          <t>16:49:09</t>
         </is>
       </c>
       <c r="B288" t="inlineStr">
         <is>
-          <t>17:35</t>
+          <t>17:21</t>
         </is>
       </c>
       <c r="C288" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D288" t="n">
-        <v>62</v>
+        <v>32</v>
       </c>
       <c r="E288" t="inlineStr">
         <is>
@@ -7553,16 +7553,16 @@
       </c>
       <c r="B289" t="inlineStr">
         <is>
-          <t>17:35</t>
+          <t>17:23</t>
         </is>
       </c>
       <c r="C289" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D289" t="n">
-        <v>62</v>
+        <v>50</v>
       </c>
       <c r="E289" t="inlineStr">
         <is>
@@ -7573,21 +7573,21 @@
     <row r="290">
       <c r="A290" t="inlineStr">
         <is>
-          <t>16:33:34</t>
+          <t>16:49:09</t>
         </is>
       </c>
       <c r="B290" t="inlineStr">
         <is>
-          <t>17:35</t>
+          <t>17:24</t>
         </is>
       </c>
       <c r="C290" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D290" t="n">
-        <v>62</v>
+        <v>35</v>
       </c>
       <c r="E290" t="inlineStr">
         <is>
@@ -7598,21 +7598,21 @@
     <row r="291">
       <c r="A291" t="inlineStr">
         <is>
-          <t>16:01:44</t>
+          <t>16:33:34</t>
         </is>
       </c>
       <c r="B291" t="inlineStr">
         <is>
-          <t>17:38</t>
+          <t>17:24</t>
         </is>
       </c>
       <c r="C291" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D291" t="n">
-        <v>97</v>
+        <v>51</v>
       </c>
       <c r="E291" t="inlineStr">
         <is>
@@ -7623,21 +7623,21 @@
     <row r="292">
       <c r="A292" t="inlineStr">
         <is>
-          <t>16:33:34</t>
+          <t>16:49:09</t>
         </is>
       </c>
       <c r="B292" t="inlineStr">
         <is>
-          <t>17:41</t>
+          <t>17:33</t>
         </is>
       </c>
       <c r="C292" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D292" t="n">
-        <v>68</v>
+        <v>44</v>
       </c>
       <c r="E292" t="inlineStr">
         <is>
@@ -7648,21 +7648,21 @@
     <row r="293">
       <c r="A293" t="inlineStr">
         <is>
-          <t>16:33:34</t>
+          <t>16:49:09</t>
         </is>
       </c>
       <c r="B293" t="inlineStr">
         <is>
-          <t>17:47</t>
+          <t>17:35</t>
         </is>
       </c>
       <c r="C293" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D293" t="n">
-        <v>74</v>
+        <v>46</v>
       </c>
       <c r="E293" t="inlineStr">
         <is>
@@ -7673,21 +7673,21 @@
     <row r="294">
       <c r="A294" t="inlineStr">
         <is>
-          <t>16:01:44</t>
+          <t>16:49:09</t>
         </is>
       </c>
       <c r="B294" t="inlineStr">
         <is>
-          <t>17:47</t>
+          <t>17:35</t>
         </is>
       </c>
       <c r="C294" t="inlineStr">
         <is>
-          <t>215_EL PELIGRO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D294" t="n">
-        <v>106</v>
+        <v>46</v>
       </c>
       <c r="E294" t="inlineStr">
         <is>
@@ -7703,16 +7703,16 @@
       </c>
       <c r="B295" t="inlineStr">
         <is>
-          <t>17:48</t>
+          <t>17:35</t>
         </is>
       </c>
       <c r="C295" t="inlineStr">
         <is>
-          <t>215_EL PELIGRO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D295" t="n">
-        <v>75</v>
+        <v>62</v>
       </c>
       <c r="E295" t="inlineStr">
         <is>
@@ -7723,21 +7723,21 @@
     <row r="296">
       <c r="A296" t="inlineStr">
         <is>
-          <t>16:33:34</t>
+          <t>16:49:09</t>
         </is>
       </c>
       <c r="B296" t="inlineStr">
         <is>
-          <t>17:51</t>
+          <t>17:37</t>
         </is>
       </c>
       <c r="C296" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D296" t="n">
-        <v>78</v>
+        <v>48</v>
       </c>
       <c r="E296" t="inlineStr">
         <is>
@@ -7753,16 +7753,16 @@
       </c>
       <c r="B297" t="inlineStr">
         <is>
-          <t>17:59</t>
+          <t>17:38</t>
         </is>
       </c>
       <c r="C297" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D297" t="n">
-        <v>118</v>
+        <v>97</v>
       </c>
       <c r="E297" t="inlineStr">
         <is>
@@ -7778,16 +7778,16 @@
       </c>
       <c r="B298" t="inlineStr">
         <is>
-          <t>17:59</t>
+          <t>17:41</t>
         </is>
       </c>
       <c r="C298" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D298" t="n">
-        <v>86</v>
+        <v>68</v>
       </c>
       <c r="E298" t="inlineStr">
         <is>
@@ -7798,21 +7798,21 @@
     <row r="299">
       <c r="A299" t="inlineStr">
         <is>
-          <t>16:33:34</t>
+          <t>16:01:44</t>
         </is>
       </c>
       <c r="B299" t="inlineStr">
         <is>
-          <t>18:00</t>
+          <t>17:47</t>
         </is>
       </c>
       <c r="C299" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>215_EL PELIGRO</t>
         </is>
       </c>
       <c r="D299" t="n">
-        <v>87</v>
+        <v>106</v>
       </c>
       <c r="E299" t="inlineStr">
         <is>
@@ -7828,16 +7828,16 @@
       </c>
       <c r="B300" t="inlineStr">
         <is>
-          <t>18:11</t>
+          <t>17:47</t>
         </is>
       </c>
       <c r="C300" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D300" t="n">
-        <v>98</v>
+        <v>74</v>
       </c>
       <c r="E300" t="inlineStr">
         <is>
@@ -7848,23 +7848,323 @@
     <row r="301">
       <c r="A301" t="inlineStr">
         <is>
+          <t>16:49:09</t>
+        </is>
+      </c>
+      <c r="B301" t="inlineStr">
+        <is>
+          <t>17:48</t>
+        </is>
+      </c>
+      <c r="C301" t="inlineStr">
+        <is>
+          <t>215_EL PELIGRO</t>
+        </is>
+      </c>
+      <c r="D301" t="n">
+        <v>59</v>
+      </c>
+      <c r="E301" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="302">
+      <c r="A302" t="inlineStr">
+        <is>
+          <t>16:49:09</t>
+        </is>
+      </c>
+      <c r="B302" t="inlineStr">
+        <is>
+          <t>17:48</t>
+        </is>
+      </c>
+      <c r="C302" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D302" t="n">
+        <v>59</v>
+      </c>
+      <c r="E302" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="303">
+      <c r="A303" t="inlineStr">
+        <is>
           <t>16:33:34</t>
         </is>
       </c>
-      <c r="B301" t="inlineStr">
+      <c r="B303" t="inlineStr">
+        <is>
+          <t>17:51</t>
+        </is>
+      </c>
+      <c r="C303" t="inlineStr">
+        <is>
+          <t>16_P MOR-SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D303" t="n">
+        <v>78</v>
+      </c>
+      <c r="E303" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="304">
+      <c r="A304" t="inlineStr">
+        <is>
+          <t>16:49:09</t>
+        </is>
+      </c>
+      <c r="B304" t="inlineStr">
+        <is>
+          <t>17:59</t>
+        </is>
+      </c>
+      <c r="C304" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D304" t="n">
+        <v>70</v>
+      </c>
+      <c r="E304" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="305">
+      <c r="A305" t="inlineStr">
+        <is>
+          <t>16:01:44</t>
+        </is>
+      </c>
+      <c r="B305" t="inlineStr">
+        <is>
+          <t>17:59</t>
+        </is>
+      </c>
+      <c r="C305" t="inlineStr">
+        <is>
+          <t>17_ROMERO</t>
+        </is>
+      </c>
+      <c r="D305" t="n">
+        <v>118</v>
+      </c>
+      <c r="E305" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="306">
+      <c r="A306" t="inlineStr">
+        <is>
+          <t>16:49:09</t>
+        </is>
+      </c>
+      <c r="B306" t="inlineStr">
+        <is>
+          <t>18:00</t>
+        </is>
+      </c>
+      <c r="C306" t="inlineStr">
+        <is>
+          <t>17_ROMERO</t>
+        </is>
+      </c>
+      <c r="D306" t="n">
+        <v>71</v>
+      </c>
+      <c r="E306" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="307">
+      <c r="A307" t="inlineStr">
+        <is>
+          <t>16:49:09</t>
+        </is>
+      </c>
+      <c r="B307" t="inlineStr">
+        <is>
+          <t>18:01</t>
+        </is>
+      </c>
+      <c r="C307" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D307" t="n">
+        <v>72</v>
+      </c>
+      <c r="E307" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="308">
+      <c r="A308" t="inlineStr">
+        <is>
+          <t>16:33:34</t>
+        </is>
+      </c>
+      <c r="B308" t="inlineStr">
+        <is>
+          <t>18:11</t>
+        </is>
+      </c>
+      <c r="C308" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D308" t="n">
+        <v>98</v>
+      </c>
+      <c r="E308" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="309">
+      <c r="A309" t="inlineStr">
+        <is>
+          <t>16:49:09</t>
+        </is>
+      </c>
+      <c r="B309" t="inlineStr">
+        <is>
+          <t>18:12</t>
+        </is>
+      </c>
+      <c r="C309" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D309" t="n">
+        <v>83</v>
+      </c>
+      <c r="E309" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="310">
+      <c r="A310" t="inlineStr">
+        <is>
+          <t>16:49:09</t>
+        </is>
+      </c>
+      <c r="B310" t="inlineStr">
+        <is>
+          <t>18:12</t>
+        </is>
+      </c>
+      <c r="C310" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D310" t="n">
+        <v>83</v>
+      </c>
+      <c r="E310" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="311">
+      <c r="A311" t="inlineStr">
+        <is>
+          <t>16:49:09</t>
+        </is>
+      </c>
+      <c r="B311" t="inlineStr">
         <is>
           <t>18:23</t>
         </is>
       </c>
-      <c r="C301" t="inlineStr">
+      <c r="C311" t="inlineStr">
         <is>
           <t>10_OLMOS</t>
         </is>
       </c>
-      <c r="D301" t="n">
+      <c r="D311" t="n">
+        <v>94</v>
+      </c>
+      <c r="E311" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="312">
+      <c r="A312" t="inlineStr">
+        <is>
+          <t>16:49:09</t>
+        </is>
+      </c>
+      <c r="B312" t="inlineStr">
+        <is>
+          <t>18:35</t>
+        </is>
+      </c>
+      <c r="C312" t="inlineStr">
+        <is>
+          <t>17X38_ROMERO</t>
+        </is>
+      </c>
+      <c r="D312" t="n">
+        <v>106</v>
+      </c>
+      <c r="E312" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="313">
+      <c r="A313" t="inlineStr">
+        <is>
+          <t>16:49:09</t>
+        </is>
+      </c>
+      <c r="B313" t="inlineStr">
+        <is>
+          <t>18:39</t>
+        </is>
+      </c>
+      <c r="C313" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D313" t="n">
         <v>110</v>
       </c>
-      <c r="E301" t="inlineStr">
+      <c r="E313" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -7881,7 +8181,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E52"/>
+  <dimension ref="A1:E53"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -7894,14 +8194,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 16:33:34</t>
+          <t>Última actualización: 16:49:09</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 47</t>
+          <t>Total filas: 48</t>
         </is>
       </c>
     </row>
@@ -9010,7 +9310,7 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>16:33:34</t>
+          <t>16:49:09</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
@@ -9024,7 +9324,7 @@
         </is>
       </c>
       <c r="D49" t="n">
-        <v>27</v>
+        <v>11</v>
       </c>
       <c r="E49" t="inlineStr">
         <is>
@@ -9085,7 +9385,7 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>16:33:34</t>
+          <t>16:49:09</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
@@ -9099,9 +9399,34 @@
         </is>
       </c>
       <c r="D52" t="n">
-        <v>75</v>
+        <v>59</v>
       </c>
       <c r="E52" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>16:49:09</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>17:48</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D53" t="n">
+        <v>59</v>
+      </c>
+      <c r="E53" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -9118,7 +9443,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E55"/>
+  <dimension ref="A1:E56"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -9131,14 +9456,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 16:33:34</t>
+          <t>Última actualización: 16:49:09</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 50</t>
+          <t>Total filas: 51</t>
         </is>
       </c>
     </row>
@@ -10372,7 +10697,7 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>14:59:00</t>
+          <t>16:49:09</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
@@ -10386,7 +10711,7 @@
         </is>
       </c>
       <c r="D54" t="n">
-        <v>117</v>
+        <v>7</v>
       </c>
       <c r="E54" t="inlineStr">
         <is>
@@ -10414,6 +10739,31 @@
         <v>112</v>
       </c>
       <c r="E55" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>16:49:09</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>18:26</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D56" t="n">
+        <v>97</v>
+      </c>
+      <c r="E56" t="inlineStr">
         <is>
           <t>L6203</t>
         </is>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 1818
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-03-21.xlsx
+++ b/data/horarios-141-2026-03-21.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E313"/>
+  <dimension ref="A1:E318"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 16:49:09</t>
+          <t>Última actualización: 16:57:49</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 308</t>
+          <t>Total filas: 313</t>
         </is>
       </c>
     </row>
@@ -1158,7 +1158,7 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D33" t="n">
@@ -1183,7 +1183,7 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D34" t="n">
@@ -1558,7 +1558,7 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D49" t="n">
@@ -1583,7 +1583,7 @@
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D50" t="n">
@@ -1908,7 +1908,7 @@
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D63" t="n">
@@ -1933,7 +1933,7 @@
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D64" t="n">
@@ -1973,7 +1973,7 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>07:27:35</t>
+          <t>07:51:37</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
@@ -1983,11 +1983,11 @@
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D66" t="n">
-        <v>52</v>
+        <v>28</v>
       </c>
       <c r="E66" t="inlineStr">
         <is>
@@ -2008,7 +2008,7 @@
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D67" t="n">
@@ -2023,7 +2023,7 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>07:51:37</t>
+          <t>07:27:35</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
@@ -2033,11 +2033,11 @@
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D68" t="n">
-        <v>28</v>
+        <v>52</v>
       </c>
       <c r="E68" t="inlineStr">
         <is>
@@ -2233,7 +2233,7 @@
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D76" t="n">
@@ -2258,7 +2258,7 @@
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D77" t="n">
@@ -2373,7 +2373,7 @@
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>07:27:35</t>
+          <t>08:50:55</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
@@ -2383,11 +2383,11 @@
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D82" t="n">
-        <v>84</v>
+        <v>1</v>
       </c>
       <c r="E82" t="inlineStr">
         <is>
@@ -2408,7 +2408,7 @@
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D83" t="n">
@@ -2423,7 +2423,7 @@
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>08:50:55</t>
+          <t>07:27:35</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
@@ -2433,11 +2433,11 @@
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D84" t="n">
-        <v>1</v>
+        <v>84</v>
       </c>
       <c r="E84" t="inlineStr">
         <is>
@@ -2698,7 +2698,7 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>08:50:55</t>
+          <t>08:14:14</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
@@ -2708,11 +2708,11 @@
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>215_EL PELIGRO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D95" t="n">
-        <v>28</v>
+        <v>64</v>
       </c>
       <c r="E95" t="inlineStr">
         <is>
@@ -2733,7 +2733,7 @@
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215_EL PELIGRO</t>
         </is>
       </c>
       <c r="D96" t="n">
@@ -2748,7 +2748,7 @@
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>08:14:14</t>
+          <t>08:50:55</t>
         </is>
       </c>
       <c r="B97" t="inlineStr">
@@ -2758,11 +2758,11 @@
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D97" t="n">
-        <v>64</v>
+        <v>28</v>
       </c>
       <c r="E97" t="inlineStr">
         <is>
@@ -2873,7 +2873,7 @@
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>08:36:09</t>
+          <t>07:51:37</t>
         </is>
       </c>
       <c r="B102" t="inlineStr">
@@ -2883,11 +2883,11 @@
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D102" t="n">
-        <v>53</v>
+        <v>98</v>
       </c>
       <c r="E102" t="inlineStr">
         <is>
@@ -2898,7 +2898,7 @@
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>07:51:37</t>
+          <t>08:36:09</t>
         </is>
       </c>
       <c r="B103" t="inlineStr">
@@ -2908,11 +2908,11 @@
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D103" t="n">
-        <v>98</v>
+        <v>53</v>
       </c>
       <c r="E103" t="inlineStr">
         <is>
@@ -2923,7 +2923,7 @@
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>09:23:24</t>
+          <t>08:14:14</t>
         </is>
       </c>
       <c r="B104" t="inlineStr">
@@ -2933,11 +2933,11 @@
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D104" t="n">
-        <v>10</v>
+        <v>79</v>
       </c>
       <c r="E104" t="inlineStr">
         <is>
@@ -2948,7 +2948,7 @@
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>08:14:14</t>
+          <t>09:23:24</t>
         </is>
       </c>
       <c r="B105" t="inlineStr">
@@ -2958,11 +2958,11 @@
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D105" t="n">
-        <v>79</v>
+        <v>10</v>
       </c>
       <c r="E105" t="inlineStr">
         <is>
@@ -3173,7 +3173,7 @@
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>09:23:24</t>
+          <t>08:50:55</t>
         </is>
       </c>
       <c r="B114" t="inlineStr">
@@ -3183,11 +3183,11 @@
       </c>
       <c r="C114" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D114" t="n">
-        <v>40</v>
+        <v>73</v>
       </c>
       <c r="E114" t="inlineStr">
         <is>
@@ -3198,7 +3198,7 @@
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>08:50:55</t>
+          <t>09:23:24</t>
         </is>
       </c>
       <c r="B115" t="inlineStr">
@@ -3208,11 +3208,11 @@
       </c>
       <c r="C115" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D115" t="n">
-        <v>73</v>
+        <v>40</v>
       </c>
       <c r="E115" t="inlineStr">
         <is>
@@ -3873,7 +3873,7 @@
     <row r="142">
       <c r="A142" t="inlineStr">
         <is>
-          <t>10:52:37</t>
+          <t>10:14:52</t>
         </is>
       </c>
       <c r="B142" t="inlineStr">
@@ -3883,11 +3883,11 @@
       </c>
       <c r="C142" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D142" t="n">
-        <v>11</v>
+        <v>49</v>
       </c>
       <c r="E142" t="inlineStr">
         <is>
@@ -3898,7 +3898,7 @@
     <row r="143">
       <c r="A143" t="inlineStr">
         <is>
-          <t>10:14:52</t>
+          <t>10:52:37</t>
         </is>
       </c>
       <c r="B143" t="inlineStr">
@@ -3908,11 +3908,11 @@
       </c>
       <c r="C143" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D143" t="n">
-        <v>49</v>
+        <v>11</v>
       </c>
       <c r="E143" t="inlineStr">
         <is>
@@ -4123,7 +4123,7 @@
     <row r="152">
       <c r="A152" t="inlineStr">
         <is>
-          <t>10:14:52</t>
+          <t>11:16:36</t>
         </is>
       </c>
       <c r="B152" t="inlineStr">
@@ -4133,11 +4133,11 @@
       </c>
       <c r="C152" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D152" t="n">
-        <v>78</v>
+        <v>16</v>
       </c>
       <c r="E152" t="inlineStr">
         <is>
@@ -4148,7 +4148,7 @@
     <row r="153">
       <c r="A153" t="inlineStr">
         <is>
-          <t>11:16:36</t>
+          <t>10:14:52</t>
         </is>
       </c>
       <c r="B153" t="inlineStr">
@@ -4158,11 +4158,11 @@
       </c>
       <c r="C153" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D153" t="n">
-        <v>16</v>
+        <v>78</v>
       </c>
       <c r="E153" t="inlineStr">
         <is>
@@ -4183,7 +4183,7 @@
       </c>
       <c r="C154" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D154" t="n">
@@ -4208,7 +4208,7 @@
       </c>
       <c r="C155" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D155" t="n">
@@ -4473,7 +4473,7 @@
     <row r="166">
       <c r="A166" t="inlineStr">
         <is>
-          <t>11:16:36</t>
+          <t>12:00:15</t>
         </is>
       </c>
       <c r="B166" t="inlineStr">
@@ -4483,11 +4483,11 @@
       </c>
       <c r="C166" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D166" t="n">
-        <v>48</v>
+        <v>4</v>
       </c>
       <c r="E166" t="inlineStr">
         <is>
@@ -4498,7 +4498,7 @@
     <row r="167">
       <c r="A167" t="inlineStr">
         <is>
-          <t>12:00:15</t>
+          <t>11:16:36</t>
         </is>
       </c>
       <c r="B167" t="inlineStr">
@@ -4508,11 +4508,11 @@
       </c>
       <c r="C167" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D167" t="n">
-        <v>4</v>
+        <v>48</v>
       </c>
       <c r="E167" t="inlineStr">
         <is>
@@ -4648,7 +4648,7 @@
     <row r="173">
       <c r="A173" t="inlineStr">
         <is>
-          <t>12:00:15</t>
+          <t>12:28:38</t>
         </is>
       </c>
       <c r="B173" t="inlineStr">
@@ -4658,11 +4658,11 @@
       </c>
       <c r="C173" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D173" t="n">
-        <v>33</v>
+        <v>5</v>
       </c>
       <c r="E173" t="inlineStr">
         <is>
@@ -4698,7 +4698,7 @@
     <row r="175">
       <c r="A175" t="inlineStr">
         <is>
-          <t>12:28:38</t>
+          <t>12:00:15</t>
         </is>
       </c>
       <c r="B175" t="inlineStr">
@@ -4708,11 +4708,11 @@
       </c>
       <c r="C175" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D175" t="n">
-        <v>5</v>
+        <v>33</v>
       </c>
       <c r="E175" t="inlineStr">
         <is>
@@ -4998,7 +4998,7 @@
     <row r="187">
       <c r="A187" t="inlineStr">
         <is>
-          <t>12:28:38</t>
+          <t>13:00:14</t>
         </is>
       </c>
       <c r="B187" t="inlineStr">
@@ -5008,11 +5008,11 @@
       </c>
       <c r="C187" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D187" t="n">
-        <v>35</v>
+        <v>3</v>
       </c>
       <c r="E187" t="inlineStr">
         <is>
@@ -5023,7 +5023,7 @@
     <row r="188">
       <c r="A188" t="inlineStr">
         <is>
-          <t>13:00:14</t>
+          <t>12:28:38</t>
         </is>
       </c>
       <c r="B188" t="inlineStr">
@@ -5033,11 +5033,11 @@
       </c>
       <c r="C188" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D188" t="n">
-        <v>3</v>
+        <v>35</v>
       </c>
       <c r="E188" t="inlineStr">
         <is>
@@ -5073,7 +5073,7 @@
     <row r="190">
       <c r="A190" t="inlineStr">
         <is>
-          <t>13:00:14</t>
+          <t>12:48:06</t>
         </is>
       </c>
       <c r="B190" t="inlineStr">
@@ -5083,11 +5083,11 @@
       </c>
       <c r="C190" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D190" t="n">
-        <v>4</v>
+        <v>16</v>
       </c>
       <c r="E190" t="inlineStr">
         <is>
@@ -5098,7 +5098,7 @@
     <row r="191">
       <c r="A191" t="inlineStr">
         <is>
-          <t>12:48:06</t>
+          <t>13:00:14</t>
         </is>
       </c>
       <c r="B191" t="inlineStr">
@@ -5108,11 +5108,11 @@
       </c>
       <c r="C191" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D191" t="n">
-        <v>16</v>
+        <v>4</v>
       </c>
       <c r="E191" t="inlineStr">
         <is>
@@ -5323,7 +5323,7 @@
     <row r="200">
       <c r="A200" t="inlineStr">
         <is>
-          <t>12:48:06</t>
+          <t>13:00:14</t>
         </is>
       </c>
       <c r="B200" t="inlineStr">
@@ -5333,11 +5333,11 @@
       </c>
       <c r="C200" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D200" t="n">
-        <v>50</v>
+        <v>38</v>
       </c>
       <c r="E200" t="inlineStr">
         <is>
@@ -5348,7 +5348,7 @@
     <row r="201">
       <c r="A201" t="inlineStr">
         <is>
-          <t>13:00:14</t>
+          <t>12:48:06</t>
         </is>
       </c>
       <c r="B201" t="inlineStr">
@@ -5358,11 +5358,11 @@
       </c>
       <c r="C201" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D201" t="n">
-        <v>38</v>
+        <v>50</v>
       </c>
       <c r="E201" t="inlineStr">
         <is>
@@ -5498,7 +5498,7 @@
     <row r="207">
       <c r="A207" t="inlineStr">
         <is>
-          <t>13:57:43</t>
+          <t>13:32:57</t>
         </is>
       </c>
       <c r="B207" t="inlineStr">
@@ -5508,11 +5508,11 @@
       </c>
       <c r="C207" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D207" t="n">
-        <v>2</v>
+        <v>27</v>
       </c>
       <c r="E207" t="inlineStr">
         <is>
@@ -5523,7 +5523,7 @@
     <row r="208">
       <c r="A208" t="inlineStr">
         <is>
-          <t>13:32:57</t>
+          <t>13:57:43</t>
         </is>
       </c>
       <c r="B208" t="inlineStr">
@@ -5533,11 +5533,11 @@
       </c>
       <c r="C208" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D208" t="n">
-        <v>27</v>
+        <v>2</v>
       </c>
       <c r="E208" t="inlineStr">
         <is>
@@ -5873,7 +5873,7 @@
     <row r="222">
       <c r="A222" t="inlineStr">
         <is>
-          <t>14:21:42</t>
+          <t>13:00:14</t>
         </is>
       </c>
       <c r="B222" t="inlineStr">
@@ -5883,11 +5883,11 @@
       </c>
       <c r="C222" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D222" t="n">
-        <v>12</v>
+        <v>93</v>
       </c>
       <c r="E222" t="inlineStr">
         <is>
@@ -5898,7 +5898,7 @@
     <row r="223">
       <c r="A223" t="inlineStr">
         <is>
-          <t>13:00:14</t>
+          <t>14:21:42</t>
         </is>
       </c>
       <c r="B223" t="inlineStr">
@@ -5908,11 +5908,11 @@
       </c>
       <c r="C223" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D223" t="n">
-        <v>93</v>
+        <v>12</v>
       </c>
       <c r="E223" t="inlineStr">
         <is>
@@ -6098,7 +6098,7 @@
     <row r="231">
       <c r="A231" t="inlineStr">
         <is>
-          <t>14:59:00</t>
+          <t>14:46:39</t>
         </is>
       </c>
       <c r="B231" t="inlineStr">
@@ -6108,11 +6108,11 @@
       </c>
       <c r="C231" t="inlineStr">
         <is>
-          <t>81_EL PELIGRO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D231" t="n">
-        <v>0</v>
+        <v>13</v>
       </c>
       <c r="E231" t="inlineStr">
         <is>
@@ -6123,7 +6123,7 @@
     <row r="232">
       <c r="A232" t="inlineStr">
         <is>
-          <t>14:46:39</t>
+          <t>14:59:00</t>
         </is>
       </c>
       <c r="B232" t="inlineStr">
@@ -6133,11 +6133,11 @@
       </c>
       <c r="C232" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>81_EL PELIGRO</t>
         </is>
       </c>
       <c r="D232" t="n">
-        <v>13</v>
+        <v>0</v>
       </c>
       <c r="E232" t="inlineStr">
         <is>
@@ -7033,7 +7033,7 @@
       </c>
       <c r="C268" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D268" t="n">
@@ -7058,7 +7058,7 @@
       </c>
       <c r="C269" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D269" t="n">
@@ -7073,7 +7073,7 @@
     <row r="270">
       <c r="A270" t="inlineStr">
         <is>
-          <t>16:33:34</t>
+          <t>16:01:44</t>
         </is>
       </c>
       <c r="B270" t="inlineStr">
@@ -7083,11 +7083,11 @@
       </c>
       <c r="C270" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D270" t="n">
-        <v>2</v>
+        <v>34</v>
       </c>
       <c r="E270" t="inlineStr">
         <is>
@@ -7098,7 +7098,7 @@
     <row r="271">
       <c r="A271" t="inlineStr">
         <is>
-          <t>16:01:44</t>
+          <t>16:33:34</t>
         </is>
       </c>
       <c r="B271" t="inlineStr">
@@ -7108,11 +7108,11 @@
       </c>
       <c r="C271" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D271" t="n">
-        <v>34</v>
+        <v>2</v>
       </c>
       <c r="E271" t="inlineStr">
         <is>
@@ -7123,7 +7123,7 @@
     <row r="272">
       <c r="A272" t="inlineStr">
         <is>
-          <t>15:34:45</t>
+          <t>14:59:00</t>
         </is>
       </c>
       <c r="B272" t="inlineStr">
@@ -7133,11 +7133,11 @@
       </c>
       <c r="C272" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D272" t="n">
-        <v>62</v>
+        <v>97</v>
       </c>
       <c r="E272" t="inlineStr">
         <is>
@@ -7148,7 +7148,7 @@
     <row r="273">
       <c r="A273" t="inlineStr">
         <is>
-          <t>14:59:00</t>
+          <t>15:34:45</t>
         </is>
       </c>
       <c r="B273" t="inlineStr">
@@ -7158,11 +7158,11 @@
       </c>
       <c r="C273" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D273" t="n">
-        <v>97</v>
+        <v>62</v>
       </c>
       <c r="E273" t="inlineStr">
         <is>
@@ -7323,7 +7323,7 @@
     <row r="280">
       <c r="A280" t="inlineStr">
         <is>
-          <t>16:01:44</t>
+          <t>16:57:49</t>
         </is>
       </c>
       <c r="B280" t="inlineStr">
@@ -7333,11 +7333,11 @@
       </c>
       <c r="C280" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D280" t="n">
-        <v>58</v>
+        <v>2</v>
       </c>
       <c r="E280" t="inlineStr">
         <is>
@@ -7348,7 +7348,7 @@
     <row r="281">
       <c r="A281" t="inlineStr">
         <is>
-          <t>16:33:34</t>
+          <t>16:57:49</t>
         </is>
       </c>
       <c r="B281" t="inlineStr">
@@ -7358,11 +7358,11 @@
       </c>
       <c r="C281" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D281" t="n">
-        <v>26</v>
+        <v>2</v>
       </c>
       <c r="E281" t="inlineStr">
         <is>
@@ -7383,7 +7383,7 @@
       </c>
       <c r="C282" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D282" t="n">
@@ -7408,7 +7408,7 @@
       </c>
       <c r="C283" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D283" t="n">
@@ -7423,7 +7423,7 @@
     <row r="284">
       <c r="A284" t="inlineStr">
         <is>
-          <t>16:49:09</t>
+          <t>16:57:49</t>
         </is>
       </c>
       <c r="B284" t="inlineStr">
@@ -7437,7 +7437,7 @@
         </is>
       </c>
       <c r="D284" t="n">
-        <v>14</v>
+        <v>6</v>
       </c>
       <c r="E284" t="inlineStr">
         <is>
@@ -7448,7 +7448,7 @@
     <row r="285">
       <c r="A285" t="inlineStr">
         <is>
-          <t>16:01:44</t>
+          <t>16:57:49</t>
         </is>
       </c>
       <c r="B285" t="inlineStr">
@@ -7462,7 +7462,7 @@
         </is>
       </c>
       <c r="D285" t="n">
-        <v>70</v>
+        <v>14</v>
       </c>
       <c r="E285" t="inlineStr">
         <is>
@@ -7523,7 +7523,7 @@
     <row r="288">
       <c r="A288" t="inlineStr">
         <is>
-          <t>16:49:09</t>
+          <t>16:57:49</t>
         </is>
       </c>
       <c r="B288" t="inlineStr">
@@ -7537,7 +7537,7 @@
         </is>
       </c>
       <c r="D288" t="n">
-        <v>32</v>
+        <v>24</v>
       </c>
       <c r="E288" t="inlineStr">
         <is>
@@ -7548,7 +7548,7 @@
     <row r="289">
       <c r="A289" t="inlineStr">
         <is>
-          <t>16:33:34</t>
+          <t>16:57:49</t>
         </is>
       </c>
       <c r="B289" t="inlineStr">
@@ -7562,7 +7562,7 @@
         </is>
       </c>
       <c r="D289" t="n">
-        <v>50</v>
+        <v>26</v>
       </c>
       <c r="E289" t="inlineStr">
         <is>
@@ -7623,7 +7623,7 @@
     <row r="292">
       <c r="A292" t="inlineStr">
         <is>
-          <t>16:49:09</t>
+          <t>16:57:49</t>
         </is>
       </c>
       <c r="B292" t="inlineStr">
@@ -7637,7 +7637,7 @@
         </is>
       </c>
       <c r="D292" t="n">
-        <v>44</v>
+        <v>36</v>
       </c>
       <c r="E292" t="inlineStr">
         <is>
@@ -7648,7 +7648,7 @@
     <row r="293">
       <c r="A293" t="inlineStr">
         <is>
-          <t>16:49:09</t>
+          <t>16:57:49</t>
         </is>
       </c>
       <c r="B293" t="inlineStr">
@@ -7658,11 +7658,11 @@
       </c>
       <c r="C293" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D293" t="n">
-        <v>46</v>
+        <v>38</v>
       </c>
       <c r="E293" t="inlineStr">
         <is>
@@ -7673,7 +7673,7 @@
     <row r="294">
       <c r="A294" t="inlineStr">
         <is>
-          <t>16:49:09</t>
+          <t>16:57:49</t>
         </is>
       </c>
       <c r="B294" t="inlineStr">
@@ -7683,11 +7683,11 @@
       </c>
       <c r="C294" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D294" t="n">
-        <v>46</v>
+        <v>38</v>
       </c>
       <c r="E294" t="inlineStr">
         <is>
@@ -7723,12 +7723,12 @@
     <row r="296">
       <c r="A296" t="inlineStr">
         <is>
-          <t>16:49:09</t>
+          <t>16:57:49</t>
         </is>
       </c>
       <c r="B296" t="inlineStr">
         <is>
-          <t>17:37</t>
+          <t>17:36</t>
         </is>
       </c>
       <c r="C296" t="inlineStr">
@@ -7737,7 +7737,7 @@
         </is>
       </c>
       <c r="D296" t="n">
-        <v>48</v>
+        <v>39</v>
       </c>
       <c r="E296" t="inlineStr">
         <is>
@@ -7748,12 +7748,12 @@
     <row r="297">
       <c r="A297" t="inlineStr">
         <is>
-          <t>16:01:44</t>
+          <t>16:49:09</t>
         </is>
       </c>
       <c r="B297" t="inlineStr">
         <is>
-          <t>17:38</t>
+          <t>17:37</t>
         </is>
       </c>
       <c r="C297" t="inlineStr">
@@ -7762,7 +7762,7 @@
         </is>
       </c>
       <c r="D297" t="n">
-        <v>97</v>
+        <v>48</v>
       </c>
       <c r="E297" t="inlineStr">
         <is>
@@ -7773,21 +7773,21 @@
     <row r="298">
       <c r="A298" t="inlineStr">
         <is>
-          <t>16:33:34</t>
+          <t>16:01:44</t>
         </is>
       </c>
       <c r="B298" t="inlineStr">
         <is>
-          <t>17:41</t>
+          <t>17:38</t>
         </is>
       </c>
       <c r="C298" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D298" t="n">
-        <v>68</v>
+        <v>97</v>
       </c>
       <c r="E298" t="inlineStr">
         <is>
@@ -7798,21 +7798,21 @@
     <row r="299">
       <c r="A299" t="inlineStr">
         <is>
-          <t>16:01:44</t>
+          <t>16:57:49</t>
         </is>
       </c>
       <c r="B299" t="inlineStr">
         <is>
-          <t>17:47</t>
+          <t>17:41</t>
         </is>
       </c>
       <c r="C299" t="inlineStr">
         <is>
-          <t>215_EL PELIGRO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D299" t="n">
-        <v>106</v>
+        <v>44</v>
       </c>
       <c r="E299" t="inlineStr">
         <is>
@@ -7823,7 +7823,7 @@
     <row r="300">
       <c r="A300" t="inlineStr">
         <is>
-          <t>16:33:34</t>
+          <t>16:57:49</t>
         </is>
       </c>
       <c r="B300" t="inlineStr">
@@ -7833,11 +7833,11 @@
       </c>
       <c r="C300" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>215_EL PELIGRO</t>
         </is>
       </c>
       <c r="D300" t="n">
-        <v>74</v>
+        <v>50</v>
       </c>
       <c r="E300" t="inlineStr">
         <is>
@@ -7848,21 +7848,21 @@
     <row r="301">
       <c r="A301" t="inlineStr">
         <is>
-          <t>16:49:09</t>
+          <t>16:57:49</t>
         </is>
       </c>
       <c r="B301" t="inlineStr">
         <is>
-          <t>17:48</t>
+          <t>17:47</t>
         </is>
       </c>
       <c r="C301" t="inlineStr">
         <is>
-          <t>215_EL PELIGRO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D301" t="n">
-        <v>59</v>
+        <v>50</v>
       </c>
       <c r="E301" t="inlineStr">
         <is>
@@ -7898,21 +7898,21 @@
     <row r="303">
       <c r="A303" t="inlineStr">
         <is>
-          <t>16:33:34</t>
+          <t>16:49:09</t>
         </is>
       </c>
       <c r="B303" t="inlineStr">
         <is>
-          <t>17:51</t>
+          <t>17:48</t>
         </is>
       </c>
       <c r="C303" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>215_EL PELIGRO</t>
         </is>
       </c>
       <c r="D303" t="n">
-        <v>78</v>
+        <v>59</v>
       </c>
       <c r="E303" t="inlineStr">
         <is>
@@ -7923,21 +7923,21 @@
     <row r="304">
       <c r="A304" t="inlineStr">
         <is>
-          <t>16:49:09</t>
+          <t>16:57:49</t>
         </is>
       </c>
       <c r="B304" t="inlineStr">
         <is>
-          <t>17:59</t>
+          <t>17:51</t>
         </is>
       </c>
       <c r="C304" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D304" t="n">
-        <v>70</v>
+        <v>54</v>
       </c>
       <c r="E304" t="inlineStr">
         <is>
@@ -7948,7 +7948,7 @@
     <row r="305">
       <c r="A305" t="inlineStr">
         <is>
-          <t>16:01:44</t>
+          <t>16:57:49</t>
         </is>
       </c>
       <c r="B305" t="inlineStr">
@@ -7962,7 +7962,7 @@
         </is>
       </c>
       <c r="D305" t="n">
-        <v>118</v>
+        <v>62</v>
       </c>
       <c r="E305" t="inlineStr">
         <is>
@@ -7973,21 +7973,21 @@
     <row r="306">
       <c r="A306" t="inlineStr">
         <is>
-          <t>16:49:09</t>
+          <t>16:57:49</t>
         </is>
       </c>
       <c r="B306" t="inlineStr">
         <is>
-          <t>18:00</t>
+          <t>17:59</t>
         </is>
       </c>
       <c r="C306" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D306" t="n">
-        <v>71</v>
+        <v>62</v>
       </c>
       <c r="E306" t="inlineStr">
         <is>
@@ -8003,16 +8003,16 @@
       </c>
       <c r="B307" t="inlineStr">
         <is>
-          <t>18:01</t>
+          <t>18:00</t>
         </is>
       </c>
       <c r="C307" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D307" t="n">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="E307" t="inlineStr">
         <is>
@@ -8023,21 +8023,21 @@
     <row r="308">
       <c r="A308" t="inlineStr">
         <is>
-          <t>16:33:34</t>
+          <t>16:49:09</t>
         </is>
       </c>
       <c r="B308" t="inlineStr">
         <is>
-          <t>18:11</t>
+          <t>18:01</t>
         </is>
       </c>
       <c r="C308" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D308" t="n">
-        <v>98</v>
+        <v>72</v>
       </c>
       <c r="E308" t="inlineStr">
         <is>
@@ -8048,21 +8048,21 @@
     <row r="309">
       <c r="A309" t="inlineStr">
         <is>
-          <t>16:49:09</t>
+          <t>16:57:49</t>
         </is>
       </c>
       <c r="B309" t="inlineStr">
         <is>
-          <t>18:12</t>
+          <t>18:11</t>
         </is>
       </c>
       <c r="C309" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D309" t="n">
-        <v>83</v>
+        <v>74</v>
       </c>
       <c r="E309" t="inlineStr">
         <is>
@@ -8073,7 +8073,7 @@
     <row r="310">
       <c r="A310" t="inlineStr">
         <is>
-          <t>16:49:09</t>
+          <t>16:57:49</t>
         </is>
       </c>
       <c r="B310" t="inlineStr">
@@ -8083,11 +8083,11 @@
       </c>
       <c r="C310" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D310" t="n">
-        <v>83</v>
+        <v>75</v>
       </c>
       <c r="E310" t="inlineStr">
         <is>
@@ -8103,16 +8103,16 @@
       </c>
       <c r="B311" t="inlineStr">
         <is>
-          <t>18:23</t>
+          <t>18:12</t>
         </is>
       </c>
       <c r="C311" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D311" t="n">
-        <v>94</v>
+        <v>83</v>
       </c>
       <c r="E311" t="inlineStr">
         <is>
@@ -8123,21 +8123,21 @@
     <row r="312">
       <c r="A312" t="inlineStr">
         <is>
-          <t>16:49:09</t>
+          <t>16:57:49</t>
         </is>
       </c>
       <c r="B312" t="inlineStr">
         <is>
-          <t>18:35</t>
+          <t>18:23</t>
         </is>
       </c>
       <c r="C312" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D312" t="n">
-        <v>106</v>
+        <v>86</v>
       </c>
       <c r="E312" t="inlineStr">
         <is>
@@ -8148,23 +8148,148 @@
     <row r="313">
       <c r="A313" t="inlineStr">
         <is>
+          <t>16:57:49</t>
+        </is>
+      </c>
+      <c r="B313" t="inlineStr">
+        <is>
+          <t>18:24</t>
+        </is>
+      </c>
+      <c r="C313" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D313" t="n">
+        <v>87</v>
+      </c>
+      <c r="E313" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="314">
+      <c r="A314" t="inlineStr">
+        <is>
+          <t>16:57:49</t>
+        </is>
+      </c>
+      <c r="B314" t="inlineStr">
+        <is>
+          <t>18:35</t>
+        </is>
+      </c>
+      <c r="C314" t="inlineStr">
+        <is>
+          <t>17X38_ROMERO</t>
+        </is>
+      </c>
+      <c r="D314" t="n">
+        <v>98</v>
+      </c>
+      <c r="E314" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="315">
+      <c r="A315" t="inlineStr">
+        <is>
+          <t>16:57:49</t>
+        </is>
+      </c>
+      <c r="B315" t="inlineStr">
+        <is>
+          <t>18:38</t>
+        </is>
+      </c>
+      <c r="C315" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D315" t="n">
+        <v>101</v>
+      </c>
+      <c r="E315" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="316">
+      <c r="A316" t="inlineStr">
+        <is>
           <t>16:49:09</t>
         </is>
       </c>
-      <c r="B313" t="inlineStr">
+      <c r="B316" t="inlineStr">
         <is>
           <t>18:39</t>
         </is>
       </c>
-      <c r="C313" t="inlineStr">
+      <c r="C316" t="inlineStr">
         <is>
           <t>11_ETCHEVERRY</t>
         </is>
       </c>
-      <c r="D313" t="n">
+      <c r="D316" t="n">
         <v>110</v>
       </c>
-      <c r="E313" t="inlineStr">
+      <c r="E316" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="317">
+      <c r="A317" t="inlineStr">
+        <is>
+          <t>16:57:49</t>
+        </is>
+      </c>
+      <c r="B317" t="inlineStr">
+        <is>
+          <t>18:51</t>
+        </is>
+      </c>
+      <c r="C317" t="inlineStr">
+        <is>
+          <t>16_P MOR-SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D317" t="n">
+        <v>114</v>
+      </c>
+      <c r="E317" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="318">
+      <c r="A318" t="inlineStr">
+        <is>
+          <t>16:57:49</t>
+        </is>
+      </c>
+      <c r="B318" t="inlineStr">
+        <is>
+          <t>18:52</t>
+        </is>
+      </c>
+      <c r="C318" t="inlineStr">
+        <is>
+          <t>14X44_ABASTO</t>
+        </is>
+      </c>
+      <c r="D318" t="n">
+        <v>115</v>
+      </c>
+      <c r="E318" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -8194,7 +8319,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 16:49:09</t>
+          <t>Última actualización: 16:57:49</t>
         </is>
       </c>
     </row>
@@ -9285,7 +9410,7 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>16:01:44</t>
+          <t>16:57:49</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
@@ -9299,7 +9424,7 @@
         </is>
       </c>
       <c r="D48" t="n">
-        <v>58</v>
+        <v>2</v>
       </c>
       <c r="E48" t="inlineStr">
         <is>
@@ -9335,7 +9460,7 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>16:01:44</t>
+          <t>16:57:49</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
@@ -9349,7 +9474,7 @@
         </is>
       </c>
       <c r="D50" t="n">
-        <v>106</v>
+        <v>50</v>
       </c>
       <c r="E50" t="inlineStr">
         <is>
@@ -9360,7 +9485,7 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>16:33:34</t>
+          <t>16:57:49</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
@@ -9374,7 +9499,7 @@
         </is>
       </c>
       <c r="D51" t="n">
-        <v>74</v>
+        <v>50</v>
       </c>
       <c r="E51" t="inlineStr">
         <is>
@@ -9443,7 +9568,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E56"/>
+  <dimension ref="A1:E57"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -9456,14 +9581,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 16:49:09</t>
+          <t>Última actualización: 16:57:49</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 51</t>
+          <t>Total filas: 52</t>
         </is>
       </c>
     </row>
@@ -10722,12 +10847,12 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>16:33:34</t>
+          <t>16:57:49</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>18:25</t>
+          <t>16:57</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
@@ -10736,7 +10861,7 @@
         </is>
       </c>
       <c r="D55" t="n">
-        <v>112</v>
+        <v>0</v>
       </c>
       <c r="E55" t="inlineStr">
         <is>
@@ -10747,23 +10872,48 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
+          <t>16:57:49</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>18:25</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D56" t="n">
+        <v>88</v>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
           <t>16:49:09</t>
         </is>
       </c>
-      <c r="B56" t="inlineStr">
+      <c r="B57" t="inlineStr">
         <is>
           <t>18:26</t>
         </is>
       </c>
-      <c r="C56" t="inlineStr">
+      <c r="C57" t="inlineStr">
         <is>
           <t>215C_LA PLATA</t>
         </is>
       </c>
-      <c r="D56" t="n">
+      <c r="D57" t="n">
         <v>97</v>
       </c>
-      <c r="E56" t="inlineStr">
+      <c r="E57" t="inlineStr">
         <is>
           <t>L6203</t>
         </is>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 1819
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-03-21.xlsx
+++ b/data/horarios-141-2026-03-21.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E318"/>
+  <dimension ref="A1:E325"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 16:57:49</t>
+          <t>Última actualización: 17:21:09</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 313</t>
+          <t>Total filas: 320</t>
         </is>
       </c>
     </row>
@@ -1158,7 +1158,7 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D33" t="n">
@@ -1183,7 +1183,7 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D34" t="n">
@@ -1558,7 +1558,7 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D49" t="n">
@@ -1583,7 +1583,7 @@
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D50" t="n">
@@ -1873,7 +1873,7 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>06:59:30</t>
+          <t>08:14:14</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
@@ -1883,11 +1883,11 @@
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D62" t="n">
-        <v>75</v>
+        <v>0</v>
       </c>
       <c r="E62" t="inlineStr">
         <is>
@@ -1898,7 +1898,7 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>08:14:14</t>
+          <t>06:59:30</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
@@ -1908,11 +1908,11 @@
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D63" t="n">
-        <v>0</v>
+        <v>75</v>
       </c>
       <c r="E63" t="inlineStr">
         <is>
@@ -1933,7 +1933,7 @@
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D64" t="n">
@@ -1998,7 +1998,7 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>07:51:37</t>
+          <t>07:27:35</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
@@ -2008,11 +2008,11 @@
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D67" t="n">
-        <v>28</v>
+        <v>52</v>
       </c>
       <c r="E67" t="inlineStr">
         <is>
@@ -2023,7 +2023,7 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>07:27:35</t>
+          <t>07:51:37</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
@@ -2033,11 +2033,11 @@
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D68" t="n">
-        <v>52</v>
+        <v>28</v>
       </c>
       <c r="E68" t="inlineStr">
         <is>
@@ -2233,7 +2233,7 @@
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D76" t="n">
@@ -2258,7 +2258,7 @@
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D77" t="n">
@@ -2698,7 +2698,7 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>08:14:14</t>
+          <t>08:50:55</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
@@ -2708,11 +2708,11 @@
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>215_EL PELIGRO</t>
         </is>
       </c>
       <c r="D95" t="n">
-        <v>64</v>
+        <v>28</v>
       </c>
       <c r="E95" t="inlineStr">
         <is>
@@ -2723,7 +2723,7 @@
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>08:50:55</t>
+          <t>08:14:14</t>
         </is>
       </c>
       <c r="B96" t="inlineStr">
@@ -2733,11 +2733,11 @@
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>215_EL PELIGRO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D96" t="n">
-        <v>28</v>
+        <v>64</v>
       </c>
       <c r="E96" t="inlineStr">
         <is>
@@ -2873,7 +2873,7 @@
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>07:51:37</t>
+          <t>08:36:09</t>
         </is>
       </c>
       <c r="B102" t="inlineStr">
@@ -2883,11 +2883,11 @@
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D102" t="n">
-        <v>98</v>
+        <v>53</v>
       </c>
       <c r="E102" t="inlineStr">
         <is>
@@ -2898,7 +2898,7 @@
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>08:36:09</t>
+          <t>07:51:37</t>
         </is>
       </c>
       <c r="B103" t="inlineStr">
@@ -2908,11 +2908,11 @@
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D103" t="n">
-        <v>53</v>
+        <v>98</v>
       </c>
       <c r="E103" t="inlineStr">
         <is>
@@ -2923,7 +2923,7 @@
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>08:14:14</t>
+          <t>09:23:24</t>
         </is>
       </c>
       <c r="B104" t="inlineStr">
@@ -2933,11 +2933,11 @@
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D104" t="n">
-        <v>79</v>
+        <v>10</v>
       </c>
       <c r="E104" t="inlineStr">
         <is>
@@ -2948,7 +2948,7 @@
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>09:23:24</t>
+          <t>08:14:14</t>
         </is>
       </c>
       <c r="B105" t="inlineStr">
@@ -2958,11 +2958,11 @@
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D105" t="n">
-        <v>10</v>
+        <v>79</v>
       </c>
       <c r="E105" t="inlineStr">
         <is>
@@ -3083,7 +3083,7 @@
       </c>
       <c r="C110" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D110" t="n">
@@ -3108,7 +3108,7 @@
       </c>
       <c r="C111" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D111" t="n">
@@ -4183,7 +4183,7 @@
       </c>
       <c r="C154" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D154" t="n">
@@ -4208,7 +4208,7 @@
       </c>
       <c r="C155" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D155" t="n">
@@ -4648,7 +4648,7 @@
     <row r="173">
       <c r="A173" t="inlineStr">
         <is>
-          <t>12:28:38</t>
+          <t>12:00:15</t>
         </is>
       </c>
       <c r="B173" t="inlineStr">
@@ -4658,11 +4658,11 @@
       </c>
       <c r="C173" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D173" t="n">
-        <v>5</v>
+        <v>33</v>
       </c>
       <c r="E173" t="inlineStr">
         <is>
@@ -4683,7 +4683,7 @@
       </c>
       <c r="C174" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D174" t="n">
@@ -4698,7 +4698,7 @@
     <row r="175">
       <c r="A175" t="inlineStr">
         <is>
-          <t>12:00:15</t>
+          <t>12:28:38</t>
         </is>
       </c>
       <c r="B175" t="inlineStr">
@@ -4708,11 +4708,11 @@
       </c>
       <c r="C175" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D175" t="n">
-        <v>33</v>
+        <v>5</v>
       </c>
       <c r="E175" t="inlineStr">
         <is>
@@ -4998,7 +4998,7 @@
     <row r="187">
       <c r="A187" t="inlineStr">
         <is>
-          <t>13:00:14</t>
+          <t>12:28:38</t>
         </is>
       </c>
       <c r="B187" t="inlineStr">
@@ -5008,11 +5008,11 @@
       </c>
       <c r="C187" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D187" t="n">
-        <v>3</v>
+        <v>35</v>
       </c>
       <c r="E187" t="inlineStr">
         <is>
@@ -5048,7 +5048,7 @@
     <row r="189">
       <c r="A189" t="inlineStr">
         <is>
-          <t>12:28:38</t>
+          <t>13:00:14</t>
         </is>
       </c>
       <c r="B189" t="inlineStr">
@@ -5058,11 +5058,11 @@
       </c>
       <c r="C189" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D189" t="n">
-        <v>35</v>
+        <v>3</v>
       </c>
       <c r="E189" t="inlineStr">
         <is>
@@ -5073,7 +5073,7 @@
     <row r="190">
       <c r="A190" t="inlineStr">
         <is>
-          <t>12:48:06</t>
+          <t>13:00:14</t>
         </is>
       </c>
       <c r="B190" t="inlineStr">
@@ -5083,11 +5083,11 @@
       </c>
       <c r="C190" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D190" t="n">
-        <v>16</v>
+        <v>4</v>
       </c>
       <c r="E190" t="inlineStr">
         <is>
@@ -5098,7 +5098,7 @@
     <row r="191">
       <c r="A191" t="inlineStr">
         <is>
-          <t>13:00:14</t>
+          <t>12:48:06</t>
         </is>
       </c>
       <c r="B191" t="inlineStr">
@@ -5108,11 +5108,11 @@
       </c>
       <c r="C191" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D191" t="n">
-        <v>4</v>
+        <v>16</v>
       </c>
       <c r="E191" t="inlineStr">
         <is>
@@ -5498,7 +5498,7 @@
     <row r="207">
       <c r="A207" t="inlineStr">
         <is>
-          <t>13:32:57</t>
+          <t>13:57:43</t>
         </is>
       </c>
       <c r="B207" t="inlineStr">
@@ -5508,11 +5508,11 @@
       </c>
       <c r="C207" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D207" t="n">
-        <v>27</v>
+        <v>2</v>
       </c>
       <c r="E207" t="inlineStr">
         <is>
@@ -5523,7 +5523,7 @@
     <row r="208">
       <c r="A208" t="inlineStr">
         <is>
-          <t>13:57:43</t>
+          <t>13:32:57</t>
         </is>
       </c>
       <c r="B208" t="inlineStr">
@@ -5533,11 +5533,11 @@
       </c>
       <c r="C208" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D208" t="n">
-        <v>2</v>
+        <v>27</v>
       </c>
       <c r="E208" t="inlineStr">
         <is>
@@ -5573,7 +5573,7 @@
     <row r="210">
       <c r="A210" t="inlineStr">
         <is>
-          <t>13:57:43</t>
+          <t>13:00:14</t>
         </is>
       </c>
       <c r="B210" t="inlineStr">
@@ -5583,11 +5583,11 @@
       </c>
       <c r="C210" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D210" t="n">
-        <v>6</v>
+        <v>63</v>
       </c>
       <c r="E210" t="inlineStr">
         <is>
@@ -5598,7 +5598,7 @@
     <row r="211">
       <c r="A211" t="inlineStr">
         <is>
-          <t>13:00:14</t>
+          <t>13:57:43</t>
         </is>
       </c>
       <c r="B211" t="inlineStr">
@@ -5608,11 +5608,11 @@
       </c>
       <c r="C211" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D211" t="n">
-        <v>63</v>
+        <v>6</v>
       </c>
       <c r="E211" t="inlineStr">
         <is>
@@ -6298,7 +6298,7 @@
     <row r="239">
       <c r="A239" t="inlineStr">
         <is>
-          <t>14:59:00</t>
+          <t>14:46:39</t>
         </is>
       </c>
       <c r="B239" t="inlineStr">
@@ -6308,11 +6308,11 @@
       </c>
       <c r="C239" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D239" t="n">
-        <v>12</v>
+        <v>25</v>
       </c>
       <c r="E239" t="inlineStr">
         <is>
@@ -6323,7 +6323,7 @@
     <row r="240">
       <c r="A240" t="inlineStr">
         <is>
-          <t>14:46:39</t>
+          <t>14:59:00</t>
         </is>
       </c>
       <c r="B240" t="inlineStr">
@@ -6333,11 +6333,11 @@
       </c>
       <c r="C240" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D240" t="n">
-        <v>25</v>
+        <v>12</v>
       </c>
       <c r="E240" t="inlineStr">
         <is>
@@ -6933,7 +6933,7 @@
       </c>
       <c r="C264" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>215_ALUAR</t>
         </is>
       </c>
       <c r="D264" t="n">
@@ -6958,7 +6958,7 @@
       </c>
       <c r="C265" t="inlineStr">
         <is>
-          <t>215_ALUAR</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D265" t="n">
@@ -7073,7 +7073,7 @@
     <row r="270">
       <c r="A270" t="inlineStr">
         <is>
-          <t>16:01:44</t>
+          <t>16:33:34</t>
         </is>
       </c>
       <c r="B270" t="inlineStr">
@@ -7083,11 +7083,11 @@
       </c>
       <c r="C270" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D270" t="n">
-        <v>34</v>
+        <v>2</v>
       </c>
       <c r="E270" t="inlineStr">
         <is>
@@ -7098,7 +7098,7 @@
     <row r="271">
       <c r="A271" t="inlineStr">
         <is>
-          <t>16:33:34</t>
+          <t>16:01:44</t>
         </is>
       </c>
       <c r="B271" t="inlineStr">
@@ -7108,11 +7108,11 @@
       </c>
       <c r="C271" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D271" t="n">
-        <v>2</v>
+        <v>34</v>
       </c>
       <c r="E271" t="inlineStr">
         <is>
@@ -7333,7 +7333,7 @@
       </c>
       <c r="C280" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D280" t="n">
@@ -7358,7 +7358,7 @@
       </c>
       <c r="C281" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D281" t="n">
@@ -7383,7 +7383,7 @@
       </c>
       <c r="C282" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D282" t="n">
@@ -7408,7 +7408,7 @@
       </c>
       <c r="C283" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D283" t="n">
@@ -7573,7 +7573,7 @@
     <row r="290">
       <c r="A290" t="inlineStr">
         <is>
-          <t>16:49:09</t>
+          <t>17:21:09</t>
         </is>
       </c>
       <c r="B290" t="inlineStr">
@@ -7587,7 +7587,7 @@
         </is>
       </c>
       <c r="D290" t="n">
-        <v>35</v>
+        <v>3</v>
       </c>
       <c r="E290" t="inlineStr">
         <is>
@@ -7623,7 +7623,7 @@
     <row r="292">
       <c r="A292" t="inlineStr">
         <is>
-          <t>16:57:49</t>
+          <t>17:21:09</t>
         </is>
       </c>
       <c r="B292" t="inlineStr">
@@ -7637,7 +7637,7 @@
         </is>
       </c>
       <c r="D292" t="n">
-        <v>36</v>
+        <v>12</v>
       </c>
       <c r="E292" t="inlineStr">
         <is>
@@ -7648,7 +7648,7 @@
     <row r="293">
       <c r="A293" t="inlineStr">
         <is>
-          <t>16:57:49</t>
+          <t>16:33:34</t>
         </is>
       </c>
       <c r="B293" t="inlineStr">
@@ -7658,11 +7658,11 @@
       </c>
       <c r="C293" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D293" t="n">
-        <v>38</v>
+        <v>62</v>
       </c>
       <c r="E293" t="inlineStr">
         <is>
@@ -7673,7 +7673,7 @@
     <row r="294">
       <c r="A294" t="inlineStr">
         <is>
-          <t>16:57:49</t>
+          <t>17:21:09</t>
         </is>
       </c>
       <c r="B294" t="inlineStr">
@@ -7687,7 +7687,7 @@
         </is>
       </c>
       <c r="D294" t="n">
-        <v>38</v>
+        <v>14</v>
       </c>
       <c r="E294" t="inlineStr">
         <is>
@@ -7698,7 +7698,7 @@
     <row r="295">
       <c r="A295" t="inlineStr">
         <is>
-          <t>16:33:34</t>
+          <t>17:21:09</t>
         </is>
       </c>
       <c r="B295" t="inlineStr">
@@ -7708,11 +7708,11 @@
       </c>
       <c r="C295" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D295" t="n">
-        <v>62</v>
+        <v>14</v>
       </c>
       <c r="E295" t="inlineStr">
         <is>
@@ -7748,7 +7748,7 @@
     <row r="297">
       <c r="A297" t="inlineStr">
         <is>
-          <t>16:49:09</t>
+          <t>17:21:09</t>
         </is>
       </c>
       <c r="B297" t="inlineStr">
@@ -7762,7 +7762,7 @@
         </is>
       </c>
       <c r="D297" t="n">
-        <v>48</v>
+        <v>16</v>
       </c>
       <c r="E297" t="inlineStr">
         <is>
@@ -7798,7 +7798,7 @@
     <row r="299">
       <c r="A299" t="inlineStr">
         <is>
-          <t>16:57:49</t>
+          <t>17:21:09</t>
         </is>
       </c>
       <c r="B299" t="inlineStr">
@@ -7812,7 +7812,7 @@
         </is>
       </c>
       <c r="D299" t="n">
-        <v>44</v>
+        <v>20</v>
       </c>
       <c r="E299" t="inlineStr">
         <is>
@@ -7833,7 +7833,7 @@
       </c>
       <c r="C300" t="inlineStr">
         <is>
-          <t>215_EL PELIGRO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D300" t="n">
@@ -7858,7 +7858,7 @@
       </c>
       <c r="C301" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>215_EL PELIGRO</t>
         </is>
       </c>
       <c r="D301" t="n">
@@ -7873,7 +7873,7 @@
     <row r="302">
       <c r="A302" t="inlineStr">
         <is>
-          <t>16:49:09</t>
+          <t>17:21:09</t>
         </is>
       </c>
       <c r="B302" t="inlineStr">
@@ -7883,11 +7883,11 @@
       </c>
       <c r="C302" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>215_EL PELIGRO</t>
         </is>
       </c>
       <c r="D302" t="n">
-        <v>59</v>
+        <v>27</v>
       </c>
       <c r="E302" t="inlineStr">
         <is>
@@ -7898,7 +7898,7 @@
     <row r="303">
       <c r="A303" t="inlineStr">
         <is>
-          <t>16:49:09</t>
+          <t>17:21:09</t>
         </is>
       </c>
       <c r="B303" t="inlineStr">
@@ -7908,11 +7908,11 @@
       </c>
       <c r="C303" t="inlineStr">
         <is>
-          <t>215_EL PELIGRO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D303" t="n">
-        <v>59</v>
+        <v>27</v>
       </c>
       <c r="E303" t="inlineStr">
         <is>
@@ -7923,7 +7923,7 @@
     <row r="304">
       <c r="A304" t="inlineStr">
         <is>
-          <t>16:57:49</t>
+          <t>17:21:09</t>
         </is>
       </c>
       <c r="B304" t="inlineStr">
@@ -7937,7 +7937,7 @@
         </is>
       </c>
       <c r="D304" t="n">
-        <v>54</v>
+        <v>30</v>
       </c>
       <c r="E304" t="inlineStr">
         <is>
@@ -7973,7 +7973,7 @@
     <row r="306">
       <c r="A306" t="inlineStr">
         <is>
-          <t>16:57:49</t>
+          <t>17:21:09</t>
         </is>
       </c>
       <c r="B306" t="inlineStr">
@@ -7987,7 +7987,7 @@
         </is>
       </c>
       <c r="D306" t="n">
-        <v>62</v>
+        <v>38</v>
       </c>
       <c r="E306" t="inlineStr">
         <is>
@@ -7998,7 +7998,7 @@
     <row r="307">
       <c r="A307" t="inlineStr">
         <is>
-          <t>16:49:09</t>
+          <t>17:21:09</t>
         </is>
       </c>
       <c r="B307" t="inlineStr">
@@ -8012,7 +8012,7 @@
         </is>
       </c>
       <c r="D307" t="n">
-        <v>71</v>
+        <v>39</v>
       </c>
       <c r="E307" t="inlineStr">
         <is>
@@ -8023,7 +8023,7 @@
     <row r="308">
       <c r="A308" t="inlineStr">
         <is>
-          <t>16:49:09</t>
+          <t>17:21:09</t>
         </is>
       </c>
       <c r="B308" t="inlineStr">
@@ -8037,7 +8037,7 @@
         </is>
       </c>
       <c r="D308" t="n">
-        <v>72</v>
+        <v>40</v>
       </c>
       <c r="E308" t="inlineStr">
         <is>
@@ -8073,7 +8073,7 @@
     <row r="310">
       <c r="A310" t="inlineStr">
         <is>
-          <t>16:57:49</t>
+          <t>17:21:09</t>
         </is>
       </c>
       <c r="B310" t="inlineStr">
@@ -8083,11 +8083,11 @@
       </c>
       <c r="C310" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D310" t="n">
-        <v>75</v>
+        <v>51</v>
       </c>
       <c r="E310" t="inlineStr">
         <is>
@@ -8098,7 +8098,7 @@
     <row r="311">
       <c r="A311" t="inlineStr">
         <is>
-          <t>16:49:09</t>
+          <t>16:57:49</t>
         </is>
       </c>
       <c r="B311" t="inlineStr">
@@ -8108,11 +8108,11 @@
       </c>
       <c r="C311" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D311" t="n">
-        <v>83</v>
+        <v>75</v>
       </c>
       <c r="E311" t="inlineStr">
         <is>
@@ -8123,21 +8123,21 @@
     <row r="312">
       <c r="A312" t="inlineStr">
         <is>
-          <t>16:57:49</t>
+          <t>17:21:09</t>
         </is>
       </c>
       <c r="B312" t="inlineStr">
         <is>
-          <t>18:23</t>
+          <t>18:14</t>
         </is>
       </c>
       <c r="C312" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D312" t="n">
-        <v>86</v>
+        <v>53</v>
       </c>
       <c r="E312" t="inlineStr">
         <is>
@@ -8148,21 +8148,21 @@
     <row r="313">
       <c r="A313" t="inlineStr">
         <is>
-          <t>16:57:49</t>
+          <t>17:21:09</t>
         </is>
       </c>
       <c r="B313" t="inlineStr">
         <is>
-          <t>18:24</t>
+          <t>18:23</t>
         </is>
       </c>
       <c r="C313" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D313" t="n">
-        <v>87</v>
+        <v>62</v>
       </c>
       <c r="E313" t="inlineStr">
         <is>
@@ -8173,21 +8173,21 @@
     <row r="314">
       <c r="A314" t="inlineStr">
         <is>
-          <t>16:57:49</t>
+          <t>17:21:09</t>
         </is>
       </c>
       <c r="B314" t="inlineStr">
         <is>
-          <t>18:35</t>
+          <t>18:24</t>
         </is>
       </c>
       <c r="C314" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D314" t="n">
-        <v>98</v>
+        <v>63</v>
       </c>
       <c r="E314" t="inlineStr">
         <is>
@@ -8198,21 +8198,21 @@
     <row r="315">
       <c r="A315" t="inlineStr">
         <is>
-          <t>16:57:49</t>
+          <t>17:21:09</t>
         </is>
       </c>
       <c r="B315" t="inlineStr">
         <is>
-          <t>18:38</t>
+          <t>18:34</t>
         </is>
       </c>
       <c r="C315" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D315" t="n">
-        <v>101</v>
+        <v>73</v>
       </c>
       <c r="E315" t="inlineStr">
         <is>
@@ -8223,21 +8223,21 @@
     <row r="316">
       <c r="A316" t="inlineStr">
         <is>
-          <t>16:49:09</t>
+          <t>17:21:09</t>
         </is>
       </c>
       <c r="B316" t="inlineStr">
         <is>
-          <t>18:39</t>
+          <t>18:35</t>
         </is>
       </c>
       <c r="C316" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D316" t="n">
-        <v>110</v>
+        <v>74</v>
       </c>
       <c r="E316" t="inlineStr">
         <is>
@@ -8253,16 +8253,16 @@
       </c>
       <c r="B317" t="inlineStr">
         <is>
-          <t>18:51</t>
+          <t>18:38</t>
         </is>
       </c>
       <c r="C317" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D317" t="n">
-        <v>114</v>
+        <v>101</v>
       </c>
       <c r="E317" t="inlineStr">
         <is>
@@ -8273,23 +8273,198 @@
     <row r="318">
       <c r="A318" t="inlineStr">
         <is>
+          <t>17:21:09</t>
+        </is>
+      </c>
+      <c r="B318" t="inlineStr">
+        <is>
+          <t>18:39</t>
+        </is>
+      </c>
+      <c r="C318" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D318" t="n">
+        <v>78</v>
+      </c>
+      <c r="E318" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="319">
+      <c r="A319" t="inlineStr">
+        <is>
+          <t>17:21:09</t>
+        </is>
+      </c>
+      <c r="B319" t="inlineStr">
+        <is>
+          <t>18:51</t>
+        </is>
+      </c>
+      <c r="C319" t="inlineStr">
+        <is>
+          <t>16_P MOR-SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D319" t="n">
+        <v>90</v>
+      </c>
+      <c r="E319" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="320">
+      <c r="A320" t="inlineStr">
+        <is>
           <t>16:57:49</t>
         </is>
       </c>
-      <c r="B318" t="inlineStr">
+      <c r="B320" t="inlineStr">
         <is>
           <t>18:52</t>
         </is>
       </c>
-      <c r="C318" t="inlineStr">
+      <c r="C320" t="inlineStr">
         <is>
           <t>14X44_ABASTO</t>
         </is>
       </c>
-      <c r="D318" t="n">
+      <c r="D320" t="n">
         <v>115</v>
       </c>
-      <c r="E318" t="inlineStr">
+      <c r="E320" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="321">
+      <c r="A321" t="inlineStr">
+        <is>
+          <t>17:21:09</t>
+        </is>
+      </c>
+      <c r="B321" t="inlineStr">
+        <is>
+          <t>18:53</t>
+        </is>
+      </c>
+      <c r="C321" t="inlineStr">
+        <is>
+          <t>14X44_ABASTO</t>
+        </is>
+      </c>
+      <c r="D321" t="n">
+        <v>92</v>
+      </c>
+      <c r="E321" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="322">
+      <c r="A322" t="inlineStr">
+        <is>
+          <t>17:21:09</t>
+        </is>
+      </c>
+      <c r="B322" t="inlineStr">
+        <is>
+          <t>19:00</t>
+        </is>
+      </c>
+      <c r="C322" t="inlineStr">
+        <is>
+          <t>17_ROMERO</t>
+        </is>
+      </c>
+      <c r="D322" t="n">
+        <v>99</v>
+      </c>
+      <c r="E322" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="323">
+      <c r="A323" t="inlineStr">
+        <is>
+          <t>17:21:09</t>
+        </is>
+      </c>
+      <c r="B323" t="inlineStr">
+        <is>
+          <t>19:09</t>
+        </is>
+      </c>
+      <c r="C323" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D323" t="n">
+        <v>108</v>
+      </c>
+      <c r="E323" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="324">
+      <c r="A324" t="inlineStr">
+        <is>
+          <t>17:21:09</t>
+        </is>
+      </c>
+      <c r="B324" t="inlineStr">
+        <is>
+          <t>19:12</t>
+        </is>
+      </c>
+      <c r="C324" t="inlineStr">
+        <is>
+          <t>81_EL PELIGRO</t>
+        </is>
+      </c>
+      <c r="D324" t="n">
+        <v>111</v>
+      </c>
+      <c r="E324" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="325">
+      <c r="A325" t="inlineStr">
+        <is>
+          <t>17:21:09</t>
+        </is>
+      </c>
+      <c r="B325" t="inlineStr">
+        <is>
+          <t>19:17</t>
+        </is>
+      </c>
+      <c r="C325" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D325" t="n">
+        <v>116</v>
+      </c>
+      <c r="E325" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -8319,7 +8494,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 16:57:49</t>
+          <t>Última actualización: 17:21:09</t>
         </is>
       </c>
     </row>
@@ -9510,7 +9685,7 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>16:49:09</t>
+          <t>17:21:09</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
@@ -9524,7 +9699,7 @@
         </is>
       </c>
       <c r="D52" t="n">
-        <v>59</v>
+        <v>27</v>
       </c>
       <c r="E52" t="inlineStr">
         <is>
@@ -9535,7 +9710,7 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>16:49:09</t>
+          <t>17:21:09</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
@@ -9549,7 +9724,7 @@
         </is>
       </c>
       <c r="D53" t="n">
-        <v>59</v>
+        <v>27</v>
       </c>
       <c r="E53" t="inlineStr">
         <is>
@@ -9568,7 +9743,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E57"/>
+  <dimension ref="A1:E58"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -9581,14 +9756,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 16:57:49</t>
+          <t>Última actualización: 17:21:09</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 52</t>
+          <t>Total filas: 53</t>
         </is>
       </c>
     </row>
@@ -10897,7 +11072,7 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>16:49:09</t>
+          <t>17:21:09</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
@@ -10911,11 +11086,36 @@
         </is>
       </c>
       <c r="D57" t="n">
-        <v>97</v>
+        <v>65</v>
       </c>
       <c r="E57" t="inlineStr">
         <is>
           <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>17:21:09</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>19:18</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>215B_LP-P MOR-1 Y 57</t>
+        </is>
+      </c>
+      <c r="D58" t="n">
+        <v>117</v>
+      </c>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>L6173</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 1820
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-03-21.xlsx
+++ b/data/horarios-141-2026-03-21.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E325"/>
+  <dimension ref="A1:E334"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 17:21:09</t>
+          <t>Última actualización: 17:47:20</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 320</t>
+          <t>Total filas: 329</t>
         </is>
       </c>
     </row>
@@ -1158,7 +1158,7 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D33" t="n">
@@ -1183,7 +1183,7 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D34" t="n">
@@ -1873,7 +1873,7 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>08:14:14</t>
+          <t>06:59:30</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
@@ -1883,11 +1883,11 @@
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D62" t="n">
-        <v>0</v>
+        <v>75</v>
       </c>
       <c r="E62" t="inlineStr">
         <is>
@@ -1898,7 +1898,7 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>06:59:30</t>
+          <t>08:14:14</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
@@ -1908,11 +1908,11 @@
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D63" t="n">
-        <v>75</v>
+        <v>0</v>
       </c>
       <c r="E63" t="inlineStr">
         <is>
@@ -1933,7 +1933,7 @@
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D64" t="n">
@@ -2233,7 +2233,7 @@
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D76" t="n">
@@ -2258,7 +2258,7 @@
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D77" t="n">
@@ -2708,7 +2708,7 @@
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>215_EL PELIGRO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D95" t="n">
@@ -2723,7 +2723,7 @@
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>08:14:14</t>
+          <t>08:50:55</t>
         </is>
       </c>
       <c r="B96" t="inlineStr">
@@ -2733,11 +2733,11 @@
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>215_EL PELIGRO</t>
         </is>
       </c>
       <c r="D96" t="n">
-        <v>64</v>
+        <v>28</v>
       </c>
       <c r="E96" t="inlineStr">
         <is>
@@ -2748,7 +2748,7 @@
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>08:50:55</t>
+          <t>08:14:14</t>
         </is>
       </c>
       <c r="B97" t="inlineStr">
@@ -2758,11 +2758,11 @@
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D97" t="n">
-        <v>28</v>
+        <v>64</v>
       </c>
       <c r="E97" t="inlineStr">
         <is>
@@ -3083,7 +3083,7 @@
       </c>
       <c r="C110" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D110" t="n">
@@ -3108,7 +3108,7 @@
       </c>
       <c r="C111" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D111" t="n">
@@ -3498,7 +3498,7 @@
     <row r="127">
       <c r="A127" t="inlineStr">
         <is>
-          <t>08:36:09</t>
+          <t>10:14:52</t>
         </is>
       </c>
       <c r="B127" t="inlineStr">
@@ -3508,11 +3508,11 @@
       </c>
       <c r="C127" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D127" t="n">
-        <v>117</v>
+        <v>19</v>
       </c>
       <c r="E127" t="inlineStr">
         <is>
@@ -3523,7 +3523,7 @@
     <row r="128">
       <c r="A128" t="inlineStr">
         <is>
-          <t>10:14:52</t>
+          <t>08:36:09</t>
         </is>
       </c>
       <c r="B128" t="inlineStr">
@@ -3533,11 +3533,11 @@
       </c>
       <c r="C128" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D128" t="n">
-        <v>19</v>
+        <v>117</v>
       </c>
       <c r="E128" t="inlineStr">
         <is>
@@ -4123,7 +4123,7 @@
     <row r="152">
       <c r="A152" t="inlineStr">
         <is>
-          <t>11:16:36</t>
+          <t>10:14:52</t>
         </is>
       </c>
       <c r="B152" t="inlineStr">
@@ -4133,11 +4133,11 @@
       </c>
       <c r="C152" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D152" t="n">
-        <v>16</v>
+        <v>78</v>
       </c>
       <c r="E152" t="inlineStr">
         <is>
@@ -4148,7 +4148,7 @@
     <row r="153">
       <c r="A153" t="inlineStr">
         <is>
-          <t>10:14:52</t>
+          <t>11:16:36</t>
         </is>
       </c>
       <c r="B153" t="inlineStr">
@@ -4158,11 +4158,11 @@
       </c>
       <c r="C153" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D153" t="n">
-        <v>78</v>
+        <v>16</v>
       </c>
       <c r="E153" t="inlineStr">
         <is>
@@ -4473,7 +4473,7 @@
     <row r="166">
       <c r="A166" t="inlineStr">
         <is>
-          <t>12:00:15</t>
+          <t>11:16:36</t>
         </is>
       </c>
       <c r="B166" t="inlineStr">
@@ -4483,11 +4483,11 @@
       </c>
       <c r="C166" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D166" t="n">
-        <v>4</v>
+        <v>48</v>
       </c>
       <c r="E166" t="inlineStr">
         <is>
@@ -4498,7 +4498,7 @@
     <row r="167">
       <c r="A167" t="inlineStr">
         <is>
-          <t>11:16:36</t>
+          <t>12:00:15</t>
         </is>
       </c>
       <c r="B167" t="inlineStr">
@@ -4508,11 +4508,11 @@
       </c>
       <c r="C167" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D167" t="n">
-        <v>48</v>
+        <v>4</v>
       </c>
       <c r="E167" t="inlineStr">
         <is>
@@ -4648,7 +4648,7 @@
     <row r="173">
       <c r="A173" t="inlineStr">
         <is>
-          <t>12:00:15</t>
+          <t>12:28:38</t>
         </is>
       </c>
       <c r="B173" t="inlineStr">
@@ -4658,11 +4658,11 @@
       </c>
       <c r="C173" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D173" t="n">
-        <v>33</v>
+        <v>5</v>
       </c>
       <c r="E173" t="inlineStr">
         <is>
@@ -4698,7 +4698,7 @@
     <row r="175">
       <c r="A175" t="inlineStr">
         <is>
-          <t>12:28:38</t>
+          <t>12:00:15</t>
         </is>
       </c>
       <c r="B175" t="inlineStr">
@@ -4708,11 +4708,11 @@
       </c>
       <c r="C175" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D175" t="n">
-        <v>5</v>
+        <v>33</v>
       </c>
       <c r="E175" t="inlineStr">
         <is>
@@ -4998,7 +4998,7 @@
     <row r="187">
       <c r="A187" t="inlineStr">
         <is>
-          <t>12:28:38</t>
+          <t>13:00:14</t>
         </is>
       </c>
       <c r="B187" t="inlineStr">
@@ -5008,11 +5008,11 @@
       </c>
       <c r="C187" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D187" t="n">
-        <v>35</v>
+        <v>3</v>
       </c>
       <c r="E187" t="inlineStr">
         <is>
@@ -5033,7 +5033,7 @@
       </c>
       <c r="C188" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D188" t="n">
@@ -5048,7 +5048,7 @@
     <row r="189">
       <c r="A189" t="inlineStr">
         <is>
-          <t>13:00:14</t>
+          <t>12:28:38</t>
         </is>
       </c>
       <c r="B189" t="inlineStr">
@@ -5058,11 +5058,11 @@
       </c>
       <c r="C189" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D189" t="n">
-        <v>3</v>
+        <v>35</v>
       </c>
       <c r="E189" t="inlineStr">
         <is>
@@ -5498,7 +5498,7 @@
     <row r="207">
       <c r="A207" t="inlineStr">
         <is>
-          <t>13:57:43</t>
+          <t>13:32:57</t>
         </is>
       </c>
       <c r="B207" t="inlineStr">
@@ -5508,11 +5508,11 @@
       </c>
       <c r="C207" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D207" t="n">
-        <v>2</v>
+        <v>27</v>
       </c>
       <c r="E207" t="inlineStr">
         <is>
@@ -5523,7 +5523,7 @@
     <row r="208">
       <c r="A208" t="inlineStr">
         <is>
-          <t>13:32:57</t>
+          <t>13:57:43</t>
         </is>
       </c>
       <c r="B208" t="inlineStr">
@@ -5533,11 +5533,11 @@
       </c>
       <c r="C208" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D208" t="n">
-        <v>27</v>
+        <v>2</v>
       </c>
       <c r="E208" t="inlineStr">
         <is>
@@ -5573,7 +5573,7 @@
     <row r="210">
       <c r="A210" t="inlineStr">
         <is>
-          <t>13:00:14</t>
+          <t>13:57:43</t>
         </is>
       </c>
       <c r="B210" t="inlineStr">
@@ -5583,11 +5583,11 @@
       </c>
       <c r="C210" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D210" t="n">
-        <v>63</v>
+        <v>6</v>
       </c>
       <c r="E210" t="inlineStr">
         <is>
@@ -5598,7 +5598,7 @@
     <row r="211">
       <c r="A211" t="inlineStr">
         <is>
-          <t>13:57:43</t>
+          <t>13:00:14</t>
         </is>
       </c>
       <c r="B211" t="inlineStr">
@@ -5608,11 +5608,11 @@
       </c>
       <c r="C211" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D211" t="n">
-        <v>6</v>
+        <v>63</v>
       </c>
       <c r="E211" t="inlineStr">
         <is>
@@ -5623,7 +5623,7 @@
     <row r="212">
       <c r="A212" t="inlineStr">
         <is>
-          <t>13:57:43</t>
+          <t>13:32:57</t>
         </is>
       </c>
       <c r="B212" t="inlineStr">
@@ -5633,11 +5633,11 @@
       </c>
       <c r="C212" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D212" t="n">
-        <v>19</v>
+        <v>44</v>
       </c>
       <c r="E212" t="inlineStr">
         <is>
@@ -5648,7 +5648,7 @@
     <row r="213">
       <c r="A213" t="inlineStr">
         <is>
-          <t>13:32:57</t>
+          <t>13:57:43</t>
         </is>
       </c>
       <c r="B213" t="inlineStr">
@@ -5658,11 +5658,11 @@
       </c>
       <c r="C213" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D213" t="n">
-        <v>44</v>
+        <v>19</v>
       </c>
       <c r="E213" t="inlineStr">
         <is>
@@ -5873,7 +5873,7 @@
     <row r="222">
       <c r="A222" t="inlineStr">
         <is>
-          <t>13:00:14</t>
+          <t>14:21:42</t>
         </is>
       </c>
       <c r="B222" t="inlineStr">
@@ -5883,11 +5883,11 @@
       </c>
       <c r="C222" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D222" t="n">
-        <v>93</v>
+        <v>12</v>
       </c>
       <c r="E222" t="inlineStr">
         <is>
@@ -5898,7 +5898,7 @@
     <row r="223">
       <c r="A223" t="inlineStr">
         <is>
-          <t>14:21:42</t>
+          <t>13:00:14</t>
         </is>
       </c>
       <c r="B223" t="inlineStr">
@@ -5908,11 +5908,11 @@
       </c>
       <c r="C223" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D223" t="n">
-        <v>12</v>
+        <v>93</v>
       </c>
       <c r="E223" t="inlineStr">
         <is>
@@ -6173,7 +6173,7 @@
     <row r="234">
       <c r="A234" t="inlineStr">
         <is>
-          <t>14:46:39</t>
+          <t>14:59:00</t>
         </is>
       </c>
       <c r="B234" t="inlineStr">
@@ -6183,11 +6183,11 @@
       </c>
       <c r="C234" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D234" t="n">
-        <v>15</v>
+        <v>2</v>
       </c>
       <c r="E234" t="inlineStr">
         <is>
@@ -6198,7 +6198,7 @@
     <row r="235">
       <c r="A235" t="inlineStr">
         <is>
-          <t>14:59:00</t>
+          <t>14:46:39</t>
         </is>
       </c>
       <c r="B235" t="inlineStr">
@@ -6208,11 +6208,11 @@
       </c>
       <c r="C235" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D235" t="n">
-        <v>2</v>
+        <v>15</v>
       </c>
       <c r="E235" t="inlineStr">
         <is>
@@ -6298,7 +6298,7 @@
     <row r="239">
       <c r="A239" t="inlineStr">
         <is>
-          <t>14:46:39</t>
+          <t>14:59:00</t>
         </is>
       </c>
       <c r="B239" t="inlineStr">
@@ -6308,11 +6308,11 @@
       </c>
       <c r="C239" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D239" t="n">
-        <v>25</v>
+        <v>12</v>
       </c>
       <c r="E239" t="inlineStr">
         <is>
@@ -6323,7 +6323,7 @@
     <row r="240">
       <c r="A240" t="inlineStr">
         <is>
-          <t>14:59:00</t>
+          <t>14:46:39</t>
         </is>
       </c>
       <c r="B240" t="inlineStr">
@@ -6333,11 +6333,11 @@
       </c>
       <c r="C240" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D240" t="n">
-        <v>12</v>
+        <v>25</v>
       </c>
       <c r="E240" t="inlineStr">
         <is>
@@ -6698,7 +6698,7 @@
     <row r="255">
       <c r="A255" t="inlineStr">
         <is>
-          <t>15:34:45</t>
+          <t>14:46:39</t>
         </is>
       </c>
       <c r="B255" t="inlineStr">
@@ -6708,11 +6708,11 @@
       </c>
       <c r="C255" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D255" t="n">
-        <v>20</v>
+        <v>68</v>
       </c>
       <c r="E255" t="inlineStr">
         <is>
@@ -6723,7 +6723,7 @@
     <row r="256">
       <c r="A256" t="inlineStr">
         <is>
-          <t>14:46:39</t>
+          <t>15:34:45</t>
         </is>
       </c>
       <c r="B256" t="inlineStr">
@@ -6733,11 +6733,11 @@
       </c>
       <c r="C256" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D256" t="n">
-        <v>68</v>
+        <v>20</v>
       </c>
       <c r="E256" t="inlineStr">
         <is>
@@ -6933,7 +6933,7 @@
       </c>
       <c r="C264" t="inlineStr">
         <is>
-          <t>215_ALUAR</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D264" t="n">
@@ -6958,7 +6958,7 @@
       </c>
       <c r="C265" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>215_ALUAR</t>
         </is>
       </c>
       <c r="D265" t="n">
@@ -7033,7 +7033,7 @@
       </c>
       <c r="C268" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D268" t="n">
@@ -7058,7 +7058,7 @@
       </c>
       <c r="C269" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D269" t="n">
@@ -7333,7 +7333,7 @@
       </c>
       <c r="C280" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D280" t="n">
@@ -7358,7 +7358,7 @@
       </c>
       <c r="C281" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D281" t="n">
@@ -7648,7 +7648,7 @@
     <row r="293">
       <c r="A293" t="inlineStr">
         <is>
-          <t>16:33:34</t>
+          <t>17:21:09</t>
         </is>
       </c>
       <c r="B293" t="inlineStr">
@@ -7658,11 +7658,11 @@
       </c>
       <c r="C293" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D293" t="n">
-        <v>62</v>
+        <v>14</v>
       </c>
       <c r="E293" t="inlineStr">
         <is>
@@ -7673,7 +7673,7 @@
     <row r="294">
       <c r="A294" t="inlineStr">
         <is>
-          <t>17:21:09</t>
+          <t>16:33:34</t>
         </is>
       </c>
       <c r="B294" t="inlineStr">
@@ -7683,11 +7683,11 @@
       </c>
       <c r="C294" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D294" t="n">
-        <v>14</v>
+        <v>62</v>
       </c>
       <c r="E294" t="inlineStr">
         <is>
@@ -7708,7 +7708,7 @@
       </c>
       <c r="C295" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D295" t="n">
@@ -7823,7 +7823,7 @@
     <row r="300">
       <c r="A300" t="inlineStr">
         <is>
-          <t>16:57:49</t>
+          <t>17:47:19</t>
         </is>
       </c>
       <c r="B300" t="inlineStr">
@@ -7833,11 +7833,11 @@
       </c>
       <c r="C300" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>215_EL PELIGRO</t>
         </is>
       </c>
       <c r="D300" t="n">
-        <v>50</v>
+        <v>0</v>
       </c>
       <c r="E300" t="inlineStr">
         <is>
@@ -7848,7 +7848,7 @@
     <row r="301">
       <c r="A301" t="inlineStr">
         <is>
-          <t>16:57:49</t>
+          <t>17:47:19</t>
         </is>
       </c>
       <c r="B301" t="inlineStr">
@@ -7858,11 +7858,11 @@
       </c>
       <c r="C301" t="inlineStr">
         <is>
-          <t>215_EL PELIGRO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D301" t="n">
-        <v>50</v>
+        <v>0</v>
       </c>
       <c r="E301" t="inlineStr">
         <is>
@@ -7883,7 +7883,7 @@
       </c>
       <c r="C302" t="inlineStr">
         <is>
-          <t>215_EL PELIGRO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D302" t="n">
@@ -7908,7 +7908,7 @@
       </c>
       <c r="C303" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>215_EL PELIGRO</t>
         </is>
       </c>
       <c r="D303" t="n">
@@ -7923,7 +7923,7 @@
     <row r="304">
       <c r="A304" t="inlineStr">
         <is>
-          <t>17:21:09</t>
+          <t>17:47:19</t>
         </is>
       </c>
       <c r="B304" t="inlineStr">
@@ -7937,7 +7937,7 @@
         </is>
       </c>
       <c r="D304" t="n">
-        <v>30</v>
+        <v>4</v>
       </c>
       <c r="E304" t="inlineStr">
         <is>
@@ -7948,7 +7948,7 @@
     <row r="305">
       <c r="A305" t="inlineStr">
         <is>
-          <t>16:57:49</t>
+          <t>17:47:19</t>
         </is>
       </c>
       <c r="B305" t="inlineStr">
@@ -7958,11 +7958,11 @@
       </c>
       <c r="C305" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D305" t="n">
-        <v>62</v>
+        <v>12</v>
       </c>
       <c r="E305" t="inlineStr">
         <is>
@@ -7973,7 +7973,7 @@
     <row r="306">
       <c r="A306" t="inlineStr">
         <is>
-          <t>17:21:09</t>
+          <t>16:57:49</t>
         </is>
       </c>
       <c r="B306" t="inlineStr">
@@ -7983,11 +7983,11 @@
       </c>
       <c r="C306" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D306" t="n">
-        <v>38</v>
+        <v>62</v>
       </c>
       <c r="E306" t="inlineStr">
         <is>
@@ -7998,7 +7998,7 @@
     <row r="307">
       <c r="A307" t="inlineStr">
         <is>
-          <t>17:21:09</t>
+          <t>17:47:19</t>
         </is>
       </c>
       <c r="B307" t="inlineStr">
@@ -8008,11 +8008,11 @@
       </c>
       <c r="C307" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D307" t="n">
-        <v>39</v>
+        <v>13</v>
       </c>
       <c r="E307" t="inlineStr">
         <is>
@@ -8023,21 +8023,21 @@
     <row r="308">
       <c r="A308" t="inlineStr">
         <is>
-          <t>17:21:09</t>
+          <t>17:47:19</t>
         </is>
       </c>
       <c r="B308" t="inlineStr">
         <is>
-          <t>18:01</t>
+          <t>18:00</t>
         </is>
       </c>
       <c r="C308" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D308" t="n">
-        <v>40</v>
+        <v>13</v>
       </c>
       <c r="E308" t="inlineStr">
         <is>
@@ -8048,21 +8048,21 @@
     <row r="309">
       <c r="A309" t="inlineStr">
         <is>
-          <t>16:57:49</t>
+          <t>17:47:19</t>
         </is>
       </c>
       <c r="B309" t="inlineStr">
         <is>
-          <t>18:11</t>
+          <t>18:01</t>
         </is>
       </c>
       <c r="C309" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D309" t="n">
-        <v>74</v>
+        <v>14</v>
       </c>
       <c r="E309" t="inlineStr">
         <is>
@@ -8073,12 +8073,12 @@
     <row r="310">
       <c r="A310" t="inlineStr">
         <is>
-          <t>17:21:09</t>
+          <t>17:47:19</t>
         </is>
       </c>
       <c r="B310" t="inlineStr">
         <is>
-          <t>18:12</t>
+          <t>18:11</t>
         </is>
       </c>
       <c r="C310" t="inlineStr">
@@ -8087,7 +8087,7 @@
         </is>
       </c>
       <c r="D310" t="n">
-        <v>51</v>
+        <v>24</v>
       </c>
       <c r="E310" t="inlineStr">
         <is>
@@ -8098,7 +8098,7 @@
     <row r="311">
       <c r="A311" t="inlineStr">
         <is>
-          <t>16:57:49</t>
+          <t>17:47:19</t>
         </is>
       </c>
       <c r="B311" t="inlineStr">
@@ -8112,7 +8112,7 @@
         </is>
       </c>
       <c r="D311" t="n">
-        <v>75</v>
+        <v>25</v>
       </c>
       <c r="E311" t="inlineStr">
         <is>
@@ -8128,16 +8128,16 @@
       </c>
       <c r="B312" t="inlineStr">
         <is>
-          <t>18:14</t>
+          <t>18:12</t>
         </is>
       </c>
       <c r="C312" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D312" t="n">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="E312" t="inlineStr">
         <is>
@@ -8153,16 +8153,16 @@
       </c>
       <c r="B313" t="inlineStr">
         <is>
-          <t>18:23</t>
+          <t>18:14</t>
         </is>
       </c>
       <c r="C313" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D313" t="n">
-        <v>62</v>
+        <v>53</v>
       </c>
       <c r="E313" t="inlineStr">
         <is>
@@ -8173,21 +8173,21 @@
     <row r="314">
       <c r="A314" t="inlineStr">
         <is>
-          <t>17:21:09</t>
+          <t>17:47:19</t>
         </is>
       </c>
       <c r="B314" t="inlineStr">
         <is>
-          <t>18:24</t>
+          <t>18:23</t>
         </is>
       </c>
       <c r="C314" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D314" t="n">
-        <v>63</v>
+        <v>36</v>
       </c>
       <c r="E314" t="inlineStr">
         <is>
@@ -8198,21 +8198,21 @@
     <row r="315">
       <c r="A315" t="inlineStr">
         <is>
-          <t>17:21:09</t>
+          <t>17:47:19</t>
         </is>
       </c>
       <c r="B315" t="inlineStr">
         <is>
-          <t>18:34</t>
+          <t>18:24</t>
         </is>
       </c>
       <c r="C315" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D315" t="n">
-        <v>73</v>
+        <v>37</v>
       </c>
       <c r="E315" t="inlineStr">
         <is>
@@ -8223,21 +8223,21 @@
     <row r="316">
       <c r="A316" t="inlineStr">
         <is>
-          <t>17:21:09</t>
+          <t>17:47:19</t>
         </is>
       </c>
       <c r="B316" t="inlineStr">
         <is>
-          <t>18:35</t>
+          <t>18:30</t>
         </is>
       </c>
       <c r="C316" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D316" t="n">
-        <v>74</v>
+        <v>43</v>
       </c>
       <c r="E316" t="inlineStr">
         <is>
@@ -8248,21 +8248,21 @@
     <row r="317">
       <c r="A317" t="inlineStr">
         <is>
-          <t>16:57:49</t>
+          <t>17:21:09</t>
         </is>
       </c>
       <c r="B317" t="inlineStr">
         <is>
-          <t>18:38</t>
+          <t>18:34</t>
         </is>
       </c>
       <c r="C317" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D317" t="n">
-        <v>101</v>
+        <v>73</v>
       </c>
       <c r="E317" t="inlineStr">
         <is>
@@ -8273,21 +8273,21 @@
     <row r="318">
       <c r="A318" t="inlineStr">
         <is>
-          <t>17:21:09</t>
+          <t>17:47:19</t>
         </is>
       </c>
       <c r="B318" t="inlineStr">
         <is>
-          <t>18:39</t>
+          <t>18:35</t>
         </is>
       </c>
       <c r="C318" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D318" t="n">
-        <v>78</v>
+        <v>48</v>
       </c>
       <c r="E318" t="inlineStr">
         <is>
@@ -8298,21 +8298,21 @@
     <row r="319">
       <c r="A319" t="inlineStr">
         <is>
-          <t>17:21:09</t>
+          <t>17:47:19</t>
         </is>
       </c>
       <c r="B319" t="inlineStr">
         <is>
-          <t>18:51</t>
+          <t>18:38</t>
         </is>
       </c>
       <c r="C319" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D319" t="n">
-        <v>90</v>
+        <v>51</v>
       </c>
       <c r="E319" t="inlineStr">
         <is>
@@ -8323,21 +8323,21 @@
     <row r="320">
       <c r="A320" t="inlineStr">
         <is>
-          <t>16:57:49</t>
+          <t>17:21:09</t>
         </is>
       </c>
       <c r="B320" t="inlineStr">
         <is>
-          <t>18:52</t>
+          <t>18:39</t>
         </is>
       </c>
       <c r="C320" t="inlineStr">
         <is>
-          <t>14X44_ABASTO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D320" t="n">
-        <v>115</v>
+        <v>78</v>
       </c>
       <c r="E320" t="inlineStr">
         <is>
@@ -8348,21 +8348,21 @@
     <row r="321">
       <c r="A321" t="inlineStr">
         <is>
-          <t>17:21:09</t>
+          <t>17:47:19</t>
         </is>
       </c>
       <c r="B321" t="inlineStr">
         <is>
-          <t>18:53</t>
+          <t>18:41</t>
         </is>
       </c>
       <c r="C321" t="inlineStr">
         <is>
-          <t>14X44_ABASTO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D321" t="n">
-        <v>92</v>
+        <v>54</v>
       </c>
       <c r="E321" t="inlineStr">
         <is>
@@ -8373,21 +8373,21 @@
     <row r="322">
       <c r="A322" t="inlineStr">
         <is>
-          <t>17:21:09</t>
+          <t>17:47:19</t>
         </is>
       </c>
       <c r="B322" t="inlineStr">
         <is>
-          <t>19:00</t>
+          <t>18:51</t>
         </is>
       </c>
       <c r="C322" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D322" t="n">
-        <v>99</v>
+        <v>64</v>
       </c>
       <c r="E322" t="inlineStr">
         <is>
@@ -8398,21 +8398,21 @@
     <row r="323">
       <c r="A323" t="inlineStr">
         <is>
-          <t>17:21:09</t>
+          <t>16:57:49</t>
         </is>
       </c>
       <c r="B323" t="inlineStr">
         <is>
-          <t>19:09</t>
+          <t>18:52</t>
         </is>
       </c>
       <c r="C323" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>14X44_ABASTO</t>
         </is>
       </c>
       <c r="D323" t="n">
-        <v>108</v>
+        <v>115</v>
       </c>
       <c r="E323" t="inlineStr">
         <is>
@@ -8423,21 +8423,21 @@
     <row r="324">
       <c r="A324" t="inlineStr">
         <is>
-          <t>17:21:09</t>
+          <t>17:47:19</t>
         </is>
       </c>
       <c r="B324" t="inlineStr">
         <is>
-          <t>19:12</t>
+          <t>18:53</t>
         </is>
       </c>
       <c r="C324" t="inlineStr">
         <is>
-          <t>81_EL PELIGRO</t>
+          <t>14X44_ABASTO</t>
         </is>
       </c>
       <c r="D324" t="n">
-        <v>111</v>
+        <v>66</v>
       </c>
       <c r="E324" t="inlineStr">
         <is>
@@ -8448,23 +8448,248 @@
     <row r="325">
       <c r="A325" t="inlineStr">
         <is>
+          <t>17:47:19</t>
+        </is>
+      </c>
+      <c r="B325" t="inlineStr">
+        <is>
+          <t>19:00</t>
+        </is>
+      </c>
+      <c r="C325" t="inlineStr">
+        <is>
+          <t>17_ROMERO</t>
+        </is>
+      </c>
+      <c r="D325" t="n">
+        <v>73</v>
+      </c>
+      <c r="E325" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="326">
+      <c r="A326" t="inlineStr">
+        <is>
+          <t>17:47:19</t>
+        </is>
+      </c>
+      <c r="B326" t="inlineStr">
+        <is>
+          <t>19:08</t>
+        </is>
+      </c>
+      <c r="C326" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D326" t="n">
+        <v>81</v>
+      </c>
+      <c r="E326" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="327">
+      <c r="A327" t="inlineStr">
+        <is>
           <t>17:21:09</t>
         </is>
       </c>
-      <c r="B325" t="inlineStr">
+      <c r="B327" t="inlineStr">
+        <is>
+          <t>19:09</t>
+        </is>
+      </c>
+      <c r="C327" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D327" t="n">
+        <v>108</v>
+      </c>
+      <c r="E327" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="328">
+      <c r="A328" t="inlineStr">
+        <is>
+          <t>17:47:19</t>
+        </is>
+      </c>
+      <c r="B328" t="inlineStr">
+        <is>
+          <t>19:12</t>
+        </is>
+      </c>
+      <c r="C328" t="inlineStr">
+        <is>
+          <t>81_EL PELIGRO</t>
+        </is>
+      </c>
+      <c r="D328" t="n">
+        <v>85</v>
+      </c>
+      <c r="E328" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="329">
+      <c r="A329" t="inlineStr">
+        <is>
+          <t>17:21:09</t>
+        </is>
+      </c>
+      <c r="B329" t="inlineStr">
         <is>
           <t>19:17</t>
         </is>
       </c>
-      <c r="C325" t="inlineStr">
+      <c r="C329" t="inlineStr">
         <is>
           <t>27_EL RETIRO</t>
         </is>
       </c>
-      <c r="D325" t="n">
+      <c r="D329" t="n">
         <v>116</v>
       </c>
-      <c r="E325" t="inlineStr">
+      <c r="E329" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="330">
+      <c r="A330" t="inlineStr">
+        <is>
+          <t>17:47:19</t>
+        </is>
+      </c>
+      <c r="B330" t="inlineStr">
+        <is>
+          <t>19:20</t>
+        </is>
+      </c>
+      <c r="C330" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D330" t="n">
+        <v>93</v>
+      </c>
+      <c r="E330" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="331">
+      <c r="A331" t="inlineStr">
+        <is>
+          <t>17:47:19</t>
+        </is>
+      </c>
+      <c r="B331" t="inlineStr">
+        <is>
+          <t>19:23</t>
+        </is>
+      </c>
+      <c r="C331" t="inlineStr">
+        <is>
+          <t>225_GOMEZ</t>
+        </is>
+      </c>
+      <c r="D331" t="n">
+        <v>96</v>
+      </c>
+      <c r="E331" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="332">
+      <c r="A332" t="inlineStr">
+        <is>
+          <t>17:47:19</t>
+        </is>
+      </c>
+      <c r="B332" t="inlineStr">
+        <is>
+          <t>19:24</t>
+        </is>
+      </c>
+      <c r="C332" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D332" t="n">
+        <v>97</v>
+      </c>
+      <c r="E332" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="333">
+      <c r="A333" t="inlineStr">
+        <is>
+          <t>17:47:19</t>
+        </is>
+      </c>
+      <c r="B333" t="inlineStr">
+        <is>
+          <t>19:36</t>
+        </is>
+      </c>
+      <c r="C333" t="inlineStr">
+        <is>
+          <t>215_EL PELIGRO</t>
+        </is>
+      </c>
+      <c r="D333" t="n">
+        <v>109</v>
+      </c>
+      <c r="E333" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="334">
+      <c r="A334" t="inlineStr">
+        <is>
+          <t>17:47:19</t>
+        </is>
+      </c>
+      <c r="B334" t="inlineStr">
+        <is>
+          <t>19:40</t>
+        </is>
+      </c>
+      <c r="C334" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D334" t="n">
+        <v>113</v>
+      </c>
+      <c r="E334" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -8481,7 +8706,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E53"/>
+  <dimension ref="A1:E55"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -8494,14 +8719,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 17:21:09</t>
+          <t>Última actualización: 17:47:20</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 48</t>
+          <t>Total filas: 50</t>
         </is>
       </c>
     </row>
@@ -9635,7 +9860,7 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>16:57:49</t>
+          <t>17:47:19</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
@@ -9649,7 +9874,7 @@
         </is>
       </c>
       <c r="D50" t="n">
-        <v>50</v>
+        <v>0</v>
       </c>
       <c r="E50" t="inlineStr">
         <is>
@@ -9660,7 +9885,7 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>16:57:49</t>
+          <t>17:47:19</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
@@ -9674,7 +9899,7 @@
         </is>
       </c>
       <c r="D51" t="n">
-        <v>50</v>
+        <v>0</v>
       </c>
       <c r="E51" t="inlineStr">
         <is>
@@ -9727,6 +9952,56 @@
         <v>27</v>
       </c>
       <c r="E53" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>17:47:19</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>19:24</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D54" t="n">
+        <v>97</v>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>17:47:19</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>19:36</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>215_EL PELIGRO</t>
+        </is>
+      </c>
+      <c r="D55" t="n">
+        <v>109</v>
+      </c>
+      <c r="E55" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -9756,7 +10031,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 17:21:09</t>
+          <t>Última actualización: 17:47:20</t>
         </is>
       </c>
     </row>
@@ -11072,7 +11347,7 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>17:21:09</t>
+          <t>17:47:19</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
@@ -11086,7 +11361,7 @@
         </is>
       </c>
       <c r="D57" t="n">
-        <v>65</v>
+        <v>39</v>
       </c>
       <c r="E57" t="inlineStr">
         <is>
@@ -11097,7 +11372,7 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>17:21:09</t>
+          <t>17:47:19</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
@@ -11111,7 +11386,7 @@
         </is>
       </c>
       <c r="D58" t="n">
-        <v>117</v>
+        <v>91</v>
       </c>
       <c r="E58" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 1821
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-03-21.xlsx
+++ b/data/horarios-141-2026-03-21.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E334"/>
+  <dimension ref="A1:E340"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 17:47:20</t>
+          <t>Última actualización: 18:01:08</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 329</t>
+          <t>Total filas: 335</t>
         </is>
       </c>
     </row>
@@ -1158,7 +1158,7 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D33" t="n">
@@ -1183,7 +1183,7 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D34" t="n">
@@ -1558,7 +1558,7 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D49" t="n">
@@ -1583,7 +1583,7 @@
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D50" t="n">
@@ -1873,7 +1873,7 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>06:59:30</t>
+          <t>08:14:14</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
@@ -1883,11 +1883,11 @@
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D62" t="n">
-        <v>75</v>
+        <v>0</v>
       </c>
       <c r="E62" t="inlineStr">
         <is>
@@ -1908,7 +1908,7 @@
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D63" t="n">
@@ -1923,7 +1923,7 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>08:14:14</t>
+          <t>06:59:30</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
@@ -1933,11 +1933,11 @@
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D64" t="n">
-        <v>0</v>
+        <v>75</v>
       </c>
       <c r="E64" t="inlineStr">
         <is>
@@ -1983,7 +1983,7 @@
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D66" t="n">
@@ -2033,7 +2033,7 @@
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D68" t="n">
@@ -2233,7 +2233,7 @@
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D76" t="n">
@@ -2258,7 +2258,7 @@
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D77" t="n">
@@ -2708,7 +2708,7 @@
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215_EL PELIGRO</t>
         </is>
       </c>
       <c r="D95" t="n">
@@ -2733,7 +2733,7 @@
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>215_EL PELIGRO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D96" t="n">
@@ -2873,7 +2873,7 @@
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>08:36:09</t>
+          <t>07:51:37</t>
         </is>
       </c>
       <c r="B102" t="inlineStr">
@@ -2883,11 +2883,11 @@
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D102" t="n">
-        <v>53</v>
+        <v>98</v>
       </c>
       <c r="E102" t="inlineStr">
         <is>
@@ -2898,7 +2898,7 @@
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>07:51:37</t>
+          <t>08:36:09</t>
         </is>
       </c>
       <c r="B103" t="inlineStr">
@@ -2908,11 +2908,11 @@
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D103" t="n">
-        <v>98</v>
+        <v>53</v>
       </c>
       <c r="E103" t="inlineStr">
         <is>
@@ -3083,7 +3083,7 @@
       </c>
       <c r="C110" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D110" t="n">
@@ -3108,7 +3108,7 @@
       </c>
       <c r="C111" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D111" t="n">
@@ -3173,7 +3173,7 @@
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>08:50:55</t>
+          <t>09:23:24</t>
         </is>
       </c>
       <c r="B114" t="inlineStr">
@@ -3183,11 +3183,11 @@
       </c>
       <c r="C114" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D114" t="n">
-        <v>73</v>
+        <v>40</v>
       </c>
       <c r="E114" t="inlineStr">
         <is>
@@ -3198,7 +3198,7 @@
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>09:23:24</t>
+          <t>08:50:55</t>
         </is>
       </c>
       <c r="B115" t="inlineStr">
@@ -3208,11 +3208,11 @@
       </c>
       <c r="C115" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D115" t="n">
-        <v>40</v>
+        <v>73</v>
       </c>
       <c r="E115" t="inlineStr">
         <is>
@@ -3598,7 +3598,7 @@
     <row r="131">
       <c r="A131" t="inlineStr">
         <is>
-          <t>09:23:24</t>
+          <t>10:14:52</t>
         </is>
       </c>
       <c r="B131" t="inlineStr">
@@ -3608,11 +3608,11 @@
       </c>
       <c r="C131" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D131" t="n">
-        <v>80</v>
+        <v>29</v>
       </c>
       <c r="E131" t="inlineStr">
         <is>
@@ -3623,7 +3623,7 @@
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t>10:14:52</t>
+          <t>09:23:24</t>
         </is>
       </c>
       <c r="B132" t="inlineStr">
@@ -3633,11 +3633,11 @@
       </c>
       <c r="C132" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D132" t="n">
-        <v>29</v>
+        <v>80</v>
       </c>
       <c r="E132" t="inlineStr">
         <is>
@@ -3873,7 +3873,7 @@
     <row r="142">
       <c r="A142" t="inlineStr">
         <is>
-          <t>10:14:52</t>
+          <t>10:52:37</t>
         </is>
       </c>
       <c r="B142" t="inlineStr">
@@ -3883,11 +3883,11 @@
       </c>
       <c r="C142" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D142" t="n">
-        <v>49</v>
+        <v>11</v>
       </c>
       <c r="E142" t="inlineStr">
         <is>
@@ -3898,7 +3898,7 @@
     <row r="143">
       <c r="A143" t="inlineStr">
         <is>
-          <t>10:52:37</t>
+          <t>10:14:52</t>
         </is>
       </c>
       <c r="B143" t="inlineStr">
@@ -3908,11 +3908,11 @@
       </c>
       <c r="C143" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D143" t="n">
-        <v>11</v>
+        <v>49</v>
       </c>
       <c r="E143" t="inlineStr">
         <is>
@@ -4183,7 +4183,7 @@
       </c>
       <c r="C154" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D154" t="n">
@@ -4208,7 +4208,7 @@
       </c>
       <c r="C155" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D155" t="n">
@@ -4998,7 +4998,7 @@
     <row r="187">
       <c r="A187" t="inlineStr">
         <is>
-          <t>13:00:14</t>
+          <t>12:28:38</t>
         </is>
       </c>
       <c r="B187" t="inlineStr">
@@ -5008,11 +5008,11 @@
       </c>
       <c r="C187" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D187" t="n">
-        <v>3</v>
+        <v>35</v>
       </c>
       <c r="E187" t="inlineStr">
         <is>
@@ -5023,7 +5023,7 @@
     <row r="188">
       <c r="A188" t="inlineStr">
         <is>
-          <t>12:28:38</t>
+          <t>13:00:14</t>
         </is>
       </c>
       <c r="B188" t="inlineStr">
@@ -5033,11 +5033,11 @@
       </c>
       <c r="C188" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D188" t="n">
-        <v>35</v>
+        <v>3</v>
       </c>
       <c r="E188" t="inlineStr">
         <is>
@@ -5073,7 +5073,7 @@
     <row r="190">
       <c r="A190" t="inlineStr">
         <is>
-          <t>13:00:14</t>
+          <t>12:48:06</t>
         </is>
       </c>
       <c r="B190" t="inlineStr">
@@ -5083,11 +5083,11 @@
       </c>
       <c r="C190" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D190" t="n">
-        <v>4</v>
+        <v>16</v>
       </c>
       <c r="E190" t="inlineStr">
         <is>
@@ -5098,7 +5098,7 @@
     <row r="191">
       <c r="A191" t="inlineStr">
         <is>
-          <t>12:48:06</t>
+          <t>13:00:14</t>
         </is>
       </c>
       <c r="B191" t="inlineStr">
@@ -5108,11 +5108,11 @@
       </c>
       <c r="C191" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D191" t="n">
-        <v>16</v>
+        <v>4</v>
       </c>
       <c r="E191" t="inlineStr">
         <is>
@@ -5248,7 +5248,7 @@
     <row r="197">
       <c r="A197" t="inlineStr">
         <is>
-          <t>12:48:06</t>
+          <t>13:00:14</t>
         </is>
       </c>
       <c r="B197" t="inlineStr">
@@ -5258,11 +5258,11 @@
       </c>
       <c r="C197" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D197" t="n">
-        <v>45</v>
+        <v>33</v>
       </c>
       <c r="E197" t="inlineStr">
         <is>
@@ -5273,7 +5273,7 @@
     <row r="198">
       <c r="A198" t="inlineStr">
         <is>
-          <t>13:00:14</t>
+          <t>12:48:06</t>
         </is>
       </c>
       <c r="B198" t="inlineStr">
@@ -5283,11 +5283,11 @@
       </c>
       <c r="C198" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D198" t="n">
-        <v>33</v>
+        <v>45</v>
       </c>
       <c r="E198" t="inlineStr">
         <is>
@@ -5573,7 +5573,7 @@
     <row r="210">
       <c r="A210" t="inlineStr">
         <is>
-          <t>13:57:43</t>
+          <t>13:00:14</t>
         </is>
       </c>
       <c r="B210" t="inlineStr">
@@ -5583,11 +5583,11 @@
       </c>
       <c r="C210" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D210" t="n">
-        <v>6</v>
+        <v>63</v>
       </c>
       <c r="E210" t="inlineStr">
         <is>
@@ -5598,7 +5598,7 @@
     <row r="211">
       <c r="A211" t="inlineStr">
         <is>
-          <t>13:00:14</t>
+          <t>13:57:43</t>
         </is>
       </c>
       <c r="B211" t="inlineStr">
@@ -5608,11 +5608,11 @@
       </c>
       <c r="C211" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D211" t="n">
-        <v>63</v>
+        <v>6</v>
       </c>
       <c r="E211" t="inlineStr">
         <is>
@@ -5623,7 +5623,7 @@
     <row r="212">
       <c r="A212" t="inlineStr">
         <is>
-          <t>13:32:57</t>
+          <t>13:57:43</t>
         </is>
       </c>
       <c r="B212" t="inlineStr">
@@ -5633,11 +5633,11 @@
       </c>
       <c r="C212" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D212" t="n">
-        <v>44</v>
+        <v>19</v>
       </c>
       <c r="E212" t="inlineStr">
         <is>
@@ -5648,7 +5648,7 @@
     <row r="213">
       <c r="A213" t="inlineStr">
         <is>
-          <t>13:57:43</t>
+          <t>13:32:57</t>
         </is>
       </c>
       <c r="B213" t="inlineStr">
@@ -5658,11 +5658,11 @@
       </c>
       <c r="C213" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D213" t="n">
-        <v>19</v>
+        <v>44</v>
       </c>
       <c r="E213" t="inlineStr">
         <is>
@@ -5873,7 +5873,7 @@
     <row r="222">
       <c r="A222" t="inlineStr">
         <is>
-          <t>14:21:42</t>
+          <t>13:00:14</t>
         </is>
       </c>
       <c r="B222" t="inlineStr">
@@ -5883,11 +5883,11 @@
       </c>
       <c r="C222" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D222" t="n">
-        <v>12</v>
+        <v>93</v>
       </c>
       <c r="E222" t="inlineStr">
         <is>
@@ -5898,7 +5898,7 @@
     <row r="223">
       <c r="A223" t="inlineStr">
         <is>
-          <t>13:00:14</t>
+          <t>14:21:42</t>
         </is>
       </c>
       <c r="B223" t="inlineStr">
@@ -5908,11 +5908,11 @@
       </c>
       <c r="C223" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D223" t="n">
-        <v>93</v>
+        <v>12</v>
       </c>
       <c r="E223" t="inlineStr">
         <is>
@@ -5983,7 +5983,7 @@
       </c>
       <c r="C226" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D226" t="n">
@@ -6008,7 +6008,7 @@
       </c>
       <c r="C227" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D227" t="n">
@@ -6173,7 +6173,7 @@
     <row r="234">
       <c r="A234" t="inlineStr">
         <is>
-          <t>14:59:00</t>
+          <t>14:46:39</t>
         </is>
       </c>
       <c r="B234" t="inlineStr">
@@ -6183,11 +6183,11 @@
       </c>
       <c r="C234" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D234" t="n">
-        <v>2</v>
+        <v>15</v>
       </c>
       <c r="E234" t="inlineStr">
         <is>
@@ -6198,7 +6198,7 @@
     <row r="235">
       <c r="A235" t="inlineStr">
         <is>
-          <t>14:46:39</t>
+          <t>14:59:00</t>
         </is>
       </c>
       <c r="B235" t="inlineStr">
@@ -6208,11 +6208,11 @@
       </c>
       <c r="C235" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D235" t="n">
-        <v>15</v>
+        <v>2</v>
       </c>
       <c r="E235" t="inlineStr">
         <is>
@@ -7033,7 +7033,7 @@
       </c>
       <c r="C268" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D268" t="n">
@@ -7058,7 +7058,7 @@
       </c>
       <c r="C269" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D269" t="n">
@@ -7073,7 +7073,7 @@
     <row r="270">
       <c r="A270" t="inlineStr">
         <is>
-          <t>16:33:34</t>
+          <t>16:01:44</t>
         </is>
       </c>
       <c r="B270" t="inlineStr">
@@ -7083,11 +7083,11 @@
       </c>
       <c r="C270" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D270" t="n">
-        <v>2</v>
+        <v>34</v>
       </c>
       <c r="E270" t="inlineStr">
         <is>
@@ -7098,7 +7098,7 @@
     <row r="271">
       <c r="A271" t="inlineStr">
         <is>
-          <t>16:01:44</t>
+          <t>16:33:34</t>
         </is>
       </c>
       <c r="B271" t="inlineStr">
@@ -7108,11 +7108,11 @@
       </c>
       <c r="C271" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D271" t="n">
-        <v>34</v>
+        <v>2</v>
       </c>
       <c r="E271" t="inlineStr">
         <is>
@@ -7383,7 +7383,7 @@
       </c>
       <c r="C282" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D282" t="n">
@@ -7408,7 +7408,7 @@
       </c>
       <c r="C283" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D283" t="n">
@@ -7648,7 +7648,7 @@
     <row r="293">
       <c r="A293" t="inlineStr">
         <is>
-          <t>17:21:09</t>
+          <t>16:33:34</t>
         </is>
       </c>
       <c r="B293" t="inlineStr">
@@ -7658,11 +7658,11 @@
       </c>
       <c r="C293" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D293" t="n">
-        <v>14</v>
+        <v>62</v>
       </c>
       <c r="E293" t="inlineStr">
         <is>
@@ -7673,7 +7673,7 @@
     <row r="294">
       <c r="A294" t="inlineStr">
         <is>
-          <t>16:33:34</t>
+          <t>17:21:09</t>
         </is>
       </c>
       <c r="B294" t="inlineStr">
@@ -7683,11 +7683,11 @@
       </c>
       <c r="C294" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D294" t="n">
-        <v>62</v>
+        <v>14</v>
       </c>
       <c r="E294" t="inlineStr">
         <is>
@@ -7883,7 +7883,7 @@
       </c>
       <c r="C302" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>215_EL PELIGRO</t>
         </is>
       </c>
       <c r="D302" t="n">
@@ -7908,7 +7908,7 @@
       </c>
       <c r="C303" t="inlineStr">
         <is>
-          <t>215_EL PELIGRO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D303" t="n">
@@ -8008,7 +8008,7 @@
       </c>
       <c r="C307" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D307" t="n">
@@ -8033,7 +8033,7 @@
       </c>
       <c r="C308" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D308" t="n">
@@ -8048,7 +8048,7 @@
     <row r="309">
       <c r="A309" t="inlineStr">
         <is>
-          <t>17:47:19</t>
+          <t>18:01:08</t>
         </is>
       </c>
       <c r="B309" t="inlineStr">
@@ -8058,11 +8058,11 @@
       </c>
       <c r="C309" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D309" t="n">
-        <v>14</v>
+        <v>0</v>
       </c>
       <c r="E309" t="inlineStr">
         <is>
@@ -8073,21 +8073,21 @@
     <row r="310">
       <c r="A310" t="inlineStr">
         <is>
-          <t>17:47:19</t>
+          <t>18:01:08</t>
         </is>
       </c>
       <c r="B310" t="inlineStr">
         <is>
-          <t>18:11</t>
+          <t>18:01</t>
         </is>
       </c>
       <c r="C310" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D310" t="n">
-        <v>24</v>
+        <v>0</v>
       </c>
       <c r="E310" t="inlineStr">
         <is>
@@ -8098,21 +8098,21 @@
     <row r="311">
       <c r="A311" t="inlineStr">
         <is>
-          <t>17:47:19</t>
+          <t>18:01:08</t>
         </is>
       </c>
       <c r="B311" t="inlineStr">
         <is>
-          <t>18:12</t>
+          <t>18:01</t>
         </is>
       </c>
       <c r="C311" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D311" t="n">
-        <v>25</v>
+        <v>0</v>
       </c>
       <c r="E311" t="inlineStr">
         <is>
@@ -8123,12 +8123,12 @@
     <row r="312">
       <c r="A312" t="inlineStr">
         <is>
-          <t>17:21:09</t>
+          <t>17:47:19</t>
         </is>
       </c>
       <c r="B312" t="inlineStr">
         <is>
-          <t>18:12</t>
+          <t>18:11</t>
         </is>
       </c>
       <c r="C312" t="inlineStr">
@@ -8137,7 +8137,7 @@
         </is>
       </c>
       <c r="D312" t="n">
-        <v>51</v>
+        <v>24</v>
       </c>
       <c r="E312" t="inlineStr">
         <is>
@@ -8148,21 +8148,21 @@
     <row r="313">
       <c r="A313" t="inlineStr">
         <is>
-          <t>17:21:09</t>
+          <t>18:01:08</t>
         </is>
       </c>
       <c r="B313" t="inlineStr">
         <is>
-          <t>18:14</t>
+          <t>18:12</t>
         </is>
       </c>
       <c r="C313" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D313" t="n">
-        <v>53</v>
+        <v>11</v>
       </c>
       <c r="E313" t="inlineStr">
         <is>
@@ -8173,21 +8173,21 @@
     <row r="314">
       <c r="A314" t="inlineStr">
         <is>
-          <t>17:47:19</t>
+          <t>18:01:08</t>
         </is>
       </c>
       <c r="B314" t="inlineStr">
         <is>
-          <t>18:23</t>
+          <t>18:12</t>
         </is>
       </c>
       <c r="C314" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D314" t="n">
-        <v>36</v>
+        <v>11</v>
       </c>
       <c r="E314" t="inlineStr">
         <is>
@@ -8198,12 +8198,12 @@
     <row r="315">
       <c r="A315" t="inlineStr">
         <is>
-          <t>17:47:19</t>
+          <t>17:21:09</t>
         </is>
       </c>
       <c r="B315" t="inlineStr">
         <is>
-          <t>18:24</t>
+          <t>18:14</t>
         </is>
       </c>
       <c r="C315" t="inlineStr">
@@ -8212,7 +8212,7 @@
         </is>
       </c>
       <c r="D315" t="n">
-        <v>37</v>
+        <v>53</v>
       </c>
       <c r="E315" t="inlineStr">
         <is>
@@ -8223,21 +8223,21 @@
     <row r="316">
       <c r="A316" t="inlineStr">
         <is>
-          <t>17:47:19</t>
+          <t>18:01:08</t>
         </is>
       </c>
       <c r="B316" t="inlineStr">
         <is>
-          <t>18:30</t>
+          <t>18:23</t>
         </is>
       </c>
       <c r="C316" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D316" t="n">
-        <v>43</v>
+        <v>22</v>
       </c>
       <c r="E316" t="inlineStr">
         <is>
@@ -8248,21 +8248,21 @@
     <row r="317">
       <c r="A317" t="inlineStr">
         <is>
-          <t>17:21:09</t>
+          <t>18:01:08</t>
         </is>
       </c>
       <c r="B317" t="inlineStr">
         <is>
-          <t>18:34</t>
+          <t>18:24</t>
         </is>
       </c>
       <c r="C317" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D317" t="n">
-        <v>73</v>
+        <v>23</v>
       </c>
       <c r="E317" t="inlineStr">
         <is>
@@ -8278,16 +8278,16 @@
       </c>
       <c r="B318" t="inlineStr">
         <is>
-          <t>18:35</t>
+          <t>18:30</t>
         </is>
       </c>
       <c r="C318" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D318" t="n">
-        <v>48</v>
+        <v>43</v>
       </c>
       <c r="E318" t="inlineStr">
         <is>
@@ -8298,21 +8298,21 @@
     <row r="319">
       <c r="A319" t="inlineStr">
         <is>
-          <t>17:47:19</t>
+          <t>18:01:08</t>
         </is>
       </c>
       <c r="B319" t="inlineStr">
         <is>
-          <t>18:38</t>
+          <t>18:33</t>
         </is>
       </c>
       <c r="C319" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D319" t="n">
-        <v>51</v>
+        <v>32</v>
       </c>
       <c r="E319" t="inlineStr">
         <is>
@@ -8328,16 +8328,16 @@
       </c>
       <c r="B320" t="inlineStr">
         <is>
-          <t>18:39</t>
+          <t>18:34</t>
         </is>
       </c>
       <c r="C320" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D320" t="n">
-        <v>78</v>
+        <v>73</v>
       </c>
       <c r="E320" t="inlineStr">
         <is>
@@ -8348,21 +8348,21 @@
     <row r="321">
       <c r="A321" t="inlineStr">
         <is>
-          <t>17:47:19</t>
+          <t>18:01:08</t>
         </is>
       </c>
       <c r="B321" t="inlineStr">
         <is>
-          <t>18:41</t>
+          <t>18:35</t>
         </is>
       </c>
       <c r="C321" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D321" t="n">
-        <v>54</v>
+        <v>34</v>
       </c>
       <c r="E321" t="inlineStr">
         <is>
@@ -8378,16 +8378,16 @@
       </c>
       <c r="B322" t="inlineStr">
         <is>
-          <t>18:51</t>
+          <t>18:38</t>
         </is>
       </c>
       <c r="C322" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D322" t="n">
-        <v>64</v>
+        <v>51</v>
       </c>
       <c r="E322" t="inlineStr">
         <is>
@@ -8398,21 +8398,21 @@
     <row r="323">
       <c r="A323" t="inlineStr">
         <is>
-          <t>16:57:49</t>
+          <t>18:01:08</t>
         </is>
       </c>
       <c r="B323" t="inlineStr">
         <is>
-          <t>18:52</t>
+          <t>18:39</t>
         </is>
       </c>
       <c r="C323" t="inlineStr">
         <is>
-          <t>14X44_ABASTO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D323" t="n">
-        <v>115</v>
+        <v>38</v>
       </c>
       <c r="E323" t="inlineStr">
         <is>
@@ -8423,21 +8423,21 @@
     <row r="324">
       <c r="A324" t="inlineStr">
         <is>
-          <t>17:47:19</t>
+          <t>18:01:08</t>
         </is>
       </c>
       <c r="B324" t="inlineStr">
         <is>
-          <t>18:53</t>
+          <t>18:41</t>
         </is>
       </c>
       <c r="C324" t="inlineStr">
         <is>
-          <t>14X44_ABASTO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D324" t="n">
-        <v>66</v>
+        <v>40</v>
       </c>
       <c r="E324" t="inlineStr">
         <is>
@@ -8448,21 +8448,21 @@
     <row r="325">
       <c r="A325" t="inlineStr">
         <is>
-          <t>17:47:19</t>
+          <t>18:01:08</t>
         </is>
       </c>
       <c r="B325" t="inlineStr">
         <is>
-          <t>19:00</t>
+          <t>18:51</t>
         </is>
       </c>
       <c r="C325" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D325" t="n">
-        <v>73</v>
+        <v>50</v>
       </c>
       <c r="E325" t="inlineStr">
         <is>
@@ -8473,21 +8473,21 @@
     <row r="326">
       <c r="A326" t="inlineStr">
         <is>
-          <t>17:47:19</t>
+          <t>16:57:49</t>
         </is>
       </c>
       <c r="B326" t="inlineStr">
         <is>
-          <t>19:08</t>
+          <t>18:52</t>
         </is>
       </c>
       <c r="C326" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>14X44_ABASTO</t>
         </is>
       </c>
       <c r="D326" t="n">
-        <v>81</v>
+        <v>115</v>
       </c>
       <c r="E326" t="inlineStr">
         <is>
@@ -8498,21 +8498,21 @@
     <row r="327">
       <c r="A327" t="inlineStr">
         <is>
-          <t>17:21:09</t>
+          <t>18:01:08</t>
         </is>
       </c>
       <c r="B327" t="inlineStr">
         <is>
-          <t>19:09</t>
+          <t>18:53</t>
         </is>
       </c>
       <c r="C327" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>14X44_ABASTO</t>
         </is>
       </c>
       <c r="D327" t="n">
-        <v>108</v>
+        <v>52</v>
       </c>
       <c r="E327" t="inlineStr">
         <is>
@@ -8523,21 +8523,21 @@
     <row r="328">
       <c r="A328" t="inlineStr">
         <is>
-          <t>17:47:19</t>
+          <t>18:01:08</t>
         </is>
       </c>
       <c r="B328" t="inlineStr">
         <is>
-          <t>19:12</t>
+          <t>19:00</t>
         </is>
       </c>
       <c r="C328" t="inlineStr">
         <is>
-          <t>81_EL PELIGRO</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D328" t="n">
-        <v>85</v>
+        <v>59</v>
       </c>
       <c r="E328" t="inlineStr">
         <is>
@@ -8548,21 +8548,21 @@
     <row r="329">
       <c r="A329" t="inlineStr">
         <is>
-          <t>17:21:09</t>
+          <t>17:47:19</t>
         </is>
       </c>
       <c r="B329" t="inlineStr">
         <is>
-          <t>19:17</t>
+          <t>19:08</t>
         </is>
       </c>
       <c r="C329" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D329" t="n">
-        <v>116</v>
+        <v>81</v>
       </c>
       <c r="E329" t="inlineStr">
         <is>
@@ -8573,21 +8573,21 @@
     <row r="330">
       <c r="A330" t="inlineStr">
         <is>
-          <t>17:47:19</t>
+          <t>18:01:08</t>
         </is>
       </c>
       <c r="B330" t="inlineStr">
         <is>
-          <t>19:20</t>
+          <t>19:09</t>
         </is>
       </c>
       <c r="C330" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D330" t="n">
-        <v>93</v>
+        <v>68</v>
       </c>
       <c r="E330" t="inlineStr">
         <is>
@@ -8598,21 +8598,21 @@
     <row r="331">
       <c r="A331" t="inlineStr">
         <is>
-          <t>17:47:19</t>
+          <t>18:01:08</t>
         </is>
       </c>
       <c r="B331" t="inlineStr">
         <is>
-          <t>19:23</t>
+          <t>19:12</t>
         </is>
       </c>
       <c r="C331" t="inlineStr">
         <is>
-          <t>225_GOMEZ</t>
+          <t>81_EL PELIGRO</t>
         </is>
       </c>
       <c r="D331" t="n">
-        <v>96</v>
+        <v>71</v>
       </c>
       <c r="E331" t="inlineStr">
         <is>
@@ -8623,21 +8623,21 @@
     <row r="332">
       <c r="A332" t="inlineStr">
         <is>
-          <t>17:47:19</t>
+          <t>18:01:08</t>
         </is>
       </c>
       <c r="B332" t="inlineStr">
         <is>
-          <t>19:24</t>
+          <t>19:17</t>
         </is>
       </c>
       <c r="C332" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D332" t="n">
-        <v>97</v>
+        <v>76</v>
       </c>
       <c r="E332" t="inlineStr">
         <is>
@@ -8653,16 +8653,16 @@
       </c>
       <c r="B333" t="inlineStr">
         <is>
-          <t>19:36</t>
+          <t>19:20</t>
         </is>
       </c>
       <c r="C333" t="inlineStr">
         <is>
-          <t>215_EL PELIGRO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D333" t="n">
-        <v>109</v>
+        <v>93</v>
       </c>
       <c r="E333" t="inlineStr">
         <is>
@@ -8673,23 +8673,173 @@
     <row r="334">
       <c r="A334" t="inlineStr">
         <is>
-          <t>17:47:19</t>
+          <t>18:01:08</t>
         </is>
       </c>
       <c r="B334" t="inlineStr">
         <is>
+          <t>19:23</t>
+        </is>
+      </c>
+      <c r="C334" t="inlineStr">
+        <is>
+          <t>225_GOMEZ</t>
+        </is>
+      </c>
+      <c r="D334" t="n">
+        <v>82</v>
+      </c>
+      <c r="E334" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="335">
+      <c r="A335" t="inlineStr">
+        <is>
+          <t>18:01:08</t>
+        </is>
+      </c>
+      <c r="B335" t="inlineStr">
+        <is>
+          <t>19:24</t>
+        </is>
+      </c>
+      <c r="C335" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D335" t="n">
+        <v>83</v>
+      </c>
+      <c r="E335" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="336">
+      <c r="A336" t="inlineStr">
+        <is>
+          <t>18:01:08</t>
+        </is>
+      </c>
+      <c r="B336" t="inlineStr">
+        <is>
+          <t>19:36</t>
+        </is>
+      </c>
+      <c r="C336" t="inlineStr">
+        <is>
+          <t>215_EL PELIGRO</t>
+        </is>
+      </c>
+      <c r="D336" t="n">
+        <v>95</v>
+      </c>
+      <c r="E336" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="337">
+      <c r="A337" t="inlineStr">
+        <is>
+          <t>18:01:08</t>
+        </is>
+      </c>
+      <c r="B337" t="inlineStr">
+        <is>
           <t>19:40</t>
         </is>
       </c>
-      <c r="C334" t="inlineStr">
+      <c r="C337" t="inlineStr">
         <is>
           <t>11_ETCHEVERRY</t>
         </is>
       </c>
-      <c r="D334" t="n">
-        <v>113</v>
-      </c>
-      <c r="E334" t="inlineStr">
+      <c r="D337" t="n">
+        <v>99</v>
+      </c>
+      <c r="E337" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="338">
+      <c r="A338" t="inlineStr">
+        <is>
+          <t>18:01:08</t>
+        </is>
+      </c>
+      <c r="B338" t="inlineStr">
+        <is>
+          <t>19:47</t>
+        </is>
+      </c>
+      <c r="C338" t="inlineStr">
+        <is>
+          <t>17X38_ROMERO</t>
+        </is>
+      </c>
+      <c r="D338" t="n">
+        <v>106</v>
+      </c>
+      <c r="E338" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="339">
+      <c r="A339" t="inlineStr">
+        <is>
+          <t>18:01:08</t>
+        </is>
+      </c>
+      <c r="B339" t="inlineStr">
+        <is>
+          <t>19:53</t>
+        </is>
+      </c>
+      <c r="C339" t="inlineStr">
+        <is>
+          <t>16_P MOR-SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D339" t="n">
+        <v>112</v>
+      </c>
+      <c r="E339" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="340">
+      <c r="A340" t="inlineStr">
+        <is>
+          <t>18:01:08</t>
+        </is>
+      </c>
+      <c r="B340" t="inlineStr">
+        <is>
+          <t>19:55</t>
+        </is>
+      </c>
+      <c r="C340" t="inlineStr">
+        <is>
+          <t>14X44_ABASTO</t>
+        </is>
+      </c>
+      <c r="D340" t="n">
+        <v>114</v>
+      </c>
+      <c r="E340" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -8719,7 +8869,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 17:47:20</t>
+          <t>Última actualización: 18:01:08</t>
         </is>
       </c>
     </row>
@@ -9960,7 +10110,7 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>17:47:19</t>
+          <t>18:01:08</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
@@ -9974,7 +10124,7 @@
         </is>
       </c>
       <c r="D54" t="n">
-        <v>97</v>
+        <v>83</v>
       </c>
       <c r="E54" t="inlineStr">
         <is>
@@ -9985,7 +10135,7 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>17:47:19</t>
+          <t>18:01:08</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
@@ -9999,7 +10149,7 @@
         </is>
       </c>
       <c r="D55" t="n">
-        <v>109</v>
+        <v>95</v>
       </c>
       <c r="E55" t="inlineStr">
         <is>
@@ -10031,7 +10181,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 17:47:20</t>
+          <t>Última actualización: 18:01:08</t>
         </is>
       </c>
     </row>
@@ -11347,7 +11497,7 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>17:47:19</t>
+          <t>18:01:08</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
@@ -11361,7 +11511,7 @@
         </is>
       </c>
       <c r="D57" t="n">
-        <v>39</v>
+        <v>25</v>
       </c>
       <c r="E57" t="inlineStr">
         <is>
@@ -11372,7 +11522,7 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>17:47:19</t>
+          <t>18:01:08</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
@@ -11386,7 +11536,7 @@
         </is>
       </c>
       <c r="D58" t="n">
-        <v>91</v>
+        <v>77</v>
       </c>
       <c r="E58" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 1822
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-03-21.xlsx
+++ b/data/horarios-141-2026-03-21.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E340"/>
+  <dimension ref="A1:E349"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 18:01:08</t>
+          <t>Última actualización: 18:35:14</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 335</t>
+          <t>Total filas: 344</t>
         </is>
       </c>
     </row>
@@ -533,7 +533,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D8" t="n">
@@ -558,7 +558,7 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D9" t="n">
@@ -758,7 +758,7 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D17" t="n">
@@ -783,7 +783,7 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D18" t="n">
@@ -1883,7 +1883,7 @@
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D62" t="n">
@@ -1898,7 +1898,7 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>08:14:14</t>
+          <t>06:59:30</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
@@ -1908,11 +1908,11 @@
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D63" t="n">
-        <v>0</v>
+        <v>75</v>
       </c>
       <c r="E63" t="inlineStr">
         <is>
@@ -1923,7 +1923,7 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>06:59:30</t>
+          <t>08:14:14</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
@@ -1933,11 +1933,11 @@
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D64" t="n">
-        <v>75</v>
+        <v>0</v>
       </c>
       <c r="E64" t="inlineStr">
         <is>
@@ -1973,7 +1973,7 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>07:51:37</t>
+          <t>07:27:35</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
@@ -1983,11 +1983,11 @@
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D66" t="n">
-        <v>28</v>
+        <v>52</v>
       </c>
       <c r="E66" t="inlineStr">
         <is>
@@ -1998,7 +1998,7 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>07:27:35</t>
+          <t>07:51:37</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
@@ -2008,11 +2008,11 @@
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D67" t="n">
-        <v>52</v>
+        <v>28</v>
       </c>
       <c r="E67" t="inlineStr">
         <is>
@@ -2033,7 +2033,7 @@
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D68" t="n">
@@ -2383,7 +2383,7 @@
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D82" t="n">
@@ -2408,7 +2408,7 @@
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D83" t="n">
@@ -2708,7 +2708,7 @@
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>215_EL PELIGRO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D95" t="n">
@@ -2733,7 +2733,7 @@
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215_EL PELIGRO</t>
         </is>
       </c>
       <c r="D96" t="n">
@@ -3173,7 +3173,7 @@
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>09:23:24</t>
+          <t>08:50:55</t>
         </is>
       </c>
       <c r="B114" t="inlineStr">
@@ -3183,11 +3183,11 @@
       </c>
       <c r="C114" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D114" t="n">
-        <v>40</v>
+        <v>73</v>
       </c>
       <c r="E114" t="inlineStr">
         <is>
@@ -3198,7 +3198,7 @@
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>08:50:55</t>
+          <t>09:23:24</t>
         </is>
       </c>
       <c r="B115" t="inlineStr">
@@ -3208,11 +3208,11 @@
       </c>
       <c r="C115" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D115" t="n">
-        <v>73</v>
+        <v>40</v>
       </c>
       <c r="E115" t="inlineStr">
         <is>
@@ -3498,7 +3498,7 @@
     <row r="127">
       <c r="A127" t="inlineStr">
         <is>
-          <t>10:14:52</t>
+          <t>08:36:09</t>
         </is>
       </c>
       <c r="B127" t="inlineStr">
@@ -3508,11 +3508,11 @@
       </c>
       <c r="C127" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D127" t="n">
-        <v>19</v>
+        <v>117</v>
       </c>
       <c r="E127" t="inlineStr">
         <is>
@@ -3523,7 +3523,7 @@
     <row r="128">
       <c r="A128" t="inlineStr">
         <is>
-          <t>08:36:09</t>
+          <t>10:14:52</t>
         </is>
       </c>
       <c r="B128" t="inlineStr">
@@ -3533,11 +3533,11 @@
       </c>
       <c r="C128" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D128" t="n">
-        <v>117</v>
+        <v>19</v>
       </c>
       <c r="E128" t="inlineStr">
         <is>
@@ -3598,7 +3598,7 @@
     <row r="131">
       <c r="A131" t="inlineStr">
         <is>
-          <t>10:14:52</t>
+          <t>09:23:24</t>
         </is>
       </c>
       <c r="B131" t="inlineStr">
@@ -3608,11 +3608,11 @@
       </c>
       <c r="C131" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D131" t="n">
-        <v>29</v>
+        <v>80</v>
       </c>
       <c r="E131" t="inlineStr">
         <is>
@@ -3623,7 +3623,7 @@
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t>09:23:24</t>
+          <t>10:14:52</t>
         </is>
       </c>
       <c r="B132" t="inlineStr">
@@ -3633,11 +3633,11 @@
       </c>
       <c r="C132" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D132" t="n">
-        <v>80</v>
+        <v>29</v>
       </c>
       <c r="E132" t="inlineStr">
         <is>
@@ -3873,7 +3873,7 @@
     <row r="142">
       <c r="A142" t="inlineStr">
         <is>
-          <t>10:52:37</t>
+          <t>10:14:52</t>
         </is>
       </c>
       <c r="B142" t="inlineStr">
@@ -3883,11 +3883,11 @@
       </c>
       <c r="C142" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D142" t="n">
-        <v>11</v>
+        <v>49</v>
       </c>
       <c r="E142" t="inlineStr">
         <is>
@@ -3898,7 +3898,7 @@
     <row r="143">
       <c r="A143" t="inlineStr">
         <is>
-          <t>10:14:52</t>
+          <t>10:52:37</t>
         </is>
       </c>
       <c r="B143" t="inlineStr">
@@ -3908,11 +3908,11 @@
       </c>
       <c r="C143" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D143" t="n">
-        <v>49</v>
+        <v>11</v>
       </c>
       <c r="E143" t="inlineStr">
         <is>
@@ -4183,7 +4183,7 @@
       </c>
       <c r="C154" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D154" t="n">
@@ -4208,7 +4208,7 @@
       </c>
       <c r="C155" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D155" t="n">
@@ -4673,7 +4673,7 @@
     <row r="174">
       <c r="A174" t="inlineStr">
         <is>
-          <t>12:28:38</t>
+          <t>12:00:15</t>
         </is>
       </c>
       <c r="B174" t="inlineStr">
@@ -4683,11 +4683,11 @@
       </c>
       <c r="C174" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D174" t="n">
-        <v>5</v>
+        <v>33</v>
       </c>
       <c r="E174" t="inlineStr">
         <is>
@@ -4698,7 +4698,7 @@
     <row r="175">
       <c r="A175" t="inlineStr">
         <is>
-          <t>12:00:15</t>
+          <t>12:28:38</t>
         </is>
       </c>
       <c r="B175" t="inlineStr">
@@ -4708,11 +4708,11 @@
       </c>
       <c r="C175" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D175" t="n">
-        <v>33</v>
+        <v>5</v>
       </c>
       <c r="E175" t="inlineStr">
         <is>
@@ -4998,7 +4998,7 @@
     <row r="187">
       <c r="A187" t="inlineStr">
         <is>
-          <t>12:28:38</t>
+          <t>13:00:14</t>
         </is>
       </c>
       <c r="B187" t="inlineStr">
@@ -5008,11 +5008,11 @@
       </c>
       <c r="C187" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D187" t="n">
-        <v>35</v>
+        <v>3</v>
       </c>
       <c r="E187" t="inlineStr">
         <is>
@@ -5023,7 +5023,7 @@
     <row r="188">
       <c r="A188" t="inlineStr">
         <is>
-          <t>13:00:14</t>
+          <t>12:28:38</t>
         </is>
       </c>
       <c r="B188" t="inlineStr">
@@ -5033,11 +5033,11 @@
       </c>
       <c r="C188" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D188" t="n">
-        <v>3</v>
+        <v>35</v>
       </c>
       <c r="E188" t="inlineStr">
         <is>
@@ -5073,7 +5073,7 @@
     <row r="190">
       <c r="A190" t="inlineStr">
         <is>
-          <t>12:48:06</t>
+          <t>13:00:14</t>
         </is>
       </c>
       <c r="B190" t="inlineStr">
@@ -5083,11 +5083,11 @@
       </c>
       <c r="C190" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D190" t="n">
-        <v>16</v>
+        <v>4</v>
       </c>
       <c r="E190" t="inlineStr">
         <is>
@@ -5098,7 +5098,7 @@
     <row r="191">
       <c r="A191" t="inlineStr">
         <is>
-          <t>13:00:14</t>
+          <t>12:48:06</t>
         </is>
       </c>
       <c r="B191" t="inlineStr">
@@ -5108,11 +5108,11 @@
       </c>
       <c r="C191" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D191" t="n">
-        <v>4</v>
+        <v>16</v>
       </c>
       <c r="E191" t="inlineStr">
         <is>
@@ -5248,7 +5248,7 @@
     <row r="197">
       <c r="A197" t="inlineStr">
         <is>
-          <t>13:00:14</t>
+          <t>12:48:06</t>
         </is>
       </c>
       <c r="B197" t="inlineStr">
@@ -5258,11 +5258,11 @@
       </c>
       <c r="C197" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D197" t="n">
-        <v>33</v>
+        <v>45</v>
       </c>
       <c r="E197" t="inlineStr">
         <is>
@@ -5273,7 +5273,7 @@
     <row r="198">
       <c r="A198" t="inlineStr">
         <is>
-          <t>12:48:06</t>
+          <t>13:00:14</t>
         </is>
       </c>
       <c r="B198" t="inlineStr">
@@ -5283,11 +5283,11 @@
       </c>
       <c r="C198" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D198" t="n">
-        <v>45</v>
+        <v>33</v>
       </c>
       <c r="E198" t="inlineStr">
         <is>
@@ -5623,7 +5623,7 @@
     <row r="212">
       <c r="A212" t="inlineStr">
         <is>
-          <t>13:57:43</t>
+          <t>13:32:57</t>
         </is>
       </c>
       <c r="B212" t="inlineStr">
@@ -5633,11 +5633,11 @@
       </c>
       <c r="C212" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D212" t="n">
-        <v>19</v>
+        <v>44</v>
       </c>
       <c r="E212" t="inlineStr">
         <is>
@@ -5648,7 +5648,7 @@
     <row r="213">
       <c r="A213" t="inlineStr">
         <is>
-          <t>13:32:57</t>
+          <t>13:57:43</t>
         </is>
       </c>
       <c r="B213" t="inlineStr">
@@ -5658,11 +5658,11 @@
       </c>
       <c r="C213" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D213" t="n">
-        <v>44</v>
+        <v>19</v>
       </c>
       <c r="E213" t="inlineStr">
         <is>
@@ -5673,7 +5673,7 @@
     <row r="214">
       <c r="A214" t="inlineStr">
         <is>
-          <t>13:00:14</t>
+          <t>13:57:43</t>
         </is>
       </c>
       <c r="B214" t="inlineStr">
@@ -5683,11 +5683,11 @@
       </c>
       <c r="C214" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D214" t="n">
-        <v>77</v>
+        <v>20</v>
       </c>
       <c r="E214" t="inlineStr">
         <is>
@@ -5698,7 +5698,7 @@
     <row r="215">
       <c r="A215" t="inlineStr">
         <is>
-          <t>13:57:43</t>
+          <t>13:00:14</t>
         </is>
       </c>
       <c r="B215" t="inlineStr">
@@ -5708,11 +5708,11 @@
       </c>
       <c r="C215" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D215" t="n">
-        <v>20</v>
+        <v>77</v>
       </c>
       <c r="E215" t="inlineStr">
         <is>
@@ -5873,7 +5873,7 @@
     <row r="222">
       <c r="A222" t="inlineStr">
         <is>
-          <t>13:00:14</t>
+          <t>14:21:42</t>
         </is>
       </c>
       <c r="B222" t="inlineStr">
@@ -5883,11 +5883,11 @@
       </c>
       <c r="C222" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D222" t="n">
-        <v>93</v>
+        <v>12</v>
       </c>
       <c r="E222" t="inlineStr">
         <is>
@@ -5898,7 +5898,7 @@
     <row r="223">
       <c r="A223" t="inlineStr">
         <is>
-          <t>14:21:42</t>
+          <t>13:00:14</t>
         </is>
       </c>
       <c r="B223" t="inlineStr">
@@ -5908,11 +5908,11 @@
       </c>
       <c r="C223" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D223" t="n">
-        <v>12</v>
+        <v>93</v>
       </c>
       <c r="E223" t="inlineStr">
         <is>
@@ -5983,7 +5983,7 @@
       </c>
       <c r="C226" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D226" t="n">
@@ -6008,7 +6008,7 @@
       </c>
       <c r="C227" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D227" t="n">
@@ -6098,7 +6098,7 @@
     <row r="231">
       <c r="A231" t="inlineStr">
         <is>
-          <t>14:46:39</t>
+          <t>14:59:00</t>
         </is>
       </c>
       <c r="B231" t="inlineStr">
@@ -6108,11 +6108,11 @@
       </c>
       <c r="C231" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>81_EL PELIGRO</t>
         </is>
       </c>
       <c r="D231" t="n">
-        <v>13</v>
+        <v>0</v>
       </c>
       <c r="E231" t="inlineStr">
         <is>
@@ -6123,7 +6123,7 @@
     <row r="232">
       <c r="A232" t="inlineStr">
         <is>
-          <t>14:59:00</t>
+          <t>14:46:39</t>
         </is>
       </c>
       <c r="B232" t="inlineStr">
@@ -6133,11 +6133,11 @@
       </c>
       <c r="C232" t="inlineStr">
         <is>
-          <t>81_EL PELIGRO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D232" t="n">
-        <v>0</v>
+        <v>13</v>
       </c>
       <c r="E232" t="inlineStr">
         <is>
@@ -6298,7 +6298,7 @@
     <row r="239">
       <c r="A239" t="inlineStr">
         <is>
-          <t>14:59:00</t>
+          <t>14:46:39</t>
         </is>
       </c>
       <c r="B239" t="inlineStr">
@@ -6308,11 +6308,11 @@
       </c>
       <c r="C239" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D239" t="n">
-        <v>12</v>
+        <v>25</v>
       </c>
       <c r="E239" t="inlineStr">
         <is>
@@ -6323,7 +6323,7 @@
     <row r="240">
       <c r="A240" t="inlineStr">
         <is>
-          <t>14:46:39</t>
+          <t>14:59:00</t>
         </is>
       </c>
       <c r="B240" t="inlineStr">
@@ -6333,11 +6333,11 @@
       </c>
       <c r="C240" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D240" t="n">
-        <v>25</v>
+        <v>12</v>
       </c>
       <c r="E240" t="inlineStr">
         <is>
@@ -7033,7 +7033,7 @@
       </c>
       <c r="C268" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D268" t="n">
@@ -7058,7 +7058,7 @@
       </c>
       <c r="C269" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D269" t="n">
@@ -7333,7 +7333,7 @@
       </c>
       <c r="C280" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D280" t="n">
@@ -7358,7 +7358,7 @@
       </c>
       <c r="C281" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D281" t="n">
@@ -7573,7 +7573,7 @@
     <row r="290">
       <c r="A290" t="inlineStr">
         <is>
-          <t>17:21:09</t>
+          <t>16:33:34</t>
         </is>
       </c>
       <c r="B290" t="inlineStr">
@@ -7583,11 +7583,11 @@
       </c>
       <c r="C290" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D290" t="n">
-        <v>3</v>
+        <v>51</v>
       </c>
       <c r="E290" t="inlineStr">
         <is>
@@ -7598,7 +7598,7 @@
     <row r="291">
       <c r="A291" t="inlineStr">
         <is>
-          <t>16:33:34</t>
+          <t>17:21:09</t>
         </is>
       </c>
       <c r="B291" t="inlineStr">
@@ -7608,11 +7608,11 @@
       </c>
       <c r="C291" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D291" t="n">
-        <v>51</v>
+        <v>3</v>
       </c>
       <c r="E291" t="inlineStr">
         <is>
@@ -7883,7 +7883,7 @@
       </c>
       <c r="C302" t="inlineStr">
         <is>
-          <t>215_EL PELIGRO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D302" t="n">
@@ -7908,7 +7908,7 @@
       </c>
       <c r="C303" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>215_EL PELIGRO</t>
         </is>
       </c>
       <c r="D303" t="n">
@@ -7948,7 +7948,7 @@
     <row r="305">
       <c r="A305" t="inlineStr">
         <is>
-          <t>17:47:19</t>
+          <t>16:57:49</t>
         </is>
       </c>
       <c r="B305" t="inlineStr">
@@ -7958,11 +7958,11 @@
       </c>
       <c r="C305" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D305" t="n">
-        <v>12</v>
+        <v>62</v>
       </c>
       <c r="E305" t="inlineStr">
         <is>
@@ -7973,7 +7973,7 @@
     <row r="306">
       <c r="A306" t="inlineStr">
         <is>
-          <t>16:57:49</t>
+          <t>17:47:19</t>
         </is>
       </c>
       <c r="B306" t="inlineStr">
@@ -7983,11 +7983,11 @@
       </c>
       <c r="C306" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D306" t="n">
-        <v>62</v>
+        <v>12</v>
       </c>
       <c r="E306" t="inlineStr">
         <is>
@@ -8008,7 +8008,7 @@
       </c>
       <c r="C307" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D307" t="n">
@@ -8033,7 +8033,7 @@
       </c>
       <c r="C308" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D308" t="n">
@@ -8083,7 +8083,7 @@
       </c>
       <c r="C310" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D310" t="n">
@@ -8108,7 +8108,7 @@
       </c>
       <c r="C311" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D311" t="n">
@@ -8158,7 +8158,7 @@
       </c>
       <c r="C313" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D313" t="n">
@@ -8183,7 +8183,7 @@
       </c>
       <c r="C314" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D314" t="n">
@@ -8373,21 +8373,21 @@
     <row r="322">
       <c r="A322" t="inlineStr">
         <is>
-          <t>17:47:19</t>
+          <t>18:35:14</t>
         </is>
       </c>
       <c r="B322" t="inlineStr">
         <is>
-          <t>18:38</t>
+          <t>18:36</t>
         </is>
       </c>
       <c r="C322" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D322" t="n">
-        <v>51</v>
+        <v>1</v>
       </c>
       <c r="E322" t="inlineStr">
         <is>
@@ -8398,12 +8398,12 @@
     <row r="323">
       <c r="A323" t="inlineStr">
         <is>
-          <t>18:01:08</t>
+          <t>18:35:14</t>
         </is>
       </c>
       <c r="B323" t="inlineStr">
         <is>
-          <t>18:39</t>
+          <t>18:37</t>
         </is>
       </c>
       <c r="C323" t="inlineStr">
@@ -8412,7 +8412,7 @@
         </is>
       </c>
       <c r="D323" t="n">
-        <v>38</v>
+        <v>2</v>
       </c>
       <c r="E323" t="inlineStr">
         <is>
@@ -8423,21 +8423,21 @@
     <row r="324">
       <c r="A324" t="inlineStr">
         <is>
-          <t>18:01:08</t>
+          <t>17:47:19</t>
         </is>
       </c>
       <c r="B324" t="inlineStr">
         <is>
-          <t>18:41</t>
+          <t>18:38</t>
         </is>
       </c>
       <c r="C324" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D324" t="n">
-        <v>40</v>
+        <v>51</v>
       </c>
       <c r="E324" t="inlineStr">
         <is>
@@ -8453,16 +8453,16 @@
       </c>
       <c r="B325" t="inlineStr">
         <is>
-          <t>18:51</t>
+          <t>18:39</t>
         </is>
       </c>
       <c r="C325" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D325" t="n">
-        <v>50</v>
+        <v>38</v>
       </c>
       <c r="E325" t="inlineStr">
         <is>
@@ -8473,21 +8473,21 @@
     <row r="326">
       <c r="A326" t="inlineStr">
         <is>
-          <t>16:57:49</t>
+          <t>18:35:14</t>
         </is>
       </c>
       <c r="B326" t="inlineStr">
         <is>
-          <t>18:52</t>
+          <t>18:41</t>
         </is>
       </c>
       <c r="C326" t="inlineStr">
         <is>
-          <t>14X44_ABASTO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D326" t="n">
-        <v>115</v>
+        <v>6</v>
       </c>
       <c r="E326" t="inlineStr">
         <is>
@@ -8498,21 +8498,21 @@
     <row r="327">
       <c r="A327" t="inlineStr">
         <is>
-          <t>18:01:08</t>
+          <t>18:35:14</t>
         </is>
       </c>
       <c r="B327" t="inlineStr">
         <is>
-          <t>18:53</t>
+          <t>18:48</t>
         </is>
       </c>
       <c r="C327" t="inlineStr">
         <is>
-          <t>14X44_ABASTO</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D327" t="n">
-        <v>52</v>
+        <v>13</v>
       </c>
       <c r="E327" t="inlineStr">
         <is>
@@ -8523,21 +8523,21 @@
     <row r="328">
       <c r="A328" t="inlineStr">
         <is>
-          <t>18:01:08</t>
+          <t>18:35:14</t>
         </is>
       </c>
       <c r="B328" t="inlineStr">
         <is>
-          <t>19:00</t>
+          <t>18:51</t>
         </is>
       </c>
       <c r="C328" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D328" t="n">
-        <v>59</v>
+        <v>16</v>
       </c>
       <c r="E328" t="inlineStr">
         <is>
@@ -8548,21 +8548,21 @@
     <row r="329">
       <c r="A329" t="inlineStr">
         <is>
-          <t>17:47:19</t>
+          <t>16:57:49</t>
         </is>
       </c>
       <c r="B329" t="inlineStr">
         <is>
-          <t>19:08</t>
+          <t>18:52</t>
         </is>
       </c>
       <c r="C329" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>14X44_ABASTO</t>
         </is>
       </c>
       <c r="D329" t="n">
-        <v>81</v>
+        <v>115</v>
       </c>
       <c r="E329" t="inlineStr">
         <is>
@@ -8573,21 +8573,21 @@
     <row r="330">
       <c r="A330" t="inlineStr">
         <is>
-          <t>18:01:08</t>
+          <t>18:35:14</t>
         </is>
       </c>
       <c r="B330" t="inlineStr">
         <is>
-          <t>19:09</t>
+          <t>18:53</t>
         </is>
       </c>
       <c r="C330" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>14X44_ABASTO</t>
         </is>
       </c>
       <c r="D330" t="n">
-        <v>68</v>
+        <v>18</v>
       </c>
       <c r="E330" t="inlineStr">
         <is>
@@ -8598,21 +8598,21 @@
     <row r="331">
       <c r="A331" t="inlineStr">
         <is>
-          <t>18:01:08</t>
+          <t>18:35:14</t>
         </is>
       </c>
       <c r="B331" t="inlineStr">
         <is>
-          <t>19:12</t>
+          <t>19:00</t>
         </is>
       </c>
       <c r="C331" t="inlineStr">
         <is>
-          <t>81_EL PELIGRO</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D331" t="n">
-        <v>71</v>
+        <v>25</v>
       </c>
       <c r="E331" t="inlineStr">
         <is>
@@ -8623,21 +8623,21 @@
     <row r="332">
       <c r="A332" t="inlineStr">
         <is>
-          <t>18:01:08</t>
+          <t>18:35:14</t>
         </is>
       </c>
       <c r="B332" t="inlineStr">
         <is>
-          <t>19:17</t>
+          <t>19:01</t>
         </is>
       </c>
       <c r="C332" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D332" t="n">
-        <v>76</v>
+        <v>26</v>
       </c>
       <c r="E332" t="inlineStr">
         <is>
@@ -8648,21 +8648,21 @@
     <row r="333">
       <c r="A333" t="inlineStr">
         <is>
-          <t>17:47:19</t>
+          <t>18:35:14</t>
         </is>
       </c>
       <c r="B333" t="inlineStr">
         <is>
-          <t>19:20</t>
+          <t>19:03</t>
         </is>
       </c>
       <c r="C333" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D333" t="n">
-        <v>93</v>
+        <v>28</v>
       </c>
       <c r="E333" t="inlineStr">
         <is>
@@ -8673,21 +8673,21 @@
     <row r="334">
       <c r="A334" t="inlineStr">
         <is>
-          <t>18:01:08</t>
+          <t>17:47:19</t>
         </is>
       </c>
       <c r="B334" t="inlineStr">
         <is>
-          <t>19:23</t>
+          <t>19:08</t>
         </is>
       </c>
       <c r="C334" t="inlineStr">
         <is>
-          <t>225_GOMEZ</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D334" t="n">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="E334" t="inlineStr">
         <is>
@@ -8698,21 +8698,21 @@
     <row r="335">
       <c r="A335" t="inlineStr">
         <is>
-          <t>18:01:08</t>
+          <t>18:35:14</t>
         </is>
       </c>
       <c r="B335" t="inlineStr">
         <is>
-          <t>19:24</t>
+          <t>19:09</t>
         </is>
       </c>
       <c r="C335" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D335" t="n">
-        <v>83</v>
+        <v>34</v>
       </c>
       <c r="E335" t="inlineStr">
         <is>
@@ -8723,21 +8723,21 @@
     <row r="336">
       <c r="A336" t="inlineStr">
         <is>
-          <t>18:01:08</t>
+          <t>18:35:14</t>
         </is>
       </c>
       <c r="B336" t="inlineStr">
         <is>
-          <t>19:36</t>
+          <t>19:12</t>
         </is>
       </c>
       <c r="C336" t="inlineStr">
         <is>
-          <t>215_EL PELIGRO</t>
+          <t>81_EL PELIGRO</t>
         </is>
       </c>
       <c r="D336" t="n">
-        <v>95</v>
+        <v>37</v>
       </c>
       <c r="E336" t="inlineStr">
         <is>
@@ -8748,21 +8748,21 @@
     <row r="337">
       <c r="A337" t="inlineStr">
         <is>
-          <t>18:01:08</t>
+          <t>18:35:14</t>
         </is>
       </c>
       <c r="B337" t="inlineStr">
         <is>
-          <t>19:40</t>
+          <t>19:17</t>
         </is>
       </c>
       <c r="C337" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D337" t="n">
-        <v>99</v>
+        <v>42</v>
       </c>
       <c r="E337" t="inlineStr">
         <is>
@@ -8773,21 +8773,21 @@
     <row r="338">
       <c r="A338" t="inlineStr">
         <is>
-          <t>18:01:08</t>
+          <t>17:47:19</t>
         </is>
       </c>
       <c r="B338" t="inlineStr">
         <is>
-          <t>19:47</t>
+          <t>19:20</t>
         </is>
       </c>
       <c r="C338" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D338" t="n">
-        <v>106</v>
+        <v>93</v>
       </c>
       <c r="E338" t="inlineStr">
         <is>
@@ -8798,21 +8798,21 @@
     <row r="339">
       <c r="A339" t="inlineStr">
         <is>
-          <t>18:01:08</t>
+          <t>18:35:14</t>
         </is>
       </c>
       <c r="B339" t="inlineStr">
         <is>
-          <t>19:53</t>
+          <t>19:23</t>
         </is>
       </c>
       <c r="C339" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>225_GOMEZ</t>
         </is>
       </c>
       <c r="D339" t="n">
-        <v>112</v>
+        <v>48</v>
       </c>
       <c r="E339" t="inlineStr">
         <is>
@@ -8823,23 +8823,248 @@
     <row r="340">
       <c r="A340" t="inlineStr">
         <is>
-          <t>18:01:08</t>
+          <t>18:35:14</t>
         </is>
       </c>
       <c r="B340" t="inlineStr">
         <is>
+          <t>19:24</t>
+        </is>
+      </c>
+      <c r="C340" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D340" t="n">
+        <v>49</v>
+      </c>
+      <c r="E340" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="341">
+      <c r="A341" t="inlineStr">
+        <is>
+          <t>18:35:14</t>
+        </is>
+      </c>
+      <c r="B341" t="inlineStr">
+        <is>
+          <t>19:36</t>
+        </is>
+      </c>
+      <c r="C341" t="inlineStr">
+        <is>
+          <t>215_EL PELIGRO</t>
+        </is>
+      </c>
+      <c r="D341" t="n">
+        <v>61</v>
+      </c>
+      <c r="E341" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="342">
+      <c r="A342" t="inlineStr">
+        <is>
+          <t>18:35:14</t>
+        </is>
+      </c>
+      <c r="B342" t="inlineStr">
+        <is>
+          <t>19:38</t>
+        </is>
+      </c>
+      <c r="C342" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D342" t="n">
+        <v>63</v>
+      </c>
+      <c r="E342" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="343">
+      <c r="A343" t="inlineStr">
+        <is>
+          <t>18:35:14</t>
+        </is>
+      </c>
+      <c r="B343" t="inlineStr">
+        <is>
+          <t>19:40</t>
+        </is>
+      </c>
+      <c r="C343" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D343" t="n">
+        <v>65</v>
+      </c>
+      <c r="E343" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="344">
+      <c r="A344" t="inlineStr">
+        <is>
+          <t>18:35:14</t>
+        </is>
+      </c>
+      <c r="B344" t="inlineStr">
+        <is>
+          <t>19:47</t>
+        </is>
+      </c>
+      <c r="C344" t="inlineStr">
+        <is>
+          <t>17X38_ROMERO</t>
+        </is>
+      </c>
+      <c r="D344" t="n">
+        <v>72</v>
+      </c>
+      <c r="E344" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="345">
+      <c r="A345" t="inlineStr">
+        <is>
+          <t>18:35:14</t>
+        </is>
+      </c>
+      <c r="B345" t="inlineStr">
+        <is>
+          <t>19:53</t>
+        </is>
+      </c>
+      <c r="C345" t="inlineStr">
+        <is>
+          <t>16_P MOR-SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D345" t="n">
+        <v>78</v>
+      </c>
+      <c r="E345" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="346">
+      <c r="A346" t="inlineStr">
+        <is>
+          <t>18:35:14</t>
+        </is>
+      </c>
+      <c r="B346" t="inlineStr">
+        <is>
           <t>19:55</t>
         </is>
       </c>
-      <c r="C340" t="inlineStr">
+      <c r="C346" t="inlineStr">
         <is>
           <t>14X44_ABASTO</t>
         </is>
       </c>
-      <c r="D340" t="n">
-        <v>114</v>
-      </c>
-      <c r="E340" t="inlineStr">
+      <c r="D346" t="n">
+        <v>80</v>
+      </c>
+      <c r="E346" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="347">
+      <c r="A347" t="inlineStr">
+        <is>
+          <t>18:35:14</t>
+        </is>
+      </c>
+      <c r="B347" t="inlineStr">
+        <is>
+          <t>20:00</t>
+        </is>
+      </c>
+      <c r="C347" t="inlineStr">
+        <is>
+          <t>81_EL PELIGRO</t>
+        </is>
+      </c>
+      <c r="D347" t="n">
+        <v>85</v>
+      </c>
+      <c r="E347" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="348">
+      <c r="A348" t="inlineStr">
+        <is>
+          <t>18:35:14</t>
+        </is>
+      </c>
+      <c r="B348" t="inlineStr">
+        <is>
+          <t>20:15</t>
+        </is>
+      </c>
+      <c r="C348" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D348" t="n">
+        <v>100</v>
+      </c>
+      <c r="E348" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="349">
+      <c r="A349" t="inlineStr">
+        <is>
+          <t>18:35:14</t>
+        </is>
+      </c>
+      <c r="B349" t="inlineStr">
+        <is>
+          <t>20:27</t>
+        </is>
+      </c>
+      <c r="C349" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D349" t="n">
+        <v>112</v>
+      </c>
+      <c r="E349" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -8856,7 +9081,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E55"/>
+  <dimension ref="A1:E56"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -8869,14 +9094,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 18:01:08</t>
+          <t>Última actualización: 18:35:14</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 50</t>
+          <t>Total filas: 51</t>
         </is>
       </c>
     </row>
@@ -10110,7 +10335,7 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>18:01:08</t>
+          <t>18:35:14</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
@@ -10124,7 +10349,7 @@
         </is>
       </c>
       <c r="D54" t="n">
-        <v>83</v>
+        <v>49</v>
       </c>
       <c r="E54" t="inlineStr">
         <is>
@@ -10135,7 +10360,7 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>18:01:08</t>
+          <t>18:35:14</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
@@ -10149,9 +10374,34 @@
         </is>
       </c>
       <c r="D55" t="n">
-        <v>95</v>
+        <v>61</v>
       </c>
       <c r="E55" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>18:35:14</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>20:15</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D56" t="n">
+        <v>100</v>
+      </c>
+      <c r="E56" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -10181,7 +10431,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 18:01:08</t>
+          <t>Última actualización: 18:35:14</t>
         </is>
       </c>
     </row>
@@ -11522,7 +11772,7 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>18:01:08</t>
+          <t>18:35:14</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
@@ -11536,7 +11786,7 @@
         </is>
       </c>
       <c r="D58" t="n">
-        <v>77</v>
+        <v>43</v>
       </c>
       <c r="E58" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 1823
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-03-21.xlsx
+++ b/data/horarios-141-2026-03-21.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E349"/>
+  <dimension ref="A1:E357"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 18:35:14</t>
+          <t>Última actualización: 18:51:25</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 344</t>
+          <t>Total filas: 352</t>
         </is>
       </c>
     </row>
@@ -1158,7 +1158,7 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D33" t="n">
@@ -1183,7 +1183,7 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D34" t="n">
@@ -1883,7 +1883,7 @@
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D62" t="n">
@@ -1933,7 +1933,7 @@
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D64" t="n">
@@ -1973,7 +1973,7 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>07:27:35</t>
+          <t>07:51:37</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
@@ -1983,11 +1983,11 @@
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D66" t="n">
-        <v>52</v>
+        <v>28</v>
       </c>
       <c r="E66" t="inlineStr">
         <is>
@@ -2023,7 +2023,7 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>07:51:37</t>
+          <t>07:27:35</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
@@ -2033,11 +2033,11 @@
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D68" t="n">
-        <v>28</v>
+        <v>52</v>
       </c>
       <c r="E68" t="inlineStr">
         <is>
@@ -2233,7 +2233,7 @@
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D76" t="n">
@@ -2258,7 +2258,7 @@
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D77" t="n">
@@ -2398,7 +2398,7 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>08:50:55</t>
+          <t>07:27:35</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
@@ -2408,11 +2408,11 @@
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D83" t="n">
-        <v>1</v>
+        <v>84</v>
       </c>
       <c r="E83" t="inlineStr">
         <is>
@@ -2423,7 +2423,7 @@
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>07:27:35</t>
+          <t>08:50:55</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
@@ -2433,11 +2433,11 @@
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D84" t="n">
-        <v>84</v>
+        <v>1</v>
       </c>
       <c r="E84" t="inlineStr">
         <is>
@@ -2698,7 +2698,7 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>08:50:55</t>
+          <t>08:14:14</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
@@ -2708,11 +2708,11 @@
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D95" t="n">
-        <v>28</v>
+        <v>64</v>
       </c>
       <c r="E95" t="inlineStr">
         <is>
@@ -2748,7 +2748,7 @@
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>08:14:14</t>
+          <t>08:50:55</t>
         </is>
       </c>
       <c r="B97" t="inlineStr">
@@ -2758,11 +2758,11 @@
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D97" t="n">
-        <v>64</v>
+        <v>28</v>
       </c>
       <c r="E97" t="inlineStr">
         <is>
@@ -4123,7 +4123,7 @@
     <row r="152">
       <c r="A152" t="inlineStr">
         <is>
-          <t>10:14:52</t>
+          <t>11:16:36</t>
         </is>
       </c>
       <c r="B152" t="inlineStr">
@@ -4133,11 +4133,11 @@
       </c>
       <c r="C152" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D152" t="n">
-        <v>78</v>
+        <v>16</v>
       </c>
       <c r="E152" t="inlineStr">
         <is>
@@ -4148,7 +4148,7 @@
     <row r="153">
       <c r="A153" t="inlineStr">
         <is>
-          <t>11:16:36</t>
+          <t>10:14:52</t>
         </is>
       </c>
       <c r="B153" t="inlineStr">
@@ -4158,11 +4158,11 @@
       </c>
       <c r="C153" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D153" t="n">
-        <v>16</v>
+        <v>78</v>
       </c>
       <c r="E153" t="inlineStr">
         <is>
@@ -4473,7 +4473,7 @@
     <row r="166">
       <c r="A166" t="inlineStr">
         <is>
-          <t>11:16:36</t>
+          <t>12:00:15</t>
         </is>
       </c>
       <c r="B166" t="inlineStr">
@@ -4483,11 +4483,11 @@
       </c>
       <c r="C166" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D166" t="n">
-        <v>48</v>
+        <v>4</v>
       </c>
       <c r="E166" t="inlineStr">
         <is>
@@ -4498,7 +4498,7 @@
     <row r="167">
       <c r="A167" t="inlineStr">
         <is>
-          <t>12:00:15</t>
+          <t>11:16:36</t>
         </is>
       </c>
       <c r="B167" t="inlineStr">
@@ -4508,11 +4508,11 @@
       </c>
       <c r="C167" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D167" t="n">
-        <v>4</v>
+        <v>48</v>
       </c>
       <c r="E167" t="inlineStr">
         <is>
@@ -4673,7 +4673,7 @@
     <row r="174">
       <c r="A174" t="inlineStr">
         <is>
-          <t>12:00:15</t>
+          <t>12:28:38</t>
         </is>
       </c>
       <c r="B174" t="inlineStr">
@@ -4683,11 +4683,11 @@
       </c>
       <c r="C174" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D174" t="n">
-        <v>33</v>
+        <v>5</v>
       </c>
       <c r="E174" t="inlineStr">
         <is>
@@ -4698,7 +4698,7 @@
     <row r="175">
       <c r="A175" t="inlineStr">
         <is>
-          <t>12:28:38</t>
+          <t>12:00:15</t>
         </is>
       </c>
       <c r="B175" t="inlineStr">
@@ -4708,11 +4708,11 @@
       </c>
       <c r="C175" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D175" t="n">
-        <v>5</v>
+        <v>33</v>
       </c>
       <c r="E175" t="inlineStr">
         <is>
@@ -5673,7 +5673,7 @@
     <row r="214">
       <c r="A214" t="inlineStr">
         <is>
-          <t>13:57:43</t>
+          <t>13:00:14</t>
         </is>
       </c>
       <c r="B214" t="inlineStr">
@@ -5683,11 +5683,11 @@
       </c>
       <c r="C214" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D214" t="n">
-        <v>20</v>
+        <v>77</v>
       </c>
       <c r="E214" t="inlineStr">
         <is>
@@ -5698,7 +5698,7 @@
     <row r="215">
       <c r="A215" t="inlineStr">
         <is>
-          <t>13:00:14</t>
+          <t>13:57:43</t>
         </is>
       </c>
       <c r="B215" t="inlineStr">
@@ -5708,11 +5708,11 @@
       </c>
       <c r="C215" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D215" t="n">
-        <v>77</v>
+        <v>20</v>
       </c>
       <c r="E215" t="inlineStr">
         <is>
@@ -5873,7 +5873,7 @@
     <row r="222">
       <c r="A222" t="inlineStr">
         <is>
-          <t>14:21:42</t>
+          <t>13:00:14</t>
         </is>
       </c>
       <c r="B222" t="inlineStr">
@@ -5883,11 +5883,11 @@
       </c>
       <c r="C222" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D222" t="n">
-        <v>12</v>
+        <v>93</v>
       </c>
       <c r="E222" t="inlineStr">
         <is>
@@ -5898,7 +5898,7 @@
     <row r="223">
       <c r="A223" t="inlineStr">
         <is>
-          <t>13:00:14</t>
+          <t>14:21:42</t>
         </is>
       </c>
       <c r="B223" t="inlineStr">
@@ -5908,11 +5908,11 @@
       </c>
       <c r="C223" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D223" t="n">
-        <v>93</v>
+        <v>12</v>
       </c>
       <c r="E223" t="inlineStr">
         <is>
@@ -5983,7 +5983,7 @@
       </c>
       <c r="C226" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D226" t="n">
@@ -6008,7 +6008,7 @@
       </c>
       <c r="C227" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D227" t="n">
@@ -6698,7 +6698,7 @@
     <row r="255">
       <c r="A255" t="inlineStr">
         <is>
-          <t>14:46:39</t>
+          <t>15:34:45</t>
         </is>
       </c>
       <c r="B255" t="inlineStr">
@@ -6708,11 +6708,11 @@
       </c>
       <c r="C255" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D255" t="n">
-        <v>68</v>
+        <v>20</v>
       </c>
       <c r="E255" t="inlineStr">
         <is>
@@ -6723,7 +6723,7 @@
     <row r="256">
       <c r="A256" t="inlineStr">
         <is>
-          <t>15:34:45</t>
+          <t>14:46:39</t>
         </is>
       </c>
       <c r="B256" t="inlineStr">
@@ -6733,11 +6733,11 @@
       </c>
       <c r="C256" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D256" t="n">
-        <v>20</v>
+        <v>68</v>
       </c>
       <c r="E256" t="inlineStr">
         <is>
@@ -6933,7 +6933,7 @@
       </c>
       <c r="C264" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>215_ALUAR</t>
         </is>
       </c>
       <c r="D264" t="n">
@@ -6958,7 +6958,7 @@
       </c>
       <c r="C265" t="inlineStr">
         <is>
-          <t>215_ALUAR</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D265" t="n">
@@ -7123,7 +7123,7 @@
     <row r="272">
       <c r="A272" t="inlineStr">
         <is>
-          <t>14:59:00</t>
+          <t>15:34:45</t>
         </is>
       </c>
       <c r="B272" t="inlineStr">
@@ -7133,11 +7133,11 @@
       </c>
       <c r="C272" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D272" t="n">
-        <v>97</v>
+        <v>62</v>
       </c>
       <c r="E272" t="inlineStr">
         <is>
@@ -7148,7 +7148,7 @@
     <row r="273">
       <c r="A273" t="inlineStr">
         <is>
-          <t>15:34:45</t>
+          <t>14:59:00</t>
         </is>
       </c>
       <c r="B273" t="inlineStr">
@@ -7158,11 +7158,11 @@
       </c>
       <c r="C273" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D273" t="n">
-        <v>62</v>
+        <v>97</v>
       </c>
       <c r="E273" t="inlineStr">
         <is>
@@ -7333,7 +7333,7 @@
       </c>
       <c r="C280" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D280" t="n">
@@ -7358,7 +7358,7 @@
       </c>
       <c r="C281" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D281" t="n">
@@ -7648,7 +7648,7 @@
     <row r="293">
       <c r="A293" t="inlineStr">
         <is>
-          <t>16:33:34</t>
+          <t>17:21:09</t>
         </is>
       </c>
       <c r="B293" t="inlineStr">
@@ -7658,11 +7658,11 @@
       </c>
       <c r="C293" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D293" t="n">
-        <v>62</v>
+        <v>14</v>
       </c>
       <c r="E293" t="inlineStr">
         <is>
@@ -7673,7 +7673,7 @@
     <row r="294">
       <c r="A294" t="inlineStr">
         <is>
-          <t>17:21:09</t>
+          <t>16:33:34</t>
         </is>
       </c>
       <c r="B294" t="inlineStr">
@@ -7683,11 +7683,11 @@
       </c>
       <c r="C294" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D294" t="n">
-        <v>14</v>
+        <v>62</v>
       </c>
       <c r="E294" t="inlineStr">
         <is>
@@ -7948,7 +7948,7 @@
     <row r="305">
       <c r="A305" t="inlineStr">
         <is>
-          <t>16:57:49</t>
+          <t>17:47:19</t>
         </is>
       </c>
       <c r="B305" t="inlineStr">
@@ -7958,11 +7958,11 @@
       </c>
       <c r="C305" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D305" t="n">
-        <v>62</v>
+        <v>12</v>
       </c>
       <c r="E305" t="inlineStr">
         <is>
@@ -7973,7 +7973,7 @@
     <row r="306">
       <c r="A306" t="inlineStr">
         <is>
-          <t>17:47:19</t>
+          <t>16:57:49</t>
         </is>
       </c>
       <c r="B306" t="inlineStr">
@@ -7983,11 +7983,11 @@
       </c>
       <c r="C306" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D306" t="n">
-        <v>12</v>
+        <v>62</v>
       </c>
       <c r="E306" t="inlineStr">
         <is>
@@ -8083,7 +8083,7 @@
       </c>
       <c r="C310" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D310" t="n">
@@ -8108,7 +8108,7 @@
       </c>
       <c r="C311" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D311" t="n">
@@ -8158,7 +8158,7 @@
       </c>
       <c r="C313" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D313" t="n">
@@ -8183,7 +8183,7 @@
       </c>
       <c r="C314" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D314" t="n">
@@ -8523,7 +8523,7 @@
     <row r="328">
       <c r="A328" t="inlineStr">
         <is>
-          <t>18:35:14</t>
+          <t>18:51:25</t>
         </is>
       </c>
       <c r="B328" t="inlineStr">
@@ -8537,7 +8537,7 @@
         </is>
       </c>
       <c r="D328" t="n">
-        <v>16</v>
+        <v>0</v>
       </c>
       <c r="E328" t="inlineStr">
         <is>
@@ -8573,7 +8573,7 @@
     <row r="330">
       <c r="A330" t="inlineStr">
         <is>
-          <t>18:35:14</t>
+          <t>18:51:25</t>
         </is>
       </c>
       <c r="B330" t="inlineStr">
@@ -8587,7 +8587,7 @@
         </is>
       </c>
       <c r="D330" t="n">
-        <v>18</v>
+        <v>2</v>
       </c>
       <c r="E330" t="inlineStr">
         <is>
@@ -8598,7 +8598,7 @@
     <row r="331">
       <c r="A331" t="inlineStr">
         <is>
-          <t>18:35:14</t>
+          <t>18:51:25</t>
         </is>
       </c>
       <c r="B331" t="inlineStr">
@@ -8612,7 +8612,7 @@
         </is>
       </c>
       <c r="D331" t="n">
-        <v>25</v>
+        <v>9</v>
       </c>
       <c r="E331" t="inlineStr">
         <is>
@@ -8623,7 +8623,7 @@
     <row r="332">
       <c r="A332" t="inlineStr">
         <is>
-          <t>18:35:14</t>
+          <t>18:51:25</t>
         </is>
       </c>
       <c r="B332" t="inlineStr">
@@ -8637,7 +8637,7 @@
         </is>
       </c>
       <c r="D332" t="n">
-        <v>26</v>
+        <v>10</v>
       </c>
       <c r="E332" t="inlineStr">
         <is>
@@ -8673,21 +8673,21 @@
     <row r="334">
       <c r="A334" t="inlineStr">
         <is>
-          <t>17:47:19</t>
+          <t>18:51:25</t>
         </is>
       </c>
       <c r="B334" t="inlineStr">
         <is>
-          <t>19:08</t>
+          <t>19:07</t>
         </is>
       </c>
       <c r="C334" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D334" t="n">
-        <v>81</v>
+        <v>16</v>
       </c>
       <c r="E334" t="inlineStr">
         <is>
@@ -8698,12 +8698,12 @@
     <row r="335">
       <c r="A335" t="inlineStr">
         <is>
-          <t>18:35:14</t>
+          <t>17:47:19</t>
         </is>
       </c>
       <c r="B335" t="inlineStr">
         <is>
-          <t>19:09</t>
+          <t>19:08</t>
         </is>
       </c>
       <c r="C335" t="inlineStr">
@@ -8712,7 +8712,7 @@
         </is>
       </c>
       <c r="D335" t="n">
-        <v>34</v>
+        <v>81</v>
       </c>
       <c r="E335" t="inlineStr">
         <is>
@@ -8723,21 +8723,21 @@
     <row r="336">
       <c r="A336" t="inlineStr">
         <is>
-          <t>18:35:14</t>
+          <t>18:51:25</t>
         </is>
       </c>
       <c r="B336" t="inlineStr">
         <is>
-          <t>19:12</t>
+          <t>19:09</t>
         </is>
       </c>
       <c r="C336" t="inlineStr">
         <is>
-          <t>81_EL PELIGRO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D336" t="n">
-        <v>37</v>
+        <v>18</v>
       </c>
       <c r="E336" t="inlineStr">
         <is>
@@ -8748,21 +8748,21 @@
     <row r="337">
       <c r="A337" t="inlineStr">
         <is>
-          <t>18:35:14</t>
+          <t>18:51:25</t>
         </is>
       </c>
       <c r="B337" t="inlineStr">
         <is>
-          <t>19:17</t>
+          <t>19:12</t>
         </is>
       </c>
       <c r="C337" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>81_EL PELIGRO</t>
         </is>
       </c>
       <c r="D337" t="n">
-        <v>42</v>
+        <v>21</v>
       </c>
       <c r="E337" t="inlineStr">
         <is>
@@ -8773,12 +8773,12 @@
     <row r="338">
       <c r="A338" t="inlineStr">
         <is>
-          <t>17:47:19</t>
+          <t>18:51:25</t>
         </is>
       </c>
       <c r="B338" t="inlineStr">
         <is>
-          <t>19:20</t>
+          <t>19:16</t>
         </is>
       </c>
       <c r="C338" t="inlineStr">
@@ -8787,7 +8787,7 @@
         </is>
       </c>
       <c r="D338" t="n">
-        <v>93</v>
+        <v>25</v>
       </c>
       <c r="E338" t="inlineStr">
         <is>
@@ -8803,16 +8803,16 @@
       </c>
       <c r="B339" t="inlineStr">
         <is>
-          <t>19:23</t>
+          <t>19:17</t>
         </is>
       </c>
       <c r="C339" t="inlineStr">
         <is>
-          <t>225_GOMEZ</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D339" t="n">
-        <v>48</v>
+        <v>42</v>
       </c>
       <c r="E339" t="inlineStr">
         <is>
@@ -8823,21 +8823,21 @@
     <row r="340">
       <c r="A340" t="inlineStr">
         <is>
-          <t>18:35:14</t>
+          <t>17:47:19</t>
         </is>
       </c>
       <c r="B340" t="inlineStr">
         <is>
-          <t>19:24</t>
+          <t>19:20</t>
         </is>
       </c>
       <c r="C340" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D340" t="n">
-        <v>49</v>
+        <v>93</v>
       </c>
       <c r="E340" t="inlineStr">
         <is>
@@ -8848,21 +8848,21 @@
     <row r="341">
       <c r="A341" t="inlineStr">
         <is>
-          <t>18:35:14</t>
+          <t>18:51:25</t>
         </is>
       </c>
       <c r="B341" t="inlineStr">
         <is>
-          <t>19:36</t>
+          <t>19:21</t>
         </is>
       </c>
       <c r="C341" t="inlineStr">
         <is>
-          <t>215_EL PELIGRO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D341" t="n">
-        <v>61</v>
+        <v>30</v>
       </c>
       <c r="E341" t="inlineStr">
         <is>
@@ -8873,21 +8873,21 @@
     <row r="342">
       <c r="A342" t="inlineStr">
         <is>
-          <t>18:35:14</t>
+          <t>18:51:25</t>
         </is>
       </c>
       <c r="B342" t="inlineStr">
         <is>
-          <t>19:38</t>
+          <t>19:23</t>
         </is>
       </c>
       <c r="C342" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>225_GOMEZ</t>
         </is>
       </c>
       <c r="D342" t="n">
-        <v>63</v>
+        <v>32</v>
       </c>
       <c r="E342" t="inlineStr">
         <is>
@@ -8898,21 +8898,21 @@
     <row r="343">
       <c r="A343" t="inlineStr">
         <is>
-          <t>18:35:14</t>
+          <t>18:51:25</t>
         </is>
       </c>
       <c r="B343" t="inlineStr">
         <is>
-          <t>19:40</t>
+          <t>19:24</t>
         </is>
       </c>
       <c r="C343" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D343" t="n">
-        <v>65</v>
+        <v>33</v>
       </c>
       <c r="E343" t="inlineStr">
         <is>
@@ -8923,21 +8923,21 @@
     <row r="344">
       <c r="A344" t="inlineStr">
         <is>
-          <t>18:35:14</t>
+          <t>18:51:25</t>
         </is>
       </c>
       <c r="B344" t="inlineStr">
         <is>
-          <t>19:47</t>
+          <t>19:36</t>
         </is>
       </c>
       <c r="C344" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>215_EL PELIGRO</t>
         </is>
       </c>
       <c r="D344" t="n">
-        <v>72</v>
+        <v>45</v>
       </c>
       <c r="E344" t="inlineStr">
         <is>
@@ -8953,16 +8953,16 @@
       </c>
       <c r="B345" t="inlineStr">
         <is>
-          <t>19:53</t>
+          <t>19:38</t>
         </is>
       </c>
       <c r="C345" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D345" t="n">
-        <v>78</v>
+        <v>63</v>
       </c>
       <c r="E345" t="inlineStr">
         <is>
@@ -8973,21 +8973,21 @@
     <row r="346">
       <c r="A346" t="inlineStr">
         <is>
-          <t>18:35:14</t>
+          <t>18:51:25</t>
         </is>
       </c>
       <c r="B346" t="inlineStr">
         <is>
-          <t>19:55</t>
+          <t>19:40</t>
         </is>
       </c>
       <c r="C346" t="inlineStr">
         <is>
-          <t>14X44_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D346" t="n">
-        <v>80</v>
+        <v>49</v>
       </c>
       <c r="E346" t="inlineStr">
         <is>
@@ -8998,21 +8998,21 @@
     <row r="347">
       <c r="A347" t="inlineStr">
         <is>
-          <t>18:35:14</t>
+          <t>18:51:25</t>
         </is>
       </c>
       <c r="B347" t="inlineStr">
         <is>
-          <t>20:00</t>
+          <t>19:40</t>
         </is>
       </c>
       <c r="C347" t="inlineStr">
         <is>
-          <t>81_EL PELIGRO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D347" t="n">
-        <v>85</v>
+        <v>49</v>
       </c>
       <c r="E347" t="inlineStr">
         <is>
@@ -9023,21 +9023,21 @@
     <row r="348">
       <c r="A348" t="inlineStr">
         <is>
-          <t>18:35:14</t>
+          <t>18:51:25</t>
         </is>
       </c>
       <c r="B348" t="inlineStr">
         <is>
-          <t>20:15</t>
+          <t>19:47</t>
         </is>
       </c>
       <c r="C348" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D348" t="n">
-        <v>100</v>
+        <v>56</v>
       </c>
       <c r="E348" t="inlineStr">
         <is>
@@ -9048,23 +9048,223 @@
     <row r="349">
       <c r="A349" t="inlineStr">
         <is>
+          <t>18:51:25</t>
+        </is>
+      </c>
+      <c r="B349" t="inlineStr">
+        <is>
+          <t>19:53</t>
+        </is>
+      </c>
+      <c r="C349" t="inlineStr">
+        <is>
+          <t>16_P MOR-SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D349" t="n">
+        <v>62</v>
+      </c>
+      <c r="E349" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="350">
+      <c r="A350" t="inlineStr">
+        <is>
+          <t>18:51:25</t>
+        </is>
+      </c>
+      <c r="B350" t="inlineStr">
+        <is>
+          <t>19:54</t>
+        </is>
+      </c>
+      <c r="C350" t="inlineStr">
+        <is>
+          <t>14X44_ABASTO</t>
+        </is>
+      </c>
+      <c r="D350" t="n">
+        <v>63</v>
+      </c>
+      <c r="E350" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="351">
+      <c r="A351" t="inlineStr">
+        <is>
           <t>18:35:14</t>
         </is>
       </c>
-      <c r="B349" t="inlineStr">
+      <c r="B351" t="inlineStr">
+        <is>
+          <t>19:55</t>
+        </is>
+      </c>
+      <c r="C351" t="inlineStr">
+        <is>
+          <t>14X44_ABASTO</t>
+        </is>
+      </c>
+      <c r="D351" t="n">
+        <v>80</v>
+      </c>
+      <c r="E351" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="352">
+      <c r="A352" t="inlineStr">
+        <is>
+          <t>18:51:25</t>
+        </is>
+      </c>
+      <c r="B352" t="inlineStr">
+        <is>
+          <t>20:00</t>
+        </is>
+      </c>
+      <c r="C352" t="inlineStr">
+        <is>
+          <t>81_EL PELIGRO</t>
+        </is>
+      </c>
+      <c r="D352" t="n">
+        <v>69</v>
+      </c>
+      <c r="E352" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="353">
+      <c r="A353" t="inlineStr">
+        <is>
+          <t>18:51:25</t>
+        </is>
+      </c>
+      <c r="B353" t="inlineStr">
+        <is>
+          <t>20:11</t>
+        </is>
+      </c>
+      <c r="C353" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D353" t="n">
+        <v>80</v>
+      </c>
+      <c r="E353" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="354">
+      <c r="A354" t="inlineStr">
+        <is>
+          <t>18:51:25</t>
+        </is>
+      </c>
+      <c r="B354" t="inlineStr">
+        <is>
+          <t>20:15</t>
+        </is>
+      </c>
+      <c r="C354" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D354" t="n">
+        <v>84</v>
+      </c>
+      <c r="E354" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="355">
+      <c r="A355" t="inlineStr">
+        <is>
+          <t>18:51:25</t>
+        </is>
+      </c>
+      <c r="B355" t="inlineStr">
         <is>
           <t>20:27</t>
         </is>
       </c>
-      <c r="C349" t="inlineStr">
+      <c r="C355" t="inlineStr">
         <is>
           <t>10_OLMOS</t>
         </is>
       </c>
-      <c r="D349" t="n">
-        <v>112</v>
-      </c>
-      <c r="E349" t="inlineStr">
+      <c r="D355" t="n">
+        <v>96</v>
+      </c>
+      <c r="E355" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="356">
+      <c r="A356" t="inlineStr">
+        <is>
+          <t>18:51:25</t>
+        </is>
+      </c>
+      <c r="B356" t="inlineStr">
+        <is>
+          <t>20:35</t>
+        </is>
+      </c>
+      <c r="C356" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D356" t="n">
+        <v>104</v>
+      </c>
+      <c r="E356" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="357">
+      <c r="A357" t="inlineStr">
+        <is>
+          <t>18:51:25</t>
+        </is>
+      </c>
+      <c r="B357" t="inlineStr">
+        <is>
+          <t>20:44</t>
+        </is>
+      </c>
+      <c r="C357" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D357" t="n">
+        <v>113</v>
+      </c>
+      <c r="E357" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -9081,7 +9281,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E56"/>
+  <dimension ref="A1:E57"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -9094,14 +9294,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 18:35:14</t>
+          <t>Última actualización: 18:51:25</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 51</t>
+          <t>Total filas: 52</t>
         </is>
       </c>
     </row>
@@ -10335,7 +10535,7 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>18:35:14</t>
+          <t>18:51:25</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
@@ -10349,7 +10549,7 @@
         </is>
       </c>
       <c r="D54" t="n">
-        <v>49</v>
+        <v>33</v>
       </c>
       <c r="E54" t="inlineStr">
         <is>
@@ -10360,7 +10560,7 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>18:35:14</t>
+          <t>18:51:25</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
@@ -10374,7 +10574,7 @@
         </is>
       </c>
       <c r="D55" t="n">
-        <v>61</v>
+        <v>45</v>
       </c>
       <c r="E55" t="inlineStr">
         <is>
@@ -10385,7 +10585,7 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>18:35:14</t>
+          <t>18:51:25</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
@@ -10399,9 +10599,34 @@
         </is>
       </c>
       <c r="D56" t="n">
-        <v>100</v>
+        <v>84</v>
       </c>
       <c r="E56" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>18:51:25</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>20:44</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D57" t="n">
+        <v>113</v>
+      </c>
+      <c r="E57" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -10418,7 +10643,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E58"/>
+  <dimension ref="A1:E59"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -10431,14 +10656,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 18:35:14</t>
+          <t>Última actualización: 18:51:25</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 53</t>
+          <t>Total filas: 54</t>
         </is>
       </c>
     </row>
@@ -11772,7 +11997,7 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>18:35:14</t>
+          <t>18:51:25</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
@@ -11786,11 +12011,36 @@
         </is>
       </c>
       <c r="D58" t="n">
-        <v>43</v>
+        <v>27</v>
       </c>
       <c r="E58" t="inlineStr">
         <is>
           <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>18:51:25</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>20:45</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D59" t="n">
+        <v>114</v>
+      </c>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>L6203</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 1824
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-03-21.xlsx
+++ b/data/horarios-141-2026-03-21.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E357"/>
+  <dimension ref="A1:E369"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 18:51:25</t>
+          <t>Última actualización: 19:12:47</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 352</t>
+          <t>Total filas: 364</t>
         </is>
       </c>
     </row>
@@ -1158,7 +1158,7 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D33" t="n">
@@ -1183,7 +1183,7 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D34" t="n">
@@ -1558,7 +1558,7 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D49" t="n">
@@ -1583,7 +1583,7 @@
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D50" t="n">
@@ -1898,7 +1898,7 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>06:59:30</t>
+          <t>08:14:14</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
@@ -1908,11 +1908,11 @@
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D63" t="n">
-        <v>75</v>
+        <v>0</v>
       </c>
       <c r="E63" t="inlineStr">
         <is>
@@ -1923,7 +1923,7 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>08:14:14</t>
+          <t>06:59:30</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
@@ -1933,11 +1933,11 @@
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D64" t="n">
-        <v>0</v>
+        <v>75</v>
       </c>
       <c r="E64" t="inlineStr">
         <is>
@@ -1973,7 +1973,7 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>07:51:37</t>
+          <t>07:27:35</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
@@ -1983,11 +1983,11 @@
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D66" t="n">
-        <v>28</v>
+        <v>52</v>
       </c>
       <c r="E66" t="inlineStr">
         <is>
@@ -2023,7 +2023,7 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>07:27:35</t>
+          <t>07:51:37</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
@@ -2033,11 +2033,11 @@
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D68" t="n">
-        <v>52</v>
+        <v>28</v>
       </c>
       <c r="E68" t="inlineStr">
         <is>
@@ -2233,7 +2233,7 @@
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D76" t="n">
@@ -2258,7 +2258,7 @@
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D77" t="n">
@@ -2373,7 +2373,7 @@
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>08:50:55</t>
+          <t>07:27:35</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
@@ -2383,11 +2383,11 @@
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D82" t="n">
-        <v>1</v>
+        <v>84</v>
       </c>
       <c r="E82" t="inlineStr">
         <is>
@@ -2398,7 +2398,7 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>07:27:35</t>
+          <t>08:50:55</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
@@ -2408,11 +2408,11 @@
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D83" t="n">
-        <v>84</v>
+        <v>1</v>
       </c>
       <c r="E83" t="inlineStr">
         <is>
@@ -2698,7 +2698,7 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>08:14:14</t>
+          <t>08:50:55</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
@@ -2708,11 +2708,11 @@
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>215_EL PELIGRO</t>
         </is>
       </c>
       <c r="D95" t="n">
-        <v>64</v>
+        <v>28</v>
       </c>
       <c r="E95" t="inlineStr">
         <is>
@@ -2733,7 +2733,7 @@
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>215_EL PELIGRO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D96" t="n">
@@ -2748,7 +2748,7 @@
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>08:50:55</t>
+          <t>08:14:14</t>
         </is>
       </c>
       <c r="B97" t="inlineStr">
@@ -2758,11 +2758,11 @@
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D97" t="n">
-        <v>28</v>
+        <v>64</v>
       </c>
       <c r="E97" t="inlineStr">
         <is>
@@ -2873,7 +2873,7 @@
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>07:51:37</t>
+          <t>08:36:09</t>
         </is>
       </c>
       <c r="B102" t="inlineStr">
@@ -2883,11 +2883,11 @@
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D102" t="n">
-        <v>98</v>
+        <v>53</v>
       </c>
       <c r="E102" t="inlineStr">
         <is>
@@ -2898,7 +2898,7 @@
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>08:36:09</t>
+          <t>07:51:37</t>
         </is>
       </c>
       <c r="B103" t="inlineStr">
@@ -2908,11 +2908,11 @@
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D103" t="n">
-        <v>53</v>
+        <v>98</v>
       </c>
       <c r="E103" t="inlineStr">
         <is>
@@ -3083,7 +3083,7 @@
       </c>
       <c r="C110" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D110" t="n">
@@ -3108,7 +3108,7 @@
       </c>
       <c r="C111" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D111" t="n">
@@ -3173,7 +3173,7 @@
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>08:50:55</t>
+          <t>09:23:24</t>
         </is>
       </c>
       <c r="B114" t="inlineStr">
@@ -3183,11 +3183,11 @@
       </c>
       <c r="C114" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D114" t="n">
-        <v>73</v>
+        <v>40</v>
       </c>
       <c r="E114" t="inlineStr">
         <is>
@@ -3198,7 +3198,7 @@
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>09:23:24</t>
+          <t>08:50:55</t>
         </is>
       </c>
       <c r="B115" t="inlineStr">
@@ -3208,11 +3208,11 @@
       </c>
       <c r="C115" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D115" t="n">
-        <v>40</v>
+        <v>73</v>
       </c>
       <c r="E115" t="inlineStr">
         <is>
@@ -3498,7 +3498,7 @@
     <row r="127">
       <c r="A127" t="inlineStr">
         <is>
-          <t>08:36:09</t>
+          <t>10:14:52</t>
         </is>
       </c>
       <c r="B127" t="inlineStr">
@@ -3508,11 +3508,11 @@
       </c>
       <c r="C127" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D127" t="n">
-        <v>117</v>
+        <v>19</v>
       </c>
       <c r="E127" t="inlineStr">
         <is>
@@ -3523,7 +3523,7 @@
     <row r="128">
       <c r="A128" t="inlineStr">
         <is>
-          <t>10:14:52</t>
+          <t>08:36:09</t>
         </is>
       </c>
       <c r="B128" t="inlineStr">
@@ -3533,11 +3533,11 @@
       </c>
       <c r="C128" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D128" t="n">
-        <v>19</v>
+        <v>117</v>
       </c>
       <c r="E128" t="inlineStr">
         <is>
@@ -4183,7 +4183,7 @@
       </c>
       <c r="C154" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D154" t="n">
@@ -4208,7 +4208,7 @@
       </c>
       <c r="C155" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D155" t="n">
@@ -4673,7 +4673,7 @@
     <row r="174">
       <c r="A174" t="inlineStr">
         <is>
-          <t>12:28:38</t>
+          <t>12:00:15</t>
         </is>
       </c>
       <c r="B174" t="inlineStr">
@@ -4683,11 +4683,11 @@
       </c>
       <c r="C174" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D174" t="n">
-        <v>5</v>
+        <v>33</v>
       </c>
       <c r="E174" t="inlineStr">
         <is>
@@ -4698,7 +4698,7 @@
     <row r="175">
       <c r="A175" t="inlineStr">
         <is>
-          <t>12:00:15</t>
+          <t>12:28:38</t>
         </is>
       </c>
       <c r="B175" t="inlineStr">
@@ -4708,11 +4708,11 @@
       </c>
       <c r="C175" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D175" t="n">
-        <v>33</v>
+        <v>5</v>
       </c>
       <c r="E175" t="inlineStr">
         <is>
@@ -5033,7 +5033,7 @@
       </c>
       <c r="C188" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D188" t="n">
@@ -5058,7 +5058,7 @@
       </c>
       <c r="C189" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D189" t="n">
@@ -5073,7 +5073,7 @@
     <row r="190">
       <c r="A190" t="inlineStr">
         <is>
-          <t>13:00:14</t>
+          <t>12:48:06</t>
         </is>
       </c>
       <c r="B190" t="inlineStr">
@@ -5083,11 +5083,11 @@
       </c>
       <c r="C190" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D190" t="n">
-        <v>4</v>
+        <v>16</v>
       </c>
       <c r="E190" t="inlineStr">
         <is>
@@ -5098,7 +5098,7 @@
     <row r="191">
       <c r="A191" t="inlineStr">
         <is>
-          <t>12:48:06</t>
+          <t>13:00:14</t>
         </is>
       </c>
       <c r="B191" t="inlineStr">
@@ -5108,11 +5108,11 @@
       </c>
       <c r="C191" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D191" t="n">
-        <v>16</v>
+        <v>4</v>
       </c>
       <c r="E191" t="inlineStr">
         <is>
@@ -5248,7 +5248,7 @@
     <row r="197">
       <c r="A197" t="inlineStr">
         <is>
-          <t>12:48:06</t>
+          <t>13:00:14</t>
         </is>
       </c>
       <c r="B197" t="inlineStr">
@@ -5258,11 +5258,11 @@
       </c>
       <c r="C197" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D197" t="n">
-        <v>45</v>
+        <v>33</v>
       </c>
       <c r="E197" t="inlineStr">
         <is>
@@ -5273,7 +5273,7 @@
     <row r="198">
       <c r="A198" t="inlineStr">
         <is>
-          <t>13:00:14</t>
+          <t>12:48:06</t>
         </is>
       </c>
       <c r="B198" t="inlineStr">
@@ -5283,11 +5283,11 @@
       </c>
       <c r="C198" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D198" t="n">
-        <v>33</v>
+        <v>45</v>
       </c>
       <c r="E198" t="inlineStr">
         <is>
@@ -5498,7 +5498,7 @@
     <row r="207">
       <c r="A207" t="inlineStr">
         <is>
-          <t>13:32:57</t>
+          <t>13:57:43</t>
         </is>
       </c>
       <c r="B207" t="inlineStr">
@@ -5508,11 +5508,11 @@
       </c>
       <c r="C207" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D207" t="n">
-        <v>27</v>
+        <v>2</v>
       </c>
       <c r="E207" t="inlineStr">
         <is>
@@ -5523,7 +5523,7 @@
     <row r="208">
       <c r="A208" t="inlineStr">
         <is>
-          <t>13:57:43</t>
+          <t>13:32:57</t>
         </is>
       </c>
       <c r="B208" t="inlineStr">
@@ -5533,11 +5533,11 @@
       </c>
       <c r="C208" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D208" t="n">
-        <v>2</v>
+        <v>27</v>
       </c>
       <c r="E208" t="inlineStr">
         <is>
@@ -5623,7 +5623,7 @@
     <row r="212">
       <c r="A212" t="inlineStr">
         <is>
-          <t>13:32:57</t>
+          <t>13:57:43</t>
         </is>
       </c>
       <c r="B212" t="inlineStr">
@@ -5633,11 +5633,11 @@
       </c>
       <c r="C212" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D212" t="n">
-        <v>44</v>
+        <v>19</v>
       </c>
       <c r="E212" t="inlineStr">
         <is>
@@ -5648,7 +5648,7 @@
     <row r="213">
       <c r="A213" t="inlineStr">
         <is>
-          <t>13:57:43</t>
+          <t>13:32:57</t>
         </is>
       </c>
       <c r="B213" t="inlineStr">
@@ -5658,11 +5658,11 @@
       </c>
       <c r="C213" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D213" t="n">
-        <v>19</v>
+        <v>44</v>
       </c>
       <c r="E213" t="inlineStr">
         <is>
@@ -5673,7 +5673,7 @@
     <row r="214">
       <c r="A214" t="inlineStr">
         <is>
-          <t>13:00:14</t>
+          <t>13:57:43</t>
         </is>
       </c>
       <c r="B214" t="inlineStr">
@@ -5683,11 +5683,11 @@
       </c>
       <c r="C214" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D214" t="n">
-        <v>77</v>
+        <v>20</v>
       </c>
       <c r="E214" t="inlineStr">
         <is>
@@ -5698,7 +5698,7 @@
     <row r="215">
       <c r="A215" t="inlineStr">
         <is>
-          <t>13:57:43</t>
+          <t>13:00:14</t>
         </is>
       </c>
       <c r="B215" t="inlineStr">
@@ -5708,11 +5708,11 @@
       </c>
       <c r="C215" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D215" t="n">
-        <v>20</v>
+        <v>77</v>
       </c>
       <c r="E215" t="inlineStr">
         <is>
@@ -5983,7 +5983,7 @@
       </c>
       <c r="C226" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D226" t="n">
@@ -6008,7 +6008,7 @@
       </c>
       <c r="C227" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D227" t="n">
@@ -6173,7 +6173,7 @@
     <row r="234">
       <c r="A234" t="inlineStr">
         <is>
-          <t>14:46:39</t>
+          <t>14:59:00</t>
         </is>
       </c>
       <c r="B234" t="inlineStr">
@@ -6183,11 +6183,11 @@
       </c>
       <c r="C234" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D234" t="n">
-        <v>15</v>
+        <v>2</v>
       </c>
       <c r="E234" t="inlineStr">
         <is>
@@ -6198,7 +6198,7 @@
     <row r="235">
       <c r="A235" t="inlineStr">
         <is>
-          <t>14:59:00</t>
+          <t>14:46:39</t>
         </is>
       </c>
       <c r="B235" t="inlineStr">
@@ -6208,11 +6208,11 @@
       </c>
       <c r="C235" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D235" t="n">
-        <v>2</v>
+        <v>15</v>
       </c>
       <c r="E235" t="inlineStr">
         <is>
@@ -6933,7 +6933,7 @@
       </c>
       <c r="C264" t="inlineStr">
         <is>
-          <t>215_ALUAR</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D264" t="n">
@@ -6958,7 +6958,7 @@
       </c>
       <c r="C265" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>215_ALUAR</t>
         </is>
       </c>
       <c r="D265" t="n">
@@ -7033,7 +7033,7 @@
       </c>
       <c r="C268" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D268" t="n">
@@ -7058,7 +7058,7 @@
       </c>
       <c r="C269" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D269" t="n">
@@ -7073,7 +7073,7 @@
     <row r="270">
       <c r="A270" t="inlineStr">
         <is>
-          <t>16:01:44</t>
+          <t>16:33:34</t>
         </is>
       </c>
       <c r="B270" t="inlineStr">
@@ -7083,11 +7083,11 @@
       </c>
       <c r="C270" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D270" t="n">
-        <v>34</v>
+        <v>2</v>
       </c>
       <c r="E270" t="inlineStr">
         <is>
@@ -7098,7 +7098,7 @@
     <row r="271">
       <c r="A271" t="inlineStr">
         <is>
-          <t>16:33:34</t>
+          <t>16:01:44</t>
         </is>
       </c>
       <c r="B271" t="inlineStr">
@@ -7108,11 +7108,11 @@
       </c>
       <c r="C271" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D271" t="n">
-        <v>2</v>
+        <v>34</v>
       </c>
       <c r="E271" t="inlineStr">
         <is>
@@ -7383,7 +7383,7 @@
       </c>
       <c r="C282" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D282" t="n">
@@ -7408,7 +7408,7 @@
       </c>
       <c r="C283" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D283" t="n">
@@ -7948,7 +7948,7 @@
     <row r="305">
       <c r="A305" t="inlineStr">
         <is>
-          <t>17:47:19</t>
+          <t>16:57:49</t>
         </is>
       </c>
       <c r="B305" t="inlineStr">
@@ -7958,11 +7958,11 @@
       </c>
       <c r="C305" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D305" t="n">
-        <v>12</v>
+        <v>62</v>
       </c>
       <c r="E305" t="inlineStr">
         <is>
@@ -7973,7 +7973,7 @@
     <row r="306">
       <c r="A306" t="inlineStr">
         <is>
-          <t>16:57:49</t>
+          <t>17:47:19</t>
         </is>
       </c>
       <c r="B306" t="inlineStr">
@@ -7983,11 +7983,11 @@
       </c>
       <c r="C306" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D306" t="n">
-        <v>62</v>
+        <v>12</v>
       </c>
       <c r="E306" t="inlineStr">
         <is>
@@ -8008,7 +8008,7 @@
       </c>
       <c r="C307" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D307" t="n">
@@ -8033,7 +8033,7 @@
       </c>
       <c r="C308" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D308" t="n">
@@ -8083,7 +8083,7 @@
       </c>
       <c r="C310" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D310" t="n">
@@ -8108,7 +8108,7 @@
       </c>
       <c r="C311" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D311" t="n">
@@ -8158,7 +8158,7 @@
       </c>
       <c r="C313" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D313" t="n">
@@ -8183,7 +8183,7 @@
       </c>
       <c r="C314" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D314" t="n">
@@ -8773,21 +8773,21 @@
     <row r="338">
       <c r="A338" t="inlineStr">
         <is>
-          <t>18:51:25</t>
+          <t>19:12:47</t>
         </is>
       </c>
       <c r="B338" t="inlineStr">
         <is>
-          <t>19:16</t>
+          <t>19:13</t>
         </is>
       </c>
       <c r="C338" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>81_EL PELIGRO</t>
         </is>
       </c>
       <c r="D338" t="n">
-        <v>25</v>
+        <v>1</v>
       </c>
       <c r="E338" t="inlineStr">
         <is>
@@ -8798,21 +8798,21 @@
     <row r="339">
       <c r="A339" t="inlineStr">
         <is>
-          <t>18:35:14</t>
+          <t>19:12:47</t>
         </is>
       </c>
       <c r="B339" t="inlineStr">
         <is>
-          <t>19:17</t>
+          <t>19:15</t>
         </is>
       </c>
       <c r="C339" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>225_GOMEZ</t>
         </is>
       </c>
       <c r="D339" t="n">
-        <v>42</v>
+        <v>3</v>
       </c>
       <c r="E339" t="inlineStr">
         <is>
@@ -8823,12 +8823,12 @@
     <row r="340">
       <c r="A340" t="inlineStr">
         <is>
-          <t>17:47:19</t>
+          <t>19:12:47</t>
         </is>
       </c>
       <c r="B340" t="inlineStr">
         <is>
-          <t>19:20</t>
+          <t>19:16</t>
         </is>
       </c>
       <c r="C340" t="inlineStr">
@@ -8837,7 +8837,7 @@
         </is>
       </c>
       <c r="D340" t="n">
-        <v>93</v>
+        <v>4</v>
       </c>
       <c r="E340" t="inlineStr">
         <is>
@@ -8848,21 +8848,21 @@
     <row r="341">
       <c r="A341" t="inlineStr">
         <is>
-          <t>18:51:25</t>
+          <t>18:35:14</t>
         </is>
       </c>
       <c r="B341" t="inlineStr">
         <is>
-          <t>19:21</t>
+          <t>19:17</t>
         </is>
       </c>
       <c r="C341" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D341" t="n">
-        <v>30</v>
+        <v>42</v>
       </c>
       <c r="E341" t="inlineStr">
         <is>
@@ -8873,21 +8873,21 @@
     <row r="342">
       <c r="A342" t="inlineStr">
         <is>
-          <t>18:51:25</t>
+          <t>17:47:19</t>
         </is>
       </c>
       <c r="B342" t="inlineStr">
         <is>
-          <t>19:23</t>
+          <t>19:20</t>
         </is>
       </c>
       <c r="C342" t="inlineStr">
         <is>
-          <t>225_GOMEZ</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D342" t="n">
-        <v>32</v>
+        <v>93</v>
       </c>
       <c r="E342" t="inlineStr">
         <is>
@@ -8898,21 +8898,21 @@
     <row r="343">
       <c r="A343" t="inlineStr">
         <is>
-          <t>18:51:25</t>
+          <t>19:12:47</t>
         </is>
       </c>
       <c r="B343" t="inlineStr">
         <is>
-          <t>19:24</t>
+          <t>19:21</t>
         </is>
       </c>
       <c r="C343" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D343" t="n">
-        <v>33</v>
+        <v>9</v>
       </c>
       <c r="E343" t="inlineStr">
         <is>
@@ -8923,21 +8923,21 @@
     <row r="344">
       <c r="A344" t="inlineStr">
         <is>
-          <t>18:51:25</t>
+          <t>19:12:47</t>
         </is>
       </c>
       <c r="B344" t="inlineStr">
         <is>
-          <t>19:36</t>
+          <t>19:23</t>
         </is>
       </c>
       <c r="C344" t="inlineStr">
         <is>
-          <t>215_EL PELIGRO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D344" t="n">
-        <v>45</v>
+        <v>11</v>
       </c>
       <c r="E344" t="inlineStr">
         <is>
@@ -8948,21 +8948,21 @@
     <row r="345">
       <c r="A345" t="inlineStr">
         <is>
-          <t>18:35:14</t>
+          <t>18:51:25</t>
         </is>
       </c>
       <c r="B345" t="inlineStr">
         <is>
-          <t>19:38</t>
+          <t>19:23</t>
         </is>
       </c>
       <c r="C345" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>225_GOMEZ</t>
         </is>
       </c>
       <c r="D345" t="n">
-        <v>63</v>
+        <v>32</v>
       </c>
       <c r="E345" t="inlineStr">
         <is>
@@ -8978,16 +8978,16 @@
       </c>
       <c r="B346" t="inlineStr">
         <is>
-          <t>19:40</t>
+          <t>19:24</t>
         </is>
       </c>
       <c r="C346" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D346" t="n">
-        <v>49</v>
+        <v>33</v>
       </c>
       <c r="E346" t="inlineStr">
         <is>
@@ -8998,21 +8998,21 @@
     <row r="347">
       <c r="A347" t="inlineStr">
         <is>
-          <t>18:51:25</t>
+          <t>19:12:47</t>
         </is>
       </c>
       <c r="B347" t="inlineStr">
         <is>
-          <t>19:40</t>
+          <t>19:31</t>
         </is>
       </c>
       <c r="C347" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D347" t="n">
-        <v>49</v>
+        <v>19</v>
       </c>
       <c r="E347" t="inlineStr">
         <is>
@@ -9023,21 +9023,21 @@
     <row r="348">
       <c r="A348" t="inlineStr">
         <is>
-          <t>18:51:25</t>
+          <t>19:12:47</t>
         </is>
       </c>
       <c r="B348" t="inlineStr">
         <is>
-          <t>19:47</t>
+          <t>19:35</t>
         </is>
       </c>
       <c r="C348" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>215_EL PELIGRO</t>
         </is>
       </c>
       <c r="D348" t="n">
-        <v>56</v>
+        <v>23</v>
       </c>
       <c r="E348" t="inlineStr">
         <is>
@@ -9053,16 +9053,16 @@
       </c>
       <c r="B349" t="inlineStr">
         <is>
-          <t>19:53</t>
+          <t>19:36</t>
         </is>
       </c>
       <c r="C349" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>215_EL PELIGRO</t>
         </is>
       </c>
       <c r="D349" t="n">
-        <v>62</v>
+        <v>45</v>
       </c>
       <c r="E349" t="inlineStr">
         <is>
@@ -9073,17 +9073,17 @@
     <row r="350">
       <c r="A350" t="inlineStr">
         <is>
-          <t>18:51:25</t>
+          <t>18:35:14</t>
         </is>
       </c>
       <c r="B350" t="inlineStr">
         <is>
-          <t>19:54</t>
+          <t>19:38</t>
         </is>
       </c>
       <c r="C350" t="inlineStr">
         <is>
-          <t>14X44_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D350" t="n">
@@ -9098,21 +9098,21 @@
     <row r="351">
       <c r="A351" t="inlineStr">
         <is>
-          <t>18:35:14</t>
+          <t>19:12:47</t>
         </is>
       </c>
       <c r="B351" t="inlineStr">
         <is>
-          <t>19:55</t>
+          <t>19:40</t>
         </is>
       </c>
       <c r="C351" t="inlineStr">
         <is>
-          <t>14X44_ABASTO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D351" t="n">
-        <v>80</v>
+        <v>28</v>
       </c>
       <c r="E351" t="inlineStr">
         <is>
@@ -9128,16 +9128,16 @@
       </c>
       <c r="B352" t="inlineStr">
         <is>
-          <t>20:00</t>
+          <t>19:40</t>
         </is>
       </c>
       <c r="C352" t="inlineStr">
         <is>
-          <t>81_EL PELIGRO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D352" t="n">
-        <v>69</v>
+        <v>49</v>
       </c>
       <c r="E352" t="inlineStr">
         <is>
@@ -9148,21 +9148,21 @@
     <row r="353">
       <c r="A353" t="inlineStr">
         <is>
-          <t>18:51:25</t>
+          <t>19:12:47</t>
         </is>
       </c>
       <c r="B353" t="inlineStr">
         <is>
-          <t>20:11</t>
+          <t>19:41</t>
         </is>
       </c>
       <c r="C353" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D353" t="n">
-        <v>80</v>
+        <v>29</v>
       </c>
       <c r="E353" t="inlineStr">
         <is>
@@ -9173,21 +9173,21 @@
     <row r="354">
       <c r="A354" t="inlineStr">
         <is>
-          <t>18:51:25</t>
+          <t>19:12:47</t>
         </is>
       </c>
       <c r="B354" t="inlineStr">
         <is>
-          <t>20:15</t>
+          <t>19:47</t>
         </is>
       </c>
       <c r="C354" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D354" t="n">
-        <v>84</v>
+        <v>35</v>
       </c>
       <c r="E354" t="inlineStr">
         <is>
@@ -9198,21 +9198,21 @@
     <row r="355">
       <c r="A355" t="inlineStr">
         <is>
-          <t>18:51:25</t>
+          <t>19:12:47</t>
         </is>
       </c>
       <c r="B355" t="inlineStr">
         <is>
-          <t>20:27</t>
+          <t>19:53</t>
         </is>
       </c>
       <c r="C355" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D355" t="n">
-        <v>96</v>
+        <v>41</v>
       </c>
       <c r="E355" t="inlineStr">
         <is>
@@ -9223,21 +9223,21 @@
     <row r="356">
       <c r="A356" t="inlineStr">
         <is>
-          <t>18:51:25</t>
+          <t>19:12:47</t>
         </is>
       </c>
       <c r="B356" t="inlineStr">
         <is>
-          <t>20:35</t>
+          <t>19:54</t>
         </is>
       </c>
       <c r="C356" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>14X44_ABASTO</t>
         </is>
       </c>
       <c r="D356" t="n">
-        <v>104</v>
+        <v>42</v>
       </c>
       <c r="E356" t="inlineStr">
         <is>
@@ -9248,23 +9248,323 @@
     <row r="357">
       <c r="A357" t="inlineStr">
         <is>
+          <t>18:35:14</t>
+        </is>
+      </c>
+      <c r="B357" t="inlineStr">
+        <is>
+          <t>19:55</t>
+        </is>
+      </c>
+      <c r="C357" t="inlineStr">
+        <is>
+          <t>14X44_ABASTO</t>
+        </is>
+      </c>
+      <c r="D357" t="n">
+        <v>80</v>
+      </c>
+      <c r="E357" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="358">
+      <c r="A358" t="inlineStr">
+        <is>
+          <t>19:12:47</t>
+        </is>
+      </c>
+      <c r="B358" t="inlineStr">
+        <is>
+          <t>20:00</t>
+        </is>
+      </c>
+      <c r="C358" t="inlineStr">
+        <is>
+          <t>81_EL PELIGRO</t>
+        </is>
+      </c>
+      <c r="D358" t="n">
+        <v>48</v>
+      </c>
+      <c r="E358" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="359">
+      <c r="A359" t="inlineStr">
+        <is>
+          <t>19:12:47</t>
+        </is>
+      </c>
+      <c r="B359" t="inlineStr">
+        <is>
+          <t>20:10</t>
+        </is>
+      </c>
+      <c r="C359" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D359" t="n">
+        <v>58</v>
+      </c>
+      <c r="E359" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="360">
+      <c r="A360" t="inlineStr">
+        <is>
+          <t>19:12:47</t>
+        </is>
+      </c>
+      <c r="B360" t="inlineStr">
+        <is>
+          <t>20:11</t>
+        </is>
+      </c>
+      <c r="C360" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D360" t="n">
+        <v>59</v>
+      </c>
+      <c r="E360" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="361">
+      <c r="A361" t="inlineStr">
+        <is>
+          <t>19:12:47</t>
+        </is>
+      </c>
+      <c r="B361" t="inlineStr">
+        <is>
+          <t>20:14</t>
+        </is>
+      </c>
+      <c r="C361" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D361" t="n">
+        <v>62</v>
+      </c>
+      <c r="E361" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="362">
+      <c r="A362" t="inlineStr">
+        <is>
           <t>18:51:25</t>
         </is>
       </c>
-      <c r="B357" t="inlineStr">
+      <c r="B362" t="inlineStr">
+        <is>
+          <t>20:15</t>
+        </is>
+      </c>
+      <c r="C362" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D362" t="n">
+        <v>84</v>
+      </c>
+      <c r="E362" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="363">
+      <c r="A363" t="inlineStr">
+        <is>
+          <t>19:12:47</t>
+        </is>
+      </c>
+      <c r="B363" t="inlineStr">
+        <is>
+          <t>20:26</t>
+        </is>
+      </c>
+      <c r="C363" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D363" t="n">
+        <v>74</v>
+      </c>
+      <c r="E363" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="364">
+      <c r="A364" t="inlineStr">
+        <is>
+          <t>18:51:25</t>
+        </is>
+      </c>
+      <c r="B364" t="inlineStr">
+        <is>
+          <t>20:27</t>
+        </is>
+      </c>
+      <c r="C364" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D364" t="n">
+        <v>96</v>
+      </c>
+      <c r="E364" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="365">
+      <c r="A365" t="inlineStr">
+        <is>
+          <t>19:12:47</t>
+        </is>
+      </c>
+      <c r="B365" t="inlineStr">
+        <is>
+          <t>20:34</t>
+        </is>
+      </c>
+      <c r="C365" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D365" t="n">
+        <v>82</v>
+      </c>
+      <c r="E365" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="366">
+      <c r="A366" t="inlineStr">
+        <is>
+          <t>18:51:25</t>
+        </is>
+      </c>
+      <c r="B366" t="inlineStr">
+        <is>
+          <t>20:35</t>
+        </is>
+      </c>
+      <c r="C366" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D366" t="n">
+        <v>104</v>
+      </c>
+      <c r="E366" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="367">
+      <c r="A367" t="inlineStr">
+        <is>
+          <t>19:12:47</t>
+        </is>
+      </c>
+      <c r="B367" t="inlineStr">
         <is>
           <t>20:44</t>
         </is>
       </c>
-      <c r="C357" t="inlineStr">
+      <c r="C367" t="inlineStr">
         <is>
           <t>215B_EL PATO</t>
         </is>
       </c>
-      <c r="D357" t="n">
-        <v>113</v>
-      </c>
-      <c r="E357" t="inlineStr">
+      <c r="D367" t="n">
+        <v>92</v>
+      </c>
+      <c r="E367" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="368">
+      <c r="A368" t="inlineStr">
+        <is>
+          <t>19:12:47</t>
+        </is>
+      </c>
+      <c r="B368" t="inlineStr">
+        <is>
+          <t>20:55</t>
+        </is>
+      </c>
+      <c r="C368" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D368" t="n">
+        <v>103</v>
+      </c>
+      <c r="E368" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="369">
+      <c r="A369" t="inlineStr">
+        <is>
+          <t>19:12:47</t>
+        </is>
+      </c>
+      <c r="B369" t="inlineStr">
+        <is>
+          <t>20:56</t>
+        </is>
+      </c>
+      <c r="C369" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D369" t="n">
+        <v>104</v>
+      </c>
+      <c r="E369" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -9281,7 +9581,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E57"/>
+  <dimension ref="A1:E61"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -9294,14 +9594,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 18:51:25</t>
+          <t>Última actualización: 19:12:47</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 52</t>
+          <t>Total filas: 56</t>
         </is>
       </c>
     </row>
@@ -10535,12 +10835,12 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>18:51:25</t>
+          <t>19:12:47</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>19:24</t>
+          <t>19:23</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
@@ -10549,7 +10849,7 @@
         </is>
       </c>
       <c r="D54" t="n">
-        <v>33</v>
+        <v>11</v>
       </c>
       <c r="E54" t="inlineStr">
         <is>
@@ -10565,16 +10865,16 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>19:36</t>
+          <t>19:24</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>215_EL PELIGRO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D55" t="n">
-        <v>45</v>
+        <v>33</v>
       </c>
       <c r="E55" t="inlineStr">
         <is>
@@ -10585,21 +10885,21 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>18:51:25</t>
+          <t>19:12:47</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>20:15</t>
+          <t>19:35</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>215_EL PELIGRO</t>
         </is>
       </c>
       <c r="D56" t="n">
-        <v>84</v>
+        <v>23</v>
       </c>
       <c r="E56" t="inlineStr">
         <is>
@@ -10615,18 +10915,118 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
+          <t>19:36</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>215_EL PELIGRO</t>
+        </is>
+      </c>
+      <c r="D57" t="n">
+        <v>45</v>
+      </c>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>19:12:47</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>20:14</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D58" t="n">
+        <v>62</v>
+      </c>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>18:51:25</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>20:15</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D59" t="n">
+        <v>84</v>
+      </c>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>19:12:47</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
           <t>20:44</t>
         </is>
       </c>
-      <c r="C57" t="inlineStr">
+      <c r="C60" t="inlineStr">
         <is>
           <t>215B_EL PATO</t>
         </is>
       </c>
-      <c r="D57" t="n">
-        <v>113</v>
-      </c>
-      <c r="E57" t="inlineStr">
+      <c r="D60" t="n">
+        <v>92</v>
+      </c>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>19:12:47</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>20:55</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D61" t="n">
+        <v>103</v>
+      </c>
+      <c r="E61" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -10643,7 +11043,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E59"/>
+  <dimension ref="A1:E61"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -10656,14 +11056,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 18:51:25</t>
+          <t>Última actualización: 19:12:47</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 54</t>
+          <t>Total filas: 56</t>
         </is>
       </c>
     </row>
@@ -11997,12 +12397,12 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>18:51:25</t>
+          <t>19:12:47</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>19:18</t>
+          <t>19:17</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
@@ -12011,7 +12411,7 @@
         </is>
       </c>
       <c r="D58" t="n">
-        <v>27</v>
+        <v>5</v>
       </c>
       <c r="E58" t="inlineStr">
         <is>
@@ -12027,18 +12427,68 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
+          <t>19:18</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>215B_LP-P MOR-1 Y 57</t>
+        </is>
+      </c>
+      <c r="D59" t="n">
+        <v>27</v>
+      </c>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>19:12:47</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>20:44</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D60" t="n">
+        <v>92</v>
+      </c>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>18:51:25</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
           <t>20:45</t>
         </is>
       </c>
-      <c r="C59" t="inlineStr">
+      <c r="C61" t="inlineStr">
         <is>
           <t>215C_LA PLATA</t>
         </is>
       </c>
-      <c r="D59" t="n">
+      <c r="D61" t="n">
         <v>114</v>
       </c>
-      <c r="E59" t="inlineStr">
+      <c r="E61" t="inlineStr">
         <is>
           <t>L6203</t>
         </is>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 1825
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-03-21.xlsx
+++ b/data/horarios-141-2026-03-21.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E369"/>
+  <dimension ref="A1:E377"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 19:12:47</t>
+          <t>Última actualización: 19:44:03</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 364</t>
+          <t>Total filas: 372</t>
         </is>
       </c>
     </row>
@@ -1883,7 +1883,7 @@
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D62" t="n">
@@ -1898,7 +1898,7 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>08:14:14</t>
+          <t>06:59:30</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
@@ -1908,11 +1908,11 @@
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D63" t="n">
-        <v>0</v>
+        <v>75</v>
       </c>
       <c r="E63" t="inlineStr">
         <is>
@@ -1923,7 +1923,7 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>06:59:30</t>
+          <t>08:14:14</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
@@ -1933,11 +1933,11 @@
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D64" t="n">
-        <v>75</v>
+        <v>0</v>
       </c>
       <c r="E64" t="inlineStr">
         <is>
@@ -2008,7 +2008,7 @@
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D67" t="n">
@@ -2033,7 +2033,7 @@
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D68" t="n">
@@ -2233,7 +2233,7 @@
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D76" t="n">
@@ -2258,7 +2258,7 @@
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D77" t="n">
@@ -2373,7 +2373,7 @@
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>07:27:35</t>
+          <t>08:50:55</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
@@ -2383,11 +2383,11 @@
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D82" t="n">
-        <v>84</v>
+        <v>1</v>
       </c>
       <c r="E82" t="inlineStr">
         <is>
@@ -2423,7 +2423,7 @@
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>08:50:55</t>
+          <t>07:27:35</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
@@ -2433,11 +2433,11 @@
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D84" t="n">
-        <v>1</v>
+        <v>84</v>
       </c>
       <c r="E84" t="inlineStr">
         <is>
@@ -2873,7 +2873,7 @@
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>08:36:09</t>
+          <t>07:51:37</t>
         </is>
       </c>
       <c r="B102" t="inlineStr">
@@ -2883,11 +2883,11 @@
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D102" t="n">
-        <v>53</v>
+        <v>98</v>
       </c>
       <c r="E102" t="inlineStr">
         <is>
@@ -2898,7 +2898,7 @@
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>07:51:37</t>
+          <t>08:36:09</t>
         </is>
       </c>
       <c r="B103" t="inlineStr">
@@ -2908,11 +2908,11 @@
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D103" t="n">
-        <v>98</v>
+        <v>53</v>
       </c>
       <c r="E103" t="inlineStr">
         <is>
@@ -3498,7 +3498,7 @@
     <row r="127">
       <c r="A127" t="inlineStr">
         <is>
-          <t>10:14:52</t>
+          <t>08:36:09</t>
         </is>
       </c>
       <c r="B127" t="inlineStr">
@@ -3508,11 +3508,11 @@
       </c>
       <c r="C127" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D127" t="n">
-        <v>19</v>
+        <v>117</v>
       </c>
       <c r="E127" t="inlineStr">
         <is>
@@ -3523,7 +3523,7 @@
     <row r="128">
       <c r="A128" t="inlineStr">
         <is>
-          <t>08:36:09</t>
+          <t>10:14:52</t>
         </is>
       </c>
       <c r="B128" t="inlineStr">
@@ -3533,11 +3533,11 @@
       </c>
       <c r="C128" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D128" t="n">
-        <v>117</v>
+        <v>19</v>
       </c>
       <c r="E128" t="inlineStr">
         <is>
@@ -3598,7 +3598,7 @@
     <row r="131">
       <c r="A131" t="inlineStr">
         <is>
-          <t>09:23:24</t>
+          <t>10:14:52</t>
         </is>
       </c>
       <c r="B131" t="inlineStr">
@@ -3608,11 +3608,11 @@
       </c>
       <c r="C131" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D131" t="n">
-        <v>80</v>
+        <v>29</v>
       </c>
       <c r="E131" t="inlineStr">
         <is>
@@ -3623,7 +3623,7 @@
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t>10:14:52</t>
+          <t>09:23:24</t>
         </is>
       </c>
       <c r="B132" t="inlineStr">
@@ -3633,11 +3633,11 @@
       </c>
       <c r="C132" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D132" t="n">
-        <v>29</v>
+        <v>80</v>
       </c>
       <c r="E132" t="inlineStr">
         <is>
@@ -3873,7 +3873,7 @@
     <row r="142">
       <c r="A142" t="inlineStr">
         <is>
-          <t>10:14:52</t>
+          <t>10:52:37</t>
         </is>
       </c>
       <c r="B142" t="inlineStr">
@@ -3883,11 +3883,11 @@
       </c>
       <c r="C142" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D142" t="n">
-        <v>49</v>
+        <v>11</v>
       </c>
       <c r="E142" t="inlineStr">
         <is>
@@ -3898,7 +3898,7 @@
     <row r="143">
       <c r="A143" t="inlineStr">
         <is>
-          <t>10:52:37</t>
+          <t>10:14:52</t>
         </is>
       </c>
       <c r="B143" t="inlineStr">
@@ -3908,11 +3908,11 @@
       </c>
       <c r="C143" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D143" t="n">
-        <v>11</v>
+        <v>49</v>
       </c>
       <c r="E143" t="inlineStr">
         <is>
@@ -4183,7 +4183,7 @@
       </c>
       <c r="C154" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D154" t="n">
@@ -4208,7 +4208,7 @@
       </c>
       <c r="C155" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D155" t="n">
@@ -4473,7 +4473,7 @@
     <row r="166">
       <c r="A166" t="inlineStr">
         <is>
-          <t>12:00:15</t>
+          <t>11:16:36</t>
         </is>
       </c>
       <c r="B166" t="inlineStr">
@@ -4483,11 +4483,11 @@
       </c>
       <c r="C166" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D166" t="n">
-        <v>4</v>
+        <v>48</v>
       </c>
       <c r="E166" t="inlineStr">
         <is>
@@ -4498,7 +4498,7 @@
     <row r="167">
       <c r="A167" t="inlineStr">
         <is>
-          <t>11:16:36</t>
+          <t>12:00:15</t>
         </is>
       </c>
       <c r="B167" t="inlineStr">
@@ -4508,11 +4508,11 @@
       </c>
       <c r="C167" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D167" t="n">
-        <v>48</v>
+        <v>4</v>
       </c>
       <c r="E167" t="inlineStr">
         <is>
@@ -4648,7 +4648,7 @@
     <row r="173">
       <c r="A173" t="inlineStr">
         <is>
-          <t>12:28:38</t>
+          <t>12:00:15</t>
         </is>
       </c>
       <c r="B173" t="inlineStr">
@@ -4658,11 +4658,11 @@
       </c>
       <c r="C173" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D173" t="n">
-        <v>5</v>
+        <v>33</v>
       </c>
       <c r="E173" t="inlineStr">
         <is>
@@ -4673,7 +4673,7 @@
     <row r="174">
       <c r="A174" t="inlineStr">
         <is>
-          <t>12:00:15</t>
+          <t>12:28:38</t>
         </is>
       </c>
       <c r="B174" t="inlineStr">
@@ -4683,11 +4683,11 @@
       </c>
       <c r="C174" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D174" t="n">
-        <v>33</v>
+        <v>5</v>
       </c>
       <c r="E174" t="inlineStr">
         <is>
@@ -4708,7 +4708,7 @@
       </c>
       <c r="C175" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D175" t="n">
@@ -4998,7 +4998,7 @@
     <row r="187">
       <c r="A187" t="inlineStr">
         <is>
-          <t>13:00:14</t>
+          <t>12:28:38</t>
         </is>
       </c>
       <c r="B187" t="inlineStr">
@@ -5008,11 +5008,11 @@
       </c>
       <c r="C187" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D187" t="n">
-        <v>3</v>
+        <v>35</v>
       </c>
       <c r="E187" t="inlineStr">
         <is>
@@ -5023,7 +5023,7 @@
     <row r="188">
       <c r="A188" t="inlineStr">
         <is>
-          <t>12:28:38</t>
+          <t>13:00:14</t>
         </is>
       </c>
       <c r="B188" t="inlineStr">
@@ -5033,11 +5033,11 @@
       </c>
       <c r="C188" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D188" t="n">
-        <v>35</v>
+        <v>3</v>
       </c>
       <c r="E188" t="inlineStr">
         <is>
@@ -5058,7 +5058,7 @@
       </c>
       <c r="C189" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D189" t="n">
@@ -5248,7 +5248,7 @@
     <row r="197">
       <c r="A197" t="inlineStr">
         <is>
-          <t>13:00:14</t>
+          <t>12:48:06</t>
         </is>
       </c>
       <c r="B197" t="inlineStr">
@@ -5258,11 +5258,11 @@
       </c>
       <c r="C197" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D197" t="n">
-        <v>33</v>
+        <v>45</v>
       </c>
       <c r="E197" t="inlineStr">
         <is>
@@ -5273,7 +5273,7 @@
     <row r="198">
       <c r="A198" t="inlineStr">
         <is>
-          <t>12:48:06</t>
+          <t>13:00:14</t>
         </is>
       </c>
       <c r="B198" t="inlineStr">
@@ -5283,11 +5283,11 @@
       </c>
       <c r="C198" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D198" t="n">
-        <v>45</v>
+        <v>33</v>
       </c>
       <c r="E198" t="inlineStr">
         <is>
@@ -5323,7 +5323,7 @@
     <row r="200">
       <c r="A200" t="inlineStr">
         <is>
-          <t>13:00:14</t>
+          <t>12:48:06</t>
         </is>
       </c>
       <c r="B200" t="inlineStr">
@@ -5333,11 +5333,11 @@
       </c>
       <c r="C200" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D200" t="n">
-        <v>38</v>
+        <v>50</v>
       </c>
       <c r="E200" t="inlineStr">
         <is>
@@ -5348,7 +5348,7 @@
     <row r="201">
       <c r="A201" t="inlineStr">
         <is>
-          <t>12:48:06</t>
+          <t>13:00:14</t>
         </is>
       </c>
       <c r="B201" t="inlineStr">
@@ -5358,11 +5358,11 @@
       </c>
       <c r="C201" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D201" t="n">
-        <v>50</v>
+        <v>38</v>
       </c>
       <c r="E201" t="inlineStr">
         <is>
@@ -5498,7 +5498,7 @@
     <row r="207">
       <c r="A207" t="inlineStr">
         <is>
-          <t>13:57:43</t>
+          <t>13:32:57</t>
         </is>
       </c>
       <c r="B207" t="inlineStr">
@@ -5508,11 +5508,11 @@
       </c>
       <c r="C207" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D207" t="n">
-        <v>2</v>
+        <v>27</v>
       </c>
       <c r="E207" t="inlineStr">
         <is>
@@ -5523,7 +5523,7 @@
     <row r="208">
       <c r="A208" t="inlineStr">
         <is>
-          <t>13:32:57</t>
+          <t>13:57:43</t>
         </is>
       </c>
       <c r="B208" t="inlineStr">
@@ -5533,11 +5533,11 @@
       </c>
       <c r="C208" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D208" t="n">
-        <v>27</v>
+        <v>2</v>
       </c>
       <c r="E208" t="inlineStr">
         <is>
@@ -5573,7 +5573,7 @@
     <row r="210">
       <c r="A210" t="inlineStr">
         <is>
-          <t>13:00:14</t>
+          <t>13:57:43</t>
         </is>
       </c>
       <c r="B210" t="inlineStr">
@@ -5583,11 +5583,11 @@
       </c>
       <c r="C210" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D210" t="n">
-        <v>63</v>
+        <v>6</v>
       </c>
       <c r="E210" t="inlineStr">
         <is>
@@ -5598,7 +5598,7 @@
     <row r="211">
       <c r="A211" t="inlineStr">
         <is>
-          <t>13:57:43</t>
+          <t>13:00:14</t>
         </is>
       </c>
       <c r="B211" t="inlineStr">
@@ -5608,11 +5608,11 @@
       </c>
       <c r="C211" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D211" t="n">
-        <v>6</v>
+        <v>63</v>
       </c>
       <c r="E211" t="inlineStr">
         <is>
@@ -5623,7 +5623,7 @@
     <row r="212">
       <c r="A212" t="inlineStr">
         <is>
-          <t>13:57:43</t>
+          <t>13:32:57</t>
         </is>
       </c>
       <c r="B212" t="inlineStr">
@@ -5633,11 +5633,11 @@
       </c>
       <c r="C212" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D212" t="n">
-        <v>19</v>
+        <v>44</v>
       </c>
       <c r="E212" t="inlineStr">
         <is>
@@ -5648,7 +5648,7 @@
     <row r="213">
       <c r="A213" t="inlineStr">
         <is>
-          <t>13:32:57</t>
+          <t>13:57:43</t>
         </is>
       </c>
       <c r="B213" t="inlineStr">
@@ -5658,11 +5658,11 @@
       </c>
       <c r="C213" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D213" t="n">
-        <v>44</v>
+        <v>19</v>
       </c>
       <c r="E213" t="inlineStr">
         <is>
@@ -5673,7 +5673,7 @@
     <row r="214">
       <c r="A214" t="inlineStr">
         <is>
-          <t>13:57:43</t>
+          <t>13:00:14</t>
         </is>
       </c>
       <c r="B214" t="inlineStr">
@@ -5683,11 +5683,11 @@
       </c>
       <c r="C214" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D214" t="n">
-        <v>20</v>
+        <v>77</v>
       </c>
       <c r="E214" t="inlineStr">
         <is>
@@ -5698,7 +5698,7 @@
     <row r="215">
       <c r="A215" t="inlineStr">
         <is>
-          <t>13:00:14</t>
+          <t>13:57:43</t>
         </is>
       </c>
       <c r="B215" t="inlineStr">
@@ -5708,11 +5708,11 @@
       </c>
       <c r="C215" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D215" t="n">
-        <v>77</v>
+        <v>20</v>
       </c>
       <c r="E215" t="inlineStr">
         <is>
@@ -5983,7 +5983,7 @@
       </c>
       <c r="C226" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D226" t="n">
@@ -6008,7 +6008,7 @@
       </c>
       <c r="C227" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D227" t="n">
@@ -6298,7 +6298,7 @@
     <row r="239">
       <c r="A239" t="inlineStr">
         <is>
-          <t>14:46:39</t>
+          <t>14:59:00</t>
         </is>
       </c>
       <c r="B239" t="inlineStr">
@@ -6308,11 +6308,11 @@
       </c>
       <c r="C239" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D239" t="n">
-        <v>25</v>
+        <v>12</v>
       </c>
       <c r="E239" t="inlineStr">
         <is>
@@ -6323,7 +6323,7 @@
     <row r="240">
       <c r="A240" t="inlineStr">
         <is>
-          <t>14:59:00</t>
+          <t>14:46:39</t>
         </is>
       </c>
       <c r="B240" t="inlineStr">
@@ -6333,11 +6333,11 @@
       </c>
       <c r="C240" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D240" t="n">
-        <v>12</v>
+        <v>25</v>
       </c>
       <c r="E240" t="inlineStr">
         <is>
@@ -6698,7 +6698,7 @@
     <row r="255">
       <c r="A255" t="inlineStr">
         <is>
-          <t>15:34:45</t>
+          <t>14:46:39</t>
         </is>
       </c>
       <c r="B255" t="inlineStr">
@@ -6708,11 +6708,11 @@
       </c>
       <c r="C255" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D255" t="n">
-        <v>20</v>
+        <v>68</v>
       </c>
       <c r="E255" t="inlineStr">
         <is>
@@ -6723,7 +6723,7 @@
     <row r="256">
       <c r="A256" t="inlineStr">
         <is>
-          <t>14:46:39</t>
+          <t>15:34:45</t>
         </is>
       </c>
       <c r="B256" t="inlineStr">
@@ -6733,11 +6733,11 @@
       </c>
       <c r="C256" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D256" t="n">
-        <v>68</v>
+        <v>20</v>
       </c>
       <c r="E256" t="inlineStr">
         <is>
@@ -6933,7 +6933,7 @@
       </c>
       <c r="C264" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>215_ALUAR</t>
         </is>
       </c>
       <c r="D264" t="n">
@@ -6958,7 +6958,7 @@
       </c>
       <c r="C265" t="inlineStr">
         <is>
-          <t>215_ALUAR</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D265" t="n">
@@ -7123,7 +7123,7 @@
     <row r="272">
       <c r="A272" t="inlineStr">
         <is>
-          <t>15:34:45</t>
+          <t>14:59:00</t>
         </is>
       </c>
       <c r="B272" t="inlineStr">
@@ -7133,11 +7133,11 @@
       </c>
       <c r="C272" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D272" t="n">
-        <v>62</v>
+        <v>97</v>
       </c>
       <c r="E272" t="inlineStr">
         <is>
@@ -7148,7 +7148,7 @@
     <row r="273">
       <c r="A273" t="inlineStr">
         <is>
-          <t>14:59:00</t>
+          <t>15:34:45</t>
         </is>
       </c>
       <c r="B273" t="inlineStr">
@@ -7158,11 +7158,11 @@
       </c>
       <c r="C273" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D273" t="n">
-        <v>97</v>
+        <v>62</v>
       </c>
       <c r="E273" t="inlineStr">
         <is>
@@ -7333,7 +7333,7 @@
       </c>
       <c r="C280" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D280" t="n">
@@ -7358,7 +7358,7 @@
       </c>
       <c r="C281" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D281" t="n">
@@ -7833,7 +7833,7 @@
       </c>
       <c r="C300" t="inlineStr">
         <is>
-          <t>215_EL PELIGRO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D300" t="n">
@@ -7858,7 +7858,7 @@
       </c>
       <c r="C301" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>215_EL PELIGRO</t>
         </is>
       </c>
       <c r="D301" t="n">
@@ -7883,7 +7883,7 @@
       </c>
       <c r="C302" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>215_EL PELIGRO</t>
         </is>
       </c>
       <c r="D302" t="n">
@@ -7908,7 +7908,7 @@
       </c>
       <c r="C303" t="inlineStr">
         <is>
-          <t>215_EL PELIGRO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D303" t="n">
@@ -8058,7 +8058,7 @@
       </c>
       <c r="C309" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D309" t="n">
@@ -8083,7 +8083,7 @@
       </c>
       <c r="C310" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D310" t="n">
@@ -8108,7 +8108,7 @@
       </c>
       <c r="C311" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D311" t="n">
@@ -8158,7 +8158,7 @@
       </c>
       <c r="C313" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D313" t="n">
@@ -8183,7 +8183,7 @@
       </c>
       <c r="C314" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D314" t="n">
@@ -8923,7 +8923,7 @@
     <row r="344">
       <c r="A344" t="inlineStr">
         <is>
-          <t>19:12:47</t>
+          <t>18:51:25</t>
         </is>
       </c>
       <c r="B344" t="inlineStr">
@@ -8933,11 +8933,11 @@
       </c>
       <c r="C344" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>225_GOMEZ</t>
         </is>
       </c>
       <c r="D344" t="n">
-        <v>11</v>
+        <v>32</v>
       </c>
       <c r="E344" t="inlineStr">
         <is>
@@ -8948,7 +8948,7 @@
     <row r="345">
       <c r="A345" t="inlineStr">
         <is>
-          <t>18:51:25</t>
+          <t>19:12:47</t>
         </is>
       </c>
       <c r="B345" t="inlineStr">
@@ -8958,11 +8958,11 @@
       </c>
       <c r="C345" t="inlineStr">
         <is>
-          <t>225_GOMEZ</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D345" t="n">
-        <v>32</v>
+        <v>11</v>
       </c>
       <c r="E345" t="inlineStr">
         <is>
@@ -9098,7 +9098,7 @@
     <row r="351">
       <c r="A351" t="inlineStr">
         <is>
-          <t>19:12:47</t>
+          <t>18:51:25</t>
         </is>
       </c>
       <c r="B351" t="inlineStr">
@@ -9108,11 +9108,11 @@
       </c>
       <c r="C351" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D351" t="n">
-        <v>28</v>
+        <v>49</v>
       </c>
       <c r="E351" t="inlineStr">
         <is>
@@ -9123,7 +9123,7 @@
     <row r="352">
       <c r="A352" t="inlineStr">
         <is>
-          <t>18:51:25</t>
+          <t>19:12:47</t>
         </is>
       </c>
       <c r="B352" t="inlineStr">
@@ -9133,11 +9133,11 @@
       </c>
       <c r="C352" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D352" t="n">
-        <v>49</v>
+        <v>28</v>
       </c>
       <c r="E352" t="inlineStr">
         <is>
@@ -9173,21 +9173,21 @@
     <row r="354">
       <c r="A354" t="inlineStr">
         <is>
-          <t>19:12:47</t>
+          <t>19:44:03</t>
         </is>
       </c>
       <c r="B354" t="inlineStr">
         <is>
-          <t>19:47</t>
+          <t>19:45</t>
         </is>
       </c>
       <c r="C354" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D354" t="n">
-        <v>35</v>
+        <v>1</v>
       </c>
       <c r="E354" t="inlineStr">
         <is>
@@ -9198,21 +9198,21 @@
     <row r="355">
       <c r="A355" t="inlineStr">
         <is>
-          <t>19:12:47</t>
+          <t>19:44:03</t>
         </is>
       </c>
       <c r="B355" t="inlineStr">
         <is>
-          <t>19:53</t>
+          <t>19:47</t>
         </is>
       </c>
       <c r="C355" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D355" t="n">
-        <v>41</v>
+        <v>3</v>
       </c>
       <c r="E355" t="inlineStr">
         <is>
@@ -9228,16 +9228,16 @@
       </c>
       <c r="B356" t="inlineStr">
         <is>
-          <t>19:54</t>
+          <t>19:53</t>
         </is>
       </c>
       <c r="C356" t="inlineStr">
         <is>
-          <t>14X44_ABASTO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D356" t="n">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="E356" t="inlineStr">
         <is>
@@ -9248,12 +9248,12 @@
     <row r="357">
       <c r="A357" t="inlineStr">
         <is>
-          <t>18:35:14</t>
+          <t>19:12:47</t>
         </is>
       </c>
       <c r="B357" t="inlineStr">
         <is>
-          <t>19:55</t>
+          <t>19:54</t>
         </is>
       </c>
       <c r="C357" t="inlineStr">
@@ -9262,7 +9262,7 @@
         </is>
       </c>
       <c r="D357" t="n">
-        <v>80</v>
+        <v>42</v>
       </c>
       <c r="E357" t="inlineStr">
         <is>
@@ -9273,21 +9273,21 @@
     <row r="358">
       <c r="A358" t="inlineStr">
         <is>
-          <t>19:12:47</t>
+          <t>19:44:03</t>
         </is>
       </c>
       <c r="B358" t="inlineStr">
         <is>
-          <t>20:00</t>
+          <t>19:55</t>
         </is>
       </c>
       <c r="C358" t="inlineStr">
         <is>
-          <t>81_EL PELIGRO</t>
+          <t>14X44_ABASTO</t>
         </is>
       </c>
       <c r="D358" t="n">
-        <v>48</v>
+        <v>11</v>
       </c>
       <c r="E358" t="inlineStr">
         <is>
@@ -9298,21 +9298,21 @@
     <row r="359">
       <c r="A359" t="inlineStr">
         <is>
-          <t>19:12:47</t>
+          <t>19:44:03</t>
         </is>
       </c>
       <c r="B359" t="inlineStr">
         <is>
-          <t>20:10</t>
+          <t>20:00</t>
         </is>
       </c>
       <c r="C359" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>81_EL PELIGRO</t>
         </is>
       </c>
       <c r="D359" t="n">
-        <v>58</v>
+        <v>16</v>
       </c>
       <c r="E359" t="inlineStr">
         <is>
@@ -9323,21 +9323,21 @@
     <row r="360">
       <c r="A360" t="inlineStr">
         <is>
-          <t>19:12:47</t>
+          <t>19:44:03</t>
         </is>
       </c>
       <c r="B360" t="inlineStr">
         <is>
-          <t>20:11</t>
+          <t>20:07</t>
         </is>
       </c>
       <c r="C360" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D360" t="n">
-        <v>59</v>
+        <v>23</v>
       </c>
       <c r="E360" t="inlineStr">
         <is>
@@ -9348,21 +9348,21 @@
     <row r="361">
       <c r="A361" t="inlineStr">
         <is>
-          <t>19:12:47</t>
+          <t>19:44:03</t>
         </is>
       </c>
       <c r="B361" t="inlineStr">
         <is>
-          <t>20:14</t>
+          <t>20:10</t>
         </is>
       </c>
       <c r="C361" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D361" t="n">
-        <v>62</v>
+        <v>26</v>
       </c>
       <c r="E361" t="inlineStr">
         <is>
@@ -9373,21 +9373,21 @@
     <row r="362">
       <c r="A362" t="inlineStr">
         <is>
-          <t>18:51:25</t>
+          <t>19:44:03</t>
         </is>
       </c>
       <c r="B362" t="inlineStr">
         <is>
-          <t>20:15</t>
+          <t>20:11</t>
         </is>
       </c>
       <c r="C362" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D362" t="n">
-        <v>84</v>
+        <v>27</v>
       </c>
       <c r="E362" t="inlineStr">
         <is>
@@ -9398,21 +9398,21 @@
     <row r="363">
       <c r="A363" t="inlineStr">
         <is>
-          <t>19:12:47</t>
+          <t>19:44:03</t>
         </is>
       </c>
       <c r="B363" t="inlineStr">
         <is>
-          <t>20:26</t>
+          <t>20:13</t>
         </is>
       </c>
       <c r="C363" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D363" t="n">
-        <v>74</v>
+        <v>29</v>
       </c>
       <c r="E363" t="inlineStr">
         <is>
@@ -9423,21 +9423,21 @@
     <row r="364">
       <c r="A364" t="inlineStr">
         <is>
-          <t>18:51:25</t>
+          <t>19:12:47</t>
         </is>
       </c>
       <c r="B364" t="inlineStr">
         <is>
-          <t>20:27</t>
+          <t>20:14</t>
         </is>
       </c>
       <c r="C364" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D364" t="n">
-        <v>96</v>
+        <v>62</v>
       </c>
       <c r="E364" t="inlineStr">
         <is>
@@ -9448,21 +9448,21 @@
     <row r="365">
       <c r="A365" t="inlineStr">
         <is>
-          <t>19:12:47</t>
+          <t>19:44:03</t>
         </is>
       </c>
       <c r="B365" t="inlineStr">
         <is>
-          <t>20:34</t>
+          <t>20:15</t>
         </is>
       </c>
       <c r="C365" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D365" t="n">
-        <v>82</v>
+        <v>31</v>
       </c>
       <c r="E365" t="inlineStr">
         <is>
@@ -9473,21 +9473,21 @@
     <row r="366">
       <c r="A366" t="inlineStr">
         <is>
-          <t>18:51:25</t>
+          <t>19:12:47</t>
         </is>
       </c>
       <c r="B366" t="inlineStr">
         <is>
-          <t>20:35</t>
+          <t>20:26</t>
         </is>
       </c>
       <c r="C366" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D366" t="n">
-        <v>104</v>
+        <v>74</v>
       </c>
       <c r="E366" t="inlineStr">
         <is>
@@ -9498,21 +9498,21 @@
     <row r="367">
       <c r="A367" t="inlineStr">
         <is>
-          <t>19:12:47</t>
+          <t>19:44:03</t>
         </is>
       </c>
       <c r="B367" t="inlineStr">
         <is>
-          <t>20:44</t>
+          <t>20:27</t>
         </is>
       </c>
       <c r="C367" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D367" t="n">
-        <v>92</v>
+        <v>43</v>
       </c>
       <c r="E367" t="inlineStr">
         <is>
@@ -9528,16 +9528,16 @@
       </c>
       <c r="B368" t="inlineStr">
         <is>
-          <t>20:55</t>
+          <t>20:34</t>
         </is>
       </c>
       <c r="C368" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D368" t="n">
-        <v>103</v>
+        <v>82</v>
       </c>
       <c r="E368" t="inlineStr">
         <is>
@@ -9548,23 +9548,223 @@
     <row r="369">
       <c r="A369" t="inlineStr">
         <is>
+          <t>19:44:03</t>
+        </is>
+      </c>
+      <c r="B369" t="inlineStr">
+        <is>
+          <t>20:35</t>
+        </is>
+      </c>
+      <c r="C369" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D369" t="n">
+        <v>51</v>
+      </c>
+      <c r="E369" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="370">
+      <c r="A370" t="inlineStr">
+        <is>
+          <t>19:44:03</t>
+        </is>
+      </c>
+      <c r="B370" t="inlineStr">
+        <is>
+          <t>20:44</t>
+        </is>
+      </c>
+      <c r="C370" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D370" t="n">
+        <v>60</v>
+      </c>
+      <c r="E370" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="371">
+      <c r="A371" t="inlineStr">
+        <is>
           <t>19:12:47</t>
         </is>
       </c>
-      <c r="B369" t="inlineStr">
+      <c r="B371" t="inlineStr">
+        <is>
+          <t>20:55</t>
+        </is>
+      </c>
+      <c r="C371" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D371" t="n">
+        <v>103</v>
+      </c>
+      <c r="E371" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="372">
+      <c r="A372" t="inlineStr">
+        <is>
+          <t>19:12:47</t>
+        </is>
+      </c>
+      <c r="B372" t="inlineStr">
         <is>
           <t>20:56</t>
         </is>
       </c>
-      <c r="C369" t="inlineStr">
+      <c r="C372" t="inlineStr">
         <is>
           <t>27_EL RETIRO</t>
         </is>
       </c>
-      <c r="D369" t="n">
+      <c r="D372" t="n">
         <v>104</v>
       </c>
-      <c r="E369" t="inlineStr">
+      <c r="E372" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="373">
+      <c r="A373" t="inlineStr">
+        <is>
+          <t>19:44:03</t>
+        </is>
+      </c>
+      <c r="B373" t="inlineStr">
+        <is>
+          <t>20:56</t>
+        </is>
+      </c>
+      <c r="C373" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D373" t="n">
+        <v>72</v>
+      </c>
+      <c r="E373" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="374">
+      <c r="A374" t="inlineStr">
+        <is>
+          <t>19:44:03</t>
+        </is>
+      </c>
+      <c r="B374" t="inlineStr">
+        <is>
+          <t>20:57</t>
+        </is>
+      </c>
+      <c r="C374" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D374" t="n">
+        <v>73</v>
+      </c>
+      <c r="E374" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="375">
+      <c r="A375" t="inlineStr">
+        <is>
+          <t>19:44:03</t>
+        </is>
+      </c>
+      <c r="B375" t="inlineStr">
+        <is>
+          <t>21:02</t>
+        </is>
+      </c>
+      <c r="C375" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D375" t="n">
+        <v>78</v>
+      </c>
+      <c r="E375" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="376">
+      <c r="A376" t="inlineStr">
+        <is>
+          <t>19:44:03</t>
+        </is>
+      </c>
+      <c r="B376" t="inlineStr">
+        <is>
+          <t>21:24</t>
+        </is>
+      </c>
+      <c r="C376" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D376" t="n">
+        <v>100</v>
+      </c>
+      <c r="E376" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="377">
+      <c r="A377" t="inlineStr">
+        <is>
+          <t>19:44:03</t>
+        </is>
+      </c>
+      <c r="B377" t="inlineStr">
+        <is>
+          <t>21:37</t>
+        </is>
+      </c>
+      <c r="C377" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D377" t="n">
+        <v>113</v>
+      </c>
+      <c r="E377" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -9581,7 +9781,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E61"/>
+  <dimension ref="A1:E62"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -9594,14 +9794,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 19:12:47</t>
+          <t>Última actualización: 19:44:03</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 56</t>
+          <t>Total filas: 57</t>
         </is>
       </c>
     </row>
@@ -10745,7 +10945,7 @@
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>215_EL PELIGRO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D50" t="n">
@@ -10770,7 +10970,7 @@
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>215_EL PELIGRO</t>
         </is>
       </c>
       <c r="D51" t="n">
@@ -10795,7 +10995,7 @@
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>215_EL PELIGRO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D52" t="n">
@@ -10820,7 +11020,7 @@
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>215_EL PELIGRO</t>
         </is>
       </c>
       <c r="D53" t="n">
@@ -10960,7 +11160,7 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>18:51:25</t>
+          <t>19:44:03</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
@@ -10974,7 +11174,7 @@
         </is>
       </c>
       <c r="D59" t="n">
-        <v>84</v>
+        <v>31</v>
       </c>
       <c r="E59" t="inlineStr">
         <is>
@@ -10985,7 +11185,7 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>19:12:47</t>
+          <t>19:44:03</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
@@ -10999,7 +11199,7 @@
         </is>
       </c>
       <c r="D60" t="n">
-        <v>92</v>
+        <v>60</v>
       </c>
       <c r="E60" t="inlineStr">
         <is>
@@ -11027,6 +11227,31 @@
         <v>103</v>
       </c>
       <c r="E61" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>19:44:03</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>20:56</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D62" t="n">
+        <v>72</v>
+      </c>
+      <c r="E62" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -11043,7 +11268,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E61"/>
+  <dimension ref="A1:E62"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -11056,14 +11281,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 19:12:47</t>
+          <t>Última actualización: 19:44:03</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 56</t>
+          <t>Total filas: 57</t>
         </is>
       </c>
     </row>
@@ -12472,7 +12697,7 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>18:51:25</t>
+          <t>19:44:03</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
@@ -12486,9 +12711,34 @@
         </is>
       </c>
       <c r="D61" t="n">
-        <v>114</v>
+        <v>61</v>
       </c>
       <c r="E61" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>19:44:03</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>21:37</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D62" t="n">
+        <v>113</v>
+      </c>
+      <c r="E62" t="inlineStr">
         <is>
           <t>L6203</t>
         </is>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 1826
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-03-21.xlsx
+++ b/data/horarios-141-2026-03-21.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E377"/>
+  <dimension ref="A1:E383"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 19:44:03</t>
+          <t>Última actualización: 19:59:19</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 372</t>
+          <t>Total filas: 378</t>
         </is>
       </c>
     </row>
@@ -533,7 +533,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D8" t="n">
@@ -558,7 +558,7 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D9" t="n">
@@ -1558,7 +1558,7 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D49" t="n">
@@ -1583,7 +1583,7 @@
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D50" t="n">
@@ -1883,7 +1883,7 @@
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D62" t="n">
@@ -1898,7 +1898,7 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>06:59:30</t>
+          <t>08:14:14</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
@@ -1908,11 +1908,11 @@
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D63" t="n">
-        <v>75</v>
+        <v>0</v>
       </c>
       <c r="E63" t="inlineStr">
         <is>
@@ -1923,7 +1923,7 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>08:14:14</t>
+          <t>06:59:30</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
@@ -1933,11 +1933,11 @@
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D64" t="n">
-        <v>0</v>
+        <v>75</v>
       </c>
       <c r="E64" t="inlineStr">
         <is>
@@ -1973,7 +1973,7 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>07:27:35</t>
+          <t>07:51:37</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
@@ -1983,11 +1983,11 @@
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D66" t="n">
-        <v>52</v>
+        <v>28</v>
       </c>
       <c r="E66" t="inlineStr">
         <is>
@@ -2023,7 +2023,7 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>07:51:37</t>
+          <t>07:27:35</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
@@ -2033,11 +2033,11 @@
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D68" t="n">
-        <v>28</v>
+        <v>52</v>
       </c>
       <c r="E68" t="inlineStr">
         <is>
@@ -2233,7 +2233,7 @@
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D76" t="n">
@@ -2258,7 +2258,7 @@
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D77" t="n">
@@ -2373,7 +2373,7 @@
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>08:50:55</t>
+          <t>07:27:35</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
@@ -2383,11 +2383,11 @@
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D82" t="n">
-        <v>1</v>
+        <v>84</v>
       </c>
       <c r="E82" t="inlineStr">
         <is>
@@ -2408,7 +2408,7 @@
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D83" t="n">
@@ -2423,7 +2423,7 @@
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>07:27:35</t>
+          <t>08:50:55</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
@@ -2433,11 +2433,11 @@
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D84" t="n">
-        <v>84</v>
+        <v>1</v>
       </c>
       <c r="E84" t="inlineStr">
         <is>
@@ -2708,7 +2708,7 @@
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>215_EL PELIGRO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D95" t="n">
@@ -2733,7 +2733,7 @@
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215_EL PELIGRO</t>
         </is>
       </c>
       <c r="D96" t="n">
@@ -2873,7 +2873,7 @@
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>07:51:37</t>
+          <t>08:36:09</t>
         </is>
       </c>
       <c r="B102" t="inlineStr">
@@ -2883,11 +2883,11 @@
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D102" t="n">
-        <v>98</v>
+        <v>53</v>
       </c>
       <c r="E102" t="inlineStr">
         <is>
@@ -2898,7 +2898,7 @@
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>08:36:09</t>
+          <t>07:51:37</t>
         </is>
       </c>
       <c r="B103" t="inlineStr">
@@ -2908,11 +2908,11 @@
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D103" t="n">
-        <v>53</v>
+        <v>98</v>
       </c>
       <c r="E103" t="inlineStr">
         <is>
@@ -2923,7 +2923,7 @@
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>09:23:24</t>
+          <t>08:14:14</t>
         </is>
       </c>
       <c r="B104" t="inlineStr">
@@ -2933,11 +2933,11 @@
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D104" t="n">
-        <v>10</v>
+        <v>79</v>
       </c>
       <c r="E104" t="inlineStr">
         <is>
@@ -2948,7 +2948,7 @@
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>08:14:14</t>
+          <t>09:23:24</t>
         </is>
       </c>
       <c r="B105" t="inlineStr">
@@ -2958,11 +2958,11 @@
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D105" t="n">
-        <v>79</v>
+        <v>10</v>
       </c>
       <c r="E105" t="inlineStr">
         <is>
@@ -3083,7 +3083,7 @@
       </c>
       <c r="C110" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D110" t="n">
@@ -3108,7 +3108,7 @@
       </c>
       <c r="C111" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D111" t="n">
@@ -4123,7 +4123,7 @@
     <row r="152">
       <c r="A152" t="inlineStr">
         <is>
-          <t>11:16:36</t>
+          <t>10:14:52</t>
         </is>
       </c>
       <c r="B152" t="inlineStr">
@@ -4133,11 +4133,11 @@
       </c>
       <c r="C152" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D152" t="n">
-        <v>16</v>
+        <v>78</v>
       </c>
       <c r="E152" t="inlineStr">
         <is>
@@ -4148,7 +4148,7 @@
     <row r="153">
       <c r="A153" t="inlineStr">
         <is>
-          <t>10:14:52</t>
+          <t>11:16:36</t>
         </is>
       </c>
       <c r="B153" t="inlineStr">
@@ -4158,11 +4158,11 @@
       </c>
       <c r="C153" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D153" t="n">
-        <v>78</v>
+        <v>16</v>
       </c>
       <c r="E153" t="inlineStr">
         <is>
@@ -4183,7 +4183,7 @@
       </c>
       <c r="C154" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D154" t="n">
@@ -4208,7 +4208,7 @@
       </c>
       <c r="C155" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D155" t="n">
@@ -4473,7 +4473,7 @@
     <row r="166">
       <c r="A166" t="inlineStr">
         <is>
-          <t>11:16:36</t>
+          <t>12:00:15</t>
         </is>
       </c>
       <c r="B166" t="inlineStr">
@@ -4483,11 +4483,11 @@
       </c>
       <c r="C166" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D166" t="n">
-        <v>48</v>
+        <v>4</v>
       </c>
       <c r="E166" t="inlineStr">
         <is>
@@ -4498,7 +4498,7 @@
     <row r="167">
       <c r="A167" t="inlineStr">
         <is>
-          <t>12:00:15</t>
+          <t>11:16:36</t>
         </is>
       </c>
       <c r="B167" t="inlineStr">
@@ -4508,11 +4508,11 @@
       </c>
       <c r="C167" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D167" t="n">
-        <v>4</v>
+        <v>48</v>
       </c>
       <c r="E167" t="inlineStr">
         <is>
@@ -4648,7 +4648,7 @@
     <row r="173">
       <c r="A173" t="inlineStr">
         <is>
-          <t>12:00:15</t>
+          <t>12:28:38</t>
         </is>
       </c>
       <c r="B173" t="inlineStr">
@@ -4658,11 +4658,11 @@
       </c>
       <c r="C173" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D173" t="n">
-        <v>33</v>
+        <v>5</v>
       </c>
       <c r="E173" t="inlineStr">
         <is>
@@ -4698,7 +4698,7 @@
     <row r="175">
       <c r="A175" t="inlineStr">
         <is>
-          <t>12:28:38</t>
+          <t>12:00:15</t>
         </is>
       </c>
       <c r="B175" t="inlineStr">
@@ -4708,11 +4708,11 @@
       </c>
       <c r="C175" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D175" t="n">
-        <v>5</v>
+        <v>33</v>
       </c>
       <c r="E175" t="inlineStr">
         <is>
@@ -5323,7 +5323,7 @@
     <row r="200">
       <c r="A200" t="inlineStr">
         <is>
-          <t>12:48:06</t>
+          <t>13:00:14</t>
         </is>
       </c>
       <c r="B200" t="inlineStr">
@@ -5333,11 +5333,11 @@
       </c>
       <c r="C200" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D200" t="n">
-        <v>50</v>
+        <v>38</v>
       </c>
       <c r="E200" t="inlineStr">
         <is>
@@ -5348,7 +5348,7 @@
     <row r="201">
       <c r="A201" t="inlineStr">
         <is>
-          <t>13:00:14</t>
+          <t>12:48:06</t>
         </is>
       </c>
       <c r="B201" t="inlineStr">
@@ -5358,11 +5358,11 @@
       </c>
       <c r="C201" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D201" t="n">
-        <v>38</v>
+        <v>50</v>
       </c>
       <c r="E201" t="inlineStr">
         <is>
@@ -5573,7 +5573,7 @@
     <row r="210">
       <c r="A210" t="inlineStr">
         <is>
-          <t>13:57:43</t>
+          <t>13:00:14</t>
         </is>
       </c>
       <c r="B210" t="inlineStr">
@@ -5583,11 +5583,11 @@
       </c>
       <c r="C210" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D210" t="n">
-        <v>6</v>
+        <v>63</v>
       </c>
       <c r="E210" t="inlineStr">
         <is>
@@ -5598,7 +5598,7 @@
     <row r="211">
       <c r="A211" t="inlineStr">
         <is>
-          <t>13:00:14</t>
+          <t>13:57:43</t>
         </is>
       </c>
       <c r="B211" t="inlineStr">
@@ -5608,11 +5608,11 @@
       </c>
       <c r="C211" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D211" t="n">
-        <v>63</v>
+        <v>6</v>
       </c>
       <c r="E211" t="inlineStr">
         <is>
@@ -5623,7 +5623,7 @@
     <row r="212">
       <c r="A212" t="inlineStr">
         <is>
-          <t>13:32:57</t>
+          <t>13:57:43</t>
         </is>
       </c>
       <c r="B212" t="inlineStr">
@@ -5633,11 +5633,11 @@
       </c>
       <c r="C212" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D212" t="n">
-        <v>44</v>
+        <v>19</v>
       </c>
       <c r="E212" t="inlineStr">
         <is>
@@ -5648,7 +5648,7 @@
     <row r="213">
       <c r="A213" t="inlineStr">
         <is>
-          <t>13:57:43</t>
+          <t>13:32:57</t>
         </is>
       </c>
       <c r="B213" t="inlineStr">
@@ -5658,11 +5658,11 @@
       </c>
       <c r="C213" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D213" t="n">
-        <v>19</v>
+        <v>44</v>
       </c>
       <c r="E213" t="inlineStr">
         <is>
@@ -5673,7 +5673,7 @@
     <row r="214">
       <c r="A214" t="inlineStr">
         <is>
-          <t>13:00:14</t>
+          <t>13:57:43</t>
         </is>
       </c>
       <c r="B214" t="inlineStr">
@@ -5683,11 +5683,11 @@
       </c>
       <c r="C214" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D214" t="n">
-        <v>77</v>
+        <v>20</v>
       </c>
       <c r="E214" t="inlineStr">
         <is>
@@ -5698,7 +5698,7 @@
     <row r="215">
       <c r="A215" t="inlineStr">
         <is>
-          <t>13:57:43</t>
+          <t>13:00:14</t>
         </is>
       </c>
       <c r="B215" t="inlineStr">
@@ -5708,11 +5708,11 @@
       </c>
       <c r="C215" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D215" t="n">
-        <v>20</v>
+        <v>77</v>
       </c>
       <c r="E215" t="inlineStr">
         <is>
@@ -6098,7 +6098,7 @@
     <row r="231">
       <c r="A231" t="inlineStr">
         <is>
-          <t>14:59:00</t>
+          <t>14:46:39</t>
         </is>
       </c>
       <c r="B231" t="inlineStr">
@@ -6108,11 +6108,11 @@
       </c>
       <c r="C231" t="inlineStr">
         <is>
-          <t>81_EL PELIGRO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D231" t="n">
-        <v>0</v>
+        <v>13</v>
       </c>
       <c r="E231" t="inlineStr">
         <is>
@@ -6123,7 +6123,7 @@
     <row r="232">
       <c r="A232" t="inlineStr">
         <is>
-          <t>14:46:39</t>
+          <t>14:59:00</t>
         </is>
       </c>
       <c r="B232" t="inlineStr">
@@ -6133,11 +6133,11 @@
       </c>
       <c r="C232" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>81_EL PELIGRO</t>
         </is>
       </c>
       <c r="D232" t="n">
-        <v>13</v>
+        <v>0</v>
       </c>
       <c r="E232" t="inlineStr">
         <is>
@@ -6298,7 +6298,7 @@
     <row r="239">
       <c r="A239" t="inlineStr">
         <is>
-          <t>14:59:00</t>
+          <t>14:46:39</t>
         </is>
       </c>
       <c r="B239" t="inlineStr">
@@ -6308,11 +6308,11 @@
       </c>
       <c r="C239" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D239" t="n">
-        <v>12</v>
+        <v>25</v>
       </c>
       <c r="E239" t="inlineStr">
         <is>
@@ -6323,7 +6323,7 @@
     <row r="240">
       <c r="A240" t="inlineStr">
         <is>
-          <t>14:46:39</t>
+          <t>14:59:00</t>
         </is>
       </c>
       <c r="B240" t="inlineStr">
@@ -6333,11 +6333,11 @@
       </c>
       <c r="C240" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D240" t="n">
-        <v>25</v>
+        <v>12</v>
       </c>
       <c r="E240" t="inlineStr">
         <is>
@@ -6933,7 +6933,7 @@
       </c>
       <c r="C264" t="inlineStr">
         <is>
-          <t>215_ALUAR</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D264" t="n">
@@ -6958,7 +6958,7 @@
       </c>
       <c r="C265" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>215_ALUAR</t>
         </is>
       </c>
       <c r="D265" t="n">
@@ -7073,7 +7073,7 @@
     <row r="270">
       <c r="A270" t="inlineStr">
         <is>
-          <t>16:33:34</t>
+          <t>16:01:44</t>
         </is>
       </c>
       <c r="B270" t="inlineStr">
@@ -7083,11 +7083,11 @@
       </c>
       <c r="C270" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D270" t="n">
-        <v>2</v>
+        <v>34</v>
       </c>
       <c r="E270" t="inlineStr">
         <is>
@@ -7098,7 +7098,7 @@
     <row r="271">
       <c r="A271" t="inlineStr">
         <is>
-          <t>16:01:44</t>
+          <t>16:33:34</t>
         </is>
       </c>
       <c r="B271" t="inlineStr">
@@ -7108,11 +7108,11 @@
       </c>
       <c r="C271" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D271" t="n">
-        <v>34</v>
+        <v>2</v>
       </c>
       <c r="E271" t="inlineStr">
         <is>
@@ -7123,7 +7123,7 @@
     <row r="272">
       <c r="A272" t="inlineStr">
         <is>
-          <t>14:59:00</t>
+          <t>15:34:45</t>
         </is>
       </c>
       <c r="B272" t="inlineStr">
@@ -7133,11 +7133,11 @@
       </c>
       <c r="C272" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D272" t="n">
-        <v>97</v>
+        <v>62</v>
       </c>
       <c r="E272" t="inlineStr">
         <is>
@@ -7148,7 +7148,7 @@
     <row r="273">
       <c r="A273" t="inlineStr">
         <is>
-          <t>15:34:45</t>
+          <t>14:59:00</t>
         </is>
       </c>
       <c r="B273" t="inlineStr">
@@ -7158,11 +7158,11 @@
       </c>
       <c r="C273" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D273" t="n">
-        <v>62</v>
+        <v>97</v>
       </c>
       <c r="E273" t="inlineStr">
         <is>
@@ -7673,7 +7673,7 @@
     <row r="294">
       <c r="A294" t="inlineStr">
         <is>
-          <t>16:33:34</t>
+          <t>17:21:09</t>
         </is>
       </c>
       <c r="B294" t="inlineStr">
@@ -7683,11 +7683,11 @@
       </c>
       <c r="C294" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D294" t="n">
-        <v>62</v>
+        <v>14</v>
       </c>
       <c r="E294" t="inlineStr">
         <is>
@@ -7698,7 +7698,7 @@
     <row r="295">
       <c r="A295" t="inlineStr">
         <is>
-          <t>17:21:09</t>
+          <t>16:33:34</t>
         </is>
       </c>
       <c r="B295" t="inlineStr">
@@ -7708,11 +7708,11 @@
       </c>
       <c r="C295" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D295" t="n">
-        <v>14</v>
+        <v>62</v>
       </c>
       <c r="E295" t="inlineStr">
         <is>
@@ -7833,7 +7833,7 @@
       </c>
       <c r="C300" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>215_EL PELIGRO</t>
         </is>
       </c>
       <c r="D300" t="n">
@@ -7858,7 +7858,7 @@
       </c>
       <c r="C301" t="inlineStr">
         <is>
-          <t>215_EL PELIGRO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D301" t="n">
@@ -7883,7 +7883,7 @@
       </c>
       <c r="C302" t="inlineStr">
         <is>
-          <t>215_EL PELIGRO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D302" t="n">
@@ -7908,7 +7908,7 @@
       </c>
       <c r="C303" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>215_EL PELIGRO</t>
         </is>
       </c>
       <c r="D303" t="n">
@@ -7948,7 +7948,7 @@
     <row r="305">
       <c r="A305" t="inlineStr">
         <is>
-          <t>16:57:49</t>
+          <t>17:47:19</t>
         </is>
       </c>
       <c r="B305" t="inlineStr">
@@ -7958,11 +7958,11 @@
       </c>
       <c r="C305" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D305" t="n">
-        <v>62</v>
+        <v>12</v>
       </c>
       <c r="E305" t="inlineStr">
         <is>
@@ -7973,7 +7973,7 @@
     <row r="306">
       <c r="A306" t="inlineStr">
         <is>
-          <t>17:47:19</t>
+          <t>16:57:49</t>
         </is>
       </c>
       <c r="B306" t="inlineStr">
@@ -7983,11 +7983,11 @@
       </c>
       <c r="C306" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D306" t="n">
-        <v>12</v>
+        <v>62</v>
       </c>
       <c r="E306" t="inlineStr">
         <is>
@@ -8158,7 +8158,7 @@
       </c>
       <c r="C313" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D313" t="n">
@@ -8183,7 +8183,7 @@
       </c>
       <c r="C314" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D314" t="n">
@@ -8923,7 +8923,7 @@
     <row r="344">
       <c r="A344" t="inlineStr">
         <is>
-          <t>18:51:25</t>
+          <t>19:12:47</t>
         </is>
       </c>
       <c r="B344" t="inlineStr">
@@ -8933,11 +8933,11 @@
       </c>
       <c r="C344" t="inlineStr">
         <is>
-          <t>225_GOMEZ</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D344" t="n">
-        <v>32</v>
+        <v>11</v>
       </c>
       <c r="E344" t="inlineStr">
         <is>
@@ -8948,7 +8948,7 @@
     <row r="345">
       <c r="A345" t="inlineStr">
         <is>
-          <t>19:12:47</t>
+          <t>18:51:25</t>
         </is>
       </c>
       <c r="B345" t="inlineStr">
@@ -8958,11 +8958,11 @@
       </c>
       <c r="C345" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>225_GOMEZ</t>
         </is>
       </c>
       <c r="D345" t="n">
-        <v>11</v>
+        <v>32</v>
       </c>
       <c r="E345" t="inlineStr">
         <is>
@@ -9298,7 +9298,7 @@
     <row r="359">
       <c r="A359" t="inlineStr">
         <is>
-          <t>19:44:03</t>
+          <t>19:59:19</t>
         </is>
       </c>
       <c r="B359" t="inlineStr">
@@ -9312,7 +9312,7 @@
         </is>
       </c>
       <c r="D359" t="n">
-        <v>16</v>
+        <v>1</v>
       </c>
       <c r="E359" t="inlineStr">
         <is>
@@ -9323,7 +9323,7 @@
     <row r="360">
       <c r="A360" t="inlineStr">
         <is>
-          <t>19:44:03</t>
+          <t>19:59:19</t>
         </is>
       </c>
       <c r="B360" t="inlineStr">
@@ -9337,7 +9337,7 @@
         </is>
       </c>
       <c r="D360" t="n">
-        <v>23</v>
+        <v>8</v>
       </c>
       <c r="E360" t="inlineStr">
         <is>
@@ -9348,7 +9348,7 @@
     <row r="361">
       <c r="A361" t="inlineStr">
         <is>
-          <t>19:44:03</t>
+          <t>19:59:19</t>
         </is>
       </c>
       <c r="B361" t="inlineStr">
@@ -9362,7 +9362,7 @@
         </is>
       </c>
       <c r="D361" t="n">
-        <v>26</v>
+        <v>11</v>
       </c>
       <c r="E361" t="inlineStr">
         <is>
@@ -9373,7 +9373,7 @@
     <row r="362">
       <c r="A362" t="inlineStr">
         <is>
-          <t>19:44:03</t>
+          <t>19:59:19</t>
         </is>
       </c>
       <c r="B362" t="inlineStr">
@@ -9387,7 +9387,7 @@
         </is>
       </c>
       <c r="D362" t="n">
-        <v>27</v>
+        <v>12</v>
       </c>
       <c r="E362" t="inlineStr">
         <is>
@@ -9448,7 +9448,7 @@
     <row r="365">
       <c r="A365" t="inlineStr">
         <is>
-          <t>19:44:03</t>
+          <t>19:59:19</t>
         </is>
       </c>
       <c r="B365" t="inlineStr">
@@ -9462,7 +9462,7 @@
         </is>
       </c>
       <c r="D365" t="n">
-        <v>31</v>
+        <v>16</v>
       </c>
       <c r="E365" t="inlineStr">
         <is>
@@ -9498,7 +9498,7 @@
     <row r="367">
       <c r="A367" t="inlineStr">
         <is>
-          <t>19:44:03</t>
+          <t>19:59:19</t>
         </is>
       </c>
       <c r="B367" t="inlineStr">
@@ -9512,7 +9512,7 @@
         </is>
       </c>
       <c r="D367" t="n">
-        <v>43</v>
+        <v>28</v>
       </c>
       <c r="E367" t="inlineStr">
         <is>
@@ -9523,21 +9523,21 @@
     <row r="368">
       <c r="A368" t="inlineStr">
         <is>
-          <t>19:12:47</t>
+          <t>19:59:19</t>
         </is>
       </c>
       <c r="B368" t="inlineStr">
         <is>
-          <t>20:34</t>
+          <t>20:28</t>
         </is>
       </c>
       <c r="C368" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D368" t="n">
-        <v>82</v>
+        <v>29</v>
       </c>
       <c r="E368" t="inlineStr">
         <is>
@@ -9548,21 +9548,21 @@
     <row r="369">
       <c r="A369" t="inlineStr">
         <is>
-          <t>19:44:03</t>
+          <t>19:59:19</t>
         </is>
       </c>
       <c r="B369" t="inlineStr">
         <is>
-          <t>20:35</t>
+          <t>20:32</t>
         </is>
       </c>
       <c r="C369" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D369" t="n">
-        <v>51</v>
+        <v>33</v>
       </c>
       <c r="E369" t="inlineStr">
         <is>
@@ -9573,21 +9573,21 @@
     <row r="370">
       <c r="A370" t="inlineStr">
         <is>
-          <t>19:44:03</t>
+          <t>19:12:47</t>
         </is>
       </c>
       <c r="B370" t="inlineStr">
         <is>
-          <t>20:44</t>
+          <t>20:34</t>
         </is>
       </c>
       <c r="C370" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D370" t="n">
-        <v>60</v>
+        <v>82</v>
       </c>
       <c r="E370" t="inlineStr">
         <is>
@@ -9598,21 +9598,21 @@
     <row r="371">
       <c r="A371" t="inlineStr">
         <is>
-          <t>19:12:47</t>
+          <t>19:59:19</t>
         </is>
       </c>
       <c r="B371" t="inlineStr">
         <is>
-          <t>20:55</t>
+          <t>20:35</t>
         </is>
       </c>
       <c r="C371" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D371" t="n">
-        <v>103</v>
+        <v>36</v>
       </c>
       <c r="E371" t="inlineStr">
         <is>
@@ -9623,21 +9623,21 @@
     <row r="372">
       <c r="A372" t="inlineStr">
         <is>
-          <t>19:12:47</t>
+          <t>19:59:19</t>
         </is>
       </c>
       <c r="B372" t="inlineStr">
         <is>
-          <t>20:56</t>
+          <t>20:44</t>
         </is>
       </c>
       <c r="C372" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D372" t="n">
-        <v>104</v>
+        <v>45</v>
       </c>
       <c r="E372" t="inlineStr">
         <is>
@@ -9648,12 +9648,12 @@
     <row r="373">
       <c r="A373" t="inlineStr">
         <is>
-          <t>19:44:03</t>
+          <t>19:12:47</t>
         </is>
       </c>
       <c r="B373" t="inlineStr">
         <is>
-          <t>20:56</t>
+          <t>20:55</t>
         </is>
       </c>
       <c r="C373" t="inlineStr">
@@ -9662,7 +9662,7 @@
         </is>
       </c>
       <c r="D373" t="n">
-        <v>72</v>
+        <v>103</v>
       </c>
       <c r="E373" t="inlineStr">
         <is>
@@ -9673,21 +9673,21 @@
     <row r="374">
       <c r="A374" t="inlineStr">
         <is>
-          <t>19:44:03</t>
+          <t>19:59:19</t>
         </is>
       </c>
       <c r="B374" t="inlineStr">
         <is>
-          <t>20:57</t>
+          <t>20:56</t>
         </is>
       </c>
       <c r="C374" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D374" t="n">
-        <v>73</v>
+        <v>57</v>
       </c>
       <c r="E374" t="inlineStr">
         <is>
@@ -9698,21 +9698,21 @@
     <row r="375">
       <c r="A375" t="inlineStr">
         <is>
-          <t>19:44:03</t>
+          <t>19:12:47</t>
         </is>
       </c>
       <c r="B375" t="inlineStr">
         <is>
-          <t>21:02</t>
+          <t>20:56</t>
         </is>
       </c>
       <c r="C375" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D375" t="n">
-        <v>78</v>
+        <v>104</v>
       </c>
       <c r="E375" t="inlineStr">
         <is>
@@ -9723,21 +9723,21 @@
     <row r="376">
       <c r="A376" t="inlineStr">
         <is>
-          <t>19:44:03</t>
+          <t>19:59:19</t>
         </is>
       </c>
       <c r="B376" t="inlineStr">
         <is>
-          <t>21:24</t>
+          <t>20:57</t>
         </is>
       </c>
       <c r="C376" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D376" t="n">
-        <v>100</v>
+        <v>58</v>
       </c>
       <c r="E376" t="inlineStr">
         <is>
@@ -9748,23 +9748,173 @@
     <row r="377">
       <c r="A377" t="inlineStr">
         <is>
+          <t>19:59:19</t>
+        </is>
+      </c>
+      <c r="B377" t="inlineStr">
+        <is>
+          <t>20:59</t>
+        </is>
+      </c>
+      <c r="C377" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D377" t="n">
+        <v>60</v>
+      </c>
+      <c r="E377" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="378">
+      <c r="A378" t="inlineStr">
+        <is>
           <t>19:44:03</t>
         </is>
       </c>
-      <c r="B377" t="inlineStr">
+      <c r="B378" t="inlineStr">
+        <is>
+          <t>21:02</t>
+        </is>
+      </c>
+      <c r="C378" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D378" t="n">
+        <v>78</v>
+      </c>
+      <c r="E378" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="379">
+      <c r="A379" t="inlineStr">
+        <is>
+          <t>19:59:19</t>
+        </is>
+      </c>
+      <c r="B379" t="inlineStr">
+        <is>
+          <t>21:24</t>
+        </is>
+      </c>
+      <c r="C379" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D379" t="n">
+        <v>85</v>
+      </c>
+      <c r="E379" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="380">
+      <c r="A380" t="inlineStr">
+        <is>
+          <t>19:44:03</t>
+        </is>
+      </c>
+      <c r="B380" t="inlineStr">
         <is>
           <t>21:37</t>
         </is>
       </c>
-      <c r="C377" t="inlineStr">
+      <c r="C380" t="inlineStr">
         <is>
           <t>15_ABASTO</t>
         </is>
       </c>
-      <c r="D377" t="n">
+      <c r="D380" t="n">
         <v>113</v>
       </c>
-      <c r="E377" t="inlineStr">
+      <c r="E380" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="381">
+      <c r="A381" t="inlineStr">
+        <is>
+          <t>19:59:19</t>
+        </is>
+      </c>
+      <c r="B381" t="inlineStr">
+        <is>
+          <t>21:49</t>
+        </is>
+      </c>
+      <c r="C381" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D381" t="n">
+        <v>110</v>
+      </c>
+      <c r="E381" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="382">
+      <c r="A382" t="inlineStr">
+        <is>
+          <t>19:59:19</t>
+        </is>
+      </c>
+      <c r="B382" t="inlineStr">
+        <is>
+          <t>21:50</t>
+        </is>
+      </c>
+      <c r="C382" t="inlineStr">
+        <is>
+          <t>84_COLONIA URQUIZA-ESC 49</t>
+        </is>
+      </c>
+      <c r="D382" t="n">
+        <v>111</v>
+      </c>
+      <c r="E382" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="383">
+      <c r="A383" t="inlineStr">
+        <is>
+          <t>19:59:19</t>
+        </is>
+      </c>
+      <c r="B383" t="inlineStr">
+        <is>
+          <t>21:52</t>
+        </is>
+      </c>
+      <c r="C383" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D383" t="n">
+        <v>113</v>
+      </c>
+      <c r="E383" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -9794,7 +9944,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 19:44:03</t>
+          <t>Última actualización: 19:59:19</t>
         </is>
       </c>
     </row>
@@ -10945,7 +11095,7 @@
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>215_EL PELIGRO</t>
         </is>
       </c>
       <c r="D50" t="n">
@@ -10970,7 +11120,7 @@
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>215_EL PELIGRO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D51" t="n">
@@ -10995,7 +11145,7 @@
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>215_EL PELIGRO</t>
         </is>
       </c>
       <c r="D52" t="n">
@@ -11020,7 +11170,7 @@
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>215_EL PELIGRO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D53" t="n">
@@ -11160,7 +11310,7 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>19:44:03</t>
+          <t>19:59:19</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
@@ -11174,7 +11324,7 @@
         </is>
       </c>
       <c r="D59" t="n">
-        <v>31</v>
+        <v>16</v>
       </c>
       <c r="E59" t="inlineStr">
         <is>
@@ -11185,7 +11335,7 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>19:44:03</t>
+          <t>19:59:19</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
@@ -11199,7 +11349,7 @@
         </is>
       </c>
       <c r="D60" t="n">
-        <v>60</v>
+        <v>45</v>
       </c>
       <c r="E60" t="inlineStr">
         <is>
@@ -11235,7 +11385,7 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>19:44:03</t>
+          <t>19:59:19</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
@@ -11249,7 +11399,7 @@
         </is>
       </c>
       <c r="D62" t="n">
-        <v>72</v>
+        <v>57</v>
       </c>
       <c r="E62" t="inlineStr">
         <is>
@@ -11281,7 +11431,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 19:44:03</t>
+          <t>Última actualización: 19:59:19</t>
         </is>
       </c>
     </row>
@@ -12697,7 +12847,7 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>19:44:03</t>
+          <t>19:59:19</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
@@ -12711,7 +12861,7 @@
         </is>
       </c>
       <c r="D61" t="n">
-        <v>61</v>
+        <v>46</v>
       </c>
       <c r="E61" t="inlineStr">
         <is>
@@ -12722,7 +12872,7 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>19:44:03</t>
+          <t>19:59:19</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
@@ -12736,7 +12886,7 @@
         </is>
       </c>
       <c r="D62" t="n">
-        <v>113</v>
+        <v>98</v>
       </c>
       <c r="E62" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 1827
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-03-21.xlsx
+++ b/data/horarios-141-2026-03-21.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E383"/>
+  <dimension ref="A1:E394"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 19:59:19</t>
+          <t>Última actualización: 20:24:55</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 378</t>
+          <t>Total filas: 389</t>
         </is>
       </c>
     </row>
@@ -758,7 +758,7 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D17" t="n">
@@ -783,7 +783,7 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D18" t="n">
@@ -1158,7 +1158,7 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D33" t="n">
@@ -1183,7 +1183,7 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D34" t="n">
@@ -1998,7 +1998,7 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>07:51:37</t>
+          <t>07:27:35</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
@@ -2008,11 +2008,11 @@
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D67" t="n">
-        <v>28</v>
+        <v>52</v>
       </c>
       <c r="E67" t="inlineStr">
         <is>
@@ -2023,7 +2023,7 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>07:27:35</t>
+          <t>07:51:37</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
@@ -2033,11 +2033,11 @@
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D68" t="n">
-        <v>52</v>
+        <v>28</v>
       </c>
       <c r="E68" t="inlineStr">
         <is>
@@ -2408,7 +2408,7 @@
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D83" t="n">
@@ -2433,7 +2433,7 @@
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D84" t="n">
@@ -2873,7 +2873,7 @@
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>08:36:09</t>
+          <t>07:51:37</t>
         </is>
       </c>
       <c r="B102" t="inlineStr">
@@ -2883,11 +2883,11 @@
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D102" t="n">
-        <v>53</v>
+        <v>98</v>
       </c>
       <c r="E102" t="inlineStr">
         <is>
@@ -2898,7 +2898,7 @@
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>07:51:37</t>
+          <t>08:36:09</t>
         </is>
       </c>
       <c r="B103" t="inlineStr">
@@ -2908,11 +2908,11 @@
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D103" t="n">
-        <v>98</v>
+        <v>53</v>
       </c>
       <c r="E103" t="inlineStr">
         <is>
@@ -3498,7 +3498,7 @@
     <row r="127">
       <c r="A127" t="inlineStr">
         <is>
-          <t>08:36:09</t>
+          <t>10:14:52</t>
         </is>
       </c>
       <c r="B127" t="inlineStr">
@@ -3508,11 +3508,11 @@
       </c>
       <c r="C127" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D127" t="n">
-        <v>117</v>
+        <v>19</v>
       </c>
       <c r="E127" t="inlineStr">
         <is>
@@ -3523,7 +3523,7 @@
     <row r="128">
       <c r="A128" t="inlineStr">
         <is>
-          <t>10:14:52</t>
+          <t>08:36:09</t>
         </is>
       </c>
       <c r="B128" t="inlineStr">
@@ -3533,11 +3533,11 @@
       </c>
       <c r="C128" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D128" t="n">
-        <v>19</v>
+        <v>117</v>
       </c>
       <c r="E128" t="inlineStr">
         <is>
@@ -3598,7 +3598,7 @@
     <row r="131">
       <c r="A131" t="inlineStr">
         <is>
-          <t>10:14:52</t>
+          <t>09:23:24</t>
         </is>
       </c>
       <c r="B131" t="inlineStr">
@@ -3608,11 +3608,11 @@
       </c>
       <c r="C131" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D131" t="n">
-        <v>29</v>
+        <v>80</v>
       </c>
       <c r="E131" t="inlineStr">
         <is>
@@ -3623,7 +3623,7 @@
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t>09:23:24</t>
+          <t>10:14:52</t>
         </is>
       </c>
       <c r="B132" t="inlineStr">
@@ -3633,11 +3633,11 @@
       </c>
       <c r="C132" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D132" t="n">
-        <v>80</v>
+        <v>29</v>
       </c>
       <c r="E132" t="inlineStr">
         <is>
@@ -3873,7 +3873,7 @@
     <row r="142">
       <c r="A142" t="inlineStr">
         <is>
-          <t>10:52:37</t>
+          <t>10:14:52</t>
         </is>
       </c>
       <c r="B142" t="inlineStr">
@@ -3883,11 +3883,11 @@
       </c>
       <c r="C142" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D142" t="n">
-        <v>11</v>
+        <v>49</v>
       </c>
       <c r="E142" t="inlineStr">
         <is>
@@ -3898,7 +3898,7 @@
     <row r="143">
       <c r="A143" t="inlineStr">
         <is>
-          <t>10:14:52</t>
+          <t>10:52:37</t>
         </is>
       </c>
       <c r="B143" t="inlineStr">
@@ -3908,11 +3908,11 @@
       </c>
       <c r="C143" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D143" t="n">
-        <v>49</v>
+        <v>11</v>
       </c>
       <c r="E143" t="inlineStr">
         <is>
@@ -4183,7 +4183,7 @@
       </c>
       <c r="C154" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D154" t="n">
@@ -4208,7 +4208,7 @@
       </c>
       <c r="C155" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D155" t="n">
@@ -4648,7 +4648,7 @@
     <row r="173">
       <c r="A173" t="inlineStr">
         <is>
-          <t>12:28:38</t>
+          <t>12:00:15</t>
         </is>
       </c>
       <c r="B173" t="inlineStr">
@@ -4658,11 +4658,11 @@
       </c>
       <c r="C173" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D173" t="n">
-        <v>5</v>
+        <v>33</v>
       </c>
       <c r="E173" t="inlineStr">
         <is>
@@ -4683,7 +4683,7 @@
       </c>
       <c r="C174" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D174" t="n">
@@ -4698,7 +4698,7 @@
     <row r="175">
       <c r="A175" t="inlineStr">
         <is>
-          <t>12:00:15</t>
+          <t>12:28:38</t>
         </is>
       </c>
       <c r="B175" t="inlineStr">
@@ -4708,11 +4708,11 @@
       </c>
       <c r="C175" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D175" t="n">
-        <v>33</v>
+        <v>5</v>
       </c>
       <c r="E175" t="inlineStr">
         <is>
@@ -5008,7 +5008,7 @@
       </c>
       <c r="C187" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D187" t="n">
@@ -5058,7 +5058,7 @@
       </c>
       <c r="C189" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D189" t="n">
@@ -5073,7 +5073,7 @@
     <row r="190">
       <c r="A190" t="inlineStr">
         <is>
-          <t>12:48:06</t>
+          <t>13:00:14</t>
         </is>
       </c>
       <c r="B190" t="inlineStr">
@@ -5083,11 +5083,11 @@
       </c>
       <c r="C190" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D190" t="n">
-        <v>16</v>
+        <v>4</v>
       </c>
       <c r="E190" t="inlineStr">
         <is>
@@ -5098,7 +5098,7 @@
     <row r="191">
       <c r="A191" t="inlineStr">
         <is>
-          <t>13:00:14</t>
+          <t>12:48:06</t>
         </is>
       </c>
       <c r="B191" t="inlineStr">
@@ -5108,11 +5108,11 @@
       </c>
       <c r="C191" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D191" t="n">
-        <v>4</v>
+        <v>16</v>
       </c>
       <c r="E191" t="inlineStr">
         <is>
@@ -5323,7 +5323,7 @@
     <row r="200">
       <c r="A200" t="inlineStr">
         <is>
-          <t>13:00:14</t>
+          <t>12:48:06</t>
         </is>
       </c>
       <c r="B200" t="inlineStr">
@@ -5333,11 +5333,11 @@
       </c>
       <c r="C200" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D200" t="n">
-        <v>38</v>
+        <v>50</v>
       </c>
       <c r="E200" t="inlineStr">
         <is>
@@ -5348,7 +5348,7 @@
     <row r="201">
       <c r="A201" t="inlineStr">
         <is>
-          <t>12:48:06</t>
+          <t>13:00:14</t>
         </is>
       </c>
       <c r="B201" t="inlineStr">
@@ -5358,11 +5358,11 @@
       </c>
       <c r="C201" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D201" t="n">
-        <v>50</v>
+        <v>38</v>
       </c>
       <c r="E201" t="inlineStr">
         <is>
@@ -5623,7 +5623,7 @@
     <row r="212">
       <c r="A212" t="inlineStr">
         <is>
-          <t>13:57:43</t>
+          <t>13:32:57</t>
         </is>
       </c>
       <c r="B212" t="inlineStr">
@@ -5633,11 +5633,11 @@
       </c>
       <c r="C212" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D212" t="n">
-        <v>19</v>
+        <v>44</v>
       </c>
       <c r="E212" t="inlineStr">
         <is>
@@ -5648,7 +5648,7 @@
     <row r="213">
       <c r="A213" t="inlineStr">
         <is>
-          <t>13:32:57</t>
+          <t>13:57:43</t>
         </is>
       </c>
       <c r="B213" t="inlineStr">
@@ -5658,11 +5658,11 @@
       </c>
       <c r="C213" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D213" t="n">
-        <v>44</v>
+        <v>19</v>
       </c>
       <c r="E213" t="inlineStr">
         <is>
@@ -5673,7 +5673,7 @@
     <row r="214">
       <c r="A214" t="inlineStr">
         <is>
-          <t>13:57:43</t>
+          <t>13:00:14</t>
         </is>
       </c>
       <c r="B214" t="inlineStr">
@@ -5683,11 +5683,11 @@
       </c>
       <c r="C214" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D214" t="n">
-        <v>20</v>
+        <v>77</v>
       </c>
       <c r="E214" t="inlineStr">
         <is>
@@ -5698,7 +5698,7 @@
     <row r="215">
       <c r="A215" t="inlineStr">
         <is>
-          <t>13:00:14</t>
+          <t>13:57:43</t>
         </is>
       </c>
       <c r="B215" t="inlineStr">
@@ -5708,11 +5708,11 @@
       </c>
       <c r="C215" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D215" t="n">
-        <v>77</v>
+        <v>20</v>
       </c>
       <c r="E215" t="inlineStr">
         <is>
@@ -5873,7 +5873,7 @@
     <row r="222">
       <c r="A222" t="inlineStr">
         <is>
-          <t>13:00:14</t>
+          <t>14:21:42</t>
         </is>
       </c>
       <c r="B222" t="inlineStr">
@@ -5883,11 +5883,11 @@
       </c>
       <c r="C222" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D222" t="n">
-        <v>93</v>
+        <v>12</v>
       </c>
       <c r="E222" t="inlineStr">
         <is>
@@ -5898,7 +5898,7 @@
     <row r="223">
       <c r="A223" t="inlineStr">
         <is>
-          <t>14:21:42</t>
+          <t>13:00:14</t>
         </is>
       </c>
       <c r="B223" t="inlineStr">
@@ -5908,11 +5908,11 @@
       </c>
       <c r="C223" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D223" t="n">
-        <v>12</v>
+        <v>93</v>
       </c>
       <c r="E223" t="inlineStr">
         <is>
@@ -5983,7 +5983,7 @@
       </c>
       <c r="C226" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D226" t="n">
@@ -6008,7 +6008,7 @@
       </c>
       <c r="C227" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D227" t="n">
@@ -6098,7 +6098,7 @@
     <row r="231">
       <c r="A231" t="inlineStr">
         <is>
-          <t>14:46:39</t>
+          <t>14:59:00</t>
         </is>
       </c>
       <c r="B231" t="inlineStr">
@@ -6108,11 +6108,11 @@
       </c>
       <c r="C231" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>81_EL PELIGRO</t>
         </is>
       </c>
       <c r="D231" t="n">
-        <v>13</v>
+        <v>0</v>
       </c>
       <c r="E231" t="inlineStr">
         <is>
@@ -6123,7 +6123,7 @@
     <row r="232">
       <c r="A232" t="inlineStr">
         <is>
-          <t>14:59:00</t>
+          <t>14:46:39</t>
         </is>
       </c>
       <c r="B232" t="inlineStr">
@@ -6133,11 +6133,11 @@
       </c>
       <c r="C232" t="inlineStr">
         <is>
-          <t>81_EL PELIGRO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D232" t="n">
-        <v>0</v>
+        <v>13</v>
       </c>
       <c r="E232" t="inlineStr">
         <is>
@@ -6698,7 +6698,7 @@
     <row r="255">
       <c r="A255" t="inlineStr">
         <is>
-          <t>14:46:39</t>
+          <t>15:34:45</t>
         </is>
       </c>
       <c r="B255" t="inlineStr">
@@ -6708,11 +6708,11 @@
       </c>
       <c r="C255" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D255" t="n">
-        <v>68</v>
+        <v>20</v>
       </c>
       <c r="E255" t="inlineStr">
         <is>
@@ -6723,7 +6723,7 @@
     <row r="256">
       <c r="A256" t="inlineStr">
         <is>
-          <t>15:34:45</t>
+          <t>14:46:39</t>
         </is>
       </c>
       <c r="B256" t="inlineStr">
@@ -6733,11 +6733,11 @@
       </c>
       <c r="C256" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D256" t="n">
-        <v>20</v>
+        <v>68</v>
       </c>
       <c r="E256" t="inlineStr">
         <is>
@@ -6933,7 +6933,7 @@
       </c>
       <c r="C264" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>215_ALUAR</t>
         </is>
       </c>
       <c r="D264" t="n">
@@ -6958,7 +6958,7 @@
       </c>
       <c r="C265" t="inlineStr">
         <is>
-          <t>215_ALUAR</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D265" t="n">
@@ -7123,7 +7123,7 @@
     <row r="272">
       <c r="A272" t="inlineStr">
         <is>
-          <t>15:34:45</t>
+          <t>14:59:00</t>
         </is>
       </c>
       <c r="B272" t="inlineStr">
@@ -7133,11 +7133,11 @@
       </c>
       <c r="C272" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D272" t="n">
-        <v>62</v>
+        <v>97</v>
       </c>
       <c r="E272" t="inlineStr">
         <is>
@@ -7148,7 +7148,7 @@
     <row r="273">
       <c r="A273" t="inlineStr">
         <is>
-          <t>14:59:00</t>
+          <t>15:34:45</t>
         </is>
       </c>
       <c r="B273" t="inlineStr">
@@ -7158,11 +7158,11 @@
       </c>
       <c r="C273" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D273" t="n">
-        <v>97</v>
+        <v>62</v>
       </c>
       <c r="E273" t="inlineStr">
         <is>
@@ -7573,7 +7573,7 @@
     <row r="290">
       <c r="A290" t="inlineStr">
         <is>
-          <t>16:33:34</t>
+          <t>17:21:09</t>
         </is>
       </c>
       <c r="B290" t="inlineStr">
@@ -7583,11 +7583,11 @@
       </c>
       <c r="C290" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D290" t="n">
-        <v>51</v>
+        <v>3</v>
       </c>
       <c r="E290" t="inlineStr">
         <is>
@@ -7598,7 +7598,7 @@
     <row r="291">
       <c r="A291" t="inlineStr">
         <is>
-          <t>17:21:09</t>
+          <t>16:33:34</t>
         </is>
       </c>
       <c r="B291" t="inlineStr">
@@ -7608,11 +7608,11 @@
       </c>
       <c r="C291" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D291" t="n">
-        <v>3</v>
+        <v>51</v>
       </c>
       <c r="E291" t="inlineStr">
         <is>
@@ -7658,7 +7658,7 @@
       </c>
       <c r="C293" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D293" t="n">
@@ -7683,7 +7683,7 @@
       </c>
       <c r="C294" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D294" t="n">
@@ -7948,7 +7948,7 @@
     <row r="305">
       <c r="A305" t="inlineStr">
         <is>
-          <t>17:47:19</t>
+          <t>16:57:49</t>
         </is>
       </c>
       <c r="B305" t="inlineStr">
@@ -7958,11 +7958,11 @@
       </c>
       <c r="C305" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D305" t="n">
-        <v>12</v>
+        <v>62</v>
       </c>
       <c r="E305" t="inlineStr">
         <is>
@@ -7973,7 +7973,7 @@
     <row r="306">
       <c r="A306" t="inlineStr">
         <is>
-          <t>16:57:49</t>
+          <t>17:47:19</t>
         </is>
       </c>
       <c r="B306" t="inlineStr">
@@ -7983,11 +7983,11 @@
       </c>
       <c r="C306" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D306" t="n">
-        <v>62</v>
+        <v>12</v>
       </c>
       <c r="E306" t="inlineStr">
         <is>
@@ -8008,7 +8008,7 @@
       </c>
       <c r="C307" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D307" t="n">
@@ -8033,7 +8033,7 @@
       </c>
       <c r="C308" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D308" t="n">
@@ -8058,7 +8058,7 @@
       </c>
       <c r="C309" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D309" t="n">
@@ -8083,7 +8083,7 @@
       </c>
       <c r="C310" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D310" t="n">
@@ -8923,7 +8923,7 @@
     <row r="344">
       <c r="A344" t="inlineStr">
         <is>
-          <t>19:12:47</t>
+          <t>18:51:25</t>
         </is>
       </c>
       <c r="B344" t="inlineStr">
@@ -8933,11 +8933,11 @@
       </c>
       <c r="C344" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>225_GOMEZ</t>
         </is>
       </c>
       <c r="D344" t="n">
-        <v>11</v>
+        <v>32</v>
       </c>
       <c r="E344" t="inlineStr">
         <is>
@@ -8948,7 +8948,7 @@
     <row r="345">
       <c r="A345" t="inlineStr">
         <is>
-          <t>18:51:25</t>
+          <t>19:12:47</t>
         </is>
       </c>
       <c r="B345" t="inlineStr">
@@ -8958,11 +8958,11 @@
       </c>
       <c r="C345" t="inlineStr">
         <is>
-          <t>225_GOMEZ</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D345" t="n">
-        <v>32</v>
+        <v>11</v>
       </c>
       <c r="E345" t="inlineStr">
         <is>
@@ -9473,12 +9473,12 @@
     <row r="366">
       <c r="A366" t="inlineStr">
         <is>
-          <t>19:12:47</t>
+          <t>20:24:55</t>
         </is>
       </c>
       <c r="B366" t="inlineStr">
         <is>
-          <t>20:26</t>
+          <t>20:25</t>
         </is>
       </c>
       <c r="C366" t="inlineStr">
@@ -9487,7 +9487,7 @@
         </is>
       </c>
       <c r="D366" t="n">
-        <v>74</v>
+        <v>1</v>
       </c>
       <c r="E366" t="inlineStr">
         <is>
@@ -9498,12 +9498,12 @@
     <row r="367">
       <c r="A367" t="inlineStr">
         <is>
-          <t>19:59:19</t>
+          <t>19:12:47</t>
         </is>
       </c>
       <c r="B367" t="inlineStr">
         <is>
-          <t>20:27</t>
+          <t>20:26</t>
         </is>
       </c>
       <c r="C367" t="inlineStr">
@@ -9512,7 +9512,7 @@
         </is>
       </c>
       <c r="D367" t="n">
-        <v>28</v>
+        <v>74</v>
       </c>
       <c r="E367" t="inlineStr">
         <is>
@@ -9528,16 +9528,16 @@
       </c>
       <c r="B368" t="inlineStr">
         <is>
-          <t>20:28</t>
+          <t>20:27</t>
         </is>
       </c>
       <c r="C368" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D368" t="n">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="E368" t="inlineStr">
         <is>
@@ -9553,16 +9553,16 @@
       </c>
       <c r="B369" t="inlineStr">
         <is>
-          <t>20:32</t>
+          <t>20:28</t>
         </is>
       </c>
       <c r="C369" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D369" t="n">
-        <v>33</v>
+        <v>29</v>
       </c>
       <c r="E369" t="inlineStr">
         <is>
@@ -9573,21 +9573,21 @@
     <row r="370">
       <c r="A370" t="inlineStr">
         <is>
-          <t>19:12:47</t>
+          <t>20:24:55</t>
         </is>
       </c>
       <c r="B370" t="inlineStr">
         <is>
-          <t>20:34</t>
+          <t>20:31</t>
         </is>
       </c>
       <c r="C370" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D370" t="n">
-        <v>82</v>
+        <v>7</v>
       </c>
       <c r="E370" t="inlineStr">
         <is>
@@ -9603,16 +9603,16 @@
       </c>
       <c r="B371" t="inlineStr">
         <is>
-          <t>20:35</t>
+          <t>20:32</t>
         </is>
       </c>
       <c r="C371" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D371" t="n">
-        <v>36</v>
+        <v>33</v>
       </c>
       <c r="E371" t="inlineStr">
         <is>
@@ -9623,21 +9623,21 @@
     <row r="372">
       <c r="A372" t="inlineStr">
         <is>
-          <t>19:59:19</t>
+          <t>20:24:55</t>
         </is>
       </c>
       <c r="B372" t="inlineStr">
         <is>
-          <t>20:44</t>
+          <t>20:34</t>
         </is>
       </c>
       <c r="C372" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D372" t="n">
-        <v>45</v>
+        <v>10</v>
       </c>
       <c r="E372" t="inlineStr">
         <is>
@@ -9648,21 +9648,21 @@
     <row r="373">
       <c r="A373" t="inlineStr">
         <is>
-          <t>19:12:47</t>
+          <t>19:59:19</t>
         </is>
       </c>
       <c r="B373" t="inlineStr">
         <is>
-          <t>20:55</t>
+          <t>20:35</t>
         </is>
       </c>
       <c r="C373" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D373" t="n">
-        <v>103</v>
+        <v>36</v>
       </c>
       <c r="E373" t="inlineStr">
         <is>
@@ -9673,21 +9673,21 @@
     <row r="374">
       <c r="A374" t="inlineStr">
         <is>
-          <t>19:59:19</t>
+          <t>20:24:55</t>
         </is>
       </c>
       <c r="B374" t="inlineStr">
         <is>
-          <t>20:56</t>
+          <t>20:43</t>
         </is>
       </c>
       <c r="C374" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D374" t="n">
-        <v>57</v>
+        <v>19</v>
       </c>
       <c r="E374" t="inlineStr">
         <is>
@@ -9698,21 +9698,21 @@
     <row r="375">
       <c r="A375" t="inlineStr">
         <is>
-          <t>19:12:47</t>
+          <t>19:59:19</t>
         </is>
       </c>
       <c r="B375" t="inlineStr">
         <is>
-          <t>20:56</t>
+          <t>20:44</t>
         </is>
       </c>
       <c r="C375" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D375" t="n">
-        <v>104</v>
+        <v>45</v>
       </c>
       <c r="E375" t="inlineStr">
         <is>
@@ -9723,21 +9723,21 @@
     <row r="376">
       <c r="A376" t="inlineStr">
         <is>
-          <t>19:59:19</t>
+          <t>20:24:55</t>
         </is>
       </c>
       <c r="B376" t="inlineStr">
         <is>
-          <t>20:57</t>
+          <t>20:49</t>
         </is>
       </c>
       <c r="C376" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D376" t="n">
-        <v>58</v>
+        <v>25</v>
       </c>
       <c r="E376" t="inlineStr">
         <is>
@@ -9748,21 +9748,21 @@
     <row r="377">
       <c r="A377" t="inlineStr">
         <is>
-          <t>19:59:19</t>
+          <t>20:24:55</t>
         </is>
       </c>
       <c r="B377" t="inlineStr">
         <is>
-          <t>20:59</t>
+          <t>20:55</t>
         </is>
       </c>
       <c r="C377" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D377" t="n">
-        <v>60</v>
+        <v>31</v>
       </c>
       <c r="E377" t="inlineStr">
         <is>
@@ -9773,21 +9773,21 @@
     <row r="378">
       <c r="A378" t="inlineStr">
         <is>
-          <t>19:44:03</t>
+          <t>19:59:19</t>
         </is>
       </c>
       <c r="B378" t="inlineStr">
         <is>
-          <t>21:02</t>
+          <t>20:56</t>
         </is>
       </c>
       <c r="C378" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D378" t="n">
-        <v>78</v>
+        <v>57</v>
       </c>
       <c r="E378" t="inlineStr">
         <is>
@@ -9798,21 +9798,21 @@
     <row r="379">
       <c r="A379" t="inlineStr">
         <is>
-          <t>19:59:19</t>
+          <t>20:24:55</t>
         </is>
       </c>
       <c r="B379" t="inlineStr">
         <is>
-          <t>21:24</t>
+          <t>20:56</t>
         </is>
       </c>
       <c r="C379" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D379" t="n">
-        <v>85</v>
+        <v>32</v>
       </c>
       <c r="E379" t="inlineStr">
         <is>
@@ -9823,21 +9823,21 @@
     <row r="380">
       <c r="A380" t="inlineStr">
         <is>
-          <t>19:44:03</t>
+          <t>19:59:19</t>
         </is>
       </c>
       <c r="B380" t="inlineStr">
         <is>
-          <t>21:37</t>
+          <t>20:57</t>
         </is>
       </c>
       <c r="C380" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D380" t="n">
-        <v>113</v>
+        <v>58</v>
       </c>
       <c r="E380" t="inlineStr">
         <is>
@@ -9853,16 +9853,16 @@
       </c>
       <c r="B381" t="inlineStr">
         <is>
-          <t>21:49</t>
+          <t>20:59</t>
         </is>
       </c>
       <c r="C381" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D381" t="n">
-        <v>110</v>
+        <v>60</v>
       </c>
       <c r="E381" t="inlineStr">
         <is>
@@ -9873,21 +9873,21 @@
     <row r="382">
       <c r="A382" t="inlineStr">
         <is>
-          <t>19:59:19</t>
+          <t>19:44:03</t>
         </is>
       </c>
       <c r="B382" t="inlineStr">
         <is>
-          <t>21:50</t>
+          <t>21:02</t>
         </is>
       </c>
       <c r="C382" t="inlineStr">
         <is>
-          <t>84_COLONIA URQUIZA-ESC 49</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D382" t="n">
-        <v>111</v>
+        <v>78</v>
       </c>
       <c r="E382" t="inlineStr">
         <is>
@@ -9898,23 +9898,298 @@
     <row r="383">
       <c r="A383" t="inlineStr">
         <is>
+          <t>20:24:55</t>
+        </is>
+      </c>
+      <c r="B383" t="inlineStr">
+        <is>
+          <t>21:03</t>
+        </is>
+      </c>
+      <c r="C383" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D383" t="n">
+        <v>39</v>
+      </c>
+      <c r="E383" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="384">
+      <c r="A384" t="inlineStr">
+        <is>
+          <t>20:24:55</t>
+        </is>
+      </c>
+      <c r="B384" t="inlineStr">
+        <is>
+          <t>21:09</t>
+        </is>
+      </c>
+      <c r="C384" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D384" t="n">
+        <v>45</v>
+      </c>
+      <c r="E384" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="385">
+      <c r="A385" t="inlineStr">
+        <is>
+          <t>20:24:55</t>
+        </is>
+      </c>
+      <c r="B385" t="inlineStr">
+        <is>
+          <t>21:23</t>
+        </is>
+      </c>
+      <c r="C385" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D385" t="n">
+        <v>59</v>
+      </c>
+      <c r="E385" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="386">
+      <c r="A386" t="inlineStr">
+        <is>
+          <t>20:24:55</t>
+        </is>
+      </c>
+      <c r="B386" t="inlineStr">
+        <is>
+          <t>21:24</t>
+        </is>
+      </c>
+      <c r="C386" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D386" t="n">
+        <v>60</v>
+      </c>
+      <c r="E386" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="387">
+      <c r="A387" t="inlineStr">
+        <is>
           <t>19:59:19</t>
         </is>
       </c>
-      <c r="B383" t="inlineStr">
+      <c r="B387" t="inlineStr">
+        <is>
+          <t>21:24</t>
+        </is>
+      </c>
+      <c r="C387" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D387" t="n">
+        <v>85</v>
+      </c>
+      <c r="E387" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="388">
+      <c r="A388" t="inlineStr">
+        <is>
+          <t>19:44:03</t>
+        </is>
+      </c>
+      <c r="B388" t="inlineStr">
+        <is>
+          <t>21:37</t>
+        </is>
+      </c>
+      <c r="C388" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D388" t="n">
+        <v>113</v>
+      </c>
+      <c r="E388" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="389">
+      <c r="A389" t="inlineStr">
+        <is>
+          <t>20:24:55</t>
+        </is>
+      </c>
+      <c r="B389" t="inlineStr">
+        <is>
+          <t>21:48</t>
+        </is>
+      </c>
+      <c r="C389" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D389" t="n">
+        <v>84</v>
+      </c>
+      <c r="E389" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="390">
+      <c r="A390" t="inlineStr">
+        <is>
+          <t>20:24:55</t>
+        </is>
+      </c>
+      <c r="B390" t="inlineStr">
+        <is>
+          <t>21:49</t>
+        </is>
+      </c>
+      <c r="C390" t="inlineStr">
+        <is>
+          <t>84_COLONIA URQUIZA-ESC 49</t>
+        </is>
+      </c>
+      <c r="D390" t="n">
+        <v>85</v>
+      </c>
+      <c r="E390" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="391">
+      <c r="A391" t="inlineStr">
+        <is>
+          <t>19:59:19</t>
+        </is>
+      </c>
+      <c r="B391" t="inlineStr">
+        <is>
+          <t>21:49</t>
+        </is>
+      </c>
+      <c r="C391" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D391" t="n">
+        <v>110</v>
+      </c>
+      <c r="E391" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="392">
+      <c r="A392" t="inlineStr">
+        <is>
+          <t>19:59:19</t>
+        </is>
+      </c>
+      <c r="B392" t="inlineStr">
+        <is>
+          <t>21:50</t>
+        </is>
+      </c>
+      <c r="C392" t="inlineStr">
+        <is>
+          <t>84_COLONIA URQUIZA-ESC 49</t>
+        </is>
+      </c>
+      <c r="D392" t="n">
+        <v>111</v>
+      </c>
+      <c r="E392" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="393">
+      <c r="A393" t="inlineStr">
+        <is>
+          <t>19:59:19</t>
+        </is>
+      </c>
+      <c r="B393" t="inlineStr">
         <is>
           <t>21:52</t>
         </is>
       </c>
-      <c r="C383" t="inlineStr">
+      <c r="C393" t="inlineStr">
         <is>
           <t>15_ABASTO</t>
         </is>
       </c>
-      <c r="D383" t="n">
+      <c r="D393" t="n">
         <v>113</v>
       </c>
-      <c r="E383" t="inlineStr">
+      <c r="E393" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="394">
+      <c r="A394" t="inlineStr">
+        <is>
+          <t>20:24:55</t>
+        </is>
+      </c>
+      <c r="B394" t="inlineStr">
+        <is>
+          <t>22:18</t>
+        </is>
+      </c>
+      <c r="C394" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D394" t="n">
+        <v>114</v>
+      </c>
+      <c r="E394" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -9931,7 +10206,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E62"/>
+  <dimension ref="A1:E63"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -9944,14 +10219,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 19:59:19</t>
+          <t>Última actualización: 20:24:55</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 57</t>
+          <t>Total filas: 58</t>
         </is>
       </c>
     </row>
@@ -11335,12 +11610,12 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>19:59:19</t>
+          <t>20:24:55</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>20:44</t>
+          <t>20:43</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
@@ -11349,7 +11624,7 @@
         </is>
       </c>
       <c r="D60" t="n">
-        <v>45</v>
+        <v>19</v>
       </c>
       <c r="E60" t="inlineStr">
         <is>
@@ -11360,21 +11635,21 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>19:12:47</t>
+          <t>19:59:19</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>20:55</t>
+          <t>20:44</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D61" t="n">
-        <v>103</v>
+        <v>45</v>
       </c>
       <c r="E61" t="inlineStr">
         <is>
@@ -11385,23 +11660,48 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
+          <t>20:24:55</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>20:55</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D62" t="n">
+        <v>31</v>
+      </c>
+      <c r="E62" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
           <t>19:59:19</t>
         </is>
       </c>
-      <c r="B62" t="inlineStr">
+      <c r="B63" t="inlineStr">
         <is>
           <t>20:56</t>
         </is>
       </c>
-      <c r="C62" t="inlineStr">
+      <c r="C63" t="inlineStr">
         <is>
           <t>215A_EL PATO</t>
         </is>
       </c>
-      <c r="D62" t="n">
+      <c r="D63" t="n">
         <v>57</v>
       </c>
-      <c r="E62" t="inlineStr">
+      <c r="E63" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -11418,7 +11718,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E62"/>
+  <dimension ref="A1:E64"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -11431,14 +11731,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 19:59:19</t>
+          <t>Última actualización: 20:24:55</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 57</t>
+          <t>Total filas: 59</t>
         </is>
       </c>
     </row>
@@ -12822,7 +13122,7 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>19:12:47</t>
+          <t>20:24:55</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
@@ -12836,7 +13136,7 @@
         </is>
       </c>
       <c r="D60" t="n">
-        <v>92</v>
+        <v>20</v>
       </c>
       <c r="E60" t="inlineStr">
         <is>
@@ -12872,25 +13172,75 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
+          <t>20:24:55</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>21:36</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D62" t="n">
+        <v>72</v>
+      </c>
+      <c r="E62" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
           <t>19:59:19</t>
         </is>
       </c>
-      <c r="B62" t="inlineStr">
+      <c r="B63" t="inlineStr">
         <is>
           <t>21:37</t>
         </is>
       </c>
-      <c r="C62" t="inlineStr">
+      <c r="C63" t="inlineStr">
         <is>
           <t>215C_LA PLATA</t>
         </is>
       </c>
-      <c r="D62" t="n">
+      <c r="D63" t="n">
         <v>98</v>
       </c>
-      <c r="E62" t="inlineStr">
+      <c r="E63" t="inlineStr">
         <is>
           <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>20:24:55</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>22:11</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>215B_LP-P MOR-1 Y 57</t>
+        </is>
+      </c>
+      <c r="D64" t="n">
+        <v>107</v>
+      </c>
+      <c r="E64" t="inlineStr">
+        <is>
+          <t>L6173</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 1828
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-03-21.xlsx
+++ b/data/horarios-141-2026-03-21.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E394"/>
+  <dimension ref="A1:E402"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 20:24:55</t>
+          <t>Última actualización: 20:44:28</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 389</t>
+          <t>Total filas: 397</t>
         </is>
       </c>
     </row>
@@ -758,7 +758,7 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D17" t="n">
@@ -783,7 +783,7 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D18" t="n">
@@ -1158,7 +1158,7 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D33" t="n">
@@ -1183,7 +1183,7 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D34" t="n">
@@ -1558,7 +1558,7 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D49" t="n">
@@ -1583,7 +1583,7 @@
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D50" t="n">
@@ -1983,7 +1983,7 @@
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D66" t="n">
@@ -2033,7 +2033,7 @@
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D68" t="n">
@@ -2373,7 +2373,7 @@
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>07:27:35</t>
+          <t>08:50:55</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
@@ -2383,11 +2383,11 @@
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D82" t="n">
-        <v>84</v>
+        <v>1</v>
       </c>
       <c r="E82" t="inlineStr">
         <is>
@@ -2408,7 +2408,7 @@
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D83" t="n">
@@ -2423,7 +2423,7 @@
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>08:50:55</t>
+          <t>07:27:35</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
@@ -2433,11 +2433,11 @@
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D84" t="n">
-        <v>1</v>
+        <v>84</v>
       </c>
       <c r="E84" t="inlineStr">
         <is>
@@ -2698,7 +2698,7 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>08:50:55</t>
+          <t>08:14:14</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
@@ -2708,11 +2708,11 @@
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D95" t="n">
-        <v>28</v>
+        <v>64</v>
       </c>
       <c r="E95" t="inlineStr">
         <is>
@@ -2748,7 +2748,7 @@
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>08:14:14</t>
+          <t>08:50:55</t>
         </is>
       </c>
       <c r="B97" t="inlineStr">
@@ -2758,11 +2758,11 @@
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D97" t="n">
-        <v>64</v>
+        <v>28</v>
       </c>
       <c r="E97" t="inlineStr">
         <is>
@@ -2923,7 +2923,7 @@
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>08:14:14</t>
+          <t>09:23:24</t>
         </is>
       </c>
       <c r="B104" t="inlineStr">
@@ -2933,11 +2933,11 @@
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D104" t="n">
-        <v>79</v>
+        <v>10</v>
       </c>
       <c r="E104" t="inlineStr">
         <is>
@@ -2948,7 +2948,7 @@
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>09:23:24</t>
+          <t>08:14:14</t>
         </is>
       </c>
       <c r="B105" t="inlineStr">
@@ -2958,11 +2958,11 @@
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D105" t="n">
-        <v>10</v>
+        <v>79</v>
       </c>
       <c r="E105" t="inlineStr">
         <is>
@@ -3173,7 +3173,7 @@
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>09:23:24</t>
+          <t>08:50:55</t>
         </is>
       </c>
       <c r="B114" t="inlineStr">
@@ -3183,11 +3183,11 @@
       </c>
       <c r="C114" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D114" t="n">
-        <v>40</v>
+        <v>73</v>
       </c>
       <c r="E114" t="inlineStr">
         <is>
@@ -3198,7 +3198,7 @@
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>08:50:55</t>
+          <t>09:23:24</t>
         </is>
       </c>
       <c r="B115" t="inlineStr">
@@ -3208,11 +3208,11 @@
       </c>
       <c r="C115" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D115" t="n">
-        <v>73</v>
+        <v>40</v>
       </c>
       <c r="E115" t="inlineStr">
         <is>
@@ -4183,7 +4183,7 @@
       </c>
       <c r="C154" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D154" t="n">
@@ -4208,7 +4208,7 @@
       </c>
       <c r="C155" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D155" t="n">
@@ -4473,7 +4473,7 @@
     <row r="166">
       <c r="A166" t="inlineStr">
         <is>
-          <t>12:00:15</t>
+          <t>11:16:36</t>
         </is>
       </c>
       <c r="B166" t="inlineStr">
@@ -4483,11 +4483,11 @@
       </c>
       <c r="C166" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D166" t="n">
-        <v>4</v>
+        <v>48</v>
       </c>
       <c r="E166" t="inlineStr">
         <is>
@@ -4498,7 +4498,7 @@
     <row r="167">
       <c r="A167" t="inlineStr">
         <is>
-          <t>11:16:36</t>
+          <t>12:00:15</t>
         </is>
       </c>
       <c r="B167" t="inlineStr">
@@ -4508,11 +4508,11 @@
       </c>
       <c r="C167" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D167" t="n">
-        <v>48</v>
+        <v>4</v>
       </c>
       <c r="E167" t="inlineStr">
         <is>
@@ -5008,7 +5008,7 @@
       </c>
       <c r="C187" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D187" t="n">
@@ -5023,7 +5023,7 @@
     <row r="188">
       <c r="A188" t="inlineStr">
         <is>
-          <t>13:00:14</t>
+          <t>12:28:38</t>
         </is>
       </c>
       <c r="B188" t="inlineStr">
@@ -5033,11 +5033,11 @@
       </c>
       <c r="C188" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D188" t="n">
-        <v>3</v>
+        <v>35</v>
       </c>
       <c r="E188" t="inlineStr">
         <is>
@@ -5048,7 +5048,7 @@
     <row r="189">
       <c r="A189" t="inlineStr">
         <is>
-          <t>12:28:38</t>
+          <t>13:00:14</t>
         </is>
       </c>
       <c r="B189" t="inlineStr">
@@ -5058,11 +5058,11 @@
       </c>
       <c r="C189" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D189" t="n">
-        <v>35</v>
+        <v>3</v>
       </c>
       <c r="E189" t="inlineStr">
         <is>
@@ -5248,7 +5248,7 @@
     <row r="197">
       <c r="A197" t="inlineStr">
         <is>
-          <t>12:48:06</t>
+          <t>13:00:14</t>
         </is>
       </c>
       <c r="B197" t="inlineStr">
@@ -5258,11 +5258,11 @@
       </c>
       <c r="C197" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D197" t="n">
-        <v>45</v>
+        <v>33</v>
       </c>
       <c r="E197" t="inlineStr">
         <is>
@@ -5273,7 +5273,7 @@
     <row r="198">
       <c r="A198" t="inlineStr">
         <is>
-          <t>13:00:14</t>
+          <t>12:48:06</t>
         </is>
       </c>
       <c r="B198" t="inlineStr">
@@ -5283,11 +5283,11 @@
       </c>
       <c r="C198" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D198" t="n">
-        <v>33</v>
+        <v>45</v>
       </c>
       <c r="E198" t="inlineStr">
         <is>
@@ -5323,7 +5323,7 @@
     <row r="200">
       <c r="A200" t="inlineStr">
         <is>
-          <t>12:48:06</t>
+          <t>13:00:14</t>
         </is>
       </c>
       <c r="B200" t="inlineStr">
@@ -5333,11 +5333,11 @@
       </c>
       <c r="C200" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D200" t="n">
-        <v>50</v>
+        <v>38</v>
       </c>
       <c r="E200" t="inlineStr">
         <is>
@@ -5348,7 +5348,7 @@
     <row r="201">
       <c r="A201" t="inlineStr">
         <is>
-          <t>13:00:14</t>
+          <t>12:48:06</t>
         </is>
       </c>
       <c r="B201" t="inlineStr">
@@ -5358,11 +5358,11 @@
       </c>
       <c r="C201" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D201" t="n">
-        <v>38</v>
+        <v>50</v>
       </c>
       <c r="E201" t="inlineStr">
         <is>
@@ -5573,7 +5573,7 @@
     <row r="210">
       <c r="A210" t="inlineStr">
         <is>
-          <t>13:00:14</t>
+          <t>13:57:43</t>
         </is>
       </c>
       <c r="B210" t="inlineStr">
@@ -5583,11 +5583,11 @@
       </c>
       <c r="C210" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D210" t="n">
-        <v>63</v>
+        <v>6</v>
       </c>
       <c r="E210" t="inlineStr">
         <is>
@@ -5598,7 +5598,7 @@
     <row r="211">
       <c r="A211" t="inlineStr">
         <is>
-          <t>13:57:43</t>
+          <t>13:00:14</t>
         </is>
       </c>
       <c r="B211" t="inlineStr">
@@ -5608,11 +5608,11 @@
       </c>
       <c r="C211" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D211" t="n">
-        <v>6</v>
+        <v>63</v>
       </c>
       <c r="E211" t="inlineStr">
         <is>
@@ -5983,7 +5983,7 @@
       </c>
       <c r="C226" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D226" t="n">
@@ -6008,7 +6008,7 @@
       </c>
       <c r="C227" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D227" t="n">
@@ -6098,7 +6098,7 @@
     <row r="231">
       <c r="A231" t="inlineStr">
         <is>
-          <t>14:59:00</t>
+          <t>14:46:39</t>
         </is>
       </c>
       <c r="B231" t="inlineStr">
@@ -6108,11 +6108,11 @@
       </c>
       <c r="C231" t="inlineStr">
         <is>
-          <t>81_EL PELIGRO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D231" t="n">
-        <v>0</v>
+        <v>13</v>
       </c>
       <c r="E231" t="inlineStr">
         <is>
@@ -6123,7 +6123,7 @@
     <row r="232">
       <c r="A232" t="inlineStr">
         <is>
-          <t>14:46:39</t>
+          <t>14:59:00</t>
         </is>
       </c>
       <c r="B232" t="inlineStr">
@@ -6133,11 +6133,11 @@
       </c>
       <c r="C232" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>81_EL PELIGRO</t>
         </is>
       </c>
       <c r="D232" t="n">
-        <v>13</v>
+        <v>0</v>
       </c>
       <c r="E232" t="inlineStr">
         <is>
@@ -6173,7 +6173,7 @@
     <row r="234">
       <c r="A234" t="inlineStr">
         <is>
-          <t>14:59:00</t>
+          <t>14:46:39</t>
         </is>
       </c>
       <c r="B234" t="inlineStr">
@@ -6183,11 +6183,11 @@
       </c>
       <c r="C234" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D234" t="n">
-        <v>2</v>
+        <v>15</v>
       </c>
       <c r="E234" t="inlineStr">
         <is>
@@ -6198,7 +6198,7 @@
     <row r="235">
       <c r="A235" t="inlineStr">
         <is>
-          <t>14:46:39</t>
+          <t>14:59:00</t>
         </is>
       </c>
       <c r="B235" t="inlineStr">
@@ -6208,11 +6208,11 @@
       </c>
       <c r="C235" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D235" t="n">
-        <v>15</v>
+        <v>2</v>
       </c>
       <c r="E235" t="inlineStr">
         <is>
@@ -6933,7 +6933,7 @@
       </c>
       <c r="C264" t="inlineStr">
         <is>
-          <t>215_ALUAR</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D264" t="n">
@@ -6958,7 +6958,7 @@
       </c>
       <c r="C265" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>215_ALUAR</t>
         </is>
       </c>
       <c r="D265" t="n">
@@ -7123,7 +7123,7 @@
     <row r="272">
       <c r="A272" t="inlineStr">
         <is>
-          <t>14:59:00</t>
+          <t>15:34:45</t>
         </is>
       </c>
       <c r="B272" t="inlineStr">
@@ -7133,11 +7133,11 @@
       </c>
       <c r="C272" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D272" t="n">
-        <v>97</v>
+        <v>62</v>
       </c>
       <c r="E272" t="inlineStr">
         <is>
@@ -7148,7 +7148,7 @@
     <row r="273">
       <c r="A273" t="inlineStr">
         <is>
-          <t>15:34:45</t>
+          <t>14:59:00</t>
         </is>
       </c>
       <c r="B273" t="inlineStr">
@@ -7158,11 +7158,11 @@
       </c>
       <c r="C273" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D273" t="n">
-        <v>62</v>
+        <v>97</v>
       </c>
       <c r="E273" t="inlineStr">
         <is>
@@ -7573,7 +7573,7 @@
     <row r="290">
       <c r="A290" t="inlineStr">
         <is>
-          <t>17:21:09</t>
+          <t>16:33:34</t>
         </is>
       </c>
       <c r="B290" t="inlineStr">
@@ -7583,11 +7583,11 @@
       </c>
       <c r="C290" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D290" t="n">
-        <v>3</v>
+        <v>51</v>
       </c>
       <c r="E290" t="inlineStr">
         <is>
@@ -7598,7 +7598,7 @@
     <row r="291">
       <c r="A291" t="inlineStr">
         <is>
-          <t>16:33:34</t>
+          <t>17:21:09</t>
         </is>
       </c>
       <c r="B291" t="inlineStr">
@@ -7608,11 +7608,11 @@
       </c>
       <c r="C291" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D291" t="n">
-        <v>51</v>
+        <v>3</v>
       </c>
       <c r="E291" t="inlineStr">
         <is>
@@ -7648,7 +7648,7 @@
     <row r="293">
       <c r="A293" t="inlineStr">
         <is>
-          <t>17:21:09</t>
+          <t>16:33:34</t>
         </is>
       </c>
       <c r="B293" t="inlineStr">
@@ -7658,11 +7658,11 @@
       </c>
       <c r="C293" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D293" t="n">
-        <v>14</v>
+        <v>62</v>
       </c>
       <c r="E293" t="inlineStr">
         <is>
@@ -7683,7 +7683,7 @@
       </c>
       <c r="C294" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D294" t="n">
@@ -7698,7 +7698,7 @@
     <row r="295">
       <c r="A295" t="inlineStr">
         <is>
-          <t>16:33:34</t>
+          <t>17:21:09</t>
         </is>
       </c>
       <c r="B295" t="inlineStr">
@@ -7708,11 +7708,11 @@
       </c>
       <c r="C295" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D295" t="n">
-        <v>62</v>
+        <v>14</v>
       </c>
       <c r="E295" t="inlineStr">
         <is>
@@ -7833,7 +7833,7 @@
       </c>
       <c r="C300" t="inlineStr">
         <is>
-          <t>215_EL PELIGRO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D300" t="n">
@@ -7858,7 +7858,7 @@
       </c>
       <c r="C301" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>215_EL PELIGRO</t>
         </is>
       </c>
       <c r="D301" t="n">
@@ -7883,7 +7883,7 @@
       </c>
       <c r="C302" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>215_EL PELIGRO</t>
         </is>
       </c>
       <c r="D302" t="n">
@@ -7908,7 +7908,7 @@
       </c>
       <c r="C303" t="inlineStr">
         <is>
-          <t>215_EL PELIGRO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D303" t="n">
@@ -8083,7 +8083,7 @@
       </c>
       <c r="C310" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D310" t="n">
@@ -8108,7 +8108,7 @@
       </c>
       <c r="C311" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D311" t="n">
@@ -8158,7 +8158,7 @@
       </c>
       <c r="C313" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D313" t="n">
@@ -8183,7 +8183,7 @@
       </c>
       <c r="C314" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D314" t="n">
@@ -9698,7 +9698,7 @@
     <row r="375">
       <c r="A375" t="inlineStr">
         <is>
-          <t>19:59:19</t>
+          <t>20:44:28</t>
         </is>
       </c>
       <c r="B375" t="inlineStr">
@@ -9712,7 +9712,7 @@
         </is>
       </c>
       <c r="D375" t="n">
-        <v>45</v>
+        <v>0</v>
       </c>
       <c r="E375" t="inlineStr">
         <is>
@@ -9748,21 +9748,21 @@
     <row r="377">
       <c r="A377" t="inlineStr">
         <is>
-          <t>20:24:55</t>
+          <t>20:44:28</t>
         </is>
       </c>
       <c r="B377" t="inlineStr">
         <is>
-          <t>20:55</t>
+          <t>20:50</t>
         </is>
       </c>
       <c r="C377" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D377" t="n">
-        <v>31</v>
+        <v>6</v>
       </c>
       <c r="E377" t="inlineStr">
         <is>
@@ -9773,12 +9773,12 @@
     <row r="378">
       <c r="A378" t="inlineStr">
         <is>
-          <t>19:59:19</t>
+          <t>20:44:28</t>
         </is>
       </c>
       <c r="B378" t="inlineStr">
         <is>
-          <t>20:56</t>
+          <t>20:55</t>
         </is>
       </c>
       <c r="C378" t="inlineStr">
@@ -9787,7 +9787,7 @@
         </is>
       </c>
       <c r="D378" t="n">
-        <v>57</v>
+        <v>11</v>
       </c>
       <c r="E378" t="inlineStr">
         <is>
@@ -9798,7 +9798,7 @@
     <row r="379">
       <c r="A379" t="inlineStr">
         <is>
-          <t>20:24:55</t>
+          <t>19:59:19</t>
         </is>
       </c>
       <c r="B379" t="inlineStr">
@@ -9808,11 +9808,11 @@
       </c>
       <c r="C379" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D379" t="n">
-        <v>32</v>
+        <v>57</v>
       </c>
       <c r="E379" t="inlineStr">
         <is>
@@ -9823,12 +9823,12 @@
     <row r="380">
       <c r="A380" t="inlineStr">
         <is>
-          <t>19:59:19</t>
+          <t>20:44:28</t>
         </is>
       </c>
       <c r="B380" t="inlineStr">
         <is>
-          <t>20:57</t>
+          <t>20:56</t>
         </is>
       </c>
       <c r="C380" t="inlineStr">
@@ -9837,7 +9837,7 @@
         </is>
       </c>
       <c r="D380" t="n">
-        <v>58</v>
+        <v>12</v>
       </c>
       <c r="E380" t="inlineStr">
         <is>
@@ -9853,16 +9853,16 @@
       </c>
       <c r="B381" t="inlineStr">
         <is>
-          <t>20:59</t>
+          <t>20:57</t>
         </is>
       </c>
       <c r="C381" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D381" t="n">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="E381" t="inlineStr">
         <is>
@@ -9873,12 +9873,12 @@
     <row r="382">
       <c r="A382" t="inlineStr">
         <is>
-          <t>19:44:03</t>
+          <t>19:59:19</t>
         </is>
       </c>
       <c r="B382" t="inlineStr">
         <is>
-          <t>21:02</t>
+          <t>20:59</t>
         </is>
       </c>
       <c r="C382" t="inlineStr">
@@ -9887,7 +9887,7 @@
         </is>
       </c>
       <c r="D382" t="n">
-        <v>78</v>
+        <v>60</v>
       </c>
       <c r="E382" t="inlineStr">
         <is>
@@ -9898,21 +9898,21 @@
     <row r="383">
       <c r="A383" t="inlineStr">
         <is>
-          <t>20:24:55</t>
+          <t>19:44:03</t>
         </is>
       </c>
       <c r="B383" t="inlineStr">
         <is>
-          <t>21:03</t>
+          <t>21:02</t>
         </is>
       </c>
       <c r="C383" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D383" t="n">
-        <v>39</v>
+        <v>78</v>
       </c>
       <c r="E383" t="inlineStr">
         <is>
@@ -9928,16 +9928,16 @@
       </c>
       <c r="B384" t="inlineStr">
         <is>
-          <t>21:09</t>
+          <t>21:03</t>
         </is>
       </c>
       <c r="C384" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D384" t="n">
-        <v>45</v>
+        <v>39</v>
       </c>
       <c r="E384" t="inlineStr">
         <is>
@@ -9948,21 +9948,21 @@
     <row r="385">
       <c r="A385" t="inlineStr">
         <is>
-          <t>20:24:55</t>
+          <t>20:44:28</t>
         </is>
       </c>
       <c r="B385" t="inlineStr">
         <is>
-          <t>21:23</t>
+          <t>21:04</t>
         </is>
       </c>
       <c r="C385" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D385" t="n">
-        <v>59</v>
+        <v>20</v>
       </c>
       <c r="E385" t="inlineStr">
         <is>
@@ -9973,21 +9973,21 @@
     <row r="386">
       <c r="A386" t="inlineStr">
         <is>
-          <t>20:24:55</t>
+          <t>20:44:28</t>
         </is>
       </c>
       <c r="B386" t="inlineStr">
         <is>
-          <t>21:24</t>
+          <t>21:06</t>
         </is>
       </c>
       <c r="C386" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D386" t="n">
-        <v>60</v>
+        <v>22</v>
       </c>
       <c r="E386" t="inlineStr">
         <is>
@@ -9998,21 +9998,21 @@
     <row r="387">
       <c r="A387" t="inlineStr">
         <is>
-          <t>19:59:19</t>
+          <t>20:24:55</t>
         </is>
       </c>
       <c r="B387" t="inlineStr">
         <is>
-          <t>21:24</t>
+          <t>21:09</t>
         </is>
       </c>
       <c r="C387" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D387" t="n">
-        <v>85</v>
+        <v>45</v>
       </c>
       <c r="E387" t="inlineStr">
         <is>
@@ -10023,21 +10023,21 @@
     <row r="388">
       <c r="A388" t="inlineStr">
         <is>
-          <t>19:44:03</t>
+          <t>20:44:28</t>
         </is>
       </c>
       <c r="B388" t="inlineStr">
         <is>
-          <t>21:37</t>
+          <t>21:22</t>
         </is>
       </c>
       <c r="C388" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D388" t="n">
-        <v>113</v>
+        <v>38</v>
       </c>
       <c r="E388" t="inlineStr">
         <is>
@@ -10048,21 +10048,21 @@
     <row r="389">
       <c r="A389" t="inlineStr">
         <is>
-          <t>20:24:55</t>
+          <t>20:44:28</t>
         </is>
       </c>
       <c r="B389" t="inlineStr">
         <is>
-          <t>21:48</t>
+          <t>21:23</t>
         </is>
       </c>
       <c r="C389" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D389" t="n">
-        <v>84</v>
+        <v>39</v>
       </c>
       <c r="E389" t="inlineStr">
         <is>
@@ -10078,16 +10078,16 @@
       </c>
       <c r="B390" t="inlineStr">
         <is>
-          <t>21:49</t>
+          <t>21:24</t>
         </is>
       </c>
       <c r="C390" t="inlineStr">
         <is>
-          <t>84_COLONIA URQUIZA-ESC 49</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D390" t="n">
-        <v>85</v>
+        <v>60</v>
       </c>
       <c r="E390" t="inlineStr">
         <is>
@@ -10103,16 +10103,16 @@
       </c>
       <c r="B391" t="inlineStr">
         <is>
-          <t>21:49</t>
+          <t>21:24</t>
         </is>
       </c>
       <c r="C391" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D391" t="n">
-        <v>110</v>
+        <v>85</v>
       </c>
       <c r="E391" t="inlineStr">
         <is>
@@ -10123,21 +10123,21 @@
     <row r="392">
       <c r="A392" t="inlineStr">
         <is>
-          <t>19:59:19</t>
+          <t>20:44:28</t>
         </is>
       </c>
       <c r="B392" t="inlineStr">
         <is>
-          <t>21:50</t>
+          <t>21:34</t>
         </is>
       </c>
       <c r="C392" t="inlineStr">
         <is>
-          <t>84_COLONIA URQUIZA-ESC 49</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D392" t="n">
-        <v>111</v>
+        <v>50</v>
       </c>
       <c r="E392" t="inlineStr">
         <is>
@@ -10148,12 +10148,12 @@
     <row r="393">
       <c r="A393" t="inlineStr">
         <is>
-          <t>19:59:19</t>
+          <t>19:44:03</t>
         </is>
       </c>
       <c r="B393" t="inlineStr">
         <is>
-          <t>21:52</t>
+          <t>21:37</t>
         </is>
       </c>
       <c r="C393" t="inlineStr">
@@ -10178,18 +10178,218 @@
       </c>
       <c r="B394" t="inlineStr">
         <is>
+          <t>21:48</t>
+        </is>
+      </c>
+      <c r="C394" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D394" t="n">
+        <v>84</v>
+      </c>
+      <c r="E394" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="395">
+      <c r="A395" t="inlineStr">
+        <is>
+          <t>20:44:28</t>
+        </is>
+      </c>
+      <c r="B395" t="inlineStr">
+        <is>
+          <t>21:49</t>
+        </is>
+      </c>
+      <c r="C395" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D395" t="n">
+        <v>65</v>
+      </c>
+      <c r="E395" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="396">
+      <c r="A396" t="inlineStr">
+        <is>
+          <t>20:24:55</t>
+        </is>
+      </c>
+      <c r="B396" t="inlineStr">
+        <is>
+          <t>21:49</t>
+        </is>
+      </c>
+      <c r="C396" t="inlineStr">
+        <is>
+          <t>84_COLONIA URQUIZA-ESC 49</t>
+        </is>
+      </c>
+      <c r="D396" t="n">
+        <v>85</v>
+      </c>
+      <c r="E396" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="397">
+      <c r="A397" t="inlineStr">
+        <is>
+          <t>20:44:28</t>
+        </is>
+      </c>
+      <c r="B397" t="inlineStr">
+        <is>
+          <t>21:50</t>
+        </is>
+      </c>
+      <c r="C397" t="inlineStr">
+        <is>
+          <t>84_COLONIA URQUIZA-ESC 49</t>
+        </is>
+      </c>
+      <c r="D397" t="n">
+        <v>66</v>
+      </c>
+      <c r="E397" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="398">
+      <c r="A398" t="inlineStr">
+        <is>
+          <t>19:59:19</t>
+        </is>
+      </c>
+      <c r="B398" t="inlineStr">
+        <is>
+          <t>21:52</t>
+        </is>
+      </c>
+      <c r="C398" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D398" t="n">
+        <v>113</v>
+      </c>
+      <c r="E398" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="399">
+      <c r="A399" t="inlineStr">
+        <is>
+          <t>20:24:55</t>
+        </is>
+      </c>
+      <c r="B399" t="inlineStr">
+        <is>
           <t>22:18</t>
         </is>
       </c>
-      <c r="C394" t="inlineStr">
+      <c r="C399" t="inlineStr">
         <is>
           <t>10_OLMOS</t>
         </is>
       </c>
-      <c r="D394" t="n">
+      <c r="D399" t="n">
         <v>114</v>
       </c>
-      <c r="E394" t="inlineStr">
+      <c r="E399" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="400">
+      <c r="A400" t="inlineStr">
+        <is>
+          <t>20:44:28</t>
+        </is>
+      </c>
+      <c r="B400" t="inlineStr">
+        <is>
+          <t>22:19</t>
+        </is>
+      </c>
+      <c r="C400" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D400" t="n">
+        <v>95</v>
+      </c>
+      <c r="E400" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="401">
+      <c r="A401" t="inlineStr">
+        <is>
+          <t>20:44:28</t>
+        </is>
+      </c>
+      <c r="B401" t="inlineStr">
+        <is>
+          <t>22:26</t>
+        </is>
+      </c>
+      <c r="C401" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D401" t="n">
+        <v>102</v>
+      </c>
+      <c r="E401" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="402">
+      <c r="A402" t="inlineStr">
+        <is>
+          <t>20:44:28</t>
+        </is>
+      </c>
+      <c r="B402" t="inlineStr">
+        <is>
+          <t>22:30</t>
+        </is>
+      </c>
+      <c r="C402" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D402" t="n">
+        <v>106</v>
+      </c>
+      <c r="E402" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -10206,7 +10406,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E63"/>
+  <dimension ref="A1:E64"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -10219,14 +10419,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 20:24:55</t>
+          <t>Última actualización: 20:44:28</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 58</t>
+          <t>Total filas: 59</t>
         </is>
       </c>
     </row>
@@ -11370,7 +11570,7 @@
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>215_EL PELIGRO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D50" t="n">
@@ -11395,7 +11595,7 @@
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>215_EL PELIGRO</t>
         </is>
       </c>
       <c r="D51" t="n">
@@ -11635,7 +11835,7 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>19:59:19</t>
+          <t>20:44:28</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
@@ -11649,7 +11849,7 @@
         </is>
       </c>
       <c r="D61" t="n">
-        <v>45</v>
+        <v>0</v>
       </c>
       <c r="E61" t="inlineStr">
         <is>
@@ -11660,7 +11860,7 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>20:24:55</t>
+          <t>20:44:28</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
@@ -11674,7 +11874,7 @@
         </is>
       </c>
       <c r="D62" t="n">
-        <v>31</v>
+        <v>11</v>
       </c>
       <c r="E62" t="inlineStr">
         <is>
@@ -11702,6 +11902,31 @@
         <v>57</v>
       </c>
       <c r="E63" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>20:44:28</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>22:26</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D64" t="n">
+        <v>102</v>
+      </c>
+      <c r="E64" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -11718,7 +11943,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E64"/>
+  <dimension ref="A1:E67"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -11731,14 +11956,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 20:24:55</t>
+          <t>Última actualización: 20:44:28</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 59</t>
+          <t>Total filas: 62</t>
         </is>
       </c>
     </row>
@@ -13172,12 +13397,12 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>20:24:55</t>
+          <t>20:44:28</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>21:36</t>
+          <t>20:46</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
@@ -13186,7 +13411,7 @@
         </is>
       </c>
       <c r="D62" t="n">
-        <v>72</v>
+        <v>2</v>
       </c>
       <c r="E62" t="inlineStr">
         <is>
@@ -13197,12 +13422,12 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>19:59:19</t>
+          <t>20:24:55</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>21:37</t>
+          <t>21:36</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
@@ -13211,7 +13436,7 @@
         </is>
       </c>
       <c r="D63" t="n">
-        <v>98</v>
+        <v>72</v>
       </c>
       <c r="E63" t="inlineStr">
         <is>
@@ -13222,23 +13447,98 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
+          <t>20:44:28</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>21:37</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D64" t="n">
+        <v>53</v>
+      </c>
+      <c r="E64" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
           <t>20:24:55</t>
         </is>
       </c>
-      <c r="B64" t="inlineStr">
+      <c r="B65" t="inlineStr">
         <is>
           <t>22:11</t>
         </is>
       </c>
-      <c r="C64" t="inlineStr">
+      <c r="C65" t="inlineStr">
         <is>
           <t>215B_LP-P MOR-1 Y 57</t>
         </is>
       </c>
-      <c r="D64" t="n">
+      <c r="D65" t="n">
         <v>107</v>
       </c>
-      <c r="E64" t="inlineStr">
+      <c r="E65" t="inlineStr">
+        <is>
+          <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>20:44:28</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>22:12</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>215B_LP-P MOR-1 Y 57</t>
+        </is>
+      </c>
+      <c r="D66" t="n">
+        <v>88</v>
+      </c>
+      <c r="E66" t="inlineStr">
+        <is>
+          <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>20:44:28</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>22:32</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>215A_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D67" t="n">
+        <v>108</v>
+      </c>
+      <c r="E67" t="inlineStr">
         <is>
           <t>L6173</t>
         </is>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 1829
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-03-21.xlsx
+++ b/data/horarios-141-2026-03-21.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E402"/>
+  <dimension ref="A1:E409"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 20:44:28</t>
+          <t>Última actualización: 20:57:52</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 397</t>
+          <t>Total filas: 404</t>
         </is>
       </c>
     </row>
@@ -533,7 +533,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D8" t="n">
@@ -558,7 +558,7 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D9" t="n">
@@ -758,7 +758,7 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D17" t="n">
@@ -783,7 +783,7 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D18" t="n">
@@ -1558,7 +1558,7 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D49" t="n">
@@ -1583,7 +1583,7 @@
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D50" t="n">
@@ -1973,7 +1973,7 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>07:51:37</t>
+          <t>07:27:35</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
@@ -1983,11 +1983,11 @@
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D66" t="n">
-        <v>28</v>
+        <v>52</v>
       </c>
       <c r="E66" t="inlineStr">
         <is>
@@ -1998,7 +1998,7 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>07:27:35</t>
+          <t>07:51:37</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
@@ -2008,11 +2008,11 @@
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D67" t="n">
-        <v>52</v>
+        <v>28</v>
       </c>
       <c r="E67" t="inlineStr">
         <is>
@@ -2033,7 +2033,7 @@
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D68" t="n">
@@ -2233,7 +2233,7 @@
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D76" t="n">
@@ -2258,7 +2258,7 @@
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D77" t="n">
@@ -2373,7 +2373,7 @@
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>08:50:55</t>
+          <t>07:27:35</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
@@ -2383,11 +2383,11 @@
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D82" t="n">
-        <v>1</v>
+        <v>84</v>
       </c>
       <c r="E82" t="inlineStr">
         <is>
@@ -2408,7 +2408,7 @@
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D83" t="n">
@@ -2423,7 +2423,7 @@
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>07:27:35</t>
+          <t>08:50:55</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
@@ -2433,11 +2433,11 @@
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D84" t="n">
-        <v>84</v>
+        <v>1</v>
       </c>
       <c r="E84" t="inlineStr">
         <is>
@@ -2698,7 +2698,7 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>08:14:14</t>
+          <t>08:50:55</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
@@ -2708,11 +2708,11 @@
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>215_EL PELIGRO</t>
         </is>
       </c>
       <c r="D95" t="n">
-        <v>64</v>
+        <v>28</v>
       </c>
       <c r="E95" t="inlineStr">
         <is>
@@ -2733,7 +2733,7 @@
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>215_EL PELIGRO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D96" t="n">
@@ -2748,7 +2748,7 @@
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>08:50:55</t>
+          <t>08:14:14</t>
         </is>
       </c>
       <c r="B97" t="inlineStr">
@@ -2758,11 +2758,11 @@
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D97" t="n">
-        <v>28</v>
+        <v>64</v>
       </c>
       <c r="E97" t="inlineStr">
         <is>
@@ -3173,7 +3173,7 @@
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>08:50:55</t>
+          <t>09:23:24</t>
         </is>
       </c>
       <c r="B114" t="inlineStr">
@@ -3183,11 +3183,11 @@
       </c>
       <c r="C114" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D114" t="n">
-        <v>73</v>
+        <v>40</v>
       </c>
       <c r="E114" t="inlineStr">
         <is>
@@ -3198,7 +3198,7 @@
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>09:23:24</t>
+          <t>08:50:55</t>
         </is>
       </c>
       <c r="B115" t="inlineStr">
@@ -3208,11 +3208,11 @@
       </c>
       <c r="C115" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D115" t="n">
-        <v>40</v>
+        <v>73</v>
       </c>
       <c r="E115" t="inlineStr">
         <is>
@@ -3498,7 +3498,7 @@
     <row r="127">
       <c r="A127" t="inlineStr">
         <is>
-          <t>10:14:52</t>
+          <t>08:36:09</t>
         </is>
       </c>
       <c r="B127" t="inlineStr">
@@ -3508,11 +3508,11 @@
       </c>
       <c r="C127" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D127" t="n">
-        <v>19</v>
+        <v>117</v>
       </c>
       <c r="E127" t="inlineStr">
         <is>
@@ -3523,7 +3523,7 @@
     <row r="128">
       <c r="A128" t="inlineStr">
         <is>
-          <t>08:36:09</t>
+          <t>10:14:52</t>
         </is>
       </c>
       <c r="B128" t="inlineStr">
@@ -3533,11 +3533,11 @@
       </c>
       <c r="C128" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D128" t="n">
-        <v>117</v>
+        <v>19</v>
       </c>
       <c r="E128" t="inlineStr">
         <is>
@@ -4123,7 +4123,7 @@
     <row r="152">
       <c r="A152" t="inlineStr">
         <is>
-          <t>10:14:52</t>
+          <t>11:16:36</t>
         </is>
       </c>
       <c r="B152" t="inlineStr">
@@ -4133,11 +4133,11 @@
       </c>
       <c r="C152" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D152" t="n">
-        <v>78</v>
+        <v>16</v>
       </c>
       <c r="E152" t="inlineStr">
         <is>
@@ -4148,7 +4148,7 @@
     <row r="153">
       <c r="A153" t="inlineStr">
         <is>
-          <t>11:16:36</t>
+          <t>10:14:52</t>
         </is>
       </c>
       <c r="B153" t="inlineStr">
@@ -4158,11 +4158,11 @@
       </c>
       <c r="C153" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D153" t="n">
-        <v>16</v>
+        <v>78</v>
       </c>
       <c r="E153" t="inlineStr">
         <is>
@@ -5073,7 +5073,7 @@
     <row r="190">
       <c r="A190" t="inlineStr">
         <is>
-          <t>13:00:14</t>
+          <t>12:48:06</t>
         </is>
       </c>
       <c r="B190" t="inlineStr">
@@ -5083,11 +5083,11 @@
       </c>
       <c r="C190" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D190" t="n">
-        <v>4</v>
+        <v>16</v>
       </c>
       <c r="E190" t="inlineStr">
         <is>
@@ -5098,7 +5098,7 @@
     <row r="191">
       <c r="A191" t="inlineStr">
         <is>
-          <t>12:48:06</t>
+          <t>13:00:14</t>
         </is>
       </c>
       <c r="B191" t="inlineStr">
@@ -5108,11 +5108,11 @@
       </c>
       <c r="C191" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D191" t="n">
-        <v>16</v>
+        <v>4</v>
       </c>
       <c r="E191" t="inlineStr">
         <is>
@@ -5248,7 +5248,7 @@
     <row r="197">
       <c r="A197" t="inlineStr">
         <is>
-          <t>13:00:14</t>
+          <t>12:48:06</t>
         </is>
       </c>
       <c r="B197" t="inlineStr">
@@ -5258,11 +5258,11 @@
       </c>
       <c r="C197" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D197" t="n">
-        <v>33</v>
+        <v>45</v>
       </c>
       <c r="E197" t="inlineStr">
         <is>
@@ -5273,7 +5273,7 @@
     <row r="198">
       <c r="A198" t="inlineStr">
         <is>
-          <t>12:48:06</t>
+          <t>13:00:14</t>
         </is>
       </c>
       <c r="B198" t="inlineStr">
@@ -5283,11 +5283,11 @@
       </c>
       <c r="C198" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D198" t="n">
-        <v>45</v>
+        <v>33</v>
       </c>
       <c r="E198" t="inlineStr">
         <is>
@@ -5323,7 +5323,7 @@
     <row r="200">
       <c r="A200" t="inlineStr">
         <is>
-          <t>13:00:14</t>
+          <t>12:48:06</t>
         </is>
       </c>
       <c r="B200" t="inlineStr">
@@ -5333,11 +5333,11 @@
       </c>
       <c r="C200" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D200" t="n">
-        <v>38</v>
+        <v>50</v>
       </c>
       <c r="E200" t="inlineStr">
         <is>
@@ -5348,7 +5348,7 @@
     <row r="201">
       <c r="A201" t="inlineStr">
         <is>
-          <t>12:48:06</t>
+          <t>13:00:14</t>
         </is>
       </c>
       <c r="B201" t="inlineStr">
@@ -5358,11 +5358,11 @@
       </c>
       <c r="C201" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D201" t="n">
-        <v>50</v>
+        <v>38</v>
       </c>
       <c r="E201" t="inlineStr">
         <is>
@@ -5623,7 +5623,7 @@
     <row r="212">
       <c r="A212" t="inlineStr">
         <is>
-          <t>13:32:57</t>
+          <t>13:57:43</t>
         </is>
       </c>
       <c r="B212" t="inlineStr">
@@ -5633,11 +5633,11 @@
       </c>
       <c r="C212" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D212" t="n">
-        <v>44</v>
+        <v>19</v>
       </c>
       <c r="E212" t="inlineStr">
         <is>
@@ -5648,7 +5648,7 @@
     <row r="213">
       <c r="A213" t="inlineStr">
         <is>
-          <t>13:57:43</t>
+          <t>13:32:57</t>
         </is>
       </c>
       <c r="B213" t="inlineStr">
@@ -5658,11 +5658,11 @@
       </c>
       <c r="C213" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D213" t="n">
-        <v>19</v>
+        <v>44</v>
       </c>
       <c r="E213" t="inlineStr">
         <is>
@@ -5673,7 +5673,7 @@
     <row r="214">
       <c r="A214" t="inlineStr">
         <is>
-          <t>13:00:14</t>
+          <t>13:57:43</t>
         </is>
       </c>
       <c r="B214" t="inlineStr">
@@ -5683,11 +5683,11 @@
       </c>
       <c r="C214" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D214" t="n">
-        <v>77</v>
+        <v>20</v>
       </c>
       <c r="E214" t="inlineStr">
         <is>
@@ -5698,7 +5698,7 @@
     <row r="215">
       <c r="A215" t="inlineStr">
         <is>
-          <t>13:57:43</t>
+          <t>13:00:14</t>
         </is>
       </c>
       <c r="B215" t="inlineStr">
@@ -5708,11 +5708,11 @@
       </c>
       <c r="C215" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D215" t="n">
-        <v>20</v>
+        <v>77</v>
       </c>
       <c r="E215" t="inlineStr">
         <is>
@@ -5983,7 +5983,7 @@
       </c>
       <c r="C226" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D226" t="n">
@@ -6008,7 +6008,7 @@
       </c>
       <c r="C227" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D227" t="n">
@@ -6698,7 +6698,7 @@
     <row r="255">
       <c r="A255" t="inlineStr">
         <is>
-          <t>15:34:45</t>
+          <t>14:46:39</t>
         </is>
       </c>
       <c r="B255" t="inlineStr">
@@ -6708,11 +6708,11 @@
       </c>
       <c r="C255" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D255" t="n">
-        <v>20</v>
+        <v>68</v>
       </c>
       <c r="E255" t="inlineStr">
         <is>
@@ -6723,7 +6723,7 @@
     <row r="256">
       <c r="A256" t="inlineStr">
         <is>
-          <t>14:46:39</t>
+          <t>15:34:45</t>
         </is>
       </c>
       <c r="B256" t="inlineStr">
@@ -6733,11 +6733,11 @@
       </c>
       <c r="C256" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D256" t="n">
-        <v>68</v>
+        <v>20</v>
       </c>
       <c r="E256" t="inlineStr">
         <is>
@@ -6933,7 +6933,7 @@
       </c>
       <c r="C264" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>215_ALUAR</t>
         </is>
       </c>
       <c r="D264" t="n">
@@ -6958,7 +6958,7 @@
       </c>
       <c r="C265" t="inlineStr">
         <is>
-          <t>215_ALUAR</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D265" t="n">
@@ -7033,7 +7033,7 @@
       </c>
       <c r="C268" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D268" t="n">
@@ -7058,7 +7058,7 @@
       </c>
       <c r="C269" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D269" t="n">
@@ -7073,7 +7073,7 @@
     <row r="270">
       <c r="A270" t="inlineStr">
         <is>
-          <t>16:01:44</t>
+          <t>16:33:34</t>
         </is>
       </c>
       <c r="B270" t="inlineStr">
@@ -7083,11 +7083,11 @@
       </c>
       <c r="C270" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D270" t="n">
-        <v>34</v>
+        <v>2</v>
       </c>
       <c r="E270" t="inlineStr">
         <is>
@@ -7098,7 +7098,7 @@
     <row r="271">
       <c r="A271" t="inlineStr">
         <is>
-          <t>16:33:34</t>
+          <t>16:01:44</t>
         </is>
       </c>
       <c r="B271" t="inlineStr">
@@ -7108,11 +7108,11 @@
       </c>
       <c r="C271" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D271" t="n">
-        <v>2</v>
+        <v>34</v>
       </c>
       <c r="E271" t="inlineStr">
         <is>
@@ -7648,7 +7648,7 @@
     <row r="293">
       <c r="A293" t="inlineStr">
         <is>
-          <t>16:33:34</t>
+          <t>17:21:09</t>
         </is>
       </c>
       <c r="B293" t="inlineStr">
@@ -7658,11 +7658,11 @@
       </c>
       <c r="C293" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D293" t="n">
-        <v>62</v>
+        <v>14</v>
       </c>
       <c r="E293" t="inlineStr">
         <is>
@@ -7673,7 +7673,7 @@
     <row r="294">
       <c r="A294" t="inlineStr">
         <is>
-          <t>17:21:09</t>
+          <t>16:33:34</t>
         </is>
       </c>
       <c r="B294" t="inlineStr">
@@ -7683,11 +7683,11 @@
       </c>
       <c r="C294" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D294" t="n">
-        <v>14</v>
+        <v>62</v>
       </c>
       <c r="E294" t="inlineStr">
         <is>
@@ -7708,7 +7708,7 @@
       </c>
       <c r="C295" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D295" t="n">
@@ -7833,7 +7833,7 @@
       </c>
       <c r="C300" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>215_EL PELIGRO</t>
         </is>
       </c>
       <c r="D300" t="n">
@@ -7858,7 +7858,7 @@
       </c>
       <c r="C301" t="inlineStr">
         <is>
-          <t>215_EL PELIGRO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D301" t="n">
@@ -7883,7 +7883,7 @@
       </c>
       <c r="C302" t="inlineStr">
         <is>
-          <t>215_EL PELIGRO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D302" t="n">
@@ -7908,7 +7908,7 @@
       </c>
       <c r="C303" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>215_EL PELIGRO</t>
         </is>
       </c>
       <c r="D303" t="n">
@@ -7948,7 +7948,7 @@
     <row r="305">
       <c r="A305" t="inlineStr">
         <is>
-          <t>16:57:49</t>
+          <t>17:47:19</t>
         </is>
       </c>
       <c r="B305" t="inlineStr">
@@ -7958,11 +7958,11 @@
       </c>
       <c r="C305" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D305" t="n">
-        <v>62</v>
+        <v>12</v>
       </c>
       <c r="E305" t="inlineStr">
         <is>
@@ -7973,7 +7973,7 @@
     <row r="306">
       <c r="A306" t="inlineStr">
         <is>
-          <t>17:47:19</t>
+          <t>16:57:49</t>
         </is>
       </c>
       <c r="B306" t="inlineStr">
@@ -7983,11 +7983,11 @@
       </c>
       <c r="C306" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D306" t="n">
-        <v>12</v>
+        <v>62</v>
       </c>
       <c r="E306" t="inlineStr">
         <is>
@@ -8923,7 +8923,7 @@
     <row r="344">
       <c r="A344" t="inlineStr">
         <is>
-          <t>18:51:25</t>
+          <t>19:12:47</t>
         </is>
       </c>
       <c r="B344" t="inlineStr">
@@ -8933,11 +8933,11 @@
       </c>
       <c r="C344" t="inlineStr">
         <is>
-          <t>225_GOMEZ</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D344" t="n">
-        <v>32</v>
+        <v>11</v>
       </c>
       <c r="E344" t="inlineStr">
         <is>
@@ -8948,7 +8948,7 @@
     <row r="345">
       <c r="A345" t="inlineStr">
         <is>
-          <t>19:12:47</t>
+          <t>18:51:25</t>
         </is>
       </c>
       <c r="B345" t="inlineStr">
@@ -8958,11 +8958,11 @@
       </c>
       <c r="C345" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>225_GOMEZ</t>
         </is>
       </c>
       <c r="D345" t="n">
-        <v>11</v>
+        <v>32</v>
       </c>
       <c r="E345" t="inlineStr">
         <is>
@@ -9848,7 +9848,7 @@
     <row r="381">
       <c r="A381" t="inlineStr">
         <is>
-          <t>19:59:19</t>
+          <t>20:57:52</t>
         </is>
       </c>
       <c r="B381" t="inlineStr">
@@ -9862,7 +9862,7 @@
         </is>
       </c>
       <c r="D381" t="n">
-        <v>58</v>
+        <v>0</v>
       </c>
       <c r="E381" t="inlineStr">
         <is>
@@ -9973,12 +9973,12 @@
     <row r="386">
       <c r="A386" t="inlineStr">
         <is>
-          <t>20:44:28</t>
+          <t>20:57:52</t>
         </is>
       </c>
       <c r="B386" t="inlineStr">
         <is>
-          <t>21:06</t>
+          <t>21:05</t>
         </is>
       </c>
       <c r="C386" t="inlineStr">
@@ -9987,7 +9987,7 @@
         </is>
       </c>
       <c r="D386" t="n">
-        <v>22</v>
+        <v>8</v>
       </c>
       <c r="E386" t="inlineStr">
         <is>
@@ -9998,21 +9998,21 @@
     <row r="387">
       <c r="A387" t="inlineStr">
         <is>
-          <t>20:24:55</t>
+          <t>20:57:52</t>
         </is>
       </c>
       <c r="B387" t="inlineStr">
         <is>
-          <t>21:09</t>
+          <t>21:05</t>
         </is>
       </c>
       <c r="C387" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D387" t="n">
-        <v>45</v>
+        <v>8</v>
       </c>
       <c r="E387" t="inlineStr">
         <is>
@@ -10028,16 +10028,16 @@
       </c>
       <c r="B388" t="inlineStr">
         <is>
-          <t>21:22</t>
+          <t>21:06</t>
         </is>
       </c>
       <c r="C388" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D388" t="n">
-        <v>38</v>
+        <v>22</v>
       </c>
       <c r="E388" t="inlineStr">
         <is>
@@ -10048,21 +10048,21 @@
     <row r="389">
       <c r="A389" t="inlineStr">
         <is>
-          <t>20:44:28</t>
+          <t>20:24:55</t>
         </is>
       </c>
       <c r="B389" t="inlineStr">
         <is>
-          <t>21:23</t>
+          <t>21:09</t>
         </is>
       </c>
       <c r="C389" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D389" t="n">
-        <v>39</v>
+        <v>45</v>
       </c>
       <c r="E389" t="inlineStr">
         <is>
@@ -10073,21 +10073,21 @@
     <row r="390">
       <c r="A390" t="inlineStr">
         <is>
-          <t>20:24:55</t>
+          <t>20:57:52</t>
         </is>
       </c>
       <c r="B390" t="inlineStr">
         <is>
-          <t>21:24</t>
+          <t>21:21</t>
         </is>
       </c>
       <c r="C390" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D390" t="n">
-        <v>60</v>
+        <v>24</v>
       </c>
       <c r="E390" t="inlineStr">
         <is>
@@ -10098,21 +10098,21 @@
     <row r="391">
       <c r="A391" t="inlineStr">
         <is>
-          <t>19:59:19</t>
+          <t>20:44:28</t>
         </is>
       </c>
       <c r="B391" t="inlineStr">
         <is>
-          <t>21:24</t>
+          <t>21:22</t>
         </is>
       </c>
       <c r="C391" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D391" t="n">
-        <v>85</v>
+        <v>38</v>
       </c>
       <c r="E391" t="inlineStr">
         <is>
@@ -10123,21 +10123,21 @@
     <row r="392">
       <c r="A392" t="inlineStr">
         <is>
-          <t>20:44:28</t>
+          <t>20:57:52</t>
         </is>
       </c>
       <c r="B392" t="inlineStr">
         <is>
-          <t>21:34</t>
+          <t>21:23</t>
         </is>
       </c>
       <c r="C392" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D392" t="n">
-        <v>50</v>
+        <v>26</v>
       </c>
       <c r="E392" t="inlineStr">
         <is>
@@ -10148,12 +10148,12 @@
     <row r="393">
       <c r="A393" t="inlineStr">
         <is>
-          <t>19:44:03</t>
+          <t>20:24:55</t>
         </is>
       </c>
       <c r="B393" t="inlineStr">
         <is>
-          <t>21:37</t>
+          <t>21:24</t>
         </is>
       </c>
       <c r="C393" t="inlineStr">
@@ -10162,7 +10162,7 @@
         </is>
       </c>
       <c r="D393" t="n">
-        <v>113</v>
+        <v>60</v>
       </c>
       <c r="E393" t="inlineStr">
         <is>
@@ -10173,21 +10173,21 @@
     <row r="394">
       <c r="A394" t="inlineStr">
         <is>
-          <t>20:24:55</t>
+          <t>19:59:19</t>
         </is>
       </c>
       <c r="B394" t="inlineStr">
         <is>
-          <t>21:48</t>
+          <t>21:24</t>
         </is>
       </c>
       <c r="C394" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D394" t="n">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="E394" t="inlineStr">
         <is>
@@ -10198,21 +10198,21 @@
     <row r="395">
       <c r="A395" t="inlineStr">
         <is>
-          <t>20:44:28</t>
+          <t>20:57:52</t>
         </is>
       </c>
       <c r="B395" t="inlineStr">
         <is>
-          <t>21:49</t>
+          <t>21:33</t>
         </is>
       </c>
       <c r="C395" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D395" t="n">
-        <v>65</v>
+        <v>36</v>
       </c>
       <c r="E395" t="inlineStr">
         <is>
@@ -10223,21 +10223,21 @@
     <row r="396">
       <c r="A396" t="inlineStr">
         <is>
-          <t>20:24:55</t>
+          <t>20:44:28</t>
         </is>
       </c>
       <c r="B396" t="inlineStr">
         <is>
-          <t>21:49</t>
+          <t>21:34</t>
         </is>
       </c>
       <c r="C396" t="inlineStr">
         <is>
-          <t>84_COLONIA URQUIZA-ESC 49</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D396" t="n">
-        <v>85</v>
+        <v>50</v>
       </c>
       <c r="E396" t="inlineStr">
         <is>
@@ -10248,21 +10248,21 @@
     <row r="397">
       <c r="A397" t="inlineStr">
         <is>
-          <t>20:44:28</t>
+          <t>19:44:03</t>
         </is>
       </c>
       <c r="B397" t="inlineStr">
         <is>
-          <t>21:50</t>
+          <t>21:37</t>
         </is>
       </c>
       <c r="C397" t="inlineStr">
         <is>
-          <t>84_COLONIA URQUIZA-ESC 49</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D397" t="n">
-        <v>66</v>
+        <v>113</v>
       </c>
       <c r="E397" t="inlineStr">
         <is>
@@ -10273,21 +10273,21 @@
     <row r="398">
       <c r="A398" t="inlineStr">
         <is>
-          <t>19:59:19</t>
+          <t>20:57:52</t>
         </is>
       </c>
       <c r="B398" t="inlineStr">
         <is>
-          <t>21:52</t>
+          <t>21:48</t>
         </is>
       </c>
       <c r="C398" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D398" t="n">
-        <v>113</v>
+        <v>51</v>
       </c>
       <c r="E398" t="inlineStr">
         <is>
@@ -10298,21 +10298,21 @@
     <row r="399">
       <c r="A399" t="inlineStr">
         <is>
-          <t>20:24:55</t>
+          <t>20:57:52</t>
         </is>
       </c>
       <c r="B399" t="inlineStr">
         <is>
-          <t>22:18</t>
+          <t>21:49</t>
         </is>
       </c>
       <c r="C399" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>84_COLONIA URQUIZA-ESC 49</t>
         </is>
       </c>
       <c r="D399" t="n">
-        <v>114</v>
+        <v>52</v>
       </c>
       <c r="E399" t="inlineStr">
         <is>
@@ -10328,16 +10328,16 @@
       </c>
       <c r="B400" t="inlineStr">
         <is>
-          <t>22:19</t>
+          <t>21:49</t>
         </is>
       </c>
       <c r="C400" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D400" t="n">
-        <v>95</v>
+        <v>65</v>
       </c>
       <c r="E400" t="inlineStr">
         <is>
@@ -10353,16 +10353,16 @@
       </c>
       <c r="B401" t="inlineStr">
         <is>
-          <t>22:26</t>
+          <t>21:50</t>
         </is>
       </c>
       <c r="C401" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>84_COLONIA URQUIZA-ESC 49</t>
         </is>
       </c>
       <c r="D401" t="n">
-        <v>102</v>
+        <v>66</v>
       </c>
       <c r="E401" t="inlineStr">
         <is>
@@ -10373,23 +10373,198 @@
     <row r="402">
       <c r="A402" t="inlineStr">
         <is>
+          <t>19:59:19</t>
+        </is>
+      </c>
+      <c r="B402" t="inlineStr">
+        <is>
+          <t>21:52</t>
+        </is>
+      </c>
+      <c r="C402" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D402" t="n">
+        <v>113</v>
+      </c>
+      <c r="E402" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="403">
+      <c r="A403" t="inlineStr">
+        <is>
+          <t>20:57:52</t>
+        </is>
+      </c>
+      <c r="B403" t="inlineStr">
+        <is>
+          <t>22:18</t>
+        </is>
+      </c>
+      <c r="C403" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D403" t="n">
+        <v>81</v>
+      </c>
+      <c r="E403" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="404">
+      <c r="A404" t="inlineStr">
+        <is>
           <t>20:44:28</t>
         </is>
       </c>
-      <c r="B402" t="inlineStr">
+      <c r="B404" t="inlineStr">
+        <is>
+          <t>22:19</t>
+        </is>
+      </c>
+      <c r="C404" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D404" t="n">
+        <v>95</v>
+      </c>
+      <c r="E404" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="405">
+      <c r="A405" t="inlineStr">
+        <is>
+          <t>20:57:52</t>
+        </is>
+      </c>
+      <c r="B405" t="inlineStr">
+        <is>
+          <t>22:24</t>
+        </is>
+      </c>
+      <c r="C405" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D405" t="n">
+        <v>87</v>
+      </c>
+      <c r="E405" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="406">
+      <c r="A406" t="inlineStr">
+        <is>
+          <t>20:57:52</t>
+        </is>
+      </c>
+      <c r="B406" t="inlineStr">
+        <is>
+          <t>22:26</t>
+        </is>
+      </c>
+      <c r="C406" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D406" t="n">
+        <v>89</v>
+      </c>
+      <c r="E406" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="407">
+      <c r="A407" t="inlineStr">
+        <is>
+          <t>20:57:52</t>
+        </is>
+      </c>
+      <c r="B407" t="inlineStr">
+        <is>
+          <t>22:29</t>
+        </is>
+      </c>
+      <c r="C407" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D407" t="n">
+        <v>92</v>
+      </c>
+      <c r="E407" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="408">
+      <c r="A408" t="inlineStr">
+        <is>
+          <t>20:44:28</t>
+        </is>
+      </c>
+      <c r="B408" t="inlineStr">
         <is>
           <t>22:30</t>
         </is>
       </c>
-      <c r="C402" t="inlineStr">
+      <c r="C408" t="inlineStr">
         <is>
           <t>15_ABASTO</t>
         </is>
       </c>
-      <c r="D402" t="n">
+      <c r="D408" t="n">
         <v>106</v>
       </c>
-      <c r="E402" t="inlineStr">
+      <c r="E408" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="409">
+      <c r="A409" t="inlineStr">
+        <is>
+          <t>20:57:52</t>
+        </is>
+      </c>
+      <c r="B409" t="inlineStr">
+        <is>
+          <t>22:48</t>
+        </is>
+      </c>
+      <c r="C409" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D409" t="n">
+        <v>111</v>
+      </c>
+      <c r="E409" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -10419,7 +10594,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 20:44:28</t>
+          <t>Última actualización: 20:57:52</t>
         </is>
       </c>
     </row>
@@ -11910,7 +12085,7 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>20:44:28</t>
+          <t>20:57:52</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
@@ -11924,7 +12099,7 @@
         </is>
       </c>
       <c r="D64" t="n">
-        <v>102</v>
+        <v>89</v>
       </c>
       <c r="E64" t="inlineStr">
         <is>
@@ -11956,7 +12131,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 20:44:28</t>
+          <t>Última actualización: 20:57:52</t>
         </is>
       </c>
     </row>
@@ -13422,7 +13597,7 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>20:24:55</t>
+          <t>20:57:52</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
@@ -13436,7 +13611,7 @@
         </is>
       </c>
       <c r="D63" t="n">
-        <v>72</v>
+        <v>39</v>
       </c>
       <c r="E63" t="inlineStr">
         <is>
@@ -13472,7 +13647,7 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>20:24:55</t>
+          <t>20:57:52</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
@@ -13486,7 +13661,7 @@
         </is>
       </c>
       <c r="D65" t="n">
-        <v>107</v>
+        <v>74</v>
       </c>
       <c r="E65" t="inlineStr">
         <is>
@@ -13522,7 +13697,7 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>20:44:28</t>
+          <t>20:57:52</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
@@ -13536,7 +13711,7 @@
         </is>
       </c>
       <c r="D67" t="n">
-        <v>108</v>
+        <v>95</v>
       </c>
       <c r="E67" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 1830
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-03-21.xlsx
+++ b/data/horarios-141-2026-03-21.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E409"/>
+  <dimension ref="A1:E415"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 20:57:52</t>
+          <t>Última actualización: 22:52:50</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 404</t>
+          <t>Total filas: 410</t>
         </is>
       </c>
     </row>
@@ -1158,7 +1158,7 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D33" t="n">
@@ -1183,7 +1183,7 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D34" t="n">
@@ -1558,7 +1558,7 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D49" t="n">
@@ -1583,7 +1583,7 @@
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D50" t="n">
@@ -1973,7 +1973,7 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>07:27:35</t>
+          <t>07:51:37</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
@@ -1983,11 +1983,11 @@
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D66" t="n">
-        <v>52</v>
+        <v>28</v>
       </c>
       <c r="E66" t="inlineStr">
         <is>
@@ -2008,7 +2008,7 @@
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D67" t="n">
@@ -2023,7 +2023,7 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>07:51:37</t>
+          <t>07:27:35</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
@@ -2033,11 +2033,11 @@
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D68" t="n">
-        <v>28</v>
+        <v>52</v>
       </c>
       <c r="E68" t="inlineStr">
         <is>
@@ -2233,7 +2233,7 @@
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D76" t="n">
@@ -2258,7 +2258,7 @@
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D77" t="n">
@@ -2408,7 +2408,7 @@
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D83" t="n">
@@ -2433,7 +2433,7 @@
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D84" t="n">
@@ -2873,7 +2873,7 @@
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>07:51:37</t>
+          <t>08:36:09</t>
         </is>
       </c>
       <c r="B102" t="inlineStr">
@@ -2883,11 +2883,11 @@
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D102" t="n">
-        <v>98</v>
+        <v>53</v>
       </c>
       <c r="E102" t="inlineStr">
         <is>
@@ -2898,7 +2898,7 @@
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>08:36:09</t>
+          <t>07:51:37</t>
         </is>
       </c>
       <c r="B103" t="inlineStr">
@@ -2908,11 +2908,11 @@
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D103" t="n">
-        <v>53</v>
+        <v>98</v>
       </c>
       <c r="E103" t="inlineStr">
         <is>
@@ -2923,7 +2923,7 @@
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>09:23:24</t>
+          <t>08:14:14</t>
         </is>
       </c>
       <c r="B104" t="inlineStr">
@@ -2933,11 +2933,11 @@
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D104" t="n">
-        <v>10</v>
+        <v>79</v>
       </c>
       <c r="E104" t="inlineStr">
         <is>
@@ -2948,7 +2948,7 @@
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>08:14:14</t>
+          <t>09:23:24</t>
         </is>
       </c>
       <c r="B105" t="inlineStr">
@@ -2958,11 +2958,11 @@
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D105" t="n">
-        <v>79</v>
+        <v>10</v>
       </c>
       <c r="E105" t="inlineStr">
         <is>
@@ -3083,7 +3083,7 @@
       </c>
       <c r="C110" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D110" t="n">
@@ -3108,7 +3108,7 @@
       </c>
       <c r="C111" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D111" t="n">
@@ -3173,7 +3173,7 @@
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>09:23:24</t>
+          <t>08:50:55</t>
         </is>
       </c>
       <c r="B114" t="inlineStr">
@@ -3183,11 +3183,11 @@
       </c>
       <c r="C114" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D114" t="n">
-        <v>40</v>
+        <v>73</v>
       </c>
       <c r="E114" t="inlineStr">
         <is>
@@ -3198,7 +3198,7 @@
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>08:50:55</t>
+          <t>09:23:24</t>
         </is>
       </c>
       <c r="B115" t="inlineStr">
@@ -3208,11 +3208,11 @@
       </c>
       <c r="C115" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D115" t="n">
-        <v>73</v>
+        <v>40</v>
       </c>
       <c r="E115" t="inlineStr">
         <is>
@@ -3598,7 +3598,7 @@
     <row r="131">
       <c r="A131" t="inlineStr">
         <is>
-          <t>09:23:24</t>
+          <t>10:14:52</t>
         </is>
       </c>
       <c r="B131" t="inlineStr">
@@ -3608,11 +3608,11 @@
       </c>
       <c r="C131" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D131" t="n">
-        <v>80</v>
+        <v>29</v>
       </c>
       <c r="E131" t="inlineStr">
         <is>
@@ -3623,7 +3623,7 @@
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t>10:14:52</t>
+          <t>09:23:24</t>
         </is>
       </c>
       <c r="B132" t="inlineStr">
@@ -3633,11 +3633,11 @@
       </c>
       <c r="C132" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D132" t="n">
-        <v>29</v>
+        <v>80</v>
       </c>
       <c r="E132" t="inlineStr">
         <is>
@@ -3873,7 +3873,7 @@
     <row r="142">
       <c r="A142" t="inlineStr">
         <is>
-          <t>10:14:52</t>
+          <t>10:52:37</t>
         </is>
       </c>
       <c r="B142" t="inlineStr">
@@ -3883,11 +3883,11 @@
       </c>
       <c r="C142" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D142" t="n">
-        <v>49</v>
+        <v>11</v>
       </c>
       <c r="E142" t="inlineStr">
         <is>
@@ -3898,7 +3898,7 @@
     <row r="143">
       <c r="A143" t="inlineStr">
         <is>
-          <t>10:52:37</t>
+          <t>10:14:52</t>
         </is>
       </c>
       <c r="B143" t="inlineStr">
@@ -3908,11 +3908,11 @@
       </c>
       <c r="C143" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D143" t="n">
-        <v>11</v>
+        <v>49</v>
       </c>
       <c r="E143" t="inlineStr">
         <is>
@@ -4123,7 +4123,7 @@
     <row r="152">
       <c r="A152" t="inlineStr">
         <is>
-          <t>11:16:36</t>
+          <t>10:14:52</t>
         </is>
       </c>
       <c r="B152" t="inlineStr">
@@ -4133,11 +4133,11 @@
       </c>
       <c r="C152" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D152" t="n">
-        <v>16</v>
+        <v>78</v>
       </c>
       <c r="E152" t="inlineStr">
         <is>
@@ -4148,7 +4148,7 @@
     <row r="153">
       <c r="A153" t="inlineStr">
         <is>
-          <t>10:14:52</t>
+          <t>11:16:36</t>
         </is>
       </c>
       <c r="B153" t="inlineStr">
@@ -4158,11 +4158,11 @@
       </c>
       <c r="C153" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D153" t="n">
-        <v>78</v>
+        <v>16</v>
       </c>
       <c r="E153" t="inlineStr">
         <is>
@@ -5008,7 +5008,7 @@
       </c>
       <c r="C187" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D187" t="n">
@@ -5023,7 +5023,7 @@
     <row r="188">
       <c r="A188" t="inlineStr">
         <is>
-          <t>12:28:38</t>
+          <t>13:00:14</t>
         </is>
       </c>
       <c r="B188" t="inlineStr">
@@ -5033,11 +5033,11 @@
       </c>
       <c r="C188" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D188" t="n">
-        <v>35</v>
+        <v>3</v>
       </c>
       <c r="E188" t="inlineStr">
         <is>
@@ -5048,7 +5048,7 @@
     <row r="189">
       <c r="A189" t="inlineStr">
         <is>
-          <t>13:00:14</t>
+          <t>12:28:38</t>
         </is>
       </c>
       <c r="B189" t="inlineStr">
@@ -5058,11 +5058,11 @@
       </c>
       <c r="C189" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D189" t="n">
-        <v>3</v>
+        <v>35</v>
       </c>
       <c r="E189" t="inlineStr">
         <is>
@@ -5248,7 +5248,7 @@
     <row r="197">
       <c r="A197" t="inlineStr">
         <is>
-          <t>12:48:06</t>
+          <t>13:00:14</t>
         </is>
       </c>
       <c r="B197" t="inlineStr">
@@ -5258,11 +5258,11 @@
       </c>
       <c r="C197" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D197" t="n">
-        <v>45</v>
+        <v>33</v>
       </c>
       <c r="E197" t="inlineStr">
         <is>
@@ -5273,7 +5273,7 @@
     <row r="198">
       <c r="A198" t="inlineStr">
         <is>
-          <t>13:00:14</t>
+          <t>12:48:06</t>
         </is>
       </c>
       <c r="B198" t="inlineStr">
@@ -5283,11 +5283,11 @@
       </c>
       <c r="C198" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D198" t="n">
-        <v>33</v>
+        <v>45</v>
       </c>
       <c r="E198" t="inlineStr">
         <is>
@@ -5873,7 +5873,7 @@
     <row r="222">
       <c r="A222" t="inlineStr">
         <is>
-          <t>14:21:42</t>
+          <t>13:00:14</t>
         </is>
       </c>
       <c r="B222" t="inlineStr">
@@ -5883,11 +5883,11 @@
       </c>
       <c r="C222" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D222" t="n">
-        <v>12</v>
+        <v>93</v>
       </c>
       <c r="E222" t="inlineStr">
         <is>
@@ -5898,7 +5898,7 @@
     <row r="223">
       <c r="A223" t="inlineStr">
         <is>
-          <t>13:00:14</t>
+          <t>14:21:42</t>
         </is>
       </c>
       <c r="B223" t="inlineStr">
@@ -5908,11 +5908,11 @@
       </c>
       <c r="C223" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D223" t="n">
-        <v>93</v>
+        <v>12</v>
       </c>
       <c r="E223" t="inlineStr">
         <is>
@@ -5983,7 +5983,7 @@
       </c>
       <c r="C226" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D226" t="n">
@@ -6008,7 +6008,7 @@
       </c>
       <c r="C227" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D227" t="n">
@@ -6098,7 +6098,7 @@
     <row r="231">
       <c r="A231" t="inlineStr">
         <is>
-          <t>14:46:39</t>
+          <t>14:59:00</t>
         </is>
       </c>
       <c r="B231" t="inlineStr">
@@ -6108,11 +6108,11 @@
       </c>
       <c r="C231" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>81_EL PELIGRO</t>
         </is>
       </c>
       <c r="D231" t="n">
-        <v>13</v>
+        <v>0</v>
       </c>
       <c r="E231" t="inlineStr">
         <is>
@@ -6123,7 +6123,7 @@
     <row r="232">
       <c r="A232" t="inlineStr">
         <is>
-          <t>14:59:00</t>
+          <t>14:46:39</t>
         </is>
       </c>
       <c r="B232" t="inlineStr">
@@ -6133,11 +6133,11 @@
       </c>
       <c r="C232" t="inlineStr">
         <is>
-          <t>81_EL PELIGRO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D232" t="n">
-        <v>0</v>
+        <v>13</v>
       </c>
       <c r="E232" t="inlineStr">
         <is>
@@ -6933,7 +6933,7 @@
       </c>
       <c r="C264" t="inlineStr">
         <is>
-          <t>215_ALUAR</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D264" t="n">
@@ -6958,7 +6958,7 @@
       </c>
       <c r="C265" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>215_ALUAR</t>
         </is>
       </c>
       <c r="D265" t="n">
@@ -7033,7 +7033,7 @@
       </c>
       <c r="C268" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D268" t="n">
@@ -7058,7 +7058,7 @@
       </c>
       <c r="C269" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D269" t="n">
@@ -7073,7 +7073,7 @@
     <row r="270">
       <c r="A270" t="inlineStr">
         <is>
-          <t>16:33:34</t>
+          <t>16:01:44</t>
         </is>
       </c>
       <c r="B270" t="inlineStr">
@@ -7083,11 +7083,11 @@
       </c>
       <c r="C270" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D270" t="n">
-        <v>2</v>
+        <v>34</v>
       </c>
       <c r="E270" t="inlineStr">
         <is>
@@ -7098,7 +7098,7 @@
     <row r="271">
       <c r="A271" t="inlineStr">
         <is>
-          <t>16:01:44</t>
+          <t>16:33:34</t>
         </is>
       </c>
       <c r="B271" t="inlineStr">
@@ -7108,11 +7108,11 @@
       </c>
       <c r="C271" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D271" t="n">
-        <v>34</v>
+        <v>2</v>
       </c>
       <c r="E271" t="inlineStr">
         <is>
@@ -7333,7 +7333,7 @@
       </c>
       <c r="C280" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D280" t="n">
@@ -7358,7 +7358,7 @@
       </c>
       <c r="C281" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D281" t="n">
@@ -7383,7 +7383,7 @@
       </c>
       <c r="C282" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D282" t="n">
@@ -7408,7 +7408,7 @@
       </c>
       <c r="C283" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D283" t="n">
@@ -7648,7 +7648,7 @@
     <row r="293">
       <c r="A293" t="inlineStr">
         <is>
-          <t>17:21:09</t>
+          <t>16:33:34</t>
         </is>
       </c>
       <c r="B293" t="inlineStr">
@@ -7658,11 +7658,11 @@
       </c>
       <c r="C293" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D293" t="n">
-        <v>14</v>
+        <v>62</v>
       </c>
       <c r="E293" t="inlineStr">
         <is>
@@ -7673,7 +7673,7 @@
     <row r="294">
       <c r="A294" t="inlineStr">
         <is>
-          <t>16:33:34</t>
+          <t>17:21:09</t>
         </is>
       </c>
       <c r="B294" t="inlineStr">
@@ -7683,11 +7683,11 @@
       </c>
       <c r="C294" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D294" t="n">
-        <v>62</v>
+        <v>14</v>
       </c>
       <c r="E294" t="inlineStr">
         <is>
@@ -7708,7 +7708,7 @@
       </c>
       <c r="C295" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D295" t="n">
@@ -8083,7 +8083,7 @@
       </c>
       <c r="C310" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D310" t="n">
@@ -8108,7 +8108,7 @@
       </c>
       <c r="C311" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D311" t="n">
@@ -8158,7 +8158,7 @@
       </c>
       <c r="C313" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D313" t="n">
@@ -8183,7 +8183,7 @@
       </c>
       <c r="C314" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D314" t="n">
@@ -9983,7 +9983,7 @@
       </c>
       <c r="C386" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D386" t="n">
@@ -10008,7 +10008,7 @@
       </c>
       <c r="C387" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D387" t="n">
@@ -10148,7 +10148,7 @@
     <row r="393">
       <c r="A393" t="inlineStr">
         <is>
-          <t>20:24:55</t>
+          <t>19:59:19</t>
         </is>
       </c>
       <c r="B393" t="inlineStr">
@@ -10158,11 +10158,11 @@
       </c>
       <c r="C393" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D393" t="n">
-        <v>60</v>
+        <v>85</v>
       </c>
       <c r="E393" t="inlineStr">
         <is>
@@ -10173,7 +10173,7 @@
     <row r="394">
       <c r="A394" t="inlineStr">
         <is>
-          <t>19:59:19</t>
+          <t>20:24:55</t>
         </is>
       </c>
       <c r="B394" t="inlineStr">
@@ -10183,11 +10183,11 @@
       </c>
       <c r="C394" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D394" t="n">
-        <v>85</v>
+        <v>60</v>
       </c>
       <c r="E394" t="inlineStr">
         <is>
@@ -10565,6 +10565,156 @@
         <v>111</v>
       </c>
       <c r="E409" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="410">
+      <c r="A410" t="inlineStr">
+        <is>
+          <t>22:52:50</t>
+        </is>
+      </c>
+      <c r="B410" t="inlineStr">
+        <is>
+          <t>22:58</t>
+        </is>
+      </c>
+      <c r="C410" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D410" t="n">
+        <v>6</v>
+      </c>
+      <c r="E410" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="411">
+      <c r="A411" t="inlineStr">
+        <is>
+          <t>22:52:50</t>
+        </is>
+      </c>
+      <c r="B411" t="inlineStr">
+        <is>
+          <t>23:19</t>
+        </is>
+      </c>
+      <c r="C411" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D411" t="n">
+        <v>27</v>
+      </c>
+      <c r="E411" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="412">
+      <c r="A412" t="inlineStr">
+        <is>
+          <t>22:52:50</t>
+        </is>
+      </c>
+      <c r="B412" t="inlineStr">
+        <is>
+          <t>23:26</t>
+        </is>
+      </c>
+      <c r="C412" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D412" t="n">
+        <v>34</v>
+      </c>
+      <c r="E412" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="413">
+      <c r="A413" t="inlineStr">
+        <is>
+          <t>22:52:50</t>
+        </is>
+      </c>
+      <c r="B413" t="inlineStr">
+        <is>
+          <t>23:29</t>
+        </is>
+      </c>
+      <c r="C413" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D413" t="n">
+        <v>37</v>
+      </c>
+      <c r="E413" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="414">
+      <c r="A414" t="inlineStr">
+        <is>
+          <t>22:52:50</t>
+        </is>
+      </c>
+      <c r="B414" t="inlineStr">
+        <is>
+          <t>23:39</t>
+        </is>
+      </c>
+      <c r="C414" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D414" t="n">
+        <v>47</v>
+      </c>
+      <c r="E414" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="415">
+      <c r="A415" t="inlineStr">
+        <is>
+          <t>22:52:50</t>
+        </is>
+      </c>
+      <c r="B415" t="inlineStr">
+        <is>
+          <t>23:48</t>
+        </is>
+      </c>
+      <c r="C415" t="inlineStr">
+        <is>
+          <t>11X44_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D415" t="n">
+        <v>56</v>
+      </c>
+      <c r="E415" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -10581,7 +10731,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E64"/>
+  <dimension ref="A1:E65"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -10594,14 +10744,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 20:57:52</t>
+          <t>Última actualización: 22:52:50</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 59</t>
+          <t>Total filas: 60</t>
         </is>
       </c>
     </row>
@@ -12102,6 +12252,31 @@
         <v>89</v>
       </c>
       <c r="E64" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>22:52:50</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>23:39</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D65" t="n">
+        <v>47</v>
+      </c>
+      <c r="E65" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -12131,7 +12306,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 20:57:52</t>
+          <t>Última actualización: 22:52:50</t>
         </is>
       </c>
     </row>

</xml_diff>